<commit_message>
Fix false positive keyword match for 생활 관리
</commit_message>
<xml_diff>
--- a/reviews_with_keywords.xlsx
+++ b/reviews_with_keywords.xlsx
@@ -691,7 +691,7 @@
         <v>이투스247학원의 학습 상담 시스템 덕분에 저의 취약 과목을 객관적으로 파악하고 구체적인 보완 계획을 세울 수 있었어요.</v>
       </c>
       <c r="K8" t="str">
-        <v>학습 관리, 학습 계획</v>
+        <v>학습 관리</v>
       </c>
     </row>
     <row r="9">
@@ -1077,7 +1077,7 @@
         <v>잠 관리가 잘 안되는 편이였는데 생활 담임 선생님들이 아침에 깨워주셔서 규칙적인 학습 루틴을 유지할 수 있었어요.</v>
       </c>
       <c r="K19" t="str">
-        <v>학습 관리, 생활 관리</v>
+        <v/>
       </c>
     </row>
     <row r="20">
@@ -1276,7 +1276,7 @@
         <v>다른 독서실처럼 일방적으로 통제하기보다는 개인 상태에 맞춘 관리가 이루어져 훨씬 집중도 높은 학습이 가능했어요.</v>
       </c>
       <c r="K24" t="str">
-        <v>학습 관리</v>
+        <v/>
       </c>
     </row>
     <row r="25">
@@ -1560,7 +1560,7 @@
         <v>면학 분위기 관리와 감독이 잘 이루어져서 학습에 집중하기 좋은 환경이었어요.</v>
       </c>
       <c r="K32" t="str">
-        <v>학습 관리, 면학 분위기</v>
+        <v>면학 분위기</v>
       </c>
     </row>
     <row r="33">
@@ -2093,7 +2093,7 @@
         <v>졸음 관리와 생활 습관 교정에도 큰 도움을 주었어요.</v>
       </c>
       <c r="K47" t="str">
-        <v>생활 관리, 졸음 관리</v>
+        <v>졸음 관리</v>
       </c>
     </row>
     <row r="48">
@@ -2715,7 +2715,7 @@
         <v>학습 기록과 계획 확인을 반복하면서 스스로를 관리하는 힘이 생겼고, 공부 흐름을 꾸준히 유지할 수 있었어요.</v>
       </c>
       <c r="K64" t="str">
-        <v>학습 관리, 학습 계획</v>
+        <v/>
       </c>
     </row>
     <row r="65">
@@ -2785,7 +2785,7 @@
         <v>수준에 맞춘 학습 코칭과 질문 해결, 휴대폰 관리 덕분에 집중하며 공부할 수 있었어요.</v>
       </c>
       <c r="K66" t="str">
-        <v>학습 관리</v>
+        <v/>
       </c>
     </row>
     <row r="67">
@@ -2855,7 +2855,7 @@
         <v>이런 생활 관리 시스템 덕분에 학습 습관이 규칙적으로 잡히고 성과 향상에 큰 도움이 되었어요.</v>
       </c>
       <c r="K68" t="str">
-        <v>학습 관리, 생활 관리</v>
+        <v>생활 관리</v>
       </c>
     </row>
     <row r="69">
@@ -3256,7 +3256,7 @@
         <v>재수 생활을 시작하며 막막했던 제게 학습코칭은 단순한 스케줄 관리를 넘어선 '터닝 포인트'였어요.</v>
       </c>
       <c r="K79" t="str">
-        <v>학습 관리, 생활 관리</v>
+        <v/>
       </c>
     </row>
     <row r="80">
@@ -3334,7 +3334,7 @@
         <v>플래너 관리 덕분에 하루 단위로 학습 계획을 구체적으로 세우고 실천할 수 있어 시간 낭비를 줄였어요.</v>
       </c>
       <c r="K81" t="str">
-        <v>학습 관리, 학습 계획, 플래너 관리</v>
+        <v>학습 계획, 플래너 관리</v>
       </c>
     </row>
     <row r="82">
@@ -3584,7 +3584,7 @@
         <v>선생님과의 학습 상황 점검, 휴대폰 관리, 모의고사 분석 덕분에 끝까지 집중하며 완주할 수 있었어요.</v>
       </c>
       <c r="K88" t="str">
-        <v>학습 관리, 모의고사</v>
+        <v>모의고사</v>
       </c>
     </row>
     <row r="89">
@@ -3619,7 +3619,7 @@
         <v>선생님이 직접 관리하는 환경 덕분에 스스로 더 긴장감을 갖고 학습에 집중할 수 있었어요.</v>
       </c>
       <c r="K89" t="str">
-        <v>학습 관리</v>
+        <v/>
       </c>
     </row>
     <row r="90" xml:space="preserve">
@@ -3936,7 +3936,7 @@
         <v>학습 환경이 적절한지 체크하며 관리해주셔서 편하게 공부할 수 있었어요.</v>
       </c>
       <c r="K98" t="str">
-        <v>학습 관리</v>
+        <v/>
       </c>
     </row>
     <row r="99">
@@ -4055,7 +4055,7 @@
         <v>학습 보조 및 관리 측면에서는 제 성적을 누군가 지속적으로 점검해준다는 점에서 항상 긴장감을 유지하며 시험에 임할 수 있어 도움이 되었어요.</v>
       </c>
       <c r="K101" t="str">
-        <v>학습 관리</v>
+        <v/>
       </c>
     </row>
     <row r="102">
@@ -4090,7 +4090,7 @@
         <v>출석 관리가 체계적으로 이루어져 스스로 학습 태도를 점검할 수 있었고, 지각이나 결석을 줄이는 데에도 도움이 되었어요.</v>
       </c>
       <c r="K102" t="str">
-        <v>학습 관리</v>
+        <v/>
       </c>
     </row>
     <row r="103">
@@ -4306,7 +4306,7 @@
         <v>하루 공부량을 체계적으로 관리할 수 있었고, 생활 패턴도 규칙적으로 유지하는 데 도움이 되었어요.</v>
       </c>
       <c r="K108" t="str">
-        <v>생활 관리</v>
+        <v/>
       </c>
     </row>
     <row r="109" xml:space="preserve">
@@ -4377,7 +4377,7 @@
         <v>생활 관리와 맞춤 학습 코칭 덕분에 올바른 공부 습관이 생기고 집중력이 올라가서 합격까지 이어졌어요.</v>
       </c>
       <c r="K110" t="str">
-        <v>학습 관리, 생활 관리</v>
+        <v>생활 관리</v>
       </c>
     </row>
     <row r="111">
@@ -4447,7 +4447,7 @@
         <v>학습계획과 플래너 관리를 통해 하루 공부 흐름을 체계적으로 정리할 수 있었고, 목표를 구체적으로 세워 실천하는 데 큰 도움이 되었어요.</v>
       </c>
       <c r="K112" t="str">
-        <v>학습 관리, 학습 계획, 플래너 관리</v>
+        <v>학습 계획, 플래너 관리</v>
       </c>
     </row>
     <row r="113">
@@ -4592,7 +4592,7 @@
         <v>개인별 실시간 피드백과 전 과목 학습 방향 제시, 면학 분위기 관리 덕분에 목표 성적을 얻었어요.</v>
       </c>
       <c r="K116" t="str">
-        <v>학습 관리, 면학 분위기</v>
+        <v>면학 분위기</v>
       </c>
     </row>
     <row r="117">
@@ -4958,7 +4958,7 @@
         <v>원장님과 선생님들께서 제 학습 상황을 세심하게 파악하고 맞춤 계획을 제시해주셔서 심적으로도 안정감을 얻을 수 있었어요.</v>
       </c>
       <c r="K126" t="str">
-        <v>학습 계획</v>
+        <v/>
       </c>
     </row>
     <row r="127">
@@ -5063,7 +5063,7 @@
         <v>체계적인 플래너 관리와 학습 계획 분석 덕분에 '막연한 불안감'을 '확실한 성취감'으로 바꿀 수 있었어요.</v>
       </c>
       <c r="K129" t="str">
-        <v>학습 관리, 학습 계획, 플래너 관리</v>
+        <v>학습 계획, 플래너 관리</v>
       </c>
     </row>
     <row r="130">
@@ -5133,7 +5133,7 @@
         <v>주기적인 학습 점검과 1:1 과목별 질문, 휴대폰 관리 덕분에 계획을 보완하며 효율적으로 공부했어요.</v>
       </c>
       <c r="K131" t="str">
-        <v>학습 관리, 학습 계획</v>
+        <v/>
       </c>
     </row>
     <row r="132">
@@ -5420,7 +5420,7 @@
         <v>졸음 방지와 면학 분위기 관리 덕분에 집중력을 유지하고, 규칙적인 학습 루틴을 이어갈 수 있었어요.</v>
       </c>
       <c r="K139" t="str">
-        <v>학습 관리, 면학 분위기, 졸음 관리</v>
+        <v>면학 분위기</v>
       </c>
     </row>
     <row r="140">
@@ -5490,7 +5490,7 @@
         <v>저에게 맞는 좋은 인강들을 추천받을 수 있어서 만족스러웠고, 선생님들의 세심한 관리 덕분에 안정적으로 공부할 수 있었어요.</v>
       </c>
       <c r="K141" t="str">
-        <v>인강 추천</v>
+        <v/>
       </c>
     </row>
     <row r="142" xml:space="preserve">
@@ -5596,7 +5596,7 @@
         <v>담임선생님의 인강, 교재 추천 덕분에 제 수준에 맞게 공부해 수학 성적 향상과 국어 학습 습관 형성에 도움이 되었어요.</v>
       </c>
       <c r="K144" t="str">
-        <v>인강 추천</v>
+        <v/>
       </c>
     </row>
     <row r="145">
@@ -5673,7 +5673,7 @@
         <v>플래너 관리로 과목별 공부 시간을 균형 있게 세우고, 매일 실천 여부를 점검하며 학습 효율을 높일 수 있었어요.</v>
       </c>
       <c r="K146" t="str">
-        <v>학습 관리, 플래너 관리</v>
+        <v>플래너 관리</v>
       </c>
     </row>
     <row r="147">
@@ -5785,7 +5785,7 @@
         <v>학원에서 이투스 인강 구독 서비스를 제공해 주셔서 편하게 강의를 들을 수 있었어요.</v>
       </c>
       <c r="K149" t="str">
-        <v>이투스 구독</v>
+        <v/>
       </c>
     </row>
     <row r="150">
@@ -6658,7 +6658,7 @@
         <v>이투스247학원의 스마트 관리는 학습뿐 아니라 생활 전반을 관리해준다는 점에서 매우 유용했어요.</v>
       </c>
       <c r="K173" t="str">
-        <v>학습 관리, 생활 관리</v>
+        <v/>
       </c>
     </row>
     <row r="174" xml:space="preserve">
@@ -7161,7 +7161,7 @@
         <v>학원 생활 중 가장 만족스러웠던 부분은 체계적인 학습 관리 시스템이었어요.</v>
       </c>
       <c r="K187" t="str">
-        <v>학습 관리, 생활 관리</v>
+        <v>학습 관리</v>
       </c>
     </row>
     <row r="188" xml:space="preserve">
@@ -7387,7 +7387,7 @@
         <v>과목별 학습 방향과 모의고사 분석, 전자기기 관리 덕분에 집중해서 공부할 수 있었어요.</v>
       </c>
       <c r="K193" t="str">
-        <v>학습 관리, 모의고사</v>
+        <v>모의고사</v>
       </c>
     </row>
     <row r="194">
@@ -7684,7 +7684,7 @@
         <v>학습에 방해되지 않게 상담 일정을 잡아주시고, 제 수준에 맞는 인강 커리큘럼과 교재를 추천해 주셔서 더 성실하게 공부할 수 있었어요.</v>
       </c>
       <c r="K201" t="str">
-        <v>인강 추천</v>
+        <v/>
       </c>
     </row>
     <row r="202">
@@ -7719,7 +7719,7 @@
         <v>매번 학습일지를 작성하고 주기적인 피드백을 받으며 공부 계획을 잡아 원동력을 잃지 않고 공부할 수 있었어요.</v>
       </c>
       <c r="K202" t="str">
-        <v>학습 계획</v>
+        <v/>
       </c>
     </row>
     <row r="203" xml:space="preserve">
@@ -7760,7 +7760,7 @@
         <v>담임선생님께서 공부 계획부터 방향까지 철저하게 잡아주시고, 즉각적인 피드백으로 올바른 학습 방향을 이어갈 수 있었어요.</v>
       </c>
       <c r="K203" t="str">
-        <v>학습 계획</v>
+        <v/>
       </c>
     </row>
     <row r="204" xml:space="preserve">
@@ -7797,7 +7797,7 @@
         <v>풍부한 입시 정보와 객관적인 조언, 전자기기 관리 덕분에 흔들릴 때마다 다시 방향을 잡을 수 있었어요.</v>
       </c>
       <c r="K204" t="str">
-        <v>입시 관리</v>
+        <v/>
       </c>
     </row>
     <row r="205">
@@ -8042,7 +8042,7 @@
         <v>학습관리 시스템 덕분에 공부 시간을 체계적으로 관리하고, 계획·실행·피드백 과정을 꾸준히 이어갈 수 있었어요.</v>
       </c>
       <c r="K211" t="str">
-        <v>학습 관리, 학습 계획</v>
+        <v>학습 관리</v>
       </c>
     </row>
     <row r="212">
@@ -8253,7 +8253,7 @@
         <v>최적의 학습 환경과 선생님의 세심한 관리로 끝까지 집중하며 긍정적인 변화와 함께 재수 성공을 이뤄내어 뿌듯해요.</v>
       </c>
       <c r="K217" t="str">
-        <v>학습 관리</v>
+        <v/>
       </c>
     </row>
     <row r="218" xml:space="preserve">
@@ -8324,7 +8324,7 @@
         <v>졸음 관리 시스템을 통해 규칙적인 생활 습관을 유지하고, 졸릴 때 적절한 환기나 스트레칭, 관리 지도를 받아 집중력을 빠르게 회복할 수 있었어요.</v>
       </c>
       <c r="K219" t="str">
-        <v>생활 관리, 졸음 관리</v>
+        <v>졸음 관리</v>
       </c>
     </row>
     <row r="220">
@@ -8430,7 +8430,7 @@
         <v>세심한 진도 체크와 관리 덕분에 처음으로 플래너를 꾸준히 지킨 덕분에 매일 성실하게 공부하는 힘이 생겼어요.</v>
       </c>
       <c r="K222" t="str">
-        <v>플래너 관리</v>
+        <v/>
       </c>
     </row>
     <row r="223" xml:space="preserve">
@@ -8651,7 +8651,7 @@
         <v>타이트한 관리로 학습량을 채우고, 나에게 꼭 맞는 강의를 추천해 주신 덕분에 성적을 올릴 수 있었어요.</v>
       </c>
       <c r="K228" t="str">
-        <v>학습 관리</v>
+        <v/>
       </c>
     </row>
     <row r="229">
@@ -8686,7 +8686,7 @@
         <v>철저한 출결 관리로 규칙적인 습관을 기르고, 학습과 휴식의 균형을 잡아 높은 집중력을 유지했어요.</v>
       </c>
       <c r="K229" t="str">
-        <v>학습 관리</v>
+        <v/>
       </c>
     </row>
     <row r="230">
@@ -9015,7 +9015,7 @@
         <v>멘탈 관리와 학습 계획 점검, 생활패턴 관리 덕분에 반수 생활을 끝까지 버티고 좋은 결과를 얻을 수 있었어요.</v>
       </c>
       <c r="K238" t="str">
-        <v>학습 관리, 학습 계획, 생활 관리</v>
+        <v>학습 계획</v>
       </c>
     </row>
     <row r="239">
@@ -9158,7 +9158,7 @@
         <v>플래너와 휴대폰 관리 덕분에 과목 편식 없이 집중했고, 깊이 있는 상담이 큰 도움이 됐어요.</v>
       </c>
       <c r="K242" t="str">
-        <v>플래너 관리</v>
+        <v/>
       </c>
     </row>
     <row r="243">
@@ -9301,7 +9301,7 @@
         <v>주기적 상담과 주간 계획표, 휴대폰 관리 덕분에 학습량이 늘고 공부의 질이 높아졌어요.</v>
       </c>
       <c r="K246" t="str">
-        <v>학습 관리, 학습 계획</v>
+        <v/>
       </c>
     </row>
     <row r="247">
@@ -9511,7 +9511,7 @@
         <v>무너졌던 생활 패턴도 꾸준한 졸음 관리와 세심한 도움 덕분에 바로잡고, 집중하는 시간을 늘릴 수 있었어요.</v>
       </c>
       <c r="K252" t="str">
-        <v>생활 관리, 졸음 관리</v>
+        <v>졸음 관리</v>
       </c>
     </row>
     <row r="253" xml:space="preserve">
@@ -9632,7 +9632,7 @@
         <v>매주 플래너를 바탕으로 학습 점검이 이뤄져서 시간을 어떻게 활용하는지 선생님께서 세밀하게 관리해 주셔서 좋았어요.</v>
       </c>
       <c r="K255" t="str">
-        <v>학습 관리, 플래너 관리</v>
+        <v/>
       </c>
     </row>
     <row r="256">
@@ -9702,7 +9702,7 @@
         <v>졸음지도 및 관리 덕분에 집중력을 유지하여, 순공시간 확보에 큰 도움이 되었어요.</v>
       </c>
       <c r="K257" t="str">
-        <v>졸음 관리</v>
+        <v/>
       </c>
     </row>
     <row r="258">
@@ -9912,7 +9912,7 @@
         <v>학생 개개인의 학습 패턴과 성향을 분석해 맞춤형 관리가 이루어진다는 점이 학원의 가장 큰 장점이라고 생각합니다.</v>
       </c>
       <c r="K263" t="str">
-        <v>학습 관리</v>
+        <v/>
       </c>
     </row>
     <row r="264" xml:space="preserve">
@@ -9950,7 +9950,7 @@
         <v>혼자 공부하면 빠뜨리는 부분이 많았는데 선생님께서 놓치지 않고 챙겨주셔서 계획한 학습량을 채울 수 있었어요!</v>
       </c>
       <c r="K264" t="str">
-        <v>학습 계획</v>
+        <v/>
       </c>
     </row>
     <row r="265">
@@ -10175,7 +10175,7 @@
         <v>개별 학습 데이터와 플래너, 방화벽 관리 덕분에 막막함을 줄이고 수험생활을 잘 마무리했어요.</v>
       </c>
       <c r="K269" t="str">
-        <v>학습 관리, 플래너 관리, 생활 관리, 방화벽</v>
+        <v>방화벽</v>
       </c>
     </row>
     <row r="270">
@@ -10316,7 +10316,7 @@
         <v>출결 관리와 시간 관리가 철저해 자연스럽게 공부에 집중할 수 있었고, 전반적인 생활 습관을 바로잡는 데 도움이 되었어요.</v>
       </c>
       <c r="K273" t="str">
-        <v>생활 관리</v>
+        <v/>
       </c>
     </row>
     <row r="274">
@@ -10606,7 +10606,7 @@
         <v>학원 밖에서의 생활 습관까지 확인해 주시면서 수면 관리를 도와주신 덕분에 학원에서 졸지 않고 공부할 수 있었어요.</v>
       </c>
       <c r="K281" t="str">
-        <v>생활 관리</v>
+        <v/>
       </c>
     </row>
     <row r="282">
@@ -10956,7 +10956,7 @@
         <v>노베이스라 인강과 교재 선택부터 막막했지만, 선생님께서 저에게 맞는 콘텐츠를 추천해 주신 덕분에 성적을 올릴 수 있었어요.</v>
       </c>
       <c r="K291" t="str">
-        <v>인강 추천</v>
+        <v/>
       </c>
     </row>
     <row r="292">
@@ -11131,7 +11131,7 @@
         <v>정기적으로 학습 상태를 점검하고, 앞으로의 계획을 선생님과 이야기 하면서 공부에 더 전념할 수 있었습니다.</v>
       </c>
       <c r="K296" t="str">
-        <v>학습 계획</v>
+        <v/>
       </c>
     </row>
     <row r="297">
@@ -11201,7 +11201,7 @@
         <v>단순히 인강을 추천해주는 것만 아니라 구체적인 학습 로드맵을 만들어 어떻게 공부하면 될지 가이드를 주셔서 도움이 많이 됐어요.</v>
       </c>
       <c r="K298" t="str">
-        <v>인강 추천</v>
+        <v/>
       </c>
     </row>
     <row r="299" xml:space="preserve">
@@ -11347,7 +11347,7 @@
         <v>하루 일정을 체계적으로 관리해 주셔서 자연스럽게 규칙적인 생활 습관을 만들 수 있어 좋았습니다.</v>
       </c>
       <c r="K302" t="str">
-        <v>생활 관리</v>
+        <v/>
       </c>
     </row>
     <row r="303">
@@ -11740,7 +11740,7 @@
         <v>재수 생활 동안 학습 계획과 생활 관리를 꾸준히 받아 끝까지 흔들리지 않고 공부할 수 있었어요.</v>
       </c>
       <c r="K313" t="str">
-        <v>학습 관리, 학습 계획, 생활 관리</v>
+        <v>학습 계획, 생활 관리</v>
       </c>
     </row>
     <row r="314">
@@ -12057,7 +12057,7 @@
         <v>플래너에서 부족한 부분을 찾아 보충하도록 도움을 주시고, 자세한 교재와 인강도 함께 추천해주셔서 도움을 많이 받았어요.</v>
       </c>
       <c r="K322" t="str">
-        <v>인강 추천</v>
+        <v/>
       </c>
     </row>
     <row r="323">
@@ -12768,7 +12768,7 @@
         <v>면학 분위기 감독과 졸음 관리는 학습 집중도를 유지하는 데 큰 도움이 되었어요.</v>
       </c>
       <c r="K342" t="str">
-        <v>학습 관리, 면학 분위기, 졸음 관리</v>
+        <v>면학 분위기, 졸음 관리</v>
       </c>
     </row>
     <row r="343">
@@ -12844,7 +12844,7 @@
         <v>수능과 동일한 시간표에 맞춰 생활 패턴을 관리할 수 있어 불필요한 시간 낭비 없이 학습에 집중할 수 있었어요.</v>
       </c>
       <c r="K344" t="str">
-        <v>학습 관리, 생활 관리</v>
+        <v/>
       </c>
     </row>
     <row r="345" xml:space="preserve">
@@ -13103,7 +13103,7 @@
         <v>꼼꼼한 출결 관리 덕분에 스스로 긴장감을 가지며 규칙적인 생활을 할 수 있었어요.</v>
       </c>
       <c r="K351" t="str">
-        <v>생활 관리</v>
+        <v/>
       </c>
     </row>
     <row r="352" xml:space="preserve">
@@ -13256,7 +13256,7 @@
         <v>학원에서 제공하는 학습계획 플래너 관리를 받으면서 공부의 질이 완전히 달라졌었어요.</v>
       </c>
       <c r="K355" t="str">
-        <v>학습 관리, 학습 계획, 플래너 관리</v>
+        <v>학습 계획, 플래너 관리</v>
       </c>
     </row>
     <row r="356">
@@ -13291,7 +13291,7 @@
         <v>수많은 인강 중에서 저에게 맞는 선생님과 난이도를 추천해 주셨는데 잘 맞아서 신기했어요!</v>
       </c>
       <c r="K356" t="str">
-        <v>인강 추천</v>
+        <v/>
       </c>
     </row>
     <row r="357">
@@ -13466,7 +13466,7 @@
         <v>이투스247학원의 학습계획이랑 플래너 관리도 도움이 많이 됐어요.</v>
       </c>
       <c r="K361" t="str">
-        <v>학습 관리, 학습 계획, 플래너 관리</v>
+        <v>학습 계획, 플래너 관리</v>
       </c>
     </row>
     <row r="362" xml:space="preserve">
@@ -13534,7 +13534,7 @@
         <v>분위기를 잡아주는 생활 관리, 학업을 책임지는 교과 지도, 그리고 최종 합격을 설계하는 입시 전략까지 다 만족했어요.</v>
       </c>
       <c r="K362" t="str">
-        <v>입시 관리, 생활 관리</v>
+        <v>생활 관리</v>
       </c>
     </row>
     <row r="363" xml:space="preserve">
@@ -13608,7 +13608,7 @@
         <v>학습 전 계획표를 작성하고, 그에 맞게 생활하며 규칙적인 생활 습관을 만들 수 있었어요!</v>
       </c>
       <c r="K364" t="str">
-        <v>학습 계획</v>
+        <v/>
       </c>
     </row>
     <row r="365">
@@ -13749,7 +13749,7 @@
         <v>면학 분위기 감독 및 졸음 관리로 학습에 집중할 수 있는 환경이 잘 조성되어 있었어요.</v>
       </c>
       <c r="K368" t="str">
-        <v>학습 관리, 면학 분위기, 졸음 관리</v>
+        <v>면학 분위기, 졸음 관리</v>
       </c>
     </row>
     <row r="369">

</xml_diff>

<commit_message>
Fix additional spacing typos
</commit_message>
<xml_diff>
--- a/reviews_with_keywords.xlsx
+++ b/reviews_with_keywords.xlsx
@@ -746,7 +746,7 @@
         <v>요즘같이 수 많은 컨텐츠가 쏟아지는 시기에 나한테 맞는 커리큘럼은 무엇인지, 등등 정확하게 현재 내게 필요한 공부만 할 수 있었습니다. 또한 성적이 나오지 않아 전전긍긍할 때에도 객관적으로 나를 평가해 올바른 방법으로 공부할 수 있도록 꾸준히 이끌어주었습니다.</v>
       </c>
       <c r="F10" t="str">
-        <v>저는 인강을 많이 듣지 않고 스스로 공부하는 것을 좋아하였는데 이때 자칫 공부량이 너무 적어질 수 있는 문제가 있었습니다. 그러나 이러한 부분들을 관리해주시고 정말 나에게 맞는 공부를 추천해주셔서 잘 할 수 있었습니다.</v>
+        <v>저는 인강을 많이 듣지 않고 스스로 공부하는 것을 좋아하였는데 이때 자칫 공부량이 너무 적어질 수 있는 문제가 있었습니다. 그러나 이러한 부분들을 관리해주시고 정말 나에게 맞는 공부를 추천해 주셔서 잘 할 수 있었습니다.</v>
       </c>
       <c r="G10" t="str">
         <v>저는 집중력이 좋지 않아 스터디카페에서는 한 문제 풀고 핸드폰 보고 하는 등의 문제가 있었는데 이러한 부분들을 핸드폰 제출로 해결할 수 있었습니다. 또한 SNS를 잘 보지 않게 돼 남들과 저를 비교하지 못하는 것도 좋았습니다.</v>
@@ -1094,7 +1094,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E20" t="str">
-        <v>학습 계획이나 모의고사 계획을 어떻기 세워야할지 막막했는데 담당 선생님께서 이에 대해 코칭해주시고 같이 내 일정에 맞게 계획을 세워주셔서 도움이 많이 되었다. 내가 들으면 좋을 만한 인강도 추천해주셔서 실제로도 영어 성적이 많이 올랐다. 항상 무계획으로 공부했던 시절과 다르게 학습 습관이 잡혀서 계획적으로 공부를 해나갈 수 있었다.</v>
+        <v>학습 계획이나 모의고사 계획을 어떻기 세워야할지 막막했는데 담당 선생님께서 이에 대해 코칭해주시고 같이 내 일정에 맞게 계획을 세워주셔서 도움이 많이 되었다. 내가 들으면 좋을 만한 인강도 추천해 주셔서 실제로도 영어 성적이 많이 올랐다. 항상 무계획으로 공부했던 시절과 다르게 학습 습관이 잡혀서 계획적으로 공부를 해나갈 수 있었다.</v>
       </c>
       <c r="F20" t="str">
         <v>솔직히 학교 선생님 제외 모르는 문제를 물어볼 사람이 마땅히 없었는데 학원 선생님께 물어보니 친절히 답변해주셔서 좋았다. 다들 학력이 높으셔서 그런지 설명도 잘 하시고 수학같은 경우엔 효율적인 문제 풀이 방법을 알려주셔서 이 점도 많은 도움이 됐었다.</v>
@@ -1187,7 +1187,7 @@
         <v>예전에는 시간에만 쫓기다가 제대로된 학습을 못했는데 이투스247에 다니면서 어떻게 공부해야 효율적으로 학습할 수 있는지 배울 수 있었습니다. 6모 전까지 어디까지 끝내야 하는지, 9모 전까지 어디까지 끝내야 하는지, N제는 어떤 교재가 좋은지 등 자세한 코칭 시스템 덕분에 계획적으로 공부할 수 있었습니다.</v>
       </c>
       <c r="F22" t="str">
-        <v>무조건 유명한 강사 뿐만이 아니라 학생 개인에게 맞는 인강과 강사를 추천해주시고 성적에 따라 단계적으로 수준에 맞는 강의를 추천해주셔서 유용했습니다. 기출이나 N제 또한 진도와 성적에 맞는 교재로 추천해주셔서 성적 향상에 더 큰 도움을 받을 수 있었습니다.</v>
+        <v>무조건 유명한 강사 뿐만이 아니라 학생 개인에게 맞는 인강과 강사를 추천해주시고 성적에 따라 단계적으로 수준에 맞는 강의를 추천해 주셔서 유용했습니다. 기출이나 N제 또한 진도와 성적에 맞는 교재로 추천해 주셔서 성적 향상에 더 큰 도움을 받을 수 있었습니다.</v>
       </c>
       <c r="G22" t="str">
         <v>면학 분위기가 굉장히 좋았습니다. 자습실도 책상마다 칸막이가 설치되어있어서 더 공부에 몰입할 수 있었고 강의실 또한 쾌적했습니다. 가끔 피곤해서 졸리기도 했지만 감독 선생님들께서 친절하게 깨워주셔서 다시 정신을 차릴 수 있었습니다.</v>
@@ -1199,7 +1199,7 @@
         <v>이투스 247 부산서면점에 다니면서 좋은 공부 습관을 기를 수 있었습니다. 졸업하고 나서도 이투스 247에서 배운 학습법을 바탕으로 대학에 가서도 유용하게 쓸 수 있을 것 같습니다.</v>
       </c>
       <c r="J22" t="str">
-        <v>기출이나 N제 또한 진도와 성적에 맞는 교재로 추천해주셔서 성적 향상에 더 큰 도움을 받을 수 있었어요.</v>
+        <v>기출이나 N제 또한 진도와 성적에 맞는 교재로 추천해 주셔서 성적 향상에 더 큰 도움을 받을 수 있었어요.</v>
       </c>
       <c r="K22" t="str">
         <v/>
@@ -1331,7 +1331,7 @@
         <v>자기주도적인학습이 잘 되지 않는 사람들은 보통 어디서부터 시작해야할지 막막한데 이투스는 한 주마다 상담을하며  어떤 커리큘럼을 탈지, 어떤 부분이 부족한지에 대해 심도있게 대화하며 계획을 같이 짜게되니 아무런 계획이 없이 그냥 들어오기만 하면 이끌어주니까 공부에 집중할 수 있는 환경이 만들어집니다</v>
       </c>
       <c r="F26" t="str">
-        <v>평소 현역시절 학원만 다녀 인강이나 교재에 대해 정보가 전무했는데 이투스 조교 선생님께서 과목별로 나의 수준에 맞는 교재와 문이과를 가리지 않고 다양한 인강 강사를 추천해주셔서 평소 인강계에 대해 관심이 없었던 사람들까지 이 학원에 온다면 자기의 학습패턴에 맞는 커리큘럼을 탈 수 있습니다</v>
+        <v>평소 현역시절 학원만 다녀 인강이나 교재에 대해 정보가 전무했는데 이투스 조교 선생님께서 과목별로 나의 수준에 맞는 교재와 문이과를 가리지 않고 다양한 인강 강사를 추천해 주셔서 평소 인강계에 대해 관심이 없었던 사람들까지 이 학원에 온다면 자기의 학습패턴에 맞는 커리큘럼을 탈 수 있습니다</v>
       </c>
       <c r="G26" t="str">
         <v>오며가며 출석과 외부 일정 관리를 하는데에 있어 수기로 체크하거나 하면 번거로운데 전자출결로 스케줄을 체크하니 잠깐이라도 낭비되는 시간을 줄일 수 있어 좋았습니다. 또한 시간을 넘기는 것에 대해 엄격해서 수능이나 모의고사와 같이 중요한 일정에 늦지 않는 습관을 길러주어 좋았습니다.</v>
@@ -1436,7 +1436,7 @@
         <v>반수생</v>
       </c>
       <c r="E29" t="str">
-        <v>성적이 낮은 과목이 있었는데 저에게 알맞은  강의를 추천해주셔서 많이 도움이 되었습니다 모의고사 성적표가 나올때마다 어떤 과목 중심으로 공부해야 효율적일지 같이 고민하고 상담해주셔서 좋았습니다</v>
+        <v>성적이 낮은 과목이 있었는데 저에게 알맞은  강의를 추천해 주셔서 많이 도움이 되었습니다 모의고사 성적표가 나올때마다 어떤 과목 중심으로 공부해야 효율적일지 같이 고민하고 상담해주셔서 좋았습니다</v>
       </c>
       <c r="F29" t="str">
         <v>매일 플래너를 쓰니까 계획적으로 학습을 할수 있어서 좋았습니다.  플래너를 쓰지 않았을때보다 더 체계적이고 효율적으로 공부할수 있었습니다. 매일 플래너를 쓰다보니 습관이 되어서 공부 계획을 잘 세우게되었습니다</v>
@@ -2875,7 +2875,7 @@
         <v>입시에 대해서 많이 무지한 편이었는데 도움을 많이 주셔서 입시 시스템이 어떻게 돌아가는지 정확하게 파악하는 걸 수월하게 할 수 있었고, 심리적으로도 대학 입시와 수능 공부 방향을 어떻게 해야할 지도 알려주셔서 많이 도움되었던 것 같았습니다.</v>
       </c>
       <c r="F69" t="str">
-        <v>자기가 무슨 인강을 들어야할 지 처음엔 감이 안잡힐 때가 많은데 제 성적과 학습 수준에 따라서 어떤 교재와 인강을 들어야할 지 추천해주셔서 좋았습니다. 방향을 잡는데 많이 도움되었다고 생각해요</v>
+        <v>자기가 무슨 인강을 들어야할 지 처음엔 감이 안잡힐 때가 많은데 제 성적과 학습 수준에 따라서 어떤 교재와 인강을 들어야할 지 추천해 주셔서 좋았습니다. 방향을 잡는데 많이 도움되었다고 생각해요</v>
       </c>
       <c r="G69" t="str">
         <v>핸드폰이 진짜 수능 준비에 가장 방해가 많이 되는 물품이라고 생각하는데, 이렇게 확실하게 강제성을 주니까 공부에만 집중하게 될 수 있는 환경이 만들어져서 정말 좋았습니다. 졸음도 가끔 들어오셔서 돌아다니시면서 깨워주시는데 그것 덕에 졸음도 깨고 공부 집중에 도움이 되었습니다.</v>
@@ -3387,7 +3387,7 @@
       </c>
       <c r="E83" t="str" xml:space="preserve">
         <v xml:space="preserve">매주 무엇을 더 공부하며 채워나가야할지나 지금 현재 부족한 점과 그것을 보완할 방법에 대해 알려주시고_x000d_
-한 선생님의 커리만 따르는 것이 아닌 내가 진짜 필요한 강좌나 교재를 추천해주셔서 내가 필요한 부분을 채우며 실력을 쌓아나갈 수 있었다</v>
+한 선생님의 커리만 따르는 것이 아닌 내가 진짜 필요한 강좌나 교재를 추천해 주셔서 내가 필요한 부분을 채우며 실력을 쌓아나갈 수 있었다</v>
       </c>
       <c r="F83" t="str">
         <v>인강과 교재를 체계적으로 추천해 주시고, 수강 관리뿐만 아니라 학습 스케줄까지 함께 관리해 주셔서 매일 해야 할 공부를 적절한 분량으로 꾸준히 해낼 수 있었다. 그 덕분에 학습 리듬이 안정적으로 유지되었고 계획적으로 공부하는 습관도 자연스럽게 형성될 수 있었다</v>
@@ -4822,7 +4822,7 @@
         <v>N수생</v>
       </c>
       <c r="E123" t="str" xml:space="preserve">
-        <v xml:space="preserve">6월 모의고사 성적과 9월 모의고사 성적을 바탕으로 선생님께서 수시원서상담을 친절하게 진행해주셔서 도움이 많이 됐어 제 성적대에 맞는 대학을 추천해주셔서 감사했습니다 과도한 상향원서 작성이_x000d_
+        <v xml:space="preserve">6월 모의고사 성적과 9월 모의고사 성적을 바탕으로 선생님께서 수시원서상담을 친절하게 진행해주셔서 도움이 많이 됐어 제 성적대에 맞는 대학을 추천해 주셔서 감사했습니다 과도한 상향원서 작성이_x000d_
 아닌 현실적으로 가능한 원서를 작성하게끔 해주셔서 안정적으로 입시를 마무리했습니다</v>
       </c>
       <c r="F123" t="str" xml:space="preserve">
@@ -5581,7 +5581,7 @@
         <v>고2때까지 내신 위주로 하다보니까 수능 공부는 제게 너무 생소했습니다. 하지만 겨울방학때 기본적인 틀을 잡아주는데 담임 선생님께서 도와주셨습니다. 특히 탐구 같은 경우 내신과 괴리감이 워낙 커서 이 부분을 좀 집중적으로 케어해주셨습니다. 또한 여름 방학때 본격적으로 수능 공부에 몰입할때 날씨랑 수시 원서 쓰는 시기가 다가왔기에 집중이 안되었지만 이부분을 제대로 잡아주셔서 25년도 하반기때 열심히 공부할수 있었습니다.</v>
       </c>
       <c r="F144" t="str">
-        <v>처음 수능 공부를 할때 인강이 생소하여 내신에서 활용했던 마플 자습서등을 이용할려고 했습니다. 하지만 담임 선생님께서 저에게 여러 인강을 추천해주셔서 여러모로 다양한 도움이 되었습니다. 특히 수학 같은 경우 제 성적에 맞는 실전개념서등을 추천해주셨고 이로 인해 제 9월 모의고사 성적은 6모보다 훨씬 높았습니다. 이외에 국어 인강도 추천해주셔서 비문학 습관은 잡을수 있어서 유용했습니다.</v>
+        <v>처음 수능 공부를 할때 인강이 생소하여 내신에서 활용했던 마플 자습서등을 이용할려고 했습니다. 하지만 담임 선생님께서 저에게 여러 인강을 추천해 주셔서 여러모로 다양한 도움이 되었습니다. 특히 수학 같은 경우 제 성적에 맞는 실전개념서등을 추천해주셨고 이로 인해 제 9월 모의고사 성적은 6모보다 훨씬 높았습니다. 이외에 국어 인강도 추천해 주셔서 비문학 습관은 잡을수 있어서 유용했습니다.</v>
       </c>
       <c r="G144" t="str">
         <v>저는 폰 사용을 한번 하면 2시간은 금방 지나기 때문에 내신때 이로 인해 많은 손해를 보았습니다. 하지만 고3 겨울방학때 부터 이투스 247을 다니면서 폰을 거두어서 확실히 공부 하는 시간이 늘었습니다</v>
@@ -7520,7 +7520,7 @@
         <v xml:space="preserve">주마다 불러내시어, 과목별로 지금 어떤 공부들을 하고 있는지 점검을 해주셔서 _x000d_
 일단 플래너와 주 학습 계획을 더 잘 세울 수 있게 되었습니다. _x000d_
 그리고 같이 어떤 공부를 어떻게 했는지 대화하다보면, 어떤 과목이 시간이 부족했으며 능률이 오르지 않았고, _x000d_
-실모 같은 경우도 어떤 유형들이 안되는지 잘 체크를 해주셔서 저의 문제점을 찾기 좋았던 것 같습니다. 또한 과목별로 제 스타일에 맞는 선생님들을 추천해주셔서 도움을 많이 받았습니다 !</v>
+실모 같은 경우도 어떤 유형들이 안되는지 잘 체크를 해주셔서 저의 문제점을 찾기 좋았던 것 같습니다. 또한 과목별로 제 스타일에 맞는 선생님들을 추천해 주셔서 도움을 많이 받았습니다 !</v>
       </c>
       <c r="G197" t="str" xml:space="preserve">
         <v xml:space="preserve">정신차리고 항상 자지 않으려고 노력은 하지만, 어쩔 수 없이 잠이 올 때 _x000d_
@@ -8306,10 +8306,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E219" t="str">
-        <v>현재 내 학습 수준과 남은 시간과 시기 등의 상황을 고려하여 적절한 강의와 커리큘럼을 추천해주셔서 학습 방향을 보다 명확하게 설정하여 불필요한 시간 낭비 없이 효율적으로 공부할 수 있게 되었고 또한 학습 상담 과정에서 세심하게 제 고민과 부족한 부분을 파악해주시고 현실적인 조언과 구체적인 학습 방법까지 제시해주셔서 신뢰가 갔으며 동기부여에도 큰 도움이 되었습니다.</v>
+        <v>현재 내 학습 수준과 남은 시간과 시기 등의 상황을 고려하여 적절한 강의와 커리큘럼을 추천해 주셔서 학습 방향을 보다 명확하게 설정하여 불필요한 시간 낭비 없이 효율적으로 공부할 수 있게 되었고 또한 학습 상담 과정에서 세심하게 제 고민과 부족한 부분을 파악해주시고 현실적인 조언과 구체적인 학습 방법까지 제시해주셔서 신뢰가 갔으며 동기부여에도 큰 도움이 되었습니다.</v>
       </c>
       <c r="F219" t="str">
-        <v>현재 내 학습 수준과 남은 시간 등을 고려하여 교재와 인강을 체계적으로 추천해주셔서 무엇부터 어떻게 공부해야 할지 명확하게 알 수 있어 매우 유용했습니다. 특히 개인에게 맞는 강의와 교재를 연결해주어 학습 효율이 높아졌고 시행착오를 줄일 수 있었습니다.</v>
+        <v>현재 내 학습 수준과 남은 시간 등을 고려하여 교재와 인강을 체계적으로 추천해 주셔서 무엇부터 어떻게 공부해야 할지 명확하게 알 수 있어 매우 유용했습니다. 특히 개인에게 맞는 강의와 교재를 연결해주어 학습 효율이 높아졌고 시행착오를 줄일 수 있었습니다.</v>
       </c>
       <c r="G219" t="str">
         <v>체계적으로 조성된 면학 분위기 덕분에 집중할 수 있는 환경이 만들어져 학습 효율이 크게 향상되었습니다. 또한 졸음 관리 및 감독 시스템을 통해 공부 중 흐트러질 수 있는 부분을 바로잡아 주셔서 꾸준한 집중력을 유지하는 데 도움이 되었고 학습 습관 형성에도 긍정적인 영향을 주었습니다.</v>
@@ -8883,8 +8883,8 @@
 단순히 질문을 받아주는 수준을 넘어서, 학습의 방향성과 문제 해결 능력을 함께 키워준다는 점에서 이투스 독재의 학습 코칭은 큰 장점이라고 생각합니다. 혼자서는 채우기 어려운 부분을 확실하게 보완해준 덕분에 끝까지 흔들리지 않고 공부를 이어갈 수 있었습니다. 실제로 많은 성적 향상을 이루었고 제가 만족할 수 있는 대학교에 오게 되었습니다.</v>
       </c>
       <c r="F235" t="str" xml:space="preserve">
-        <v xml:space="preserve">이투스 독학재수학원을 다니면서 좋았던 점 중 하나는 인강이나 교재 추천 시스템이 정말 체계적이었다는 점입니다. 저는 검정고시를 보고 수능을 준비한 케이스라서, 어떤 교재를 써야 하는지, 어떤 인강을 들어야 하는지에 대한 기준이 거의 없는 상태였습니다. 혼자였다면 수준에 맞지 않는 교재를 선택하거나, 방향 없이 이것저것 건드리다가 시간만 낭비했을 가능성이 컸다고 생각합니다. 그런데 학습 코칭을 통해 현재 제 실력에 맞는 교재와 인강을 추천해주셔서 공부 방향을 잡는 데 큰 도움이 되었습니다. 특히 단순히 유명한 교재를 추천하는 것이 아니라, 제 수준에 맞는 단계별 교재를 골라주셨던 점이 인상적이었습니다. 실제로 학습에서는 자신의 수준에 맞는 교재 선택이 굉장히 중요한데, 난이도가 맞지 않으면 학습 효율이 떨어질 수 있다는 점에서도 이런 추천이 큰 도움이 되었습니다. _x000d_
-또한 교재와 인강이 서로 연계되도록 추천해주셔서, 개념 이해 → 문제 적용 → 복습까지 자연스럽게 이어지는 학습 흐름을 만들 수 있었습니다. 덕분에 막연하게 공부하는 느낌이 아니라, 체계적으로 실력이 쌓여가는 느낌을 받을 수 있었습니다._x000d_
+        <v xml:space="preserve">이투스 독학재수학원을 다니면서 좋았던 점 중 하나는 인강이나 교재 추천 시스템이 정말 체계적이었다는 점입니다. 저는 검정고시를 보고 수능을 준비한 케이스라서, 어떤 교재를 써야 하는지, 어떤 인강을 들어야 하는지에 대한 기준이 거의 없는 상태였습니다. 혼자였다면 수준에 맞지 않는 교재를 선택하거나, 방향 없이 이것저것 건드리다가 시간만 낭비했을 가능성이 컸다고 생각합니다. 그런데 학습 코칭을 통해 현재 제 실력에 맞는 교재와 인강을 추천해 주셔서 공부 방향을 잡는 데 큰 도움이 되었습니다. 특히 단순히 유명한 교재를 추천하는 것이 아니라, 제 수준에 맞는 단계별 교재를 골라주셨던 점이 인상적이었습니다. 실제로 학습에서는 자신의 수준에 맞는 교재 선택이 굉장히 중요한데, 난이도가 맞지 않으면 학습 효율이 떨어질 수 있다는 점에서도 이런 추천이 큰 도움이 되었습니다. _x000d_
+또한 교재와 인강이 서로 연계되도록 추천해 주셔서, 개념 이해 → 문제 적용 → 복습까지 자연스럽게 이어지는 학습 흐름을 만들 수 있었습니다. 덕분에 막연하게 공부하는 느낌이 아니라, 체계적으로 실력이 쌓여가는 느낌을 받을 수 있었습니다._x000d_
 특히 저처럼 기초가 부족한 상태에서 시작한 경우에는 무엇을 먼저 해야 할지 몰라서 방황하기 쉬운데, 이런 부분을 잡아주고 학습 로드맵을 제시해준 점이 가장 큰 장점이라고 느꼈습니다. 혼자 했다면 절대 만들기 어려웠을 공부 방향을 잡아줬다는 점에서 매우 만족스러웠습니다.</v>
       </c>
       <c r="G235" t="str" xml:space="preserve">
@@ -10371,7 +10371,7 @@
         <v>전반적인 성적, 부족한 과목과 파트를 자세히 파악해주시고 이를 토대로 구체적인 학습 방향을 제시해주셔서 학습계획 수립에 큰 도움이 되었습니다. 특히 저는 수학과 탐구 과목이 부족하였는데, 제시해주신 학습 방향대로 공부하니 성적향상을 거둘 수 있었습니다.</v>
       </c>
       <c r="F275" t="str">
-        <v>수많은 콘텐츠가 넘쳐나는 현재 대학 입시 상황에서 무슨 교재와 강의를 선택해야 저의 현재 성적대에 도움이 될지 잘 모르겠어서 힘들었었는데 분석하신 제 성적을 바탕으로 각 과목의 교재와 강의를 꼼꼼히 추천해주셔서 크게 도움이 되었습니다.</v>
+        <v>수많은 콘텐츠가 넘쳐나는 현재 대학 입시 상황에서 무슨 교재와 강의를 선택해야 저의 현재 성적대에 도움이 될지 잘 모르겠어서 힘들었었는데 분석하신 제 성적을 바탕으로 각 과목의 교재와 강의를 꼼꼼히 추천해 주셔서 크게 도움이 되었습니다.</v>
       </c>
       <c r="G275" t="str">
         <v>아무래도 수험생활의 가장 큰 적은 인터넷으로 즐길 수 있는 오락거리와 미디어라고 생각합니다. 하지만 이투스 247에서는 와이파이 방화벽을 통해 애초에 접속 가능성을 막고 학습사이트만 들어갈 수 있게 설계되어있어 스스로 자제력이 부족해 인터넷 사용시간이 많았던 저에게 도움이 되었습니다.</v>
@@ -10406,7 +10406,7 @@
         <v>선생님이 과목별로 있어서 학습 방법과 출제경향을 잘 아셔서 좋았습니다. 어려운 유형도 질문하면 잘 알려주시고, 부족한 부분을 채우는 방법도 알려주셔서 좋았습니다. 이투스 선생님이 과목별로 상주하는 시간마다 질문할 수 있어서 하루에 여러 번, 다른 과목 질문이 수월했습니다.</v>
       </c>
       <c r="F276" t="str">
-        <v>학원 스케쥴과 이투스 학원을 병행하여 스케쥴 관리에 어려움이 있었습니다. 하지만 이투스 등원을 처음 했을 때, 적절하게 스케쥴 관리표를 짜주시고 인강과 학원을 적절히 병행하도록 추천해주셔서, 균형잡힌 공부를 할 수 있었습니다.</v>
+        <v>학원 스케쥴과 이투스 학원을 병행하여 스케쥴 관리에 어려움이 있었습니다. 하지만 이투스 등원을 처음 했을 때, 적절하게 스케쥴 관리표를 짜주시고 인강과 학원을 적절히 병행하도록 추천해 주셔서, 균형잡힌 공부를 할 수 있었습니다.</v>
       </c>
       <c r="G276" t="str">
         <v>핸드폰을 가지고 있으면 확실히 집중이 분산되고 중간에 딴짓을 할 가능성이 높아지는데, 기본적으로 항상 스마트폰을 수거하여 공부가 지치더라도 스마트폰을 붙들지 않을 수 있어서 좋았습니다</v>
@@ -10696,7 +10696,7 @@
         <v>재수 중 초반 갈피가 안 잡혔을 때나 흐트러질 때쯤 혼자서 관리하기 어려운(핸드폰) 부분들을 관리해주시고 상담할 때 이제 거의 다 끝났다, 열심히 하라는 등의 격려 말을 해주셔서 멘탈 관리에 도움이 되었습니다.</v>
       </c>
       <c r="F284" t="str">
-        <v>잘 모르는 커리큘럼을 잘 설명해주시고 제가 어떤 시기에 어떤 커리큘럼을 들어야하는지 자세히 조언해주시고 추천해주셔서 좋았습니다. 제가 고민할 때 방향을 확실하게  잡아주셔서 유익했습니다.</v>
+        <v>잘 모르는 커리큘럼을 잘 설명해주시고 제가 어떤 시기에 어떤 커리큘럼을 들어야하는지 자세히 조언해주시고 추천해 주셔서 좋았습니다. 제가 고민할 때 방향을 확실하게  잡아주셔서 유익했습니다.</v>
       </c>
       <c r="G284" t="str">
         <v>제가 아침에 정말 많이 자고 사실 계속 잘 때 깨우실 때는 속으로 너무 짜증났는데 계속 깨워주시고 상담 때 일침도 날려주신 후에 정말 거짓말처럼 쭈욱 안 자서 너무 좋았습니다. 열정적으로 깨워주셔서 감사했습니다!</v>
@@ -11198,7 +11198,7 @@
         <v>선생님들 잘 지내고 계시나요? 목표를 이루고 싶은데, 혼자 불안정하게 있었을 수도 있던 제게 길잡이가 되어주셔서 감사합니다. 한 해 동안 공부, 생활 관리를 넘어서 정말 많은 부분에서 도움을 받은 것 같아서 애틋한 마음이 드네요. 지금은 대학생이 되어 캠퍼스를 돌아다니는데, 그때의 제가 본다면 좋아할 것 같아요. 선생님들 덕분에 제가 끝까지 놓지 않고 헤쳐나갈 수 있던 것 같아요. 공부 이외에도 제게 많은 것들을 가르쳐주셔서 정말 감사합니다.</v>
       </c>
       <c r="J298" t="str">
-        <v>단순히 인강을 추천해주는 것만 아니라 구체적인 학습 로드맵을 만들어 어떻게 공부하면 될지 가이드를 주셔서 도움이 많이 됐어요.</v>
+        <v>단순히 인강을 추천해 주는 것만 아니라 구체적인 학습 로드맵을 만들어 어떻게 공부하면 될지 가이드를 주셔서 도움이 많이 됐어요.</v>
       </c>
       <c r="K298" t="str">
         <v/>
@@ -12042,7 +12042,7 @@
         <v>과목별로 학습 진행 상황에 대해 자세히 파악하고, 어떤 방향으로 나아가야할지 구체적으로 조언해주셨다. 또한 과목별로 구체적인 공부 방법도 알려주셔서 좋았다. 매주 플래너 검사도 꼼꼼히 해주시고 부족한 과목을 찾아내어 채울 수 있도록 도움을 주셔서 유용했다.</v>
       </c>
       <c r="F322" t="str">
-        <v>플래너를 검사하고 학습 진행 상황을 파악하여 단계에 맞는 학습 방법을 알려주셔서 유용하였다. 또한 플래너에서 부족한 부분을 찾아 보충하도록 도움을 주시고, 자세한 교재와 인강도 함께 추천해주셔서 도움을 많이 받았다.</v>
+        <v>플래너를 검사하고 학습 진행 상황을 파악하여 단계에 맞는 학습 방법을 알려주셔서 유용하였다. 또한 플래너에서 부족한 부분을 찾아 보충하도록 도움을 주시고, 자세한 교재와 인강도 함께 추천해 주셔서 도움을 많이 받았다.</v>
       </c>
       <c r="G322" t="str">
         <v>자제력이 부족하여 태블릿이 눈 앞에 있으면 딴 짓을 많이 하였는데 와이파이 방회벽이 막아주어 불필요한 행동을 하지 않아 공부에 더욱 집중할 수 있었다. 또한, 노래도 못듣게 통제해주어서 노래 들으면서 공부하는 습관을 고치게 되었고 더욱 집중할 수 있는 상태로 만들어주어 유용하였습니다.</v>
@@ -12054,7 +12054,7 @@
         <v>공부뿐만 아니라 생활이나 친구 관계에도 항상 신경 써주셔서 감사했습니다!! 덕분에 사소한 것에 흔들리지 않고 끝까지 열심히 공부할 수 있었습니다. 수업하시는 선생님들도 항상 열정적으로 수업해주시고 상담도 꼼꼼히 해주셔서 정말 도움이 많이 되었습니다. 다시 한번 감사드립니다!</v>
       </c>
       <c r="J322" t="str">
-        <v>플래너에서 부족한 부분을 찾아 보충하도록 도움을 주시고, 자세한 교재와 인강도 함께 추천해주셔서 도움을 많이 받았어요.</v>
+        <v>플래너에서 부족한 부분을 찾아 보충하도록 도움을 주시고, 자세한 교재와 인강도 함께 추천해 주셔서 도움을 많이 받았어요.</v>
       </c>
       <c r="K322" t="str">
         <v/>

</xml_diff>

<commit_message>
Fix additional wording and spacing typos
</commit_message>
<xml_diff>
--- a/reviews_with_keywords.xlsx
+++ b/reviews_with_keywords.xlsx
@@ -778,7 +778,7 @@
         <v>N수생</v>
       </c>
       <c r="E11" t="str">
-        <v>문제집을 풀면서 모르는 문제가 있을때 매번 답지만 보며 시간을 많이 썼는데 학습 상담을 통해서 시간을 효율적으로 쓸  수 있었고 이해하는데도 도움이 많이 되었습니다. 그리고 공부 커리큘럼을 어떻게 짜야할지 몰랐는데 학습상담을 통해서 어떻게 공부해야할지 감을 잡고 공부할 수 있었습니다.</v>
+        <v>문제집을 풀면서 모르는 문제가 있을때 매번 답지만 보며 시간을 많이 썼는데 학습 상담을 통해서 시간을 효율적으로 쓸  수 있었고 이해하는데도 도움이 많이 되었습니다. 그리고 공부 커리큘럼을 어떻게 짜야할지 몰랐는데 학습 상담을 통해서 어떻게 공부해야할지 감을 잡고 공부할 수 있었습니다.</v>
       </c>
       <c r="F11" t="str">
         <v>보통 문제집을 풀면 강의가 없어 답지를 보고 문제를 혼자 이해했어야하는데 1:1로 질의 응답을 해주셔서 이해하는데 도움이 많이 되었습니다. 제가 모르는 부분을 더 집중적으로 자세하게 설명을 들을 수 있었고 못하는 부분을 보완하기 위해 무엇을 공부 해야하는지도 알 수 있어 좋았습니다.</v>
@@ -813,8 +813,8 @@
         <v>N수생</v>
       </c>
       <c r="E12" t="str" xml:space="preserve">
-        <v xml:space="preserve">이것 저것 다 해야할 것 같은 조급함에 이러지도 저러지도 못하고 있을때 담임선생님과의 학습상담을 통해서 저와 맞는 학습 계획을 세우고 저만의 템포로 공부할 수 있어서 좋았습니다_x000d_
-또한, 저는 맞는 인강쌤을 찾기 힘들어 많이 왔다갔다 거리는 인강 유목민이었습니다. 인강이 없으면 안된다고 생각했는데 학습상담을 통해 인강이 맞지 않는 과목의 경우여도 독학으로 좋은 성적을 받을 수 있음을 알게되었습니다. 머리가 복잡한 수험생을 옳은 길로 잘 이끌어주셨습니다</v>
+        <v xml:space="preserve">이것 저것 다 해야할 것 같은 조급함에 이러지도 저러지도 못하고 있을때 담임선생님과의 학습 상담을 통해서 저와 맞는 학습 계획을 세우고 저만의 템포로 공부할 수 있어서 좋았습니다_x000d_
+또한, 저는 맞는 인강쌤을 찾기 힘들어 많이 왔다갔다 거리는 인강 유목민이었습니다. 인강이 없으면 안된다고 생각했는데 학습 상담을 통해 인강이 맞지 않는 과목의 경우여도 독학으로 좋은 성적을 받을 수 있음을 알게되었습니다. 머리가 복잡한 수험생을 옳은 길로 잘 이끌어주셨습니다</v>
       </c>
       <c r="F12" t="str">
         <v>앞서 언급했듯 다양한 방면으로 공부법을 제시해주시고, 결정하게 해주셔서 좋았습니다. 사람마다 맞는 공부법이 다르기에 그것을 찾아 정착하는데에는 꽤 오랜 시간이 걸린다고 생각합니다. 이투스 담임선생님과의 꾸준한 소통과 학습 관리 시스템을 통해 시간낭비를 줄일 수 있었던 것 같습니다</v>
@@ -829,7 +829,7 @@
         <v>여러모로 학생만큼 고생하셨을텐데 길다면 긴, 짧다면 짧은 기간동안 감사했습니다! 선생님들의 격려와 응원, 도움이 없었다면 힘든 수험생활 진작에 무너졌을 것 같아요,, 제 수험생활에 함께해주셔서 감사합니다</v>
       </c>
       <c r="J12" t="str">
-        <v>수업이 없으면 안된다고 생각했는데 학습상담을 통해 저에게 맞는 공부법을 알려주셔서 좋은 성적을 받을 수 있었어요.</v>
+        <v>수업이 없으면 안된다고 생각했는데 학습 상담을 통해 저에게 맞는 공부법을 알려주셔서 좋은 성적을 받을 수 있었어요.</v>
       </c>
       <c r="K12" t="str">
         <v>학습 관리</v>
@@ -1219,7 +1219,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E23" t="str">
-        <v>재수학원에서 받은 학습상담은 나의 학습 방향을 구체적으로 설정하는 데 큰 도움이 되었다. 특히 상담을 통해 모든 과목을 동일하게 끌어올리기보다는, 부족한 과목은 기본 점수를 확보하는 수준으로 관리하고 자신 있는 과목은 최대한 점수를 끌어올리는 전략이 효과적이라는 점을 배웠다. 이에 따라 취약 과목은 핵심 개념 위주로 최소한의 점수를 확보하는 데 집중하고, 강점 과목에는 더 많은 시간을 투자해 고득점을 목표로 학습 계획을 세웠다. 이러한 전략적 접근 덕분에 전체적인 성적 균형을 유지하면서도 총점을 효율적으로 높일 수 있었고, 학습에 대한 부담도 줄일 수 있었다.</v>
+        <v>재수학원에서 받은 학습 상담은 나의 학습 방향을 구체적으로 설정하는 데 큰 도움이 되었다. 특히 상담을 통해 모든 과목을 동일하게 끌어올리기보다는, 부족한 과목은 기본 점수를 확보하는 수준으로 관리하고 자신 있는 과목은 최대한 점수를 끌어올리는 전략이 효과적이라는 점을 배웠다. 이에 따라 취약 과목은 핵심 개념 위주로 최소한의 점수를 확보하는 데 집중하고, 강점 과목에는 더 많은 시간을 투자해 고득점을 목표로 학습 계획을 세웠다. 이러한 전략적 접근 덕분에 전체적인 성적 균형을 유지하면서도 총점을 효율적으로 높일 수 있었고, 학습에 대한 부담도 줄일 수 있었다.</v>
       </c>
       <c r="F23" t="str">
         <v>재수학원의 1대1 질의응답 시스템은 모르는 문제를 단순히 해결하는 것을 넘어, 문제를 접근하는 방법 자체를 배우는 데 유용했다. 특히 모의고사 이후 틀린 문제를 질문하면 단순한 해설이 아니라 문제를 푸는 과정과 공략법을 단계적으로 설명해 주어, 같은 유형의 문제를 다시 만났을 때 스스로 해결할 수 있는 능력을 기를 수 있었다. 또한 과목별로 효율적인 풀이 순서와 시간 배분 방법 등 구체적인 학습방법까지 제시해 주어, 실전에서의 문제 해결 능력을 높이는 데 도움이 되었다. 이를 통해 단순 암기 중심의 공부에서 벗어나 전략적으로 문제를 해결하는 학습 습관을 형성할 수 있었다.</v>
@@ -1293,10 +1293,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E25" t="str">
-        <v>헉습에 집중할수있더록 멘탈관리를 잘해주셨습니다 주기적인 상담을 해주셨고 멘탈이 떨어질때 여러방법으로 상담을 주셔서 이갸낼수있었습니다 모의고사를 보고나면 과목별 학습상담이 도움이 되었습니다</v>
+        <v>헉습에 집중할수있더록 멘탈관리를 잘해주셨습니다 주기적인 상담을 해주셨고 멘탈이 떨어질때 여러방법으로 상담을 주셔서 이갸낼수있었습니다 모의고사를 보고나면 과목별 학습 상담이 도움이 되었습니다</v>
       </c>
       <c r="F25" t="str">
-        <v>과목별 성적변화에 대한 상담이 도움이되었고 그에따른 과목별 시간배분과 교재선정및 학습계획에 대해 도움을 받았습니다 어떤과목에 현재 더 시간을 쏟아야할지 가이드라인을 해주셨습니다 한과목에 치중하지않도록 시건배분에대한 계획에 도움을 받았습니다</v>
+        <v>과목별 성적변화에 대한 상담이 도움이되었고 그에따른 과목별 시간배분과 교재선정및 학습 계획에 대해 도움을 받았습니다 어떤과목에 현재 더 시간을 쏟아야할지 가이드라인을 해주셨습니다 한과목에 치중하지않도록 시건배분에대한 계획에 도움을 받았습니다</v>
       </c>
       <c r="G25" t="str">
         <v>기숙을 들어온 가장 중요한 목적이테블릿 핸드폰 관리인데 스스로 제어하기힘들기에 도움이 필요했습니다 필요할때 인강을 듣고 그외 방화벽이 있어 제어할수있어가장 큰 도움이 되었습니다 기숙을 들어온 가장 큰 목적이 스마트기기 관리인데 적절하게 관리가 되어 좋았어요</v>
@@ -1577,7 +1577,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E33" t="str">
-        <v>학습상담을 통해 내 수준과 목표에 맞는 공부 커리큘럼을 세우는 데 큰 도움을 받았다.공부 계획을 구체적으로 정리할 수 있었고, 부족한 부분을 보완할 방향도 명확해졌다. 덕분에 더 체계적으로 공부할 수 있게 되었다.</v>
+        <v>학습 상담을 통해 내 수준과 목표에 맞는 공부 커리큘럼을 세우는 데 큰 도움을 받았다.공부 계획을 구체적으로 정리할 수 있었고, 부족한 부분을 보완할 방향도 명확해졌다. 덕분에 더 체계적으로 공부할 수 있게 되었다.</v>
       </c>
       <c r="F33" t="str">
         <v>공부 계획을 잡는데 어려움이 많이 줄었다. 특히 나에게 맞는 인강과 교재를 추천해주어 불필요한 시행착오를 줄일 수 있었고, 방향성에 대한 확신이 생겼다. 그 결과 꾸준히 안정적인 학습을 이어갈 수 있었다.</v>
@@ -1722,7 +1722,7 @@
         <v>반수생</v>
       </c>
       <c r="E37" t="str">
-        <v>반수를 시작했을 때는 이미 늦었다는 생각이 들어 불안했지만, 이투스247재수학원에서 체계적인 관리와 상담을 받으며 더 빠르게 방향을 잡을 수 있었던 것 같다. 학습상담을 통해 현재 실력을 정확히 파악하고 효율적인 공부 방법을 제시받아 시간 낭비를 줄일 수 있었고, 생활상담을 통해 흐트러지기 쉬운 생활 패턴도 안정적으로 유지할 수 있었다. 또한 입시상담에서는 현실적인 조언과 전략을 통해 목표를 구체화할 수 있어 막연했던 불안이 많이 해소되었다. 전반적으로 늦게 시작했음에도 불구하고 빠르게 중심을 잡고 끝까지 버틸 수 있도록 큰 도움을 받은 만족스러운 경험이었다.</v>
+        <v>반수를 시작했을 때는 이미 늦었다는 생각이 들어 불안했지만, 이투스247재수학원에서 체계적인 관리와 상담을 받으며 더 빠르게 방향을 잡을 수 있었던 것 같다. 학습 상담을 통해 현재 실력을 정확히 파악하고 효율적인 공부 방법을 제시받아 시간 낭비를 줄일 수 있었고, 생활상담을 통해 흐트러지기 쉬운 생활 패턴도 안정적으로 유지할 수 있었다. 또한 입시상담에서는 현실적인 조언과 전략을 통해 목표를 구체화할 수 있어 막연했던 불안이 많이 해소되었다. 전반적으로 늦게 시작했음에도 불구하고 빠르게 중심을 잡고 끝까지 버틸 수 있도록 큰 도움을 받은 만족스러운 경험이었다.</v>
       </c>
       <c r="F37" t="str">
         <v>인강 추천이 체계적이고 수준에 맞게 이루어져서 공부 효율이 크게 올라갔다. 과목별로 필요한 강의를 정확히 짚어주어 불필요한 선택 고민이 줄었고, 덕분에 시간 낭비 없이 핵심 내용에 집중할 수 있어 전체적인 학습 만족도가 높았다.</v>
@@ -2288,7 +2288,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E53" t="str">
-        <v>이투스247 학원의 학습상담 코칭 시스템은 단순히 공부하라고 방향만 잡아주는 게 아니라, 내 현재 수준이랑 약점을 정확하게 짚어주고 그에 맞는 공부 계획을 같이 세워준다는 점에서 유용했다. 특히 혼자 공부하다 보면 내가 제대로 하고 있는지 불안할 때가 많았는데, 주기적으로 상담을 하면서 방향을 점검받을 수 있어서 시간 낭비를 줄이고 효율적으로 공부할 수 있었다.</v>
+        <v>이투스247 학원의 학습 상담 코칭 시스템은 단순히 공부하라고 방향만 잡아주는 게 아니라, 내 현재 수준이랑 약점을 정확하게 짚어주고 그에 맞는 공부 계획을 같이 세워준다는 점에서 유용했다. 특히 혼자 공부하다 보면 내가 제대로 하고 있는지 불안할 때가 많았는데, 주기적으로 상담을 하면서 방향을 점검받을 수 있어서 시간 낭비를 줄이고 효율적으로 공부할 수 있었다.</v>
       </c>
       <c r="F53" t="str">
         <v>질의응답 시스템은 혼자 공부하면서 막히는 부분을 바로 해결할 수 있다는 점에서 유용했다. 문제를 풀다가 이해가 안 되는 부분이 생기면 오래 끌지 않고 질문해서 바로 개념을 잡을 수 있었고, 단순히 답만 알려주는 게 아니라 풀이 과정이나 접근 방법까지 설명해줘서 비슷한 문제를 풀 때도 도움이 됐다. 혼자 독학할 때 생기는 답답함을 줄여주고 공부 흐름이 끊기지 않게 해준다는 점이 가장 좋았다.</v>
@@ -4072,10 +4072,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E102" t="str">
-        <v>학습상담을 할때 전체적으로 계획표를 작성하는법을 배웠다.또한 계획표를 작성하며 각각의 과목 시간과 과목 공부법에 대해 배웠다.그렇게 하나하나 딱잡아줘서 좋았다.그리고 내가 계획표를 잡고 익숙해지면 나만의 방법이 생겨서 하려고 할때 자유롭게 할수 있게 해주어서 좋았다.</v>
+        <v>학습 상담을 할때 전체적으로 계획표를 작성하는법을 배웠다.또한 계획표를 작성하며 각각의 과목 시간과 과목 공부법에 대해 배웠다.그렇게 하나하나 딱잡아줘서 좋았다.그리고 내가 계획표를 잡고 익숙해지면 나만의 방법이 생겨서 하려고 할때 자유롭게 할수 있게 해주어서 좋았다.</v>
       </c>
       <c r="F102" t="str">
-        <v>학원에서 설문조사를 통해 개인의 학습 성향과 목표를 파악한 뒤 맞춤형 학습계획을 세워준 점이 매우 좋았습니다. 단순히 일률적인 계획이 아니라 나에게 맞는 속도와 방식으로 공부할 수 있어 효율이 높아졌고, 학습 방향이 명확해져 꾸준히 실천하는 데 큰 도움이 되었습니다.</v>
+        <v>학원에서 설문조사를 통해 개인의 학습 성향과 목표를 파악한 뒤 맞춤형 학습 계획을 세워준 점이 매우 좋았습니다. 단순히 일률적인 계획이 아니라 나에게 맞는 속도와 방식으로 공부할 수 있어 효율이 높아졌고, 학습 방향이 명확해져 꾸준히 실천하는 데 큰 도움이 되었습니다.</v>
       </c>
       <c r="G102" t="str">
         <v>전자출결 시스템을 통해 출석 관리가 체계적으로 이루어져 스스로 학습 태도를 점검할 수 있었고, 지각이나 결석을 줄이는 데에도 도움이 되었습니다. 이런 점들이 학습 집중도를 높이는 데 큰 역할을 했습니다.</v>
@@ -4429,10 +4429,10 @@
         <v>N수생</v>
       </c>
       <c r="E112" t="str">
-        <v>학습상담을 통해 제 공부 습관과 문제점을 객관적으로 파악할 수 있었고, 개인에 맞는 구체적인 학습 계획을 세울 수 있어 큰 도움이 되었습니다. 단순한 조언이 아니라 실천 가능한 방법을 제시해 주셔서 꾸준히 실력을 향상시킬 수 있었고, 공부 방향에 대한 불안도 줄어들었습니다.</v>
+        <v>학습 상담을 통해 제 공부 습관과 문제점을 객관적으로 파악할 수 있었고, 개인에 맞는 구체적인 학습 계획을 세울 수 있어 큰 도움이 되었습니다. 단순한 조언이 아니라 실천 가능한 방법을 제시해 주셔서 꾸준히 실력을 향상시킬 수 있었고, 공부 방향에 대한 불안도 줄어들었습니다.</v>
       </c>
       <c r="F112" t="str">
-        <v>학습계획과 플래너 관리를 통해 하루 공부 흐름을 체계적으로 정리할 수 있었고, 목표를 구체적으로 세워 실천하는 데 큰 도움이 되었습니다. 계획 대비 실천 여부를 점검하며 부족한 부분을 바로 보완할 수 있었고, 꾸준한 관리 덕분에 학습 습관이 안정적으로 자리 잡았습니다.</v>
+        <v>학습 계획과 플래너 관리를 통해 하루 공부 흐름을 체계적으로 정리할 수 있었고, 목표를 구체적으로 세워 실천하는 데 큰 도움이 되었습니다. 계획 대비 실천 여부를 점검하며 부족한 부분을 바로 보완할 수 있었고, 꾸준한 관리 덕분에 학습 습관이 안정적으로 자리 잡았습니다.</v>
       </c>
       <c r="G112" t="str">
         <v>와이파이를 끊고 핸드폰을 제출하면서 불필요한 자극이 차단되어 공부에 온전히 집중할 수 있었습니다. 자연스럽게 딴짓이 줄어들고 몰입 시간이 늘어나 학습 효율이 크게 향상되었습니다. 또한 규칙적인 생활 습관이 형성되어 자기관리 능력도 함께 키울 수 있었습니다.</v>
@@ -4444,7 +4444,7 @@
         <v>학원에서의 시간 동안 체계적인 학습 관리와 세심한 상담 덕분에 흔들리지 않고 목표를 향해 나아갈 수 있었습니다. 항상 학생 한 명 한 명을 진심으로 신경 써주시고, 필요한 조언과 격려를 아끼지 않아 큰 힘이 되었습니다. 덕분에 공부 습관과 자신감을 함께 키울 수 있었습니다. 진심으로 감사드립니다. 덕분에 원하는 대학에 합격한거같습니다!</v>
       </c>
       <c r="J112" t="str">
-        <v>학습계획과 플래너 관리를 통해 하루 공부 흐름을 체계적으로 정리할 수 있었고, 목표를 구체적으로 세워 실천하는 데 큰 도움이 되었어요.</v>
+        <v>학습 계획과 플래너 관리를 통해 하루 공부 흐름을 체계적으로 정리할 수 있었고, 목표를 구체적으로 세워 실천하는 데 큰 도움이 되었어요.</v>
       </c>
       <c r="K112" t="str">
         <v>학습 계획, 플래너 관리</v>
@@ -5840,7 +5840,7 @@
         <v>국어 공부가 가장하기도 어렵고 어떻게 해야할지 막막했는데 저한테 맞춰서 정말 세세하게 신경써주시면서 코핑해주셔서 좋았습니다. 코칭 할때마다 국어 공부는 어떤지 어떤부분이 잘안되는지 물어봐주셔서 공부하는데 많은 도움이 되었습니다</v>
       </c>
       <c r="F151" t="str">
-        <v>아침에 꾸준히 학습계획을 쓰게 되면서 하루 목표 공부량과 시간을 정확히 알 수 있어서 좋았고 꾸준히 쓰다보니 진도도 안밀리고 부족한부분 보완할점도 같이 알려주셔서 공부하는데 많은 도움을 받았습니다</v>
+        <v>아침에 꾸준히 학습 계획을 쓰게 되면서 하루 목표 공부량과 시간을 정확히 알 수 있어서 좋았고 꾸준히 쓰다보니 진도도 안밀리고 부족한부분 보완할점도 같이 알려주셔서 공부하는데 많은 도움을 받았습니다</v>
       </c>
       <c r="G151" t="str">
         <v>잠이 많아서 정말 자주 졸아서 공부 집중시간도 짧고 순공시간도 짧았는데 계속 돌아다니시면서 깨워주셔서 갈 수록 덜 졸게되고 집중시간도 길어지고 공부도 집중해서 더 잘 할 수 있었던 것 같아 좋았습니다.</v>
@@ -6473,7 +6473,7 @@
         <v>N수생</v>
       </c>
       <c r="E169" t="str">
-        <v>담임선생님과 함께 본인에 맞는 커리큘럼을 짜며 소통할수있어 좋았고 달별로 점검 받으며 부족한 과목의 공부량을 더 늘리거나 하는등의 즉각적인 학습계획수정이 용이했음,또한 자주 특강을 개설하여 선택학생에게  공부중 부족한 부분을 추가로 공부할수 있도록 하게해서 좋았음.</v>
+        <v>담임선생님과 함께 본인에 맞는 커리큘럼을 짜며 소통할수있어 좋았고 달별로 점검 받으며 부족한 과목의 공부량을 더 늘리거나 하는등의 즉각적인 학습 계획수정이 용이했음,또한 자주 특강을 개설하여 선택학생에게  공부중 부족한 부분을 추가로 공부할수 있도록 하게해서 좋았음.</v>
       </c>
       <c r="F169" t="str">
         <v>2주마다 학습멘토와 함께 공부를 점검하며 한무동안 소홀하거나 잘했던 부분을 확인하고 다음주의 공부게획을 점검하는 점이좋았고,학습매니저에게 공부를 점검받아야하므로 공부를 계속 하게되서 좋았고,학습 매니저에게 모르는 부분을 물어보면서 공부할수있는점도 좋았다</v>
@@ -7108,7 +7108,7 @@
         <v>N수생</v>
       </c>
       <c r="E186" t="str">
-        <v>이투스247 하남점에서의 학습상담은 현재 나의 학습 상태를 객관적으로 파악하는 데 큰 도움이 되었다. 특히 과목별 취약점을 구체적으로 짚어주고, 이에 맞는 학습 방법과 계획을 제시해 주어 효율적인 공부 방향을 설정할 수 있었다. 또한 꾸준한 상담을 통해 학습 동기를 유지하고 스스로를 점검할 수 있는 계기가 되었다.</v>
+        <v>이투스247 하남점에서의 학습 상담은 현재 나의 학습 상태를 객관적으로 파악하는 데 큰 도움이 되었다. 특히 과목별 취약점을 구체적으로 짚어주고, 이에 맞는 학습 방법과 계획을 제시해 주어 효율적인 공부 방향을 설정할 수 있었다. 또한 꾸준한 상담을 통해 학습 동기를 유지하고 스스로를 점검할 수 있는 계기가 되었다.</v>
       </c>
       <c r="F186" t="str">
         <v>성적 리포팅 및 관리는 나의 학습 결과를 체계적으로 확인하고 분석하는 데 큰 도움이 되었다. 정기적으로 성적 변화를 확인하면서 부족한 과목과 단원을 파악할 수 있었고, 이를 바탕으로 학습 계획을 보완할 수 있었다. 또한 성적 추이를 통해 자신의 노력과 성과를 객관적으로 인식할 수 있어 학습 동기 유지에도 긍정적인 영향을 주었다.</v>
@@ -7255,7 +7255,7 @@
       </c>
       <c r="F190" t="str" xml:space="preserve">
         <v xml:space="preserve">작년 수능 저의 영어는 6등급으로 처참했습니다. 영어를 올리는게 가장 시_x000d_
-급하였고 따라서 이투스 247에서 영어선생님과의 1대1 질의응담을 진행했었는데 모르는 문제에 답변해 주실 뿐만 아니라 영어 학습을 어떻게 진행하는지 전체적인 학습계획과 방법을 함께 진향해 주신 부분이 너무 만족스러웠습니다. 그결과, 수능에서 3등급이라는 점수를 받을 수 있었습니다.</v>
+급하였고 따라서 이투스 247에서 영어선생님과의 1대1 질의응담을 진행했었는데 모르는 문제에 답변해 주실 뿐만 아니라 영어 학습을 어떻게 진행하는지 전체적인 학습 계획과 방법을 함께 진향해 주신 부분이 너무 만족스러웠습니다. 그결과, 수능에서 3등급이라는 점수를 받을 수 있었습니다.</v>
       </c>
       <c r="G190" t="str">
         <v>체력이 약했던 저는 수업시간에 자주 졸곤 했었는데 그럴 때 마다 감독 선생님께서 잊지 않고 매번 깨워주셨습니다. 그 날 하루를 다 날려먹을 수도 있었던 저를 항상 5분 이내로 깨워주셔서 감사했던 기억이 납니다.</v>
@@ -7369,7 +7369,7 @@
         <v>N수생</v>
       </c>
       <c r="E193" t="str">
-        <v>매주 정기적으로 듣고 싶은 과목의 선생님과 학습상담을 할 수 있어서 좋았습니다. 매일 앉아서 공부만 하다보니 내가 지금 잘하고 있는 건가 하는 불안감에 오히려 공부에 집중을 하지 못할때가 있었는데 그럴때마다 배정받은 과목 선생님께 가서 상담을 하면서 다시 마음을 다잡고 공부할수 있었습니다.</v>
+        <v>매주 정기적으로 듣고 싶은 과목의 선생님과 학습 상담을 할 수 있어서 좋았습니다. 매일 앉아서 공부만 하다보니 내가 지금 잘하고 있는 건가 하는 불안감에 오히려 공부에 집중을 하지 못할때가 있었는데 그럴때마다 배정받은 과목 선생님께 가서 상담을 하면서 다시 마음을 다잡고 공부할수 있었습니다.</v>
       </c>
       <c r="F193" t="str">
         <v>독학 기숙인데도 불구하고 주요 과목 강사님들과 일대일 질문시간을 가질 수 있어서 궁금한 문제에 대한 선생님의 답변시간을 기다리느라 시간을 낭비하지 않고 바로바로 모르는 문제를 해결할 수 있었습니다.</v>
@@ -7992,7 +7992,7 @@
         <v>선생님들께서 주기적으로 상담해주시면서 과목별로 자세히 어떻게 공부해야하는지 알려주셨고, 단체로 실전 모의고사를 친 후에 상담했던 것도 도움이 많이 되었고, 학습 뿐만 아니라 마음가짐에 대해서 알려주신 것도 유용했습니다.</v>
       </c>
       <c r="F210" t="str">
-        <v>일주일 단위로 자세히 학습계획표를 짜게 하셨는데, 구체적이고 정확한 목표를 정하고 나니까 오늘은 무엇을 하고 어디까지 끝내야 할지가 눈에 보여서 학습량이 늘어나는 데 도움이 되었습니다.</v>
+        <v>일주일 단위로 자세히 학습 계획표를 짜게 하셨는데, 구체적이고 정확한 목표를 정하고 나니까 오늘은 무엇을 하고 어디까지 끝내야 할지가 눈에 보여서 학습량이 늘어나는 데 도움이 되었습니다.</v>
       </c>
       <c r="G210" t="str">
         <v>원래 혼자서 공부할때는 공부하다가도 수시로 휴대폰을 확인하는 습관이 있었는데, 핸드폰을 강제로 걷어가시니까 공부중 딴 짓을 하는 시간이 줄어들고 공부의 질이 향상되는 것을 느꼈습니다.</v>
@@ -8561,7 +8561,7 @@
         <v>반수생</v>
       </c>
       <c r="E226" t="str">
-        <v>코치시스템을 통해 혼자 공부할때의 방향을 설정하는데 큰 도움을 받았습니다. 현재 공부 상태를 점검하고 부족한 부분을 알 수 있었고 그에 맞는 학습계획을 새울 수 있었습니다. 이로 인해 집중도도 높아지고 공부시간을 더 효과적으로 사용할 수 있었습니다.</v>
+        <v>코치시스템을 통해 혼자 공부할때의 방향을 설정하는데 큰 도움을 받았습니다. 현재 공부 상태를 점검하고 부족한 부분을 알 수 있었고 그에 맞는 학습 계획을 새울 수 있었습니다. 이로 인해 집중도도 높아지고 공부시간을 더 효과적으로 사용할 수 있었습니다.</v>
       </c>
       <c r="F226" t="str">
         <v>혼자 공부하다가 계속 모르는 문제들을 바로바로 선생님들께 여쭈어 볼 수 있어서 좋았습니다. 질문하는 것에 대해 부담이 있었는데 1:1 질문 시스템 덕분에 궁금한 점을 물어볼 수 있었습니다. 덕분에 문제들을 정확히 알고 넘어갈 수 있었습니다.</v>
@@ -8846,7 +8846,7 @@
         <v>가장 좋았던 건 물어보고 싶을 때 언제든지 물어볼 수 있는 것이었습니다. 항상 멘토, 선생님들이 상주해계시고 할때마다 친절하고 자세히 알려주셔서 정말 좋았습니다. 또 한분한분 진심으로 알게해주려고 하셔서 감사했습니다. 단순한 문재풀이 뿐만 아니라 접근방법도 상세히 알려주십니다.</v>
       </c>
       <c r="F234" t="str">
-        <v>독학재수학원이기 때문에 자기관리가 힘들 수 있습니다. 하지만 과목별로 주기적인 상담을 통해 본인 진도에 맞춰서 알맞은 계획을 세워주십니다. 저는 학습계획을 세우는 것에 있어서 어려움을 느꼈는데 학습 관리 시스템 덕분에 계획 짜는 법에 도움을 많이 받았습니다.</v>
+        <v>독학재수학원이기 때문에 자기관리가 힘들 수 있습니다. 하지만 과목별로 주기적인 상담을 통해 본인 진도에 맞춰서 알맞은 계획을 세워주십니다. 저는 학습 계획을 세우는 것에 있어서 어려움을 느꼈는데 학습 관리 시스템 덕분에 계획 짜는 법에 도움을 많이 받았습니다.</v>
       </c>
       <c r="G234" t="str">
         <v>수험생활 중 굉장히 힘든 점 중 하나가 스마트폰 관리라고 생각합니다. 이투스 247에서는 강제적으로라도 휴대폰을 수거해서 처음에는 조금 힘들 수 있지만 결국에는 많은 도움을 받았던 것 같습니다.</v>
@@ -9070,7 +9070,7 @@
         <v>처음에 시작할 때 아무 방향 없이 시작 했었는데, 개별 학습 데이터를 바탕으로 취약점과 공부 방향에 개인의 방향을 알려주어 좋았다. 특히 점수대 별에 맞춰, 시기별로 어떤 전략으로 공부하며 좋을지 알려주어서, 혼자서 공부할 때의 막막함을 해소 할 수 있어서 좋았다.</v>
       </c>
       <c r="F240" t="str">
-        <v>나는 원래 공부할 때 학습계획은 대략적으로 만 세우고, 플레너는 쓰지도 않았었다. 하지만 이투스247에서 제공하는 프로그램으로 학습계획과 플레너를 쓰면서, 객관적인 공부시간을 시각적으로 파악하며, 따로 큰 힘을 들이지 않아도 공부계획을 세울 수 있었다. 그리고 완료한 항목에 체크 표시를 해 나가면서 성취감도 얻을 수 있었고, 나의 기록을 보며 특정과목에만 치우치지 않게 공부양을 조절하며, 매일 기록을 복기하며 어려웠던 부분을 마스터 할 수 있었다.</v>
+        <v>나는 원래 공부할 때 학습 계획은 대략적으로 만 세우고, 플레너는 쓰지도 않았었다. 하지만 이투스247에서 제공하는 프로그램으로 학습 계획과 플레너를 쓰면서, 객관적인 공부시간을 시각적으로 파악하며, 따로 큰 힘을 들이지 않아도 공부계획을 세울 수 있었다. 그리고 완료한 항목에 체크 표시를 해 나가면서 성취감도 얻을 수 있었고, 나의 기록을 보며 특정과목에만 치우치지 않게 공부양을 조절하며, 매일 기록을 복기하며 어려웠던 부분을 마스터 할 수 있었다.</v>
       </c>
       <c r="G240" t="str" xml:space="preserve">
         <v xml:space="preserve">나의 공부에서 가장 큰 문제는 공부시간을 제대로 활용하지 못하고 딴 짓을 한다는 것이었다. 그런데 와이파이 장벽은 스스로 자기 통제가 어려운 수험 생활 초반에 올바른 공부 습관을 형성하는데 큰 도움을 주었다. _x000d_
@@ -9318,7 +9318,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E247" t="str">
-        <v>각 과목별로 코칭을 받을 수 있어서 너무 좋았어요. 학습상담을 통해 과목별로 제가 부족한 부분과 취약한 부분을 잘 보완할 수 있었어요. 또한 부족한 점을 베꿀 수 있는 자세한 대안까지 제안해주신 덕에 떨어졌던 자신감을 얻을 수 있었던 기회이기도 했습니다.</v>
+        <v>각 과목별로 코칭을 받을 수 있어서 너무 좋았어요. 학습 상담을 통해 과목별로 제가 부족한 부분과 취약한 부분을 잘 보완할 수 있었어요. 또한 부족한 점을 베꿀 수 있는 자세한 대안까지 제안해주신 덕에 떨어졌던 자신감을 얻을 수 있었던 기회이기도 했습니다.</v>
       </c>
       <c r="F247" t="str">
         <v>공부를 어디서부터 어떻게 시작해야되고 계획해야되는지 막막한 저에게 공부할 큰 틀을 제안해주고 계획을 세우는 방법을 알려주는 이 시스템이 정날 유용했습니다. 제가 계획을 세우면 선생님께서 보고 피드백을 주셨기 때문에 더 효율적이고 도움이 되는 공부계획을 세우고 실천할 수 있었습니다.</v>
@@ -9458,7 +9458,7 @@
         <v>N수생</v>
       </c>
       <c r="E251" t="str">
-        <v>학창시절 공부를 해본적이 없어서 어떤식으로 공부를 해가야 할지 몰랐는데 학습상담으로 공부하는 방법을 알려주셨고 과목별 공부시간 배분과 하루 최소할당치 같은 양을 정해주는게 큰 도움이 됐습니다</v>
+        <v>학창시절 공부를 해본적이 없어서 어떤식으로 공부를 해가야 할지 몰랐는데 학습 상담으로 공부하는 방법을 알려주셨고 과목별 공부시간 배분과 하루 최소할당치 같은 양을 정해주는게 큰 도움이 됐습니다</v>
       </c>
       <c r="F251" t="str">
         <v>학창시절에 공부를 안했었고 당연히 수능 인강에 대해 무지하던 시절에 모의평가 성적을 보고 저에게 맞을만한 인강 강사를 추천해 준 것과 올해 수능에서 끝을 내기 위해 몇일까지 어느정도를 들어놔야 한다는 것을 알려주는게 시간관리 측면에서 도움이 되었습니다</v>
@@ -9528,10 +9528,10 @@
         <v>반수생</v>
       </c>
       <c r="E253" t="str" xml:space="preserve">
-        <v xml:space="preserve">재수학원에서 진행된 학습상담은 단순히 공부 방법을 듣는 것을 넘어서, 제 공부 습관과 문제점을 객관적으로 돌아볼 수 있는 계기가 되었습니다. 특히 스스로는 잘 인지하지 못했던 시간 관리의 비효율성과 과목별 학습 편차를 구체적으로 짚어주어 학습 방향을 다시 설정하는 데 큰 도움이 되었습니다._x000d_
+        <v xml:space="preserve">재수학원에서 진행된 학습 상담은 단순히 공부 방법을 듣는 것을 넘어서, 제 공부 습관과 문제점을 객관적으로 돌아볼 수 있는 계기가 되었습니다. 특히 스스로는 잘 인지하지 못했던 시간 관리의 비효율성과 과목별 학습 편차를 구체적으로 짚어주어 학습 방향을 다시 설정하는 데 큰 도움이 되었습니다._x000d_
 또한 상담을 통해 과목별로 자주 틀리는 문제 유형을 분석하고, 이에 맞는 보완 방법을 제시받을 수 있었습니다. 예를 들어 오답노트 정리 방식이나 문제 풀이 순서를 조정하는 방법 등을 적용하면서, 단순히 문제를 많이 푸는 것이 아니라 틀린 이유를 이해하는 데 집중하게 되었습니다. 그 결과 학습의 효율이 높아졌다고 느꼈습니다._x000d_
 더불어 멘탈 관리 측면에서도 많은 도움이 되었습니다. 재수 과정에서 생기는 불안감이나 슬럼프에 대해 현실적인 조언을 들을 수 있었고, 이를 바탕으로 꾸준히 공부를 이어갈 수 있는 루틴을 만들 수 있었습니다._x000d_
-이처럼 학습상담은 제게 맞는 공부 방법을 찾고 이를 지속할 수 있도록 도와준 중요한 경험이었다고 생각합니다.</v>
+이처럼 학습 상담은 제게 맞는 공부 방법을 찾고 이를 지속할 수 있도록 도와준 중요한 경험이었다고 생각합니다.</v>
       </c>
       <c r="F253" t="str" xml:space="preserve">
         <v xml:space="preserve">학습 계획 플래너는 하루 공부를 체계적으로 관리하는 데 큰 도움이 되었습니다. 이전에는 해야 할 공부를 막연하게 생각하고 넘어가는 경우가 많았는데, 플래너를 사용하면서 하루 목표를 구체적으로 설정하고 이를 실제로 실천하는 습관을 기를 수 있었습니다._x000d_
@@ -9731,7 +9731,7 @@
         <v>사이트 들어가서 영어듣기 평가를 자주 했었다 솔직히 영어듣기는 따로 종이책 사기는 부담스러운데 그냥 간편하게 패드로 답 체크하고 들을 수 있어서 편했다 특히 학원에서 이용하니 다른 sns에 안 들어가고 바로 사이트&gt;영듣 들어가서 할 수 있었다</v>
       </c>
       <c r="I258" t="str">
-        <v>학원 다니는 학생들도 엄청 많았는데 1명씩 다 돌봐주신 거에 감사드려요 매일 학습상담도 다 받아주시고 사소한 고민도 다 들어주셔서 감사했습니다 또 재수생이어도 혼자가 아니고 어딘가에 소속되어있다는 사실이 가장 든든했습니다</v>
+        <v>학원 다니는 학생들도 엄청 많았는데 1명씩 다 돌봐주신 거에 감사드려요 매일 학습 상담도 다 받아주시고 사소한 고민도 다 들어주셔서 감사했습니다 또 재수생이어도 혼자가 아니고 어딘가에 소속되어있다는 사실이 가장 든든했습니다</v>
       </c>
       <c r="J258" t="str">
         <v>짧은 반수 기간에도 상담과 맞춤 교재 추천, 휴대폰 관리와 모의고사 덕분에 집중력을 높이고 성적을 올릴 수 있었어요.</v>
@@ -9929,7 +9929,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E264" t="str">
-        <v>공부를 하다보면 막막할때가 잦은데, 입시를 성공하신 선생님들의 학습상담이 있어서 슬럼프나 막막할때 잘 넘어갈수 있었고, 때로는 엄격하지만 때로는 진중하고 재밌게 지친 수험생활을 위로해주신점이 유용했습니다.</v>
+        <v>공부를 하다보면 막막할때가 잦은데, 입시를 성공하신 선생님들의 학습 상담이 있어서 슬럼프나 막막할때 잘 넘어갈수 있었고, 때로는 엄격하지만 때로는 진중하고 재밌게 지친 수험생활을 위로해주신점이 유용했습니다.</v>
       </c>
       <c r="F264" t="str" xml:space="preserve">
         <v xml:space="preserve">노베상태에서, 인강이나 책 선택조차 막막할 시기가 있었는데, 선생님이 계셔서 어떤 책을 어떻게 공부해야할지 알수 있어서 유용했습니다._x000d_
@@ -9967,7 +9967,7 @@
         <v>반수생</v>
       </c>
       <c r="E265" t="str">
-        <v>반수하고 6월에 기숙학원에 들어와서 어떤 선생님에 수업을 들어야할지 고민하던 중 이투스 이천 기숙학원에 계시는 담당 선생님의 학습상담을 통해 빠르게 공부의 방향을 잡고 진도를 나갈 수 있었습니다.</v>
+        <v>반수하고 6월에 기숙학원에 들어와서 어떤 선생님에 수업을 들어야할지 고민하던 중 이투스 이천 기숙학원에 계시는 담당 선생님의 학습 상담을 통해 빠르게 공부의 방향을 잡고 진도를 나갈 수 있었습니다.</v>
       </c>
       <c r="F265" t="str">
         <v>이투스 이천 247 기숙학원에 계시는 담당선생님께서 매주 상담을 진행하시며 플레너에 계획한 계획을 잘 지켰는지 매주 검사하고 방향성을 정하는 시간을 가졌는데요. 이 덕분에 학습 분량 조절을 원활히 할 수 있었습니다</v>
@@ -10102,7 +10102,7 @@
         <v>항상 진심을 다해 학생들을 대해주시는 것이 느껴져서 재수기간 동안 우울하지 않고 즐겁게 공부할 수 있었던 것 같습니다. 이투스를 선택한 것이 제가 한 선택 중 가장 최고의 선택이었습니다. 이투스 덕분에 좋은 결과를 이룰 수 있었던 것 같습니다!</v>
       </c>
       <c r="J267" t="str">
-        <v>학습계획을 세우는 데 어려움이 있었는데, 학습 전문 선생님 덕분에 계획을 어떻게 짜야 하는지 많은 도움을 받을 수 있었어요.</v>
+        <v>학습 계획을 세우는 데 어려움이 있었는데, 학습 전문 선생님 덕분에 계획을 어떻게 짜야 하는지 많은 도움을 받을 수 있었어요.</v>
       </c>
       <c r="K267" t="str">
         <v>학습 계획</v>
@@ -10137,10 +10137,10 @@
         <v>덕분에 좋은 학교 입학할 수 있었습니다! 감사합니다. 모의고사 성적이 잘 나오는데도 끝까지 수시로 대학 갈 생각만 했더라면, 수능 때 미끄러질까 봐 걱정하고 수시 원서를 낮게만 넣었다면 정말 후회할 뻔했습니다. 저는 지금 수시 원서 6장 중 가장 높게 적었던 학교보다도 높은 학교를 입학하게 되었으며, 이러한 입학 전략을 짜게 해 주신 선생님께 감사합니다.</v>
       </c>
       <c r="J268" t="str">
-        <v>입시 상담과 빠른 질의응답, 체계적인 면학 관리 덕분에 좋은 환경에서 재수를 마쳤어요.</v>
+        <v>입시 상담과 빠른 질의응답, 체계적인 면학 분위기 관리 덕분에 좋은 환경에서 재수를 마쳤어요.</v>
       </c>
       <c r="K268" t="str">
-        <v>입시 관리, 질의응답</v>
+        <v>입시 관리, 질의응답, 면학 분위기</v>
       </c>
     </row>
     <row r="269">
@@ -10157,7 +10157,7 @@
         <v>반수생</v>
       </c>
       <c r="E269" t="str">
-        <v>학습상담을 진행하면서 공부 방향을 정하고 그에 맞춰서 공부하면서 열심히 공부 할 수 있었던것 같다. 당일 할 일을 정하여 그것만큼은 꼭 해결하려한 것이 공부에 큰 도움이 됐다고 생각했다.</v>
+        <v>학습 상담을 진행하면서 공부 방향을 정하고 그에 맞춰서 공부하면서 열심히 공부 할 수 있었던것 같다. 당일 할 일을 정하여 그것만큼은 꼭 해결하려한 것이 공부에 큰 도움이 됐다고 생각했다.</v>
       </c>
       <c r="F269" t="str">
         <v>평소에 계획을 세우고 공부하기보다는 그냥 마구잡이로 공부를 하는 성향이 있었다. 하지만 계획을 세우면서 공부하니 좀 더 효과적으로 공부할 수 있었던 것 같다. 계획을 세우는 습관을 들임으로써 앞으로도 나에게 큰 도움이 될 것 같다고 생각이 든다.</v>
@@ -10368,7 +10368,7 @@
         <v>N수생</v>
       </c>
       <c r="E275" t="str">
-        <v>전반적인 성적, 부족한 과목과 파트를 자세히 파악해주시고 이를 토대로 구체적인 학습 방향을 제시해주셔서 학습계획 수립에 큰 도움이 되었습니다. 특히 저는 수학과 탐구 과목이 부족하였는데, 제시해주신 학습 방향대로 공부하니 성적향상을 거둘 수 있었습니다.</v>
+        <v>전반적인 성적, 부족한 과목과 파트를 자세히 파악해주시고 이를 토대로 구체적인 학습 방향을 제시해주셔서 학습 계획 수립에 큰 도움이 되었습니다. 특히 저는 수학과 탐구 과목이 부족하였는데, 제시해주신 학습 방향대로 공부하니 성적향상을 거둘 수 있었습니다.</v>
       </c>
       <c r="F275" t="str">
         <v>수많은 콘텐츠가 넘쳐나는 현재 대학 입시 상황에서 무슨 교재와 강의를 선택해야 저의 현재 성적대에 도움이 될지 잘 모르겠어서 힘들었었는데 분석하신 제 성적을 바탕으로 각 과목의 교재와 강의를 꼼꼼히 추천해 주셔서 크게 도움이 되었습니다.</v>
@@ -10438,9 +10438,9 @@
         <v>N수생</v>
       </c>
       <c r="E277" t="str" xml:space="preserve">
-        <v xml:space="preserve">학습상담을 하면서 이후의 공부 계획과 방향성을 잡기 좋아서 만족스러웠다._x000d_
+        <v xml:space="preserve">학습 상담을 하면서 이후의 공부 계획과 방향성을 잡기 좋아서 만족스러웠다._x000d_
 _x000d_
-그동안 공부해온 산물들을 들고 담임 선생님과 이후에 어떻게 공부해내가면 좋을지를 얘기하였었는데 수시라면 수시전략대로 정시라면 정시대로 구체적 성적 향상에 도움 될만한 이야기를 해주셔서 그 학습상담이 목표 대학에 합격하는 것에 대해 큰 도움이 되었던 것 같다.</v>
+그동안 공부해온 산물들을 들고 담임 선생님과 이후에 어떻게 공부해내가면 좋을지를 얘기하였었는데 수시라면 수시전략대로 정시라면 정시대로 구체적 성적 향상에 도움 될만한 이야기를 해주셔서 그 학습 상담이 목표 대학에 합격하는 것에 대해 큰 도움이 되었던 것 같다.</v>
       </c>
       <c r="F277" t="str" xml:space="preserve">
         <v xml:space="preserve">언제든지 궁금한 게 생기면 1:1로 질문할 수 있다는 점이 큰 메리트를 가지고 있었던 것 같다._x000d_
@@ -10988,7 +10988,7 @@
         <v>덕분에 공부하는 방법을 알았고 공부의 재미를 깨달았습니다. 선생님들께 상담하고 질문하며 해당 과목을 더 깊게 파고들 수 있었고, 성적을 많이 올렸습니다. 아침마다 반갑게 인사해 주시고, 담임선생님이 아니더라도 관심 가지고 성적 체크해 주셔서 감사했습니다!</v>
       </c>
       <c r="J292" t="str">
-        <v>반수로 들어왔는데 담임 선생님이 매주 학습계획을 점검하고 방향성을 잡아주셔서 빠르게 진도를 나갈 수 있었습니다.</v>
+        <v>반수로 들어왔는데 담임 선생님이 매주 학습 계획을 점검하고 방향성을 잡아주셔서 빠르게 진도를 나갈 수 있었습니다.</v>
       </c>
       <c r="K292" t="str">
         <v>학습 계획</v>
@@ -11151,7 +11151,7 @@
         <v>생활상담 코칭 시스템은 학습 외적인 고민까지 함께 다룰 수 있어 정서적 안정에 큰 도움이 되었습니다. 재수 생활에서 느끼는 불안감이나 스트레스를 주기적으로 점검하고 조언을 받을 수 있어 집중력을 유지하는 데 유익했습니다. 또한 개인의 생활 패턴을 점검하고 개선 방향을 제시해 주어 보다 규칙적이고 효율적인 학습 습관을 형성하는 데에도 긍정적인 역할을 했습니다.</v>
       </c>
       <c r="F297" t="str">
-        <v>학습계획 및 플래너 관리 시스템은 하루와 주간 단위로 목표를 구체적으로 설정하고 점검할 수 있어 학습 방향을 명확하게 잡는 데 도움이 되었습니다. 계획 대비 실천 여부를 확인하면서 스스로 부족한 부분을 파악하고 보완할 수 있었고, 시간 관리 능력도 자연스럽게 향상되었습니다. 또한 꾸준한 기록을 통해 학습 습관을 체계적으로 유지하는 데에도 큰 도움이 되었습니다.</v>
+        <v>학습 계획 및 플래너 관리 시스템은 하루와 주간 단위로 목표를 구체적으로 설정하고 점검할 수 있어 학습 방향을 명확하게 잡는 데 도움이 되었습니다. 계획 대비 실천 여부를 확인하면서 스스로 부족한 부분을 파악하고 보완할 수 있었고, 시간 관리 능력도 자연스럽게 향상되었습니다. 또한 꾸준한 기록을 통해 학습 습관을 체계적으로 유지하는 데에도 큰 도움이 되었습니다.</v>
       </c>
       <c r="G297" t="str">
         <v>출석관리 시스템은 규칙적인 생활을 유지하는 데 큰 도움이 되었습니다. 매일 정해진 시간에 등원하고 체크를 받는 과정이 학습 리듬을 안정적으로 만들어 주었고, 지각이나 결석을 줄이려는 책임감도 자연스럽게 생겼습니다. 또한 출석 기록을 통해 자신의 생활 태도를 객관적으로 확인할 수 있어 스스로를 관리하는 데 긍정적인 영향을 주었습니다.</v>
@@ -11757,7 +11757,7 @@
         <v>N수생</v>
       </c>
       <c r="E314" t="str">
-        <v>담당 과목 선생님들께서 상주하시면서 매주 학습상담과 질의응답을 받아주셔서 정말 좋았습니다. 모르는 점이 있으면 바로 질의응답이 가능하다는 점이 수험생활에서 심리적으로 매우 중요하다는 점을 느낄 수 있었습니다</v>
+        <v>담당 과목 선생님들께서 상주하시면서 매주 학습 상담과 질의응답을 받아주셔서 정말 좋았습니다. 모르는 점이 있으면 바로 질의응답이 가능하다는 점이 수험생활에서 심리적으로 매우 중요하다는 점을 느낄 수 있었습니다</v>
       </c>
       <c r="F314" t="str">
         <v>질의응답을 바로바로 할 수 있다는 점이 좋았습니다. 어찌보면 당연한 것이겠지만 수험생활에서 질의응답이 대면으로 가능하다는 것은 매우 큰 힘이 됐습니다 그렇기에 질의응답이 가장 좋았던거 같습니다</v>
@@ -11772,7 +11772,7 @@
         <v>잘 이끌어주셔서 감사합니다 덕분에 좋은 결과가 있었던구 같습니다 힘든 수험생활에도 불구하고 견딜 수 있었던 이유는 선생님들께서 열심히 독려해주시고 이끌어주셔서 그랬던거 같습니다 감사합니다</v>
       </c>
       <c r="J314" t="str">
-        <v>담당 과목 선생님들께서 상주하시면서 매주 학습상담과 질의응답을 받아주셔서 정말 좋았어요.</v>
+        <v>담당 과목 선생님들께서 상주하시면서 매주 학습 상담과 질의응답을 받아주셔서 정말 좋았어요.</v>
       </c>
       <c r="K314" t="str">
         <v>학습 관리, 질의응답</v>
@@ -11972,7 +11972,7 @@
         <v>이투스247을 다니기 전에는 혼자서 생활 관리가 안돼서 핸드폰을 하루종일 붙잡고 있었고 순공시간이 적었습니다. 생활 관리가 이투스를 통해 된 후부터 순공시간이 늘어났고 성적이 오르기 시작했습니다.</v>
       </c>
       <c r="F320" t="str">
-        <v>학습계획을 혼자서 공부할때는 세우지않고 그때그때 원하는대로 공부하다보니 진도가 잘 나가지 않고 하는 과목만 계속하는 문제가 있었습니다. 플래너를 통해 각 과목별로 시간을 정해서 하다보니 모든과목의 성적을 올릴수 있어서 좋았습니다</v>
+        <v>학습 계획을 혼자서 공부할때는 세우지않고 그때그때 원하는대로 공부하다보니 진도가 잘 나가지 않고 하는 과목만 계속하는 문제가 있었습니다. 플래너를 통해 각 과목별로 시간을 정해서 하다보니 모든과목의 성적을 올릴수 있어서 좋았습니다</v>
       </c>
       <c r="G320" t="str">
         <v>수험생의 가장 큰 적은 핸드폰이라고 생각합니다. 저도 혼자서 핸드폰때문에 공부에 많은 방해를 받았는데요, 이투스에서 공부를 시작한 이후로 휴대폰 없이 하루에 14시간씩 있다보니 자동으로 공부하는 시간이 많아져서 성적이 많이 올랐습니다</v>
@@ -12222,7 +12222,7 @@
         <v>이투스247의 생활상담 코칭 시스템은 그냥 공부만 시키는 방식이 아니라, 학생 생활 전체를 같이 본다는 점에서 확실히 도움됐다. 수험생활은 계획만 세운다고 굴러가는 게 아니라 수면, 식사, 멘탈, 루틴이 다 연결돼 있어서 한 부분만 무너지면 하루가 쉽게 흔들리는데, 이걸 혼자 계속 잡기는 생각보다 어렵다. 그럴 때 현재 상태를 같이 점검해주고 흐트러진 부분을 바로바로 정리해주는 게 꽤 컸다. 막연하게 불안해하기보다 왜 공부가 안 되는지 원인을 빨리 찾게 되고, 생활 패턴도 조금씩 안정되면서 결국 공부 효율까지 같이 올라가는 느낌이었다. 혼자 버티는 수험생활보다 훨씬 덜 막막하게 만들어주는 시스템이라고 생각한다.</v>
       </c>
       <c r="F327" t="str">
-        <v>이투스247에서 학습계획이랑 플래너 관리가 유용했던 건, 그냥 “공부해라”가 아니라 뭘 얼마나 어떻게 해야 하는지를 계속 보이게 만들어준다는 점이었다. 혼자 계획 짜면 욕심만 앞서서 비현실적으로 세우거나, 밀리면 아예 손 놓게 되는 경우가 많은데 여기서는 현재 수준이랑 해야 할 양을 기준으로 좀 더 현실적으로 흐름을 잡아주는 느낌이 있었다. 플래너도 단순 기록용이 아니라 내가 하루를 제대로 쓰고 있는지 확인하게 해줘서 좋았다. 계획 세우고 끝이 아니라 실제로 했는지, 어디서 막혔는지까지 보이니까 흐트러져도 다시 복구하기가 훨씬 쉬웠고, 공부를 막연하게 하는 시간이 줄어드는 게 꽤 크게 느껴졌다.</v>
+        <v>이투스247에서 학습 계획이랑 플래너 관리가 유용했던 건, 그냥 “공부해라”가 아니라 뭘 얼마나 어떻게 해야 하는지를 계속 보이게 만들어준다는 점이었다. 혼자 계획 짜면 욕심만 앞서서 비현실적으로 세우거나, 밀리면 아예 손 놓게 되는 경우가 많은데 여기서는 현재 수준이랑 해야 할 양을 기준으로 좀 더 현실적으로 흐름을 잡아주는 느낌이 있었다. 플래너도 단순 기록용이 아니라 내가 하루를 제대로 쓰고 있는지 확인하게 해줘서 좋았다. 계획 세우고 끝이 아니라 실제로 했는지, 어디서 막혔는지까지 보이니까 흐트러져도 다시 복구하기가 훨씬 쉬웠고, 공부를 막연하게 하는 시간이 줄어드는 게 꽤 크게 느껴졌다.</v>
       </c>
       <c r="G327" t="str">
         <v>이투스247의 면학 분위기 감독은 단순히 조용한 독서실 분위기를 만든다는 의미보다, 학생이 공부 외의 데에 에너지를 빼앗기지 않게 해준다는 점에서 유용했다. 수험생활을 하다 보면 은근히 주변 소음, 자리 분위기, 흐트러진 생활 태도 같은 사소한 요소들이 집중력에 크게 영향을 주는데, 이런 부분이 꾸준히 관리되니까 공부 흐름이 덜 끊겼다. 혼자였다면 한 번쯤은 느슨해졌을 순간에도 자연스럽게 다시 책상에 앉게 되는 분위기가 있었고, 결국 의지에만 기대지 않고 공부할 수 있는 환경이 유지된다는 점이 꽤 크게 느껴졌다.</v>
@@ -12360,7 +12360,7 @@
       </c>
       <c r="E331" t="str" xml:space="preserve">
         <v xml:space="preserve">입시 시스템과 입시 체계에 대해서 잘 모르는 저에게 선생님과의 일대일 상담은 유익한 도움이 되었습니다. 대학입시를 위해 어떤 목표를 잡아야 하고 어느정도의 성적을 만들어야 특정대학에 들어갈수 있는지 알 수 있었습니다. 이러한 상담 시스템에 도움을 입어 논술 전략이나 성적 전략을 구체적으로 계획할 수 있어서 좋았습니다._x000d_
-또한 입시상담은 입시관련 논술학원이나 인강또한 많이 추천해주셨기 때문에,제가 듣고 있었던 강의에 국한되지 않고 많은 강의들을 들어보면서 제 수준을 파악할 수 있었습니다. 분당 정자학원의 입시상담은 꼼꼼하였기 때문에 제 학습계획에 구체적으로 도움이 되었던 것 같습니다.</v>
+또한 입시상담은 입시관련 논술학원이나 인강또한 많이 추천해주셨기 때문에,제가 듣고 있었던 강의에 국한되지 않고 많은 강의들을 들어보면서 제 수준을 파악할 수 있었습니다. 분당 정자학원의 입시상담은 꼼꼼하였기 때문에 제 학습 계획에 구체적으로 도움이 되었던 것 같습니다.</v>
       </c>
       <c r="F331" t="str">
         <v>학생 스스로의 시간으로는 강사 한명 한명을 다 자세히 알지 못하는데, 선생님의 도움을 받으니 제 학습 스타일과 딱 맞는 인강 강사를 추천받을 수 있어서 좋았습니다. 또한 학원 추천 또한 많이 받았는데, 이러한 추천으로 인해 제가 부족했던 성적 부분 들을 잘 채워나갈 수 있었던 것 같습니다. 전략적으로 부실한 부분도 많아서 하마터면 비효율적인 강의를 선택할 수도 있었는데, 일대일 추천을 통해 제게 맞는 학습 스타일을 잘 찾아갈 수 있었습니다. 따라서 제 입시 생활에 도움이 되었다고 생각하고, 유용하다고 생각합니다.</v>
@@ -12399,7 +12399,7 @@
         <v>N수생</v>
       </c>
       <c r="E332" t="str">
-        <v>공부를 늦게 시작한 학생으로서 수능 커리큘럼과 공부법에 전혀 정보와 감이 없을때 여러해의 입시경험과 국영수 전공자 선생님들께서 주기적으로 학습계획을 세우는데 도와주었으며 지속적인 진도 체크와 성적 향상을 바탕으로 유기적이고 나에게 맞춤으로 코칭해주셨던 것이 수능을 독학으로 공부하는데 큰 도움이 되었다.</v>
+        <v>공부를 늦게 시작한 학생으로서 수능 커리큘럼과 공부법에 전혀 정보와 감이 없을때 여러해의 입시경험과 국영수 전공자 선생님들께서 주기적으로 학습 계획을 세우는데 도와주었으며 지속적인 진도 체크와 성적 향상을 바탕으로 유기적이고 나에게 맞춤으로 코칭해주셨던 것이 수능을 독학으로 공부하는데 큰 도움이 되었다.</v>
       </c>
       <c r="F332" t="str">
         <v>일반 독서실이나 관리형 독서실들과는 다르게 핵심과목인 국어,영어,수학 전공자 선생님들께서 상주하고 계셔서 문제를 풀다가 막힘이 오거나 특정과목에 대한 상담이 필요할때 즉각적인 질의응답을 통한 학습이 가능하다는 점이 가장 큰 장점이였다. 온라인 강의와 사이트를 이용하다보면 강의와 개념, 문제들에 대한 질문을 qna 게시판을 통해서만 질문이 가능한데 이는 시간도 오래걸리고 대면으로 질문하는것이 아니기에 한계가 존재했었다. 또한 이투스 247 목동 졸업생들이 멘토로 근무를 하여 특정 탐구 과목들에 대한 피드백과 질문, 조언들을 얻을 수 있다는 점에서 이투스 247 목동만의 독보적이고 차별적인 시스템이다.</v>
@@ -12714,7 +12714,7 @@
         <v>반수생</v>
       </c>
       <c r="E341" t="str">
-        <v>매주 학습계획표를 짜서 학습 하는 과정이 수월했습니다. 계획을 짜는 과정에서 부족한 부분과 필요하지 않은 학습에 대해 인지하는 시간을 가질 수 있었습니다. 또한 수준에 맞는 교재와 실모를 추천 받을 수 있어서 좋았습니다.</v>
+        <v>매주 학습 계획표를 짜서 학습 하는 과정이 수월했습니다. 계획을 짜는 과정에서 부족한 부분과 필요하지 않은 학습에 대해 인지하는 시간을 가질 수 있었습니다. 또한 수준에 맞는 교재와 실모를 추천 받을 수 있어서 좋았습니다.</v>
       </c>
       <c r="F341" t="str">
         <v>본인 수준에 맞는 인강과 교재를 통해 무리하지 않은 학습을 할 수 있었습니다. 그덕에 문풀 실력과 성적이 한단계씩 오르는 경험을 하였습니다. 학업 성취를 느끼는 기회가 되었습니다.</v>
@@ -12729,7 +12729,7 @@
         <v>얼마 안되는 기간동안 좌절에 빠지는 시간도 종종 있었는데 닦달않고 북돋아주셔서 감사했습니다. 덕분에 반수기간 동안 학습적인 부분을 제외하고도 심리적으로도 도움을 많이 받았습니다. 감사인사를 전할 기회가 이렇게 생겨서 다행입니다.</v>
       </c>
       <c r="J341" t="str">
-        <v>매주 학습계획표를 짜서 학습 하는 과정이 수월했어요.</v>
+        <v>매주 학습 계획표를 짜서 학습 하는 과정이 수월했어요.</v>
       </c>
       <c r="K341" t="str">
         <v>학습 계획</v>
@@ -12820,7 +12820,7 @@
         <v>N수생</v>
       </c>
       <c r="E344" t="str" xml:space="preserve">
-        <v xml:space="preserve">독학재수를 선택하며 학습계획 설정에 대한 걱정이 많았는데요, 코칭 시스템을 통해 단기부터 수능까지의 장기 목표를 체계적으로 설정할 수 있었고, 1:1 상담을 통해 나에게 맞는 학습 방법과 교재, 인강을 추천받아 효율적인 공부법을 확립할 수 있었습니다. 또한 모의고사 이후 성적을 세부적으로 분석하고 보완 전략을 함께 세우며, 더욱 체계적이고 확실한 학습을 이어갈 수 있었습니다._x000d_
+        <v xml:space="preserve">독학재수를 선택하며 학습 계획 설정에 대한 걱정이 많았는데요, 코칭 시스템을 통해 단기부터 수능까지의 장기 목표를 체계적으로 설정할 수 있었고, 1:1 상담을 통해 나에게 맞는 학습 방법과 교재, 인강을 추천받아 효율적인 공부법을 확립할 수 있었습니다. 또한 모의고사 이후 성적을 세부적으로 분석하고 보완 전략을 함께 세우며, 더욱 체계적이고 확실한 학습을 이어갈 수 있었습니다._x000d_
 더불어 선생님께서 항상 상주하시며 저의 공부 과정을 지켜봐 주셨기 때문에, 1년간의 학습 패턴과 습관을 반영한 꼼꼼한 개인 학습 관리를 받을 수 있었습니다. 공부 중 막히는 부분이 있을 때마다 친절하게 함께 해결해 주셔서 부담 없이 도움을 요청할 수 있었던 점도 큰 도움이 되었습니다.</v>
       </c>
       <c r="F344" t="str" xml:space="preserve">
@@ -13085,7 +13085,7 @@
         <v>N수생</v>
       </c>
       <c r="E351" t="str">
-        <v>정기적인 학습상담을 통해 제 공부 상태를 객관적으로 점검할 수 있었고, 그에 맞는 방향을 제시받은 점이 가장 유용했습니다. 스스로는 잘 보지 못했던 문제점들을 짚어주셔서 공부 습관을 개선하는 데 큰 도움이 되었습니다.</v>
+        <v>정기적인 학습 상담을 통해 제 공부 상태를 객관적으로 점검할 수 있었고, 그에 맞는 방향을 제시받은 점이 가장 유용했습니다. 스스로는 잘 보지 못했던 문제점들을 짚어주셔서 공부 습관을 개선하는 데 큰 도움이 되었습니다.</v>
       </c>
       <c r="F351" t="str">
         <v>학습 계획과 플래너 관리를 통해 하루 공부량과 시간 분배를 체계적으로 정리할 수 있었던 점이 가장 유용했습니다. 계획을 세우고 점검하는 과정에서 스스로의 부족한 부분을 파악할 수 있었고, 꾸준한 관리 덕분에 공부 습관을 안정적으로 유지하는 데 큰 도움이 되었습니다.</v>
@@ -13238,7 +13238,7 @@
         <v>개인적으로 몸이 좋지 않았는데 이를 배려를 정말 많이 해주셔서 에어컨 세기도 약하게 조절해주시고 룸메이트도 최대한 저랑 맞는 사람이랑 쓸 수 있도록 도와주셨습니다. 또한 교무실에 상비약이 배치되어 있어 가벼운 감기는 상비약을 먹으면서 회복하고 심한 감기일 때는 밖에 있는 병원에 갈 수 있어서 좋았습니다</v>
       </c>
       <c r="F355" t="str" xml:space="preserve">
-        <v xml:space="preserve">평소 의욕만 앞서 무리하게 계획을 세우거나, 기분에 따라 학습량이 들쑥날쑥해지는 편이었습니다. 하지만 학원에서 제공하는 학습계획 플래너 관리를 받으면서 공부의 질이 완전히 달라졌습니다._x000d_
+        <v xml:space="preserve">평소 의욕만 앞서 무리하게 계획을 세우거나, 기분에 따라 학습량이 들쑥날쑥해지는 편이었습니다. 하지만 학원에서 제공하는 학습 계획 플래너 관리를 받으면서 공부의 질이 완전히 달라졌습니다._x000d_
 ​가장 좋았던 점은 단순히 할 일을 나열하는 것이 아니라, 과목별 균형을 맞추고 실현 가능한 구체적인 목표를 설정하도록 세심하게 지도해 주신 점입니다.  혼자였다면 금방 포기했을 슬럼프 시기에도 정해진 루틴을 지키며 흔들림 없이 공부를 이어갈 수 있었습니다.</v>
       </c>
       <c r="G355" t="str" xml:space="preserve">
@@ -13253,7 +13253,7 @@
         <v>담임 선생님, 실장 선생님 , 사감선생님, 영양사선생님 등등 전부 감사인사를 드립니다. 덕분에 수험생활을 잘 마칠 수 있었습니다. 항상 하는 일마다 행운이 깃들기를 기원하겠습니다!</v>
       </c>
       <c r="J355" t="str">
-        <v>학원에서 제공하는 학습계획 플래너 관리를 받으면서 공부의 질이 완전히 달라졌었어요.</v>
+        <v>학원에서 제공하는 학습 계획 플래너 관리를 받으면서 공부의 질이 완전히 달라졌었어요.</v>
       </c>
       <c r="K355" t="str">
         <v>학습 계획, 플래너 관리</v>
@@ -13311,7 +13311,7 @@
         <v>긴 n수생활로 생활루틴을 어떻게잡을지도 지쳐있고 매번 정해지지않은 상태로 그날그날에 끌리는 과목만 공부하는정도였는데 이투스247에서 담임선생님과의 일주일에 한번씩 생활루틴을 상담받으면서 점차 제 루틴이 정립되었고 그게쌓이면서 수능때 좋은성적을 받게되었던것같습니다</v>
       </c>
       <c r="F357" t="str">
-        <v>항상 과목시간도 정해놓지않고 끌리는대로만 공부를 하던상황이라 제가 인지하지도 못한 채 성적이 잘나오는 과목만 더 열심히 하게되고, 잘 안나오는 과목은 후순위로 두는 실수를 두게되었는데 담임선생님이 제가 쓴 학습계획서를 꼼꼼히 봐주면서 지금 제가 어느과목을 회피하고있는지 명확히 알려주시고 해야한다에 그치지않고 그 과목이 부족한이유와 그 수준에맞는 새로운 공부법과 문제집을 계속 추천해주시면서 부족한과목을 놓지않게하여 결국 수능날 전체과목의 평균이 높은상태로 마무리되어 평균자체가 높아 유리한 교대에 합격하게된것같습니다</v>
+        <v>항상 과목시간도 정해놓지않고 끌리는대로만 공부를 하던상황이라 제가 인지하지도 못한 채 성적이 잘나오는 과목만 더 열심히 하게되고, 잘 안나오는 과목은 후순위로 두는 실수를 두게되었는데 담임선생님이 제가 쓴 학습 계획서를 꼼꼼히 봐주면서 지금 제가 어느과목을 회피하고있는지 명확히 알려주시고 해야한다에 그치지않고 그 과목이 부족한이유와 그 수준에맞는 새로운 공부법과 문제집을 계속 추천해주시면서 부족한과목을 놓지않게하여 결국 수능날 전체과목의 평균이 높은상태로 마무리되어 평균자체가 높아 유리한 교대에 합격하게된것같습니다</v>
       </c>
       <c r="G357" t="str">
         <v>아무래도 태블릿과 핸드폰이 수험생활에서 제일 큰 방해요인이 아닐까라고 생각이 드는데, 이투스247김포점은 말로만 태블릿과 핸드폰을 하지말라고만 하는게 아니라 방화벽까지 꼼꼼하게 막아두고 재원학생들의 태블릿을 등록시켜놔서 딴짓을 하고있는지 계속 주의하면서 실제로 2분정도 딴짓을 하기위해 이 정도면 모르시겠지하고 인터넷을 들어갔는데 바로 감시중이던 선생님이 인터넷 접속을 원격으로 끊으셔서 오히려 딴짓할까 생각도 하지못하고 오히려 딴짓도 못하는데 공부라도 열심히해야겠다라는 마인드로 바로 바뀌었던것같습니다 그만큼 태블릿관리를 말로만하지않으시고 실제계속된감시와 주의로 학생들이 공부에만 집중할수있게 면학 분위기를 조성시킨게 정말 큰 도움이되었던것같습니다</v>
@@ -13451,7 +13451,7 @@
         <v>이투스247을 다니면서 좋았던 점은 담임선생님과의 학습 상담이었습니다. 독학이다 보니까 방향을 잡는 게 어려웠는데, 상담하면서 제 상태를 정확하게 알 수 있어서 도움이 되었습니다.  그냥 열심히 하라고만 하는 게 아니라, 제 성적과 공부 습관을 보고 현실적으로 할 수 있는 계획을 같이 짜주셔서 좋았습니다. 그래서 막막할 때마다 다시 방향을 잡는 데 도움이 되었습니다.  또 분위기도 부담스럽지 않아서 편하게 질문하거나 고민을 말할 수 있었고, 그때마다 바로 피드백을 받을 수 있어서 좋았습니다. 혼자 공부하는데도 혼자 하는 느낌이 덜해서 계속 유지하는 데 도움이 되었습니다. 전체적으로 상담 덕분에 공부 방향이 덜 흔들렸고, 관리받는 느낌이 있어서 만족했습니다. 혼자 수험생활을 보내는 것에 부담이 있다면 이투스 247이 좋은 선택일 것 같습니다.</v>
       </c>
       <c r="F361" t="str">
-        <v>이투스247의 학습계획이랑 플래너 관리도 도움이 많이 됐습니다. 혼자 하면 계획을 세워도 잘 안 지키게 되는 경우가 많은데, 여기서는 계속 체크를 받으니까 더 신경 쓰게 됐습니다. 처음에 계획을 세울 때도 무리하게 잡는 게 아니라, 실제로 지킬 수 있는 수준으로 맞춰서 짜주셔서 현실적으로 공부할 수 있었습니다. 그래서 중간에 포기하는 일이 줄어든 것 같습니다. 플래너도 그냥 쓰고 끝나는 게 아니라, 매일 점검을 받으니까 제가 얼마나 했는지 바로 확인할 수 있어서 좋았습니다. 계획 대비 얼마나 했는지도 보이니까 스스로 반성도 하게 되고, 다음 날 계획 세우는 데도 도움이 됐습니다. 전체적으로 계획 세우고 실행하는 흐름이 잡혀서, 혼자 공부할 때보다 훨씬 안정적으로 공부할 수 있었습니다. 무엇보다 플래너를 쓰고나서 끝인 게 아니고, 선생님께 확인 받아야한다는 생각에 더욱 잘 지킬 수 있었습니다.</v>
+        <v>이투스247의 학습 계획이랑 플래너 관리도 도움이 많이 됐습니다. 혼자 하면 계획을 세워도 잘 안 지키게 되는 경우가 많은데, 여기서는 계속 체크를 받으니까 더 신경 쓰게 됐습니다. 처음에 계획을 세울 때도 무리하게 잡는 게 아니라, 실제로 지킬 수 있는 수준으로 맞춰서 짜주셔서 현실적으로 공부할 수 있었습니다. 그래서 중간에 포기하는 일이 줄어든 것 같습니다. 플래너도 그냥 쓰고 끝나는 게 아니라, 매일 점검을 받으니까 제가 얼마나 했는지 바로 확인할 수 있어서 좋았습니다. 계획 대비 얼마나 했는지도 보이니까 스스로 반성도 하게 되고, 다음 날 계획 세우는 데도 도움이 됐습니다. 전체적으로 계획 세우고 실행하는 흐름이 잡혀서, 혼자 공부할 때보다 훨씬 안정적으로 공부할 수 있었습니다. 무엇보다 플래너를 쓰고나서 끝인 게 아니고, 선생님께 확인 받아야한다는 생각에 더욱 잘 지킬 수 있었습니다.</v>
       </c>
       <c r="G361" t="str">
         <v>평소에 핸드폰을 많이 보는 편이어서 공부하다가도 자꾸 확인하게 되고 집중이 끊기는 경우가 많았는데, 수거되니까 아예 볼 수 없어서 그런 상황이 줄어들었습니다. 자연스럽게 핸드폰 쓰던 시간이 공부 시간으로 넘어가게 돼서 시간 활용 면에서도 도움이 많이 됐습니다.  또 중간에 알림이나 SNS 때문에 흐름이 끊기지 않으니까 한 번 집중하면 더 오래 유지할 수 있었고, 공부 효율도 올라간 느낌이었습니다. 처음에는 조금 불편하다고 느꼈지만, 오히려 이런 환경이 있어서 공부에 더 몰입할 수 있었던 것 같습니다.  전체적으로 핸드폰 사용을 강제로라도 줄여주는 환경이 만들어져서 스스로 통제하기 어려운 부분을 잡아줬고, 그 덕분에 공부 시간과 집중도가 같이 올라간 점에서 만족스러웠습니다.</v>
@@ -13463,7 +13463,7 @@
         <v>데스크 선생님과 담임 선생님 모두 항상 웃는 얼굴로 대해주셔서 좋았습니다. 학원에 갈 때마다 밝게 인사해주시고 친절하게 대해주셔서 수험생활 중에 작은 부분이지만 힘이 많이 됐습니다. 혼자 공부하다 보면 지치거나 기분이 다운될 때가 많은데, 그런 분위기 덕분에 조금이나마 편하게 다닐 수 있었던 것 같습니다.  또 중간에 성적이 잘 안 나오거나 공부가 잘 안 풀려서 낙담할 때도 있었는데, 그럴 때마다 항상 응원해주시고 괜찮다고 말해주셔서 다시 마음 잡는 데 도움이 됐습니다. 단순한 관리만 하는 게 아니라 학생 입장에서 이해해주시고 말해주시는 느낌이 들어서 더 의지가 됐습니다.  전체적으로 공부 환경뿐만 아니라 사람적인 부분에서도 도움을 많이 받았고, 그런 점들이 수험생활을 버티는 데 큰 힘이 됐다고 생각합니다.</v>
       </c>
       <c r="J361" t="str">
-        <v>이투스247학원의 학습계획이랑 플래너 관리도 도움이 많이 됐어요.</v>
+        <v>이투스247학원의 학습 계획이랑 플래너 관리도 도움이 많이 됐어요.</v>
       </c>
       <c r="K361" t="str">
         <v>학습 계획, 플래너 관리</v>
@@ -13598,7 +13598,7 @@
         <v>휴대폰과 전자기기와의 차단을 통해서 오로지 잡생각 안 하고 학습에만 집중할 수 있어서 단기간에 성적향상도 이루고 멘탈관리도 되어서 전자기기 사용금지 시스템이 유용하다고 생각을 했습니다</v>
       </c>
       <c r="H364" t="str">
-        <v>학원 내 모의고사를 봄으로써 내가 아는 것과 모르는 것 어중간하게 아는 것을 구분을 할 수 있어서 추후 학습계획을 세우고 오답정리를 할 때 취약점을 빠르게 보완하고 성적향상을 이룰 수 있게 해줘서 원내 모의고사가 좋았습니다</v>
+        <v>학원 내 모의고사를 봄으로써 내가 아는 것과 모르는 것 어중간하게 아는 것을 구분을 할 수 있어서 추후 학습 계획을 세우고 오답정리를 할 때 취약점을 빠르게 보완하고 성적향상을 이룰 수 있게 해줘서 원내 모의고사가 좋았습니다</v>
       </c>
       <c r="I364" t="str" xml:space="preserve">
         <v xml:space="preserve">2월부터 11월까지 잘 지도해주셔서 감사합니다 전역 후에 입시하느라 되게 막막하고 불안하고 했었는데 여기서 빡세게 공부해서 숭실대 잘 다니고 있어요_x000d_

</xml_diff>

<commit_message>
Apply batch spacing and typo corrections
</commit_message>
<xml_diff>
--- a/reviews_with_keywords.xlsx
+++ b/reviews_with_keywords.xlsx
@@ -580,10 +580,10 @@
         <v>현역때에는 학교에서 보는 교육청과 전국연합 평가원 모의고사가 전부였는데 이투스 전용 모의사를 통해서 새로운 유형의 문제들을 접해보면서 새로운 문제에 대한 두려움이 사라지고 모의고사에 적응이 되면서 수능날에 긴장감이 줄어들었던 것 같습니다.</v>
       </c>
       <c r="I5" t="str">
-        <v>원장선생님과 출결관리를 해주셨던 선생님 그리고 플레너 관리를 해주셨던 선생님 정말 감사합니다!!!!!항상 건강하실 바라겠습니다!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!</v>
+        <v>원장 선생님과 출결 관리를 해주셨던 선생님 그리고 플레너 관리를 해주셨던 선생님 정말 감사합니다!!!!!항상 건강하실 바라겠습니다!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!</v>
       </c>
       <c r="J5" t="str">
-        <v>원장선생님과 출결관리를 해주셨던 선생님 그리고 플레너 관리를 해주셨던 선생님 정말 감사했어요.</v>
+        <v>원장 선생님과 출결 관리를 해주셨던 선생님 그리고 플레너 관리를 해주셨던 선생님 정말 감사했어요.</v>
       </c>
       <c r="K5" t="str">
         <v/>
@@ -603,13 +603,13 @@
         <v>N수생</v>
       </c>
       <c r="E6" t="str">
-        <v>재수하면서 멘탈이 흔들릴때가 많았는데 그때마다 상담하면서 중심을 잡을 수 있었던것 같습니다. 그리고 담당선생님이 열심히 쪼아주셔서 나태해질때마다 다시 정신 붙잡고 공부할수 있었고 후반에는 공부를 어떻게 해야되는지 안 것 같은 느낌이었습니다</v>
+        <v>재수하면서 멘탈이 흔들릴때가 많았는데 그때마다 상담하면서 중심을 잡을 수 있었던것 같습니다. 그리고 담당 선생님이 열심히 쪼아주셔서 나태해질때마다 다시 정신 붙잡고 공부할 수 있었고 후반에는 공부를 어떻게 해야되는지 안 것 같은 느낌이었습니다</v>
       </c>
       <c r="F6" t="str">
         <v>앞서 말한것과 비슷하게 개인적인 성향이 혼자둬도 공부 엔간히 하지만 옆에 두고 관리해주실때 공부 효율이 더 나는 사람이라 플래너라든지 공부 방향 관리해주신게 좋았습니다! 효율적으로 공부하게 되는 느낌이었어여</v>
       </c>
       <c r="G6" t="str">
-        <v>다른건 막 좋지는 않았는데 그냥 그랬어여 그나마 나은게 출결이었음. 그냥 빨리 일어나니까 생활습관 잡히고 아침에 뇌가 깨어 있는 느낌? 좋았습니다. 근데 다른건 개선 할게 좀 있어여</v>
+        <v>다른건 막 좋지는 않았는데 그냥 그랬어여 그나마 나은게 출결이었음. 그냥 빨리 일어나니까 생활 습관 잡히고 아침에 뇌가 깨어 있는 느낌? 좋았습니다. 근데 다른건 개선 할게 좀 있어여</v>
       </c>
       <c r="H6" t="str">
         <v>무제한으로 볼 수 있었다는게 제일 큰 장점이었구여 다른거는 제가 활용을 잘 안해서 그런지 장단점을 잘 모르겠어여 근데 이투스 모의고사 국어는 진짜 좋았음 다른 사설 시험지 보다 더 평가원스러운게 적응하기 좋았어여 다른 과목은 몰라도 국어는 인정!!</v>
@@ -618,7 +618,7 @@
         <v>쌤 덕분에 대학 갔어여 솔직히 수능은 좀 큰일났긴했지만..;;논술로 붙었으면 된거 아니겠습니까 학원 한번 놀러갈게여!! 근데 반수 또 할거라 어쩌면 다시 볼 수 있을지도..??앙💕 제가 밥 사겠습니다! 저 요즘 알바해여</v>
       </c>
       <c r="J6" t="str">
-        <v>출결에 신경쓰면서 아침에 빨리 일어나니까 생활습관이 잡히고 아침에 뇌가 깨어 있는 느낌이었어요.</v>
+        <v>출결에 신경 쓰면서 아침에 빨리 일어나니까 생활 습관이 잡히고 아침에 뇌가 깨어 있는 느낌이었어요.</v>
       </c>
       <c r="K6" t="str">
         <v/>
@@ -778,7 +778,7 @@
         <v>N수생</v>
       </c>
       <c r="E11" t="str">
-        <v>문제집을 풀면서 모르는 문제가 있을때 매번 답지만 보며 시간을 많이 썼는데 학습 상담을 통해서 시간을 효율적으로 쓸  수 있었고 이해하는데도 도움이 많이 되었습니다. 그리고 공부 커리큘럼을 어떻게 짜야할지 몰랐는데 학습 상담을 통해서 어떻게 공부해야할지 감을 잡고 공부할 수 있었습니다.</v>
+        <v>문제집을 풀면서 모르는 문제가 있을때 매번 답지만 보며 시간을 많이 썼는데 학습 상담을 통해서 시간을 효율적으로 쓸  수 있었고 이해하는데도 도움이 많이 되었습니다. 그리고 공부 커리큘럼을 어떻게 짜야할지 몰랐는데 학습 상담을 통해서 어떻게 공부해야 할지 감을 잡고 공부할 수 있었습니다.</v>
       </c>
       <c r="F11" t="str">
         <v>보통 문제집을 풀면 강의가 없어 답지를 보고 문제를 혼자 이해했어야하는데 1:1로 질의 응답을 해주셔서 이해하는데 도움이 많이 되었습니다. 제가 모르는 부분을 더 집중적으로 자세하게 설명을 들을 수 있었고 못하는 부분을 보완하기 위해 무엇을 공부 해야하는지도 알 수 있어 좋았습니다.</v>
@@ -790,10 +790,10 @@
         <v>공부하는데 제일 중요한것은 감을 잃지 않는 것인데 모의고사를 통해서 수능을 볼때의 감을 잃지 않을 수 있었고 지금 제가 어느정도의 실력을 갖고 있는지 정검할 수 있어서 더 부족하다고 생각하는 과목의 공부를 하는데 도움이 되었습니다.</v>
       </c>
       <c r="I11" t="str">
-        <v>이투스247에 다니는 동안 상담과 출결 관리까지 꼼꼼히 신경 써주셔서 감사합니다. 공부하기 좋은 환경과 힘들게 공부할 때 많이 챙겨 주셔서 재수생활을 버티는데 도움이 많이 되었습니다. 선생님들의 덕분에 공부에 도움이 많이 되었고, 좋은 결과로 이어질 수 있었습니다. 감사합니다</v>
+        <v>이투스247에 다니는 동안 상담과 출결 관리까지 꼼꼼히 신경 써주셔서 감사합니다. 공부하기 좋은 환경과 힘들게 공부할 때 많이 챙겨 주셔서 재수 생활을 버티는데 도움이 많이 되었습니다. 선생님들의 덕분에 공부에 도움이 많이 되었고, 좋은 결과로 이어질 수 있었습니다. 감사합니다</v>
       </c>
       <c r="J11" t="str">
-        <v>힘들게 공부할 때 많이 챙겨 주셔서 재수생활을 버티는데 도움이 많이 되었어요.</v>
+        <v>힘들게 공부할 때 많이 챙겨 주셔서 재수 생활을 버티는데 도움이 많이 되었어요.</v>
       </c>
       <c r="K11" t="str">
         <v/>
@@ -813,20 +813,20 @@
         <v>N수생</v>
       </c>
       <c r="E12" t="str" xml:space="preserve">
-        <v xml:space="preserve">이것 저것 다 해야할 것 같은 조급함에 이러지도 저러지도 못하고 있을때 담임선생님과의 학습 상담을 통해서 저와 맞는 학습 계획을 세우고 저만의 템포로 공부할 수 있어서 좋았습니다_x000d_
+        <v xml:space="preserve">이것 저것 다 해야 할 것 같은 조급함에 이러지도 저러지도 못하고 있을때 담임 선생님과의 학습 상담을 통해서 저와 맞는 학습 계획을 세우고 저만의 템포로 공부할 수 있어서 좋았습니다_x000d_
 또한, 저는 맞는 인강쌤을 찾기 힘들어 많이 왔다갔다 거리는 인강 유목민이었습니다. 인강이 없으면 안된다고 생각했는데 학습 상담을 통해 인강이 맞지 않는 과목의 경우여도 독학으로 좋은 성적을 받을 수 있음을 알게되었습니다. 머리가 복잡한 수험생을 옳은 길로 잘 이끌어주셨습니다</v>
       </c>
       <c r="F12" t="str">
-        <v>앞서 언급했듯 다양한 방면으로 공부법을 제시해주시고, 결정하게 해주셔서 좋았습니다. 사람마다 맞는 공부법이 다르기에 그것을 찾아 정착하는데에는 꽤 오랜 시간이 걸린다고 생각합니다. 이투스 담임선생님과의 꾸준한 소통과 학습 관리 시스템을 통해 시간낭비를 줄일 수 있었던 것 같습니다</v>
+        <v>앞서 언급했듯 다양한 방면으로 공부법을 제시해주시고, 결정하게 해주셔서 좋았습니다. 사람마다 맞는 공부법이 다르기에 그것을 찾아 정착하는데에는 꽤 오랜 시간이 걸린다고 생각합니다. 이투스 담임 선생님과의 꾸준한 소통과 학습 관리 시스템을 통해 시간낭비를 줄일 수 있었던 것 같습니다</v>
       </c>
       <c r="G12" t="str">
-        <v>사실 휴대폰과 태블릿의 유혹에 수험생이 가장 취약하다고 생각하는데요. 하지만 이런 유혹은 수험생활을 쉽게 망치기 일쑤입니다. 이투스 학원을 다니며 이러한 유혹에 견딜 수 있는데에 와이파이 방화벽이 큰 기여를 했다고 생각합니다</v>
+        <v>사실 휴대폰과 태블릿의 유혹에 수험생이 가장 취약하다고 생각하는데요. 하지만 이런 유혹은 수험 생활을 쉽게 망치기 일쑤입니다. 이투스 학원을 다니며 이러한 유혹에 견딜 수 있는데에 와이파이 방화벽이 큰 기여를 했다고 생각합니다</v>
       </c>
       <c r="H12" t="str">
         <v>저는 메가패스와 대성패스만 보유하고 있었는데요. 연계공부를 압축적으로 해야하는 상황이었는데 이투스 패스 덕분에 김민정쌤을 들을 수 있었습니다. 그때 들었던 작품들이 운이 좋게도 전부 수능에 나와 문학을 다 맞을 수 있었습니다!!</v>
       </c>
       <c r="I12" t="str">
-        <v>여러모로 학생만큼 고생하셨을텐데 길다면 긴, 짧다면 짧은 기간동안 감사했습니다! 선생님들의 격려와 응원, 도움이 없었다면 힘든 수험생활 진작에 무너졌을 것 같아요,, 제 수험생활에 함께해주셔서 감사합니다</v>
+        <v>여러모로 학생만큼 고생하셨을텐데 길다면 긴, 짧다면 짧은 기간동안 감사했습니다! 선생님들의 격려와 응원, 도움이 없었다면 힘든 수험 생활 진작에 무너졌을 것 같아요,, 제 수험 생활에 함께해주셔서 감사합니다</v>
       </c>
       <c r="J12" t="str">
         <v>수업이 없으면 안된다고 생각했는데 학습 상담을 통해 저에게 맞는 공부법을 알려주셔서 좋은 성적을 받을 수 있었어요.</v>
@@ -896,7 +896,7 @@
         <v>이투스 인강에서 국어, 사문 등 여러가지 강의를 보면서 도움이 되었던 거 같습니다. 다른 사이트에서 인강도 많이 봤지만 국어, 사문은 이투스 인강에서 더 도움을 많이 받은 거 같습니다.</v>
       </c>
       <c r="I14" t="str">
-        <v>1년동안 제가 공부에 온전히 집중 할 수 있고, 다른 것에 신경 팔리지 않게 도움을 주셔서 정말 감사했습니다. 그 외에도 제가 힘들면 상담을 해주시고 저에게 방향성을 제시해 주셔서 감사했습니다</v>
+        <v>1년 동안 제가 공부에 온전히 집중 할 수 있고, 다른 것에 신경 팔리지 않게 도움을 주셔서 정말 감사했습니다. 그 외에도 제가 힘들면 상담을 해주시고 저에게 방향성을 제시해 주셔서 감사했습니다</v>
       </c>
       <c r="J14" t="str">
         <v>제가 모의고사를 풀거나 공부를 하며 많은 스트레스를 받았을 때 담임 선생님께 상담을 받아 많은 도움이 되었던 거 같아요.</v>
@@ -919,10 +919,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E15" t="str">
-        <v>원장선생님께서 재원생 한명한명을 기억하시고, 마주치실때마다 공부잘되어가는지 여쭤봐주십니다. 또한 원장선생님, 부원장 선생님을 비롯한 선생님들께서 정말 언제든 시간을 내어 적극적으로 상담해주셔서 좋았어요</v>
+        <v>원장 선생님께서 재원생 한명한명을 기억하시고, 마주치실때마다 공부잘되어가는지 여쭤봐주십니다. 또한 원장 선생님, 부원장 선생님을 비롯한 선생님들께서 정말 언제든 시간을 내어 적극적으로 상담해주셔서 좋았어요</v>
       </c>
       <c r="F15" t="str">
-        <v>부원장선생님과 국어 상담을 몇 번 진행했는데, 타 인강 강사 선생님들의 세부적인 특징들을 모두 말해주시면서 저와 가장 잘 맞아보이는 선생님을 추천해주셨어요. 다른 학원 선생님들과도 많이 상담해봤지만 정말 친절하다는게 느껴질 정도였고, 아직도 감사한 기억으로 남습니다</v>
+        <v>부원장 선생님과 국어 상담을 몇 번 진행했는데, 타 인강 강사 선생님들의 세부적인 특징들을 모두 말해주시면서 저와 가장 잘 맞아보이는 선생님을 추천해주셨어요. 다른 학원 선생님들과도 많이 상담해봤지만 정말 친절하다는게 느껴질 정도였고, 아직도 감사한 기억으로 남습니다</v>
       </c>
       <c r="G15" t="str">
         <v>고3시절 아무리 공부를 해야한다는 압박감에도 불구하고 학습용 아이패드로 sns를 들어가보는게 습관이되었습니다. 하지만 이투스 방화벽시스템으로 아예 들어가는것 자체가 불가하니까sns생각이 안나서 너무 좋았어요</v>
@@ -931,10 +931,10 @@
         <v>매달 치르는 다양한 사설 모의고사들로 굳은살 배기듯이 익숙해져서 수능 당시는 정말 긴장을 안했어요 11월 모의고사를 치르는 심정으로 편하게 시험칠 수 있었어요! 다른 친구들에게 모의고사 시스템 하나는 정말 강력 추천하고싶어요</v>
       </c>
       <c r="I15" t="str">
-        <v>선생님 따로 연락은 제대로 못 드렸지만 언제나 학원에서 인사해주시고 공부잘되어가는지 힘든건 없는지 여쭤봐주셔서 감사했어요. 길고 긴 수험생활이었지만 이투스 덕분에 저에게 과분한 대학에 오게된 것 같아 아직도 감사합니다. ㅎㅎ</v>
+        <v>선생님 따로 연락은 제대로 못 드렸지만 언제나 학원에서 인사해주시고 공부잘되어가는지 힘든건 없는지 여쭤봐주셔서 감사했어요. 길고 긴 수험 생활이었지만 이투스 덕분에 저에게 과분한 대학에 오게된 것 같아 아직도 감사합니다. ㅎㅎ</v>
       </c>
       <c r="J15" t="str">
-        <v>원장선생님께서 재원생 한 명, 한 명을 기억하시고, 마주치실 때마다 공부는 잘 되는지 항상 체크해주셨어요.</v>
+        <v>원장 선생님께서 재원생 한 명, 한 명을 기억하시고, 마주치실 때마다 공부는 잘 되는지 항상 체크해주셨어요.</v>
       </c>
       <c r="K15" t="str">
         <v/>
@@ -954,13 +954,13 @@
         <v>N수생</v>
       </c>
       <c r="E16" t="str">
-        <v>수능 대비를 어떻게 시작해야하고 또 1년간의 로드맵을 어떻게 주체적으로 구성할지 모르는 학생들에게 강좌, 선택과목 등에 대한 방향성을 제시해줄 수 있습니다. 그리고 상담이 수시로 의무적으로 잡혀있어, 학습 현황과 실력 점검, 모의평가 및 수능준비 과정 등에 대해 꼼꼼한 피드백을 받을 수 있고, 더불어 멘탈과 수험생활 관련한 상담도 받을 수 있어 좋습니다. 수능을 준비하면서 마주칠 여러 중간 과정과 난관 그리고 좌절이 있을 수 있습니다. 그 부분을 잘 다스리는데 큰 도움을 받을 수 있을 것입니다.</v>
+        <v>수능 대비를 어떻게 시작해야하고 또 1년간의 로드맵을 어떻게 주체적으로 구성할지 모르는 학생들에게 강좌, 선택과목 등에 대한 방향성을 제시해줄 수 있습니다. 그리고 상담이 수시로 의무적으로 잡혀있어, 학습 현황과 실력 점검, 모의평가 및 수능준비 과정 등에 대해 꼼꼼한 피드백을 받을 수 있고, 더불어 멘탈과 수험 생활 관련한 상담도 받을 수 있어 좋습니다. 수능을 준비하면서 마주칠 여러 중간 과정과 난관 그리고 좌절이 있을 수 있습니다. 그 부분을 잘 다스리는데 큰 도움을 받을 수 있을 것입니다.</v>
       </c>
       <c r="F16" t="str">
-        <v>플래너는 결국 학생 개인의 공부 계획과 그 성취 여부를 잘 정리해놓은 자료입니다. 여기서 그 학생이 1년간 진행하고자 마음먹은 공부의 내용과 현황을 구체적으로 살필 수 있기에 이를 토대로 학습관리 상담을 하는 것이 결국 중요합니다. 해서 개인에게 맞춘 상담을 진행할 때 플래너를 중심으로 첨삭하고 피드백 받는 과정이 가장 뼈와 살이 된다고 생각하며, 그 과정에서 수강 강좌 및 성적(실력) 체크 그리고 전체적인 비전을 가져갈 수 있는 것이 좋았다고 봅니다.</v>
+        <v>플래너는 결국 학생 개인의 공부 계획과 그 성취 여부를 잘 정리해놓은 자료입니다. 여기서 그 학생이 1년간 진행하고자 마음먹은 공부의 내용과 현황을 구체적으로 살필 수 있기에 이를 토대로 학습 관리 상담을 하는 것이 결국 중요합니다. 해서 개인에게 맞춘 상담을 진행할 때 플래너를 중심으로 첨삭하고 피드백 받는 과정이 가장 뼈와 살이 된다고 생각하며, 그 과정에서 수강 강좌 및 성적(실력) 체크 그리고 전체적인 비전을 가져갈 수 있는 것이 좋았다고 봅니다.</v>
       </c>
       <c r="G16" t="str">
-        <v>결국 입시와 수험생활을 자기 욕구와의 싸움이자 절제가 핵심입니다. 혼자의 의지로는 정말 실천하기 어려운 부분이 다름아닌 미디어와 전자기기를 학습의 용도에 맞게 제대로 사용하고 인터넷과 SNS, 기타 엔터테인먼트 같은 방해 요소를 차단하여 자기주도적으로 몰입 (가능한 환경을 조성)하는 것입니다. 이런 면에서 외부의 콘텐츠 및 학습에 무관한 미디어들을 원천 차단해주는 학습 케어가 상당히 강력했다고 생각합니다. 휴대폰을 반납하는 것도 그렇지만 학습의 용도로 태블릿 같은 미디어 재생 기기의 힘을 빌리는 것이 불가피한데, 그 과정에서 수반되는 학습 방해요소라든지 이런 점을 잘 관리해준다고 생각합니다.</v>
+        <v>결국 입시와 수험 생활을 자기 욕구와의 싸움이자 절제가 핵심입니다. 혼자의 의지로는 정말 실천하기 어려운 부분이 다름아닌 미디어와 전자기기를 학습의 용도에 맞게 제대로 사용하고 인터넷과 SNS, 기타 엔터테인먼트 같은 방해 요소를 차단하여 자기주도적으로 몰입 (가능한 환경을 조성)하는 것입니다. 이런 면에서 외부의 콘텐츠 및 학습에 무관한 미디어들을 원천 차단해주는 학습 케어가 상당히 강력했다고 생각합니다. 휴대폰을 반납하는 것도 그렇지만 학습의 용도로 태블릿 같은 미디어 재생 기기의 힘을 빌리는 것이 불가피한데, 그 과정에서 수반되는 학습 방해요소라든지 이런 점을 잘 관리해준다고 생각합니다.</v>
       </c>
       <c r="H16" t="str">
         <v>VOCA 테스트는 일견 사소해보일 수 있으나, 사실 수능을 공부하면서 타 과목들에 치여 가장 경시하기 쉬우면서도 또 일일이 챙기기에는 골치아파 개인의 의지력이 많이 부족해지기 쉬운 부분입니다. 학원에서 매일 아침 루틴적으로 테스트를 실시해 자기도 모르는 사이 효과적으로 영어 기본기를 잘 잡아주는 면이 집에서 독학하는 것과 정말 큰 차이점 중 하나를 만들어낸다고 생각합니다.</v>
@@ -1024,7 +1024,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E18" t="str">
-        <v>클리닉 수업에서는 ”부족한 점 위주로 보완“ 하는 프로그램이 이루어진다고 느꼈습니다. 단순히 진도를 빼는 수업이 아니라, 학생이 뭐가 부족하고, 어떻게 보완해야할지를 제시해주셨습니다</v>
+        <v>클리닉 수업에서는 ”부족한 점 위주로 보완“ 하는 프로그램이 이루어진다고 느꼈습니다. 단순히 진도를 빼는 수업이 아니라, 학생이 뭐가 부족하고, 어떻게 보완해야 할지를 제시해주셨습니다</v>
       </c>
       <c r="F18" t="str">
         <v>스스로 해결하기 어려운 질문들을 1:1 질의응답을 통해 해결할 수 있었고, 과목별 공부법이나, 일일테스트 질문까지 가능하여 학습에 유용했습니다. 뿐만 아니라, 질문을 해결하고 어떤걸 추가로 학습하면 좋을지도 제시해주셔서 학습 방향을 올바르게 잡는데도 도움이 돠었습니다</v>
@@ -1106,7 +1106,7 @@
         <v>영어는 매일 꾸준히 안하면 감을 잃기 쉽다. 특히나 요즘 상대평가인 영어가 많이 어려워지고 있는 추세에 영단어 암기가 많이 중요해지고 있다. 또한 한번 단어 암기를 안하게 되면 계속 미루고 안하게 돼서 매일 꾸준히 영단어 테스트를 보고 검사받는 시스템이 마음에 들었다.</v>
       </c>
       <c r="I20" t="str">
-        <v>솔직히 모의고사 공부를 제대로 시작한게 고3때라 너무 막막했는데 같이 계획도 세워주시고 무엇보다 모르는것을 친절하게 알려주셔서 많은 도움이 되었습니다. 물론 수시로 대학에 갔지만 수능 공부하면서도 많은것을 얻을 수 있었어요! 내년에 한번 찾아뵐게요(이유는 그때가서 말씀드릴게요) 감사합니다!!</v>
+        <v>솔직히 모의고사 공부를 제대로 시작한게 고3 때라 너무 막막했는데 같이 계획도 세워주시고 무엇보다 모르는것을 친절하게 알려주셔서 많은 도움이 되었습니다. 물론 수시로 대학에 갔지만 수능 공부하면서도 많은것을 얻을 수 있었어요! 내년에 한번 찾아뵐게요(이유는 그때가서 말씀드릴게요) 감사합니다!!</v>
       </c>
       <c r="J20" t="str">
         <v>휴대폰을 제출하여 공부에 집중할 수 있었고, 뿐만 아니라 다른 생활 관리 시스템으로 관리를 해주셔서 공부에 집중할 수 있었어요.</v>
@@ -1135,7 +1135,7 @@
         <v>독학재수는 쉽지 않다. 이투스 등록 전까진 아무리 플래너를 그럴듯하게 써놔도 막상 달성률은 처참했다. 누군가 옆에서 잡아주고 감시해주는 사람이 없으니, 자기합리화를 계속 하며 미루고 미루다 결국 할 일이 엄청 불어났다. 그러나 학원에 오게 되면, 선생님들이 플래너를 매주 검사하신다. 현재 내가 모든 과목을 균형있게 골고루 공부하고 있는지, 계획이 너무 무리하진 않은지 플래너를 세세히 보시고 하나하나 피드백해 주신다. 덕분에 학원에 온 지 한 달만에 미루는 습관을 교정하게 될 수 있었다.</v>
       </c>
       <c r="G21" t="str" xml:space="preserve">
-        <v xml:space="preserve">나는 잠에 정말 약하다. 고3때 모의고사를 볼 때도 몽롱한 정신으로 풀었고, 아침잠이 너무 많은 탓에 결국 현역 수능 1교시 시작 직전까지 하품을 쩍쩍 하다 결국 처참한 국어 성적을 받았다. 학원에 온 이후로는 선생님들께서 졸음 관리를 해 주셔서 좋았다. 항상 공부를 할 땐 나도 모르는 사이 꾸벅꾸벅 졸곤 했었는데, 그럴 때 마다 감독 선생님들께서 안마봉으로 깨워주셨다._x000d_
+        <v xml:space="preserve">나는 잠에 정말 약하다. 고3 때 모의고사를 볼 때도 몽롱한 정신으로 풀었고, 아침잠이 너무 많은 탓에 결국 현역 수능 1교시 시작 직전까지 하품을 쩍쩍 하다 결국 처참한 국어 성적을 받았다. 학원에 온 이후로는 선생님들께서 졸음 관리를 해 주셔서 좋았다. 항상 공부를 할 땐 나도 모르는 사이 꾸벅꾸벅 졸곤 했었는데, 그럴 때 마다 감독 선생님들께서 안마봉으로 깨워주셨다._x000d_
 이 뿐만 아니라, 담임 선생님과의 상담을 통해 어떻게 하면 컨디션 조절을 잘 할 수 있을지에 대해 많은 이야기를 나누었다. 덕분에 재수때는 꽤 괜찮은 컨디션으로 수능을 쳤다.</v>
       </c>
       <c r="H21" t="str" xml:space="preserve">
@@ -1157,7 +1157,7 @@
 나름대로 이 과정에서 얻어가는게 많았고, 반수 전후로 제 마인드가 크게 변했다는 것을 요즘 체감하고 있습니다_x000d_
 _x000d_
 _x000d_
-사실 이투스에 처음 왔을때는 조금 걱정됐습니다. 고등학교 3학년 때는 담임선생님이랑 트러블이 엄청 심했었고, 그거 때문에 스트레스도 엄청 받았어요. 하지만 이투스 선생님들은 너무 친절하고 따뜻해서 좋았습니다..돌이켜 보면, 현역때는 학교 가기 싫다는 생각을 수도없이 했었는데,막상 반수를 할 때는 학원 가기 싫다는 생각은 거의 하지 않은 것 같아요_x000d_
+사실 이투스에 처음 왔을때는 조금 걱정됐습니다. 고등학교 3학년 때는 담임 선생님이랑 트러블이 엄청 심했었고, 그거 때문에 스트레스도 엄청 받았어요. 하지만 이투스 선생님들은 너무 친절하고 따뜻해서 좋았습니다..돌이켜 보면, 현역때는 학교 가기 싫다는 생각을 수도없이 했었는데,막상 반수를 할 때는 학원 가기 싫다는 생각은 거의 하지 않은 것 같아요_x000d_
 _x000d_
 옆에서 지켜봐주시고 코칭해주신 선생님들께 정말 감사하다는 말씀을 드리고 싶습니다.. 각박한 반수생활 속에서 따뜻한 선생님들 덕분에 힘든 시기를 잘 보낼 수 있었어요_x000d_
 _x000d_
@@ -1293,7 +1293,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E25" t="str">
-        <v>헉습에 집중할수있더록 멘탈관리를 잘해주셨습니다 주기적인 상담을 해주셨고 멘탈이 떨어질때 여러방법으로 상담을 주셔서 이갸낼수있었습니다 모의고사를 보고나면 과목별 학습 상담이 도움이 되었습니다</v>
+        <v>헉습에 집중할 수있더록 멘탈관리를 잘해주셨습니다 주기적인 상담을 해주셨고 멘탈이 떨어질때 여러방법으로 상담을 주셔서 이갸낼수있었습니다 모의고사를 보고나면 과목별 학습 상담이 도움이 되었습니다</v>
       </c>
       <c r="F25" t="str">
         <v>과목별 성적변화에 대한 상담이 도움이되었고 그에따른 과목별 시간배분과 교재선정및 학습 계획에 대해 도움을 받았습니다 어떤과목에 현재 더 시간을 쏟아야할지 가이드라인을 해주셨습니다 한과목에 치중하지않도록 시건배분에대한 계획에 도움을 받았습니다</v>
@@ -1328,7 +1328,7 @@
         <v>반수생</v>
       </c>
       <c r="E26" t="str">
-        <v>자기주도적인학습이 잘 되지 않는 사람들은 보통 어디서부터 시작해야할지 막막한데 이투스는 한 주마다 상담을하며  어떤 커리큘럼을 탈지, 어떤 부분이 부족한지에 대해 심도있게 대화하며 계획을 같이 짜게되니 아무런 계획이 없이 그냥 들어오기만 하면 이끌어주니까 공부에 집중할 수 있는 환경이 만들어집니다</v>
+        <v>자기주도적인학습이 잘 되지 않는 사람들은 보통 어디서부터 시작해야 할지 막막한데 이투스는 한 주마다 상담을하며  어떤 커리큘럼을 탈지, 어떤 부분이 부족한지에 대해 심도있게 대화하며 계획을 같이 짜게되니 아무런 계획이 없이 그냥 들어오기만 하면 이끌어주니까 공부에 집중할 수 있는 환경이 만들어집니다</v>
       </c>
       <c r="F26" t="str">
         <v>평소 현역시절 학원만 다녀 인강이나 교재에 대해 정보가 전무했는데 이투스 조교 선생님께서 과목별로 나의 수준에 맞는 교재와 문이과를 가리지 않고 다양한 인강 강사를 추천해 주셔서 평소 인강계에 대해 관심이 없었던 사람들까지 이 학원에 온다면 자기의 학습패턴에 맞는 커리큘럼을 탈 수 있습니다</v>
@@ -1340,10 +1340,10 @@
         <v>모의고사의 양이 절대적으로 중요한 학생들에게 이투스 모의고사라는 자체적인 컨텐츠를 제공하는 점이 좋았습니다. 또 그 컨텐츠가 단순히 기출을 짜깁기한 것이 아니라 새롭고 퀄리티 있는 시험지라는 점에서 너무나도 큰 도움이 되었습니다.</v>
       </c>
       <c r="I26" t="str">
-        <v>재학 기간 동안 많은 건강적인 문제가 있었는데 많은 편의를 봐주셔서 오랫동안 공부하며 꾸준히 노력할 수 있었습니다 감사합니다. 또 지칠때 응원해주시며 동기부여해주시는게 수험생활의 소소한 낙이었습니다. 감사드립니다</v>
+        <v>재학 기간 동안 많은 건강적인 문제가 있었는데 많은 편의를 봐주셔서 오랫동안 공부하며 꾸준히 노력할 수 있었습니다 감사합니다. 또 지칠 때 응원해주시며 동기부여해주시는게 수험 생활의 소소한 낙이었습니다. 감사드립니다</v>
       </c>
       <c r="J26" t="str">
-        <v>지칠때 응원해주시며 동기부여해주시는게 수험생활의 소소한 낙이었어요.</v>
+        <v>지칠 때 응원해주시며 동기부여해주시는게 수험 생활의 소소한 낙이었어요.</v>
       </c>
       <c r="K26" t="str">
         <v/>
@@ -1402,7 +1402,7 @@
 스트레스 없이 아이가 입시 공부에만 집중 할 수 있는 분위기 조성도 잘 해주신것 같습니다.</v>
       </c>
       <c r="F28" t="str">
-        <v>일대일 코칭 선생님께서 부족한 부분을 잘 파악 하시고 점수를 올리기 위해서 추가로 공부 해야할 부분들을 잘 코칭해 주셨고 실제로 성적 향상이 되었습니다 . 또한 따뜻한 격려의 말씀도 너무 감사하고 도움이 많이 되었습니다</v>
+        <v>일대일 코칭 선생님께서 부족한 부분을 잘 파악 하시고 점수를 올리기 위해서 추가로 공부 해야 할 부분들을 잘 코칭해 주셨고 실제로 성적 향상이 되었습니다 . 또한 따뜻한 격려의 말씀도 너무 감사하고 도움이 많이 되었습니다</v>
       </c>
       <c r="G28" t="str">
         <v>졸음이 올때면 엄마 마냥 깨워 주셔서 감사드립니다. 모든것이 예민한 시기인데 마음까지 잘 헤아려 주시는 원장님과 모든 선생님들께 너무 감사드립니다. 외출 관리도 너무 하나하나 잘 해 주셨습니다.</v>
@@ -1439,7 +1439,7 @@
         <v>성적이 낮은 과목이 있었는데 저에게 알맞은  강의를 추천해 주셔서 많이 도움이 되었습니다 모의고사 성적표가 나올때마다 어떤 과목 중심으로 공부해야 효율적일지 같이 고민하고 상담해주셔서 좋았습니다</v>
       </c>
       <c r="F29" t="str">
-        <v>매일 플래너를 쓰니까 계획적으로 학습을 할수 있어서 좋았습니다.  플래너를 쓰지 않았을때보다 더 체계적이고 효율적으로 공부할수 있었습니다. 매일 플래너를 쓰다보니 습관이 되어서 공부 계획을 잘 세우게되었습니다</v>
+        <v>매일 플래너를 쓰니까 계획적으로 학습을 할수 있어서 좋았습니다.  플래너를 쓰지 않았을때보다 더 체계적이고 효율적으로 공부할 수 있었습니다. 매일 플래너를 쓰다보니 습관이 되어서 공부 계획을 잘 세우게되었습니다</v>
       </c>
       <c r="G29" t="str">
         <v>혼자 공부하면 5분만 눈을 붙인다는 게 1시간이 되기 일쑤인데 선생님이 주기적으로 순회하며 즉각 깨워주니 흐름이 끊기지 않았습니다. 졸음이 확산되기 전에 차단해주는 강제성이 가장 큰 장점이었습니다</v>
@@ -1451,7 +1451,7 @@
         <v>선생님 1년정도의 기간동안 잘 코칭해주셔서 정말 감사했습니다ㅎㅎ 덕분에 수험기간 잘 버텨낼수 있었어용! 쌤덕분에 수능때 영어도 3등급 받아냈어요~~ 앞으로 행복하세요!! 독서도 열심히 할게요</v>
       </c>
       <c r="J29" t="str">
-        <v>플래너를 쓰지 않았을때보다 더 체계적이고 효율적으로 공부할수 있었어요.</v>
+        <v>플래너를 쓰지 않았을때보다 더 체계적이고 효율적으로 공부할 수 있었어요.</v>
       </c>
       <c r="K29" t="str">
         <v/>
@@ -1507,7 +1507,7 @@
         <v>N수생</v>
       </c>
       <c r="E31" t="str">
-        <v>일주일에 한 번씩 상담을 했는데 지금까지 얼마나 진도를 나갔는지 말씀드리고 하루에 이정도는 해야 진도를 다 끝낼수있고 마무리할 수 있다 이렇게 도움을 주셔서 학습에 큰 도움이 됐습니다 하다보니 진도 나가는 시간도 빨라졌고 공부하는데에 엄청 도움이 됐습니다 또 상담시간 아니여도 질문을 할 수 있는데 평소에도 선생님이 계시고 질문을 많이 할수있어서 학습에 큰 도움이 됐습니다</v>
+        <v>일주일에 한 번씩 상담을 했는데 지금까지 얼마나 진도를 나갔는지 말씀드리고 하루에 이정도는 해야 진도를 다 끝낼수있고 마무리할 수 있다 이렇게 도움을 주셔서 학습에 큰 도움이 됐습니다 하다보니 진도 나가는 시간도 빨라졌고 공부하는 데에 엄청 도움이 됐습니다 또 상담시간 아니여도 질문을 할 수 있는데 평소에도 선생님이 계시고 질문을 많이 할수있어서 학습에 큰 도움이 됐습니다</v>
       </c>
       <c r="F31" t="str">
         <v>일단 모의고사를 주기적으로 정말 많이 봤습니다 평가원 뿐만 아니라 사설 모의고사도 많이 봤는데 볼 때마다 성적이 어느정도 나오는지 어느 학교가 적정인지 알려주는 그래프와 수치를 맨날 받았습니다 그걸 보고 어떤 과목이 부족했고 더 열심히해야하는지 알 수 있어서 도움이 됐어요</v>
@@ -1617,14 +1617,14 @@
 그리고 매일 영단어 시험, 영어 듣기 테스트, 문제 질문첨삭 상담 등 코칭 시스템이 다양하고 풍부하여 유용하게 활용하였습니다</v>
       </c>
       <c r="F34" t="str">
-        <v>신뢰할 수 있는 대학생 멘토쌤과 언제든지 1:1 질의응답을 할 수 있는게 되게 유용했습니다. 문제에 관한 질문뿐만 아니라 학습법, 학습방향, 선택과목 설정 등 공부 고민에 대한 질문도 할 수 있다는게 좋았습니다. 실제로 6모 후 선택과목을 바꿀때 많은 도움이 되었고 그 외 걱정거리 또한 멘토샘들이 친절하게 상담해주셔서 많이 도움 받았습니다. 수험생이라면 1년동안 공부 고민이 많을텐데 그때 1:1 질의응답을 이용해도 유용할 것 같습니다</v>
+        <v>신뢰할 수 있는 대학생 멘토쌤과 언제든지 1:1 질의응답을 할 수 있는게 되게 유용했습니다. 문제에 관한 질문뿐만 아니라 학습법, 학습방향, 선택과목 설정 등 공부 고민에 대한 질문도 할 수 있다는게 좋았습니다. 실제로 6모 후 선택과목을 바꿀때 많은 도움이 되었고 그 외 걱정거리 또한 멘토샘들이 친절하게 상담해주셔서 많이 도움 받았습니다. 수험생이라면 1년 동안 공부 고민이 많을텐데 그때 1:1 질의응답을 이용해도 유용할 것 같습니다</v>
       </c>
       <c r="G34" t="str" xml:space="preserve">
         <v xml:space="preserve">혼자 공부할때 가장 힘든게 핸드폰, 태블릿 사용인데 학원에서 관리해주니 정말 좋았습니다. 공부 할때 내내 감시받는 기분이라 딴짓은 절대 못하고 _x000d_
 공부에만 몰입할 수 있어 많이 유용하였습니다. 전자기기 사용 욕구 또한 많이 줄어들어 학원이 끝나고도, 일상생활에서도 전자기기에 의존하지 않을 수 있게 되었습니다.</v>
       </c>
       <c r="H34" t="str">
-        <v>저같은 경우에는 영어단어 외우기가 굉장히 귀찮았고 실제로 영어 공부시간 또한 현저히 적었습니다. 그러나 이투스247을 다니고나선 매일 VOCA 테스트를 보니깐 강제로 영어단어를 외우게 되어 좋았습니다. 매일 보는 단어테스트가 누적되어 수능날이 되면 결코 무시하지 못할 양의 단어를 외운 셈이고 또한 한권을 몇바퀴 돌리고 다음 단어책으로 넘어가 복습까지 자동으로 되었습니다.</v>
+        <v>저같은 경우에는 영어단어 외우기가 굉장히 귀찮았고 실제로 영어 공부 시간 또한 현저히 적었습니다. 그러나 이투스247을 다니고나선 매일 VOCA 테스트를 보니깐 강제로 영어단어를 외우게 되어 좋았습니다. 매일 보는 단어테스트가 누적되어 수능날이 되면 결코 무시하지 못할 양의 단어를 외운 셈이고 또한 한권을 몇바퀴 돌리고 다음 단어책으로 넘어가 복습까지 자동으로 되었습니다.</v>
       </c>
       <c r="I34" t="str" xml:space="preserve">
         <v xml:space="preserve">선생님들 모두모두 친절하게 대해주시고 생활 관리도 잘해주셔서 정말 감사했습니다.  덕분에 윈터스쿨, 썸머스쿨동안 공부 열심히 할 수 있었던 것 같습니다.  _x000d_
@@ -1761,7 +1761,7 @@
         <v>국어 선생님께서 국어를 어떻기 학습해야 할지 자세히 알려주셔서 좋았습니다. 특히 저는 현대소설이 약했는데, 9월 평가원에서 현대소설이 어렵게 출제되어 오답에 부담을 느끼고 있었는데 담임 선생님께서 오답을 하는 가이드라인을 제시해주셔서 도움을 많이 받았던 기억이 있습니다.</v>
       </c>
       <c r="F38" t="str">
-        <v>저는 2주에 한번씩 학습 상담울 받았었는데요, 저는 못하는 과목을 기피하는 성향이 있었는데,특히 영어가 그랬던 것 같습니다. 하지만 선생님께서 영어를 꾸준히 학습할 수 있게끔 단어 테스트를 치게 하는 등으로 도움을 꾸준히 주셔서 영어 공부를 놓치 않고 지속적으로 할 수 있었습니다.</v>
+        <v>저는 2주에 한 번씩 학습 상담울 받았었는데요, 저는 못하는 과목을 기피하는 성향이 있었는데,특히 영어가 그랬던 것 같습니다. 하지만 선생님께서 영어를 꾸준히 학습할 수 있게끔 단어 테스트를 치게 하는 등으로 도움을 꾸준히 주셔서 영어 공부를 놓치 않고 지속적으로 할 수 있었습니다.</v>
       </c>
       <c r="G38" t="str">
         <v>저희 학원에서는 순찰을 자주 도셨는데요, 한 자리에 오래 앉아있다 보면 자세도 흐트러지고 집중력도 떨어지고, 졸음도 오기 마련인데 선생님들께서 순찰을 자주 돌아주셔서 어느정도 긴장감을 꾸준히 유지하면서 집중해서 공부를 할 수 있었던 것 같습니다.</v>
@@ -1773,7 +1773,7 @@
         <v>언제나 진심으로 최선을 다해서 학생들을 관리해주셔서 감사합니다. 덕분에 알찬 일년을 보낼 수 있었던 것 같습니다. 만약 주변에서 독학재수학원을 고민하는 지인이 있다면, 저는 고민없이 이투스247을 추천랄 것 같습니다.</v>
       </c>
       <c r="J38" t="str">
-        <v>저는 2주에 한번씩 학습 상담울 받았었는데요, 상담을 받으면서 기피하는 과목을 가까이 하는 방법에 대해 많은 조언을 해주셨어요.</v>
+        <v>저는 2주에 한 번씩 학습 상담울 받았었는데요, 상담을 받으면서 기피하는 과목을 가까이 하는 방법에 대해 많은 조언을 해주셨어요.</v>
       </c>
       <c r="K38" t="str">
         <v>학습 관리</v>
@@ -1832,7 +1832,7 @@
         <v>기숙이라 여러모로 불편한 점이 많았는데 상담을 통해 격려와 응원을 받았고 시설 문제가 생겼을 때 대처해주려 노력하시는 부분이 좋았습니다…또한 타 학생의 방해행동에 대해 서로 불편하지 않는 선에서 해결해주셨습니다..</v>
       </c>
       <c r="F40" t="str">
-        <v>각 과목별로 담당선생님께 질의응답을 신청하여 문제를 해결할 수 있었던 점이 좋았습니다. 특히 수학같은경우 담당선생님께서 시간이 오버되면 또 다른 시간을 잡아서라도 끝까지 설명해주셔서 감사했습니다.</v>
+        <v>각 과목별로 담당 선생님께 질의응답을 신청하여 문제를 해결할 수 있었던 점이 좋았습니다. 특히 수학같은경우 담당 선생님께서 시간이 오버되면 또 다른 시간을 잡아서라도 끝까지 설명해주셔서 감사했습니다.</v>
       </c>
       <c r="G40" t="str">
         <v>물론 방화벽을 뚫는 학생들도 보았습니다. 하지만 저는 막아둔 것에 의미가 있다고 생각하여 틀안에서 벗어나지 않으려했는데요, 인터넷에 노출되지않아 잡생각과 유혹등에 현혹되지않을수 있어서 좋았던 것 같습니다.</v>
@@ -1844,7 +1844,7 @@
         <v>비록 수능날에 긴장을 너무많이해서 실력발휘를 못한것이 너무나 아쉽긴하지만, 실력은 확실히 늘었음을 체감할 수 있었습니다. 약 일년간 지도해주시느라 수고많으셨고 현역때의 아쉬움을 해결하고 넘어갈수있어서 좋았습니다. 서포트해주셔서 감사합니다.</v>
       </c>
       <c r="J40" t="str">
-        <v>각 과목별로 담당선생님께 질의응답을 신청하여 문제를 해결할 수 있었던 점이 좋았어요.</v>
+        <v>각 과목별로 담당 선생님께 질의응답을 신청하여 문제를 해결할 수 있었던 점이 좋았어요.</v>
       </c>
       <c r="K40" t="str">
         <v>질의응답</v>
@@ -1899,13 +1899,13 @@
         <v>N수생</v>
       </c>
       <c r="E42" t="str">
-        <v>지점마다 차이가 있겠지만 다른 독학재수학원에 비해 학생당 선생님 수가 많아서 디테일한 상담이 가능했고 이로 하여금 담임선생님께서 잘하고 있는 점부터 약한 과목에 대한 보충방법까지 잘 설명해주셨다.</v>
+        <v>지점마다 차이가 있겠지만 다른 독학재수학원에 비해 학생당 선생님 수가 많아서 디테일한 상담이 가능했고 이로 하여금 담임 선생님께서 잘하고 있는 점부터 약한 과목에 대한 보충방법까지 잘 설명해주셨다.</v>
       </c>
       <c r="F42" t="str">
-        <v>주기적으로 일정기간동안 작성한 플래너를 검사받으면서 담임선생님과 어떤 교재나 강의 그리고 공부계획등을 언제까지 끝낼지, 또 그 계획이 잘 이루어졌는지를 확인할 수 있어 좋았다. 이로 하여금 계획을 잘 마치겠다는 생각이 계속 공부를 열심히 하게 된 계기가 되었다.</v>
+        <v>주기적으로 일정기간동안 작성한 플래너를 검사받으면서 담임 선생님과 어떤 교재나 강의 그리고 공부 계획등을 언제까지 끝낼지, 또 그 계획이 잘 이루어졌는지를 확인할 수 있어 좋았다. 이로 하여금 계획을 잘 마치겠다는 생각이 계속 공부를 열심히 하게 된 계기가 되었다.</v>
       </c>
       <c r="G42" t="str">
-        <v>수험생활 중 책상에 오래 앉아있다보니 졸리기 십상인데, 이때 혼자서는 졸음을 이겨내기 어렵다고 생각한다. 이투스247에서는 선생님들이 짧고 불규칙한 간격으로 졸음 순찰을 하신다. 그래서 걸릴 수도 있겠다는 생각에 잠을 더 깰 수 있던 것 같고 정말 깜빡 잠들었을때도 다시 공부에 집중할 수 있었던 듯 하다.</v>
+        <v>수험 생활 중 책상에 오래 앉아있다보니 졸리기 십상인데, 이때 혼자서는 졸음을 이겨내기 어렵다고 생각한다. 이투스247에서는 선생님들이 짧고 불규칙한 간격으로 졸음 순찰을 하신다. 그래서 걸릴 수도 있겠다는 생각에 잠을 더 깰 수 있던 것 같고 정말 깜빡 잠들었을때도 다시 공부에 집중할 수 있었던 듯 하다.</v>
       </c>
       <c r="H42" t="str">
         <v>특정 지점에서는 이투스 인강 패스를 재원기간 내에 한정하여 무료로 증정하는데, 처음 공부를 시작하거나 인강을 처음 들어보는 수험생들이 인강에 적응할 수 있게, 또 좋은 선생님의 강의를 듣게 해주었다.</v>
@@ -1981,7 +1981,7 @@
         <v>영어단어를 꾸준히 외우는게 생각보다 쉽지 않은데 학원에서 프린트물+테스트를 봐야해서 꾸준히 외울 수 있었던 거 같습니다. 또 중요단어들을 계속 볼 수 있어서 좋았습니다! 단어 외우는 습관을 잡을 수 있는게 가장 좋았어요</v>
       </c>
       <c r="I44" t="str">
-        <v>항상 친절하게 답해주시고 응원해주셔서 넘 감사했어용. 가끔 지칠때도 있었는데 그때마다 진지하게 함께 고민해주시고 위로도 해주셨고 성적 올리는데도 많은 도움 주셨습니다. 공부습관 잡는데 큰 도움 됐어요</v>
+        <v>항상 친절하게 답해주시고 응원해주셔서 넘 감사했어용. 가끔 지칠 때도 있었는데 그때마다 진지하게 함께 고민해주시고 위로도 해주셨고 성적 올리는데도 많은 도움 주셨습니다. 공부습관 잡는데 큰 도움 됐어요</v>
       </c>
       <c r="J44" t="str">
         <v>규칙적인 생활 습관도 함께 잡을 수 있었고 집중하는 시간도 점점 늘어서 학습에 도움이 많이 됐어요.</v>
@@ -2040,13 +2040,13 @@
       </c>
       <c r="E46" t="str" xml:space="preserve">
         <v xml:space="preserve">선생님들이 친절하시고 사려 깊으셔서 정신적으로 힘든 N수생들도 한 번더 노력해 볼려고 해 볼 수 있을 것 같습니다._x000d_
-  저 같은 경우는 아쉽게도 끝까지 완수하지 못하였지만 다른 학생들 같은 경우 선생님들 덕분에 힘든 수험생활을 넘길수도 있는 분도 있을겁니다.</v>
+  저 같은 경우는 아쉽게도 끝까지 완수하지 못하였지만 다른 학생들 같은 경우 선생님들 덕분에 힘든 수험 생활을 넘길수도 있는 분도 있을겁니다.</v>
       </c>
       <c r="F46" t="str">
-        <v>수험생의 상태를 성적뿐 아니라 그 이외의 것 들도 수험생활에 집중 할 수 있도록 상담해주십니다. 건강이 좋지 않아도 한 번은 이투스247학원에서 수험생활을 노력해볼수 있을 거라고 생각합니다.</v>
+        <v>수험생의 상태를 성적뿐 아니라 그 이외의 것 들도 수험 생활에 집중 할 수 있도록 상담해주십니다. 건강이 좋지 않아도 한 번은 이투스247학원에서 수험 생활을 노력해볼수 있을 거라고 생각합니다.</v>
       </c>
       <c r="G46" t="str">
-        <v>솔직히 방금 네가지 선택지 다 별로였는데 와이파이 방화벽은 비교적 도움이 돼었지만, 핸드폰 반납같은 경우 혼자서 수험생활을 준비하는 학생의 경우 꽤 불편합니다.  학원 와서도 핸드폰으로 딴짓 하면 그것은 개인의 의지 문제이고 선생님들이 관리도 하시니 이 부분은 추후에 더 효율적으로 관리되었으면 합니다.</v>
+        <v>솔직히 방금 네가지 선택지 다 별로였는데 와이파이 방화벽은 비교적 도움이 돼었지만, 핸드폰 반납같은 경우 혼자서 수험 생활을 준비하는 학생의 경우 꽤 불편합니다.  학원 와서도 핸드폰으로 딴짓 하면 그것은 개인의 의지 문제이고 선생님들이 관리도 하시니 이 부분은 추후에 더 효율적으로 관리되었으면 합니다.</v>
       </c>
       <c r="H46" t="str">
         <v>수능까지 아직 시간이 많이 남은 경우이 한가지 과목만 공부하는 날이 많은데,  그런 날 다른과목을 최소한으로라도 학습량을 챙길수 있어서 감각이 떨어지지 않거나 덜 떨어트릴 수 있는 콘텐츠라고 생각합니다.</v>
@@ -2055,7 +2055,7 @@
         <v>몸도 마음도 힘들었지만 재원하는동안 사정봐주시고 신경 써주셔서 너무 감사합니다. 저 같은 수험생은 보지않고 싶으실것 같습니다. 그래도 신경써주셔서 그나마 덜 힘들었습니다. 학생 개개인 별로 사정을 파악하고 조치를 취하시는게 어려울것 같습니다만 그렇게 해주셔서 감사합니다</v>
       </c>
       <c r="J46" t="str">
-        <v>성적뿐만 아니라 그 이외의 것 들도 수험생활에 집중 할 수 있도록 상담해주셨어요.</v>
+        <v>성적뿐만 아니라 그 이외의 것 들도 수험 생활에 집중 할 수 있도록 상담해주셨어요.</v>
       </c>
       <c r="K46" t="str">
         <v/>
@@ -2110,7 +2110,7 @@
         <v>N수생</v>
       </c>
       <c r="E48" t="str">
-        <v>학습 도중에 공부에 대한 막막함과 학습 방법에 대해 어떤식으로 해야할지 모르겠을 때에 저에게 맞는 해결법을 주신다는 점에서 유용하다 느꼈습니다. 그리고 또 학습 상담뿐만 아니라 졸음을 느낄 때, 집중력이 흐려질 때 등 생활 상담에 대해서도 해답을 주셔서 좋았습니다.</v>
+        <v>학습 도중에 공부에 대한 막막함과 학습 방법에 대해 어떤식으로 해야 할지 모르겠을 때에 저에게 맞는 해결법을 주신다는 점에서 유용하다 느꼈습니다. 그리고 또 학습 상담뿐만 아니라 졸음을 느낄 때, 집중력이 흐려질 때 등 생활 상담에 대해서도 해답을 주셔서 좋았습니다.</v>
       </c>
       <c r="F48" t="str">
         <v>헷갈리는 문제에 대해서 어떤 질문을 하더라도 친절하게 설명해주십니다. 이해가 되지 않아 쩔쩔매고 있을 때에도 문제에 대해 비유를 해주시는 등 열정적으로 이해가 쏙쏙되게 알려주십니다.</v>
@@ -2151,7 +2151,7 @@
         <v>매일 작성하는 일간 학습 플래너를 토대로 하교시 제출 후, 다음날 바로 바로 피드백을 해주셔서 좋았다. 놓치고 있는 부분을 보완할 수 있도록 바로 바로 체크해주시고 진도나간 부분을 다시 한번 복습할 수 있는 시스템이 좋았다</v>
       </c>
       <c r="G49" t="str">
-        <v>매 시간 선생님들께서 돌아다니시면서 조는 친구들을 깨워주시니 자연스럽게 면학 분위기도 잡혀서 좋았다. 또한 와이파이 방화벽 시스템을 통해, 자칫 자제하기 힘들뻔한 인터넷 사용을 강제적으로 막아주어 마음을 다잡고 재수생활을 보낼 수 있었다</v>
+        <v>매 시간 선생님들께서 돌아다니시면서 조는 친구들을 깨워주시니 자연스럽게 면학 분위기도 잡혀서 좋았다. 또한 와이파이 방화벽 시스템을 통해, 자칫 자제하기 힘들뻔한 인터넷 사용을 강제적으로 막아주어 마음을 다잡고 재수 생활을 보낼 수 있었다</v>
       </c>
       <c r="H49" t="str">
         <v>이투스 구독권을 제공받는게 상당히 유용했다. 박광일, 김동환 선생님의 수업과 이지영 선생님과 같은 1타 강사의 인강을 들을 수 있는게 상당히 유용했다. 격월로 이투스 모의고사를 통해 나의 위치를 확인하고 계속하여 앞으로 나아갈 수 있었다</v>
@@ -2219,7 +2219,7 @@
         <v>학습뿐만 아니라 생활방면에서도 학생들의 멘탈케어를 위해 생활담임 선생님들께서 관심을 가지고 대해주셨던 점이 힘든 기숙학원 생활에서 도움이 많이 되었습니다. 가끔씩 설명회를 열어 리프레시를 할 수 있던 경험도 생각이 납니다.</v>
       </c>
       <c r="F51" t="str">
-        <v>매달 치는 모의고사를 통해 담임선생님과 상담을 하면서 취약 과목 분석, 방향성 제시, 나의 위치 등의 전문적인 정보를 얻을 수 있었습니다. 독학이지만 이런 부분은 혼자서 하기 어렵기 때문에 필요한 방면에서 선생님들이 서포트해주시는 점이 좋았습니다.</v>
+        <v>매달 치는 모의고사를 통해 담임 선생님과 상담을 하면서 취약 과목 분석, 방향성 제시, 나의 위치 등의 전문적인 정보를 얻을 수 있었습니다. 독학이지만 이런 부분은 혼자서 하기 어렵기 때문에 필요한 방면에서 선생님들이 서포트해주시는 점이 좋았습니다.</v>
       </c>
       <c r="G51" t="str">
         <v>아무래도 태블릿으로 공부하다 보면 딴짓을 하고 싶은 욕구가 강하게 드는데 애초에 와이파이가 학습 외 어플을 차단해주가 때문에 오롯이 공부에만 집중하고 쉴 때도 체력충전을 할 수 있기 때문에 가장 좋았습니다.</v>
@@ -2231,7 +2231,7 @@
         <v>항상 학생들을 위해 힘써주시고 친근하게 다가와 주셔서 감사했습니다! 기숙학원에 틀어박혀서 예민해지고 매일 같은 사람들만 마주치다 보니 트러블이 생기기도 했는데 그럴 때마다 최대한 학생들을 배려하며 해결해주시는 모습이 인상 깊었어요</v>
       </c>
       <c r="J51" t="str">
-        <v>매달 치는 모의고사를 통해 담임선생님과 상담을 하면서 취약 과목 분석, 방향성 제시, 나의 위치 등의 전문적인 정보를 얻을 수 있었어요.</v>
+        <v>매달 치는 모의고사를 통해 담임 선생님과 상담을 하면서 취약 과목 분석, 방향성 제시, 나의 위치 등의 전문적인 정보를 얻을 수 있었어요.</v>
       </c>
       <c r="K51" t="str">
         <v>모의고사</v>
@@ -2251,12 +2251,12 @@
         <v>반수생</v>
       </c>
       <c r="E52" t="str" xml:space="preserve">
-        <v xml:space="preserve">국어가 맨날 5~6등급이었지만 국어 멘토링덕분에 2,3,4등급은 안정적으로 받을수있는 수준으로 발전하였다_x000d_
-또한 탐구를 담임선생님께서 잘 체크해주셔서 빠뜨리지 않고 잘 공부할수있었다</v>
+        <v xml:space="preserve">국어가 맨날 5~6등급이었지만 국어 멘토링덕분에 2,3,4등급은 안정적으로 받을 수있는 수준으로 발전하였다_x000d_
+또한 탐구를 담임 선생님께서 잘 체크해주셔서 빠뜨리지 않고 잘 공부할 수있었다</v>
       </c>
       <c r="F52" t="str" xml:space="preserve">
         <v xml:space="preserve">오늘 할일을 처음 아침에 앉아 생각해볼수있었고 그것을 실천하여_x000d_
-최대한의 효율과 무리를 하지않고 공부할수있었던것 같다 또한 공부끝나고 오늘 한일을 체크하고 피드백하는과정에서 부족한부분도 체크할수있어서 좋았다</v>
+최대한의 효율과 무리를 하지않고 공부할 수있었던것 같다 또한 공부끝나고 오늘 한일을 체크하고 피드백하는과정에서 부족한부분도 체크할수있어서 좋았다</v>
       </c>
       <c r="G52" t="str">
         <v>개인적으로 잠이 많고 졸음이 많은데 선생님께서 졸지말라고 잘 깨워주셨고 다른 좌석에서 친구들이 잘때소리나는 코고는소리 숨소리를 모두 체크해주셔서 면학 분위기에 좋은 영향을 끼칠수있었던것 같다</v>
@@ -2268,7 +2268,7 @@
         <v>모든 선생님들 지도해주셔서 감사했습니다 특히 태민선생님 상담 잘해주시고 피드백 잘해주셔서 감사했습니다 찾아뵙고싶었는데 못찾아뵈었네요 죄송합니다 다음에 기회가 된다면 꼭 찾아뵙고싶습니다</v>
       </c>
       <c r="J52" t="str">
-        <v>6등급이었지만 국어 멘토링덕분에 2,3,4등급은 안정적으로 받을수있는 수준으로 발전하였어요.</v>
+        <v>6등급이었지만 국어 멘토링덕분에 2,3,4등급은 안정적으로 받을 수있는 수준으로 발전하였어요.</v>
       </c>
       <c r="K52" t="str">
         <v/>
@@ -2396,7 +2396,7 @@
         <v>독학공부를 하다보니 학습방향성에 대해 자주 불안했었는데 친절하신 담당과목 선생님들과의 상담이 자유로워 불안을 즉시 해결할 수 있었음. 더 나아가 장기적으로 보았을 때 수험생 멘탈관리 부분에서도 효과적이었던 것 같음.</v>
       </c>
       <c r="F56" t="str">
-        <v>혼자 공부를 하다보면 나태해져 과목편식이 심해졌었는데 관리를 받으니 하기 싫은 과목도 꾸준히 하게 되는 점이 좋았다. 플래너 쓰기 귀찮아서 대충 썼었는데 플래너 검사를 통해 해야 되는 것을 가시화하는 습관을 만들게 되어 수험생활에 큰 도움이 되었음.</v>
+        <v>혼자 공부를 하다보면 나태해져 과목편식이 심해졌었는데 관리를 받으니 하기 싫은 과목도 꾸준히 하게 되는 점이 좋았다. 플래너 쓰기 귀찮아서 대충 썼었는데 플래너 검사를 통해 해야 되는 것을 가시화하는 습관을 만들게 되어 수험 생활에 큰 도움이 되었음.</v>
       </c>
       <c r="G56" t="str">
         <v>일반 독서실에 가면 아무리 휴대폰을 안 보려 해도 자꾸만 손이 가는게 스트레스였는데 강제로 휴대폰을 수거해 가서 공부에 집중할 수 있다는 점이 좋았음. 점심,저녁시간에도 휴대폰을 못 쓰니 자연스럽게 휴대폰 의존도가  낮아져 평소 집중력도 올라건 것 같음.</v>
@@ -2408,7 +2408,7 @@
         <v>이투스 선생님들 좋은 면학 분위기를 위해 노력해주시고 훌륭한 지도 해주셔서 감사합니다. 덕분에 성적 향상과 좋은 습관을 얻은 것 같습니다. 후배들이나 다시 도전하는 친구들에게 좋을 말 많이 전할게요</v>
       </c>
       <c r="J56" t="str">
-        <v>플래너 점검을 통해 해야 할 일을 한눈에 정리하는 습관이 생겨 수험생활에 큰 도움이 되었어요.</v>
+        <v>플래너 점검을 통해 해야 할 일을 한눈에 정리하는 습관이 생겨 수험 생활에 큰 도움이 되었어요.</v>
       </c>
       <c r="K56" t="str">
         <v/>
@@ -2428,19 +2428,19 @@
         <v>N수생</v>
       </c>
       <c r="E57" t="str">
-        <v>매달 담당선생님이 직접 찾아오셔서 부르셔서 학습 과제 학습 진행 상태 등을 직접 점검해주시고 직접 과목마다 인터넷강의 강사와 교재등을 추천해주시고 가끔 간식같은것도 챙겨주시고 덕담,응원의 말들을 많이 해주셔서 많이 힘이 됐습니다.</v>
+        <v>매달 담당 선생님이 직접 찾아오셔서 부르셔서 학습 과제 학습 진행 상태 등을 직접 점검해주시고 직접 과목마다 인터넷강의 강사와 교재등을 추천해주시고 가끔 간식같은것도 챙겨주시고 덕담,응원의 말들을 많이 해주셔서 많이 힘이 됐습니다.</v>
       </c>
       <c r="F57" t="str">
-        <v>학습 관리를 담당선생님이 세심하게 해주시고 모의고사 끝날때마다 4층으로 부르셔서 각 과목 담당선생님이 시험난이도나 등급컷 어려운 문제 해설 등등을 해주셔서 도움이 많이 되었습니다. 그리고 제가 졸거나 집중 못하고있을때 확인하셔서 깨워주시는게 도움되었습니다.</v>
+        <v>학습 관리를 담당 선생님이 세심하게 해주시고 모의고사 끝날때마다 4층으로 부르셔서 각 과목 담당 선생님이 시험난이도나 등급컷 어려운 문제 해설 등등을 해주셔서 도움이 많이 되었습니다. 그리고 제가 졸거나 집중 못하고있을때 확인하셔서 깨워주시는게 도움되었습니다.</v>
       </c>
       <c r="G57" t="str">
-        <v>생활 관리 시스템중에서 특히 유용했던점은 전자출결 시스템을 이용해서 일일이 확인하는일이 없어 서로 번거로운일 없이 출석체크가 가능합니다. 그리고 외출하거나 조퇴하는 일이 있을때 일일이 담당선생님께 말씀드리고 확인받고 갈 필요없이 전자출결로 조회를 해놓으면 되니 매우 편리하고 도움이 많이되는 시스템이었다고 생각되었습니다.</v>
+        <v>생활 관리 시스템중에서 특히 유용했던점은 전자출결 시스템을 이용해서 일일이 확인하는일이 없어 서로 번거로운일 없이 출석체크가 가능합니다. 그리고 외출하거나 조퇴하는 일이 있을때 일일이 담당 선생님께 말씀드리고 확인받고 갈 필요없이 전자출결로 조회를 해놓으면 되니 매우 편리하고 도움이 많이되는 시스템이었다고 생각되었습니다.</v>
       </c>
       <c r="H57" t="str">
         <v>교육청,평가원에서 실시하는 전국 모의고사 뿐만이 아니라 이투스 학원에서 제공하는 이투스 모의고사를 추가로 풀고 답을 확인하고 해설을 들으니 더 철저히 수능을 준비할수 있었고 모르는 개념도 추가로 확인하고 얻어갈수있었고 시험을 여러번 보다보니 수능 당일날 크게 긴장하지 않는 마인드셋을 가질수있었던것 같습니다.</v>
       </c>
       <c r="I57" t="str">
-        <v>학원에 있는동안 친절하게 도와주시고 응원해주셔서 감사합니다! 국어 선생님은 항상 친절하게 문학,독서 관련 팁들을 알려주셔서 도움이 많이 되었고 수학 선생님은 본인도 n수 경험이 있다며 현실적인 경험담과 조언을 많이 해주셨고 영어 선생님은 제 담임선생님으로써 많이 케어해주셨습니다 모두 도움이 많이 되었습니다 늘 감사합니다!</v>
+        <v>학원에 있는동안 친절하게 도와주시고 응원해주셔서 감사합니다! 국어 선생님은 항상 친절하게 문학,독서 관련 팁들을 알려주셔서 도움이 많이 되었고 수학 선생님은 본인도 n수 경험이 있다며 현실적인 경험담과 조언을 많이 해주셨고 영어 선생님은 제 담임 선생님으로써 많이 케어해주셨습니다 모두 도움이 많이 되었습니다 늘 감사합니다!</v>
       </c>
       <c r="J57" t="str">
         <v>전자출결 시스템 덕분에 번거로운 확인 과정 없이 편하게 출석 체크를 할 수 있었어요.</v>
@@ -2468,7 +2468,7 @@
 좋은 공부습관을 잡아주기 위한 개인 코칭이 기억에 남음.</v>
       </c>
       <c r="F58" t="str" xml:space="preserve">
-        <v xml:space="preserve">앞서 말했듯 담임의 개인 코칭에 따른 학습관리가 기억에 남음._x000d_
+        <v xml:space="preserve">앞서 말했듯 담임의 개인 코칭에 따른 학습 관리가 기억에 남음._x000d_
 개인별 맞춤 관리에 공부를 하고자 하는 의욕이 생겼었음._x000d_
 이투스 홈페이지에 게시되어있는 온라인 학습 관리 시스템을 사용한 기억은 없음._x000d_
 따라서 이 유용성에 대해 할 말은 없음.</v>
@@ -2518,7 +2518,7 @@
 더불어 내가 어떤 곳에서 실수했는지 셀프 피드백을 손으로 써보며 다음번에는 같은 실수를 반복하지 않게 됐고 객관적인 사후 판단을 할 수 있는점이 좋았습니다</v>
       </c>
       <c r="G59" t="str">
-        <v>제가 잠이 많은 편이라서 졸때가 많았는데 그때마다 잠을 깨워주고 다시 공부를 하게 만들어주는 점이 좋았습니다 또한 규칙적인게 아닌 불규칙적으로 돌면서 계속 긴장감을 유지해주는 점도 좋았습니다 일정한 시간에만 돌면 그 시간을 피해서 잘 수도 있는데 그런 점을 감안한 선생님들의 배려가 좋았습니다</v>
+        <v>제가 잠이 많은 편이라서 졸 때가 많았는데 그때마다 잠을 깨워주고 다시 공부를 하게 만들어주는 점이 좋았습니다 또한 규칙적인게 아닌 불규칙적으로 돌면서 계속 긴장감을 유지해주는 점도 좋았습니다 일정한 시간에만 돌면 그 시간을 피해서 잘 수도 있는데 그런 점을 감안한 선생님들의 배려가 좋았습니다</v>
       </c>
       <c r="H59" t="str" xml:space="preserve">
         <v xml:space="preserve">공부를 하다보면 암기 위주의 공부가 질릴수도 있는데 매일매일 선생님들이 프린트를 바꿔주는 노력을 보고 저도 동기를 받아 열심히 외웠던거 같습니다_x000d_
@@ -2552,7 +2552,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E60" t="str">
-        <v>1대1 상담과 스케줄표 작성을 담당선생님께서 모두 함께 도와주셔서 혼자서도 어렵지 않게 공부법과 시간을 정할 수 있었고 스케줄관리에 딱히 큰 시간을 투자하지 않아도 된다는 점이 유용했습니다</v>
+        <v>1대1 상담과 스케줄표 작성을 담당 선생님께서 모두 함께 도와주셔서 혼자서도 어렵지 않게 공부법과 시간을 정할 수 있었고 스케줄관리에 딱히 큰 시간을 투자하지 않아도 된다는 점이 유용했습니다</v>
       </c>
       <c r="F60" t="str">
         <v>멘토 선생님들이 한 분만 계시는 것이 아니라 질문에 대한 여러가지 답을 얻을 수 있어서 좋았고 선생님들의 성적도 매우 우수하셔서 쉬운 풀이법이나 이해 방법을 터득할 수 있다는 점이 유용했습니다</v>
@@ -2587,7 +2587,7 @@
         <v>N수생</v>
       </c>
       <c r="E61" t="str">
-        <v>어떤 강의를 들어야 할지 어떤 책으로 공부해야할지 몰랐는데 처음부터 자세히 알려주셔서 공부를 시작하고 탐구과목도 뭘 할지 몰랐던 제게 이기상 선생님이라는 좋은 강사님을 알려주셔서 탐구 한과목을 좋은 성적을 냈던 기억이있습니다. 모의고사가 끝나면 오답도 하면서 더시 복습을 함으로써 다음 시험을 준비할 수 있게 해주었습니다</v>
+        <v>어떤 강의를 들어야 할지 어떤 책으로 공부해야 할지 몰랐는데 처음부터 자세히 알려주셔서 공부를 시작하고 탐구과목도 뭘 할지 몰랐던 제게 이기상 선생님이라는 좋은 강사님을 알려주셔서 탐구 한과목을 좋은 성적을 냈던 기억이있습니다. 모의고사가 끝나면 오답도 하면서 더시 복습을 함으로써 다음 시험을 준비할 수 있게 해주었습니다</v>
       </c>
       <c r="F61" t="str" xml:space="preserve">
         <v xml:space="preserve">앞에서 말했다시피 탐구과목을 고르고 강의를 선택해준게 제일 좋았고 강사님을 해보고 맞지 않았다고 느꼈을때 같이 골라주셔서 국어도 저에게 맞는 강사님으로 고르게 되었습니다._x000d_
@@ -2661,7 +2661,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E63" t="str">
-        <v>과목별로 바로바로 질문을 해결할 수 있었으며 과목별 공부방법에 대해 꿀팁을 얻을 수 있다. 모으고사 틀린문제를 직접 분석해주시며 개인별 부족한점과 보완할점을 각각 알려주셔 성적향상에 큰 도움이 되었다</v>
+        <v>과목별로 바로바로 질문을 해결할 수 있었으며 과목별 공부방법에 대해 꿀팁을 얻을 수 있다. 모으고사 틀린문제를 직접 분석해주시며 개인별 부족한점과 보완할점을 각각 알려주셔 성적 향상에 큰 도움이 되었다</v>
       </c>
       <c r="F63" t="str">
         <v>취약한 부분에 대해 알 수 있고, 입시라는 현실에 부딪히게 해주어서 과목 편식과 같은 습관들로부터 벗어날 수 있었다 또한 나의 문제점을 바로 확인할 수 있었다. 질문을 바로 해결할 수 있다.</v>
@@ -2703,7 +2703,7 @@
         <v>독학재수를 하면서 가장 어려웠던 점은 혼자 공부하다 보니 쉽게 방향을 잃고 시간 관리가 흐트러진다는 것이었습니다. 학습 관리 시스템을 사용한 이후로는 매일 해야 할 공부량과 목표를 정리할 수 있어 훨씬 계획적으로 공부할 수 있었고, 공부 시간과 진행 상황을 기록하면서 스스로를 객관적으로 돌아볼 수 있었습니다. 특히 꾸준히 기록하다 보니 집중력도 자연스럽게 유지되어 전체적인 학습 효율이 높아졌다고 느꼈습니다.</v>
       </c>
       <c r="G64" t="str">
-        <v>감독을 공부시간에 계속해서 받는 느낌이라 혼자 공부하면서도 쉽게 나태해지지 않게 잡아주는 점이 특히 좋았습니다. 누가 직접 옆에서 관리해주는 것은 아니지만, 기록을 남기고 계획을 확인하는 과정 자체가 스스로를 통제하게 만들어서 공부 흐름이 끊기지 않았습니다. 덕분에 하루 공부량을 보다 꾸준히 유지할 수 있었고, 전반적인 학습 태도도 이전보다 훨씬 안정적으로 바뀌었다고 느꼈습니다.</v>
+        <v>감독을 공부 시간에 계속해서 받는 느낌이라 혼자 공부하면서도 쉽게 나태해지지 않게 잡아주는 점이 특히 좋았습니다. 누가 직접 옆에서 관리해주는 것은 아니지만, 기록을 남기고 계획을 확인하는 과정 자체가 스스로를 통제하게 만들어서 공부 흐름이 끊기지 않았습니다. 덕분에 하루 공부량을 보다 꾸준히 유지할 수 있었고, 전반적인 학습 태도도 이전보다 훨씬 안정적으로 바뀌었다고 느꼈습니다.</v>
       </c>
       <c r="H64" t="str">
         <v>이투스 전국모의고사라는 모의고사를 통해 현재 나의 실력을 객관적으로 확인할 수 있었고, 부족한 부분이 무엇인지 구체적으로 파악할 수 있었습니다. 특히 실제 시험과 유사한 환경에서 문제를 풀어보면서 시간 관리 능력과 문제 해결 전략을 점검할 수 있었고, 이후 학습 방향을 설정하는 데에도 큰 도움이 되었습니다.</v>
@@ -2802,7 +2802,7 @@
         <v>N수생</v>
       </c>
       <c r="E67" t="str">
-        <v>혼자 입시를 하는경우 입시정보나 중요한 정보들을 얻기도 힘들고 알기도 힘든데 그런 정보들을 알수있어서 좋았고 담당선생님께서 그것을바탕으로 상담을 하거나 전략을 짜서 공부방향이나 공부전략 등 입시에 도움을 주셔서 유용했습니다.</v>
+        <v>혼자 입시를 하는경우 입시정보나 중요한 정보들을 얻기도 힘들고 알기도 힘든데 그런 정보들을 알수있어서 좋았고 담당 선생님께서 그것을바탕으로 상담을 하거나 전략을 짜서 공부방향이나 공부전략 등 입시에 도움을 주셔서 유용했습니다.</v>
       </c>
       <c r="F67" t="str">
         <v>혼자서 하면 모르는것을 질문하기 어렵습니다. 인강의 QnA질문을 해도 빨라도 하루는 걸리는 질의응답을 실시간으로 궁굼한 점이 생기면 바로바로 질문하고 답변받을 수 있어서 좋았습니다.</v>
@@ -2814,7 +2814,7 @@
         <v>이투스에 듣고싶은 강사가 있었는데 한분만 듣고싶어서  구독하기에는 부담이 되는 상황이였습니다 그런데 이투스247를 다니면 이투스구독 서비스가 제공되어서 강의를 듣게 되어서 좋았습니다.</v>
       </c>
       <c r="I67" t="str">
-        <v>1년동안 감사했습니다. 출결관리도 해주시고 졸거나 집중안될 때 도와주시고 면학 분위기 조성해주셔서 감사했습니다. 이것저것 도움되라고 간식등 챙겨주신것도 감사합니다. 일상에서 간간히 대화했던 것도 힘들지않고 공부하는데 도움많이됐습니다 감사합니다!</v>
+        <v>1년 동안 감사했습니다. 출결 관리도 해주시고 졸거나 집중안될 때 도와주시고 면학 분위기 조성해주셔서 감사했습니다. 이것저것 도움되라고 간식등 챙겨주신것도 감사합니다. 일상에서 간간히 대화했던 것도 힘들지않고 공부하는데 도움많이됐습니다 감사합니다!</v>
       </c>
       <c r="J67" t="str">
         <v>졸리거나 집중력이 흐트러질 때 도와주셔서 좋은 면학 분위기 속에서 공부할 수 있었어요.</v>
@@ -2872,7 +2872,7 @@
         <v>N수생</v>
       </c>
       <c r="E69" t="str">
-        <v>입시에 대해서 많이 무지한 편이었는데 도움을 많이 주셔서 입시 시스템이 어떻게 돌아가는지 정확하게 파악하는 걸 수월하게 할 수 있었고, 심리적으로도 대학 입시와 수능 공부 방향을 어떻게 해야할 지도 알려주셔서 많이 도움되었던 것 같았습니다.</v>
+        <v>입시에 대해서 많이 무지한 편이었는데 도움을 많이 주셔서 입시 시스템이 어떻게 돌아가는지 정확하게 파악하는 걸 수월하게 할 수 있었고, 심리적으로도 대학 입시와 수능 공부 방향을 어떻게 해야 할 지도 알려주셔서 많이 도움되었던 것 같았습니다.</v>
       </c>
       <c r="F69" t="str">
         <v>자기가 무슨 인강을 들어야할 지 처음엔 감이 안잡힐 때가 많은데 제 성적과 학습 수준에 따라서 어떤 교재와 인강을 들어야할 지 추천해 주셔서 좋았습니다. 방향을 잡는데 많이 도움되었다고 생각해요</v>
@@ -2884,7 +2884,7 @@
         <v>아무래도 모의고사이다 보니까 실전 연습을 자주하게 되어서 수능 시험에 많이 익숙해지도록 하게 되었던 것 같습니다. 물론 학원 내, 자기 자리에서 하는 시험이다보니 실질적으로 수능 시험장에서의 긴장감만큼 긴장이 되진 않지만, 실전 연습이라는 점에서 메리트가 상당하다고 생각합니다.</v>
       </c>
       <c r="I69" t="str">
-        <v>1년 동안 수능 공부 도와주시고 학원 생활 잘하게끔 많이 이끌어주시고 도와주셔서 감사하다고 말씀 드리고 싶어요. 대학에 지금은 합격해서 다니고 있고, 적응 잘해서 졸업까지 무사히 달려가 앞으로 열심히 인생 살아가보겠습니다. 1년동안 감사했습니다.</v>
+        <v>1년 동안 수능 공부 도와주시고 학원 생활 잘하게끔 많이 이끌어주시고 도와주셔서 감사하다고 말씀 드리고 싶어요. 대학에 지금은 합격해서 다니고 있고, 적응 잘해서 졸업까지 무사히 달려가 앞으로 열심히 인생 살아가보겠습니다. 1년 동안 감사했습니다.</v>
       </c>
       <c r="J69" t="str">
         <v>돌아다니시면서 깨워주시는데 그것 덕에 졸음도 깨고 공부 집중에 도움이 되었어요.</v>
@@ -2910,7 +2910,7 @@
         <v>아침 기상 시간을 맞춰 매우 효율적으로 움직일 수 있는 점이 좋았습니다. 6시반에 기상하여 7시50분까지 착석하면 되는 일정이었으나 아침 산책 및 간단한 식사 후 7시까지 자리에 앉아 아침 공부를 하며 루틴을 만들어 생활패턴을 지킬 수 있다는 점이 가장 좋았습니다.</v>
       </c>
       <c r="F70" t="str">
-        <v>학습에 관해 고민이 있거나 번아웃이 오면 담임선생님께 편하게 질문, 상담한 것이 좋았습니다. 기숙이라는 답답할 수 있는 공간에서 털어놓을 수 있어 힘든 순간이 와도 다시 마음을 다잡을 수 있었던 것 같습니다.</v>
+        <v>학습에 관해 고민이 있거나 번아웃이 오면 담임 선생님께 편하게 질문, 상담한 것이 좋았습니다. 기숙이라는 답답할 수 있는 공간에서 털어놓을 수 있어 힘든 순간이 와도 다시 마음을 다잡을 수 있었던 것 같습니다.</v>
       </c>
       <c r="G70" t="str">
         <v>학습 시간 도중 딴짓을 하지 못하게 방화벽으로 외부 사이트가 차단되어있었으나 일부 막히지않은 사이트, 또는 개인적으로 집중력이 너무 흐려져서 딴짓을 하게된 순간이 몇 번 있었는데 선생님들이 교시마다 돌아다니며 학생들을 점검한 점이 매우 좋았습니다. 또한 식곤증이나 아침잠이 왔을 때도 졸지 않게 깨워주셔서 잘 공부할 수 있었던 것 같습니다. 복도의 스탠딩 책상을 이용할 수 있는 점도 좋았습니다.</v>
@@ -2919,10 +2919,10 @@
         <v>6,9월 모의고사만으로는 수능 시험장을 체감하기에 너무 적은 횟수이기에 실모를 한달에 한번은 풀로 봐야한다고 생각해서 이투스전국모고가 유용했습니다. 모의고사의 퀄리티와 별개로 하루를 통으로 써서 모의고사를 볼 수 있다는 점 자체로 아주 큰 메리트가 되었던 것 같습니다. 또한 그 성적을 바탕으로 상담도 해주셔서 앞으로 해나갈 공부 방향을 잘 잡을 수 있었습니다.</v>
       </c>
       <c r="I70" t="str">
-        <v>반년동안 새로운, 그리고 힘들었던 시간이었는데, 다시 생각해보면 그 안에서 선생님들 덕분에 이겨낼 수 있었던 순간이 꽤나 있었던 것 같습니다.  다른 핑계 없이 나 자신에게 부끄럽지 않게 살아가라는 담임선생님 말씀이 아직까지 기억에 남는데 앞으로도 기숙학원에서만큼 열심히 살진 못하더라도, 그 경험을 바탕으로 부끄럽지 않게 살도록 노력해보겠습니다. 감사합니다!</v>
+        <v>반년동안 새로운, 그리고 힘들었던 시간이었는데, 다시 생각해보면 그 안에서 선생님들 덕분에 이겨낼 수 있었던 순간이 꽤나 있었던 것 같습니다.  다른 핑계 없이 나 자신에게 부끄럽지 않게 살아가라는 담임 선생님 말씀이 아직까지 기억에 남는데 앞으로도 기숙학원에서만큼 열심히 살진 못하더라도, 그 경험을 바탕으로 부끄럽지 않게 살도록 노력해보겠습니다. 감사합니다!</v>
       </c>
       <c r="J70" t="str">
-        <v>학습에 관해 고민이 있거나 번아웃이 오면 담임선생님께 편하게 질문, 상담한 것이 좋았어요.</v>
+        <v>학습에 관해 고민이 있거나 번아웃이 오면 담임 선생님께 편하게 질문, 상담한 것이 좋았어요.</v>
       </c>
       <c r="K70" t="str">
         <v/>
@@ -2942,7 +2942,7 @@
         <v>N수생</v>
       </c>
       <c r="E71" t="str">
-        <v>선생님께서 특화된 입시 프로그램을 이용하여 전문적으로 입시 상담을 해주신다. 뿐만 아니라 보통 1년동안 담당 해주실 담임 선생님이 정해지기 때문에 계속 같은 데이터와 정보를 가지고 상담 해주신다.</v>
+        <v>선생님께서 특화된 입시 프로그램을 이용하여 전문적으로 입시 상담을 해주신다. 뿐만 아니라 보통 1년 동안 담당 해주실 담임 선생님이 정해지기 때문에 계속 같은 데이터와 정보를 가지고 상담 해주신다.</v>
       </c>
       <c r="F71" t="str">
         <v>내가 직접 시험 점수를 분석하지 않아도 다양하고 많은 표본을 가지고 내 성적을 분석해준다. 한눈에 보기 편하다. 나의 위치가 어느정도인지 직관적으로, 객관적으로 알 수 있다. 때문에 공부를 위한 원동력이 되기도 한다.</v>
@@ -2957,7 +2957,7 @@
         <v>민호쌤 짱 민호쌤 술 끊으시고 담배 끊으시고 오래오래 건강하시고 맨날 속썩여서 죄송하고 아이스크림 많이 사주셔서 감사합니다 사실 선생님이 제일 좋았어요^^ 과정이 어떻게 됐든 덕분에 완주할 수 있었습니다</v>
       </c>
       <c r="J71" t="str">
-        <v>1년동안 담당 해주실 담임 선생님이 정해지기 때문에 계속 같은 데이터와 정보를 가지고 상담 해주셨어요.</v>
+        <v>1년 동안 담당 해주실 담임 선생님이 정해지기 때문에 계속 같은 데이터와 정보를 가지고 상담 해주셨어요.</v>
       </c>
       <c r="K71" t="str">
         <v/>
@@ -3052,7 +3052,7 @@
         <v>반수생</v>
       </c>
       <c r="E74" t="str">
-        <v>과목별 담당 선생님이 계시고 제일 취약한 과목 선생님을 담임 선생님으로 배정해주셔서 매주 담임선생님과 학습 진도 확인을 할 수 있다는 점이 좋았습니다. 추가로 필요할 때마다 질문을 할 수 있는 점이 좋았습니다.</v>
+        <v>과목별 담당 선생님이 계시고 제일 취약한 과목 선생님을 담임 선생님으로 배정해주셔서 매주 담임 선생님과 학습 진도 확인을 할 수 있다는 점이 좋았습니다. 추가로 필요할 때마다 질문을 할 수 있는 점이 좋았습니다.</v>
       </c>
       <c r="F74" t="str">
         <v>질문이나 학습고민이 생겼을 때 질문 대기자 명단에 이름을 작성하면 따로 불러서 봐주신다는 점이 좋았습니다. 또 대학생 선생님이 아니라 경력이 있으신 분들이 계셔서 더 믿음이 갔던 것 같습니다</v>
@@ -3173,7 +3173,7 @@
         <v>영어단어를 혼자 테스트없이 외우게되면 동기가 없고 의욕도 안생겨서 미루게되는데 강제적으로 테스트를 보게돼서 억지로라도 단어를 외운 것이 매우 좋았습니다 그래서 예전에는 단어책 하나 끝내기도 어려웠는데 이투스를 다니는 동안 매우 많은 단어를 외우게 되었습니다</v>
       </c>
       <c r="I77" t="str">
-        <v>수험생활을 하면서 힘든 점이 많긴해도 응원해주시고 최대한 공부에 집중할 수 있는 환경을 만들어주실려고 노력해주신 선생님들께 매우 감사합니다 앞으로 대학에서도 좋은 결과를 내보겠습니다</v>
+        <v>수험 생활을 하면서 힘든 점이 많긴해도 응원해주시고 최대한 공부에 집중할 수 있는 환경을 만들어주실려고 노력해주신 선생님들께 매우 감사합니다 앞으로 대학에서도 좋은 결과를 내보겠습니다</v>
       </c>
       <c r="J77" t="str">
         <v>과목별 상담과 질문 해결, 와이파이 방화벽 덕분에 집보다 훨씬 집중도 높은 공부가 가능했어요.</v>
@@ -3202,7 +3202,7 @@
       </c>
       <c r="F78" t="str" xml:space="preserve">
         <v xml:space="preserve">매일매일 내가 학습한 공부량을 확인할 수 있어 좋았고 내가 공부한 부분을 정리함으로써 한번 더 상기된 것 같다_x000d_
-또한 매일 기록표를 제출하고 담임선생님 피드백을 확인하는 과정에서 의무감과 책임감응 느껴 긴입시기간동안 풀어지지 않는 생활을 한 것 같아요</v>
+또한 매일 기록표를 제출하고 담임 선생님 피드백을 확인하는 과정에서 의무감과 책임감응 느껴 긴입시기간동안 풀어지지 않는 생활을 한 것 같아요</v>
       </c>
       <c r="G78" t="str">
         <v>학원 전자 출결은 학생의 출석 상황을 실시간으로 확인할 수 있어 관리가 편리하다. 또한 학부모에게 즉시 알림이 전달되어 안전성을 높이고, 데이터가 자동 저장되어 기록 관리와 통계 분석에도 유용했습니다</v>
@@ -3273,10 +3273,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E80" t="str">
-        <v>한 교재를 다 마치고 나면, 그다음엔 무엇을 공부해야 할지, 어떤 인강이 내 학습에 도움이 될지를 매번 망설였었는데 담임선생님께서 같이 고민해 주시고 추천해 주시는 게 많은 도움이 되어 좋았습니다.</v>
+        <v>한 교재를 다 마치고 나면, 그다음엔 무엇을 공부해야 할지, 어떤 인강이 내 학습에 도움이 될지를 매번 망설였었는데 담임 선생님께서 같이 고민해 주시고 추천해 주시는 게 많은 도움이 되어 좋았습니다.</v>
       </c>
       <c r="F80" t="str">
-        <v>매일 뭘 해야 할지 막막하고 혼자 계획을 짜고 공부했을 땐 매번 계획을 제대로 지키지 않는다던가, 좋아하는 과목 위주로만 공부를 하고 그랬는데 이투스 담임선생님과 매주마다 같이 계획을 짜나가고 공부하는 과정을 점검받아 오늘 하루 해야 할 일을 매일매일 더 열심히 하게 되어 좋았습니다.</v>
+        <v>매일 뭘 해야 할지 막막하고 혼자 계획을 짜고 공부했을 땐 매번 계획을 제대로 지키지 않는다던가, 좋아하는 과목 위주로만 공부를 하고 그랬는데 이투스 담임 선생님과 매주마다 같이 계획을 짜나가고 공부하는 과정을 점검받아 오늘 하루 해야 할 일을 매일매일 더 열심히 하게 되어 좋았습니다.</v>
       </c>
       <c r="G80" t="str">
         <v>집이나 스터디 카페에서 혼자 공부하는 것보다, 졸면 깨워주시고 졸음관리를 학원에서 철저하게 해 주시는 게 학습시간을 늘리고, 또 면학 분위기도 좋아 집중을 향상하는 데에 큰 도움이 되어 좋았습니다.</v>
@@ -3285,10 +3285,10 @@
         <v>혼자서는 테스트하듯 단어를 암기하여도 실제 학원에서 시험을 보는듯한 효과는 가지지 못한다고 생각합니다. 꾸준하게 영어단어책을 매일매일 암기하고 시험 보는 것이 단어암기에 좋았습니다.</v>
       </c>
       <c r="I80" t="str">
-        <v>이투스 학원을 재원 하며 많은 선생님들께 도움을 받았습니다. 등원하고 하원할 때마다 반갑게 맞아주시는 카운터 선생님들 감사를 드리고 상담도 잘해주시고 항상 학생들 예뻐해 주시는 원장선생님께도 감사드립니다. 또 이투스 학원 재원 중 제 담임선생님이셨던 모든 선생님들께 정말 감사하다고 말씀드리고 싶습니다. 시험을 망쳐 하루종일이 우울했던 날 저에게 힘을 북돋아주시고 다시 공부할 수 있게 일으켜주셨던 준태선생님께 정말 감사했다고 전하고 싶습니다.</v>
+        <v>이투스 학원을 재원 하며 많은 선생님들께 도움을 받았습니다. 등원하고 하원할 때마다 반갑게 맞아주시는 카운터 선생님들 감사를 드리고 상담도 잘해주시고 항상 학생들 예뻐해 주시는 원장 선생님께도 감사드립니다. 또 이투스 학원 재원 중 제 담임 선생님이셨던 모든 선생님들께 정말 감사하다고 말씀드리고 싶습니다. 시험을 망쳐 하루종일이 우울했던 날 저에게 힘을 북돋아주시고 다시 공부할 수 있게 일으켜주셨던 준태선생님께 정말 감사했다고 전하고 싶습니다.</v>
       </c>
       <c r="J80" t="str">
-        <v>늘 반갑게 맞아주시는 선생님들과 따뜻하게 상담해주시는 원장선생님 덕분에 수험생활에 큰 힘을 얻었어요.</v>
+        <v>늘 반갑게 맞아주시는 선생님들과 따뜻하게 상담해주시는 원장 선생님 덕분에 수험 생활에 큰 힘을 얻었어요.</v>
       </c>
       <c r="K80" t="str">
         <v/>
@@ -3322,7 +3322,7 @@
 또한 체계적인 오답분석을  통해 부족한 부분을 보완하며 학습 방향을 잡는 데 큰 도움을 받을 수 있었던거같습니다.</v>
       </c>
       <c r="I81" t="str" xml:space="preserve">
-        <v xml:space="preserve">선생님들! 어쩌면 가장 힘든 수험생활_x000d_
+        <v xml:space="preserve">선생님들! 어쩌면 가장 힘든 수험 생활_x000d_
 학생들을 위해 최선을 다해주셔서 감사합니다._x000d_
 세심한 관리때문에 성장할수있었고_x000d_
 힘들었던 순간마다 선생님들의 한마디가 큰 힘이 되어 버틸수있었습니다_x000d_
@@ -3351,7 +3351,7 @@
         <v>N수생</v>
       </c>
       <c r="E82" t="str">
-        <v>매달 치르는 모의고사 성적표로 개인 상담을 진행했을때 과목별로 현재 부족한 점과 보안할 점을 자세히 알려주셨습니다. 뿐만아니라 모르는 문제가 생기거나 고민이 있을때마다 언제든 상담실로 내려가서 국/영/수 선생님께 질문할 수 있었던 점이 매우 좋았습니다.</v>
+        <v>매달 치르는 모의고사 성적표로 개인 상담을 진행했을때 과목별로 현재 부족한 점과 보완할 점을 자세히 알려주셨습니다. 뿐만아니라 모르는 문제가 생기거나 고민이 있을때마다 언제든 상담실로 내려가서 국/영/수 선생님께 질문할 수 있었던 점이 매우 좋았습니다.</v>
       </c>
       <c r="F82" t="str">
         <v>저는 수학선생님께 가장 많이 질문했지만 국어,영어,지구과학 선생님도 학원에 계셨기에 언제든 1:1로 질의응답이 가능했습니다. 혼자 공부하다가 모르는 문제가 생기면 편하게 질문할 수 있어서 좋았고 학원을 다니지않고 혼자 개인적으로 공부하기보다 선생님께 질문하면서 배워나가는 과정이 중요하다고 생각하기때문에 유용했습니다.</v>
@@ -3366,7 +3366,7 @@
         <v>항상 제 터무니없는 질문들도 너그럽게 받아주셔서 너무 감사했습니다. 특히 수학선생님의 수학 특강이 정말 많은 도움이 되었고 실제로 수능장에서도 써먹은 것이 정말 많았습니다!! 덕분에 행복한 대학생활 하고있는것 같아요 ㅎ감사합니다</v>
       </c>
       <c r="J82" t="str">
-        <v>매달 치르는 모의고사 성적표로 개인 상담을 진행했을때 과목별로 현재 부족한 점과 보안할 점을 자세히 알려주셨어요.</v>
+        <v>매달 치르는 모의고사 성적표로 개인 상담을 진행했을때 과목별로 현재 부족한 점과 보완할 점을 자세히 알려주셨어요.</v>
       </c>
       <c r="K82" t="str">
         <v>모의고사</v>
@@ -3396,7 +3396,7 @@
         <v>면학 분위기가 잘 조성되어 있어 자연스럽게 공부에 집중할 수 있었고 흐트러지지 않고 학습을 이어갈 수 있었다. 특히 졸음 관리를 위해 하루에 20분씩 두 번 짧게 휴식을 취할 수 있었던게  피로를 효과적으로 해소할 수 있었고 그 덕분에 공부할 때 잠오고 집중이 안되는 상태로 억지로 이어나가는 것이 아닌  더 또렷한 상태로 집중력을 유지할 수 있었다</v>
       </c>
       <c r="H83" t="str">
-        <v>영어가 절대평가다보니 공부시간이 다른 과목에 비해 적었고 특히 고3이 되니 영단어에 소홀해져서 스스로 외우는 시간이 줄어들어 독해를 할 때 종종 어려움을 겪었었는데 보카 테스트를 통해 매일 꾸준히 단어를 점검할 수 있었고 반복 학습이 자연스럽게 이루어져 암기 효율이 높아졌다.</v>
+        <v>영어가 절대평가다보니 공부 시간이 다른 과목에 비해 적었고 특히 고3이 되니 영단어에 소홀해져서 스스로 외우는 시간이 줄어들어 독해를 할 때 종종 어려움을 겪었었는데 보카 테스트를 통해 매일 꾸준히 단어를 점검할 수 있었고 반복 학습이 자연스럽게 이루어져 암기 효율이 높아졌다.</v>
       </c>
       <c r="I83" t="str">
         <v>학습과 생활 전반을 꼼꼼히 챙겨 주셔서 진심으로 감사드립니다. 고3 재학생인지라 학교에서 수시를 쓰고 공부하지 않는 친구들도 많았는데 덕분에 흔들리지 않고 꾸준히 공부할 수 있었습니다. 수능공부릉 한번도 해보지 않았던 제가 공부를 하다가 흔들릴때도 스스로에 대한 믿음을 가질 수 있었습니다. 앞으로도 배운 점을 바탕으로 더 성실하게 노력하겠습니다.</v>
@@ -3422,19 +3422,19 @@
         <v>N수생</v>
       </c>
       <c r="E84" t="str">
-        <v>예를 들어 제 약점과목이었던 국어의 경우 담임선생님과의 상담을 통해 어떤강사의 인강을추천해주시는지를 현재 제 상태에 맞게 알려주시고 타과목들또한 제 당시수준에 맞추어 학습설계를 해주신점이 좋았습니다</v>
+        <v>예를 들어 제 약점과목이었던 국어의 경우 담임 선생님과의 상담을 통해 어떤강사의 인강을추천해주시는지를 현재 제 상태에 맞게 알려주시고 타과목들또한 제 당시수준에 맞추어 학습설계를 해주신점이 좋았습니다</v>
       </c>
       <c r="F84" t="str">
-        <v>모의고사 시행직후 담임선생님과의 상담을 통해 현재 학습수준을 판단하고 이를 토대로 수준에 맞게 인강강사와 커리큘럼을 구체적으로 과목별로 상담해주셔서 좋았고, 추천뿐만 아니라 모의고사전까지 들었던 강의들에대한 진단? 상담?도 해주셔서 좋았습니다</v>
+        <v>모의고사 시행직후 담임 선생님과의 상담을 통해 현재 학습수준을 판단하고 이를 토대로 수준에 맞게 인강강사와 커리큘럼을 구체적으로 과목별로 상담해주셔서 좋았고, 추천뿐만 아니라 모의고사전까지 들었던 강의들에대한 진단? 상담?도 해주셔서 좋았습니다</v>
       </c>
       <c r="G84" t="str">
-        <v>기본적으로 매달 정기휴가를 제외하고는 대입실에 휴대폰을 보관하도록하니 이게 기숙학원의 큰장점이라고 느꼈고, 휴대폰 사용 적발시 바로 퇴원조치라는 강한 규정이 있어서 더욱 공부에 집중할수있었던것 같습니다</v>
+        <v>기본적으로 매달 정기휴가를 제외하고는 대입실에 휴대폰을 보관하도록하니 이게 기숙학원의 큰장점이라고 느꼈고, 휴대폰 사용 적발시 바로 퇴원조치라는 강한 규정이 있어서 더욱 공부에 집중할 수있었던것 같습니다</v>
       </c>
       <c r="H84" t="str">
         <v>메가스터디와 이투스 패스를 둘다 사용한 저로써 대표적으로 이투스의 국어박광일 강사의 강의가 매우 도움이많이됐고, 다른 타과목의 강사진들 또한 경쟁력있으신분들이 많아서 좋았던것같습니다</v>
       </c>
       <c r="I84" t="str">
-        <v>Tm반 담임 송상윤 선생님 1년동안 열정과 관심으로 저희 tm반 신경쓰고 관리해주셔서 감사했습니다. 종례때마다 해주시는 덕담과 조언이 재수생활 많은 도움이 됐던것 같습니다. 뿐만 아니라 주간,야간,타반 전략 담임선생님분들 모두 1년동안 감사했습니다</v>
+        <v>Tm반 담임 송상윤 선생님 1년 동안 열정과 관심으로 저희 tm반 신경쓰고 관리해주셔서 감사했습니다. 종례때마다 해주시는 덕담과 조언이 재수 생활 많은 도움이 됐던것 같습니다. 뿐만 아니라 주간,야간,타반 전략 담임 선생님분들 모두 1년 동안 감사했습니다</v>
       </c>
       <c r="J84" t="str">
         <v>종례 때마다 해주시는 덕담과 조언이 재수 생활에 많은 도움이 됐던것 같아요.</v>
@@ -3529,21 +3529,21 @@
         <v>N수생</v>
       </c>
       <c r="E87" t="str">
-        <v>멘토선생님들께서 거의다 재수생활을 하셨던 경험이 있으셔서 제가 들려리는 학습에 관한 고민들에대해서 공감해주시고 명쾌한 해결책들을 제시해 주셔서 학습에 관한 고민들에 대해서 해결해 주셨었습니다. 또한 생활에대한 문제들이나 집중력에대한 문제들 또한 좋은 해결책들을 제안해주셔서 너무 유용했습니다</v>
+        <v>멘토선생님들께서 거의다 재수 생활을 하셨던 경험이 있으셔서 제가 들려리는 학습에 관한 고민들에대해서 공감해주시고 명쾌한 해결책들을 제시해 주셔서 학습에 관한 고민들에 대해서 해결해 주셨었습니다. 또한 생활에대한 문제들이나 집중력에대한 문제들 또한 좋은 해결책들을 제안해주셔서 너무 유용했습니다</v>
       </c>
       <c r="F87" t="str" xml:space="preserve">
-        <v xml:space="preserve">매주 멘토선생님께서 상담을 해주시면서 생활에 관해 답답하거나 잘모르겠는 부분들을 상담해주셨었습니다. 또한 친절하고 친근하게 대해 주셔서 재수생활동안 받았던 압박들을 해소해주셨습니다. _x000d_
+        <v xml:space="preserve">매주 멘토선생님께서 상담을 해주시면서 생활에 관해 답답하거나 잘모르겠는 부분들을 상담해주셨었습니다. 또한 친절하고 친근하게 대해 주셔서 재수 생활동안 받았던 압박들을 해소해주셨습니다. _x000d_
 학습멘토 선생님들은 국어, 수학 두분이셨는데 특히나 수학에서 너무나많은 도움을 받았었습니다. 제가 잘모르는 부분이나 어려워하는 유형의 문제들을 친절히 설명해주셨습니다.</v>
       </c>
       <c r="G87" t="str">
         <v>평소 공부할때 핸드폰을 절제하지 못해 힘들었던 부분들이 있었습니다. 그런데 학원에서 핸드폰을 수거해서 관리해주니 핸드폰에 관련된 문제들이 전부다 사라져서 좋았습니다. 그래서 학습에 한층더 집중할 수 있어서 좋았습니다. 그리고 다른 사람들의 핸드폰으로 인한 소음들이 생기지 않아 너무 좋았습니다.</v>
       </c>
       <c r="H87" t="str" xml:space="preserve">
-        <v xml:space="preserve">재수하면서 영어공부가 가장 귀찮은 부분이고, 영어중 단어가 가장 중요한 부분인데 그걸 강제함으로써 할수있었고 그결과 공부시간을 많이 쏟지 않고도 영어에서 작년대비 좋은 성적을 얻을 수 있어서  좋았습니다. _x000d_
+        <v xml:space="preserve">재수하면서 영어공부가 가장 귀찮은 부분이고, 영어중 단어가 가장 중요한 부분인데 그걸 강제함으로써 할수있었고 그결과 공부 시간을 많이 쏟지 않고도 영어에서 작년대비 좋은 성적을 얻을 수 있어서  좋았습니다. _x000d_
 영어 단어 테스트를 하는것이 하루의 루틴으로 자리 잡아서 하다보니 강제성이 없어도 스스로 알아서 하게되었습니다.</v>
       </c>
       <c r="I87" t="str">
-        <v>1년동안 이런저런 고민거리 들어주시고 해결책을 제시해주셔서 감사했고, 불편한점을 해결해주시기 위해서 노력해주셔서 감사했습니다. 덕분에 공부에 집중할 수 있었습니다. 저 때문에 고생도 많이 하셨습니다. 앞으로 건강히 잘지내세요</v>
+        <v>1년 동안 이런저런 고민거리 들어주시고 해결책을 제시해주셔서 감사했고, 불편한점을 해결해주시기 위해서 노력해주셔서 감사했습니다. 덕분에 공부에 집중할 수 있었습니다. 저 때문에 고생도 많이 하셨습니다. 앞으로 건강히 잘지내세요</v>
       </c>
       <c r="J87" t="str">
         <v>과목별 선생님과 꾸준한 상담으로 재수 생활의 부담을 덜 수 있었고, 어려운 문제도 차근차근 해결할 수 있었어요.</v>
@@ -3572,7 +3572,7 @@
         <v>어느정도 진행했는지 스스로 체크하기 어려웠는데 멘토님들과 확인하며 양을 늘리거나 이렇게 보충할 수 있었습니다 지구과학 같은 경우 베이스가 많이 없는 상황이었는데 양을 늘리는 것을 통해 실력을 쌓아 어느정도의 점수를 획득할 수 있었습니다</v>
       </c>
       <c r="G88" t="str">
-        <v>휴대폰이 공부의 가장 큰 적인데 제출하니 공부가 흥미의 대상이 되어 내용 자체에 재미를 가지고 공부한 기억이 있습니다 저녁에 다시 가져가면서 휴대폰하며 도파민 충전을 했습니다 1년동안 최대한 집중하고 많은 시간을 확보하기 위해 꼭 필요한 재재인것 같습니다</v>
+        <v>휴대폰이 공부의 가장 큰 적인데 제출하니 공부가 흥미의 대상이 되어 내용 자체에 재미를 가지고 공부한 기억이 있습니다 저녁에 다시 가져가면서 휴대폰하며 도파민 충전을 했습니다 1년 동안 최대한 집중하고 많은 시간을 확보하기 위해 꼭 필요한 재재인것 같습니다</v>
       </c>
       <c r="H88" t="str">
         <v>적당한 난이도로 구성되어 실제 제 실력을 평가하기에 좋은 모의고사였습니다 국어를 특히 어려워했는데 분석하고 문학도 다양한 부분을 점검해볼 수 있는 기회가 되었습니다 그리고 이후 나오는 성적 분석서도 제 실력을 객관적으로 볼 수 있는 지표가 되었습니다</v>
@@ -3672,7 +3672,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E91" t="str">
-        <v>다른 학원들과는 다르게 매달 정기적상담과 2주에 한번씩 하는 학습점검들로 인해 공부를 할수밖에 없는 시스템이 조성되서 도움이 많이 되었던거 같습니다. 또 질답 시스템도 잘 갖춰져 있어서 많이 도움이 되었던거 같습니다</v>
+        <v>다른 학원들과는 다르게 매달 정기적상담과 2주에 한 번씩 하는 학습점검들로 인해 공부를 할수밖에 없는 시스템이 조성되서 도움이 많이 되었던거 같습니다. 또 질답 시스템도 잘 갖춰져 있어서 많이 도움이 되었던거 같습니다</v>
       </c>
       <c r="F91" t="str">
         <v>매달 자신이 나간 진도와 목표로 했던 진도를 확인하고 점검을 받고 새로운 목표와 계획을 수립하도록 도와주셔서 공부방향이 올바르게 가고있는지 잘 점검할수 있었고 혹시 잘못된 곳으로 가고있다면 다시 잘 잡아주셔서 좋았습니다</v>
@@ -3793,7 +3793,7 @@
         <v>수능을 5개월 앞두고 입학해 약 3개월 동안 이곳에서 공부하며 정말 많은 도움을 받았습니다. 비록 수능 2개월을 남겨두고 논술 준비를 위해 학원을 그만두게 되었지만, 짧다면 짧은 그 시간 동안 선생님들께서 보여주신 진심 어린 정성은 제 수험 생활의 큰 버팀목이었습니다. 특히 코치님께서 등원할 때마다 항상 밝은 미소로 인사를 건네주시고, 현실적인 조언으로 멘탈을 잡아주셔서 정말 든든했습니다. 무엇보다 제가 핸드폰을 사용하다 걸렸을 때도 모른 척해주시며 믿고 기회를 주셨던 배려에 진심으로 감사드립니다. 그 따뜻한 배려 덕분에 제 행동을 반성하고 남은 기간 더 집중할 수 있었습니다. 짧은 인연이었지만 저를 한 명의 제자로 소중히 아껴주신 마음 잊지 않겠습니다. 선생님들 덕분에 이투스에서 기분 좋게 공부하고 나갑니다. 정말 감사합니다!</v>
       </c>
       <c r="J94" t="str">
-        <v>개인별 1:1 상담에서 제 상황에 맞는 현실적인 피드백을 받을 수 있어 수험생활에 큰 도움이 되었어요.</v>
+        <v>개인별 1:1 상담에서 제 상황에 맞는 현실적인 피드백을 받을 수 있어 수험 생활에 큰 도움이 되었어요.</v>
       </c>
       <c r="K94" t="str">
         <v/>
@@ -3819,16 +3819,16 @@
         <v>학원에 시간을 맞춰 가야 한다는 강제성으로 아침에 알람시계의 도움 없이도 일어날수 았게되었고 잠을 효율적으로 자는 일이 잦아짐 그러지 않으면 공부의 질이 떨어지기 때문에 직접 찾아보게됨</v>
       </c>
       <c r="G95" t="str">
-        <v>출결 관리를 사람이 하는게 아닌 기계로 자동적으로 처리하다 보니 사람이 할때와는 달리 번거로움이 없고 선생님들도 이를 파악하기 쉬워져 학생 개개인에게 집중할수있었음으로 유용한점에 이를 택함</v>
+        <v>출결 관리를 사람이 하는게 아닌 기계로 자동적으로 처리하다 보니 사람이 할때와는 달리 번거로움이 없고 선생님들도 이를 파악하기 쉬워져 학생 개개인에게 집중할 수있었음으로 유용한점에 이를 택함</v>
       </c>
       <c r="H95" t="str">
         <v>나머지 3가지 컨텐츠는 진행하지 못하여 이를 선택함 하지만 모의고사를 볼때 시험장 분위기와 실전적 진행을 역설적이게도 적절한 자유도의 조화가 완벽했다는점이 칭찬할만한 범이 아닌가 싶음</v>
       </c>
       <c r="I95" t="str">
-        <v>1년동안 관리해주셔서 감사합니다 이투스덕분에 많은것을 얻고 가는것 같네요 비록 이번 수능은 실패로 끝났지만 여기서 얻은 경험을 바탕으로 마지막 수험생활 제대로 끝마치겠습니다 감사합니다</v>
+        <v>1년 동안 관리해주셔서 감사합니다 이투스덕분에 많은것을 얻고 가는것 같네요 비록 이번 수능은 실패로 끝났지만 여기서 얻은 경험을 바탕으로 마지막 수험 생활 제대로 끝마치겠습니다 감사합니다</v>
       </c>
       <c r="J95" t="str">
-        <v>담임선생님께서 수면 시간 조절하는 방법에 도움을 주셔서 생활 리듬을 바로 잡아 공부의 질과 양이 높아졌어요.</v>
+        <v>담임 선생님께서 수면 시간 조절하는 방법에 도움을 주셔서 생활 리듬을 바로 잡아 공부의 질과 양이 높아졌어요.</v>
       </c>
       <c r="K95" t="str">
         <v/>
@@ -4040,10 +4040,10 @@
         <v>이투스 247 독학재수학원을 다니며, 국어선생님께 도움을 많이 받았던 것 같습니다. 계속 봐도 이해가 되지 않았던 국어 문제가 있으면 선생님께서 개념부터 찬찬히 알려주셔서 끝으로 제 힘으로 문제를 사고하는 능력을 키워주셨던 것 같습니다!  개인적으로 국어 과외는 별로 선호하지 않는 편이었고, 헷갈리고 이해 안 가는 몇몇 문제들만 누군가 도와주셨으면 좋겠다 하는 입장이었어서 이투스의 코칭 시스템이 맘에 들었습니다.</v>
       </c>
       <c r="F101" t="str">
-        <v>앞에서 작성한 바와 같이 국영수 중심의 코칭 시스템이 특히 마음에 들었습니다. 또한 학습 보조 및 관리 측면에서는 제 성적을 누군가 지속적으로 점검해준다는 점에서 항상 긴장감을 유지하며 시험에 임할 수 있어 도움이 되었습니다. 매달 모의고사를 통해 성적을 확인하는 시간을 담임선생님과 가질 때면 떨리기도 하고, 앞으로 더 열심히 공부해야겠다는 다짐을 할 수 있는 기회가 되었어서 좋았습니다.</v>
+        <v>앞에서 작성한 바와 같이 국영수 중심의 코칭 시스템이 특히 마음에 들었습니다. 또한 학습 보조 및 관리 측면에서는 제 성적을 누군가 지속적으로 점검해준다는 점에서 항상 긴장감을 유지하며 시험에 임할 수 있어 도움이 되었습니다. 매달 모의고사를 통해 성적을 확인하는 시간을 담임 선생님과 가질 때면 떨리기도 하고, 앞으로 더 열심히 공부해야겠다는 다짐을 할 수 있는 기회가 되었어서 좋았습니다.</v>
       </c>
       <c r="G101" t="str">
-        <v>저는 수험생 때, 같은 자습실이나 교실을 쓰는 친구들이 자고 있는 분위기 속에서는 공부 의지가 떨어지는 듯한 느낌을 받았습니다. 한두명이 졸고 있어도 신경이 쓰였습니다. 같은 방의 경쟁자들까지 졸지 않고 공부하는 ’간절한 분위기‘ 속에서 공부하고 싶었기 때문입니다. 이투스247에서는 적어도 30분에 한번씩은 감독관이나 선생님들께서 돌아다니며 졸고 있는 아이들을 깨워주셨습니다. 그 덕분에 모든 친구들이 공부에만 열중할 수 있었던 것 같고, 그 점이 참 마음에 들었습니다.</v>
+        <v>저는 수험생 때, 같은 자습실이나 교실을 쓰는 친구들이 자고 있는 분위기 속에서는 공부 의지가 떨어지는 듯한 느낌을 받았습니다. 한두명이 졸고 있어도 신경이 쓰였습니다. 같은 방의 경쟁자들까지 졸지 않고 공부하는 ’간절한 분위기‘ 속에서 공부하고 싶었기 때문입니다. 이투스247에서는 적어도 30분에 한 번씩은 감독관이나 선생님들께서 돌아다니며 졸고 있는 아이들을 깨워주셨습니다. 그 덕분에 모든 친구들이 공부에만 열중할 수 있었던 것 같고, 그 점이 참 마음에 들었습니다.</v>
       </c>
       <c r="H101" t="str">
         <v>모의고사 퀄리티가 괜찮았었기 때문에 실력 점검을 위한 테스트로 좋았습니다~ 하지만 수학은 너무 어려웠습니다…🥹🥹 국어 영어 시험지 퀄리티는 정말 마음에 들었었던 것으로 기억해요! 혼자서 보는 모의고사와  학원에서 단체로 보는 모의고사는 느낌이 천차만별이기 때문에 다같이 으쌰으쌰하는 분위기 속에서 시험 보는 게 넘 좋았네용</v>
@@ -4119,10 +4119,10 @@
         <v>인강이나 이투스의 여러 학습관련 시스템 등 필요한 부분이 많이 있었는데 학원를 다니면서 이투스 구독을 할 수 있게 해줬기 때문에 인강을 들으면서 학습 정리도 하고 큐앤에이나 여러 시스템들을 통해 더 많은 도움을 받을 수 있었습니다.</v>
       </c>
       <c r="I103" t="str">
-        <v>학습습관 형성 및 성적향상을 위한 여러 지도 감사드립니다. 덕분에 전년도와는 다른 공부 습관 및 방법들을 터득하고 이를 통해 성적향상 뿐만 아니라 앞으로의 공부에 도움이 많이 될만한 것들을 얻어갈 수 있었습니다.</v>
+        <v>학습 습관 형성 및 성적 향상을 위한 여러 지도 감사드립니다. 덕분에 전년도와는 다른 공부 습관 및 방법들을 터득하고 이를 통해 성적 향상 뿐만 아니라 앞으로의 공부에 도움이 많이 될만한 것들을 얻어갈 수 있었습니다.</v>
       </c>
       <c r="J103" t="str">
-        <v>학습습관 형성 및 성적향상을 위한 여러 지도 감사드립다.</v>
+        <v>학습 습관 형성 및 성적 향상을 위한 여러 지도 감사드립다.</v>
       </c>
       <c r="K103" t="str">
         <v/>
@@ -4180,7 +4180,7 @@
         <v>선생님께서 매일 종례를 하셨는데 그때 학생들의 상태를 확인하시고 항상 명언과 같은 동기부여의 말, 응원의 말을 해주셔서 정신적으로 도움을 받았습니다. 학생들을 정말 진심으로 아끼시는 분이 담임이라 버틸 수 있었습니다.</v>
       </c>
       <c r="F105" t="str">
-        <v>어느 부분을 더 집중적으로 보완해야하는지 콕 찝어서 말씀해주셔서 부족한 점을 채울 수 있었습니다. 혼자서라면 무엇을 해야할지 막막했을텐데 선생님과 상의할  수 있었다는게 큰 도움이 되었습니다.</v>
+        <v>어느 부분을 더 집중적으로 보완해야하는지 콕 찝어서 말씀해주셔서 부족한 점을 채울 수 있었습니다. 혼자서라면 무엇을 해야 할지 막막했을텐데 선생님과 상의할  수 있었다는게 큰 도움이 되었습니다.</v>
       </c>
       <c r="G105" t="str">
         <v>기숙학원에선 주변 사람들이 자신의 목표를 위해 열심히 노력하는 모습을 보고 포기하고 싶을 때마다 다시 힘을 낼 수 있었습니다. 혼자하면 쉽게 흐트러졌을거같은데 다 같이 열심히 하는 분위기가 좋았습니다.</v>
@@ -4212,7 +4212,7 @@
         <v>N수생</v>
       </c>
       <c r="E106" t="str" xml:space="preserve">
-        <v xml:space="preserve">담임쌤이랑 매주 한번씩 공부방법,피드백,고쳐야 할점 등등 학습에 도움되는 이야기를 할 수 있어서 좋았고_x000d_
+        <v xml:space="preserve">담임쌤이랑 매주 한 번씩 공부방법,피드백,고쳐야 할점 등등 학습에 도움되는 이야기를 할 수 있어서 좋았고_x000d_
 큐엔에이도 과목마다 다양한 선생님들이랑 당일날에 바로바로 대면으로 해결할수있어서 좋있습니다</v>
       </c>
       <c r="F106" t="str" xml:space="preserve">
@@ -4220,15 +4220,15 @@
 학습량과 커리큘럼을 조정할수있어서 좋았습니다 또한 선생님들의 경험을 토대로 추천해주신 인강을 듣고 부족했던 부분을 선생님이 채워주시기도 하셔서 좋았습니다</v>
       </c>
       <c r="G106" t="str">
-        <v>고등학생때 생각해보면 스카에서나 학교에서나 휴대폰 본다고 공부시간을 날리고 집중도 못하고 그랬었는데 관리형 독재학원을 다니니 이런 부분에서 강제적으로 제한이 되니 환경적 부분에서 공부하시가 훨씬 좋아졌습니다</v>
+        <v>고등학생때 생각해보면 스카에서나 학교에서나 휴대폰 본다고 공부 시간을 날리고 집중도 못하고 그랬었는데 관리형 독재학원을 다니니 이런 부분에서 강제적으로 제한이 되니 환경적 부분에서 공부하시가 훨씬 좋아졌습니다</v>
       </c>
       <c r="H106" t="str" xml:space="preserve">
         <v xml:space="preserve">하반기에 이투스 모의고사를 통해 _x000d_
-지금 내 실력이 어떤지 확인할수있게 되었고 피드백을 통해 부족한 부분을 채우면서 성적 향상에 지름길이 되었던거 같아서 좋았습니다 하반기로 갈수록 공부시간에 모의고사 분량이 늘어나는데 _x000d_
+지금 내 실력이 어떤지 확인할수있게 되었고 피드백을 통해 부족한 부분을 채우면서 성적 향상에 지름길이 되었던거 같아서 좋았습니다 하반기로 갈수록 공부 시간에 모의고사 분량이 늘어나는데 _x000d_
 퀄리티 좋은 모의고사로 수능대비를 할수있어서 좋았습니다</v>
       </c>
       <c r="I106" t="str" xml:space="preserve">
-        <v xml:space="preserve">1년동안 함께 달려주셔서 감사했습니다_x000d_
+        <v xml:space="preserve">1년 동안 함께 달려주셔서 감사했습니다_x000d_
 아쉽게도 수능에서는 높은 성과를 내지는 못하였지만 재수경험을 발판삼아 더 높은 목표를 향해 달려갈수있게 되었습니다 _x000d_
 모두 감사했고 수고하셨습니다</v>
       </c>
@@ -4259,7 +4259,7 @@
         <v>다른 친구들은 방심하다가 놓칠 수도 있는 평가원 모의고사나 유명한 사설 모의고사, 학원에서만 받을 수 있는 간쓸개 같은 프로그램을 시즌마다 복도에 붙여 놓치는 일 없도록 도와주신 점이 학습에 차질이 생기지 않게 해주셨다고 생각합니다</v>
       </c>
       <c r="G107" t="str">
-        <v>핸드폰을 갖게 되면 사진 찍거나 잠깐 연락하다가 공부시간을 통으로 날리게 되는데, 핸드폰을 사용하지 못하며 아이패드에도 방화벽이 적용되어 할 수 있는 것이 공부밖에 없는 것이 좋았고 도움이 많이 되었습니다</v>
+        <v>핸드폰을 갖게 되면 사진 찍거나 잠깐 연락하다가 공부 시간을 통으로 날리게 되는데, 핸드폰을 사용하지 못하며 아이패드에도 방화벽이 적용되어 할 수 있는 것이 공부밖에 없는 것이 좋았고 도움이 많이 되었습니다</v>
       </c>
       <c r="H107" t="str">
         <v>단어시험은 강제성이 부여되지 않으면 하루하루 꾸준히 하기 힘든데 점심시간에 나갔다 오면 자리에 놓여있는 시험지때문에 하기싫은 날이라도 외워서 시험을 보는 것이 꾸준함에 도움이 됐습니다</v>
@@ -4339,7 +4339,7 @@
         <v>1년이라는 긴 시간 동안 지치지 않게 곁에서 이끌어주신 선생님들께 진심으로 감사드립니다. 단순히 지식을 전달해주시는 것을 넘어, 따뜻한 격려와 세심한 생활 관리로 무너질 뻔한 의지를 다잡아주신 덕분에 끝까지 완주할 수 있었던 거 같아요.</v>
       </c>
       <c r="J109" t="str">
-        <v>생활 상담을 통해 흐트러진 습관을 바로잡고, 동기부여를 받으며 수험생활을 끝까지 이어갈 힘을 얻었어요.</v>
+        <v>생활 상담을 통해 흐트러진 습관을 바로잡고, 동기부여를 받으며 수험 생활을 끝까지 이어갈 힘을 얻었어요.</v>
       </c>
       <c r="K109" t="str">
         <v>생활 관리</v>
@@ -4371,7 +4371,7 @@
         <v>평소에 의지박약으로 단어를 외웠다가 안외웠다가 갈팡질팡 공부했었는데 학원을 다니면서 의무적으로 매일 아침마다 보는 단어시험으로 비몽사몽한 뇌를 깨우는 데에도 매우 도움이되었고 단어도 처음으로 꾸준히 암기 할 수 있었던 부분에서 매우 유용했습니다.</v>
       </c>
       <c r="I110" t="str">
-        <v>평소에 몸이 자주 안 좋아 아팠었는데 그럼에도 불구하고, 그런 저를 수험생활 끝까지 다정하게 잘 관리해주시고 이끌어주시고 감독해주셔서 입시의 끝을 합격으로 만들어주셔서 정말 감사합니다!</v>
+        <v>평소에 몸이 자주 안 좋아 아팠었는데 그럼에도 불구하고, 그런 저를 수험 생활 끝까지 다정하게 잘 관리해주시고 이끌어주시고 감독해주셔서 입시의 끝을 합격으로 만들어주셔서 정말 감사합니다!</v>
       </c>
       <c r="J110" t="str">
         <v>생활 관리와 맞춤 학습 코칭 덕분에 올바른 공부 습관이 생기고 집중력이 올라가서 합격까지 이어졌어요.</v>
@@ -4476,7 +4476,7 @@
         <v>이투스 무료 구독권을 통해서 듣고 싶었던 강의를 마음 편히 들을 수 있었습니다. 이투스 패스를 사기에는 부담스러웠는데, 학원에서 제공해 주어서 좋았습니다. 덕분에 부족한 점을 메꿀 수 있었고, 실력이 향상되었습니다.</v>
       </c>
       <c r="I113" t="str">
-        <v>1년동안 변함없이 응원해주시고, 코칭해주신 선생님들 감사합니다! 불편한 부분들을 말씀드리면 곧바로 해결해주셔서 생활의 질이 높은 수험 생활이 되었던 것 같습니다. 부족한 부분들에 대해 함께 의논해 주시고, 격려해 주셔서 감사합니다.</v>
+        <v>1년 동안 변함없이 응원해주시고, 코칭해주신 선생님들 감사합니다! 불편한 부분들을 말씀드리면 곧바로 해결해주셔서 생활의 질이 높은 수험 생활이 되었던 것 같습니다. 부족한 부분들에 대해 함께 의논해 주시고, 격려해 주셔서 감사합니다.</v>
       </c>
       <c r="J113" t="str">
         <v>휴대폰 수거와 와이파이 방화벽 시스템으로 학습 맞춤 환경 덕분에 온전히 공부에만 집중할 수 있었어요.</v>
@@ -4502,7 +4502,7 @@
         <v>원서를 어디에 써야하는지 몰라서 헤매고 있을 때 상담을 성적에 맞게 잘 해주셔서 너무 좋았습니다. 생각지도 못한 방법을 제시해주신 부분도 있어서 안심할 수 있었습니다. 모르는 부분도 잘 알려주시고, 앞으로의 방향성도 계속 잡아주셔서 좋았습니다.</v>
       </c>
       <c r="F114" t="str">
-        <v>일주일마다 한번씩 상담 해주셨습니다. 제가 쓴 플래너를 보시고 공부를 잘 하고 있는지 미흡한 부분은 어디인지 알려주셔서 좋았습니다. 제가 저번주에 공부한 부분도 가끔 물어보셔서 그 질문에 답할려고 자동적으로 복습까지 하게 되어서 좋았습니다.</v>
+        <v>일주일마다 한 번씩 상담 해주셨습니다. 제가 쓴 플래너를 보시고 공부를 잘 하고 있는지 미흡한 부분은 어디인지 알려주셔서 좋았습니다. 제가 저번주에 공부한 부분도 가끔 물어보셔서 그 질문에 답할려고 자동적으로 복습까지 하게 되어서 좋았습니다.</v>
       </c>
       <c r="G114" t="str">
         <v>공부하는 공간에서 졸고 있으면 깨워주셔서 좋았습니다. 1시간 정도 텀을 두면서 계속 돌아다니면서 깨워주셔서 정말 많이 도움이 되었습니다. 너무 졸리면 쉬는 방에서 자도 되는데 거기도 가끔 들어오셔서 깨워주셔서 딱 피곤함만 사라지게 잘 수 있어서 너무 좋았습니다.</v>
@@ -4577,7 +4577,7 @@
         <v>제가 어떤 부분을 어떻게 모르는지를 정확히 알려드리고 그에 대한 피드백을 정확히 받을 수 있어서 좋았습니다 또한 실시간으로 진행되었기 때문에 온라인으로 진행되는 Q&amp;A와 같은 제도 보다 더 유용했습니다</v>
       </c>
       <c r="F116" t="str">
-        <v>어떤 방향으로 공부를 해나갈지에 대한 고민이 있었는데 제 상황에 맞게 어떤 문제집을 풀고 어떻게 공부해야할지 알려주셔서 좋았습니다 그게 특정 과목이 아니라 전과목을 기준으로 이루어졌기 때문에 학습에 큰 도움이 되었습니다</v>
+        <v>어떤 방향으로 공부를 해나갈지에 대한 고민이 있었는데 제 상황에 맞게 어떤 문제집을 풀고 어떻게 공부해야 할지 알려주셔서 좋았습니다 그게 특정 과목이 아니라 전과목을 기준으로 이루어졌기 때문에 학습에 큰 도움이 되었습니다</v>
       </c>
       <c r="G116" t="str">
         <v>옆에서 자고 졸면 학습 분위기에 방해가 되었기 때문에 일반 스터디카페를 지양했었는데, 이투스 관리 시스템 덕분에 모두가 공부에 집중하는 분위기 속에서 학습을 진행하였기 때문에 학습 효율을 향상할 수 있었던 점이 좋았습니다</v>
@@ -4651,17 +4651,17 @@
 근데 내 수준에서 듣기엔 너무 어려운 내용들이었고 그런 것들을 파악해서 알려주셔서 내 수준에 맞는 공부를 할 수 있었다</v>
       </c>
       <c r="G118" t="str">
-        <v>혼자 공부하게 되면 옆에 공부하고 있는 사람들이 보이지 않아서 자꾸 딴짓을 하게 되고 집중도 잘 못하다가 집에 가는 경우가 많았다 근데 학원 내에서는 실장님들이 조는 사람들은 깨우고 딴 짓도 못하도록 관리해 주시니까 다들 열심히 공부하고 있어서 나도 그 분위기에 따라 공부를 열심히 하게 됐다 그래서 딴짓하는 시간이 줄어서 공부시간도 늘어나고 공부의 질도 올라가는 것 같았다</v>
+        <v>혼자 공부하게 되면 옆에 공부하고 있는 사람들이 보이지 않아서 자꾸 딴짓을 하게 되고 집중도 잘 못하다가 집에 가는 경우가 많았다 근데 학원 내에서는 실장님들이 조는 사람들은 깨우고 딴 짓도 못하도록 관리해 주시니까 다들 열심히 공부하고 있어서 나도 그 분위기에 따라 공부를 열심히 하게 됐다 그래서 딴짓하는 시간이 줄어서 공부 시간도 늘어나고 공부의 질도 올라가는 것 같았다</v>
       </c>
       <c r="H118" t="str">
         <v>이투스 모의고사를 보면서 나의 실력을 체크할 수 있고 어려워하는 부분이나 잘 모르는 부분을 체크할 수 있으며 어느부분이 부족한지 파악하고 그 부분을 중점적으로 공부할 수 있도록 도와준 것 같다</v>
       </c>
       <c r="I118" t="str" xml:space="preserve">
-        <v xml:space="preserve">삭막한 재수생활에 원장님과 실장님들이 친근하게 말 걸어주셔서 너무 감사했어요 그리고 한 번도 가져본 적 없던 규칙적인 생활패턴이 생겨서 너무 도움됐어요_x000d_
+        <v xml:space="preserve">삭막한 재수 생활에 원장님과 실장님들이 친근하게 말 걸어주셔서 너무 감사했어요 그리고 한 번도 가져본 적 없던 규칙적인 생활패턴이 생겨서 너무 도움됐어요_x000d_
 뭘 요청하거나 질문을 했을 때 잘 답변해주셔서 감사합니다</v>
       </c>
       <c r="J118" t="str">
-        <v>내 수준에 맞는 강의와 공부 방향을 잡아주고, 규칙적인 생활습관 형성에 큰 도움이 됐어요.</v>
+        <v>내 수준에 맞는 강의와 공부 방향을 잡아주고, 규칙적인 생활 습관 형성에 큰 도움이 됐어요.</v>
       </c>
       <c r="K118" t="str">
         <v/>
@@ -4684,7 +4684,7 @@
         <v>3,4,5,6,7,8,9,10월 모의고사 분석 및 기타 사설 모의고사까지 모르는 문제에 대해서 질문하면 풀이를 자세하게 설명해주십니다. 또한 과목별 학습방법 및 풀이 진행 방법까지 다방면으로 도움을 주십니다.</v>
       </c>
       <c r="F119" t="str">
-        <v>개개인의 학습 태도 및 공부계획을 잡아주어 공부에 집중할 수 있도록 해주었습니다. 그리고 과목별 취약점과 개선점을 체크할때 유용했습니다. 이를 통해 과목별로 학습 방법과 풀이법을 변경해가며 성장할 수 있습니다.</v>
+        <v>개개인의 학습 태도 및 공부 계획을 잡아주어 공부에 집중할 수 있도록 해주었습니다. 그리고 과목별 취약점과 개선점을 체크할때 유용했습니다. 이를 통해 과목별로 학습 방법과 풀이법을 변경해가며 성장할 수 있습니다.</v>
       </c>
       <c r="G119" t="str">
         <v>공부에 도움이 되기도하고 방해도 되는 핸드폰을 거두어가고 오로지 아이패드, 태블릿으로만 학습을 할 수 있어서 전자기기를 사용하더라도 공부에만 집중할 수 있게 됩니다. 또한 핸드폰으로 인해 버려지는 시간도 챙길 수 있어서 좋습니다</v>
@@ -4755,7 +4755,7 @@
         <v>타 학원에 비해 다양한 과목의 선생님들이 많이 계셔서 모르는게 생겼을 때 좋았다. 개개인에 맞춰 학습 일정을 짜 주셔서 조급해하지 않으면서 나의 일정에 맞춰 꾸준히 공부할 수 있었다.</v>
       </c>
       <c r="F121" t="str">
-        <v>내 진도에 맞춰서 학습관리를 하니 다른사람을 신경쓰느라 에너지를 빼앗기지 않아서 좋았고 조급하지 않을 수 있었다. 또한 할 수 있을 만큼만 계획을 짜서 더 효율적으로 공부할 수 있었다.</v>
+        <v>내 진도에 맞춰서 학습 관리를 하니 다른사람을 신경쓰느라 에너지를 빼앗기지 않아서 좋았고 조급하지 않을 수 있었다. 또한 할 수 있을 만큼만 계획을 짜서 더 효율적으로 공부할 수 있었다.</v>
       </c>
       <c r="G121" t="str">
         <v>태블릿으로 인강을 보다가도 나도 모르는 사이에 sns의 유혹에 넘어가거나 친구들의 메시지 알람을 클릭하는 일이 많았는데 방호벽 덕분에 공부 외의 것에 시간을 버리지 않을 수 있어서 좋았다.</v>
@@ -4787,7 +4787,7 @@
         <v>N수생</v>
       </c>
       <c r="E122" t="str">
-        <v>수험생활의 기본적인 방향을 잡는 데에는 충분히 도움이 됐다. 학습 점검이나 간단한 피드백을 통해 내가 공부를 제대로 하고 있는지 점검할 수 있었고, 혼자 공부하다 보면 흐트러지기 쉬운 부분을 잡아주는 역할을 했다. 특히 완전히 방치되는 느낌이 아니라, 필요할 때 도움을 받을 수 있다는 점에서 심리적으로 안정감이 있었다. 과하게 간섭하지 않으면서도 최소한의 관리가 이루어진다는 점이 오히려 나에게는 잘 맞았던 것 같다.</v>
+        <v>수험 생활의 기본적인 방향을 잡는 데에는 충분히 도움이 됐다. 학습 점검이나 간단한 피드백을 통해 내가 공부를 제대로 하고 있는지 점검할 수 있었고, 혼자 공부하다 보면 흐트러지기 쉬운 부분을 잡아주는 역할을 했다. 특히 완전히 방치되는 느낌이 아니라, 필요할 때 도움을 받을 수 있다는 점에서 심리적으로 안정감이 있었다. 과하게 간섭하지 않으면서도 최소한의 관리가 이루어진다는 점이 오히려 나에게는 잘 맞았던 것 같다.</v>
       </c>
       <c r="F122" t="str">
         <v>성취도 진단 테스트는 내 현재 실력을 객관적으로 확인할 수 있다는 점에서 의미가 있었다. 생각보다 부족한 단원이 어디인지 명확하게 드러나서, 이후 공부 방향을 잡는 데 도움이 됐다. 다만 시험 자체가 엄청 자세한 분석까지 이어지진 않아서, 결과를 바탕으로 스스로 복습 계획을 세우는 게 중요하다고 느꼈다. 그래도 막연하게 공부하는 것보다 기준점을 잡아준다는 점에서 충분히 유용했다.</v>
@@ -4799,7 +4799,7 @@
         <v>인강 구독권을 무료로 제공해준 점은 확실히 도움이 됐다. 따로 강의를 결제하지 않아도 필요한 과목을 바로 들을 수 있어서 부담이 줄었고, 부족한 부분을 보완하는 데 유용했다. 다만 모든 강의를 다 활용하기보다는, 본인에게 필요한 강의만 선택해서 듣는 게 더 중요하다고 느꼈다. 그래도 기본적인 학습 환경을 갖춰준다는 점에서 충분히 만족스러운 혜택이었다.</v>
       </c>
       <c r="I122" t="str">
-        <v>담임선생님부터, 생활 관리 선생님들, 기숙 사감 선생님들 덕에 좋은 습관으로 공부 할 수 있었습니다!선생님들께서 항상 친절하게 대해주시고, 필요할 때마다 도움을 주셔서 감사했다. 공부를 하면서 힘들 때도 있었지만, 응원해주시고 방향을 잡아주신 덕분에 끝까지 버틸 수 있었던 것 같다. 과하게 간섭하기보다는 필요한 순간에 도움을 주시는 방식이 오히려 더 편하게 느껴졌고, 그 점이 특히 좋았다. 진심으로 감사드립니다.</v>
+        <v>담임 선생님부터, 생활 관리 선생님들, 기숙 사감 선생님들 덕에 좋은 습관으로 공부 할 수 있었습니다!선생님들께서 항상 친절하게 대해주시고, 필요할 때마다 도움을 주셔서 감사했다. 공부를 하면서 힘들 때도 있었지만, 응원해주시고 방향을 잡아주신 덕분에 끝까지 버틸 수 있었던 것 같다. 과하게 간섭하기보다는 필요한 순간에 도움을 주시는 방식이 오히려 더 편하게 느껴졌고, 그 점이 특히 좋았다. 진심으로 감사드립니다.</v>
       </c>
       <c r="J122" t="str">
         <v>일정한 생활 패턴을 유지하고, 공부에만 집중할 수 있는 환경 속에서 자연스럽게 학습 루틴을 잡을 수 있었어요.</v>
@@ -4910,11 +4910,11 @@
       </c>
       <c r="I125" t="str" xml:space="preserve">
         <v xml:space="preserve">감사했습니다_x000d_
-힘들때도 많았지만 잘 다잡아주셔서 수험생활 잘 마무리 한것 같습니다_x000d_
+힘들 때도 많았지만 잘 다잡아주셔서 수험 생활 잘 마무리 한것 같습니다_x000d_
 학습 선생님과 카윤터에 계신 선생님들 모두 정말 감사했습니다 항상 친절하게 대해주시고 잘 잡아주셔서 너무 좋았습니다</v>
       </c>
       <c r="J125" t="str">
-        <v>힘들때도 많았지만 잘 다잡아주셔서 수험생활 잘 마무리 한것 같아요.</v>
+        <v>힘들 때도 많았지만 잘 다잡아주셔서 수험 생활 잘 마무리 한것 같아요.</v>
       </c>
       <c r="K125" t="str">
         <v/>
@@ -4981,7 +4981,7 @@
         <v>1대1 질의응답시스템을 전 수학을 매우 유용하게 사용했습니다. 코칭 선생님께서 제가 모르는부분을 시원하게 잘 알려주셔서 다른 공부를 하며 있었던 스트레스와 답답함 까지 해소되는 시간으로 기억되는거 같습니다. 그리고 같이 토론형식으로 수학문제에 대해 얘기했던것이 향상에 도움이 됬습니다</v>
       </c>
       <c r="G127" t="str">
-        <v>저는 옛날부터 핸드폰같은 노는것에 대한 자제력이 좋지 못해, 고등학교 3학년때 수업시간에 공부를 하다가도 폰을 하기도 했습니다. 그런데 재수를 시작하고 여기 독서실에서 핸드폰 수거를 하니 핸드폰을 못하게되여 많이 집중할수 있게, 성장할수 있게된거같습니더 ㅣ</v>
+        <v>저는 옛날부터 핸드폰같은 노는것에 대한 자제력이 좋지 못해, 고등학교 3학년때 수업시간에 공부를 하다가도 폰을 하기도 했습니다. 그런데 재수를 시작하고 여기 독서실에서 핸드폰 수거를 하니 핸드폰을 못하게되여 많이 집중할 수 있게, 성장할수 있게된거같습니더 ㅣ</v>
       </c>
       <c r="H127" t="str">
         <v>고등학교 3학년때에는 학교에서 시행된 모의고사만 치뤘었는데 n수생이 빠진 표본이라 저의 실력을 가늠하기 어령웠습니다 하지만 이쿠스 전국모의고사라는 컨텐츠를 통해 재수생을 포함한 표본을 알수있게됬고 성적에 맞는 대학을 확인 할수있는거도 좋았습니다</v>
@@ -5010,19 +5010,19 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E128" t="str">
-        <v>평소 자습하는 습관이 없고 학원만 많은 공부습관을 가져서 어떻게 시작해야할지 막막했었다. 그런데 이투스에서 시간표를 추천해주고 어떤 교재, 방법으로 공부해야할지 방향성을 제시해줘서 공부하는 습관을 잡아가고 성적도 함께 얻을 수 있었던 것 같다</v>
+        <v>평소 자습하는 습관이 없고 학원만 많은 공부습관을 가져서 어떻게 시작해야 할지 막막했었다. 그런데 이투스에서 시간표를 추천해주고 어떤 교재, 방법으로 공부해야 할지 방향성을 제시해줘서 공부하는 습관을 잡아가고 성적도 함께 얻을 수 있었던 것 같다</v>
       </c>
       <c r="F128" t="str">
         <v>평소 영어 성적이 낮2~높3으로 애매하게 나와서 확실하게 등급을 올리고 싶었다. 이 고민을 말씀드렸고 선생님께서 강의와 교재를 추천해주셨다. 그 방법을 매일 꾸준히 하니 수능에서도  확실하게 등급을 올릴 수 있었다</v>
       </c>
       <c r="G128" t="str">
-        <v>우선 공부 흐름에 제일 방해가 되는것이 핸드폰이라고 생각한다. 그 방해 요소를 없애는 것이 공부시간에도 집중력에도 많이 도움이 된 것 같았고 그 습관을 그대로 지금도 여전히 공부하거나 집중해야될 때는 핸드폰을 다른데 두고 하게된다</v>
+        <v>우선 공부 흐름에 제일 방해가 되는것이 핸드폰이라고 생각한다. 그 방해 요소를 없애는 것이 공부 시간에도 집중력에도 많이 도움이 된 것 같았고 그 습관을 그대로 지금도 여전히 공부하거나 집중해야될 때는 핸드폰을 다른데 두고 하게된다</v>
       </c>
       <c r="H128" t="str">
         <v>매일 요일마다 다른 과목으로  수능특강이나 수능완성 등 수능에서 보는 시험과 관련된 교재로 테스트를 보는것이 사실상 가장 큰 메리트 였다고 본다. 학교에서는 딱히 수능을 위한 시험이 많이 없어서 아쉬웠지만 이투스에서는 시험형태로 보기 때문에 도움이 되었다고 생각한다</v>
       </c>
       <c r="I128" t="str">
-        <v>초반에는 자리가 불편하진 않는지 전체적인 방 분위기가 괜찮은지 계속 여쭤봐주시고 쉬는시간이나 점심시간에 계속 힘내라고 말씀해주신 덕분에 지치지 않고 수험생활을 잘 보낼 수 있었습니다 감사합니다</v>
+        <v>초반에는 자리가 불편하진 않는지 전체적인 방 분위기가 괜찮은지 계속 여쭤봐주시고 쉬는시간이나 점심시간에 계속 힘내라고 말씀해주신 덕분에 지치지 않고 수험 생활을 잘 보낼 수 있었습니다 감사합니다</v>
       </c>
       <c r="J128" t="str">
         <v>나만의 시간표와 교재·학습 방법 안내 덕분에 공부를 시작하는 방향을 잡고, 꾸준한 학습 습관까지 만들 수 있었어요.</v>
@@ -5223,10 +5223,10 @@
         <v>진학사에서 대학을 선택하는 것에 있어서 칸수만 보고 결정하는 것이 아니라 분석하는 방법을 알려준 것이 도움이 되었다. 덕분에 상향이어도 붙을 확률이 높은 상향임을 알 수 있어서 성적에 비해 아쉬운 대학을 가지 않은 거 같다.</v>
       </c>
       <c r="F134" t="str">
-        <v>원래 수기로 직접 플래너를 쓰면서 공부를 했었는데, 프로그램으로 계획을 작성을 하니까 나의 공부시간 비중, 패턴을 쉽게 파악할 수 있었다. 그래서 매주 과목 공부 비중을 신경쓰면서 계획을 짤 수 있었다.</v>
+        <v>원래 수기로 직접 플래너를 쓰면서 공부를 했었는데, 프로그램으로 계획을 작성을 하니까 나의 공부 시간 비중, 패턴을 쉽게 파악할 수 있었다. 그래서 매주 과목 공부 비중을 신경 쓰면서 계획을 짤 수 있었다.</v>
       </c>
       <c r="G134" t="str">
-        <v>공부를 할 때 제일 방해가 되는 것이 핸드폰이다. 집이나 다른 곳에서 공부를 하게 되면 핸드폰을 보게 되어 공부에 집중을 못하는 경우가 종종 발생한다.이투스 학원을 다니면서 핸드폰을 제출함으로써 공부시간은 물론 쉬는시간에도 핸드폰을 못하니까 순공시간이 늘어나게 되었다.</v>
+        <v>공부를 할 때 제일 방해가 되는 것이 핸드폰이다. 집이나 다른 곳에서 공부를 하게 되면 핸드폰을 보게 되어 공부에 집중을 못하는 경우가 종종 발생한다.이투스 학원을 다니면서 핸드폰을 제출함으로써 공부 시간은 물론 쉬는시간에도 핸드폰을 못하니까 순공시간이 늘어나게 되었다.</v>
       </c>
       <c r="H134" t="str">
         <v>영어공부 중에서 단어를 외우는 것은 중요하다. 그치만 단어를 스스로 외우는 것은 쉽지 않은 일이다. 학원에서 단어테스트를 진행함으로써 강제적으로 단어를 매일매일 외울 수 있어서 도움이 되었다.</v>
@@ -5235,7 +5235,7 @@
         <v>등원할 때, 하원할 때 항상 밝은 얼굴로 인사해주셔서 감사했어요. 짧은 인사지만 덕분에 저도 웃으면서 학원에 들어오고 나올 수 있었어요! 그리고 매번 모의고사 볼 때마다 꼼꼼하게 신경써주셔서 감사합니다.</v>
       </c>
       <c r="J134" t="str">
-        <v>MY 247에서 온라인으로 계획을 작성을 하니까 나의 공부시간 비중, 패턴을 쉽게 파악할 수 있었어요.</v>
+        <v>MY 247에서 온라인으로 계획을 작성을 하니까 나의 공부 시간 비중, 패턴을 쉽게 파악할 수 있었어요.</v>
       </c>
       <c r="K134" t="str">
         <v/>
@@ -5290,13 +5290,13 @@
         <v>N수생</v>
       </c>
       <c r="E136" t="str">
-        <v>담임선생님께서 인강으로만 공부할 경우에 템포가 느려지는 걸 방지하기 위해 다음 상담까지 해야할 분량을 다 정해주고  집중 해야 할 부분을 딱 집어주어 학습이 편하게 진행되었다. 상담뿐만이 아니라 학원 시스템에 잘 적응하도록 많이 신경써주었다</v>
+        <v>담임 선생님께서 인강으로만 공부할 경우에 템포가 느려지는 걸 방지하기 위해 다음 상담까지 해야 할 분량을 다 정해주고  집중 해야 할 부분을 딱 집어주어 학습이 편하게 진행되었다. 상담뿐만이 아니라 학원 시스템에 잘 적응하도록 많이 신경써주었다</v>
       </c>
       <c r="F136" t="str">
         <v>원래 플래너를 자주 쓰는 성격이 아니다 mbti도 완전 p라서 평소에는 절대 안쓰는데 학원에 들어오고 플래너 관리를 너무 잘해주어 J가 되었고, 덕분에 인강도 안밀리고 잘 보았다. 학원에서 나눠주는 플래너를 사용했다.</v>
       </c>
       <c r="G136" t="str">
-        <v>정말 필요한 만큼만 핸드폰 수거하는게 가장 좋았다. 점심시간과 저녁시간에는 핸드폰 사용이 가능해서 다른 학원에 비해 부담이 매우 적었다. 핸드폰 중독이 심한 사람은 핸드폰을 장시간 사용 못하면 불안하여 오히려 집중이 더 안되는데, 딱 필요한 공부시간만 수거하는게 좋았다</v>
+        <v>정말 필요한 만큼만 핸드폰 수거하는게 가장 좋았다. 점심시간과 저녁시간에는 핸드폰 사용이 가능해서 다른 학원에 비해 부담이 매우 적었다. 핸드폰 중독이 심한 사람은 핸드폰을 장시간 사용 못하면 불안하여 오히려 집중이 더 안되는데, 딱 필요한 공부 시간만 수거하는게 좋았다</v>
       </c>
       <c r="H136" t="str">
         <v>학력평가와 평가원 모의고사 뿐만 아니라 이투스 모의고사를 정기적으로 봄으로써 좋은 성적을 긴장을 놓치지 않고 유지 할 수 있었다. 모의고사도 퀄리티가 좋아서 공부 할 때도 매우 도움이 되었다</v>
@@ -5305,7 +5305,7 @@
         <v>학원에서 공부하는데 지루하지 않게 자주 이벤트를 많이 준비해주어 좋았습니다!! 계속 학원에서 공부만 하면 지루한데 유쾌한 분위기로 만들어주어 오히려 집중력 향상에 도움 되었어요!! 감사했습니다!!!</v>
       </c>
       <c r="J136" t="str">
-        <v>담임선생님께서 상담마다 학습 분량과 취약점을 확인해 주시고, 학원 시스템 적응까지 세심하게 도와주셔서 편하게 공부할 수 있었어요.</v>
+        <v>담임 선생님께서 상담마다 학습 분량과 취약점을 확인해 주시고, 학원 시스템 적응까지 세심하게 도와주셔서 편하게 공부할 수 있었어요.</v>
       </c>
       <c r="K136" t="str">
         <v/>
@@ -5449,7 +5449,7 @@
         <v>단어를 외우는 과정은 학습의 기초를 다지는 데 매우 유용했다. 특히 영어 지문을 읽을 때 모르는 단어가 줄어들어 해석 속도가 빨라졌고, 문제 풀이 시간도 단축되었다. 또한 반복적으로 단어를 암기하면서 기억력이 향상되고, 유사한 단어들까지 함께 익힐 수 있어 어휘력이 전반적으로 늘어났다. 이러한 변화는 독해뿐만 아니라 듣기와 쓰기에도 긍정적인 영향을 주었다.</v>
       </c>
       <c r="I140" t="str">
-        <v>선생님 감사합니다! 제 질문도 꼼꼼히 잘 받아주시고 문제풀이 팁같은 것도 많이 알려주셔서 감사합니다. 그리고 휴대폰을 걷고 매시간마다 졸음 관리 이런 것도 면학 분위기 형성에 많이 도움 되었습니다. 학습관리도 잘되어 많이 도움됐습니다.</v>
+        <v>선생님 감사합니다! 제 질문도 꼼꼼히 잘 받아주시고 문제풀이 팁같은 것도 많이 알려주셔서 감사합니다. 그리고 휴대폰을 걷고 매시간마다 졸음 관리 이런 것도 면학 분위기 형성에 많이 도움 되었습니다. 학습 관리도 잘되어 많이 도움됐습니다.</v>
       </c>
       <c r="J140" t="str">
         <v>모두가 같은 학습 환경을 유지해 분위기가 흐트러지지 않았고, 자연스럽게 공부에 더 집중할 수 있었어요.</v>
@@ -5543,10 +5543,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E143" t="str">
-        <v>항상 내신 공부에만 집중했어서 수능공부를 제대로 해본적이 없었다. 그 고3 여름방학에 수능공부를 하려는데 막막한 부분이 정말 많았다. 그러나 일주일에 한 두번씩 담당선생님과 상담을 하면서 과목 별 어떻게 공부하면 더 효과적인지를 알 수 있었다. 특히 국어 과목을 너무 못했어서 고민이 많았는데 담당선생님께서 어떤 순서로 풀지, 어떻게 글을 읽는게 나에게 더 효과적일지 등을 직접적으로 설명해주셔서 정말 도움이 많이 되었고 그렇게 코칭을 받고 실제로 한 두등급 성적이 향상 되었다</v>
+        <v>항상 내신 공부에만 집중했어서 수능공부를 제대로 해본적이 없었다. 그 고3 여름방학에 수능공부를 하려는데 막막한 부분이 정말 많았다. 그러나 일주일에 한 두번씩 담당 선생님과 상담을 하면서 과목 별 어떻게 공부하면 더 효과적인지를 알 수 있었다. 특히 국어 과목을 너무 못했어서 고민이 많았는데 담당 선생님께서 어떤 순서로 풀지, 어떻게 글을 읽는게 나에게 더 효과적일지 등을 직접적으로 설명해주셔서 정말 도움이 많이 되었고 그렇게 코칭을 받고 실제로 한 두등급 성적이 향상 되었다</v>
       </c>
       <c r="F143" t="str">
-        <v>담당 선생님께서 내가 풀었던 시험지를 직접 보시고 어떤점을 어떻게 풀었고 왜이렇게 생각했는지 등 자세히 물어보면서 내 약점은 무엇이고 항상 하는 실수는 왜 하게 되는지를 같이 찾아봐주시면서 내가 가장 부족한 부분이 뭔지 잘 알려주셨다. 또한 담당선생님의 노하우도 알려주시면서 그 부족한 점을 메꾸어나가게 지속적인 티칭을 하셨고 그러한 점이 성적향상에 보탬이 됐다고 생각한다.</v>
+        <v>담당 선생님께서 내가 풀었던 시험지를 직접 보시고 어떤점을 어떻게 풀었고 왜이렇게 생각했는지 등 자세히 물어보면서 내 약점은 무엇이고 항상 하는 실수는 왜 하게 되는지를 같이 찾아봐주시면서 내가 가장 부족한 부분이 뭔지 잘 알려주셨다. 또한 담당 선생님의 노하우도 알려주시면서 그 부족한 점을 메꾸어나가게 지속적인 티칭을 하셨고 그러한 점이 성적 향상에 보탬이 됐다고 생각한다.</v>
       </c>
       <c r="G143" t="str">
         <v>이투스 다니기 이전에 스카나 집에서 자율적인 공부를 했을 때 가장 공부에 방해됐던 것은 휴대폰이었다. 아무리 휴대폰을 사용하지 않으려고 꺼두고 다른 곳에 두고 공부를 해도 자꾸만 그 유혹에 이끌렸었다. 하지만 이투스를 다니면서 휴대폰을 아예 제출하고 점심/저녁 휴식 시간에도 휴대폰을 보지 않으니까 공부할 때 집중력이 눈에 띄게 향상했다.</v>
@@ -5578,7 +5578,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E144" t="str">
-        <v>고2때까지 내신 위주로 하다보니까 수능 공부는 제게 너무 생소했습니다. 하지만 겨울방학때 기본적인 틀을 잡아주는데 담임 선생님께서 도와주셨습니다. 특히 탐구 같은 경우 내신과 괴리감이 워낙 커서 이 부분을 좀 집중적으로 케어해주셨습니다. 또한 여름 방학때 본격적으로 수능 공부에 몰입할때 날씨랑 수시 원서 쓰는 시기가 다가왔기에 집중이 안되었지만 이부분을 제대로 잡아주셔서 25년도 하반기때 열심히 공부할수 있었습니다.</v>
+        <v>고2때까지 내신 위주로 하다보니까 수능 공부는 제게 너무 생소했습니다. 하지만 겨울방학때 기본적인 틀을 잡아주는데 담임 선생님께서 도와주셨습니다. 특히 탐구 같은 경우 내신과 괴리감이 워낙 커서 이 부분을 좀 집중적으로 케어해주셨습니다. 또한 여름 방학때 본격적으로 수능 공부에 몰입할때 날씨랑 수시 원서 쓰는 시기가 다가왔기에 집중이 안되었지만 이부분을 제대로 잡아주셔서 25년도 하반기때 열심히 공부할 수 있었습니다.</v>
       </c>
       <c r="F144" t="str">
         <v>처음 수능 공부를 할때 인강이 생소하여 내신에서 활용했던 마플 자습서등을 이용할려고 했습니다. 하지만 담임 선생님께서 저에게 여러 인강을 추천해 주셔서 여러모로 다양한 도움이 되었습니다. 특히 수학 같은 경우 제 성적에 맞는 실전개념서등을 추천해주셨고 이로 인해 제 9월 모의고사 성적은 6모보다 훨씬 높았습니다. 이외에 국어 인강도 추천해 주셔서 비문학 습관은 잡을수 있어서 유용했습니다.</v>
@@ -5587,13 +5587,13 @@
         <v>저는 폰 사용을 한번 하면 2시간은 금방 지나기 때문에 내신때 이로 인해 많은 손해를 보았습니다. 하지만 고3 겨울방학때 부터 이투스 247을 다니면서 폰을 거두어서 확실히 공부 하는 시간이 늘었습니다</v>
       </c>
       <c r="H144" t="str">
-        <v>이투스 인강 좋았습니다. 특히 정승제 너무 좋았고 이지영 좋았습니다. 이투스 247을 다니면서 이투스 패스를 무료로 받을수 있어서 메가패스와 함께 사용하여 제 학습에 시너지 효과를 얻었습니다</v>
+        <v>이투스 인강 좋았습니다. 특히 정승제 너무 좋았고 이지영 좋았습니다. 이투스 247을 다니면서 이투스 패스를 무료로 받을 수 있어서 메가패스와 함께 사용하여 제 학습에 시너지 효과를 얻었습니다</v>
       </c>
       <c r="I144" t="str">
-        <v>수능 끝나고 수시 면접 때문에 너무 바빠서 이투스 선생님들께 인사를 못 드려서 너무 아쉽습니다… 수능을 앞두고 하루에 12시간 이상 공부하면서 많이 외롭고 힘들때도 있어지만 이투스 선생님들 덕분에 극복할수 있었습니다. 비록 결과가 아쉽지만 정말 감사했습니다</v>
+        <v>수능 끝나고 수시 면접 때문에 너무 바빠서 이투스 선생님들께 인사를 못 드려서 너무 아쉽습니다… 수능을 앞두고 하루에 12시간 이상 공부하면서 많이 외롭고 힘들 때도 있어지만 이투스 선생님들 덕분에 극복할수 있었습니다. 비록 결과가 아쉽지만 정말 감사했습니다</v>
       </c>
       <c r="J144" t="str">
-        <v>담임선생님의 인강, 교재 추천 덕분에 제 수준에 맞게 공부해 수학 성적 향상과 국어 학습 습관 형성에 도움이 되었어요.</v>
+        <v>담임 선생님의 인강, 교재 추천 덕분에 제 수준에 맞게 공부해 수학 성적 향상과 국어 학습 습관 형성에 도움이 되었어요.</v>
       </c>
       <c r="K144" t="str">
         <v/>
@@ -5619,7 +5619,7 @@
         <v>학습 계획을 짜며 여러가지 고려할 점이 많아 혼자하기 어렵다고 생각하여 계획없이 공부하였는데 이투스 247에 와서 전문적인 선생님들이 계획을 짜주니 걱정없이 할 수 있었다. 인강에 진도나 개인의 취향 , 성격까지 고려하여 시간표를 짜주는 모습에 정말 감동받았고 이로 인해 성적을 정말 많이 향상시킬 수 있었다.</v>
       </c>
       <c r="G145" t="str">
-        <v>공부하며 졸리거나 피곤할때는 반드시 온다. 그러나 옆에서 깨워주는 사람이 있으면 다시 정신차리고 공부할 수 있다고 생각한다. 피곤하거나 졸때 한 번씩 다독여주며 응원해주는 모습이 나에게는 정말 감동이었고 공부를 할 수 있는 원동력이 되었다. 그냥 깨워주는 것이 아니라 응원해주는 조교님들 모습에서 많은 감동을 받았다.</v>
+        <v>공부하며 졸리거나 피곤할때는 반드시 온다. 그러나 옆에서 깨워주는 사람이 있으면 다시 정신차리고 공부할 수 있다고 생각한다. 피곤하거나 졸 때 한 번씩 다독여주며 응원해주는 모습이 나에게는 정말 감동이었고 공부를 할 수 있는 원동력이 되었다. 그냥 깨워주는 것이 아니라 응원해주는 조교님들 모습에서 많은 감동을 받았다.</v>
       </c>
       <c r="H145" t="str">
         <v>이투스 전국 모의고사는 실제 수능과 유사한 난이도와 출제 경향을 반영해 실전 대비에 효과적이며, 상세한 성적 분석과 약점 파악이 가능해 학습 방향 설정에 도움을 주었다. 학원에서 다른 학생들과 함께 푸니 더욱 실전같고 도움이 되었다.</v>
@@ -5690,7 +5690,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E147" t="str">
-        <v>늦은 시간까지 공부를 하다보니까 낮에 잠이 많이 오는 상황이었음. 카페인 섭취를 많이 하다보니까 건강이 안 좋아져서 카페인 섭취를 줄이려고 했는데 피곤해서 어떻게 해야할지 고민인 상황이었는데 생활 상담을 통해서 해결책을 찾고 적용함.</v>
+        <v>늦은 시간까지 공부를 하다보니까 낮에 잠이 많이 오는 상황이었음. 카페인 섭취를 많이 하다보니까 건강이 안 좋아져서 카페인 섭취를 줄이려고 했는데 피곤해서 어떻게 해야 할지 고민인 상황이었는데 생활 상담을 통해서 해결책을 찾고 적용함.</v>
       </c>
       <c r="F147" t="str">
         <v>국어: 계속해서 공부를 하지만 성적이 오르지 않아 공부 방법이 잘못됐다고 생각해서 상담을 받았음. 상담 후 공부 방법을 조금 바꿨을 뿐인데 성적이 점점 오르기 시작함. 또한 문제를 볼 때 어떻게 봐야하는지, 글을 어떻게 읽어야 하는지 알려주셔서 큰 도움이 되었음</v>
@@ -5705,7 +5705,7 @@
         <v>항상 따뜻한 마음으로 지도해주시고, 공부에 집중할 수 있는 좋은 환경을 만들어주셔서 진심으로 감사드립니다. 선생님들의 세심한 배려와 응원 덕분에 더욱 성실하게 노력할 수 있었습니다.</v>
       </c>
       <c r="J147" t="str">
-        <v>국어가 가장 취약 과목이였는데, 담임선생님과의 상담을 통해 공부 방법과 글 읽는 방향을 바로 잡아 성적 향상에 큰 도움이 되었어요.</v>
+        <v>국어가 가장 취약 과목이였는데, 담임 선생님과의 상담을 통해 공부 방법과 글 읽는 방향을 바로 잡아 성적 향상에 큰 도움이 되었어요.</v>
       </c>
       <c r="K147" t="str">
         <v/>
@@ -5737,14 +5737,14 @@
         <v>제가 영어가 가장 취약한 과목이였는데 고3에는 매일 단어를 외우지 않았습니다 하지만 이투스 247학원에 오면서 매일 의무적으로 단어를 40개씩 외우게 해주셔서 영어 실력의 기본기가 갖춰지게 된거 같습니다 또 일일테스트 뿐만 아니라 토요일에 실행하는 단어 총정리 테스트를 통해 복습을 꾸준하게 진행할 수 있어서 좋았습니다</v>
       </c>
       <c r="I148" t="str" xml:space="preserve">
-        <v xml:space="preserve">재수생활 함께 해주셔서 감사합니다_x000d_
-재수생활 함께 해주셔서 감사합니다_x000d_
-재수생활 함께 해주셔서 감사합니다_x000d_
-재수생활 함께 해주셔서 감사합니다_x000d_
-재수생활 함께 해주셔서 감사합니다_x000d_
-재수생활 함께 해주셔서 감사합니다_x000d_
-재수생활 함께 해주셔서 감사합니다_x000d_
-재수생활 함께 해주셔서 감사합니다</v>
+        <v xml:space="preserve">재수 생활 함께 해주셔서 감사합니다_x000d_
+재수 생활 함께 해주셔서 감사합니다_x000d_
+재수 생활 함께 해주셔서 감사합니다_x000d_
+재수 생활 함께 해주셔서 감사합니다_x000d_
+재수 생활 함께 해주셔서 감사합니다_x000d_
+재수 생활 함께 해주셔서 감사합니다_x000d_
+재수 생활 함께 해주셔서 감사합니다_x000d_
+재수 생활 함께 해주셔서 감사합니다</v>
       </c>
       <c r="J148" t="str">
         <v>모의고사 후 바로 피드백을 받고, 궁금한 문제도 빠르게 질문하며 해결할 수 있어 공부 흐름을 이어가기 좋았어요.</v>
@@ -5767,7 +5767,7 @@
         <v>N수생</v>
       </c>
       <c r="E149" t="str">
-        <v>제가 어떻게 학습을 시작해야할지 막막했는데 한 가지 방법만 조언해주시는게 아닌, 과목별로 방향성을 잡아주셔서 저의 기존 방법과 선생님이 조언해주신 방법들이 적절히 섞일 수 있었던 점이 가장 좋았습니다!</v>
+        <v>제가 어떻게 학습을 시작해야 할지 막막했는데 한 가지 방법만 조언해주시는게 아닌, 과목별로 방향성을 잡아주셔서 저의 기존 방법과 선생님이 조언해주신 방법들이 적절히 섞일 수 있었던 점이 가장 좋았습니다!</v>
       </c>
       <c r="F149" t="str">
         <v>가장 좋았던 코칭 시스템과 연관된 내용으로 여러 방향 중에서 각각 방향에 맞는 인강이나 교재 혹은 문제 하나하나 마저도 알려주셨던게 가장 도움이 되고, 특히 문제 추천은 제가 부족한 부분을 집중적으로 채울 수 있어서 가장 유용했습니다.</v>
@@ -5802,7 +5802,7 @@
         <v>N수생</v>
       </c>
       <c r="E150" t="str">
-        <v>계획을 짜는게 쉽지 않고 지키기 쉽지 않았는데 매주 학습상황을 점검하며 계속 학습 습관을 잡아준다는게 좋았습니다 아직 입시학습을 어떻게 해야할지 잘 모르겠는 학생들에게 매우 유용한 시스템입니다.</v>
+        <v>계획을 짜는게 쉽지 않고 지키기 쉽지 않았는데 매주 학습상황을 점검하며 계속 학습 습관을 잡아준다는게 좋았습니다 아직 입시학습을 어떻게 해야 할지 잘 모르겠는 학생들에게 매우 유용한 시스템입니다.</v>
       </c>
       <c r="F150" t="str">
         <v>방금 질문에서 말한 내용과 같습니다 계속해서 학습진행도를 점검해주고 무리한 계획이었다면 조금 줄이고 널널했다면 조금 늘려주는 방식으로 나에게 맞는 학습양을 알수있었습니다 코칭시스템덕분에 1년을 잘 달렸다고 생각합니다</v>
@@ -5811,7 +5811,7 @@
         <v>아무래도 학습에서 제일 방해되는게 휴대폰이라고 생각하는데 학습할때 물리적으로 분리를 도와주니 확실히 학습에 도음이 되었습니다 원래 휴대폰이 없으면 못사는 사람인데 덕분에 좋은 결과를 얻을수있어서 정말 좋은 시스템이라고 생각합니더</v>
       </c>
       <c r="H150" t="str">
-        <v>저는 사회탐구를 수능때 봤습니다 수험생활동안 이지영선생님 수업이 꼭 듣고싶었는데 패스를 사기에는 애매하고 그렇다고 안듣자니 너무 아쉬웠습니다 하지만 학원에서 제공하는 이투스 패스로 이지영선생님을 수강하고 생윤 1등급을 달성했습니다</v>
+        <v>저는 사회탐구를 수능때 봤습니다 수험 생활동안 이지영선생님 수업이 꼭 듣고싶었는데 패스를 사기에는 애매하고 그렇다고 안듣자니 너무 아쉬웠습니다 하지만 학원에서 제공하는 이투스 패스로 이지영선생님을 수강하고 생윤 1등급을 달성했습니다</v>
       </c>
       <c r="I150" t="str">
         <v>코칭선생님에게 목표를 이뤘다고 꼭 전해드리고싶습니다 감사합니다. 제가 목표를 말하고 상담할때마다 제 걱정을 덜어주시며 힘을 주신덕분에 원하는 결과를 이룰수있었습니다. 감사합니다! 잘 지내시는지 궁금하기도하네요</v>
@@ -5837,7 +5837,7 @@
         <v>N수생</v>
       </c>
       <c r="E151" t="str">
-        <v>국어 공부가 가장하기도 어렵고 어떻게 해야할지 막막했는데 저한테 맞춰서 정말 세세하게 신경써주시면서 코핑해주셔서 좋았습니다. 코칭 할때마다 국어 공부는 어떤지 어떤부분이 잘안되는지 물어봐주셔서 공부하는데 많은 도움이 되었습니다</v>
+        <v>국어 공부가 가장하기도 어렵고 어떻게 해야 할지 막막했는데 저한테 맞춰서 정말 세세하게 신경써주시면서 코핑해주셔서 좋았습니다. 코칭 할때마다 국어 공부는 어떤지 어떤부분이 잘안되는지 물어봐주셔서 공부하는데 많은 도움이 되었습니다</v>
       </c>
       <c r="F151" t="str">
         <v>아침에 꾸준히 학습 계획을 쓰게 되면서 하루 목표 공부량과 시간을 정확히 알 수 있어서 좋았고 꾸준히 쓰다보니 진도도 안밀리고 부족한부분 보완할점도 같이 알려주셔서 공부하는데 많은 도움을 받았습니다</v>
@@ -5849,7 +5849,7 @@
         <v>혼자공부할때는 영어단어 안외우고 계속 미루게되었는데 이투스247에서는 아침마다 테스트를 보고 통과했어야하기 때문에 꾸준히 외우게되서 전보다 암기량과 암기속도 모두 좋아져서 도움이 되었습니다.</v>
       </c>
       <c r="I151" t="str">
-        <v>현역때 공부를 정말 많이 안했어서 재수를 어떻게 시작해야할지 공부는 어떻게해야하는지 정말 막막했었는데 공부법이랑 공부관리.상담 잘해주시고 1년동안 재수하는데 많은 도움주셔서 정말 감사합니다.</v>
+        <v>현역때 공부를 정말 많이 안했어서 재수를 어떻게 시작해야 할지 공부는 어떻게해야하는지 정말 막막했었는데 공부법이랑 공부관리.상담 잘해주시고 1년 동안 재수하는데 많은 도움주셔서 정말 감사합니다.</v>
       </c>
       <c r="J151" t="str">
         <v>아침마다 영단어 테스트를 보며 꾸준히 암기한 덕분에 암기량과 속도를 함께 높일 수 있었어요.</v>
@@ -5872,7 +5872,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E152" t="str">
-        <v>고3이 되고 나서 학습을 어떤 방식으로 해야할지 몰랐기에 독재 학원에 가기로 다짐했습니다. 그때 수능과 수시 준비는 다르게 하되 어떤 점을 공통으로 갖고 공부해야 하는지 왜 그렇게 해야하는 지 등 다양한 공부 방법들을 저의 수준에 맞게 알려주시고 계속 앞으로 나갈 수 있게 도와주셨습니다.</v>
+        <v>고3이 되고 나서 학습을 어떤 방식으로 해야 할지 몰랐기에 독재 학원에 가기로 다짐했습니다. 그때 수능과 수시 준비는 다르게 하되 어떤 점을 공통으로 갖고 공부해야 하는지 왜 그렇게 해야하는 지 등 다양한 공부 방법들을 저의 수준에 맞게 알려주시고 계속 앞으로 나갈 수 있게 도와주셨습니다.</v>
       </c>
       <c r="F152" t="str">
         <v>어떤 부분이 취약한지에 관해 약점부터 보고 그에 맞는 공부 방법을 많이 추천해주셨습니다. 저는 국어 부분에서 특히 문학이 엄청 약했습니다. 특히 문학에서 단어 차이로 계속 틀리니 많은 단어를 암기하는 게 아닌 계속 접하면서 활용하는 방법을 알려주시고 또한 글을 읽고 문제를 풀 때 어떤 방식으로 풀어야하는지에 관해 알려주셨습니다.</v>
@@ -5922,7 +5922,7 @@
         <v>윈터스쿨때 다니며 저의 공부 습관을 잡을 수 있었던 것 같습니다. 주기적인 학습 관리와 조언을 해주시고, 학습에 방해가 되지 않도록 휴대폰 관리, 학습 관리에 있어서 도와주신 선생님들께 감사합니다.</v>
       </c>
       <c r="J153" t="str">
-        <v>저는 공부하다가 많이 조는 유형인데 졸때마다 깨워주시는것과 공부하는 것을 관리, 감독해주시는게 도움이 많이 됐어요.</v>
+        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는것과 공부하는 것을 관리, 감독해주시는게 도움이 많이 됐어요.</v>
       </c>
       <c r="K153" t="str">
         <v/>
@@ -6030,7 +6030,7 @@
         <v>짧은 시간이었지만 모든 과목의 학습 뿐 아니라 생활 관리나 계획 수립 등 공부하는데 여러 부분을 세심하게 잘 봐주셔서 수험 성공하는데 큰 도움 되었습니다. 독학하는데 있어서 정보나 플랜 수립에 부족한 부분도 많았는데 잘 봐주셔서 감사했습니다.</v>
       </c>
       <c r="J156" t="str">
-        <v>매주 해야할 공부를 각자에 맞게 상담해주어서 도움이 되었어요.</v>
+        <v>매주 해야 할 공부를 각자에 맞게 상담해주어서 도움이 되었어요.</v>
       </c>
       <c r="K156" t="str">
         <v/>
@@ -6050,10 +6050,10 @@
         <v>반수생</v>
       </c>
       <c r="E157" t="str">
-        <v>국어 담당선생님이신 장유지쌤이 담임을 해주셨는데 공부 계획부터 방향성까지 아주 철저하게 이끌어주셨고 앞에서 문제도 풀면서 즉각적으로 피드백도 받고 혼자 할때는 공부를 이상한 방향으로 할 수도 있었을텐데 선생님이 계셔서 계속 방향을 잡아주셨던게 정말 좋았습니다</v>
+        <v>국어 담당 선생님이신 장유지쌤이 담임을 해주셨는데 공부 계획부터 방향성까지 아주 철저하게 이끌어주셨고 앞에서 문제도 풀면서 즉각적으로 피드백도 받고 혼자 할때는 공부를 이상한 방향으로 할 수도 있었을텐데 선생님이 계셔서 계속 방향을 잡아주셨던게 정말 좋았습니다</v>
       </c>
       <c r="F157" t="str">
-        <v>2주마다 담임선생님과 상담을 했던게 정말 큰 도움이 됐습니다. 만약에 혼자 공부를 했다면 내가 이 방향으로 가는것이 맞는건가? 라는 생각과 불안함이 많이 들었을텐데 계속 옆에서 방향을 잡아주셨었고, 내가 하루에 이정도 공부는 해야한다를 정해주셔서 그걸 나의 페이스대로 성실하게 할 수 있었고 그걸 계속 체크하면서 검사해주셔서 대충하지 않고 열심히 할 수 있었습니다</v>
+        <v>2주마다 담임 선생님과 상담을 했던게 정말 큰 도움이 됐습니다. 만약에 혼자 공부를 했다면 내가 이 방향으로 가는것이 맞는건가? 라는 생각과 불안함이 많이 들었을텐데 계속 옆에서 방향을 잡아주셨었고, 내가 하루에 이정도 공부는 해야한다를 정해주셔서 그걸 나의 페이스대로 성실하게 할 수 있었고 그걸 계속 체크하면서 검사해주셔서 대충하지 않고 열심히 할 수 있었습니다</v>
       </c>
       <c r="G157" t="str">
         <v>일단 원래 앉는 고정좌석이 있었는데 사실 처음에는 너무 답답하지 않을까 걱정을 많이 했었는데 생활해보니까 오히려 옆자리를 신경 쓰지 않아도 되고 집중이 너무 잘 돼서 일차적으로 그게 좋았습니다. 그리고 리프레쉬 룸이나 밖에도 서서 공부하거나 답답하지 않게 공부 할 수 있능 공간이 있는게 너무 좋았고 다들 집중해서 공부하는 모습을 보고 자극도 많이 받으면서 잘 공부했습니다</v>
@@ -6062,7 +6062,7 @@
         <v>매달 마다 이투스 모의고사를 보면서 나의 위치가 어느정도이고 내가 어느위치인지를 확인 하면서 공부를 하다보니 나의 부족한 점과 채울 부분을 많이 알게 됐다. 그리고 모의고사를 매달 보다보니 모의고사에서 많은 변수를 만나게 됐고 내가 만났던 그런 변수들이 실제 수능에서도 큰 도움이 됐습니다. 그리고 질 좋은 문제들이 매우 많았고 해설지도 양질로 매우 도움이 됐습니다</v>
       </c>
       <c r="I157" t="str">
-        <v>일단 국어, 수학 담당선생님들 너무 질문도 잘 받아주시고 제 사고의 능력을 향상시켜주셨고 다른 데스크 쌤들도 너무 친절하셨습니다. 가장 감사한건 담임선생님이셨고 많은 시간을 대화하면서 어떻게 해야 더 성적을 올릴 수 있었을까를 고민했던 시간이 꽤나 즐거웠고 기억에 남는 경험이지 않았나 싶고 너무 감사합니디</v>
+        <v>일단 국어, 수학 담당 선생님들 너무 질문도 잘 받아주시고 제 사고의 능력을 향상시켜주셨고 다른 데스크 쌤들도 너무 친절하셨습니다. 가장 감사한건 담임 선생님이셨고 많은 시간을 대화하면서 어떻게 해야 더 성적을 올릴 수 있었을까를 고민했던 시간이 꽤나 즐거웠고 기억에 남는 경험이지 않았나 싶고 너무 감사합니디</v>
       </c>
       <c r="J157" t="str">
         <v>학습 관리 시스템을 통해 제 성적과 학습 상태를 바탕으로 필요한 강의를 추천해주신 점이 큰 도움이 되었어요.</v>
@@ -6120,19 +6120,19 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E159" t="str">
-        <v>계속 공부만 하다가는 쉽게 지칠 수 있는데 생활상담을 통해서 머리를 리프레쉬 할 수 있었고, 입시생활에서 어떤 과목을 어떻게 공부하고 얼마나 할지, 과목당 공부시간배분 등 많은 부분에서 궁금하거나 의견을 묻고 싶을때 명확하게 답변을 해주셔서 도움이 많이 되었습니다.</v>
+        <v>계속 공부만 하다가는 쉽게 지칠 수 있는데 생활상담을 통해서 머리를 리프레쉬 할 수 있었고, 입시생활에서 어떤 과목을 어떻게 공부하고 얼마나 할지, 과목당 공부 시간배분 등 많은 부분에서 궁금하거나 의견을 묻고 싶을때 명확하게 답변을 해주셔서 도움이 많이 되었습니다.</v>
       </c>
       <c r="F159" t="str">
         <v>원래 플래너를 적지 않았었는데, 이투스를 다니면서 학습 플래너나 학습 일기를 통해서 본인 스스로 오늘 했던 공부나 보완할 점들을 생각할 수 있었고, 어떤 과목을 앞으로 얼마큼 공부하고, 또 어떻게 공부할지에 관해서 윤곽을 쉽게 잡을 수 있었고, 전반적인 공부의 방향을 정할 수 있어서 좋았습니다.</v>
       </c>
       <c r="G159" t="str">
-        <v>저는 공부하다가 많이 조는 유형인데 졸때마다 깨워주시는것과 공부하는 것을 관리, 감독해주시는게 도움이 많이 됐습니다. 또한 혼자 독서실을 가면 핸드폰을 보거나 공부 이외의 딴짓을 자주 하는데 핸드폰을 제출하고 독서실에 들어가고, 지속적으로 감시를 해주시는것이 무척 좋았습니다.</v>
+        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는것과 공부하는 것을 관리, 감독해주시는게 도움이 많이 됐습니다. 또한 혼자 독서실을 가면 핸드폰을 보거나 공부 이외의 딴짓을 자주 하는데 핸드폰을 제출하고 독서실에 들어가고, 지속적으로 감시를 해주시는것이 무척 좋았습니다.</v>
       </c>
       <c r="H159" t="str">
         <v>결국 수능에서의 실전 감각이 매우 중요하다고 생각하는데 저는 고3현역이여서 학원에서 다 같이 시험을 보지는 못하였지만 담당 선생님이 모의고사를 챙겨주셔서 주말에 모의고사를 풀 수 있었고, 이러한 실전 경험들이 쌓여서 매우 큰 성적 향상을 이뤄낼 수 있었다고 생각합니다. 또한 문제의 퀄리티 역시 매우 뛰어나고, EBS 반영까지 잘 되어 있어서 실전 연습을 하기에 적합하다고 생각합니다.</v>
       </c>
       <c r="I159" t="str">
-        <v>2월부터 다니기 시작해서 거의 9-10달을 다녔는데 고된 수험기간동안 항상 밝고 친절하게 대해주셔서 감사합니다 덕분에 힘든 수험생활을 잘 지낼 수 있었습니다 만약 이투스를 다니지 않았더라면 성적이 이렇게 많이 오를수도 없었다고 생각합니다. 지금 대학을 다니면서 항상 바로 앞 지하철역을 지날때마다 이투스 247 독서실과 계시던 선생님들이 생각납니다! 오히러 그때가 더 좋았었던거 같기도…..  그동안 정말 감사했습니다!!</v>
+        <v>2월부터 다니기 시작해서 거의 9-10달을 다녔는데 고된 수험기간동안 항상 밝고 친절하게 대해주셔서 감사합니다 덕분에 힘든 수험 생활을 잘 지낼 수 있었습니다 만약 이투스를 다니지 않았더라면 성적이 이렇게 많이 오를수도 없었다고 생각합니다. 지금 대학을 다니면서 항상 바로 앞 지하철역을 지날때마다 이투스 247 독서실과 계시던 선생님들이 생각납니다! 오히러 그때가 더 좋았었던거 같기도…..  그동안 정말 감사했습니다!!</v>
       </c>
       <c r="J159" t="str">
         <v>학습 상태를 꾸준히 점검해주고 안정적인 루틴을 만들어줘 공부에만 집중할 수 있었어요.</v>
@@ -6155,7 +6155,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E160" t="str">
-        <v>수험생활을 하다보면 불안함이 가장 크기 때문에 내가 지금 하고 있는 공부가 괜찮은지, 더 나은 방법은 없는지 궁금할 때가 많은데 그런 궁금증을 바로바로 해소할 수 있다는 점에서 많은 도움을 받았다.</v>
+        <v>수험 생활을 하다보면 불안함이 가장 크기 때문에 내가 지금 하고 있는 공부가 괜찮은지, 더 나은 방법은 없는지 궁금할 때가 많은데 그런 궁금증을 바로바로 해소할 수 있다는 점에서 많은 도움을 받았다.</v>
       </c>
       <c r="F160" t="str">
         <v>사실 플래너는 강제성이 없다면 빼먹기도하고 계획없이 하루를 보내게 되는데 이럴 경우 하루를 밀도있게 보내기 어렵다. 이투스에서의 관리 덕분에 플래너를 매일매일 쓰게 되고, 하루를 보내더라도 버리는 시간이 적어질 수 있었던 것 같다.</v>
@@ -6167,7 +6167,7 @@
         <v>다른 과목들에 비해서 영어 반영 비율이 적기 때문에 영어에 시간 투자를 상대적으로 덜 하게 된다. 단어 시험 덕분에 의식적으로 더 단어를 외우게 되면서 공부량이 적어졌더라도 해석을 좀 더 수월하게 할 수 있었고 한 단어장을 여러 번 반복하면서 제대로 암기할 수 있어서 큰 도움이 되었다.</v>
       </c>
       <c r="I160" t="str">
-        <v>고3생활 1년동안 불안한 적도 많았고 고민도 되게 많았었는데 항상 상담을 통해 잘 들어주시고 좋은 해결책들도 많이 주셨어서 큰 도움을 받았습니다. 자주 돌아다녀주시면서 졸릴 때 깨워주시고 분위기도 좋게 유지해주셔서 편하게 다녔던 것 같습니다. 그리고 항상 밝게 인사해주시고 응원해주셔서 하루하루 열심히 다닐 수 있었습니다. 감사합니다!</v>
+        <v>고3생활 1년 동안 불안한 적도 많았고 고민도 되게 많았었는데 항상 상담을 통해 잘 들어주시고 좋은 해결책들도 많이 주셨어서 큰 도움을 받았습니다. 자주 돌아다녀주시면서 졸릴 때 깨워주시고 분위기도 좋게 유지해주셔서 편하게 다녔던 것 같습니다. 그리고 항상 밝게 인사해주시고 응원해주셔서 하루하루 열심히 다닐 수 있었습니다. 감사합니다!</v>
       </c>
       <c r="J160" t="str">
         <v>공부 계획 짜는 법을 자세히 알려주시고, 매주 점검해 주셨어요.</v>
@@ -6190,7 +6190,7 @@
         <v>N수생</v>
       </c>
       <c r="E161" t="str">
-        <v>현재 내 상황에서 알맞는 강의 및 문제집을 추천해주시는게 굉장히 맘에 들았습니다. 솔직히 처음 공부를 시작할 때는 뭐부터 해야할지 감을 잡기 어려웠는데 덕분에 수월하게 진도를 나간 것 같아요</v>
+        <v>현재 내 상황에서 알맞는 강의 및 문제집을 추천해주시는게 굉장히 맘에 들았습니다. 솔직히 처음 공부를 시작할 때는 뭐부터 해야 할지 감을 잡기 어려웠는데 덕분에 수월하게 진도를 나간 것 같아요</v>
       </c>
       <c r="F161" t="str">
         <v>제 MBTI가 P성향인지라 계획 세우기를 엄청 어려워 했었는데, 선생님이 플래너 작성과 계획 세우기를 코칭해주시고,적극적으로 조언을 해주셔서 체계적인 학습을 수행하는데 아주 큰 도움이 되었습니다.</v>
@@ -6235,7 +6235,7 @@
         <v>내가 인스타나 유튜브같은 SNS를 자제 못하는 편인데 강제로 관리해줘서 좋았던거 같다. 또한 패드로 강의는 따로 들을 수 있어 자신이 원하는 수업은 현강으로 듣고 원하지 않는 수업은 인강으로 대체할 수 있어서 좋았다</v>
       </c>
       <c r="H162" t="str">
-        <v>더프리미엄과 서바이벌 프로와 같이 매번 모의고사를 쳐야하는데 비용이 만만치가 않다. 하지만 이투스247 재원생이라면 이투스 모의고사를 달마다 한번씩 무료로 칠수 있어 돈도 절약 할 슈 있고 퀄리티도 나쁘지 않아서 좋았다</v>
+        <v>더프리미엄과 서바이벌 프로와 같이 매번 모의고사를 쳐야하는데 비용이 만만치가 않다. 하지만 이투스247 재원생이라면 이투스 모의고사를 달마다 한 번씩 무료로 칠수 있어 돈도 절약 할 슈 있고 퀄리티도 나쁘지 않아서 좋았다</v>
       </c>
       <c r="I162" t="str">
         <v>한덕원 수학선생님 감사합니다. 또 저의 전반적인 생활을 관리해주시고 각종 다양한 샹활을 관리해주는 태민티처 감사합니다. 솔찍히 몇몇 선생님들은 조금 마음에 안들었지만 다들 열심히 한거라 그래도 감사합니다</v>
@@ -6277,7 +6277,7 @@
         <v>학생 한 명 한 명을 신경 써 주시며 도와주시고 응원해 주신 덕분에 끝까지 포기하지 않고 노력할 수 있었습니다. 올바른 공부 방법과 태도를 배울 수 있어 더욱 의미 있는 시간이었던 것 같습니다. 앞으로도 선생님들께 배운 것을 바탕으로 더 성장할 수 있도록 노력하겠습니다. 진심으로 감사드립니다!</v>
       </c>
       <c r="J163" t="str">
-        <v>고3때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던건 선생님들의 탁월한 입시전략과 상담, 생활환경 조성 덕분이었어요.</v>
+        <v>고3 때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던건 선생님들의 탁월한 입시전략과 상담, 생활환경 조성 덕분이었어요.</v>
       </c>
       <c r="K163" t="str">
         <v/>
@@ -6312,7 +6312,7 @@
         <v>낯선 기숙학원 생활에 적응하느라 몸도 마음도 힘들 때 곁에서 잡아주신 선생님들 덕분에 포기하지 않고 끝까지 완주할 수 있었습니다. 이른 새벽부터 늦은 밤까지 학생들의 사소한 고민까지 귀 기울여 주시던 그 정성 덕분에, 불안했던 수험 공부가 확신으로 바뀔 수 있었다고 생각합니다. 혼자였다면 절대 버티지 못했을 이 길을 함께 걸어주시고, 공부에만 전념할 수 있는 최고의 환경을 만들어주신 선생님들께 진심으로 깊은 감사의 인사를 전하고 싶습니다.</v>
       </c>
       <c r="J164" t="str">
-        <v>휴대폰이 공부하는데에 가장 방해되는 요인인데 입실할때 휴대폰 내고 나갈때 받을 수 있도록 철저하게 관리해주시니 정말 오직 공부에만 집중할 수 있었어요.</v>
+        <v>휴대폰이 공부하는 데에 가장 방해되는 요인인데 입실할때 휴대폰 내고 나갈때 받을 수 있도록 철저하게 관리해주시니 정말 오직 공부에만 집중할 수 있었어요.</v>
       </c>
       <c r="K164" t="str">
         <v/>
@@ -6335,7 +6335,7 @@
         <v>3월부터 이투스247에 다니게 되었는데 수능 전까지 거의 감시가 널널했던적이 없이 졸고 있으면 바로 깨워주시고 웬만한 시간에 자주 학습실에 들어와 관리를 해주시고 상담 일정도 주기적으로 매칭을 해주어 좋았다</v>
       </c>
       <c r="F165" t="str">
-        <v>모르는 문제가 있으면 이투스 어플에 들어가 바로 상담신청을 하면 조교 선생님께서 문제를 알려주어 당일에 해결을 할수 있었고 중간중간 정신적으로 힘들때 마다 저의 조교 담당 선생님과 멘탈 관리를 받아서 힘들았던 재수 생활이였지만 버틸수 있었던거 같다</v>
+        <v>모르는 문제가 있으면 이투스 어플에 들어가 바로 상담신청을 하면 조교 선생님께서 문제를 알려주어 당일에 해결을 할수 있었고 중간중간 정신적으로 힘들 때 마다 저의 조교 담당 선생님과 멘탈 관리를 받아서 힘들았던 재수 생활이였지만 버틸수 있었던거 같다</v>
       </c>
       <c r="G165" t="str">
         <v>다른 지점 같은 경우는 들리는 말로는 몰래 다른 활동을 할수 있다고 들었는데 이투스 247은 와이파이가 막혀있어 다른 사이트가 접속이 안되니 오로지 인강 사이트에 집중 할수 있었던거 같고 집중이 안될때에도 어쩔수 없이 인강만 들을수 있으니 다시 집중하여 들을수 있었던거 같다</v>
@@ -6344,7 +6344,7 @@
         <v>매일매일 단어 시험만 보는것이 아닌 우리 지점은 주마다 매주 국어 시험과 수학을 시험을 보았는데 영어 단어도 평소에 나였으면 가끔 드문드문 보았을거 같은데 매일 시험을 보게하여 도움이 되었던거 같고 수학 국어시험을 매주보아 감을 잃지 않아 성적유지 및 향상에 도움이 되었다</v>
       </c>
       <c r="I165" t="str">
-        <v>다닐때는 정말 힘들었지만 돌아보니 열심히 할수 있게 되었던거 같습니다 비록 원하는 대학까지 가지는 못하였으나 1년동안 좋은 추억이였고 앞으로 도움이 되었을 1년인거 같습니다. 감사합니다</v>
+        <v>다닐때는 정말 힘들었지만 돌아보니 열심히 할수 있게 되었던거 같습니다 비록 원하는 대학까지 가지는 못하였으나 1년 동안 좋은 추억이였고 앞으로 도움이 되었을 1년인거 같습니다. 감사합니다</v>
       </c>
       <c r="J165" t="str">
         <v>담임 선생님 덕분에 플래너 작성을 더 잘 할 수 있게 되었어요.</v>
@@ -6406,7 +6406,7 @@
         <v>입시 상담을 받으면서 상담과 코칭 시스템이었다. 정기 상담을 통해 내 약점을 정확히 파악할 수 있었고, 맞춤 피드백으로 공부 방향을 잡는 데 도움이 되었다. 또한 매일 학습 계획을 점검받으며 꾸준히 공부 습관을 유지할 수 있었던 점이 가장 유용했다.</v>
       </c>
       <c r="F167" t="str">
-        <v>학습관리 시스템은 내 공부 시간을 체계적으로 관리하고 계획-실행-피드백 과정을 반복할 수 있게 해준 점에서 유용했다. 매일 학습량과 진도를 기록하고 점검하면서 부족한 부분을 빠르게 보완할 수 있었고, 꾸준한 공부 습관을 유지하는 데 큰 도움이 되었다.</v>
+        <v>학습 관리 시스템은 내 공부 시간을 체계적으로 관리하고 계획-실행-피드백 과정을 반복할 수 있게 해준 점에서 유용했다. 매일 학습량과 진도를 기록하고 점검하면서 부족한 부분을 빠르게 보완할 수 있었고, 꾸준한 공부 습관을 유지하는 데 큰 도움이 되었다.</v>
       </c>
       <c r="G167" t="str">
         <v>졸음관리와 학습서비스는 공부 집중력을 유지하는 데 큰 도움이 되었다. 졸릴 때는 관리 시스템을 통해 바로 환기하거나 리프레시할 수 있어 흐름이 끊기지 않았고, 학습서비스를 통해 필요한 자료나 질문을 바로 해결할 수 있어 시간을 효율적으로 사용할 수 있었다.</v>
@@ -6438,7 +6438,7 @@
         <v>N수생</v>
       </c>
       <c r="E168" t="str">
-        <v>매주 해야할 공부를 각자에 맞게 상담해주어서 도움이 되었습니다. 매주 할게 생기니 스트레스 받지 않고 했던거 같습니다. 성적 상승에도 도움이 되었네요 또한 본인이 하고 싶은 공부가 있으면 그 방향도 잡아주어서 하고 싶은 공부를 할 수 있었던거 같습니다</v>
+        <v>매주 해야 할 공부를 각자에 맞게 상담해주어서 도움이 되었습니다. 매주 할게 생기니 스트레스 받지 않고 했던거 같습니다. 성적 상승에도 도움이 되었네요 또한 본인이 하고 싶은 공부가 있으면 그 방향도 잡아주어서 하고 싶은 공부를 할 수 있었던거 같습니다</v>
       </c>
       <c r="F168" t="str">
         <v>모르는 문제들을 전문가분들이 가르쳐 주니 좋았고 예약 시스템으로 질의응답 시간을 가졌기 때문에 바로바로 밀리지 않고 할 수 있었어서 좋았습니다 뿐만 아니라 문제가 아닌 전체적인 학습방법도 가르쳐주어 좋았습니다</v>
@@ -6473,16 +6473,16 @@
         <v>N수생</v>
       </c>
       <c r="E169" t="str">
-        <v>담임선생님과 함께 본인에 맞는 커리큘럼을 짜며 소통할수있어 좋았고 달별로 점검 받으며 부족한 과목의 공부량을 더 늘리거나 하는등의 즉각적인 학습 계획수정이 용이했음,또한 자주 특강을 개설하여 선택학생에게  공부중 부족한 부분을 추가로 공부할수 있도록 하게해서 좋았음.</v>
+        <v>담임 선생님과 함께 본인에 맞는 커리큘럼을 짜며 소통할수있어 좋았고 달별로 점검 받으며 부족한 과목의 공부량을 더 늘리거나 하는등의 즉각적인 학습 계획수정이 용이했음,또한 자주 특강을 개설하여 선택학생에게  공부중 부족한 부분을 추가로 공부할 수 있도록 하게해서 좋았음.</v>
       </c>
       <c r="F169" t="str">
-        <v>2주마다 학습멘토와 함께 공부를 점검하며 한무동안 소홀하거나 잘했던 부분을 확인하고 다음주의 공부게획을 점검하는 점이좋았고,학습매니저에게 공부를 점검받아야하므로 공부를 계속 하게되서 좋았고,학습 매니저에게 모르는 부분을 물어보면서 공부할수있는점도 좋았다</v>
+        <v>2주마다 학습멘토와 함께 공부를 점검하며 한무동안 소홀하거나 잘했던 부분을 확인하고 다음주의 공부게획을 점검하는 점이좋았고,학습매니저에게 공부를 점검받아야하므로 공부를 계속 하게되서 좋았고,학습 매니저에게 모르는 부분을 물어보면서 공부할 수있는점도 좋았다</v>
       </c>
       <c r="G169" t="str">
-        <v>출석할때 핸드폰을 수거해서 공부외에 사소하고 잡다한 다른 요소들을 배제할수 있어 공부에 더 집중할수있도록 환경을 만들어준 점이 좋았고,저녁에 핸드폰을 가져가면서 학원에서 공부가 끝나고 집갈때  핸드폰을 보며 마음편하게 쉴수있었던것같다</v>
+        <v>출석할때 핸드폰을 수거해서 공부외에 사소하고 잡다한 다른 요소들을 배제할수 있어 공부에 더 집중할 수있도록 환경을 만들어준 점이 좋았고,저녁에 핸드폰을 가져가면서 학원에서 공부가 끝나고 집갈때  핸드폰을 보며 마음편하게 쉴수있었던것같다</v>
       </c>
       <c r="H169" t="str" xml:space="preserve">
-        <v xml:space="preserve">매일 시험을 보게해서 학생들이 나태하고 해이해질쯤에도 공부할수있도록 공부습관을 만들어주어 큰도움이 됐고 시험에서 일정점수 이하를 받으면 재시험을 보게해서 실제 시험처럼 긴장감있는 연습을 할수있었다_x000d_
+        <v xml:space="preserve">매일 시험을 보게해서 학생들이 나태하고 해이해질쯤에도 공부할 수있도록 공부습관을 만들어주어 큰도움이 됐고 시험에서 일정점수 이하를 받으면 재시험을 보게해서 실제 시험처럼 긴장감있는 연습을 할수있었다_x000d_
 또 시험을 통해 부족한부분을 점검할수있어 공부에 정말좋았다</v>
       </c>
       <c r="I169" t="str" xml:space="preserve">
@@ -6620,7 +6620,7 @@
         <v>약 1년 동안 많은 학생들을 케어하기 힘드셨을텐데 그럼에도 항상 질문에 대해 친절하게 답변해주시고 성적이 잘 나오지 않아 답답해서 힘들어 할 때도 격려해주셔서 끝까지 포기하지 않고 꾸준히 1년을 달릴 수 있었던 것 같아서 감사합니다.</v>
       </c>
       <c r="J172" t="str">
-        <v>수시원서를 쓰기전에 한명씩 친절하게 상담을 해주셨어요.</v>
+        <v>수시원서를 쓰기전에 한 명씩 친절하게 상담을 해주셨어요.</v>
       </c>
       <c r="K172" t="str">
         <v/>
@@ -6643,7 +6643,7 @@
         <v>여러 사설 모의고사와 평가원 모의고사 등을 보았을 때 나의 수준이 어느정도인지, 취약한 과목이 무엇인지 등을 분석해주시고 어떤식으로 공부방향을 잡아야 할지를 알려주셨던게 매우 유용하였다</v>
       </c>
       <c r="F173" t="str">
-        <v>중간중간에 무엇을 해야할지 몰라 막막했던 상황이 꽤 있었는데 무엇을 하면 좋을지 명확하게 알려주셔서 낭비하는 시간 없이 재수하는 1년을 꽉꽉 채워 보낼 수 있었던 것 같아 유용했다.</v>
+        <v>중간중간에 무엇을 해야 할지 몰라 막막했던 상황이 꽤 있었는데 무엇을 하면 좋을지 명확하게 알려주셔서 낭비하는 시간 없이 재수하는 1년을 꽉꽉 채워 보낼 수 있었던 것 같아 유용했다.</v>
       </c>
       <c r="G173" t="str">
         <v>와이파이 방화벽 때문에 다른 행동을 못하니 점심시간이나 저녁시간 등 남는 시간에 제대로 된 휴식을 취하거나(수면) 부족한 공부를 하게 되어 시간을 매우 알뜰하게 쓰게된 것 같아 유용하였다.</v>
@@ -6675,7 +6675,7 @@
         <v>N수생</v>
       </c>
       <c r="E174" t="str">
-        <v>경험이 많으신 담임선생님 덕분에  공부방향을  잡고  또 숙소 친구들과  원만하게  잘 지낼 수 있어서 학습에  도움이 되었고  본인에  다시 열심히  공부한다면  이투스환경이 도움이 됩니다</v>
+        <v>경험이 많으신 담임 선생님 덕분에  공부방향을  잡고  또 숙소 친구들과  원만하게  잘 지낼 수 있어서 학습에  도움이 되었고  본인에  다시 열심히  공부한다면  이투스환경이 도움이 됩니다</v>
       </c>
       <c r="F174" t="str" xml:space="preserve">
         <v xml:space="preserve">부족한 부분이 뭔지를  잘 파악해서 상담하고 관리 해주심_x000d_
@@ -6726,14 +6726,14 @@
         <v>나는 집중력이 약한편이라 현역때는 일반 스터디카페가서 유튜브를 보며 놀면서 공부하며 공부했다고 스스로 위로를 했었는데 여기는 다 막혀있으니까 오직 학원에서는 공부만 할수있어 좋았다 이 시스템이 없었다면 아마 난 재수를 실패했을지도 모른다고 생각해서 나는 이 시스템이 가장 유용한거 같다고 생각한다.</v>
       </c>
       <c r="H175" t="str">
-        <v>거의 매달 모의고사를 보다보니까 내가 얼마나 성장했는지 알수있어 좋았고 내가 몇등인지 파악할수 있어 동기부여도 되고 열정이 더욱 더 생겨 더 열심히 할수있었던거 같다 게다가 매번 모의고사를 치면서 성적이 오르는게 눈에 보이니까 더 공부를 많이하고 공부를 하는게 즐거워졌다 이 콘텐츠를 통해 나는 매번 모의고사 성적을 올리면서 수능때 내가 받았던 성적중 가장 높은 등급을 받을수 있었던 거같아</v>
+        <v>거의 매달 모의고사를 보다보니까 내가 얼마나 성장했는지 알수있어 좋았고 내가 몇등인지 파악할수 있어 동기부여도 되고 열정이 더욱 더 생겨 더 열심히 할수있었던거 같다 게다가 매번 모의고사를 치면서 성적이 오르는게 눈에 보이니까 더 공부를 많이하고 공부를 하는게 즐거워졌다 이 콘텐츠를 통해 나는 매번 모의고사 성적을 올리면서 수능때 내가 받았던 성적중 가장 높은 등급을 받을 수 있었던 거같아</v>
       </c>
       <c r="I175" t="str" xml:space="preserve">
         <v xml:space="preserve">재수 생활 동안 늘 옆에서 지도해 주셔서 진심으로 감사드립니다. 처음에는 집중도 잘 안 되고 많이 흔들렸는데, 선생님들 덕분에 끝까지 포기하지 않고 버틸 수 있었습니다. 특히 공부에만 집중할 수 있는 환경과 꾸준히 관리해 주신 덕분에 저 스스로도 많이 달라졌다고 느낍니다._x000d_
 선생님들 덕분에 재수 성공할수 있었어요 감사합니다.</v>
       </c>
       <c r="J175" t="str">
-        <v>학원을 다니면서 집중도도 높아지고 공부시간을 더 효과적으로 사용할 수 있었어요.</v>
+        <v>학원을 다니면서 집중도도 높아지고 공부 시간을 더 효과적으로 사용할 수 있었어요.</v>
       </c>
       <c r="K175" t="str">
         <v/>
@@ -6765,7 +6765,7 @@
         <v>모의고사를 많이 볼 기회가 없었는데 이투스 모의고사가 있어서 양질의 실전 연습을 중간중간마다 할 수 있어서 실전 감각을 기르고 내 위치를 점검하고 약점을 발견하며 크게 실력이 늘을 수 있게 된 것 같다.</v>
       </c>
       <c r="I176" t="str">
-        <v>선생님께서 질문도 받아주시고 마주칠 때마다 좋은 말씀 많이 해주시고 밥 먹을 때마다 맛있게 먹으라고 따뜻하게 말해주시고 등원, 하원 할 때마다 따뜻하게 인사로 맞이해주셔서 힘든 수험생활에 큰 힘이 되었던 것 같습니다. 정말 감사드립니다!</v>
+        <v>선생님께서 질문도 받아주시고 마주칠 때마다 좋은 말씀 많이 해주시고 밥 먹을 때마다 맛있게 먹으라고 따뜻하게 말해주시고 등원, 하원 할 때마다 따뜻하게 인사로 맞이해주셔서 힘든 수험 생활에 큰 힘이 되었던 것 같습니다. 정말 감사드립니다!</v>
       </c>
       <c r="J176" t="str">
         <v>면학 분위기에 대한 관리도 세심하게 해주셔서 집중해서 공부할 수 있었어요.</v>
@@ -6826,7 +6826,7 @@
         <v>이투스247 학원에 다니면서 가장 좋았던 점은 엘리트 선생님들이 직접 멘토 역할을 해주시며 세심하게 지도해주신다는 것이었습니다. 단순히 수업만 하는 것이 아니라 성적 관리부터 학습 계획까지 함께 고민해주시고 방향을 잡아주셔서 공부에 대한 부담이 훨씬 줄었습니다. 또한 지각 관리 시스템도 체계적으로 운영되어 스스로 생활 습관을 잡는 데 큰 도움이 되었고, 전반적으로 학습 분위기가 잘 형성되어 있어 꾸준히 집중할 수 있었습니다.</v>
       </c>
       <c r="F178" t="str">
-        <v>학습관리시스템이 매우 체계적으로 운영되어 공부의 흐름을 꾸준히 유지하는 데 큰 도움이 되었습니다. 출결과 지각 관리가 엄격하게 이루어져 자연스럽게 생활 습관이 잡혔고, 개인별 학습 계획과 성적까지 꼼꼼하게 관리해주어 스스로 부족한 부분을 정확히 파악하고 보완할 수 있었습니다. 덕분에 학습 방향을 잃지 않고 꾸준히 목표를 향해 나아갈 수 있었습니다.</v>
+        <v>학습 관리시스템이 매우 체계적으로 운영되어 공부의 흐름을 꾸준히 유지하는 데 큰 도움이 되었습니다. 출결과 지각 관리가 엄격하게 이루어져 자연스럽게 생활 습관이 잡혔고, 개인별 학습 계획과 성적까지 꼼꼼하게 관리해주어 스스로 부족한 부분을 정확히 파악하고 보완할 수 있었습니다. 덕분에 학습 방향을 잃지 않고 꾸준히 목표를 향해 나아갈 수 있었습니다.</v>
       </c>
       <c r="G178" t="str">
         <v>생활 관리시스템이 매우 체계적으로 운영되어 규칙적인 생활 습관을 형성하는 데 큰 도움이 되었습니다. 출결과 지각 관리가 철저하게 이루어져 자연스럽게 시간 관리를 하게 되었고, 학습 외적인 부분까지도 세심하게 신경 써주어 흐트러지지 않고 꾸준히 생활 리듬을 유지할 수 있었습니다. 이러한 환경 덕분에 공부에 더욱 집중할 수 있었습니다.</v>
@@ -6947,7 +6947,7 @@
         <v>이른 아침부터 데스크에서 학생들을 맞아주시던 인자하신 어르신 직원분과 다른 직원분들 너무 감사합니다 ㅎㅎ 덕분에 여름에는 시원하고 겨울에는 따뜻한 환경에서 공부할 수 있었어요. 쾌적한 공부환경을 제공해 공부 외에는 신경쓰지 않아도 되게 해주셔서 감사했습니다. 그리고 대학생 코칭선생님에게도 학습 관련한 도움도 많이 받았고, 대학생같은 옷을 입고 다니시는 걸 보며 나도 올해 꼭 합격해서 대학 다녀야지 라고 결심하는 계기가 되었어요 ㅎㅎ 매일 맛있는 급식 제공해주신 급식업체 직원분들께도 감사드려요!</v>
       </c>
       <c r="J181" t="str">
-        <v>이투스247학원의 학습관리는 진짜 체계적이라 놀라웠었어요.</v>
+        <v>이투스247학원의 학습 관리는 진짜 체계적이라 놀라웠었어요.</v>
       </c>
       <c r="K181" t="str">
         <v>학습 관리</v>
@@ -6979,7 +6979,7 @@
         <v>혼자서 단어를 외우면 하기 싫은 날도 있고 작심삼일이 되었을 수도 있는데 매일 일정한 양을 외우고 시험 보는 게 좋았고 잘 외우지 못했을 땐 재시험을 보며 제대로 학습할 수 있어 유용했습니다</v>
       </c>
       <c r="I182" t="str">
-        <v>이투스247에서 함께해주신 선생님들께 진심으로 감사드립니다. 항상 따뜻하게 응원해주시고, 함께 방향을 잡아주셔서 끝까지 포기하지 않을 수 있었습니다. 세심한 상담과 진심 어린 조언 덕분에 한층 더 성장할 수 있었고, 그 과정이 큰 힘이 되었습니다. 1년동안 학습에 집중할 수 있도록 힘써주셔서 감사합니다.</v>
+        <v>이투스247에서 함께해주신 선생님들께 진심으로 감사드립니다. 항상 따뜻하게 응원해주시고, 함께 방향을 잡아주셔서 끝까지 포기하지 않을 수 있었습니다. 세심한 상담과 진심 어린 조언 덕분에 한층 더 성장할 수 있었고, 그 과정이 큰 힘이 되었습니다. 1년 동안 학습에 집중할 수 있도록 힘써주셔서 감사합니다.</v>
       </c>
       <c r="J182" t="str">
         <v>공부에 집중할 수 있는 환경을 만드는 데 큰 도움이 되었어요.</v>
@@ -7037,13 +7037,13 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E184" t="str">
-        <v>자기주도학습이 부족한 저에게 꼼꼼한 피드백을 해주시고 공부시간도 짜주셨습니다 코칭으로 몰랐던 부분을 채워가며 더 나은 학습환경이 만들어졌습니다 모르는 부분을 친절하게 답해주는 것도 좋았습니다</v>
+        <v>자기주도학습이 부족한 저에게 꼼꼼한 피드백을 해주시고 공부 시간도 짜주셨습니다 코칭으로 몰랐던 부분을 채워가며 더 나은 학습환경이 만들어졌습니다 모르는 부분을 친절하게 답해주는 것도 좋았습니다</v>
       </c>
       <c r="F184" t="str">
         <v>나에게 맞는 학습전략을 세워주며 더 효율적으로 공부할 수 있는 방법을 제공해주셨습니다 또 언제든 상담을 받을 수 있어 고민이 생기면 물어볼 수 있어서 좋았습니다 항상 친절하게 답변해주셨습니다</v>
       </c>
       <c r="G184" t="str">
-        <v>핸드폰이 공부에 제일 안좋은 물건인데 들어가자마자 핸드폰을 내는것이 제일 좋았습니다 또 졸고있을 때 깨워주시는것도 좋았습니다 또 출결관리로 지각하지 않는 습관을 만들어주는것도 좋았습니다</v>
+        <v>핸드폰이 공부에 제일 안좋은 물건인데 들어가자마자 핸드폰을 내는것이 제일 좋았습니다 또 졸고있을 때 깨워주시는것도 좋았습니다 또 출결 관리로 지각하지 않는 습관을 만들어주는것도 좋았습니다</v>
       </c>
       <c r="H184" t="str">
         <v>인강사이트를 무료로 사용할 수 있는것이 좋았고 이투스 모의고사도 칠 수 있어서 좋았습니다 사설이라 어렵긴 해도 내 위치가 어느정도인지 파악할 수 있어서 좋았습니다 또 이투스구독으로 다양한 수업을 들을 수 있는것도 좋았습니다</v>
@@ -7072,7 +7072,7 @@
         <v>반수생</v>
       </c>
       <c r="E185" t="str">
-        <v>이투스 학원에서 제공하는 멘토링 시스템이 좋았습니다. 모르는 문제가 있거나 어떻게 공부해야할지 모를때 멘토 분들이 하나하나 알려주시고 모르는 문제에 대한 해답이 바로 납득가기 쉽게 설명해주셔서 이부분이 가장 좋았던 것 같습니다</v>
+        <v>이투스 학원에서 제공하는 멘토링 시스템이 좋았습니다. 모르는 문제가 있거나 어떻게 공부해야 할지 모를때 멘토 분들이 하나하나 알려주시고 모르는 문제에 대한 해답이 바로 납득가기 쉽게 설명해주셔서 이부분이 가장 좋았던 것 같습니다</v>
       </c>
       <c r="F185" t="str" xml:space="preserve">
         <v xml:space="preserve">1:1질의응답에서 몰랐던 부분의 개념이나 활용방법 등등 알지 못했던 부분을 채워주셔서 더욱 더 배움에 있어 단단해 졌던 것 같습니다. 그리고 앞으로 공부를 어떻게 해야 할지도 알려주셔서 맘편하게_x000d_
@@ -7082,13 +7082,13 @@
         <v>학생들이 화장실에서 떠들거나 휴개실에사 떠들면 지도를 해주시고 졸거나 하면 깨워주셔서 수능시간 때 졸거나 피곤하지 않게 잘 관리해주신 것 같아 좋았습니다. 또 마음에 들지 않는 점이 있다면 잘 들어주셨습니다</v>
       </c>
       <c r="H185" t="str">
-        <v>이투스 전국모의고사를 지원해줘서 한달에 한번씩 감을 찾을 수 있었고 어느 부분이 부족한지 지표로 나오고 내가 지금 이 성적으로 어디를 갈 수 있는지 알 수 있어서 공부 의욕을 향상하는데 좋았던 것 같고</v>
+        <v>이투스 전국모의고사를 지원해줘서 한달에 한 번씩 감을 찾을 수 있었고 어느 부분이 부족한지 지표로 나오고 내가 지금 이 성적으로 어디를 갈 수 있는지 알 수 있어서 공부 의욕을 향상하는데 좋았던 것 같고</v>
       </c>
       <c r="I185" t="str">
         <v>선생님들이 부족함 없이 챙겨주셔서 편하게 학원을 다닌 것 같습니다. 몰랏던 부분 부족한 부분을 친절하게 채워주셔서 감사했습니다. 선생님들 덕분에 좋은 대학 간 것 같습니다.! 감사합니다!!</v>
       </c>
       <c r="J185" t="str">
-        <v>제가 계획을 세우면 선생님께서 보고 피드백을 주셨기 때문에 더 효율적이고 도움이 되는 공부계획을 세우고 실천할 수 있었어요.</v>
+        <v>제가 계획을 세우면 선생님께서 보고 피드백을 주셨기 때문에 더 효율적이고 도움이 되는 공부 계획을 세우고 실천할 수 있었어요.</v>
       </c>
       <c r="K185" t="str">
         <v/>
@@ -7265,7 +7265,7 @@
 고마운 존재였습니다. 결코 쉽지 않은 난이도로 항상 저를 당황시켰는데 오히려 시험준비에 더 열심히 임할 수 있었던 것 같습니다.</v>
       </c>
       <c r="I190" t="str">
-        <v>작년, 걱정과 불안이 가득한 입시상담을 받았던게 새록새록 떠오르는데 저는 지금 그 때의 상담에서 선생님께서 말씀하신 대학의 학과에 입학했습니다! 고3때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던건 이투스 강서지점 선생님들의 탁월한 입시전략과 상담, 생활환경 조성 덕분이었습니다. 저의 처음이자 마지막 재수를 성공적으로 마치게 해주신 이투스 강서지점 선생님들께 감사를 표합니다!</v>
+        <v>작년, 걱정과 불안이 가득한 입시상담을 받았던게 새록새록 떠오르는데 저는 지금 그 때의 상담에서 선생님께서 말씀하신 대학의 학과에 입학했습니다! 고3 때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던건 이투스 강서지점 선생님들의 탁월한 입시전략과 상담, 생활환경 조성 덕분이었습니다. 저의 처음이자 마지막 재수를 성공적으로 마치게 해주신 이투스 강서지점 선생님들께 감사를 표합니다!</v>
       </c>
       <c r="J190" t="str">
         <v>생활 상담을 포함한 코칭 시스템은 공부 외적인 부분까지 함께 관리해 준다는 점에서 의미가 있었어요.</v>
@@ -7288,7 +7288,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E191" t="str" xml:space="preserve">
-        <v xml:space="preserve">생활 상담이 가장 인상 깊었습니다. 단순히 공부 시간만 관리하는 것이 아니라, 수험생활 전반을 어떻게 유지해야 하는지에 대해 구체적이고 현실적으로 지도해주셔서 큰 도움이 되었습니다. 수면 시간, 식사 습관, 휴식 타이밍 같은 기본적인 생활 패턴부터 집중력이 떨어질 때 대처하는 방법까지 세세하게 알려주셔서 스스로를 관리하는 기준이 생겼습니다._x000d_
+        <v xml:space="preserve">생활 상담이 가장 인상 깊었습니다. 단순히 공부 시간만 관리하는 것이 아니라, 수험 생활 전반을 어떻게 유지해야 하는지에 대해 구체적이고 현실적으로 지도해주셔서 큰 도움이 되었습니다. 수면 시간, 식사 습관, 휴식 타이밍 같은 기본적인 생활 패턴부터 집중력이 떨어질 때 대처하는 방법까지 세세하게 알려주셔서 스스로를 관리하는 기준이 생겼습니다._x000d_
 특히 좋았던 점은 실천 가능한 수준으로 디테일하게 설명해주셨다는 점입니다. 하루 루틴을 어떻게 짜야 하는지, 쉬는 시간은 어느 정도가 적절한지, 컨디션이 무너질 때는 어떻게 회복해야 하는지 등 실제 상황을 고려한 조언을 해주셔서 바로 적용할 수 있었습니다._x000d_
 또한 단순히 규칙을 제시하는 데서 끝나는 것이 아니라, 왜 그렇게 해야 하는지 이유까지 설명해주셔서 납득하면서 생활 습관을 바꿀 수 있었습니다. 덕분에 억지로 버티는 느낌이 아니라 스스로 조절하면서 안정적으로 공부할 수 있게 되었습니다._x000d_
 전체적으로 생활 상담을 통해 공부 외적인 부분까지 체계적으로 관리할 수 있게 되었고, 그 덕분에 장기적으로 흔들리지 않고 공부를 이어갈 수 있는 힘을 얻었다고 느꼈습니다.</v>
@@ -7300,7 +7300,7 @@
 전체적으로 학습 관리 시스템이 단순한 조언이 아니라, 실제 성적 향상으로 이어질 수 있는 맞춤형 전략이라는 느낌을 받아서 매우 만족했습니다.</v>
       </c>
       <c r="G191" t="str" xml:space="preserve">
-        <v xml:space="preserve">생활 관리 측면에서 세심하게 챙겨주신 부분이 특히 좋았습니다. 단순히 공부만 강조하는 것이 아니라, 실제로 공부를 지속할 수 있는 컨디션을 유지하도록 도와주신 점이 인상 깊었습니다. 수험생활을 하다 보면 졸음이 쏟아지거나 집중력이 떨어지는 순간이 많은데, 그럴 때마다 적절하게 깨워주시고 현재 상태를 체크해주셔서 흐름이 끊기지 않도록 관리해주셨습니다._x000d_
+        <v xml:space="preserve">생활 관리 측면에서 세심하게 챙겨주신 부분이 특히 좋았습니다. 단순히 공부만 강조하는 것이 아니라, 실제로 공부를 지속할 수 있는 컨디션을 유지하도록 도와주신 점이 인상 깊었습니다. 수험 생활을 하다 보면 졸음이 쏟아지거나 집중력이 떨어지는 순간이 많은데, 그럴 때마다 적절하게 깨워주시고 현재 상태를 체크해주셔서 흐름이 끊기지 않도록 관리해주셨습니다._x000d_
 특히 “괜찮겠지” 하고 그냥 넘어갈 수 있는 부분까지도 수시로 확인해주시면서, 졸거나 집중이 흐트러질 때 바로 잡아주신 점이 도움이 많이 되었습니다. 덕분에 스스로 놓치기 쉬운 생활 리듬이나 집중 상태를 꾸준히 유지할 수 있었고, 혼자였다면 무너졌을 타이밍도 잘 넘길 수 있었습니다._x000d_
 또한 단순히 깨워주는 데서 끝나는 것이 아니라, 언제 쉬는 게 좋은지, 어떻게 다시 집중을 끌어올려야 하는지까지 함께 지도해주셔서 효율적으로 하루를 운영할 수 있었습니다. 이런 세심한 생활 관리 덕분에 공부 시간의 질 자체가 올라갔다고 느꼈습니다.</v>
       </c>
@@ -7310,11 +7310,11 @@
 또한 매일 꾸준히 쌓이는 방식이라 부담스럽지 않으면서도 학습량이 자연스럽게 누적되는 점이 인상적이었습니다. 이런 시스템 덕분에 영어 단어에 대한 기본기가 탄탄해졌고, 독해를 할 때도 훨씬 수월해졌다고 느꼈습니다.</v>
       </c>
       <c r="I191" t="str" xml:space="preserve">
-        <v xml:space="preserve">수험생활 동안 단순히 공부만 도와주신 것이 아니라, 방향을 잃지 않도록 계속해서 이끌어주시고 세심하게 관리해주신 덕분에 끝까지 버틸 수 있었습니다. 항상 학생 한 명 한 명의 상태를 신경 써주시고, 필요한 부분을 놓치지 않고 챙겨주시는 모습이 정말 인상 깊었습니다._x000d_
-공부뿐만 아니라 생활적인 부분까지 꼼꼼하게 지도해주셔서 안정적으로 수험생활을 이어갈 수 있었고, 힘들 때마다 해주신 말 한마디, 작은 관심 하나가 큰 힘이 되었습니다. 덕분에 포기하지 않고 계속 나아갈 수 있었던 것 같습니다.</v>
+        <v xml:space="preserve">수험 생활 동안 단순히 공부만 도와주신 것이 아니라, 방향을 잃지 않도록 계속해서 이끌어주시고 세심하게 관리해주신 덕분에 끝까지 버틸 수 있었습니다. 항상 학생 한 명 한 명의 상태를 신경 써주시고, 필요한 부분을 놓치지 않고 챙겨주시는 모습이 정말 인상 깊었습니다._x000d_
+공부뿐만 아니라 생활적인 부분까지 꼼꼼하게 지도해주셔서 안정적으로 수험 생활을 이어갈 수 있었고, 힘들 때마다 해주신 말 한마디, 작은 관심 하나가 큰 힘이 되었습니다. 덕분에 포기하지 않고 계속 나아갈 수 있었던 것 같습니다.</v>
       </c>
       <c r="J191" t="str">
-        <v>혼자 공부했으면 하루를 어떻게 보내야 할지 효율적으로 계획하는 것이 힘들었을 텐데 일주일 단위로 공부해야할 것을 계획할 수 있어서 좋았어요.</v>
+        <v>혼자 공부했으면 하루를 어떻게 보내야 할지 효율적으로 계획하는 것이 힘들었을 텐데 일주일 단위로 공부해야 할 것을 계획할 수 있어서 좋았어요.</v>
       </c>
       <c r="K191" t="str">
         <v/>
@@ -7334,7 +7334,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E192" t="str">
-        <v>원장선생님과 상담할 때 정말 평소 쌓였던 고민들과 걱정이 모두 뻥 사라지는 느낌이었습니다. 수시와 정시를 둘 다 챙기는 게 맞을 지, 과학 공부 방법과 등급 상승 방법 등등 혼자 끙끙 앓던 것들을 질문하니까 정말 명료하게 해결해주셨던 기억이 납니다. 잘하고 있다고 항상 응원해주시고 격려 많이해주셔서 학원 상담이 기다려졌던 것 같네요!</v>
+        <v>원장 선생님과 상담할 때 정말 평소 쌓였던 고민들과 걱정이 모두 뻥 사라지는 느낌이었습니다. 수시와 정시를 둘 다 챙기는 게 맞을 지, 과학 공부 방법과 등급 상승 방법 등등 혼자 끙끙 앓던 것들을 질문하니까 정말 명료하게 해결해주셨던 기억이 납니다. 잘하고 있다고 항상 응원해주시고 격려 많이해주셔서 학원 상담이 기다려졌던 것 같네요!</v>
       </c>
       <c r="F192" t="str">
         <v>평소 궁금했던 것을 해결할 수 있는 점이 좋았고 팁 주신 것들을 다음주에 다시 여쭤보시니까 더 열심히 지키려고 노력했던 것 같습니다. 개인적으로 봐주시는 시간이 있어서 성적 상승과 동기부여에 좋은 영향을 미쳤던 것 같습니다.</v>
@@ -7369,7 +7369,7 @@
         <v>N수생</v>
       </c>
       <c r="E193" t="str">
-        <v>매주 정기적으로 듣고 싶은 과목의 선생님과 학습 상담을 할 수 있어서 좋았습니다. 매일 앉아서 공부만 하다보니 내가 지금 잘하고 있는 건가 하는 불안감에 오히려 공부에 집중을 하지 못할때가 있었는데 그럴때마다 배정받은 과목 선생님께 가서 상담을 하면서 다시 마음을 다잡고 공부할수 있었습니다.</v>
+        <v>매주 정기적으로 듣고 싶은 과목의 선생님과 학습 상담을 할 수 있어서 좋았습니다. 매일 앉아서 공부만 하다보니 내가 지금 잘하고 있는 건가 하는 불안감에 오히려 공부에 집중을 하지 못할때가 있었는데 그럴때마다 배정받은 과목 선생님께 가서 상담을 하면서 다시 마음을 다잡고 공부할 수 있었습니다.</v>
       </c>
       <c r="F193" t="str">
         <v>독학 기숙인데도 불구하고 주요 과목 강사님들과 일대일 질문시간을 가질 수 있어서 궁금한 문제에 대한 선생님의 답변시간을 기다리느라 시간을 낭비하지 않고 바로바로 모르는 문제를 해결할 수 있었습니다.</v>
@@ -7404,10 +7404,10 @@
         <v>N수생</v>
       </c>
       <c r="E194" t="str">
-        <v>담임선생님과 성적 고민을 부담없이 나눌 수 있어 좋았고 멘토 선생님과 얘기를 하며 학습 향상에 도움이 되었다. 해야되는 공부량을 일주일에 한번씩 대면하면서 모의고사나 더프 등 시험볼 때의 팁들을 알아갈 수 있어서 좋았다.</v>
+        <v>담임 선생님과 성적 고민을 부담없이 나눌 수 있어 좋았고 멘토 선생님과 얘기를 하며 학습 향상에 도움이 되었다. 해야되는 공부량을 일주일에 한 번씩 대면하면서 모의고사나 더프 등 시험볼 때의 팁들을 알아갈 수 있어서 좋았다.</v>
       </c>
       <c r="F194" t="str">
-        <v>평소에는 계획을 잘 세우지 않는편이라 공부할 때 방향성을 잡기 쉽지 않았는데 매일 내가 한 학습량과 앞으로 해야할 것들을 정리하면서 하루하루 성취감도 생기고 공부 계획을 철저하게 세울 수 있어 도움이 되었다.</v>
+        <v>평소에는 계획을 잘 세우지 않는편이라 공부할 때 방향성을 잡기 쉽지 않았는데 매일 내가 한 학습량과 앞으로 해야 할 것들을 정리하면서 하루하루 성취감도 생기고 공부 계획을 철저하게 세울 수 있어 도움이 되었다.</v>
       </c>
       <c r="G194" t="str">
         <v>한 자리에서 계속 공부를 하면 지치거나 졸릴때도 있어 체력적으로 힘든데 학습 분위기를 조교 선생님들이 관리해주셔서 더 편안했다. 집중을 잘 할 수 있는 분위기를 만들어주셔서 믿고 온전히 공부에만 집중할 수 있었다.</v>
@@ -7416,10 +7416,10 @@
         <v>수능 입시를 준비하다보면 평가원 모의고사 뿐만이 아니라 많은 사설 모의고사들도 풀어보며 시험 볼 때의 태도를 많이 연습할 수 있는데 이투스 모의고사를 의무로 봄으로써 학원에서 강제적으로라도 나의 시험 태도를 확인할 수 있어서 좋았다.</v>
       </c>
       <c r="I194" t="str">
-        <v>항상 아침에 웃는 얼굴로 인사해주시고 대학 상담이나 여쭙고 싶은게 있을 때 언제든지 환영해주셔서 감사했습니다. 수능 후 논술 대비까지 응원해주셔서 덕분에 좋은 재수생활을 하고 합격할 수 있었던 것 같아요. 감사합니다!</v>
+        <v>항상 아침에 웃는 얼굴로 인사해주시고 대학 상담이나 여쭙고 싶은게 있을 때 언제든지 환영해주셔서 감사했습니다. 수능 후 논술 대비까지 응원해주셔서 덕분에 좋은 재수 생활을 하고 합격할 수 있었던 것 같아요. 감사합니다!</v>
       </c>
       <c r="J194" t="str">
-        <v>취약 유형을 담임선생님과 상담하면서 집중적으로 끌어올릴 수 있었어요.</v>
+        <v>취약 유형을 담임 선생님과 상담하면서 집중적으로 끌어올릴 수 있었어요.</v>
       </c>
       <c r="K194" t="str">
         <v/>
@@ -7440,7 +7440,7 @@
       </c>
       <c r="E195" t="str" xml:space="preserve">
         <v xml:space="preserve">재수생의 맞는 학습 패턴과 함께 올바른 공부 방법을 지도하여 주시며_x000d_
-수험 생활에서의 어려움을 공감하며 본인의 경험과 함께 더불어 뜻깊은 조언을 해주신다. 또 외로운 수험생활에서 일상의 대화가 되어주시기도 하며 더욱 공부에 집중할 수 있도록 최선을 다해주셔서 생활에 도움이 많이 되었다.</v>
+수험 생활에서의 어려움을 공감하며 본인의 경험과 함께 더불어 뜻깊은 조언을 해주신다. 또 외로운 수험 생활에서 일상의 대화가 되어주시기도 하며 더욱 공부에 집중할 수 있도록 최선을 다해주셔서 생활에 도움이 많이 되었다.</v>
       </c>
       <c r="F195" t="str">
         <v>혼자서 독학 재수를 하는 점에서 가장 불편하고도 어려운 부분이 즉각적인 질의 응답이 되어지지 않는 것인데 이 부분을 해결해주며 또 각 과목 마다 선생님이 배정되어 있으셔서 빠르게 피드백을 받고 질문을 할 수 있었다.</v>
@@ -7453,7 +7453,7 @@
       </c>
       <c r="I195" t="str" xml:space="preserve">
         <v xml:space="preserve">공부에 집중하는 수험생들을 위해 늘 최선을 다해 도와주시고 신경 써 주셔서 정말 감사합니다._x000d_
-또 매 주 상담을 해주시며 공부외 개인적인 고민도 들어주려 하시며 학생들과 함께 수험생활을 하는 것 처럼 임하여 주심에 감사드립니다.</v>
+또 매 주 상담을 해주시며 공부외 개인적인 고민도 들어주려 하시며 학생들과 함께 수험 생활을 하는 것 처럼 임하여 주심에 감사드립니다.</v>
       </c>
       <c r="J195" t="str">
         <v>월별, 주간별, 일별 계획을 세워 공부하는 법을 학원을 통해 알게 되면서 좋은 습관을 가지고 공부할 수 있었어요!</v>
@@ -7482,7 +7482,7 @@
         <v>자신에게 맞는 인강 선생님을 고르는게 수험 공부에 있어 중요한 부분을 차지한다고 생각하는데 그런 점에 있어서 많은 도움을 받았던거 같습니다. 꾸준히 진도 체크해주면서 인강 수강을 하니 좋은 결과를 얻을 수 있었습니다.</v>
       </c>
       <c r="G196" t="str">
-        <v>휴대폰이 공부하는데에 가장 방해되는 요인인데 입실할때 휴대폰 내고 나갈때 받을 수 있도록 철저하게 관리해주시니 정말 오직 공부에만 집중할 수 있었습니다. 특히 식사시간에 휴대폰을 보지 않고 차라리 산책을 갔다오니 멘탈적으로 많은 도움이 됐습니다.</v>
+        <v>휴대폰이 공부하는 데에 가장 방해되는 요인인데 입실할때 휴대폰 내고 나갈때 받을 수 있도록 철저하게 관리해주시니 정말 오직 공부에만 집중할 수 있었습니다. 특히 식사시간에 휴대폰을 보지 않고 차라리 산책을 갔다오니 멘탈적으로 많은 도움이 됐습니다.</v>
       </c>
       <c r="H196" t="str">
         <v>수능이 다가오다보면 영어에 소홀해지기 마련인데 게속 단어 테스트 보면서 영어 감을 익히고 단어도 외우다보니까 영어에서 이익을 볼 수 있었습니다. 특히 올해같이 어려웠던 영어 수능에서 많은 도움이 되었습니다.</v>
@@ -7524,7 +7524,7 @@
       </c>
       <c r="G197" t="str" xml:space="preserve">
         <v xml:space="preserve">정신차리고 항상 자지 않으려고 노력은 하지만, 어쩔 수 없이 잠이 올 때 _x000d_
-수시로 깨워주시고 태도가 좋지 않을 때에도 잘 잡아주셔서 공부가 잘 되었던 것 같습니다. 그리고 학생의 컨디션도 잘 체크를 해주셔서 제가 몸이 좋지 않을때에는 제 편의를 봐주시면서 학습관리 체크를 해주셨는데, n수 할때 도움이 많이 되었던 것 같습니다</v>
+수시로 깨워주시고 태도가 좋지 않을 때에도 잘 잡아주셔서 공부가 잘 되었던 것 같습니다. 그리고 학생의 컨디션도 잘 체크를 해주셔서 제가 몸이 좋지 않을때에는 제 편의를 봐주시면서 학습 관리 체크를 해주셨는데, n수 할때 도움이 많이 되었던 것 같습니다</v>
       </c>
       <c r="H197" t="str" xml:space="preserve">
         <v xml:space="preserve">공부를 시작하기에 앞서, 20-30분 정도 일일테스트로 머리를 깨우고 공부를 하는게 도움이 많이 되었습니다. _x000d_
@@ -7675,7 +7675,7 @@
       </c>
       <c r="I201" t="str" xml:space="preserve">
         <v xml:space="preserve">모든 분께 감사했습니다._x000d_
-제가 항상 배가 아파서 아침에 좀 상당히 지각했어도 봐주셨던 카운터 선생님, 저를 항상 믿어주시며 널널하게 봐주셨던 윤성재 담임선생님 덕분에 엄청난 성적 상승은 아니지만 적당한 상승으로 인서울을 하게 되었습니다._x000d_
+제가 항상 배가 아파서 아침에 좀 상당히 지각했어도 봐주셨던 카운터 선생님, 저를 항상 믿어주시며 널널하게 봐주셨던 윤성재 담임 선생님 덕분에 엄청난 성적 상승은 아니지만 적당한 상승으로 인서울을 하게 되었습니다._x000d_
 _x000d_
 이 결과물은 선생님들의 노고가 더해져 만들어진 결과물이라고 생각합니다._x000d_
 덕분에 현재 좋은 대학 생활을 보내고 있는 것에 그저 감사드립니다.</v>
@@ -7701,7 +7701,7 @@
         <v>N수생</v>
       </c>
       <c r="E202" t="str">
-        <v>선생님께서 효율적이고 저에게 맞는  시간표를 짤 수 있게 도움을 많이 주십니다! 혼자서 1년간의 시간을 분배하기에는 어려운 부분이 있었어서 좋았어요 공부할 때 자주 돌아다니면서 상태 체크해주셔서 계속 집중해서 공부할수 있었습니다. 어려운 문제를 질문하몀 천천히 잘 설명해주셔서 이해가 잘 됐어요</v>
+        <v>선생님께서 효율적이고 저에게 맞는  시간표를 짤 수 있게 도움을 많이 주십니다! 혼자서 1년간의 시간을 분배하기에는 어려운 부분이 있었어서 좋았어요 공부할 때 자주 돌아다니면서 상태 체크해주셔서 계속 집중해서 공부할 수 있었습니다. 어려운 문제를 질문하몀 천천히 잘 설명해주셔서 이해가 잘 됐어요</v>
       </c>
       <c r="F202" t="str">
         <v>혼자서는 꾸준히 규칙적으로 계속 공부하는걸 이어나가는게 힘든데 학습 관리 시스템 덕분에 도움을 많이 받았습니다 세세한 부분까지 관리받을 수 있어서 딴생각 안하고 공부만 잘 할수 있었던거같아요</v>
@@ -7713,7 +7713,7 @@
         <v>이투스 구독을 무료로 할 수 있어서 구독 갱신 같은 거 신경 안쓰고 학습 효율을 크게 높일수있었습니다! 이투스 안에 다양한 강의가 있어서 듣고싶은 거 제약없이 다 들을 수 있어서 좋았어요 무엇보다!!! 학원비에 구독비를 추가로 낼 필요가 없으니까 별도의 비용 부담 없이 이투스 강의를 들을수 있어서 경제적인 측면에서도 매우 좋앗습니다 ㅎㅎ</v>
       </c>
       <c r="I202" t="str">
-        <v>이투스에서 항상 저를 위해 신경써주셧던 선생님들께 진심으로 감사드립니다 !! 힘들고 지칠 때마다 따뜻한 말도 해주시고 현실적인 말도 해주셔서 다시 마음을 다잡고 할수있었어요 늘 묵묵히 응원도 해주시고 세심하게 관리해주셔서 큰 힘이 되었습니다! 덕분에 학원에서 열심히 공부할수있었어요</v>
+        <v>이투스에서 항상 저를 위해 신경써주셧던 선생님들께 진심으로 감사드립니다 !! 힘들고 지칠 때마다 따뜻한 말도 해주시고 현실적인 말도 해주셔서 다시 마음을 다잡고 할수있었어요 늘 묵묵히 응원도 해주시고 세심하게 관리해주셔서 큰 힘이 되었습니다! 덕분에 학원에서 열심히 공부할 수있었어요</v>
       </c>
       <c r="J202" t="str">
         <v>매번 학습일지를 작성하고 주기적인 피드백을 받으며 공부 계획을 잡아 원동력을 잃지 않고 공부할 수 있었어요.</v>
@@ -7736,7 +7736,7 @@
         <v>N수생</v>
       </c>
       <c r="E203" t="str">
-        <v>등원 첫 날 부터 끝날 때까지 학생 개개인에 맞는 문제집과 강의 추천이 가장 유용했다. 한 달에 한 번씩 상담을 하며 어느정도까지 진도가 나갔는지, 성장했는지 확인 받으며 문제집과 강의를 추천 받았는데 그 점이 가장 유용했고 또 성적향상에 큰 도움이 되었다.</v>
+        <v>등원 첫 날 부터 끝날 때까지 학생 개개인에 맞는 문제집과 강의 추천이 가장 유용했다. 한 달에 한 번씩 상담을 하며 어느정도까지 진도가 나갔는지, 성장했는지 확인 받으며 문제집과 강의를 추천 받았는데 그 점이 가장 유용했고 또 성적 향상에 큰 도움이 되었다.</v>
       </c>
       <c r="F203" t="str" xml:space="preserve">
         <v xml:space="preserve">학원에서 한 달에 한 번씩 개개인 성적과 어느 정도까지 진도가 나갔는지 확인을 했는데 함께 보면서 자신이 어느정도 인지 메타인지를 가능하게 하였습니다._x000d_
@@ -7757,7 +7757,7 @@
 다시 한 번 감사드립니다</v>
       </c>
       <c r="J203" t="str">
-        <v>담임선생님께서 공부 계획부터 방향까지 철저하게 잡아주시고, 즉각적인 피드백으로 올바른 학습 방향을 이어갈 수 있었어요.</v>
+        <v>담임 선생님께서 공부 계획부터 방향까지 철저하게 잡아주시고, 즉각적인 피드백으로 올바른 학습 방향을 이어갈 수 있었어요.</v>
       </c>
       <c r="K203" t="str">
         <v/>
@@ -7817,7 +7817,7 @@
         <v>재수를 시작하고 저의 공부상태를 점검해주시고 저의 수준과 목표를 고려하여 어떤 강사의 어떤 커리큘럼을 따라가야할지에 대한 방향성을 잡아주었습니다. 또한 모의고사 성적관리도 꼼꼼히 해주며 부족한 부분들을 보완해주시려고 노력해주었습니다.</v>
       </c>
       <c r="F205" t="str">
-        <v>모의고사 성적들을 봐주시고 어떤점이 부족한지 보완해야할점은 무엇인지를 같이 고민해주셨습니다. 또한 제가 필요한 자료들을 찾아주셔서 학습에 많은 도움이 되었습니다. 자습시간때도 지속적케어로 많은 도움을 받았습니다.</v>
+        <v>모의고사 성적들을 봐주시고 어떤점이 부족한지 보완해야 할점은 무엇인지를 같이 고민해주셨습니다. 또한 제가 필요한 자료들을 찾아주셔서 학습에 많은 도움이 되었습니다. 자습시간때도 지속적케어로 많은 도움을 받았습니다.</v>
       </c>
       <c r="G205" t="str">
         <v>30분정도마다 감독관선생님이 순찰을 도셔서 졸거나 자는친구들을 깨워주십니다. 옆에 친구가 자거나 혹은 제가 자면 전체적인 공부분위기가 잡히지 않을 수 있는데 지속적으로 순찰하시며 공부 분위기를 잡으려 해주셨습니다.</v>
@@ -7896,7 +7896,7 @@
         <v>여러 단어들을 자주 시험치게 되니 어떤 단어를 내가 모르고, 헷갈리는 것이 무엇인지 주기적으로 체크하고 보완할 수 있었습니다. 이 덕분에 영단어 실력이 크게 상승되고 유지할 수 있었습니다.</v>
       </c>
       <c r="I207" t="str">
-        <v>재원하는 동안 항상 친절하게 관리해주셔서 정말 감사했습니다. 덕분에 힘든 수험생활을 그나마 재밌고 쾌적하게 할 수 있었습니다! 항상 파이팅하시고 좋은 일들만 있으시길 기원합니다😊</v>
+        <v>재원하는 동안 항상 친절하게 관리해주셔서 정말 감사했습니다. 덕분에 힘든 수험 생활을 그나마 재밌고 쾌적하게 할 수 있었습니다! 항상 파이팅하시고 좋은 일들만 있으시길 기원합니다😊</v>
       </c>
       <c r="J207" t="str">
         <v>제 수준에 맞는 강의와 커리큘럼을 추천받고, 질의응답을 통해 못 푼 문제를 다시 풀어보며 부족한 부분을 채울 수 있었어요.</v>
@@ -8039,7 +8039,7 @@
         <v>진짜 감사했습니다.  내원생이름도 외우시고 안부도 여쭤봐주시고 아침 일찍 출근하시고 상담도 해주시고 수험생들 공부 환경 만들어 주시려 애썼던것들 모두 감사합니다. 이 외에도 해주신것들이 많았던것 같은데 진짜 감사합니다.</v>
       </c>
       <c r="J211" t="str">
-        <v>학습관리 시스템 덕분에 공부 시간을 체계적으로 관리하고, 계획·실행·피드백 과정을 꾸준히 이어갈 수 있었어요.</v>
+        <v>학습 관리 시스템 덕분에 공부 시간을 체계적으로 관리하고, 계획·실행·피드백 과정을 꾸준히 이어갈 수 있었어요.</v>
       </c>
       <c r="K211" t="str">
         <v>학습 관리</v>
@@ -8074,7 +8074,7 @@
         <v>작년 입시 준비 기간 동안 이투스 247 관리형독서실에서 많은 도움을 받았습니다. 체계적인 관리와 학습 환경 덕분에 공부에 집중할 수 있었고, 수험 생활을 끝까지 버틸 수 있었습니다. 그때의 경험과 도움이 지금 대학 생활을 하는 데에도 큰 밑바탕이 되었다고 생각합니다. 그동안 신경 써주신 모든 분들께 감사드립니다.</v>
       </c>
       <c r="J212" t="str">
-        <v>담임선생님과 맞춤 커리큘럼을 짜고 월별 점검과 오답 분석을 통해 부족한 과목을 바로 보완할 수 있었어요.</v>
+        <v>담임 선생님과 맞춤 커리큘럼을 짜고 월별 점검과 오답 분석을 통해 부족한 과목을 바로 보완할 수 있었어요.</v>
       </c>
       <c r="K212" t="str">
         <v/>
@@ -8094,7 +8094,7 @@
         <v>N수생</v>
       </c>
       <c r="E213" t="str">
-        <v>공부 중에 막히는 부분이 생길 때, 즉각적으로 질문을 할 수 있었던게 무척 좋았습니다. 아무래도 인강으로만 공부를 하는 것이 한계가 있다보니 전 학습 상담을 하며 저의 지식의 폭을 넓힐 수 있었던 것이 큰 장점이 아닐까 하고 생각해요. 특히 수학 선생님께 도움을 많이 받았습니다!! 학습 상담을 하면서 담임선생님께서 제게 하셨던 말씀들도 아직까지 기억에 남아 있어요. 무작정 잘 될 거라는 말보다 선생님의 담백한 충고와 현실적인 조언들이 제게 큰 힘이 되었고, 앞으로 나아갈 수 있는 좋은 발판이 되었습니다.</v>
+        <v>공부 중에 막히는 부분이 생길 때, 즉각적으로 질문을 할 수 있었던게 무척 좋았습니다. 아무래도 인강으로만 공부를 하는 것이 한계가 있다보니 전 학습 상담을 하며 저의 지식의 폭을 넓힐 수 있었던 것이 큰 장점이 아닐까 하고 생각해요. 특히 수학 선생님께 도움을 많이 받았습니다!! 학습 상담을 하면서 담임 선생님께서 제게 하셨던 말씀들도 아직까지 기억에 남아 있어요. 무작정 잘 될 거라는 말보다 선생님의 담백한 충고와 현실적인 조언들이 제게 큰 힘이 되었고, 앞으로 나아갈 수 있는 좋은 발판이 되었습니다.</v>
       </c>
       <c r="F213" t="str">
         <v>수학 선생님과 가깝게 지내서 저의 수준에 맞는 수학 교재를 추천 받곤 했습니다. 너무 쉽지도 너무 어렵지도 않은 딱 적합한 문제지를 추천해 주시거나 당신의 교재를 저에게 주시는 경우도 있었어요. 이래저래 너무 도움을 많이 받아서 유익했다고 말 할 수 밖에 없을 것 같습니다.. 또 영어 선생님께 수능 디데이 별로 어떤 교재를 쓰면 좋을지 질문을 했을 때도 명쾌하게 답을 해 주셨어요. 갈팡질팡하는 도중 선생님들의 말씀으로 갈 길을 바로 잡은 경우가 많아서 유용했습니다!</v>
@@ -8103,7 +8103,7 @@
         <v>요즘 같은 시대에 공부에 가장 방해가 되는 요소는 아무래도 휴대전화일 것 같은데요. 아침에 등원 하자마자 휴대폰을 제출하는 시스템이기 때문에 휴대폰을 보며 시간을 날리는 경우가 현저히 줄 수 밖에 없어서 좋았습니다. 서포터즈를 하는 경우와 같이 특수한 일이 있을 때는 허락을 받고 사용할 수 있어서 불편함이 없었습니다.</v>
       </c>
       <c r="H213" t="str">
-        <v>혼자 자습만 하다 보면 실전 모의고사를 푸는 감을 잃어버릴 수가 있어요. 하지만 매달 더프 모의고사와 이투스 모의고사와 같은 사설 모의고사를 치면서 그 감을 유지 할 수 있었습니다. 또 시험 후 결과를 보고 선생님께서 보완해야할 부분과 방향을 제시해 주셔서 정말 좋았어요. 수학 모의고사 같은 경우는 무료로 풀이도 다 해주시고 1:1 상담도 해주셔서 무척이나 유용했던 기억이 있습니다!!</v>
+        <v>혼자 자습만 하다 보면 실전 모의고사를 푸는 감을 잃어버릴 수가 있어요. 하지만 매달 더프 모의고사와 이투스 모의고사와 같은 사설 모의고사를 치면서 그 감을 유지 할 수 있었습니다. 또 시험 후 결과를 보고 선생님께서 보완해야 할 부분과 방향을 제시해 주셔서 정말 좋았어요. 수학 모의고사 같은 경우는 무료로 풀이도 다 해주시고 1:1 상담도 해주셔서 무척이나 유용했던 기억이 있습니다!!</v>
       </c>
       <c r="I213" t="str">
         <v>이투스 학원을 졸업?한지 벌써 6개월이 흘렀네요.. 작년 2월부터 10월 말까지 직접적이든 간접적이든 저와 함께 해주셨던 선생님들이 계셨기에 지금 제가 서울에서 즐거운 시간을 보낼 수 있다고 생각해요. 솔직히 재수라는 게 절대 행복한 시간으로 기억 될 수다 없다고 생각했는데, 왜인지 저에게는 좋은 기억으로 남아 있습니다. 제가 있었던 부산 서면 이투스 247학원은 정이 넘치는 따뜻한 공간이었던 것 같아요!! 저의 인생에 좋은 영향을 주셔서 너무 감사합니다! 항상 무탈하세요!!</v>
@@ -8142,7 +8142,7 @@
 모의고사 말고도 이투스에서 자체적인 모의고사를 보면서 모의고사를 보는 횟수를 늘리니 수능장에서의 감을 익히기 더 좋았습니다</v>
       </c>
       <c r="I214" t="str">
-        <v>짧은 시간동안 다녔지만 정말 의미있는 공부시간을 보낸것같아 좋았습니다 조금 더 빨리 왔으면 좋았겠다는 후회를 많이 했어요 항상 친절하게 대해주셔서 감사했습니다ㅠㅠ 항상 건강하시구 좋은 일만 생기시길 빌게요 서울강동이투스화이띵</v>
+        <v>짧은 시간동안 다녔지만 정말 의미있는 공부 시간을 보낸것같아 좋았습니다 조금 더 빨리 왔으면 좋았겠다는 후회를 많이 했어요 항상 친절하게 대해주셔서 감사했습니다ㅠㅠ 항상 건강하시구 좋은 일만 생기시길 빌게요 서울강동이투스화이띵</v>
       </c>
       <c r="J214" t="str">
         <v>평가원 모의고사와 실전 모의고사 후 과목별 상담을 통해 틀린 이유를 분석하고, 다음 시험을 위한 학습 방향을 잡을 수 있었어요.</v>
@@ -8171,7 +8171,7 @@
         <v>재수하기 전, 인강을 들을 때 수강율에 집착하고 주변 친구들의 추천을 통해 강의만 마구잡이로 많이 들어 그 해 수능에서 그닥 효과를 보지 못한 경험이 있었다. 이투스 학원에서 제공한 인강 추천 및 수강 관리 시스템으로 나에게 맞는 인강 강사 선생님을 나보다 인강에 대해 잘 아시는 분이 추천해주시니 한 인강 선생님의 커리큘럼을 성실하게 수행해내었다. 또 주마다 수강율 체크로 내가 지금 그 주에 소홀히 하고 있는 과목을 파악하고 이에 맞추어 그 주 인강 계획을 자세하게 수정해주시니 내가 그에 들일 노력을 대신 해주셔서 시간이 절약되는 효과를 누렸다.</v>
       </c>
       <c r="G215" t="str">
-        <v>현역 때, 독서실이나 스터디카페에서는 인강 시청을 위해 패드를 키고 공부를 하는 것이 아닌 패드로 유튜브를 보거나 소셜미디어 앱으로 노는 경향이 있었고 이로 인해 순공시간이 확실히 떨어졌다. 강제성이 부족해 실패를 겪으니, 이투스 학원에서 제공해주는 감독 시스템으로 패드를 통해 딴 짓을 못하게 되니 순공시간이 비약적으로 늘고 공부에만 오로지 집중할 수 있는 환경이 만들어졌다. 또 공부시간에 잠이 와 졸거나 책상에서 쪽잠을 잘때 감독관 선생님이 와서 깨워주시니 순공시간이 늘어나는 효과와 함께 최대한 졸음을 깨우기 위해 노력하고 긴장감을 가지는 습관을 들게 되었다. 이를 통해 수능에서 현역 때의 수능 보다 좋은 결과를 얻은 것 같아 이투스의 생활 관리 시스템이 유용했다고 생각한다.</v>
+        <v>현역 때, 독서실이나 스터디카페에서는 인강 시청을 위해 패드를 키고 공부를 하는 것이 아닌 패드로 유튜브를 보거나 소셜미디어 앱으로 노는 경향이 있었고 이로 인해 순공시간이 확실히 떨어졌다. 강제성이 부족해 실패를 겪으니, 이투스 학원에서 제공해주는 감독 시스템으로 패드를 통해 딴 짓을 못하게 되니 순공시간이 비약적으로 늘고 공부에만 오로지 집중할 수 있는 환경이 만들어졌다. 또 공부 시간에 잠이 와 졸거나 책상에서 쪽잠을 잘때 감독관 선생님이 와서 깨워주시니 순공시간이 늘어나는 효과와 함께 최대한 졸음을 깨우기 위해 노력하고 긴장감을 가지는 습관을 들게 되었다. 이를 통해 수능에서 현역 때의 수능 보다 좋은 결과를 얻은 것 같아 이투스의 생활 관리 시스템이 유용했다고 생각한다.</v>
       </c>
       <c r="H215" t="str">
         <v>이투스에서 제공해주는 전국 모의고사 시스템으로, 재수하는 동안 전국 재수생 간의 성적 지표를 알 수 있는 기회를 더 프리미엄 모의고사나 평가원 모의고사 외에 하나를 더 제공해주어 좋았다. 시험 후, 성적에 관한 분석 자료와 지금 성적으로 갈 수 있는 대학 등을 알려주어 지금 나의 상태에 대한 평가와 더 높은 성적을 위한 각오를 심어주어 학원을 다니는 동안 나에게 좋은 자극을 주었다. 달마다 모의고사를 정해진 시간에 수능 시스템으로 시험을 치르니, 후에 볼 수능을 연습해 볼 기회가 늘어나 매우 유용했다.</v>
@@ -8376,13 +8376,13 @@
         <v>반수생</v>
       </c>
       <c r="E221" t="str">
-        <v>수시원서를 쓰기전에 한명씩 친절하게 상담을 해주십니다. 각자의 모의고사와 실모, 내신 성적을 기반으로 같은 성적이여도 최선의 선택이 될 수 있게 같이 고민해주십니다. 입시전형요강에 댜해 빠삭하게 알고 있고 관련 설명도 자주 진행합니다.</v>
+        <v>수시원서를 쓰기전에 한 명씩 친절하게 상담을 해주십니다. 각자의 모의고사와 실모, 내신 성적을 기반으로 같은 성적이여도 최선의 선택이 될 수 있게 같이 고민해주십니다. 입시전형요강에 댜해 빠삭하게 알고 있고 관련 설명도 자주 진행합니다.</v>
       </c>
       <c r="F221" t="str">
         <v>일요일마다 모의고사를 보고 며칠 뒤에 성적표를 나눠준다. 더프처럼 다같이 보는 모의고사가 아니더라도 학원내에서 평균과 컷을 산출하여 알려주는 점이 매 모의고사에 진심으로 임하게 되는 것 같다.</v>
       </c>
       <c r="G221" t="str">
-        <v>기숙의 가장 큰 장점이 외부와 차단되는 것이라고 생각하는데 정말 방화벽이 잘 되어있어서 태블릿으로 딴짓할 수 없고 그만큼 그 시간들이 공부시간으로 이어지기 때문에 가장 공부에 도움이 된다</v>
+        <v>기숙의 가장 큰 장점이 외부와 차단되는 것이라고 생각하는데 정말 방화벽이 잘 되어있어서 태블릿으로 딴짓할 수 없고 그만큼 그 시간들이 공부 시간으로 이어지기 때문에 가장 공부에 도움이 된다</v>
       </c>
       <c r="H221" t="str" xml:space="preserve">
         <v xml:space="preserve">전국 모의고사라는 게 전국 학생들과 비교하여 나의 위치를 파악할 수 있고_x000d_
@@ -8424,7 +8424,7 @@
         <v>모의고사는 수능장에서 일어날 수 있는 많은 상황에 대비할 수 있고 자신의 위치를 파악할 수 있는 가장 좋은 방법입니다. 컨디션이 좋든 나쁘든 매달 모의고사를 실시하여 다양한 경험을 할 수 있었습니다.</v>
       </c>
       <c r="I222" t="str">
-        <v>길어진 수험생 생활로 자존감도 떨어지고 항상 생각만 많아져서 고민만 하면서 무기력하게 생활했는데 선생님들이 잘 받아주셔서 무사히 완주한거 같습니다. 담임선생님 항상 무기력한 학생이였는데 매번 친절하게 상담해주셔서 감사합니다🙂</v>
+        <v>길어진 수험생 생활로 자존감도 떨어지고 항상 생각만 많아져서 고민만 하면서 무기력하게 생활했는데 선생님들이 잘 받아주셔서 무사히 완주한거 같습니다. 담임 선생님 항상 무기력한 학생이였는데 매번 친절하게 상담해주셔서 감사합니다🙂</v>
       </c>
       <c r="J222" t="str">
         <v>세심한 진도 체크와 관리 덕분에 처음으로 플래너를 꾸준히 지킨 덕분에 매일 성실하게 공부하는 힘이 생겼어요.</v>
@@ -8500,7 +8500,7 @@
         <v>수능은 1년에 한번밖에 없고, N수생일수록 내신보다 수능에 대한 의존도가 높아져서 더욱 긴장되고 실수하기 쉬운데 주기적으로 제공되는 모의고사 컨텐츠 덕분에 시험장에서의 적응력을 키울 수 있었습니다. 또한 모의고사 기출을 계속 반복하다보면 이게 진짜 내 실력인지, 순수하게 처음 보는 문제가 맞는지, 점수가 지문에 익숙해져서 오른건지 내 실력이 늘어서 오른건지 구분이 안 갈때도 있었는데 새로운 문제들로 이런 복잡한 생각을 환기시킬 수 있어 좋았습니다. 현역때보다 재수생때 수능장에서 긴장을 덜 하고 더 상쾌한 상태로 시험을 봤는데, 이는 이투스 자체 모의고사 덕이 가장 컸던 것 같습니다.</v>
       </c>
       <c r="I224" t="str">
-        <v>선생님들 1년동안 너무 고생하셨고 매일 챙겨주셔서 정말 감사했습니다. 재수를 결심하고 학원을 끊었던 연초엔 막막하기만 했는데 지금 와서 되돌아보니 이 학원에 제 인생의 터닝포인트가 된 것 같습니다!!</v>
+        <v>선생님들 1년 동안 너무 고생하셨고 매일 챙겨주셔서 정말 감사했습니다. 재수를 결심하고 학원을 끊었던 연초엔 막막하기만 했는데 지금 와서 되돌아보니 이 학원에 제 인생의 터닝포인트가 된 것 같습니다!!</v>
       </c>
       <c r="J224" t="str">
         <v>규칙적인 생활 관리와 집중할 수 있는 환경 덕분에 공부 효율이 높아졌고, 자기 통제력과 책임감도 자연스럽게 길러졌어요.</v>
@@ -8527,7 +8527,7 @@
 지속적으로 선생님들께서 학원생활도 체크해주시고 스몰토크도 하면서 긴장도 풀리고 해낼수있다는 자신감도 조금씩 생겼던것같습니다</v>
       </c>
       <c r="F225" t="str" xml:space="preserve">
-        <v xml:space="preserve">특히 수학 부분에서 원장선생님께서_x000d_
+        <v xml:space="preserve">특히 수학 부분에서 원장 선생님께서_x000d_
 지금 제 수준과 시기에 풀어야하는 교재들과 괜찮은 사설 모의고사들을 추천해주신게 도움이 많이 되었습니다._x000d_
 얼마남지 않은 시기에 최고의 효율을 발휘해 예체능임에도 불구하고 2등급이라는 좋은 성적을 받을 수 있었습니다.</v>
       </c>
@@ -8561,13 +8561,13 @@
         <v>반수생</v>
       </c>
       <c r="E226" t="str">
-        <v>코치시스템을 통해 혼자 공부할때의 방향을 설정하는데 큰 도움을 받았습니다. 현재 공부 상태를 점검하고 부족한 부분을 알 수 있었고 그에 맞는 학습 계획을 새울 수 있었습니다. 이로 인해 집중도도 높아지고 공부시간을 더 효과적으로 사용할 수 있었습니다.</v>
+        <v>코치시스템을 통해 혼자 공부할때의 방향을 설정하는데 큰 도움을 받았습니다. 현재 공부 상태를 점검하고 부족한 부분을 알 수 있었고 그에 맞는 학습 계획을 새울 수 있었습니다. 이로 인해 집중도도 높아지고 공부 시간을 더 효과적으로 사용할 수 있었습니다.</v>
       </c>
       <c r="F226" t="str">
         <v>혼자 공부하다가 계속 모르는 문제들을 바로바로 선생님들께 여쭈어 볼 수 있어서 좋았습니다. 질문하는 것에 대해 부담이 있었는데 1:1 질문 시스템 덕분에 궁금한 점을 물어볼 수 있었습니다. 덕분에 문제들을 정확히 알고 넘어갈 수 있었습니다.</v>
       </c>
       <c r="G226" t="str" xml:space="preserve">
-        <v xml:space="preserve">학원의 면학 분위기 조성을 위하여 매 공부시간마다 선생님들께서 돌아다니시면서 자는 사람들을 깨우고 공부에 집중 할 수 있도록 하셨습니다._x000d_
+        <v xml:space="preserve">학원의 면학 분위기 조성을 위하여 매 공부 시간마다 선생님들께서 돌아다니시면서 자는 사람들을 깨우고 공부에 집중 할 수 있도록 하셨습니다._x000d_
 또한 시끄러운 사람이 있어 선생님들께 이야기하면 바로 조치를 취해주셔서 편안하게 조용한 환경에서 공부를 할 수 있었습니다.</v>
       </c>
       <c r="H226" t="str">
@@ -8680,7 +8680,7 @@
         <v>매달 이투스 모의고사를 봐서 내가 어느 위치인지 어느과목을 올려야 할지 좋은 모의고사라서 도움이 됬습니다. 그리고 모의고사 본 후 원장쌤과 상담도 하면서 저의 부족한 부분을 채울 수 있어서 좋았습니다</v>
       </c>
       <c r="I229" t="str">
-        <v>1년 동안 공부는 어려웠지만 선생님들의 도움 덕분에 수리 논술로 합격 되었습니다. 논술 합격은 선생님들의 코치, 방향성을 가르쳐 주신 덕분에 된것같습니다. 1년동안 감사 했습니다!!</v>
+        <v>1년 동안 공부는 어려웠지만 선생님들의 도움 덕분에 수리 논술로 합격 되었습니다. 논술 합격은 선생님들의 코치, 방향성을 가르쳐 주신 덕분에 된것같습니다. 1년 동안 감사 했습니다!!</v>
       </c>
       <c r="J229" t="str">
         <v>철저한 출결 관리로 규칙적인 습관을 기르고, 학습과 휴식의 균형을 잡아 높은 집중력을 유지했어요.</v>
@@ -8738,10 +8738,10 @@
         <v>N수생</v>
       </c>
       <c r="E231" t="str">
-        <v>독학으로 공부하는 시스템에서 학습 상담을 과목별로 일주일에 한 번씩 점검함으로써 공부 방향과 목표를 설정하는데에 도움이 되었다. 또한 이 시스템을 함으로써 독학하면서 어려웠던 부분이나 질문해야할 부분을 모아놓고 질문할 수 있어 학습에 많은 도움이 되었다.</v>
+        <v>독학으로 공부하는 시스템에서 학습 상담을 과목별로 일주일에 한 번씩 점검함으로써 공부 방향과 목표를 설정하는데에 도움이 되었다. 또한 이 시스템을 함으로써 독학하면서 어려웠던 부분이나 질문해야 할 부분을 모아놓고 질문할 수 있어 학습에 많은 도움이 되었다.</v>
       </c>
       <c r="F231" t="str">
-        <v>스스로 학습 플래너를 쓰고 하면서 놓치거나 빠지는 과목, 부분들이 꽤 많았었는데 학습 관리 시스템을 활용함으로써 내가 빠뜨린 부분이나 조금 더 보완해야할 부분들에 대해서 자세하게 피드백을 받을 수 있는 점이 유용했다. 또한 과목의 하나의 커리가 끝나게 되면 그에 맞는 다음 커리큘럼을 짜주고 공부 설정 방향을 설정해주는 점에서 많은 도움을 받을 수 있었다.</v>
+        <v>스스로 학습 플래너를 쓰고 하면서 놓치거나 빠지는 과목, 부분들이 꽤 많았었는데 학습 관리 시스템을 활용함으로써 내가 빠뜨린 부분이나 조금 더 보완해야 할 부분들에 대해서 자세하게 피드백을 받을 수 있는 점이 유용했다. 또한 과목의 하나의 커리가 끝나게 되면 그에 맞는 다음 커리큘럼을 짜주고 공부 설정 방향을 설정해주는 점에서 많은 도움을 받을 수 있었다.</v>
       </c>
       <c r="G231" t="str">
         <v>평소 핸드폰을 일상생활에서 분리하지 않고 외부에서 스스로 공부 할 때에는 아무리 핸드폰을 꺼놓아도 규제나 관리가 없었기에 수시로 확인하는 일이 많았다. 하지만 이와 같은 생활 관리 시스템이 이루어짐으로써 공부에 조금 더 집중 할 수 있는 환경이 만들어져서 좋았다.</v>
@@ -8750,7 +8750,7 @@
         <v>단어는 혼자서 외우다 보면 어느정도 알고 있다는 생각을 가지게 됨으로써 복습하거나 따로 공부하지 않게 되었다. 하지만 보카 시험 콘텐츠가 있기에 매일매일 최소 30개의 단어를 외우고 볼 수 있었던 점이 영어 공부에 생각보다 더 많은 도움이 되었다. 또한 시험이기에 시간이 나거나 집중이 되지 않을 때 틈틈히 외운 것도 도움이 되었다.</v>
       </c>
       <c r="I231" t="str">
-        <v>면학 분위기 지도, 학습관리, 학업 상담 등의 부분에서 많은 도움을 주셔서 감사합니다. 선생님들의 도움으로 앞으로 저의 미래에 있는 꿈에 한발자국 더 가까이 갈 수 있었습니다. 스스로 공부할 때에는 제가 세운 규칙들을 어기는 일이 많았지만 선생님들의 도움으로 오로지 공부에만 집중하는 시간이 늘어났습니다.</v>
+        <v>면학 분위기 지도, 학습 관리, 학업 상담 등의 부분에서 많은 도움을 주셔서 감사합니다. 선생님들의 도움으로 앞으로 저의 미래에 있는 꿈에 한발자국 더 가까이 갈 수 있었습니다. 스스로 공부할 때에는 제가 세운 규칙들을 어기는 일이 많았지만 선생님들의 도움으로 오로지 공부에만 집중하는 시간이 늘어났습니다.</v>
       </c>
       <c r="J231" t="str">
         <v>해주시는 학습 관리가 단순한 조언에 그치지 않고, 실제 성적 향상으로 이어질 수 있는 맞춤형 전략처럼 느껴져 매우 만족했어요.</v>
@@ -8776,7 +8776,7 @@
         <v>주도적으로 학습 계획을 세울 수 있다는 점이 좋아서 독학 재수 학원을 등록하였는데, 계획을 세우는 과정에서 확신을 가지고 선택을 하지 못하고 있을 때 담당 선생님께서 방향성을 잡는데에 도움을 많이 주셨다. 다른 사람의 조언을 들어도 나에게 맞는지에 대해 계속 의심해보는 성격인데, 과목에 맞는 실질적인 공부 방법도 보다 정확히 알려주셔서 믿음이 갔다.</v>
       </c>
       <c r="F232" t="str">
-        <v>믿음이 가는 사람이 나를 지속적으로 체크해준다는 점이 마음에 들었다. 선생님들께서도 학생들에게 신경을 많이 써주신다는 느낌을 받아서 좋았다. 사소한 부분에서까지 세심하게 의견을 나눌 수 있어 내가 의지하면서도 믿을 수 있고 나를 잘 아는 존재가 있다는게 수험생활에 소소한 행복이었다.</v>
+        <v>믿음이 가는 사람이 나를 지속적으로 체크해준다는 점이 마음에 들었다. 선생님들께서도 학생들에게 신경을 많이 써주신다는 느낌을 받아서 좋았다. 사소한 부분에서까지 세심하게 의견을 나눌 수 있어 내가 의지하면서도 믿을 수 있고 나를 잘 아는 존재가 있다는게 수험 생활에 소소한 행복이었다.</v>
       </c>
       <c r="G232" t="str">
         <v>기록이 남으니까 더 성실하게 다닐 수 있었던 것 같다. 혼자 독서실에서 공부했을 때 가장 문제였던 점이 식사 시간에 늘어지는 것이었는데, 점심 산책 시간도 정해져 있고 그게 기록에 남게 되어있다보니 공부에 투자할 수 있는 시간이 확실하게 보장될 수 있다는 점이 좋았다.</v>
@@ -8788,7 +8788,7 @@
         <v>학생관리팀 선생님들께 제일 감사했어요… 일 진짜 많으셨는데 항상 꼼꼼하게 챙겨주셨고 학생들한테도 친절하셨고 편의도 많이 봐주셨어요 진짜 학관쌤 아니었으면 더 빨리 그만 뒀을 거 같아요.. 담당 선생님들도 너무 도움 많이 돼서 기억에 많이 남습니다.</v>
       </c>
       <c r="J232" t="str">
-        <v>원장선생님과 상담할 때마다 평소 쌓였던 고민과 걱정이 한결 가벼워지는 느낌이었어요.</v>
+        <v>원장 선생님과 상담할 때마다 평소 쌓였던 고민과 걱정이 한결 가벼워지는 느낌이었어요.</v>
       </c>
       <c r="K232" t="str">
         <v/>
@@ -8808,19 +8808,19 @@
         <v>N수생</v>
       </c>
       <c r="E233" t="str">
-        <v>다시 공부를 시작했을 때 어떻게 공부를 해야할지 많은 고민이 있었습니다. 이투스247학원을 다니면서 각과목의 선생님과 공부의 방향성을 잡을 수 있었던 점이 가장 좋았습니다. 초반 방향성만 잡는것이 아니라 공부를 하면서 여러번의 상담을 통해 공부가 제대로 되고있는지 확인할 수 있던 것이 좋았습니다.</v>
+        <v>다시 공부를 시작했을 때 어떻게 공부를 해야 할지 많은 고민이 있었습니다. 이투스247학원을 다니면서 각과목의 선생님과 공부의 방향성을 잡을 수 있었던 점이 가장 좋았습니다. 초반 방향성만 잡는것이 아니라 공부를 하면서 여러번의 상담을 통해 공부가 제대로 되고있는지 확인할 수 있던 것이 좋았습니다.</v>
       </c>
       <c r="F233" t="str">
         <v>1년을 쉬고 시작한 수능공부라서 초반 방향성을 잡은 후 성적이 생각보다 좋지 않아 걱정을 했지만 거의 매달 시험을 보면서 성적과 시험 본 내용을 기반으로 어떤부분이 부족한지, 어떤부분을 보완해야 성적이 오를지 선생님과 상담하는것이 도움이 많이 되었습니다. 초반 성적과 비교했을 때 어떤부분에서 성장해고 여전히 어떤부분이 약한지 파악하였던 것도 많이 도움이 되었습니다.</v>
       </c>
       <c r="G233" t="str">
-        <v>시간표에 따라 생활을 하면서 생활습관과 공부습관을 함께 잡을 수 있어서 좋았던 것 같습니다. 특히 아침 잠이 좀 많은 편이라서 혼자 공부할 때 아침시간에 조는  경우가 많았는데 졸음 관리를 통해서 공부 시간을 더 확보할 수 있었고 습관을 길러서 수능이 다가올수록 조는 시간이 줄어들어 많은 도움이 되었습니다.</v>
+        <v>시간표에 따라 생활을 하면서 생활 습관과 공부습관을 함께 잡을 수 있어서 좋았던 것 같습니다. 특히 아침 잠이 좀 많은 편이라서 혼자 공부할 때 아침시간에 조는  경우가 많았는데 졸음 관리를 통해서 공부 시간을 더 확보할 수 있었고 습관을 길러서 수능이 다가올수록 조는 시간이 줄어들어 많은 도움이 되었습니다.</v>
       </c>
       <c r="H233" t="str">
         <v>수능 준비에서 중요한 부분 중 하나는 실전연습이라고 생각합니다. 하루를 온전히 수능날처럼 지내며 실제 수능처럼 모의고사를 통해 연습할 수 있었던 것이 수능 당일 긴장감을 줄이는데 많은 도움이 되었습니다. 또한 단순히 혼자 공부하는 것에서 그치는것이 아니라 이투스 전국 모의고사를 통해서 같은 수험생들 사이에 내가 어느위치에 있는지 나의 성적으로 어느학교에 갈 수 있는지를 체크할 수 있었던 점이 유용했습니다.</v>
       </c>
       <c r="I233" t="str">
-        <v>이투스 247강북점에서 일년간 저를 도와주신 모든 선생님들께 너무나도 감사합니다. 각과목의 선생님들 덕분에 과목별로 공부 방향을 잘 잡을 수 있었고 지루한 수험생활이 아니라 공부에 흥미를 가지고 노력할 수 있었던 것 같습니다. 감사합니다</v>
+        <v>이투스 247강북점에서 일년간 저를 도와주신 모든 선생님들께 너무나도 감사합니다. 각과목의 선생님들 덕분에 과목별로 공부 방향을 잘 잡을 수 있었고 지루한 수험 생활이 아니라 공부에 흥미를 가지고 노력할 수 있었던 것 같습니다. 감사합니다</v>
       </c>
       <c r="J233" t="str">
         <v>매주 정기적으로 원하는 과목의 선생님과 학습 상담을 할 수 있어서 좋았어요.</v>
@@ -8849,7 +8849,7 @@
         <v>독학재수학원이기 때문에 자기관리가 힘들 수 있습니다. 하지만 과목별로 주기적인 상담을 통해 본인 진도에 맞춰서 알맞은 계획을 세워주십니다. 저는 학습 계획을 세우는 것에 있어서 어려움을 느꼈는데 학습 관리 시스템 덕분에 계획 짜는 법에 도움을 많이 받았습니다.</v>
       </c>
       <c r="G234" t="str">
-        <v>수험생활 중 굉장히 힘든 점 중 하나가 스마트폰 관리라고 생각합니다. 이투스 247에서는 강제적으로라도 휴대폰을 수거해서 처음에는 조금 힘들 수 있지만 결국에는 많은 도움을 받았던 것 같습니다.</v>
+        <v>수험 생활 중 굉장히 힘든 점 중 하나가 스마트폰 관리라고 생각합니다. 이투스 247에서는 강제적으로라도 휴대폰을 수거해서 처음에는 조금 힘들 수 있지만 결국에는 많은 도움을 받았던 것 같습니다.</v>
       </c>
       <c r="H234" t="str">
         <v>영어공부에 있어서 영단어 공부는 매우 필수적이지만 스스로 하기에 쉽지 않다고 생각합니다. 다른 공부보다 항상 후순위로 밀려 생각보다 시간을 내서 공부하기 힘들기 때문입니다. 영단어 테스트를 매일, 반복적으로 보기 때문에 많은 도움을 받았던 것 같습니다.</v>
@@ -8858,7 +8858,7 @@
         <v>학원에 계시는 모든 분들 정말 진심으로 응원해주시고 관리해주신다는 걸  정말 많이 느꼈습니다. 가끔 쓴소리도 해주시지만 그것또한 다 잘되라고 하시는 거라는 걸 잘 알고 있습니다. 수험기간 동안 수고많이해주셔서 정말 감사했습니다.</v>
       </c>
       <c r="J234" t="str">
-        <v>담임선생님과 성적 고민을 부담없이 나눌 수 있어 좋았고, 멘토 선생님과 얘기를 하며 학습 향상에 도움이 되었어요.</v>
+        <v>담임 선생님과 성적 고민을 부담없이 나눌 수 있어 좋았고, 멘토 선생님과 얘기를 하며 학습 향상에 도움이 되었어요.</v>
       </c>
       <c r="K234" t="str">
         <v/>
@@ -8899,7 +8899,7 @@
         <v>마지막으로 영어 선생님과 실장님께 감사 인사를 드리고 싶습니다. 수험 생활을 하다 보면 예민해지고 작은 일에도 흔들리는 순간들이 많았는데, 그럴 때마다 항상 다정하게 대해주시고 질문에도 친절하게 답해주셔서 큰 힘이 되었습니다. 특히 ‘할 수 있다’고 계속해서 격려해주신 말들이 지칠 때마다 다시 버틸 수 있게 해주는 원동력이 되었습니다. 또 항상 밝게 인사해주시고 먼저 따뜻하게 말 걸어주셔서 학원에 오는 것 자체가 덜 부담스럽게 느껴졌던 것 같습니다. 사소해 보일 수 있지만 그런 분위기가 하루하루를 버티는 데 정말 큰 힘이 되었습니다. 중간중간 챙겨주신 맛있는 간식들도 큰 위로가 되었고, 덕분에 힘든 시기에도 포기하지 않고 끝까지 버틸 수 있었습니다. 1년이라는 시간을 무사히 버틸 수 있었던 데에는 선생님과 실장님의 도움이 정말 컸다고 생각합니다. 진심으로 감사드립니다.</v>
       </c>
       <c r="J235" t="str">
-        <v>담임선생님께서 일상의 대화로 힘이 되어주시고, 공부에 집중할 수 있도록 세심하게 도와주셔서 큰 도움이 되었어요.</v>
+        <v>담임 선생님께서 일상의 대화로 힘이 되어주시고, 공부에 집중할 수 있도록 세심하게 도와주셔서 큰 도움이 되었어요.</v>
       </c>
       <c r="K235" t="str">
         <v/>
@@ -9000,7 +9000,7 @@
         <v>이투스 학습 상담은 진짜 놀라울 정도로 친절하다. 이렇게까지 부담 없이 상담을 해줄 수 있나 싶을 정도로 편하게 얘기해주고, 누구에게나 적용 가능한 보편적인 조언을 꾸준히 유지해주는 일관성도 인상적이다. 특히 “열심히 하라”는 핵심 메시지를 여러 방식으로 반복해줘서 절대 잊을 수 없게 만들어주는 점이 굉장히 체계적이다. 덕분에 특별한 해결책은 없지만 마음만은 확실히 다잡게 되는 신기한 경험이었다.</v>
       </c>
       <c r="F238" t="str">
-        <v>이투스 학습관리는 진짜 체계적이라 놀라웠다. 이렇게까지 모든 학생을 비슷한 방식으로 꼼꼼하게 관리해줄 수 있다는 게 신기할 정도다. 계획도 항상 깔끔하게 잡아주고, 실천은 알아서 하게 만드는 자율성까지 완벽하게 보장해준다. 특히 꾸준히 “열심히 해야 한다”는 핵심을 잊지 않게 관리해주는 점이 인상적이라, 결국 성적이 안 오르면 이유를 명확하게 알 수 있게 해주는 친절한 시스템이다.</v>
+        <v>이투스 학습 관리는 진짜 체계적이라 놀라웠다. 이렇게까지 모든 학생을 비슷한 방식으로 꼼꼼하게 관리해줄 수 있다는 게 신기할 정도다. 계획도 항상 깔끔하게 잡아주고, 실천은 알아서 하게 만드는 자율성까지 완벽하게 보장해준다. 특히 꾸준히 “열심히 해야 한다”는 핵심을 잊지 않게 관리해주는 점이 인상적이라, 결국 성적이 안 오르면 이유를 명확하게 알 수 있게 해주는 친절한 시스템이다.</v>
       </c>
       <c r="G238" t="str">
         <v>면학 분위기 감독 및 관리는 정말 인상 깊었다. 굳이 안 자는지 공부하는지 세세하게 확인하지 않아서 학생 입장에서는 너무 편했고, 자고 있어도 크게 방해받지 않아서 쉬기에 좋은 환경이었다. 이렇게까지 학생 자율성을 존중해주는 곳은 흔치 않은 것 같다. 덕분에 공부하러 왔는지 수면 보충하러 왔는지 헷갈릴 정도로 배려가 넘쳤고, 관리가 느슨해서 오히려 더 기억에 남는다.</v>
@@ -9070,18 +9070,18 @@
         <v>처음에 시작할 때 아무 방향 없이 시작 했었는데, 개별 학습 데이터를 바탕으로 취약점과 공부 방향에 개인의 방향을 알려주어 좋았다. 특히 점수대 별에 맞춰, 시기별로 어떤 전략으로 공부하며 좋을지 알려주어서, 혼자서 공부할 때의 막막함을 해소 할 수 있어서 좋았다.</v>
       </c>
       <c r="F240" t="str">
-        <v>나는 원래 공부할 때 학습 계획은 대략적으로 만 세우고, 플레너는 쓰지도 않았었다. 하지만 이투스247에서 제공하는 프로그램으로 학습 계획과 플레너를 쓰면서, 객관적인 공부시간을 시각적으로 파악하며, 따로 큰 힘을 들이지 않아도 공부계획을 세울 수 있었다. 그리고 완료한 항목에 체크 표시를 해 나가면서 성취감도 얻을 수 있었고, 나의 기록을 보며 특정과목에만 치우치지 않게 공부양을 조절하며, 매일 기록을 복기하며 어려웠던 부분을 마스터 할 수 있었다.</v>
+        <v>나는 원래 공부할 때 학습 계획은 대략적으로 만 세우고, 플레너는 쓰지도 않았었다. 하지만 이투스247에서 제공하는 프로그램으로 학습 계획과 플레너를 쓰면서, 객관적인 공부 시간을 시각적으로 파악하며, 따로 큰 힘을 들이지 않아도 공부 계획을 세울 수 있었다. 그리고 완료한 항목에 체크 표시를 해 나가면서 성취감도 얻을 수 있었고, 나의 기록을 보며 특정과목에만 치우치지 않게 공부양을 조절하며, 매일 기록을 복기하며 어려웠던 부분을 마스터 할 수 있었다.</v>
       </c>
       <c r="G240" t="str" xml:space="preserve">
-        <v xml:space="preserve">나의 공부에서 가장 큰 문제는 공부시간을 제대로 활용하지 못하고 딴 짓을 한다는 것이었다. 그런데 와이파이 장벽은 스스로 자기 통제가 어려운 수험 생활 초반에 올바른 공부 습관을 형성하는데 큰 도움을 주었다. _x000d_
-이 덕분에 공부시간을 확보하고, 관성력으로 후반 공부까지 딴짓을 안 하고 잘 이어나갈 수 있었다.</v>
+        <v xml:space="preserve">나의 공부에서 가장 큰 문제는 공부 시간을 제대로 활용하지 못하고 딴 짓을 한다는 것이었다. 그런데 와이파이 장벽은 스스로 자기 통제가 어려운 수험 생활 초반에 올바른 공부 습관을 형성하는데 큰 도움을 주었다. _x000d_
+이 덕분에 공부 시간을 확보하고, 관성력으로 후반 공부까지 딴짓을 안 하고 잘 이어나갈 수 있었다.</v>
       </c>
       <c r="H240" t="str">
         <v>일일 테스트는 게임을 하듯이 복습을 하고, 모르는 부분을 체크 할 수 있다는 점이 가장 큰 장점이다. 탐구과목과 같은 과목의 기출을 가벼운 마음으로 게임을 하듯이 풀 수 있고, 유형 파악을 할 수 있어, 공부 한다는 생각이 안 들게 공부를 할 수 있어서 좋았다.</v>
       </c>
       <c r="I240" t="str" xml:space="preserve">
-        <v xml:space="preserve">6월말에 뒤늦게 수험생활을 시작해서 막막 했었는데, 이투스 247 수원시청점과 함께 해서 막막함이 많이 사라졌었습니다. _x000d_
-덕분에 수험생활을 잘 마무리 할 수 있었습니다. 감사합니다~!</v>
+        <v xml:space="preserve">6월말에 뒤늦게 수험 생활을 시작해서 막막 했었는데, 이투스 247 수원시청점과 함께 해서 막막함이 많이 사라졌었습니다. _x000d_
+덕분에 수험 생활을 잘 마무리 할 수 있었습니다. 감사합니다~!</v>
       </c>
       <c r="J240" t="str">
         <v>매일 매리트를 풀면서 간단하게 문제를 풀어보면서 과목마다 감을 잃지 않도록 만들어줘서 매우 유용했습니다.</v>
@@ -9152,7 +9152,7 @@
         <v>모든 사이트의 패스를 다 사려면 금액이 상당히 많이 드는데 이투스는 패스까지 무료로 준다는 게 금전적으로 메리트가 크다고 생각합니다! 저는 사회탐구를 이지영 선생님의 커리를 들었기 때문에 이투스 패스를 잘 활용했던 것 같습니다</v>
       </c>
       <c r="I242" t="str">
-        <v>항상 친절하게 관리해 주시고 상담도 해주시고 수업도 해주셔서 감사합니다. 상담하면서 심리적인 스트레스들을 해소할 수 있었던 것 같아서 좋았아요. 덕분에 1년동안 편안한 환경에서 공부하여 대학에 올 수 있었습니다!</v>
+        <v>항상 친절하게 관리해 주시고 상담도 해주시고 수업도 해주셔서 감사합니다. 상담하면서 심리적인 스트레스들을 해소할 수 있었던 것 같아서 좋았아요. 덕분에 1년 동안 편안한 환경에서 공부하여 대학에 올 수 있었습니다!</v>
       </c>
       <c r="J242" t="str">
         <v>플래너와 휴대폰 관리 덕분에 과목 편식 없이 집중했고, 깊이 있는 상담이 큰 도움이 됐어요.</v>
@@ -9251,7 +9251,7 @@
         <v>인강을 들으면서도 복습법이나 예습법 같은 상세한 공부 방법까지 피드백을 받을 수는 없었기 때문에 그 빈자리를 대신해주는 학습 관리 시스템의 역할이 저에게는 큰 도움이 되었습니다. 특히 사회문화 공부에서 어려움을 느끼고 있을 때 모의고사 학습법을 배운 것이 가장 큰 도움이 되었고, 이외에도 심리적 부분에서도 큰 도움을 받았습니다.</v>
       </c>
       <c r="G245" t="str">
-        <v>저는 스마트폰을 재수하는 기간 내내 단 한 번도 사용하지 않았습니다. 친구들과의 관계가 단절되고 홀로 견디는 수험생활이 처음엔 외롭고 어딘가 허전했지만, 수능이 다가올수록 제게 주어졌던 오직 저에게만 집중할 수 있는 1년이 얼마나 소중한 것이었던가를 느낄 수 있었습니다. 주변에 있는 작은 것들에서 기쁨과 감사를 느끼고 존재의 소중함을 느낄 수 있었던 1년이었습니다.</v>
+        <v>저는 스마트폰을 재수하는 기간 내내 단 한 번도 사용하지 않았습니다. 친구들과의 관계가 단절되고 홀로 견디는 수험 생활이 처음엔 외롭고 어딘가 허전했지만, 수능이 다가올수록 제게 주어졌던 오직 저에게만 집중할 수 있는 1년이 얼마나 소중한 것이었던가를 느낄 수 있었습니다. 주변에 있는 작은 것들에서 기쁨과 감사를 느끼고 존재의 소중함을 느낄 수 있었던 1년이었습니다.</v>
       </c>
       <c r="H245" t="str">
         <v>모의고사를 매월 보면서 저의 실력을 측정하는 것은 물론이고 실전 연습과 경험을 정말 많이 할 수 있었습니다. 특히 모의고사 전날이 정말 수능 전날인 것처럼 준비하고, 당일 아침부터 시험이 끝날 때까지의 시간을 고스란히 느끼면서 저만의 리듬과 루틴을 만들어 나갔던 것이 큰 도움이 되었습니다.</v>
@@ -9321,7 +9321,7 @@
         <v>각 과목별로 코칭을 받을 수 있어서 너무 좋았어요. 학습 상담을 통해 과목별로 제가 부족한 부분과 취약한 부분을 잘 보완할 수 있었어요. 또한 부족한 점을 베꿀 수 있는 자세한 대안까지 제안해주신 덕에 떨어졌던 자신감을 얻을 수 있었던 기회이기도 했습니다.</v>
       </c>
       <c r="F247" t="str">
-        <v>공부를 어디서부터 어떻게 시작해야되고 계획해야되는지 막막한 저에게 공부할 큰 틀을 제안해주고 계획을 세우는 방법을 알려주는 이 시스템이 정날 유용했습니다. 제가 계획을 세우면 선생님께서 보고 피드백을 주셨기 때문에 더 효율적이고 도움이 되는 공부계획을 세우고 실천할 수 있었습니다.</v>
+        <v>공부를 어디서부터 어떻게 시작해야되고 계획해야되는지 막막한 저에게 공부할 큰 틀을 제안해주고 계획을 세우는 방법을 알려주는 이 시스템이 정날 유용했습니다. 제가 계획을 세우면 선생님께서 보고 피드백을 주셨기 때문에 더 효율적이고 도움이 되는 공부 계획을 세우고 실천할 수 있었습니다.</v>
       </c>
       <c r="G247" t="str">
         <v>앉아서 공부하면 잠이 올 때가 정말 많은데 복도에서 공부할 수 있는 자리도 마련되어있고 그 외에 공부할 수 있는 공간도 엄청 다양해서 좋았습니다. 집중이 안될때 환경을 바꾸면서 공부하니 더 효율적으로 공부할 수 있었습니다. 또한 각 공간마다 감독도 잘 해주셔서 쾌적한 환경에서 공부에 집중할 수 있었어요.</v>
@@ -9400,7 +9400,7 @@
         <v>하반기에 풀었던 모의고사 덕분에 실전 감각을 익힐 수 있어서 좋았습니다. 특히 실전에서 긴장을 되게 많이 하는 성격인데 평소 연습을 많이 할 수 있는 기회를 주셔서 긴장이 아예 없어진 것은 아니지만 긴장을 어느정도 통제할 수 있는 위치에 도달한 것 같아서 좋았습니다.</v>
       </c>
       <c r="I249" t="str">
-        <v>한 해 동안 열심히 꾸준히 수험생활을 도와주셔서 정말 감사했습니다! 1년동안의 학원 분위기와 장소, 그 때 노력했던 마음 등은 절대 잊을 수가 없을 것 같습니다! 항상 건강하시길 바라겠습니다!</v>
+        <v>한 해 동안 열심히 꾸준히 수험 생활을 도와주셔서 정말 감사했습니다! 1년 동안의 학원 분위기와 장소, 그 때 노력했던 마음 등은 절대 잊을 수가 없을 것 같습니다! 항상 건강하시길 바라겠습니다!</v>
       </c>
       <c r="J249" t="str">
         <v>막히는 부분은 즉각 질문하여 바로 해결하고, 선생님의 현실적인 조언 덕분에 큰 힘을 얻어 끝까지 완주할 수 있었어요.</v>
@@ -9435,7 +9435,7 @@
         <v>매일 진행되는 영단어 테스트가 큰 도움이 되었습니다. 원래 영어 실력이 나쁘지 않은 편이었지만, 꾸준히 영단어를 반복해서 학습하도록 관리해 주셔서 자연스럽게 어휘력이 더 강화되었습니다. 덕분에 따로 영어 공부에 많은 시간을 투자하지 않아도 안정적으로 좋은 성적을 유지할 수 있었습니다.</v>
       </c>
       <c r="I250" t="str">
-        <v>선생님들 덕분에 흐트러지지 않고 끝까지 체계적으로 준비하여 입시를 잘 마무리할 수 있었습니다! 항상 응원해주신 EM반 담임선생님께 특히나 더 감사드립니다 안성이투스에서 공부하면서 정말정말 힘이 많이 되었습니다 감사합니다</v>
+        <v>선생님들 덕분에 흐트러지지 않고 끝까지 체계적으로 준비하여 입시를 잘 마무리할 수 있었습니다! 항상 응원해주신 EM반 담임 선생님께 특히나 더 감사드립니다 안성이투스에서 공부하면서 정말정말 힘이 많이 되었습니다 감사합니다</v>
       </c>
       <c r="J250" t="str">
         <v>수능을 앞두고 상담을 통해 긴장을 덜고, 모의고사와 학습 조언으로 실전 감각을 키웠어요.</v>
@@ -9458,7 +9458,7 @@
         <v>N수생</v>
       </c>
       <c r="E251" t="str">
-        <v>학창시절 공부를 해본적이 없어서 어떤식으로 공부를 해가야 할지 몰랐는데 학습 상담으로 공부하는 방법을 알려주셨고 과목별 공부시간 배분과 하루 최소할당치 같은 양을 정해주는게 큰 도움이 됐습니다</v>
+        <v>학창시절 공부를 해본적이 없어서 어떤식으로 공부를 해가야 할지 몰랐는데 학습 상담으로 공부하는 방법을 알려주셨고 과목별 공부 시간 배분과 하루 최소할당치 같은 양을 정해주는게 큰 도움이 됐습니다</v>
       </c>
       <c r="F251" t="str">
         <v>학창시절에 공부를 안했었고 당연히 수능 인강에 대해 무지하던 시절에 모의평가 성적을 보고 저에게 맞을만한 인강 강사를 추천해 준 것과 올해 수능에서 끝을 내기 위해 몇일까지 어느정도를 들어놔야 한다는 것을 알려주는게 시간관리 측면에서 도움이 되었습니다</v>
@@ -9557,7 +9557,7 @@
 앞으로도 선생님들께 배운 점을 바탕으로 더 노력하는 모습 보여드리겠습니다. 다시 한 번 진심으로 감사드립니다</v>
       </c>
       <c r="J253" t="str">
-        <v>학원에서 처음으로 저의 학습 성향을 알게 되면서 어떻게 공부를 해야할 지 습관을 바로 잡을 수 있어서 좋았습니다.</v>
+        <v>학원에서 처음으로 저의 학습 성향을 알게 되면서 어떻게 공부를 해야 할 지 습관을 바로 잡을 수 있어서 좋았습니다.</v>
       </c>
       <c r="K253" t="str">
         <v/>
@@ -9626,7 +9626,7 @@
         <v>재수생이다보니 영어단어를 외울 시간이 부족했고 영어에 시간투자를 하는것이 아깝다고 생각해서 영어를 다른 과목에 비해 덜 공부했었는데 단어시험은 매일 보다보니 어쩔 수 없이 공부했고 그에 따라 매일 일정량씩 단어를 외워야 되서 영어에 많은 도움이 되었다.</v>
       </c>
       <c r="I255" t="str">
-        <v>1년동안 재수하는 것이 너무 힘들것이라고 생각했었는데 이투스학원 선생님들이 계속 신경써주시고 상담도 자주해주셔서 버틸 수 있었던 것 같아요. 성적이 떨어져도 제 멘탈케어를 해주셔서 꾸준히 공부할 수 있었던 것 같습니다. 감사합니다.</v>
+        <v>1년 동안 재수하는 것이 너무 힘들것이라고 생각했었는데 이투스학원 선생님들이 계속 신경써주시고 상담도 자주해주셔서 버틸 수 있었던 것 같아요. 성적이 떨어져도 제 멘탈케어를 해주셔서 꾸준히 공부할 수 있었던 것 같습니다. 감사합니다.</v>
       </c>
       <c r="J255" t="str">
         <v>매주 플래너를 바탕으로 학습 점검이 이뤄져서 시간을 어떻게 활용하는지 선생님께서 세밀하게 관리해 주셔서 좋았어요.</v>
@@ -9684,7 +9684,7 @@
         <v>N수생</v>
       </c>
       <c r="E257" t="str">
-        <v>공부를 시작할 때 어떤 걸 해야할 지 모르겠는 막막함과 두려움이 있었습니다. 하지만 이투스 코칭 시스템을 통해 올바른 방향으로 공부를 할 수 있어서 심리적으로 안정감도 들고 도움이 많이 되었습니다.</v>
+        <v>공부를 시작할 때 어떤 걸 해야 할 지 모르겠는 막막함과 두려움이 있었습니다. 하지만 이투스 코칭 시스템을 통해 올바른 방향으로 공부를 할 수 있어서 심리적으로 안정감도 들고 도움이 많이 되었습니다.</v>
       </c>
       <c r="F257" t="str">
         <v>인강 콘텐츠들이 넘쳐나는 요즘 시대에서 나한테 맞고 좋은 선생님들 찾는데 시간이 많이 걸리고 지치는 일이 많았습니다. 하지만 이투스학원에서 추천해주시고 알려주시는 덕분에 스트레스 받는 일도 덜 했고 효과적이었습니다.</v>
@@ -9696,7 +9696,7 @@
         <v>각 인강 사이트마다 자신한테 맞는 선생들이 계시기 때문에 여러 패스를 끊어서 맞는 분을 찾는게 제일이지만 패스를 끊는 것도 비용이 들기 때문에 부담이 컸습니다. 그러나 이투스 247을 다니면 이투스 패스를 주어서 인강 선생님들 뵐 수 있다는 것이 비용적으로 부담이 줄었고 좋았습니다.</v>
       </c>
       <c r="I257" t="str">
-        <v>어떻게 공부를 해야할 지 모르던 저에게 올바른 방향을 제시해주시고 멘탈이 흔들릴 때나 지칠 때 잡아주시고 따뜻하게 대해주셔서 정말 감사했습니다. 덕분에 긴 수험생활 잘 버틴 것 같습니다.!!</v>
+        <v>어떻게 공부를 해야 할 지 모르던 저에게 올바른 방향을 제시해주시고 멘탈이 흔들릴 때나 지칠 때 잡아주시고 따뜻하게 대해주셔서 정말 감사했습니다. 덕분에 긴 수험 생활 잘 버틴 것 같습니다.!!</v>
       </c>
       <c r="J257" t="str">
         <v>졸음지도 및 관리 덕분에 집중력을 유지하여, 순공시간 확보에 큰 도움이 되었어요.</v>
@@ -9719,7 +9719,7 @@
         <v>N수생</v>
       </c>
       <c r="E258" t="str">
-        <v>공부 방법을 효율적으로 알려주시는 것에 그치지 않고 이를 실행할 수 있게 도와주심 또한 꾸준히 열심히 할 수 있게 계획을 세우는 것도 도와주심 생활습관 및 사소한 것들도 공부에 도움이 되는 방향으로 교정해주심</v>
+        <v>공부 방법을 효율적으로 알려주시는 것에 그치지 않고 이를 실행할 수 있게 도와주심 또한 꾸준히 열심히 할 수 있게 계획을 세우는 것도 도와주심 생활 습관 및 사소한 것들도 공부에 도움이 되는 방향으로 교정해주심</v>
       </c>
       <c r="F258" t="str">
         <v>출석체크를 통한 규칙적인 생활의 강제성, 꾸준함 그리고 만약 혼자 공부했더라면 전자기기 케어를 못하고 유튜브만 봤을 텐데 누군가가 날 지켜보고 있다고 생각하니 딴 짓을 안 하게 됨</v>
@@ -9789,10 +9789,10 @@
         <v>N수생</v>
       </c>
       <c r="E260" t="str">
-        <v>이투스 시스템이 담임선생님이 부여되고 담임선생님과 상담으로 하는식으로 이루어지는데 담임선생님과 많은 이야기를 할수있었고 수학 국어 선생님들이 있어서 질문을 할수있다는점에서 좋았습니다</v>
+        <v>이투스 시스템이 담임 선생님이 부여되고 담임 선생님과 상담으로 하는식으로 이루어지는데 담임 선생님과 많은 이야기를 할수있었고 수학 국어 선생님들이 있어서 질문을 할수있다는점에서 좋았습니다</v>
       </c>
       <c r="F260" t="str">
-        <v>매 모의고사나 이투스내에서 치는 고사같은 경우 시험을 보고난뒤 담임선생님과의 성적 상담이 들어갔는데 점수대와 틀린유형을 보고 어떤 부분에서 더 열심히 해야 하는지 알려주었고 그 피드백을 수용하여 공부하는데에 도움이 되었던거같습니다</v>
+        <v>매 모의고사나 이투스내에서 치는 고사같은 경우 시험을 보고난뒤 담임 선생님과의 성적 상담이 들어갔는데 점수대와 틀린유형을 보고 어떤 부분에서 더 열심히 해야 하는지 알려주었고 그 피드백을 수용하여 공부하는 데에 도움이 되었던거같습니다</v>
       </c>
       <c r="G260" t="str">
         <v>사실 성실한 사람이여도 피곤한날이있고 힘든날이있는데 그럴때에 공부를 놔버리면 공부의 증진이 어려운데 조는거같으먼 1분도 안되어 데스크 선생님께서 깨워주셔서 졸음퇴치에 도움이되었습니다</v>
@@ -9824,7 +9824,7 @@
         <v>N수생</v>
       </c>
       <c r="E261" t="str">
-        <v>저의 약점을 파악해 주시고 이를 바탕으로 학습 플래너를 세워주신 점이 인상 깊었습니다. 그동안 자기 객관화가 부족해 점수 향상이 어려웠지만, 담임선생님과의 상담을 통해 부족한 부분을 보완할 수 있었고, 그 결과 점수 상승으로 이어질 수 있었습니다.</v>
+        <v>저의 약점을 파악해 주시고 이를 바탕으로 학습 플래너를 세워주신 점이 인상 깊었습니다. 그동안 자기 객관화가 부족해 점수 향상이 어려웠지만, 담임 선생님과의 상담을 통해 부족한 부분을 보완할 수 있었고, 그 결과 점수 상승으로 이어질 수 있었습니다.</v>
       </c>
       <c r="F261" t="str">
         <v>부족한 부분을 보완하기 위해 수강해야 할 인강과, 해당 인강을 통해 무엇을 얻어야 하는지, 그리고 어떻게 공부해야 하는지까지 구체적으로 알려주셔서 올바른 방법으로 공부할 수 있었습니다. 학원을 다니지 않을 때에는 인강 선택에 어려움과 모호함이 있었지만, 이투스 247을 다니면서 이러한 문제를 해결할 수 있었습니다.</v>
@@ -9900,7 +9900,7 @@
         <v>혼자 재수할땐 그런 부분은 다 알수가 없고 전문가가 아니어서 정보를 다른곳에서 하나하나 얻어야 해서 힘들었는데 학원을 통해 필요한 정보만 알 수 있어서 좋았습니다. 꼭 n수를 안하더라도 고등학생이 다니기도 좋을 것 같습니다</v>
       </c>
       <c r="G263" t="str">
-        <v>전 잠도 많고 집중력도 안좋아서 다 잡아주시는게 좋았습니다. 1년동안 다니면서 학습 습관이 정말 좋아졌습니다. 딴짓하거나 졸어나 집중력이 흐트러질때 잘 잡아주셔서 감사했습니다. 재수학원이어서 추천하겠다는 말이 욕처럼 들릴진 모르겠지만 그냥 공부 습관 잡는겸 다니는것도 나쁘지 않을것같습니다</v>
+        <v>전 잠도 많고 집중력도 안좋아서 다 잡아주시는게 좋았습니다. 1년 동안 다니면서 학습 습관이 정말 좋아졌습니다. 딴짓하거나 졸어나 집중력이 흐트러질때 잘 잡아주셔서 감사했습니다. 재수학원이어서 추천하겠다는 말이 욕처럼 들릴진 모르겠지만 그냥 공부 습관 잡는겸 다니는것도 나쁘지 않을것같습니다</v>
       </c>
       <c r="H263" t="str">
         <v>모의고사를 매주 보기때문에 미리 연습하는겸 준비해볼수 있어서 좋았습니다. 전 긴장을 정말 많이 하는 사람이기때문에 모의고사를 많이 푸는 것 많으로 마음에 준비를 할 수 있었습니다.</v>
@@ -9929,17 +9929,17 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E264" t="str">
-        <v>공부를 하다보면 막막할때가 잦은데, 입시를 성공하신 선생님들의 학습 상담이 있어서 슬럼프나 막막할때 잘 넘어갈수 있었고, 때로는 엄격하지만 때로는 진중하고 재밌게 지친 수험생활을 위로해주신점이 유용했습니다.</v>
+        <v>공부를 하다보면 막막할때가 잦은데, 입시를 성공하신 선생님들의 학습 상담이 있어서 슬럼프나 막막할때 잘 넘어갈수 있었고, 때로는 엄격하지만 때로는 진중하고 재밌게 지친 수험 생활을 위로해주신점이 유용했습니다.</v>
       </c>
       <c r="F264" t="str" xml:space="preserve">
-        <v xml:space="preserve">노베상태에서, 인강이나 책 선택조차 막막할 시기가 있었는데, 선생님이 계셔서 어떤 책을 어떻게 공부해야할지 알수 있어서 유용했습니다._x000d_
+        <v xml:space="preserve">노베상태에서, 인강이나 책 선택조차 막막할 시기가 있었는데, 선생님이 계셔서 어떤 책을 어떻게 공부해야 할지 알수 있어서 유용했습니다._x000d_
 선생님이 추천해주신 책을 읽고 공부하니 비약적인 성적 상승을 이뤄서 기분이 좋았습니다.</v>
       </c>
       <c r="G264" t="str">
         <v>고3 생활은 피곤한게 일상이였습니다. 학교를 끝나고 가는거다보니 상당히 심신이 지쳐있는 상태였고, 저녁을 먹고나면 졸기 십상인 상태였습니다. 하지먼 선생님들의 코칭 하에 면학 분위기를 형성해주시고, 잠을 쫓아주셔서 유용하고 좋았습니다.</v>
       </c>
       <c r="H264" t="str">
-        <v>여러 사설모의고사가 있지만, 이투스 모의고사를 통해 수능에 나올 유형이나 내용, 또한 나오진 않지만 공부에 도움이 되는 유형까지 다양하게 공부할수 있었고, 수능 직전에 시간계산을 할때도 이투스 모의고사가 약방의 감초역할을 해줬습니다.</v>
+        <v>여러 사설모의고사가 있지만, 이투스 모의고사를 통해 수능에 나올 유형이나 내용, 또한 나오진 않지만 공부에 도움이 되는 유형까지 다양하게 공부할 수 있었고, 수능 직전에 시간계산을 할때도 이투스 모의고사가 약방의 감초역할을 해줬습니다.</v>
       </c>
       <c r="I264" t="str" xml:space="preserve">
         <v xml:space="preserve">항상 공부에 도움 주셔서 감사했고, 추후에 다시 입시를 하게될때도 이투스를 찾고싶습니다._x000d_
@@ -9970,7 +9970,7 @@
         <v>반수하고 6월에 기숙학원에 들어와서 어떤 선생님에 수업을 들어야할지 고민하던 중 이투스 이천 기숙학원에 계시는 담당 선생님의 학습 상담을 통해 빠르게 공부의 방향을 잡고 진도를 나갈 수 있었습니다.</v>
       </c>
       <c r="F265" t="str">
-        <v>이투스 이천 247 기숙학원에 계시는 담당선생님께서 매주 상담을 진행하시며 플레너에 계획한 계획을 잘 지켰는지 매주 검사하고 방향성을 정하는 시간을 가졌는데요. 이 덕분에 학습 분량 조절을 원활히 할 수 있었습니다</v>
+        <v>이투스 이천 247 기숙학원에 계시는 담당 선생님께서 매주 상담을 진행하시며 플레너에 계획한 계획을 잘 지켰는지 매주 검사하고 방향성을 정하는 시간을 가졌는데요. 이 덕분에 학습 분량 조절을 원활히 할 수 있었습니다</v>
       </c>
       <c r="G265" t="str">
         <v>독서실에 있으면 다른 생각이 들기 마련인데, 와이파이 방화벽이 정말 잘 되어있어 공부에만 집중할 수 있었습니다. 그 덕분에 이투스247 기숙학원에 있는 동안에는 공부에만 몰두하여 좋은 성적을 거둘 수 있었던 거 같습니다.</v>
@@ -9979,10 +9979,10 @@
         <v>이투스 전국모의고사를 매달 보는 것이 좋았습니다. 이투스 전국모의고사를 통해 다른 친구들과 나의 실력을 비교하는 기회를 제공받을 수 있었고, 무엇이 부족한지 파악할 수 있었습니다.</v>
       </c>
       <c r="I265" t="str">
-        <v>기숙학원에 있는동안 잘 케어해주셔서 감사합니다. 담임선생님의 철저한 학습관리와 멘토링 덕분에 반수에 성공해서 더 좋은 대학에 다닐 수 있게 되었습니다. 이투스247 기숙학원에서 관리해주셔서 감사합니다.</v>
+        <v>기숙학원에 있는동안 잘 케어해주셔서 감사합니다. 담임 선생님의 철저한 학습 관리와 멘토링 덕분에 반수에 성공해서 더 좋은 대학에 다닐 수 있게 되었습니다. 이투스247 기숙학원에서 관리해주셔서 감사합니다.</v>
       </c>
       <c r="J265" t="str">
-        <v>사소한 부분까지 함께 의견을 나누며 의지할 수 있는 선생님이 계셨다는 점이 수험생활의 작은 힘이 되었어요.</v>
+        <v>사소한 부분까지 함께 의견을 나누며 의지할 수 있는 선생님이 계셨다는 점이 수험 생활의 작은 힘이 되었어요.</v>
       </c>
       <c r="K265" t="str">
         <v/>
@@ -10002,20 +10002,20 @@
         <v>N수생</v>
       </c>
       <c r="E266" t="str" xml:space="preserve">
-        <v xml:space="preserve">독재학원에서의 코칭 시스템은 단순한 학습 관리 수준을 넘어, 수험생활 전반을 안정적으로 유지할 수 있도록 돕는 장치라는 점에서 특히 유용했습니다. 그중에서도 생활상담 중심의 멘토링은 제가 공부를 지속할 수 있게 만든 핵심 요소였습니다._x000d_
+        <v xml:space="preserve">독재학원에서의 코칭 시스템은 단순한 학습 관리 수준을 넘어, 수험 생활 전반을 안정적으로 유지할 수 있도록 돕는 장치라는 점에서 특히 유용했습니다. 그중에서도 생활상담 중심의 멘토링은 제가 공부를 지속할 수 있게 만든 핵심 요소였습니다._x000d_
 _x000d_
-우선, 수험생활은 장기간 이어지기 때문에 집중력이나 의지가 일정하게 유지되기 어렵습니다. 실제로 하루 공부량보다 더 중요한 것은 ‘흐름을 유지하는 것’인데, 생활상담을 통해 이 흐름이 무너지지 않도록 지속적으로 점검받을 수 있었습니다. 예를 들어, 수면 패턴이 흐트러지거나 식사 시간이 불규칙해질 때 이를 바로 잡아주는 피드백을 받을 수 있었고, 이는 곧 학습 효율의 회복으로 이어졌습니다._x000d_
+우선, 수험 생활은 장기간 이어지기 때문에 집중력이나 의지가 일정하게 유지되기 어렵습니다. 실제로 하루 공부량보다 더 중요한 것은 ‘흐름을 유지하는 것’인데, 생활상담을 통해 이 흐름이 무너지지 않도록 지속적으로 점검받을 수 있었습니다. 예를 들어, 수면 패턴이 흐트러지거나 식사 시간이 불규칙해질 때 이를 바로 잡아주는 피드백을 받을 수 있었고, 이는 곧 학습 효율의 회복으로 이어졌습니다._x000d_
 _x000d_
 또한, 단순히 공부 계획만을 점검하는 것이 아니라 개인의 상태를 함께 고려해주는 점이 인상적이었습니다. 슬럼프가 오거나 잡생각이 많아질 때, 이를 방치하지 않고 상담을 통해 원인을 짚어주고 해결 방향을 제시해 주었기 때문에 감정적인 소모를 줄일 수 있었습니다. 특히 재수 기간에는 스스로를 객관적으로 바라보기 어려운데, 코치 선생님과의 대화를 통해 현재 상태를 정리하고 다시 집중할 수 있는 계기를 만들 수 있었습니다._x000d_
 _x000d_
 코칭 시스템의 또 다른 장점은 ‘강제성 없는 관리’였습니다. 단순히 규칙을 따르게 하는 방식이 아니라, 스스로 납득하고 실천할 수 있도록 유도하는 구조였기 때문에 부담감 없이 지속할 수 있었습니다. 이는 단기적인 성과보다는 장기적인 습관 형성에 도움이 되었고, 결과적으로 안정적인 공부 루틴을 만드는 데 큰 역할을 했습니다._x000d_
 _x000d_
-마지막으로, 생활상담을 포함한 코칭 시스템은 공부 외적인 부분까지 함께 관리해 준다는 점에서 의미가 있었습니다. 수험생활은 공부만 잘한다고 해결되는 것이 아니라, 체력, 멘탈, 생활습관이 균형을 이루어야 한다는 것을 느꼈고, 이 시스템은 그 균형을 유지하도록 도와주었습니다._x000d_
+마지막으로, 생활상담을 포함한 코칭 시스템은 공부 외적인 부분까지 함께 관리해 준다는 점에서 의미가 있었습니다. 수험 생활은 공부만 잘한다고 해결되는 것이 아니라, 체력, 멘탈, 생활 습관이 균형을 이루어야 한다는 것을 느꼈고, 이 시스템은 그 균형을 유지하도록 도와주었습니다._x000d_
 _x000d_
 이러한 점에서 이투스247의 코칭 시스템은 단순한 관리가 아니라 ‘지속 가능한 공부 환경’을 만들어주는 중요한 기반이었다고 생각합니다.</v>
       </c>
       <c r="F266" t="str" xml:space="preserve">
-        <v xml:space="preserve">이투스247학원의 학습 관리 시스템 중에서 가장 만족스러웠던 부분은 1:1 질의응답 시스템이었습니다. 수험생활에서 가장 큰 비효율 중 하나는 ‘막힌 상태로 시간을 보내는 것’인데, 이 시스템은 그 비효율을 최소화해 준다는 점에서 매우 유용했습니다._x000d_
+        <v xml:space="preserve">이투스247학원의 학습 관리 시스템 중에서 가장 만족스러웠던 부분은 1:1 질의응답 시스템이었습니다. 수험 생활에서 가장 큰 비효율 중 하나는 ‘막힌 상태로 시간을 보내는 것’인데, 이 시스템은 그 비효율을 최소화해 준다는 점에서 매우 유용했습니다._x000d_
 _x000d_
 공부를 하다 보면 개념이 완전히 이해되지 않거나, 문제 풀이 과정에서 특정 단계가 납득되지 않는 순간이 반드시 생깁니다. 이때 혼자서 해결하려고 오래 붙잡고 있으면 시간만 소모되고 집중력도 떨어지기 쉬운데, 1:1 질의응답을 통해 필요한 순간에 바로 질문하고 피드백을 받을 수 있었습니다. 특히 단순히 정답이나 풀이를 알려주는 데서 그치는 것이 아니라, 제가 어떤 부분에서 막혔는지를 짚어주고 사고 과정을 교정해 준다는 점이 큰 도움이 되었습니다._x000d_
 _x000d_
@@ -10025,25 +10025,25 @@
 _x000d_
 또한 재수 기간에는 혼자 공부하는 시간이 길어지면서 확신이 흔들릴 때가 많은데, 질의응답을 통해 내가 이해한 방향이 맞는지 확인받을 수 있다는 점에서도 심리적으로 안정감을 얻을 수 있었습니다. 단순히 지식을 전달받는 것을 넘어, 공부 방향에 대한 확신을 강화해 주는 역할을 했다고 생각합니다._x000d_
 _x000d_
-결과적으로 1:1 질의응답 시스템은 시간 낭비를 줄이고, 학습의 정확도를 높이며, 스스로의 약점을 인식하게 만드는 데 기여했습니다. 이러한 점에서 이 시스템은 수험생활의 효율과 안정성을 동시에 높여주는 핵심적인 요소였다고 느꼈습니다.</v>
+결과적으로 1:1 질의응답 시스템은 시간 낭비를 줄이고, 학습의 정확도를 높이며, 스스로의 약점을 인식하게 만드는 데 기여했습니다. 이러한 점에서 이 시스템은 수험 생활의 효율과 안정성을 동시에 높여주는 핵심적인 요소였다고 느꼈습니다.</v>
       </c>
       <c r="G266" t="str" xml:space="preserve">
         <v xml:space="preserve">이투스247학원의 생활 관리 시스템 중에서 가장 효과적이었다고 느낀 것은 태블릿 모니터링과 와이파이 방화벽 시스템입니다. 이 두 가지는 단순한 통제가 아니라, 공부에만 집중할 수밖에 없는 환경을 만들어 준다는 점에서 큰 의미가 있었습니다._x000d_
 _x000d_
-수험생활을 하면서 느낀 것은, 집중이 안 되는 이유가 단순히 의지가 부족해서라기보다는 주변 환경의 영향이 크다는 점이었습니다. 책상 앞에 앉아 있어도 무의식적으로 다른 사이트를 들어가거나, 잠깐 쉬려던 시간이 길어지는 경우가 자주 생깁니다. 그런데 태블릿 모니터링과 와이파이 방화벽이 이러한 요소들을 자연스럽게 차단해 주면서, 공부 외적인 선택지를 줄여주는 환경이 만들어졌습니다._x000d_
+수험 생활을 하면서 느낀 것은, 집중이 안 되는 이유가 단순히 의지가 부족해서라기보다는 주변 환경의 영향이 크다는 점이었습니다. 책상 앞에 앉아 있어도 무의식적으로 다른 사이트를 들어가거나, 잠깐 쉬려던 시간이 길어지는 경우가 자주 생깁니다. 그런데 태블릿 모니터링과 와이파이 방화벽이 이러한 요소들을 자연스럽게 차단해 주면서, 공부 외적인 선택지를 줄여주는 환경이 만들어졌습니다._x000d_
 _x000d_
 특히 태블릿 모니터링 시스템은 단순히 통제받는 느낌이 아니라, 스스로를 점검하게 만드는 역할을 했습니다. ‘지금 내가 제대로 공부에 집중하고 있는지’를 계속 인식하게 해 주었고, 그 덕분에 흐트러질 수 있는 순간들을 빠르게 바로잡을 수 있었습니다. 혼자 공부할 때는 놓치기 쉬운 부분들을 잡아주면서, 하루 공부의 흐름을 안정적으로 유지하는 데 도움이 되었습니다._x000d_
 _x000d_
 와이파이 방화벽 역시 실질적인 도움이 컸습니다. 인터넷 강의를 듣는 과정에서 다른 사이트나 SNS로 쉽게 넘어갈 수 있는 상황 자체가 차단되기 때문에, 굳이 의지로 참으려고 하지 않아도 자연스럽게 공부에 집중할 수 있었습니다. 선택지가 줄어들수록 오히려 집중은 더 쉬워진다는 것을 체감할 수 있었습니다._x000d_
 _x000d_
-이 시스템의 가장 큰 장점은 자기통제에 대한 부담을 줄여준다는 점이라고 생각합니다. 보통 수험생활은 스스로를 계속 통제해야 한다는 압박이 큰데, 이투스247에서는 그 부담을 환경이 어느 정도 대신 나눠 갖는 구조였습니다. 덕분에 에너지를 버티는 데 쓰기보다 실제 공부에 집중할 수 있었고, 장기적으로도 지치지 않고 루틴을 유지할 수 있었습니다._x000d_
+이 시스템의 가장 큰 장점은 자기통제에 대한 부담을 줄여준다는 점이라고 생각합니다. 보통 수험 생활은 스스로를 계속 통제해야 한다는 압박이 큰데, 이투스247에서는 그 부담을 환경이 어느 정도 대신 나눠 갖는 구조였습니다. 덕분에 에너지를 버티는 데 쓰기보다 실제 공부에 집중할 수 있었고, 장기적으로도 지치지 않고 루틴을 유지할 수 있었습니다._x000d_
 _x000d_
 또한 이러한 환경은 단순한 제한에 그치지 않고, 공부 습관을 형성하는 데에도 영향을 주었습니다. 처음에는 다소 불편하게 느껴질 수 있었지만, 시간이 지나면서 자연스럽게 집중하는 패턴이 자리 잡았고, 이후에는 별도의 통제가 없어도 스스로 몰입 상태를 유지할 수 있게 되었습니다._x000d_
 _x000d_
-결과적으로 태블릿 모니터링과 와이파이 방화벽은 단순한 관리 수단이 아니라, 수험생활의 효율과 지속성을 높여주는 핵심적인 시스템이었다고 생각합니다. 공부에 방해가 되는 요소를 줄이고, 안정적인 학습 환경을 만들어 준다는 점에서 가장 만족스러웠습니다.</v>
+결과적으로 태블릿 모니터링과 와이파이 방화벽은 단순한 관리 수단이 아니라, 수험 생활의 효율과 지속성을 높여주는 핵심적인 시스템이었다고 생각합니다. 공부에 방해가 되는 요소를 줄이고, 안정적인 학습 환경을 만들어 준다는 점에서 가장 만족스러웠습니다.</v>
       </c>
       <c r="H266" t="str" xml:space="preserve">
-        <v xml:space="preserve">이투스247학원의 콘텐츠 중에서 가장 만족스러웠던 부분은 이투스 구독권 제공이었습니다. 수험생활에서 인강은 선택이 아니라 필수에 가까운데, 다양한 강의를 자유롭게 활용할 수 있다는 점에서 매우 큰 도움이 되었습니다._x000d_
+        <v xml:space="preserve">이투스247학원의 콘텐츠 중에서 가장 만족스러웠던 부분은 이투스 구독권 제공이었습니다. 수험 생활에서 인강은 선택이 아니라 필수에 가까운데, 다양한 강의를 자유롭게 활용할 수 있다는 점에서 매우 큰 도움이 되었습니다._x000d_
 _x000d_
 우선 가장 큰 장점은 ‘선택의 폭’이 넓어진다는 점이었습니다. 과목별로 강의 스타일이나 설명 방식이 다르기 때문에, 나에게 맞는 강사를 찾는 과정이 중요한데, 구독권이 제공되면서 여러 강의를 부담 없이 비교하고 선택할 수 있었습니다. 덕분에 특정 강사에 얽매이지 않고, 내 이해도에 맞는 강의를 찾아가는 과정이 훨씬 수월해졌습니다._x000d_
 _x000d_
@@ -10056,13 +10056,13 @@
 결과적으로 이투스 구독권은 단순한 ‘혜택’이 아니라, 학습의 방향성과 효율을 동시에 높여주는 핵심적인 콘텐츠라고 느꼈습니다. 다양한 강의를 자유롭게 활용할 수 있는 환경이 만들어지면서, 스스로에게 맞는 공부 방식을 찾아가는 데 큰 도움이 되었고, 이는 장기적인 학습 지속에도 긍정적인 영향을 주었습니다.</v>
       </c>
       <c r="I266" t="str" xml:space="preserve">
-        <v xml:space="preserve">수험생활 동안 항상 곁에서 방향을 잡아주시고, 흔들릴 때마다 다시 중심을 잡을 수 있도록 도와주신 선생님들께 진심으로 감사드립니다._x000d_
+        <v xml:space="preserve">수험 생활 동안 항상 곁에서 방향을 잡아주시고, 흔들릴 때마다 다시 중심을 잡을 수 있도록 도와주신 선생님들께 진심으로 감사드립니다._x000d_
 _x000d_
 긴 시간 혼자 공부하다 보면 지치고 불안해질 때가 많았는데, 그럴 때마다 선생님들께서 건네주신 한마디 한마디가 큰 힘이 되었습니다. 단순히 공부를 관리해 주시는 것을 넘어서, 학생 한 명 한 명의 상태를 살피고 진심으로 응원해 주신다는 느낌을 많이 받았습니다._x000d_
 _x000d_
 특히 생활 관리와 학습 코칭을 통해 제가 무너지지 않고 끝까지 버틸 수 있었던 것 같습니다. 스스로는 잘하고 있는지 확신이 없을 때도 많았지만, 선생님들께서 방향을 짚어주시고 꾸준히 점검해 주신 덕분에 흔들리지 않고 제 페이스를 유지할 수 있었습니다._x000d_
 _x000d_
-수험생활을 돌아보면 힘들었던 순간들도 많았지만, 그 과정에서 선생님들의 도움과 응원이 있었기 때문에 끝까지 해낼 수 있었다고 생각합니다. 단순히 성적 향상을 넘어서, 스스로를 관리하고 버티는 힘을 기를 수 있었던 시간이었다는 점에서 더욱 의미가 깊습니다._x000d_
+수험 생활을 돌아보면 힘들었던 순간들도 많았지만, 그 과정에서 선생님들의 도움과 응원이 있었기 때문에 끝까지 해낼 수 있었다고 생각합니다. 단순히 성적 향상을 넘어서, 스스로를 관리하고 버티는 힘을 기를 수 있었던 시간이었다는 점에서 더욱 의미가 깊습니다._x000d_
 _x000d_
 그동안 정말 감사했습니다. 앞으로도 이투스247학원이 많은 학생들에게 좋은 방향을 제시해 주는 공간으로 남기를 진심으로 응원하겠습니다.</v>
       </c>
@@ -10087,10 +10087,10 @@
         <v>N수생</v>
       </c>
       <c r="E267" t="str">
-        <v>공부를 어떻게 해야할지 갈피를 잡을 수 있었고 마음이 흔들릴 때마다 벗어나지 않고 꾸준히 공부를 이어갈 수 있었다. 또한 공부 관련해서 방법이 고민될 때 물어볼 수 있는 사람이 있다는 것이 좋았다.</v>
+        <v>공부를 어떻게 해야 할지 갈피를 잡을 수 있었고 마음이 흔들릴 때마다 벗어나지 않고 꾸준히 공부를 이어갈 수 있었다. 또한 공부 관련해서 방법이 고민될 때 물어볼 수 있는 사람이 있다는 것이 좋았다.</v>
       </c>
       <c r="F267" t="str">
-        <v>혼자 공부했으면 하루를 어떻게 보내야 할지 효율적으로 계획하는 것이 힘들었을 텐데 일주일 단위로 공부해야할 것을 계획할 수 있어서 좋았다. 또한 공부가 얼마나진행되었는지 확인할 수 있어서 밀리지 않고 꾸준히 할 수 있었던 것 같다.</v>
+        <v>혼자 공부했으면 하루를 어떻게 보내야 할지 효율적으로 계획하는 것이 힘들었을 텐데 일주일 단위로 공부해야 할 것을 계획할 수 있어서 좋았다. 또한 공부가 얼마나진행되었는지 확인할 수 있어서 밀리지 않고 꾸준히 할 수 있었던 것 같다.</v>
       </c>
       <c r="G267" t="str">
         <v>다른 어플들을 들어갈 수 있었으면 인강을 듣거나 공부를 할 때 유튜브 등을 보고 싶은 마음을 제어하기가 힘들었을 텐데 강제적으로 그런 것들을 막아주니까 공부에만 집중을 할 수 있었다.</v>
@@ -10172,7 +10172,7 @@
         <v>저는 1년이 아닌 6개월만 다녔지만 1년간 수고 많으셨습니다! 매년 많은 학생들을 만나고 학샹들을 위해 희생해주셔서 감사합니다. 선생님들의 노력으로 많은 학생들이 도움을 받고 꿈을 펼치러 갈 수 있었고 갈 것 입니다! 다시 한 번 수고많으셨습니다!</v>
       </c>
       <c r="J269" t="str">
-        <v>개별 학습 데이터와 플래너, 방화벽 관리 덕분에 막막함을 줄이고 수험생활을 잘 마무리했어요.</v>
+        <v>개별 학습 데이터와 플래너, 방화벽 관리 덕분에 막막함을 줄이고 수험 생활을 잘 마무리했어요.</v>
       </c>
       <c r="K269" t="str">
         <v>방화벽</v>
@@ -10233,7 +10233,7 @@
         <v>의대생,스카이생의 똑똑한 해설을 그날 그날 질문을 할 수 있는게 너무 좋았어요. 시간도 20분정도로 넉넉했고 뒤에 사람이 없으면 더 질문할 수도 있었어요. 또한 고민 상담, 멘탈 관리, 공부 팁 등도 자주 알려주셔서 너무 유용하게 잘 이용했습니다.</v>
       </c>
       <c r="G271" t="str">
-        <v>앞에서 말했듯이 쉬는시간에 피곤해서 자는 경우가 많은데 스카에서 자게되면 깨워줄 사람의 부재로 너무 오래 잠들까 걱정돼서 맘편히 못자는데 이투스에선 선생님들이 돌아가면서 깨워주셔서 맘편히 깊게 잠들 수 있어요. 또한 수업시간에 졸 때도 깨워주시고 한번씩 잠 깨라고 사탕도 주셨는데 너무 도움이 많이 됐습니다.</v>
+        <v>앞에서 말했듯이 쉬는시간에 피곤해서 자는 경우가 많은데 스카에서 자게되면 깨워줄 사람의 부재로 너무 오래 잠들까 걱정돼서 맘편히 못자는데 이투스에선 선생님들이 돌아가면서 깨워주셔서 맘편히 깊게 잠들 수 있어요. 또한 수업시간에 졸 때도 깨워주시고 한 번씩 잠 깨라고 사탕도 주셨는데 너무 도움이 많이 됐습니다.</v>
       </c>
       <c r="H271" t="str">
         <v>정승제 선생님같이 좋은 선생님이신데 이투스를 구독하거나 단일 강의는 듣기엔 돈이 아까워서 못듣는 이투스 강사들을 부담없이 필요한 부분만 들을 수 있는게 좋았고, 그만큼 들을 수 있는 강사가 늘어난거니 그 강사의 모의고사나 엔제 등을 더 잘 접할 수 있게 됐습니다.</v>
@@ -10345,7 +10345,7 @@
         <v>모의고사지를 지금은 용지를 파는 데가 많아 졌지만 없었을때는 용지의 느낌을 살려 실제 시험지와 최대한 비슷한 느낌을 살려준 느낌과 실제 시험과 유사한 경향의 문제 유형이 나와주어서 이투스 모의고사지 월마다 풀어본 경험이 도움이 많이 되었다.</v>
       </c>
       <c r="I274" t="str">
-        <v>강지희 선생님 외 영어 국어 선생님 지난 1년동안 여러 공부 방법과 계획의 방향을 알려주셔서 감사합니다. 또한 출석 담당자 선생님과 풀이 담당 선생님께서도 항상 최선을 다하시는 모습을 보여 주셔서 감사합니다. 또한 맨 처음 들어 갔을때 학원 소개와 저의 다짐을 물어보시고 신중히 결정하라는 원장 선생님과 부원장 선생님께도 감사 인사를 드립니다.</v>
+        <v>강지희 선생님 외 영어 국어 선생님 지난 1년 동안 여러 공부 방법과 계획의 방향을 알려주셔서 감사합니다. 또한 출석 담당자 선생님과 풀이 담당 선생님께서도 항상 최선을 다하시는 모습을 보여 주셔서 감사합니다. 또한 맨 처음 들어 갔을때 학원 소개와 저의 다짐을 물어보시고 신중히 결정하라는 원장 선생님과 부원장 선생님께도 감사 인사를 드립니다.</v>
       </c>
       <c r="J274" t="str">
         <v>저의 루틴을 유지할 수 있도록 많은 도움을 주시고 살펴주신 선생님께 감사하다고 말씀드리고 싶어요.</v>
@@ -10368,13 +10368,13 @@
         <v>N수생</v>
       </c>
       <c r="E275" t="str">
-        <v>전반적인 성적, 부족한 과목과 파트를 자세히 파악해주시고 이를 토대로 구체적인 학습 방향을 제시해주셔서 학습 계획 수립에 큰 도움이 되었습니다. 특히 저는 수학과 탐구 과목이 부족하였는데, 제시해주신 학습 방향대로 공부하니 성적향상을 거둘 수 있었습니다.</v>
+        <v>전반적인 성적, 부족한 과목과 파트를 자세히 파악해주시고 이를 토대로 구체적인 학습 방향을 제시해주셔서 학습 계획 수립에 큰 도움이 되었습니다. 특히 저는 수학과 탐구 과목이 부족하였는데, 제시해주신 학습 방향대로 공부하니 성적 향상을 거둘 수 있었습니다.</v>
       </c>
       <c r="F275" t="str">
         <v>수많은 콘텐츠가 넘쳐나는 현재 대학 입시 상황에서 무슨 교재와 강의를 선택해야 저의 현재 성적대에 도움이 될지 잘 모르겠어서 힘들었었는데 분석하신 제 성적을 바탕으로 각 과목의 교재와 강의를 꼼꼼히 추천해 주셔서 크게 도움이 되었습니다.</v>
       </c>
       <c r="G275" t="str">
-        <v>아무래도 수험생활의 가장 큰 적은 인터넷으로 즐길 수 있는 오락거리와 미디어라고 생각합니다. 하지만 이투스 247에서는 와이파이 방화벽을 통해 애초에 접속 가능성을 막고 학습사이트만 들어갈 수 있게 설계되어있어 스스로 자제력이 부족해 인터넷 사용시간이 많았던 저에게 도움이 되었습니다.</v>
+        <v>아무래도 수험 생활의 가장 큰 적은 인터넷으로 즐길 수 있는 오락거리와 미디어라고 생각합니다. 하지만 이투스 247에서는 와이파이 방화벽을 통해 애초에 접속 가능성을 막고 학습사이트만 들어갈 수 있게 설계되어있어 스스로 자제력이 부족해 인터넷 사용시간이 많았던 저에게 도움이 되었습니다.</v>
       </c>
       <c r="H275" t="str">
         <v>영어가 현재 수능 체제에서 절대평가 과목이기도 해서 영어를 소홀히 하는 경향도 있었고 특히나 단어같은 경우는 귀찮아서 안 외우는 경우가 많았습니다. 단어를 선별해서 자료를 주신 덕에 외우기도 편리했고 다같이 시험을 봐 강제성이 생긴 덕분에 꾸준히 단어를 외울 수 있었습니다.</v>
@@ -10455,7 +10455,7 @@
 실제로 국어 김민정 선생님을 구독권을 받은 이후에 알고 강의 들으면서 국어 공부에 많이 도움이 되었다.</v>
       </c>
       <c r="I277" t="str">
-        <v>과목 선생님들, 담임선생님들, 오전/오후/야간 선생님들 모두 덕분에 좋은 환경에서 때론 웃고 울면서 1년을 보낼 수 있었습니다. 특히 이천기숙 선생님들 더더 위로 가시고 돈 많이 버세요 감사했습니다 ♥</v>
+        <v>과목 선생님들, 담임 선생님들, 오전/오후/야간 선생님들 모두 덕분에 좋은 환경에서 때론 웃고 울면서 1년을 보낼 수 있었습니다. 특히 이천기숙 선생님들 더더 위로 가시고 돈 많이 버세요 감사했습니다 ♥</v>
       </c>
       <c r="J277" t="str">
         <v>선생님께서 매주 저의 학습을 점검해 주시는 것이 무척이나 든든하게 느껴졌고, 그래서 더욱 열심히 공부할 수 있었습니다!</v>
@@ -10478,7 +10478,7 @@
         <v>N수생</v>
       </c>
       <c r="E278" t="str">
-        <v>취약 유형을 담임선생님과 상담하면서 집중적으로 끌어올릴 수 있었다.또한 공부하다가 막히는 부분을 혼자 해결하기 힘들었는데 선생님과 상담하면서 방향성을 잡을 수 있게 되었다.독재의 단점이 혼자 공부하면서 방향성을 잡기 힘든건데 수원정자점에서 담임샘과 상담이 이러한 부분을 해결해주었다</v>
+        <v>취약 유형을 담임 선생님과 상담하면서 집중적으로 끌어올릴 수 있었다.또한 공부하다가 막히는 부분을 혼자 해결하기 힘들었는데 선생님과 상담하면서 방향성을 잡을 수 있게 되었다.독재의 단점이 혼자 공부하면서 방향성을 잡기 힘든건데 수원정자점에서 담임샘과 상담이 이러한 부분을 해결해주었다</v>
       </c>
       <c r="F278" t="str">
         <v>인강의 경우 정말 괜찮은 강의가 많다 보니 그 중에 어떤것을 들어야 할지 많이 고민이 되었다. 그럴때마다 담임샘께 여쭤보면서 지금 나한태 적절한 수준의 강의는 무엇일지 알려주시고 추천을 해주셨다. 교재도 담임샘이 추천해주신 교재로 사용했었고 실제로 많이 도움되었다고 생각했다</v>
@@ -10490,7 +10490,7 @@
         <v>정시 공부를 하다보면 빠질 수 없는것이 실전 연습이다.이투스 학원에서 주관하는 실전 모의고사 연습은 실전 대비하기에 가장 효과적이었다. 매달 나오는 성적으로 현재 내 위치가 어느 정도인지 체감할 수 있었고 그에 따라 공부 계획도 수정할 수 있었다</v>
       </c>
       <c r="I278" t="str">
-        <v>수능공부 1년동안 옆에서 많이 도와주시고 지켜봐주셔서 감사합니다! 공부하면서 많이 힘들고 불안할때마다 선생님들께서 조언주신것이 너무 도움되었어요.그리고 이벤트도 자주 진행해주셔서 버틸 수 있었습니다 감사합니다!</v>
+        <v>수능공부 1년 동안 옆에서 많이 도와주시고 지켜봐주셔서 감사합니다! 공부하면서 많이 힘들고 불안할때마다 선생님들께서 조언주신것이 너무 도움되었어요.그리고 이벤트도 자주 진행해주셔서 버틸 수 있었습니다 감사합니다!</v>
       </c>
       <c r="J278" t="str">
         <v>주기적인 학습 상담과 1:1 질의응답, 휴대폰 관리와 모의고사 덕분에 끝까지 차분하게 공부할 수 있었어요.</v>
@@ -10525,7 +10525,7 @@
         <v>평소 영어에서 단어가 부족해서 많이 헤매고 그러면서도 열심히 외우다가 어느순간 안하게 됐습니다. 하지만 이투스에 와서 매일 시험을 보고 시험을 위해서라도 꾸준히 외우니 실력이 많이 늘어서 좋았어요</v>
       </c>
       <c r="I279" t="str">
-        <v>짧은 썸머기간동안 만나뵀지만 모두 진심으로 응원하고 격려해주셔서 너무 감사했습니다. 기숙 사감 선생님들도 생활 관리 선생님들도 과목 담당 선생님,논술 선생님, 그리고 저희 담당선생님 모두 최적의 공부환경과 효율적인 학습을 위해 최선을 다해주셨어요! 덕분에 기숙생활 힘들지 않고 보람있게 마무리했습니다!</v>
+        <v>짧은 썸머기간동안 만나뵀지만 모두 진심으로 응원하고 격려해주셔서 너무 감사했습니다. 기숙 사감 선생님들도 생활 관리 선생님들도 과목 담당 선생님,논술 선생님, 그리고 저희 담당 선생님 모두 최적의 공부환경과 효율적인 학습을 위해 최선을 다해주셨어요! 덕분에 기숙생활 힘들지 않고 보람있게 마무리했습니다!</v>
       </c>
       <c r="J279" t="str">
         <v>스마트폰은 통제하기 어렵고 가장 큰 방해가 되는 요인인데 휴대폰을 제출하여 더 잘 집중할 수 있었어요.</v>
@@ -10871,7 +10871,7 @@
         <v>궁금한 정보를 다 알수있고 정보를 많이 알수록 수시나 정시 기회도 더 많아지고 그 걸 할지말지 선택만 하면 돼서 좋았다 모르고 못한거랑 알고 안한건 다르니까 재수도 아니라 고3이라 학교도 다니면서 병행하는게 오히려 더 좋았던 거 같다 하루종일 학원에 있는 것보다 학교랑 왔다갔다 공부환경 바꿔가며 하는게 오히려 집중도 더 잘되고 뿌듯했다</v>
       </c>
       <c r="F289" t="str">
-        <v>학원을 등록한 제일 큰 이유가 혼자서 공부하면 과목 편식을 너무 많이 하기도 하고 어디서부터 시작해야 될지 막막해서였는데 이투스에서 준 플래너는 주간 플래너라 일주일에 얼마나 공부하는지 다 보이고 과목마다 공부시간도 아니까 과목편식을 안하게 됐다</v>
+        <v>학원을 등록한 제일 큰 이유가 혼자서 공부하면 과목 편식을 너무 많이 하기도 하고 어디서부터 시작해야 될지 막막해서였는데 이투스에서 준 플래너는 주간 플래너라 일주일에 얼마나 공부하는지 다 보이고 과목마다 공부 시간도 아니까 과목편식을 안하게 됐다</v>
       </c>
       <c r="G289" t="str">
         <v>핸드폰이 제일 집중흐트리기 쉬운 물건인데 등원하면 핸드폰을 수거해서 방해요소 없이 집중하기 좋았다 눈에 핸드폰이 안보이는게 제일 큰 장점이다 하원해도 핸드폰 수거함에서 폰 안챙겨가면 그 날 저녁에 잠도 일찍 자고 폰을 맡길데가 있다는 게 좋았다</v>
@@ -10903,10 +10903,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E290" t="str">
-        <v>고3 현역이었는데 N수생에 비해 입시경험이 부족할 수 밖에 없고 처음 보는 수능이라 뭘 해야할지 몰라 방황했었습니다. 이투스247에서 입시상담을 통해 수능을 보기위해 어떤식으로 공부하면 좋을지 방향성을 잡을 수 있어서 좋았습니다. 또한 과목별로 상담을 통해 어떤 점이 부족한지 알 수 있었던 점 또한 매우 유용했다고 생각합니다.</v>
+        <v>고3 현역이었는데 N수생에 비해 입시경험이 부족할 수 밖에 없고 처음 보는 수능이라 뭘 해야 할지 몰라 방황했었습니다. 이투스247에서 입시상담을 통해 수능을 보기위해 어떤식으로 공부하면 좋을지 방향성을 잡을 수 있어서 좋았습니다. 또한 과목별로 상담을 통해 어떤 점이 부족한지 알 수 있었던 점 또한 매우 유용했다고 생각합니다.</v>
       </c>
       <c r="F290" t="str">
-        <v>평소 계획을 세우고 공부하는 편은 아니었으며 생각없이 문제만 풀다보니 성적이 정체되어있는 느낌을 받았었습니다. 플래너 작성법을 배우고 같이 공부계획을 짜며 체계적으로 공부하다보니 성적이 상승할 수 있었던 것 같고 유용했습니다.</v>
+        <v>평소 계획을 세우고 공부하는 편은 아니었으며 생각없이 문제만 풀다보니 성적이 정체되어있는 느낌을 받았었습니다. 플래너 작성법을 배우고 같이 공부 계획을 짜며 체계적으로 공부하다보니 성적이 상승할 수 있었던 것 같고 유용했습니다.</v>
       </c>
       <c r="G290" t="str">
         <v>학원에만 계속있다보면 놀고싶기도하고 공부도 잘 안될 때도 있는데 감독관분들께서 마음 다잡아주시고 상담등의 여러방식으로 공부에 집중할 수 있게 도와주신 점이 좋았습니다. 여름방학때 많이 헤이해졌던 것 같은데 도움 많이 받았던 것 같습니다.</v>
@@ -10938,13 +10938,13 @@
         <v>N수생</v>
       </c>
       <c r="E291" t="str">
-        <v>매주 담임선생님과의 학습 상담을 과목별 맞춤 전략을 세우며 지속적으로 변하는 저의 학습 진행상황에 맞도록 공부할 수 있는 점이 좋았습니다. 또한 자주 치르는 실전 모의고사에서의 피드백도 매번 진행되어 실전적 측면에서의 도움도 많이 받을 수 있었습니다.</v>
+        <v>매주 담임 선생님과의 학습 상담을 과목별 맞춤 전략을 세우며 지속적으로 변하는 저의 학습 진행상황에 맞도록 공부할 수 있는 점이 좋았습니다. 또한 자주 치르는 실전 모의고사에서의 피드백도 매번 진행되어 실전적 측면에서의 도움도 많이 받을 수 있었습니다.</v>
       </c>
       <c r="F291" t="str">
-        <v>저는 고3때 정시를 준비하던 학생이었습니다. 전과목의 성적을 모두 챙기는 것이 중요한 정시 전형에서, 제가 흥미를 느끼는 과목만을 선택적으로 공부하는 저의 학습 패턴은 실패요인이었습니다. 그리고 이투스247 학원을 다니며 이를 매주 진행되는 일주일 간의 학습 일정 조정을 통해 극복할 수 있었고, 모든 과목을 골고루 공부하는데 큰 도움이 되었습니다.</v>
+        <v>저는 고3 때 정시를 준비하던 학생이었습니다. 전과목의 성적을 모두 챙기는 것이 중요한 정시 전형에서, 제가 흥미를 느끼는 과목만을 선택적으로 공부하는 저의 학습 패턴은 실패요인이었습니다. 그리고 이투스247 학원을 다니며 이를 매주 진행되는 일주일 간의 학습 일정 조정을 통해 극복할 수 있었고, 모든 과목을 골고루 공부하는데 큰 도움이 되었습니다.</v>
       </c>
       <c r="G291" t="str">
-        <v>아침8시부터 밤12시까지 오랜시간의 공부를 특별한 여가생활 없이 매일 반복해낸다는 것은 저에게 정신적,체력적으로 상당한 부담이 되었습니다. 그렇기에 피로해진 상태의 저는 늘 졸음과 싸우고는 했습니다. 이때 이투스247의 졸음지도 및 관리는 집중력을 유지하여 공부하는 순공부시간 확보에 큰 도움이 되었습니다.</v>
+        <v>아침8시부터 밤12시까지 오랜시간의 공부를 특별한 여가생활 없이 매일 반복해낸다는 것은 저에게 정신적,체력적으로 상당한 부담이 되었습니다. 그렇기에 피로해진 상태의 저는 늘 졸음과 싸우고는 했습니다. 이때 이투스247의 졸음지도 및 관리는 집중력을 유지하여 공부하는 순공부 시간 확보에 큰 도움이 되었습니다.</v>
       </c>
       <c r="H291" t="str">
         <v>우선, 매일 등원과 동시에 아침에 풀어야하는 국어 지문 1지문은 평가원 및 교육청 기출을 자주 접할 수 있도록 도와주었을 뿐 아니라 하루의 집중력을 긴 글을 통해 깨워주어 효율적의 학습의 시작을 마련해주었습니다. 그에 더해 매일 치러지는 영단어시험은 수능에 필요한 영단어들을 반복적으로 학습할 수 있도록 해주어 어휘력을 기르는데 큰 도움을 주었습니다.</v>
@@ -10973,7 +10973,7 @@
         <v>N수생</v>
       </c>
       <c r="E292" t="str">
-        <v>학습코칭이 가장 유용했습니다. 국어, 영어, 수학 과목별로 담당 선생님들이 한 분씩 계셔서 모르는 문제를 질문하거나 세부 학습플랜을 세우는 데에 큰 도움을 받았습니다. 담임선생님께 입시상담을 하고, 과목별 담당 선생님들께 코칭을 받은 덕에 성적을 빨리 향상시킬 수 있었습니다.</v>
+        <v>학습코칭이 가장 유용했습니다. 국어, 영어, 수학 과목별로 담당 선생님들이 한 분씩 계셔서 모르는 문제를 질문하거나 세부 학습플랜을 세우는 데에 큰 도움을 받았습니다. 담임 선생님께 입시상담을 하고, 과목별 담당 선생님들께 코칭을 받은 덕에 성적을 빨리 향상시킬 수 있었습니다.</v>
       </c>
       <c r="F292" t="str">
         <v>성적 리포팅 및 관리가 도움이 되었습니다. 모의고사 응시 성적과 수능 예상 점수까지 리포팅되어 직관적으로 저의 위치를 알 수 있었고, 과목 간의 밸런스를 맞추기에도 수월했습니다. 월별로 성적 추이를 비교하며 공부하니 동기부여가 되어 더 열심히 공부했던 거 같습니다.</v>
@@ -10985,7 +10985,7 @@
         <v>원래는 타 인강사이트의 패스를 수강하다가, 이투스 247 학원에서 재원생 콘텐츠로 이투스구독을 제공한 덕에 이투스 인강을 처음 수강했습니다. 스타강사들의 강의를 무료로 수강할 수 있다는게 정말 큰 메리트였습니다. 특히나 박광일, 정승제 선생님의 도움을 정말 많이 받았습니다.</v>
       </c>
       <c r="I292" t="str">
-        <v>덕분에 공부하는 방법을 알았고 공부의 재미를 깨달았습니다. 선생님들께 상담하고 질문하며 해당 과목을 더 깊게 파고들 수 있었고, 성적을 많이 올렸습니다. 아침마다 반갑게 인사해 주시고, 담임선생님이 아니더라도 관심 가지고 성적 체크해 주셔서 감사했습니다!</v>
+        <v>덕분에 공부하는 방법을 알았고 공부의 재미를 깨달았습니다. 선생님들께 상담하고 질문하며 해당 과목을 더 깊게 파고들 수 있었고, 성적을 많이 올렸습니다. 아침마다 반갑게 인사해 주시고, 담임 선생님이 아니더라도 관심 가지고 성적 체크해 주셔서 감사했습니다!</v>
       </c>
       <c r="J292" t="str">
         <v>반수로 들어왔는데 담임 선생님이 매주 학습 계획을 점검하고 방향성을 잡아주셔서 빠르게 진도를 나갈 수 있었습니다.</v>
@@ -11046,7 +11046,7 @@
         <v>모르는 문제를 구체적으로 잘 알려주고 헷갈리는 유형과 관련된 문제들을 찾아주셔서  공부하는데 많이 도움됐습니다. 공부루틴도 잡아주시고 공부에 대한 상담까지 잘 이루어져 효율적인 공부를 할 수 있었습니다.</v>
       </c>
       <c r="F294" t="str">
-        <v>시험지를 보고 상담이 잘 이루어졌으며 모르거나 헷갈리는 문제만 골라내어 그 유형에 집즁할 수 있도록 플래너를 짜주시고 관련 문제들을 뽑아주셔서 성적향상에 도움되었습니다. 그에 대한 오답과 정답률도 체크해주는 시스템이 좋았습니다</v>
+        <v>시험지를 보고 상담이 잘 이루어졌으며 모르거나 헷갈리는 문제만 골라내어 그 유형에 집즁할 수 있도록 플래너를 짜주시고 관련 문제들을 뽑아주셔서 성적 향상에 도움되었습니다. 그에 대한 오답과 정답률도 체크해주는 시스템이 좋았습니다</v>
       </c>
       <c r="G294" t="str">
         <v>등원과 지각, 결석 등을 매일 확실하게 체크할 수 있기 때문에 일상 루틴이 잘 잡혔습니다. 매일 똑같은 시간대로 움직여 공부하기 때문에 공부하는 루틴이 몸에 잡혀서 매일 정해둔 시간표대로 모든 공부를 할 수 있었습니다</v>
@@ -11081,7 +11081,7 @@
         <v>주기적인 학원 생활상담 코칭은 단순히 공부 방법을 알려주는 것을 넘어, 생활 전반을 점검하고 균형을 맞출 수 있도록 도와주었습니다. 규칙적인 생활 습관을 형성하게 되어 체력과 집중력이 향상되었고, 불안한 마음을 안정시키는 데 큰 도움이 되었습니다. 상담 선생님과의 대화를 통해 학습 계획을 구체적으로 세 울 수 있었고, 작은 고민도 함께 나누며 해결책을 찾을 수 있어 학원 생활이 훨씬 수월해졌습니다.</v>
       </c>
       <c r="F295" t="str">
-        <v>학원의 학습관리 시스템은 단순히 공부 계획을 세우는 것을 넘어, 학생 개개인의 학습 패턴과 성향 을 분석해 맞춤형 관리가 이루어지는 점이 가장 큰 장점입니다. 매일 학습 진도를 점검하고 부족한 부분 을 빠르게 보완할 수 있도록 피드백을 제공해 주며, 체계적인 시간 관리와 목표 설정을 통해 자기주도 학습 능력을 키울 수 있었습니다. 또한 상담과 관리가 병행되어 학습 동기 부여가 지속적으로 이루어져, 장기적인 재수 생활에서도 안정감을 느낄 수 있었습니다.</v>
+        <v>학원의 학습 관리 시스템은 단순히 공부 계획을 세우는 것을 넘어, 학생 개개인의 학습 패턴과 성향 을 분석해 맞춤형 관리가 이루어지는 점이 가장 큰 장점입니다. 매일 학습 진도를 점검하고 부족한 부분 을 빠르게 보완할 수 있도록 피드백을 제공해 주며, 체계적인 시간 관리와 목표 설정을 통해 자기주도 학습 능력을 키울 수 있었습니다. 또한 상담과 관리가 병행되어 학습 동기 부여가 지속적으로 이루어져, 장기적인 재수 생활에서도 안정감을 느낄 수 있었습니다.</v>
       </c>
       <c r="G295" t="str">
         <v>학원의 생활 관리 시스템은 학습 외적인 부분까지 세심하게 챙겨주어 큰 도움이 됩니다. 규칙적인 생활 패턴을 유지할 수 있도록 기상 시간, 식사, 휴식, 운동까지 관리해 주며, 이를 통해 체력과 집중력이 안정적으로 유지됩니다. 또한 생활 태도와 습관을 점검해 불필요한 시간 낭비를 줄이고 자기 주도적인 생활을 할 수 있도록 지도해 줍니다. 상담을 통해 생활 전반에 대한 피드백을 받으면서 학습과 생활의 균형을 맞출 수 있었고, 장기적인 재수 생활에서도 흔들림 없이 목표를 향해 나아갈 수 있는 기반이 마 련되었습니다.</v>
@@ -11340,8 +11340,8 @@
         <v>이투스 구독을 통해 정승제 선생님, 이지영 선생님 등 유명 강사들의 다양한 인강을 추가 비용 없이 수강할 수 있어 큰 도움이 되었습니다 수준 높은 강의를 활용해 부족한 부분을 보완하고, 효율적으로 공부하며 성적을 꾸준히 향상시킬 수 있었습니다</v>
       </c>
       <c r="I302" t="str" xml:space="preserve">
-        <v xml:space="preserve">1년동안 저를 지도해주신 모든 선생님들께 정말 감사합니다 덕분에 지금 제가 대학생이 되어 캠퍼스 생활도 하고 즐겁게 지낼 수 있다고 생각합니다_x000d_
-특히 멘탈관리에 많은 도움을 주신 em반 담임선생님 정은숙 선생님, 항상 맛있는 밥을 만들어주셨던 동원홈푸드 영양사님께 감사합니다!</v>
+        <v xml:space="preserve">1년 동안 저를 지도해주신 모든 선생님들께 정말 감사합니다 덕분에 지금 제가 대학생이 되어 캠퍼스 생활도 하고 즐겁게 지낼 수 있다고 생각합니다_x000d_
+특히 멘탈관리에 많은 도움을 주신 em반 담임 선생님 정은숙 선생님, 항상 맛있는 밥을 만들어주셨던 동원홈푸드 영양사님께 감사합니다!</v>
       </c>
       <c r="J302" t="str">
         <v>하루 일정을 체계적으로 관리해 주셔서 자연스럽게 규칙적인 생활 습관을 만들 수 있어 좋았습니다.</v>
@@ -11376,7 +11376,7 @@
         <v>이투스 모의고사는 실제 시험 현장과 매우 유사한 분위기 속에서 시험을 경험해볼 수 있다는 자체가 도움이 되는 경험이라고 생각합니다. 전국 단위에서 제 위치를 알아보고 부족한 점을 파악할 수 있고, 이투스 강사님들의 해설강의도 제공되어서 효과적으로 오답 정리를 할 수 있었습니다.</v>
       </c>
       <c r="I303" t="str">
-        <v>담임선생님, 주간팀 및 야간팀 선생님들이 학원에 아무 불편함 없이 학업에 전념할 수 있는 환경을 만들어주셔서 좋은 결과가 있었던 것 같습니다! 힘들 때 기댈 수 있는 선생님 분들이 있다는 것 자체가 1년 내내 큰 힘이 되었습니다. 감사합니다!</v>
+        <v>담임 선생님, 주간팀 및 야간팀 선생님들이 학원에 아무 불편함 없이 학업에 전념할 수 있는 환경을 만들어주셔서 좋은 결과가 있었던 것 같습니다! 힘들 때 기댈 수 있는 선생님 분들이 있다는 것 자체가 1년 내내 큰 힘이 되었습니다. 감사합니다!</v>
       </c>
       <c r="J303" t="str">
         <v>어느 순간 성적이 오르지 않는다 생각이 들었을 때 담임 선생님과 상담을 하면서 해결 방안을 찾을 수 있었습니다.</v>
@@ -11446,7 +11446,7 @@
         <v>이투스 전국 모의고사는 실제 수능과 유사한 환경에서 시험을 치를 수 있어 실전 감각을 극대화하는 데 매우 유용했습니다. 평가원이나 교육청 모의고사 사이의 공백기에도 매달 긴장감을 유지하며 시험을 치를 수 있었고, 정해진 시간 내에 OMR 마킹까지 완료하는 연습을 반복하며 시간 배분 능력을 크게 키울 수 있었습니다. 특히 실제 수능 시간표에 맞춰 진행되는 경험 덕분에 시험장에서 느낄 수 있는 막연한 불안감을 줄이고, 자신만의 문제 풀이 루틴을 확립하는 데 결정적인 도움을 받았습니다.</v>
       </c>
       <c r="I305" t="str">
-        <v>올바른 공부 방향을 잡지 못해 방황하던 저를 믿고 이끌어주신 모든 선생님께 감사의 인사를 전합니다. 매일 아침 밝은 모습으로 맞아주시고, 엄격하면서도 애정 어린 생활 관리로 제가 올바른 학습 습관을 형성할 수 있도록 도와주셔서 감사합니다. 특히 상담 때마다 주셨던 실질적인 입시 데이터와 전략적인 조언들은 제 목표를 더 명확하게 만들어 주었습니다. 선생님들의 헌신적인 관리 덕분에 성적뿐만 아니라 마음가짐까지 한층 성장할 수 있었습니다. 원장선생님, 담임 선생님, 데스크 실장님, 영어 선생님 다 너무 감사했습니다 ❤️</v>
+        <v>올바른 공부 방향을 잡지 못해 방황하던 저를 믿고 이끌어주신 모든 선생님께 감사의 인사를 전합니다. 매일 아침 밝은 모습으로 맞아주시고, 엄격하면서도 애정 어린 생활 관리로 제가 올바른 학습 습관을 형성할 수 있도록 도와주셔서 감사합니다. 특히 상담 때마다 주셨던 실질적인 입시 데이터와 전략적인 조언들은 제 목표를 더 명확하게 만들어 주었습니다. 선생님들의 헌신적인 관리 덕분에 성적뿐만 아니라 마음가짐까지 한층 성장할 수 있었습니다. 원장 선생님, 담임 선생님, 데스크 실장님, 영어 선생님 다 너무 감사했습니다 ❤️</v>
       </c>
       <c r="J305" t="str">
         <v>반복적으로 틀리는 유형에 대하여 제 수준에 맞는 설명으로 깔끔한 해법을 제시해 주신 점이 성적 향상에 도움이 됐어요!</v>
@@ -11504,10 +11504,10 @@
         <v>N수생</v>
       </c>
       <c r="E307" t="str">
-        <v>아무래도 기숙 특성상 자습 시간이 많은 편이었는데 현역 때 공부를 거의 안 해봤던지라 그 많은 자습 시간을 어떻게 활용해야할지에 대한 고민이 많았는데, 학습 상담을 통해 갈피를 잡고 공부를 할 수 있었습니다. 플래너 쓰는 것도 어려워하던 저에게 공부 계획을 어떻게 체계적이고 효율적이게 세울 수 있는지를 알려주셨습니다. 또한, 시기마다 어떤 컨텐츠를 풀면 효율적일지 추천해주셨습니다. 꾸준히 공부를 열심히 함으로써 성적이 지난 수능에 비해 많이 오를 수 있도록 도와주셨습니다.</v>
+        <v>아무래도 기숙 특성상 자습 시간이 많은 편이었는데 현역 때 공부를 거의 안 해봤던지라 그 많은 자습 시간을 어떻게 활용해야 할지에 대한 고민이 많았는데, 학습 상담을 통해 갈피를 잡고 공부를 할 수 있었습니다. 플래너 쓰는 것도 어려워하던 저에게 공부 계획을 어떻게 체계적이고 효율적이게 세울 수 있는지를 알려주셨습니다. 또한, 시기마다 어떤 컨텐츠를 풀면 효율적일지 추천해주셨습니다. 꾸준히 공부를 열심히 함으로써 성적이 지난 수능에 비해 많이 오를 수 있도록 도와주셨습니다.</v>
       </c>
       <c r="F307" t="str">
-        <v>플래너를 처음에 짤 때는 아무래도 미숙하다보니 날마다 공부하는 과목들의 비율이 이상했는데 이와 관련해서 큰 도움을 받았던 것 같습니다. 한 과목에만 치중하거나 싫어하는 한 과목만 버리지 않도록 잘 지도해주셨습니다. 또한 공부시간이 터무니 없게 적은 날들은 따끔하게 혼도 나며 정신을 차릴 수 있도록 도와주셨습니다.</v>
+        <v>플래너를 처음에 짤 때는 아무래도 미숙하다보니 날마다 공부하는 과목들의 비율이 이상했는데 이와 관련해서 큰 도움을 받았던 것 같습니다. 한 과목에만 치중하거나 싫어하는 한 과목만 버리지 않도록 잘 지도해주셨습니다. 또한 공부 시간이 터무니 없게 적은 날들은 따끔하게 혼도 나며 정신을 차릴 수 있도록 도와주셨습니다.</v>
       </c>
       <c r="G307" t="str">
         <v>현역 때 수능을 망한 원인이 핸드폰과 아이패드, 인터넷이었다고 해도 과언이 아닐 정도로 원래의 저는 인터넷 중독이었습니다. 이천 이투스247 기숙학원에 들어간 후 강제로 핸드폰을 뺏기고 와이파이 방화벽 덕에 강제로 하루종일 인터넷을 못하는 상황이 만들어지니 공부에만 집중할 수 있었습니다. 제 이번 수능 성공요인들 중 정말 큰 요인은 인터넷을 하지 않은 것이었습니다. 1월 초에 조기선발반으로 입소한 후 단 1초도 방화벽을 뚫지 않음으로써 수능날 작년 수능에 비해 과탐과탐러임에도 불구하고 무려 평균 백분위가 25이상 상승하는 쾌거를 이룰 수 있었습니다.</v>
@@ -11617,7 +11617,7 @@
         <v>반수생</v>
       </c>
       <c r="E310" t="str">
-        <v>다양한 대학교와 목표하는 대학교의 입결과 대학별로 더 중요치를 두는 과목 등에 대해서 자세하게 설명해주셔서 어느부분의 공부에 더욱 집중하여 학습해야할 지 알 수 있어서 많은 도움이 되았습니다!</v>
+        <v>다양한 대학교와 목표하는 대학교의 입결과 대학별로 더 중요치를 두는 과목 등에 대해서 자세하게 설명해주셔서 어느부분의 공부에 더욱 집중하여 학습해야 할 지 알 수 있어서 많은 도움이 되았습니다!</v>
       </c>
       <c r="F310" t="str">
         <v>매주 보는 개인 모의고사라던지, 평가원 모의고사, 달마다 학원에서 전체시행하는 더프모의고사같은 모의고사를 보고 나서 혼자서 사고하기 어려웠던 부분들에 대해 여쭈어보면 친절하게 알려주시고 그렇게 배운 부분이 하나의 자양분이 되어서 좋은 성적의 발판이 되었다고 생각합니다!</v>
@@ -11699,7 +11699,7 @@
         <v>수능을 앞두고 모의고사 문제를 푸는 것이 실전감각을 키우는데 매우 중요하다고 생각하는데 이투스 모의고사는 실제 모의고사와 비슷한 형태이며 학원에서 다같이 보기 때문에 수능을 준비하는데 도움이 되었습니다.</v>
       </c>
       <c r="I312" t="str">
-        <v>1년동안 학생들의 학습코칭뿐만 아니라 멘탈관리와 지친 학생들을 위한 간식 이벤트 등 많은 도움을 주셔서 매우 감사합니다! 덕분에 1년을 포기하지 않고  끝까지 잘 버틸 수 있었습니다.</v>
+        <v>1년 동안 학생들의 학습코칭뿐만 아니라 멘탈관리와 지친 학생들을 위한 간식 이벤트 등 많은 도움을 주셔서 매우 감사합니다! 덕분에 1년을 포기하지 않고  끝까지 잘 버틸 수 있었습니다.</v>
       </c>
       <c r="J312" t="str">
         <v>학습 코칭뿐만 아니라 지친 학생들을 위해 다양한 이벤트도 진행해 주시고, 심리 상담도 해주셔서 끝까지 해낼 수 있었어요.</v>
@@ -11722,19 +11722,19 @@
         <v>N수생</v>
       </c>
       <c r="E313" t="str">
-        <v>재수를 하다보면 쓸쓸하고 외롭게 되어서 공부하다 보면 환기도 할겸 대화 할 상대가 필요합니다. 그럴때 일주일에 한번씩 담당 선생님과 일주일동안 무슨 공부를 했는지 체크하고 또 다음 한주동안에 목표를 잡고 힘들었던 점들을 하소연 하면서 한주 한주를 버틸수 있던거 같습니다.</v>
+        <v>재수를 하다보면 쓸쓸하고 외롭게 되어서 공부하다 보면 환기도 할겸 대화 할 상대가 필요합니다. 그럴때 일주일에 한 번씩 담당 선생님과 일주일동안 무슨 공부를 했는지 체크하고 또 다음 한주동안에 목표를 잡고 힘들었던 점들을 하소연 하면서 한주 한주를 버틸수 있던거 같습니다.</v>
       </c>
       <c r="F313" t="str">
-        <v>원래 현역 고3때 공부할때는 계획 짜는것이 의미 없다고 생각되어서 플래너를 따로 작성하지 않았습니다. 하지만 재수를 하면서 이투스학원에서 플래너를 무상으로 지급을 해주는데 매일 공부를 다하고 집에 가기전에 다음날 무엇을 할지 플래너를 작성해놓으면 다음날 학원에 왔을때 목표치가 설정되어 있어서 좀 더 공부하는데 수월했던것 같습니다.</v>
+        <v>원래 현역 고3 때 공부할때는 계획 짜는것이 의미 없다고 생각되어서 플래너를 따로 작성하지 않았습니다. 하지만 재수를 하면서 이투스학원에서 플래너를 무상으로 지급을 해주는데 매일 공부를 다하고 집에 가기전에 다음날 무엇을 할지 플래너를 작성해놓으면 다음날 학원에 왔을때 목표치가 설정되어 있어서 좀 더 공부하는데 수월했던것 같습니다.</v>
       </c>
       <c r="G313" t="str">
         <v>핸드폰이 자기 수중에 있게 되면 공부하다가 연락이 오거나 알람이 떴을 때  어쩔수 없이 보다가 시간을 허비하고 집중력이 깨지는 경우가 많습니다. 이투스에서는 핸드폰을 아침시간 출석과 동시에 걷기때문에 핸드폰의 유혹에서 벗어나 좀 더 유용한 환경에서 공부 할수가 있었습니다.</v>
       </c>
       <c r="H313" t="str">
-        <v>재수를 하면서 수 많은 기출들과 모의고사들을 풀게 되는데 막판으로 갈수록 양질의 모의고사들을 얻기가 어려워집니다. 1달~2달에 한번씩 치뤄지는 이투스 모의고사로 자기의 요즘 컨디션과 얼마나 성장했는지 체크도 하고 또 피드백까지 할수 있었던게 굉장한 도움이 되었던거 같습니다. 또 퀄리티 또한 입증이 되있기에 이투스에서 현장감을 느끼며 풀면서 실전성도 높일수가 있습니다.</v>
+        <v>재수를 하면서 수 많은 기출들과 모의고사들을 풀게 되는데 막판으로 갈수록 양질의 모의고사들을 얻기가 어려워집니다. 1달~2달에 한 번씩 치뤄지는 이투스 모의고사로 자기의 요즘 컨디션과 얼마나 성장했는지 체크도 하고 또 피드백까지 할수 있었던게 굉장한 도움이 되었던거 같습니다. 또 퀄리티 또한 입증이 되있기에 이투스에서 현장감을 느끼며 풀면서 실전성도 높일수가 있습니다.</v>
       </c>
       <c r="I313" t="str">
-        <v>1년동안 질문에 친절히 답해주시고 힘들때 격려로 끝까지 열심히 공부할수 있게 도와주셔서 너무 감사합니다. 선생님들의 격려와 덕담이 없었더라면 끝까지 완주하지 못 했을거라고 생각합니다. 특히 제 담임이셨던 국어선생님 정말로 감사합니다.</v>
+        <v>1년 동안 질문에 친절히 답해주시고 힘들 때 격려로 끝까지 열심히 공부할 수 있게 도와주셔서 너무 감사합니다. 선생님들의 격려와 덕담이 없었더라면 끝까지 완주하지 못 했을거라고 생각합니다. 특히 제 담임이셨던 국어선생님 정말로 감사합니다.</v>
       </c>
       <c r="J313" t="str">
         <v>재수 생활 동안 학습 계획과 생활 관리를 꾸준히 받아 끝까지 흔들리지 않고 공부할 수 있었어요.</v>
@@ -11757,19 +11757,19 @@
         <v>N수생</v>
       </c>
       <c r="E314" t="str">
-        <v>담당 과목 선생님들께서 상주하시면서 매주 학습 상담과 질의응답을 받아주셔서 정말 좋았습니다. 모르는 점이 있으면 바로 질의응답이 가능하다는 점이 수험생활에서 심리적으로 매우 중요하다는 점을 느낄 수 있었습니다</v>
+        <v>담당 과목 선생님들께서 상주하시면서 매주 학습 상담과 질의응답을 받아주셔서 정말 좋았습니다. 모르는 점이 있으면 바로 질의응답이 가능하다는 점이 수험 생활에서 심리적으로 매우 중요하다는 점을 느낄 수 있었습니다</v>
       </c>
       <c r="F314" t="str">
-        <v>질의응답을 바로바로 할 수 있다는 점이 좋았습니다. 어찌보면 당연한 것이겠지만 수험생활에서 질의응답이 대면으로 가능하다는 것은 매우 큰 힘이 됐습니다 그렇기에 질의응답이 가장 좋았던거 같습니다</v>
+        <v>질의응답을 바로바로 할 수 있다는 점이 좋았습니다. 어찌보면 당연한 것이겠지만 수험 생활에서 질의응답이 대면으로 가능하다는 것은 매우 큰 힘이 됐습니다 그렇기에 질의응답이 가장 좋았던거 같습니다</v>
       </c>
       <c r="G314" t="str">
-        <v>선생님들 모두 매시간마다 돌아다니시면서  다들 공부하는 분위기를 만들어주셔서 좋았던거 같습니다 모두가 지치고 힘든 수험생활을 보다 독려 될 수 있게 만들어주셨던거 같아서 감사했습니다</v>
+        <v>선생님들 모두 매시간마다 돌아다니시면서  다들 공부하는 분위기를 만들어주셔서 좋았던거 같습니다 모두가 지치고 힘든 수험 생활을 보다 독려 될 수 있게 만들어주셨던거 같아서 감사했습니다</v>
       </c>
       <c r="H314" t="str">
         <v>주기적인 모의고사로 내 위치를 확인할 수 있었던 점이 가장 좋아ㅛ습니다 수능 당일에 어떻게 하는것이 좋을지 어떤 루틴을 따를지 미리 생각할 수 있었던거 같아 좋았습니다 그래서 이투스 모의고사가 가장 좋았던거 같습니다</v>
       </c>
       <c r="I314" t="str">
-        <v>잘 이끌어주셔서 감사합니다 덕분에 좋은 결과가 있었던구 같습니다 힘든 수험생활에도 불구하고 견딜 수 있었던 이유는 선생님들께서 열심히 독려해주시고 이끌어주셔서 그랬던거 같습니다 감사합니다</v>
+        <v>잘 이끌어주셔서 감사합니다 덕분에 좋은 결과가 있었던구 같습니다 힘든 수험 생활에도 불구하고 견딜 수 있었던 이유는 선생님들께서 열심히 독려해주시고 이끌어주셔서 그랬던거 같습니다 감사합니다</v>
       </c>
       <c r="J314" t="str">
         <v>담당 과목 선생님들께서 상주하시면서 매주 학습 상담과 질의응답을 받아주셔서 정말 좋았어요.</v>
@@ -11874,7 +11874,7 @@
         <v>영어 단어 일일테스트만 해도 외워야 하는 단어의 양이 충족되는 느낌이었다. 실제로 영어공부를 하나도 하지 않았는데도 단어 외운 것으로  커버가 되어서 노력 대비 성과가 좋게 나타났다. 그리고 꾸준히 해야한다는 강제성이 부여된게 좋았다.</v>
       </c>
       <c r="I317" t="str">
-        <v>선생님 덕분에 이름 들어본 대학에 오게 되었어요. 1년동안 제 불안들 받아주시고 따듯하게 답변해주신거 정말 감사해요. 덕분에 많은 도움 되었고 많이 성장했습니다. 저도 선생님을 본받아서 남에게 친절을 베풀 수 있는 멋진 어른으로 성장하겠습니다.</v>
+        <v>선생님 덕분에 이름 들어본 대학에 오게 되었어요. 1년 동안 제 불안들 받아주시고 따듯하게 답변해주신거 정말 감사해요. 덕분에 많은 도움 되었고 많이 성장했습니다. 저도 선생님을 본받아서 남에게 친절을 베풀 수 있는 멋진 어른으로 성장하겠습니다.</v>
       </c>
       <c r="J317" t="str">
         <v>혼자서 찾기 어려운 입시 정보를 학원에서 제공해 주셔서 원서 준비에 많은 도움이 됐어요.</v>
@@ -11932,10 +11932,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E319" t="str">
-        <v>입시 생활을 하면서 자꾸만 더 해야 할 것 같다는 생각이 들고 불안했던 적이 많았었는데 이 부분에 대해서 같이 이야기할 수 있다는 점이 많이 의지가 되었습니다. 또 입시 당시 대학생이신 멘토 분과 질의응답을 진행하고 이투스 모의고사를 풀어보고 무한 오답을 진행했던 것이 개념을 까먹지 않고 문제 풀이 시간을 줄이는 데 도움이 많이 되었다고 생각합니다. 또 추가로 특정 과목이 힘들었을 때 담임선생님께서 특정 과목 담당 선생님께 학습 관련 상담을 요청해 주셔서 막막함을 해결할 수 있었던 점도 좋았습니다.</v>
+        <v>입시 생활을 하면서 자꾸만 더 해야 할 것 같다는 생각이 들고 불안했던 적이 많았었는데 이 부분에 대해서 같이 이야기할 수 있다는 점이 많이 의지가 되었습니다. 또 입시 당시 대학생이신 멘토 분과 질의응답을 진행하고 이투스 모의고사를 풀어보고 무한 오답을 진행했던 것이 개념을 까먹지 않고 문제 풀이 시간을 줄이는 데 도움이 많이 되었다고 생각합니다. 또 추가로 특정 과목이 힘들었을 때 담임 선생님께서 특정 과목 담당 선생님께 학습 관련 상담을 요청해 주셔서 막막함을 해결할 수 있었던 점도 좋았습니다.</v>
       </c>
       <c r="F319" t="str">
-        <v>입시 생활을 하면서 자꾸만 더 해야 할 것 같다는 생각이 들고 불안했던 적이 많았었는데 이 부분에 대해서 일대일로 담임선생님과 같이 이야기할 수 있다는 점이 많이 의지가 되었습니다. 또 입시 당시 대학생이신 멘토 분과 일대일로 질의응답을 진행하고 이투스 모의고사를 풀어본 후 무한 오답을 진행했던 것이 개념을 까먹지 않고 문제 풀이 시간을 줄이는 데 도움이 많이 되었다고 생각합니다. 또 추가로 특정 과목이 힘들었을 때 담임선생님께서 특정 과목 담당 선생님께 일대일로 학습 관련 상담을 요청해 주셔서 막막함을 해결할 수 있었던 점도 좋았습니다.</v>
+        <v>입시 생활을 하면서 자꾸만 더 해야 할 것 같다는 생각이 들고 불안했던 적이 많았었는데 이 부분에 대해서 일대일로 담임 선생님과 같이 이야기할 수 있다는 점이 많이 의지가 되었습니다. 또 입시 당시 대학생이신 멘토 분과 일대일로 질의응답을 진행하고 이투스 모의고사를 풀어본 후 무한 오답을 진행했던 것이 개념을 까먹지 않고 문제 풀이 시간을 줄이는 데 도움이 많이 되었다고 생각합니다. 또 추가로 특정 과목이 힘들었을 때 담임 선생님께서 특정 과목 담당 선생님께 일대일로 학습 관련 상담을 요청해 주셔서 막막함을 해결할 수 있었던 점도 좋았습니다.</v>
       </c>
       <c r="G319" t="str">
         <v>와이파이 방화벽으로 다른 데에 한눈을 팔지 않고 공부에만 온전히 집중할 수 있는 습관을 만드는 데 도움이 되었습니다. 혼자서 공부를 하면 다른 곳에 현혹되기 쉬운데 학원에서는 와이파이 방화벽으로 면학 분위기도 좋고 집중도도 높아졌다고 생각합니다.</v>
@@ -11946,7 +11946,7 @@
 또한 정승제, 이지영과 같은 업계 최정상급 강사진의 모든 강의를 제한 없이 들을 수 있어 취약한 과목을 집중적으로 보완하기에 최적의 환경을 제공했습니다. 특히 강의를 시청한 시간만큼 현금성 포인트를 돌려받는 페이백 시스템은 자칫 나태해질 수 있는 수험 생활에 강력한 학습 동기를 부여해 주었습니다. 단순히 강의를 파는 것을 넘어 학생이 공부한 만큼 보상을 주는 구조 덕분에 꾸준히 책상 앞에 앉아 있을 수 있었으며, 결과적으로 고퀄리티의 콘텐츠를 가장 효율적이고 경제적인 방법으로 누릴 수 있었던 최고의 선택이었습니다.</v>
       </c>
       <c r="I319" t="str">
-        <v>담임선생님, 원장 선생님, 사감 선생님, 멘토 선생님, 급식 담당 선생님 등의 모든 목동 이투스 247 선생님들께 그동안 격려해 주시고 제 고민과 모르는 부분 등에 대해서 친절히 상담해 주셔서 감사했습니다. 맛있는 급식 제공해 주셔서 감사했습니다.</v>
+        <v>담임 선생님, 원장 선생님, 사감 선생님, 멘토 선생님, 급식 담당 선생님 등의 모든 목동 이투스 247 선생님들께 그동안 격려해 주시고 제 고민과 모르는 부분 등에 대해서 친절히 상담해 주셔서 감사했습니다. 맛있는 급식 제공해 주셔서 감사했습니다.</v>
       </c>
       <c r="J319" t="str">
         <v>과목 담당 선생님이 따로 있어 특정 과목에 대한 학습 상담을 할 수 있어 좋았어요!</v>
@@ -12004,22 +12004,22 @@
         <v>N수생</v>
       </c>
       <c r="E321" t="str">
-        <v>담임선생님들이 계셔서 학습 외적인 부분에서도 도움을 받을 수 있다는 점이 좋았습니다. 기숙학원에서 재수를 하다보니 아무래도 정신적으로 힘들고 흔들릴 때가 많았는데 그럴 때마다 담임선생님과의 대화를 통해 버티고 이겨낼 수 있었던 것 같습니다. 담임선생님들이 진심으로 대해주셔서 좋았습니다.</v>
+        <v>담임 선생님들이 계셔서 학습 외적인 부분에서도 도움을 받을 수 있다는 점이 좋았습니다. 기숙학원에서 재수를 하다보니 아무래도 정신적으로 힘들고 흔들릴 때가 많았는데 그럴 때마다 담임 선생님과의 대화를 통해 버티고 이겨낼 수 있었던 것 같습니다. 담임 선생님들이 진심으로 대해주셔서 좋았습니다.</v>
       </c>
       <c r="F321" t="str">
-        <v>혼자서는 알아볼 수 없는 것들을 알 수 있어 좋았습니다. 또한, 성적분석만 나오는 것이 아니라 점수 변동 추이, 가능한 대학과 학과까지 자세하기 볼 수 있어 수험생활 중 궁금증이 많이 해소되었습니다.</v>
+        <v>혼자서는 알아볼 수 없는 것들을 알 수 있어 좋았습니다. 또한, 성적분석만 나오는 것이 아니라 점수 변동 추이, 가능한 대학과 학과까지 자세하기 볼 수 있어 수험 생활 중 궁금증이 많이 해소되었습니다.</v>
       </c>
       <c r="G321" t="str">
-        <v>아무래도 수험생활을 하다보면 전자기기의 유혹에 빠지기 쉬운데, 사용하는 와이파이 자체에서 그런 사이트들을 다 차단하다보니 자연스럽게 SNS 등 수험생활에 도움이 되지 않는 사이트를 사용하지 않을 수 있었습니다. 자기 자신을 잘 제어하지 못해서 간 기숙학원이라 이런 시스템이 매우 도움되었습니다.</v>
+        <v>아무래도 수험 생활을 하다보면 전자기기의 유혹에 빠지기 쉬운데, 사용하는 와이파이 자체에서 그런 사이트들을 다 차단하다보니 자연스럽게 SNS 등 수험 생활에 도움이 되지 않는 사이트를 사용하지 않을 수 있었습니다. 자기 자신을 잘 제어하지 못해서 간 기숙학원이라 이런 시스템이 매우 도움되었습니다.</v>
       </c>
       <c r="H321" t="str">
         <v>독학기숙이다보니 인터넷강의만을 활용하여 공부하는데 이투스 구독권을 받아 무료로 이투스 강의를 들을 수 있다는 점이 좋았습니다. 더욱 더 선택지가 많아지고,  비용적으로 부담이 되는 인터넷강의를 무료로 들을 수 있어 평소에 궁금했던 선생님의 강의를 들어볼 수 있는게 좋았습니다.</v>
       </c>
       <c r="I321" t="str">
-        <v>대학 진학 결과가 제 생각만큼 좋지 않아서 이런 글을 써도 될까 고민했습니다. 그러나 작년 한해동안 학원에서 지내면서 정말 많이 배웠고 성장했습니다. 특히 제가 많이 울었는데 옆에서 같이 걱정해주시고 위로해주셨던 담임선생님, 그리고 다른 반 담임선생님이지만 상담시간 쪼개서 제 학습 상담까지 봐주셨던 선생님 정말 감사했습니다.</v>
+        <v>대학 진학 결과가 제 생각만큼 좋지 않아서 이런 글을 써도 될까 고민했습니다. 그러나 작년 한해동안 학원에서 지내면서 정말 많이 배웠고 성장했습니다. 특히 제가 많이 울었는데 옆에서 같이 걱정해주시고 위로해주셨던 담임 선생님, 그리고 다른 반 담임 선생님이지만 상담시간 쪼개서 제 학습 상담까지 봐주셨던 선생님 정말 감사했습니다.</v>
       </c>
       <c r="J321" t="str">
-        <v>담임선생님들이 계셔서 학습 외적인 부분에서도 도움을 받을 수 있다는 점이 좋았어요.</v>
+        <v>담임 선생님들이 계셔서 학습 외적인 부분에서도 도움을 받을 수 있다는 점이 좋았어요.</v>
       </c>
       <c r="K321" t="str">
         <v/>
@@ -12077,10 +12077,10 @@
         <v>먼저 한약학과라는 학과를 소개해주시고 망설이는 저에게 확신을 갖게 해주는 선생님께 너무너무 감사드립니다. 또한 제 생기부와 수시 등급을 가지고 현실적으로 갈수 있는 곳을 알려주셔서 그때 당시에는 가슴아팠지만.. 장기적으로는 너무 다행이였습니다</v>
       </c>
       <c r="F323" t="str">
-        <v>여러 다양한 인강 선생님들을 알수 있었고 2주에 한번씩 상담을 하면서 최대한 인강을 안미루게 듣게되고 mbti가 p 90퍼인 저도 계획을 가지고 인강을 들을수 있게 되었습니다..ㅎㅎ</v>
+        <v>여러 다양한 인강 선생님들을 알수 있었고 2주에 한 번씩 상담을 하면서 최대한 인강을 안미루게 듣게되고 mbti가 p 90퍼인 저도 계획을 가지고 인강을 들을수 있게 되었습니다..ㅎㅎ</v>
       </c>
       <c r="G323" t="str">
-        <v>지금도 대학공부를 하며 핸드폰을 하고 있는 저로썬 만약 핸드폰 수거를 안했다면은 한 공부시간의 30퍼는 핸드폰을 하고 있지 않았을까라고 조심스럽게 추측해봅니다..따라서 핸드폰 수거는 정말정말 좋은 시스템인것같아요</v>
+        <v>지금도 대학공부를 하며 핸드폰을 하고 있는 저로썬 만약 핸드폰 수거를 안했다면은 한 공부 시간의 30퍼는 핸드폰을 하고 있지 않았을까라고 조심스럽게 추측해봅니다..따라서 핸드폰 수거는 정말정말 좋은 시스템인것같아요</v>
       </c>
       <c r="H323" t="str">
         <v>이투스 전국 모의고사.. 일단 너무 어렵지 않아서 좋았고 성적이 담임 선생님께 공개가 되니깐 더 책임감?을 가지고 임할수 있어서 좋았어요. 또 모고날을 기준으로 계획세우기도 좋았습니다</v>
@@ -12182,13 +12182,13 @@
         <v>N수생</v>
       </c>
       <c r="E326" t="str">
-        <v>학습 방향성을 잡아줌. 한 주에 한번씩 진행하여 그 기간 동안 내가 올바르게 공부하였는지, 못했다면 무엇이 문제였는지를 같이 연구하고 개선 및 실제 적용 방안을 찾는 시간이었음. 무엇보다 그 과정에서 정신적 케어도 같이 진행되어 상당히 긍정적이었음.</v>
+        <v>학습 방향성을 잡아줌. 한 주에 한 번씩 진행하여 그 기간 동안 내가 올바르게 공부하였는지, 못했다면 무엇이 문제였는지를 같이 연구하고 개선 및 실제 적용 방안을 찾는 시간이었음. 무엇보다 그 과정에서 정신적 케어도 같이 진행되어 상당히 긍정적이었음.</v>
       </c>
       <c r="F326" t="str">
         <v>여름, 느슨해진 나에게 긴장감을 선사해주심. 역시 밍기적거리는 사람에겐 불러다가 닦아주는 것이 만능 특효약. 무엇보다 내 수준이 어디인지, 얼마나 더 올려야 원하는 곳에 갈 수 있는지 등을 알려주고 머리 깨뜨려서 정신차리게 해주는 시간이었음.</v>
       </c>
       <c r="G326" t="str">
-        <v>나는 내 자신을 믿지 못하기 때문에, 핸드폰이 있었다면 공부시간 12시간 중 1시간도 못했을 것임. 강제로 핸드폰을 내 몸과 분리시켜줌으로써, 또한 그래도 점심 저녁시간에는 돌려줬기에, 공부 열심히 하면 보상으로 폰 받는 느낌이어서 상당히 좋았음.</v>
+        <v>나는 내 자신을 믿지 못하기 때문에, 핸드폰이 있었다면 공부 시간 12시간 중 1시간도 못했을 것임. 강제로 핸드폰을 내 몸과 분리시켜줌으로써, 또한 그래도 점심 저녁시간에는 돌려줬기에, 공부 열심히 하면 보상으로 폰 받는 느낌이어서 상당히 좋았음.</v>
       </c>
       <c r="H326" t="str">
         <v>학평이나 모평보고 우쭐해진 나에게 정의의 철퇴를 내려주신 단비같은 모의고사. 모의고사 한 두개 잘보고 우쭐해진 나를, 읍참마속의 심정으로 친히 내 오만함을 깨뜨려 부숴주심으로써, 현실에 안주하지 않고 끝까지 달려나갈 수 있는 원동력이 되었음.</v>
@@ -12219,13 +12219,13 @@
         <v>반수생</v>
       </c>
       <c r="E327" t="str">
-        <v>이투스247의 생활상담 코칭 시스템은 그냥 공부만 시키는 방식이 아니라, 학생 생활 전체를 같이 본다는 점에서 확실히 도움됐다. 수험생활은 계획만 세운다고 굴러가는 게 아니라 수면, 식사, 멘탈, 루틴이 다 연결돼 있어서 한 부분만 무너지면 하루가 쉽게 흔들리는데, 이걸 혼자 계속 잡기는 생각보다 어렵다. 그럴 때 현재 상태를 같이 점검해주고 흐트러진 부분을 바로바로 정리해주는 게 꽤 컸다. 막연하게 불안해하기보다 왜 공부가 안 되는지 원인을 빨리 찾게 되고, 생활 패턴도 조금씩 안정되면서 결국 공부 효율까지 같이 올라가는 느낌이었다. 혼자 버티는 수험생활보다 훨씬 덜 막막하게 만들어주는 시스템이라고 생각한다.</v>
+        <v>이투스247의 생활상담 코칭 시스템은 그냥 공부만 시키는 방식이 아니라, 학생 생활 전체를 같이 본다는 점에서 확실히 도움됐다. 수험 생활은 계획만 세운다고 굴러가는 게 아니라 수면, 식사, 멘탈, 루틴이 다 연결돼 있어서 한 부분만 무너지면 하루가 쉽게 흔들리는데, 이걸 혼자 계속 잡기는 생각보다 어렵다. 그럴 때 현재 상태를 같이 점검해주고 흐트러진 부분을 바로바로 정리해주는 게 꽤 컸다. 막연하게 불안해하기보다 왜 공부가 안 되는지 원인을 빨리 찾게 되고, 생활 패턴도 조금씩 안정되면서 결국 공부 효율까지 같이 올라가는 느낌이었다. 혼자 버티는 수험 생활보다 훨씬 덜 막막하게 만들어주는 시스템이라고 생각한다.</v>
       </c>
       <c r="F327" t="str">
         <v>이투스247에서 학습 계획이랑 플래너 관리가 유용했던 건, 그냥 “공부해라”가 아니라 뭘 얼마나 어떻게 해야 하는지를 계속 보이게 만들어준다는 점이었다. 혼자 계획 짜면 욕심만 앞서서 비현실적으로 세우거나, 밀리면 아예 손 놓게 되는 경우가 많은데 여기서는 현재 수준이랑 해야 할 양을 기준으로 좀 더 현실적으로 흐름을 잡아주는 느낌이 있었다. 플래너도 단순 기록용이 아니라 내가 하루를 제대로 쓰고 있는지 확인하게 해줘서 좋았다. 계획 세우고 끝이 아니라 실제로 했는지, 어디서 막혔는지까지 보이니까 흐트러져도 다시 복구하기가 훨씬 쉬웠고, 공부를 막연하게 하는 시간이 줄어드는 게 꽤 크게 느껴졌다.</v>
       </c>
       <c r="G327" t="str">
-        <v>이투스247의 면학 분위기 감독은 단순히 조용한 독서실 분위기를 만든다는 의미보다, 학생이 공부 외의 데에 에너지를 빼앗기지 않게 해준다는 점에서 유용했다. 수험생활을 하다 보면 은근히 주변 소음, 자리 분위기, 흐트러진 생활 태도 같은 사소한 요소들이 집중력에 크게 영향을 주는데, 이런 부분이 꾸준히 관리되니까 공부 흐름이 덜 끊겼다. 혼자였다면 한 번쯤은 느슨해졌을 순간에도 자연스럽게 다시 책상에 앉게 되는 분위기가 있었고, 결국 의지에만 기대지 않고 공부할 수 있는 환경이 유지된다는 점이 꽤 크게 느껴졌다.</v>
+        <v>이투스247의 면학 분위기 감독은 단순히 조용한 독서실 분위기를 만든다는 의미보다, 학생이 공부 외의 데에 에너지를 빼앗기지 않게 해준다는 점에서 유용했다. 수험 생활을 하다 보면 은근히 주변 소음, 자리 분위기, 흐트러진 생활 태도 같은 사소한 요소들이 집중력에 크게 영향을 주는데, 이런 부분이 꾸준히 관리되니까 공부 흐름이 덜 끊겼다. 혼자였다면 한 번쯤은 느슨해졌을 순간에도 자연스럽게 다시 책상에 앉게 되는 분위기가 있었고, 결국 의지에만 기대지 않고 공부할 수 있는 환경이 유지된다는 점이 꽤 크게 느껴졌다.</v>
       </c>
       <c r="H327" t="str">
         <v>이투스 전국 모의고사는 현재 내 위치를 객관적으로 확인할 수 있다는 점에서 도움이 됐다. 평소엔 내가 어느 정도 하고 있는지 감이 애매할 때가 많은데, 실제 시험처럼 점검해보면 약한 부분이 훨씬 선명하게 보인다. 특히 실전 시간 관리나 멘탈 흐름까지 같이 체크할 수 있어서 그냥 문제 푸는 거랑은 확실히 다르게 느껴졌다. 막연하게 불안해하기보다, 뭘 보완해야 하는지 방향을 잡는 데 유용했다.</v>
@@ -12266,7 +12266,7 @@
         <v>저는 이투스 모의고사를 치고 난 다음 강윤구 수학 선생님을 알게 되었는데, 평소라면 보지도 않았을 선생님을 우연한 계기로 만나게 해준 모의고사라서 저에게 정말 뜻이 깊었던 것 같습니다</v>
       </c>
       <c r="I328" t="str">
-        <v>1년동안 수고하셨고, 앞으로 들어오는 신입생들도 잘 챙겨주셨으면 좋겠습니다! 덕분에 서울에 상경해서 즐거운 대학 생활을 즐기고 있는데, 부산에 가게 될 일이 있으면 찾아뵙겠습니다!!</v>
+        <v>1년 동안 수고하셨고, 앞으로 들어오는 신입생들도 잘 챙겨주셨으면 좋겠습니다! 덕분에 서울에 상경해서 즐거운 대학 생활을 즐기고 있는데, 부산에 가게 될 일이 있으면 찾아뵙겠습니다!!</v>
       </c>
       <c r="J328" t="str">
         <v>불안정형 수험생이던 저를 차분하게 진정시켜 주시고, 필요한 것도 바로 챙겨주셔서 감사했습니다.</v>
@@ -12289,7 +12289,7 @@
         <v>N수생</v>
       </c>
       <c r="E329" t="str">
-        <v>과목별 선생님이 따로 계셔서 각 과목에 대해 보다 전문적이고 깊이 있는 지도를 받을 수 있었던 점이 매우 유용했습니다. 또한 담임선생님과 주간선생님이 함께 학생을 관리해 주셔서 학습 상황뿐만 아니라 전반적인 생활까지 균형 있게 점검받을 수 있었습니다. 필요할 때마다 편하게 상담을 요청드릴 수 있어 학습에 대한 고민이나 어려움을 신속하게 해결할 수 있었던 점도 큰 장점이었습니다.</v>
+        <v>과목별 선생님이 따로 계셔서 각 과목에 대해 보다 전문적이고 깊이 있는 지도를 받을 수 있었던 점이 매우 유용했습니다. 또한 담임 선생님과 주간선생님이 함께 학생을 관리해 주셔서 학습 상황뿐만 아니라 전반적인 생활까지 균형 있게 점검받을 수 있었습니다. 필요할 때마다 편하게 상담을 요청드릴 수 있어 학습에 대한 고민이나 어려움을 신속하게 해결할 수 있었던 점도 큰 장점이었습니다.</v>
       </c>
       <c r="F329" t="str">
         <v>학습 관리 시스템은 학습 중 딴짓을 하지 않도록 환경을 만들어 주어 집중력을 유지하는 데 큰 도움이 되었습니다. 또한 스스로 하기 어려운 유혹을 자연스럽게 뿌리칠 수 있게 해주었으며, 타 학생들과 함께 관리되면서 서로에게 피해를 주지 않도록 책임감을 가지게 해주었습니다. 더불어 학습이 힘들 때에는 상담을 통해 어려움을 해소할 수 있어 지속적으로 학습을 이어가는 데 매우 유용했습니다.</v>
@@ -12405,7 +12405,7 @@
         <v>일반 독서실이나 관리형 독서실들과는 다르게 핵심과목인 국어,영어,수학 전공자 선생님들께서 상주하고 계셔서 문제를 풀다가 막힘이 오거나 특정과목에 대한 상담이 필요할때 즉각적인 질의응답을 통한 학습이 가능하다는 점이 가장 큰 장점이였다. 온라인 강의와 사이트를 이용하다보면 강의와 개념, 문제들에 대한 질문을 qna 게시판을 통해서만 질문이 가능한데 이는 시간도 오래걸리고 대면으로 질문하는것이 아니기에 한계가 존재했었다. 또한 이투스 247 목동 졸업생들이 멘토로 근무를 하여 특정 탐구 과목들에 대한 피드백과 질문, 조언들을 얻을 수 있다는 점에서 이투스 247 목동만의 독보적이고 차별적인 시스템이다.</v>
       </c>
       <c r="G332" t="str">
-        <v>공부를 하는 학생 입장에서 독학재수학원을 생각할때 중요시하게 고려하는 요소가 면학 분위기 입니다. 그러한점에서 목동 이투스 247은 다양한 시스템을 통한 최고의 면학 분위기를 제공해주었습니다. 우선 매너타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경쓰이지 않고 다같이 집중 할 수 있는 공부 환경을 제공해줍니다. 또한 학생들이 학습중 자지 않도록 상시로 감독 선생님께서 자습실을 비롯한 공용학습 공간까지 꼼꼼히 돌아다니시며 모든 학생이 열심히 공부를 할 수 있게 도와주십니다.</v>
+        <v>공부를 하는 학생 입장에서 독학재수학원을 생각할때 중요시하게 고려하는 요소가 면학 분위기 입니다. 그러한점에서 목동 이투스 247은 다양한 시스템을 통한 최고의 면학 분위기를 제공해주었습니다. 우선 매너타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다같이 집중 할 수 있는 공부 환경을 제공해줍니다. 또한 학생들이 학습중 자지 않도록 상시로 감독 선생님께서 자습실을 비롯한 공용학습 공간까지 꼼꼼히 돌아다니시며 모든 학생이 열심히 공부를 할 수 있게 도와주십니다.</v>
       </c>
       <c r="H332" t="str">
         <v>목동 이투스 247점에서는 단어테스트반을 모집하여 매주 영단어 테스트를 봅니다. 학생들이 가장 귀찮아하고 소홀히하는 영단어 외우기를 같은 학생들과 함께 매주 테스트를 보며 매주 빼먹지 않게 외우게된다는 장점이 있습니다.</v>
@@ -12414,7 +12414,7 @@
         <v>항상 입시 스트레스로와 몸 건강으로 인해 학원에게 피해를 많이 끼쳤지만 그럼에도 불구하고 항상 격려해주시고 힘을 내게 도와주셔서 덕분에 끝까지 입시를 마칠 수 있었습니다. 모두 선생님들 덕분입니다. 제 입시에서 이투스 247 선생님들을 만난것이 가장 큰 행운이였습니다 감사합니다..!</v>
       </c>
       <c r="J332" t="str">
-        <v>매너 타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경쓰이지 않고 다같이 집중 할 수 있는 공부 환경을 제공해주셨어요.</v>
+        <v>매너 타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다같이 집중 할 수 있는 공부 환경을 제공해주셨어요.</v>
       </c>
       <c r="K332" t="str">
         <v/>
@@ -12469,7 +12469,7 @@
         <v>N수생</v>
       </c>
       <c r="E334" t="str">
-        <v>선생님들이 과목별로 다르게 저한테 맞는 공부법을 알려주셨습니다. 선생님 본인의 수험생활에서 효과를 보셨던 방법들부터 선배님들의 방법까지 소개해주셔서 도움이 많이 됐습니다. 학습 뿐만아니라 생활부분에서도 힘든 점이나 어려운 점이 있으면 쉽게 말할 수 있는 분위기여서 학원 생활에 있어 큰 어려움은 없었습니다. 선생님들 덕분에 수월한 수험생활을 한 것 같습니다.</v>
+        <v>선생님들이 과목별로 다르게 저한테 맞는 공부법을 알려주셨습니다. 선생님 본인의 수험 생활에서 효과를 보셨던 방법들부터 선배님들의 방법까지 소개해주셔서 도움이 많이 됐습니다. 학습 뿐만아니라 생활부분에서도 힘든 점이나 어려운 점이 있으면 쉽게 말할 수 있는 분위기여서 학원 생활에 있어 큰 어려움은 없었습니다. 선생님들 덕분에 수월한 수험 생활을 한 것 같습니다.</v>
       </c>
       <c r="F334" t="str">
         <v>매달 정기고사나 모의고사가 끝나면 필수로 해야하는 상담이 있었는데 결과가 좋든 좋지 않든 선생님께서 편안하게 상담을 진행해주셨고, 잘 한 부분은 아낌없는 칭찬과 아쉬운 부분은 어떻게 해결해나가야하는지에 대해 보완점도 제시해주셔서 유용했습니다.</v>
@@ -12481,7 +12481,7 @@
         <v>원내에서 자신의 위치, 전국단위에서의 자신의 위치를 확인할 수 있어서 위치파악에 유용했고, 매달 정기고사가 있다는 점 자체에 긴장감을 심어주어 공부에 자극이 되고 다음번에는 더 좋은 성적을 받아야 되겠다는 원동력이 되기도 했습니다.</v>
       </c>
       <c r="I334" t="str">
-        <v>선생님들! 수험생활 내내 옆에서 정신적 지지를 해주셔서 감사합니다. 선생님들이 있어서 지루하고 무료했던 제 수험 생활이 조금이나마 즐거웠던 것 같습니다. 항상 생각했던 건데 저는 다시 돌아가도 꼳 이투스 독학 기숙을 선택할 것 같습니다.</v>
+        <v>선생님들! 수험 생활 내내 옆에서 정신적 지지를 해주셔서 감사합니다. 선생님들이 있어서 지루하고 무료했던 제 수험 생활이 조금이나마 즐거웠던 것 같습니다. 항상 생각했던 건데 저는 다시 돌아가도 꼳 이투스 독학 기숙을 선택할 것 같습니다.</v>
       </c>
       <c r="J334" t="str">
         <v>과목별로 공부 방법을 추천해 주셨는데 저와 너무 잘 맞아서 성적 올리는 데 도움이 됐어요.</v>
@@ -12513,7 +12513,7 @@
         <v>학원에서 선생님들이 학습실을 쉬는 시간이나 점심시간 전후로 돌아다니시면서 가끔씩 너무 졸려서 자는 친구들을 깨워주시고 면학 분위기를 조성하기 위해 열심히 노력해주시는 모습이 도움이 되었다.</v>
       </c>
       <c r="H335" t="str">
-        <v>학력평가나 모의평가를 시행하지 않는 달에 이투스 모의고사로 나의 실력을 점검할 수 있는 기회를 주어 현재 나의 상황을 점검하고 앞으로의 공부계획을 세울 수 있도록 도와주어서 좋았던 것 같다.</v>
+        <v>학력평가나 모의평가를 시행하지 않는 달에 이투스 모의고사로 나의 실력을 점검할 수 있는 기회를 주어 현재 나의 상황을 점검하고 앞으로의 공부 계획을 세울 수 있도록 도와주어서 좋았던 것 같다.</v>
       </c>
       <c r="I335" t="str">
         <v>선생님들 안녕하세요! 오랜만에 이렇게 후기를 남기면서 인사드립니다. 사실 학원 들어올 때까지만 해도 지방대 공대에 다니고 있어서 잘해봐야 국숭세단 정도 갈 줄 알았는데 학원에와서 5개월 정도 공부하고 이제는 제가 중앙대에 다니고 있네요. 이게 다 저를 잘 캐어해주신 선생님들 덕분인 듯 합니다. 정말 감사드려요!</v>
@@ -12545,7 +12545,7 @@
         <v>처음 기숙학원에 들어왔을 때 무엇을 할지 몰라서 일단 제가 좋아하는 과목을 위주로 공부를 해 각 과목 점수의 편차가 컸습니다.그러나 선생님께서 플래너를 작성하고 어떻게 활용해야 하는 지를 알려주고 난 후, 과목 불균형을 해소하여 시험을 볼때 대부분 과목들이 비슷한 등급을 받았습니다. 또한 자신이 어디까지 공부했고 어디가 부족한지 표시하여 그다음날 무엇을 더집중적으로 하고, 또 무엇을 보충할지 등 더 체계적으로 공부할 수 있었습니다.</v>
       </c>
       <c r="G336" t="str">
-        <v>제가 제일 공부할때 방해되는것이 인터넷 이였습니다. 공부를 하다가도 집중이 안되면 핸드폰을 보며 유튜브를 들어가거나 게임을 하기도 했었습니다. 그러나 이투스 기숙학원에 들어오고나서 핸드폰을 걷고 학원 태블릿을 이용하여 강의만 들을 수 있어서  처음에는 그게 불만이였지만 나중에는 유튜브나 인터넷에 못들어가니 공부에 더 집중할수 있었습니다.</v>
+        <v>제가 제일 공부할때 방해되는것이 인터넷 이였습니다. 공부를 하다가도 집중이 안되면 핸드폰을 보며 유튜브를 들어가거나 게임을 하기도 했었습니다. 그러나 이투스 기숙학원에 들어오고나서 핸드폰을 걷고 학원 태블릿을 이용하여 강의만 들을 수 있어서  처음에는 그게 불만이였지만 나중에는 유튜브나 인터넷에 못들어가니 공부에 더 집중할 수 있었습니다.</v>
       </c>
       <c r="H336" t="str">
         <v>제가 궁금한건 어떻게 공부해야 할지 였습니다. 모의고사를 보고나서 이걸 어떻게 분석해야하는지가 문제였는데 이투스 모의고사를 보고 어디 단원을 공부해야하고 어디가 부족하고 다른사람들은 어느정도 맞췄는지, 그리고 이점수로 어느 대학에 진학할수 있는지를 알려주어서 큰 도움이 되었습니다.</v>
@@ -12574,13 +12574,13 @@
         <v>반수생</v>
       </c>
       <c r="E337" t="str">
-        <v>선생님께서 공부를 전체적으로 어떤 방식으로 해나가야하는지 계속해서 조언해주셔서 도움아 돠었습니다.또 모의고사를 본 후 선생님께서 개선해야할점을 알려주신점도 도움이 많이 되었습니다.어떤부분에 대해 내가 약하고 어떤 부분에서 실수가 계속해서 일어나는지 알게 되고 고치게 도움을 많이 주십니다</v>
+        <v>선생님께서 공부를 전체적으로 어떤 방식으로 해나가야하는지 계속해서 조언해주셔서 도움아 돠었습니다.또 모의고사를 본 후 선생님께서 개선해야 할점을 알려주신점도 도움이 많이 되었습니다.어떤부분에 대해 내가 약하고 어떤 부분에서 실수가 계속해서 일어나는지 알게 되고 고치게 도움을 많이 주십니다</v>
       </c>
       <c r="F337" t="str">
         <v>인터넷강의의 가장 큰 단점은 커리가 너무 많다는점인데 선생님과 상담후 나에게 딱 맞는 강의를 수강하는데 도움이 많이 되었습니다.반수생이었던 저는 시간이 부족해 선택과 집중이 되게 중요했는데 선생님의 도움이 없었더라면 혼자 방황했을꺼 같습니다.</v>
       </c>
       <c r="G337" t="str">
-        <v>현역때의 수능실패 원인을 되돌아보자면 휴대폰이었습니다.공부를 하러 도서관애 갔어도 휴대폰만 하고 돌아오던 시간이 대부분이었습니다.휴대폰을 등교때 제출함으로써 집중력 분산도 안되고 온전히 공부에만 집중할수있는 환경이 만들어졌습니다.</v>
+        <v>현역때의 수능실패 원인을 되돌아보자면 휴대폰이었습니다.공부를 하러 도서관애 갔어도 휴대폰만 하고 돌아오던 시간이 대부분이었습니다.휴대폰을 등교때 제출함으로써 집중력 분산도 안되고 온전히 공부에만 집중할 수있는 환경이 만들어졌습니다.</v>
       </c>
       <c r="H337" t="str">
         <v>유명하신 선생님들의 강의를 무료로 수강할수있어서 좋았습니다.특히 국어영역의 김민경 선생님의 강의중 ebs 연계에 대한 강의를 자투리 시간에 수강함으로써 ebs 독서 연계에 대해 대비를 더욱 철저히 하게 될 수 있었습니다.</v>
@@ -12589,7 +12589,7 @@
         <v>5개월 동안 성적을 끌어올랄수 았었던건 이투스 247 선생님분들이 있었기에 가능했습니다.혼자였다면 백분위 10이 절대로 상승하지 못했을것입니다.5개월 동안 신경써주셔서 정말 감사했습니다</v>
       </c>
       <c r="J337" t="str">
-        <v>휴대폰을 등교때 제출함으로써 집중력 분산도 안되고 온전히 공부에만 집중할수있는 환경이 만들어졌었어요.</v>
+        <v>휴대폰을 등교때 제출함으로써 집중력 분산도 안되고 온전히 공부에만 집중할 수있는 환경이 만들어졌었어요.</v>
       </c>
       <c r="K337" t="str">
         <v/>
@@ -12615,13 +12615,13 @@
         <v>고등학교 재학 시절에는 정해진 시간표대로 수업을 듣고, 정해진 일정대로 공부했으나, 재수를 시작하고 모든 것을 직접 계획하고 설계해야 하기에 벅찬 느낌이 있었습니다. 그러나 이투스247의 학습 계획 및 플래너 상담 시스템을 통해 더 계획적이고 정교한 수험 생활을 이어갈 수 있었습니다. 단순히 계획을 제가 일방적으로 보고하는 시스템이 아니라 서로 상의하고 더 나은 방향으로 발전시키는 시스템이기 때문에 정말 유용했던 것 같습니다.</v>
       </c>
       <c r="G338" t="str">
-        <v>이투스247의 면학 분위기 관리와 졸음 관리가 제 수험생활에 정말 많은 도움이 되었습니다. 현역 수능이 끝나고 다소 공부에서 멀어진 삶을 살다 다시 수험생활로 돌아오니, 생각보다 공부에 적응하는 것에 어려움이 있었는데요. 잘 형성된 면학 분위기 속에서 공부하며, 혹시 졸더라도 선생님 분들이 깨워주시어 다시 몰입할 수 있는 환경이었기에 다시금 수험 생활에 빠르게 적응할 수 있었습니다.</v>
+        <v>이투스247의 면학 분위기 관리와 졸음 관리가 제 수험 생활에 정말 많은 도움이 되었습니다. 현역 수능이 끝나고 다소 공부에서 멀어진 삶을 살다 다시 수험 생활로 돌아오니, 생각보다 공부에 적응하는 것에 어려움이 있었는데요. 잘 형성된 면학 분위기 속에서 공부하며, 혹시 졸더라도 선생님 분들이 깨워주시어 다시 몰입할 수 있는 환경이었기에 다시금 수험 생활에 빠르게 적응할 수 있었습니다.</v>
       </c>
       <c r="H338" t="str">
         <v>이투스247에서 제공하는 VOCA 콘텐츠를 통해 꾸준하고 접근성 편한 영어 단어 공부를 이어갈 수 있었습니다. 사실 영어라는 과목이 수능에서 차지하는 비중이 적다보니 선뜻 공부할 마음이 생기지 않을 때도 있고, 지속적인 학습이 어렵습니다. 하지만 이투스247의 VOCA 콘텐츠 덕분에 영어 학습을 저의 학습 루틴에 포함시키고 꾸준하게 영어 실력을 키워나갈 수 있었기에 매우 유용했습니다.</v>
       </c>
       <c r="I338" t="str">
-        <v>끝나지 않을 것 같던 수험생활도 어느새 끝이 나고 그렇게 바라던 약학대학에 입학해 즐겁게 다니고 있습니다. 이투스247 학원의 선생님들께서 진심으로 임해주신 덕분이라고 언제나 생각합니다. 제 인생에서 잊을 수 없는 한 페이지가 될 것 같아요. 정말 감사했습니다!</v>
+        <v>끝나지 않을 것 같던 수험 생활도 어느새 끝이 나고 그렇게 바라던 약학대학에 입학해 즐겁게 다니고 있습니다. 이투스247 학원의 선생님들께서 진심으로 임해주신 덕분이라고 언제나 생각합니다. 제 인생에서 잊을 수 없는 한 페이지가 될 것 같아요. 정말 감사했습니다!</v>
       </c>
       <c r="J338" t="str">
         <v>학습 상담 외에도 생활, 멘탈 관련 상담도 해주셔서 단단해진 마음으로 공부에 임할 수 있었어요.</v>
@@ -12650,7 +12650,7 @@
         <v>국영수탐구 뿐만 아니라 논술 전형 응시 예정이었어서 특정 학교 논술 관련해서 궁금한 점을 여쭤본 적이 있었는데 선생님께서 저에게 도움이 될 수 있는 답변을 해주셔서 실제로 논술을 준비하는 과정에서 도움이 되었던 경험이 있습니다</v>
       </c>
       <c r="G339" t="str">
-        <v>아무래도 스카 혹은 집에서 독학 재수를 하는 경우에는 휴대폰을 가끔은 보게 되어 온전히 집중하지 못하는 경우가 많은데 이투스에서는 등원하면서 휴대폰을 제출해서 하루종일 공부와 해야할 일에만 집중할 수 있었다는 점이 좋았습니다</v>
+        <v>아무래도 스카 혹은 집에서 독학 재수를 하는 경우에는 휴대폰을 가끔은 보게 되어 온전히 집중하지 못하는 경우가 많은데 이투스에서는 등원하면서 휴대폰을 제출해서 하루종일 공부와 해야 할 일에만 집중할 수 있었다는 점이 좋았습니다</v>
       </c>
       <c r="H339" t="str">
         <v>타사 인강들만 사용하고 있었어서 이투스 강의를 듣지 못하는 점이 아쉬웠었는데 구독을 통해서 이투스에서만 들을 수 있는 선생님들의 강의를 필요할 때마다 수강할 수 있었다는 점이 학습적인 측면에서 매우 좋았던 것 같습니다</v>
@@ -12788,7 +12788,7 @@
         <v>어떻게 하면 수능에서 고득점을 받을 수 있을지 구체적인 공부법들을 제안해주셨다. 공부를 하다보면 자칫 객관성을 잃고 잘못된 방향으로 빠질 수도 있는데, 매일 밴드로 적절한 공부방법과 동기부여를 올려주셔서 1년 동안 제대로 된 방향으로 공부할 수 있었다. 또한 수능이라는 시험에 대한 이해도를 높여주셔서 나중에는 스스로 올바른 공부방법을 찾아나갈 수 있었다.</v>
       </c>
       <c r="F343" t="str">
-        <v>온라인으로 미리 예약한 후 질의응답하는 시스템을 통해 1분 1초가 아까운 수험생활에서 시간을 허비할 일이 없어서 좋았다. 선생님들 또한 질문을 가지고 가면 열정적으로 답변해주셨으며, 문제 풀이 뿐만 아니라 학습 상담까지 친절하게 해주셨다.</v>
+        <v>온라인으로 미리 예약한 후 질의응답하는 시스템을 통해 1분 1초가 아까운 수험 생활에서 시간을 허비할 일이 없어서 좋았다. 선생님들 또한 질문을 가지고 가면 열정적으로 답변해주셨으며, 문제 풀이 뿐만 아니라 학습 상담까지 친절하게 해주셨다.</v>
       </c>
       <c r="G343" t="str">
         <v>옆에서 자는 학생이 있으면 공부할 때 방해가 될 수 있는데, 선생님들께서 자습 시간에 돌아다니시며 졸거나 자는 학생들을 깨워주셔서 열정적인 면학 분위기가 형성될 수 있었다. 학생들을 방치하지 않는 덕분에 졸릴 때도 정신을 차리고 공부할 수 있어서 좋았다.</v>
@@ -12824,7 +12824,7 @@
 더불어 선생님께서 항상 상주하시며 저의 공부 과정을 지켜봐 주셨기 때문에, 1년간의 학습 패턴과 습관을 반영한 꼼꼼한 개인 학습 관리를 받을 수 있었습니다. 공부 중 막히는 부분이 있을 때마다 친절하게 함께 해결해 주셔서 부담 없이 도움을 요청할 수 있었던 점도 큰 도움이 되었습니다.</v>
       </c>
       <c r="F344" t="str" xml:space="preserve">
-        <v xml:space="preserve">저의 경우 강점 과목과 약점 과목이 뚜렷하고, 고3 때와 다른 과목으로 수능을 준비해야 했기 때문에 과목별 학습 분량과 시기별 진도를 계획하는 데 어려움이 있었습니다. 그러나 학습관리시스템을 통해 일별·주별·월별로 과목별 학습 목표와 시간을 설정하고, 수능과 유사한 시간표로 체계적으로 공부할 수 있어 큰 도움이 되었습니다._x000d_
+        <v xml:space="preserve">저의 경우 강점 과목과 약점 과목이 뚜렷하고, 고3 때와 다른 과목으로 수능을 준비해야 했기 때문에 과목별 학습 분량과 시기별 진도를 계획하는 데 어려움이 있었습니다. 그러나 학습 관리시스템을 통해 일별·주별·월별로 과목별 학습 목표와 시간을 설정하고, 수능과 유사한 시간표로 체계적으로 공부할 수 있어 큰 도움이 되었습니다._x000d_
 또한 주기적으로 선생님과 플래너 상담을 진행하며 학습이 계획대로 이루어지고 있는지 점검하고, 진도가 늦어지거나 예상보다 빠른 경우에는 상황에 맞는 추가 학습 솔루션을 제공받을 수 있었습니다. 그 결과 매일 평균 13시간의 순공 시간을 달성할 수 있었고, 그 안에서 저에게 맞는 학습 타임테이블을 구축해 더욱 효율적이고 집중도 높은 공부를 이어갈 수 있었습니다.</v>
       </c>
       <c r="G344" t="str" xml:space="preserve">
@@ -12945,7 +12945,7 @@
         <v>N수생</v>
       </c>
       <c r="E347" t="str">
-        <v>상담이 필요할때마다 상담을 최대한 빠르게 응해주신 점이 좋았습니다. 모의고사를 본 후에 최대한 빠른 시간에 모의고사를 직접 검토해주시고 아직 부족한 점이나 채워야할 점들을 피드백해주셔서 좋았습니다. 또 모의고사와 플래너를 함께 피드백해주셔서 앞으로의 방향을 가르쳐주신 점이 도움이 되었습니다. 상담을 하면서 가지고 있는 고민이나 생활습관 같은 사소한 것들도 마음 편하게 얘기할 수 있어서 외로운 수험생활동안 학원에서만큼이라도 공부에만 집중할 수 있었던 것 같습니다.</v>
+        <v>상담이 필요할때마다 상담을 최대한 빠르게 응해주신 점이 좋았습니다. 모의고사를 본 후에 최대한 빠른 시간에 모의고사를 직접 검토해주시고 아직 부족한 점이나 채워야할 점들을 피드백해주셔서 좋았습니다. 또 모의고사와 플래너를 함께 피드백해주셔서 앞으로의 방향을 가르쳐주신 점이 도움이 되었습니다. 상담을 하면서 가지고 있는 고민이나 생활 습관 같은 사소한 것들도 마음 편하게 얘기할 수 있어서 외로운 수험 생활동안 학원에서만큼이라도 공부에만 집중할 수 있었던 것 같습니다.</v>
       </c>
       <c r="F347" t="str">
         <v>독학재수에서의 가장 큰 단점이 자신이 어느정도까지 공부를 했는지, 어느정도에 위치해 있는지, 어떤 점이 잘못되었는지 를 스스로 알아차리기 힘든 것인데, 성적 레포팅과 피드백을 거치면서 내가 어떤 잘못된 공부 방법을 가지고 있는지 내가 이때까지 성장했는지를 제 3자의 눈으로 볼 수 있었다는 점이 가장 좋았습니다.</v>
@@ -12957,7 +12957,7 @@
         <v>영어단어 외우기를 평소에 너무 귀찮아해서 항상 영어단어가 부족했었는데 보카테스트를 정해진 요일에 하면서 귀찮더라도 억지로 암기 습관을 들이며 매주 응시하면서 점차 영어단어에 대한 거부감도 사라지고 매주하다보니 점차 아는 단어가 많아지면서 문제가 잘 풀리다보니 점점 더 영어 공부에 애정을 가지게 되어 재밌게 공부할 수 있었습니다.</v>
       </c>
       <c r="I347" t="str">
-        <v>이투스 대구 달서점 선생님들 모두 친절하게 항상 도와주셔서 다들 너무 감사드립니다. 그리고 현역, 재수 모두 맡아주신 담임선생님도 특히 감사드리고 일요일마다 아침일찍 나올 수 있게 도와주신 토,일 담당 선생님도 감사드립니다🥹</v>
+        <v>이투스 대구 달서점 선생님들 모두 친절하게 항상 도와주셔서 다들 너무 감사드립니다. 그리고 현역, 재수 모두 맡아주신 담임 선생님도 특히 감사드리고 일요일마다 아침일찍 나올 수 있게 도와주신 토,일 담당 선생님도 감사드립니다🥹</v>
       </c>
       <c r="J347" t="str">
         <v>정해진 날마다 영단어 테스트를 진행해서 귀찮아도 미루지 않고 공부할 수 있어요!</v>
@@ -12983,7 +12983,7 @@
         <v>담임 선생님께서 상담하실 때 마다 각 과목 별 공부가 어떻게 진행되고 있는지 구체적으로 상담해주시고(예를 들면 어떤 인강을 듣고 있는지, 또는 어떤 문제집을 풀고 있는지) 해당 내용이 끝난 다음에는 어떤 커리큘럼을 밟으면 좋은지 상담해주시는 등 구체적인 공부방향 설정에 큰 도움을 주셨습니다.</v>
       </c>
       <c r="F348" t="str">
-        <v>플래너를 주기적으로 검사함을 통해 하루에 몇 시간 정도 공부하는지 또 과목별로 균형있게 학습하고 있는 지를 확인해 주시고 그에 따라 학습 피드백을 해주시는 것이 좋았습니다. 또 상담을 통해 또는 스스로 세운 계획을 얼마나 잘 지키고 있는지 점검함을 통해 학습관리를 잘 해주신 부분이 좋았습니다.</v>
+        <v>플래너를 주기적으로 검사함을 통해 하루에 몇 시간 정도 공부하는지 또 과목별로 균형있게 학습하고 있는 지를 확인해 주시고 그에 따라 학습 피드백을 해주시는 것이 좋았습니다. 또 상담을 통해 또는 스스로 세운 계획을 얼마나 잘 지키고 있는지 점검함을 통해 학습 관리를 잘 해주신 부분이 좋았습니다.</v>
       </c>
       <c r="G348" t="str">
         <v>담임 선생님들이 주기적으로 면학 분위기 조성에 힘쓰시는 것이 느껴졌습니다. 일단 오전, 오후마다 선생님들이 졸고 있는 학생들을 깨우셨고 휴가 전후로 전체적으로 분위기가 헤이해지면 더 강하게 면학 분위기 관리에 힘을 쓰셨습니다. 덕분에 분위기에 휩쓸리지 않고 공부할 수 있어서 좋았습니다.</v>
@@ -13128,7 +13128,7 @@
         <v>6월과 9월 평가원 모의고사를 보고나서 나름 선방했다는 생각에 방심하고 있었으나, 담당 선생님과 모의고사 후 면담을 통해 제 점수대를 객관적으로 파악할 수 있었고, 매주 응시하는 실전 모의고사 채점 결과를 토대로 부족한 부분이 무엇인지 빠르게 알 수 있었습니다.</v>
       </c>
       <c r="G352" t="str">
-        <v>앞 질문 중 하나에서 답했듯이 아침, 점심, 저녁 식후 가장 졸음이 많이 쏟아지는 시간대에 자주 돌아다니시며 지도 선생님들이 깨워주셨습니다. 또한 공부 외에 어떤 것에도 신경쓰이지 않게 면학 분위기 조성을 위해 노력하시는 모습이 보였습니다.</v>
+        <v>앞 질문 중 하나에서 답했듯이 아침, 점심, 저녁 식후 가장 졸음이 많이 쏟아지는 시간대에 자주 돌아다니시며 지도 선생님들이 깨워주셨습니다. 또한 공부 외에 어떤 것에도 신경 쓰이지 않게 면학 분위기 조성을 위해 노력하시는 모습이 보였습니다.</v>
       </c>
       <c r="H352" t="str">
         <v>사실 영단어 외우기는 강제성이 없으면 스스로 매일 하기 힘든 컨텐츠입니다. 이투스에서는 매일 점심시간에 60개의 영단어를 외우는 프로그램을 필수로 하여 실제 모의고사 등을 응시할 때 정말 도움이 되었습니다.</v>
@@ -13203,7 +13203,7 @@
         <v>가나다군의 입시전략을 세우는 데에 유용했다. 진학사 칸수만으로는 알기 힘든 정보로 좀 더 현실적인 전략을 세워주셨다. 지난 학생들의 정보를 통해 몇칸정도 채워지면 어느정도 가능성이 있는지 알려주셨고 그대로 들어맞아 결국 원하는 대학에 합격할 수 있었다.</v>
       </c>
       <c r="F354" t="str">
-        <v>문제를 풀다보면 인강이나 답지만으로는 해결할 수 없는 경우가 종종 있다. 이때 혼자서 해결하려고 했으면 막막했을텐데 담당선생님께 여쭈어 바로바로 해결할 수 있어 학습이 원활했다. 또 다양한 풀이방법을 선생님과 함께 고민할 수 있어 학업능력이 향상되었다</v>
+        <v>문제를 풀다보면 인강이나 답지만으로는 해결할 수 없는 경우가 종종 있다. 이때 혼자서 해결하려고 했으면 막막했을텐데 담당 선생님께 여쭈어 바로바로 해결할 수 있어 학습이 원활했다. 또 다양한 풀이방법을 선생님과 함께 고민할 수 있어 학업능력이 향상되었다</v>
       </c>
       <c r="G354" t="str">
         <v>공부하기 싫어도 감시받고 있다는 느낌이 들어 공부를 하게 되고 잠을 자고 싶다가도 선생님들 발자국 소리가 들리면 잠이 확 깼다. 또 나도 모르게 졸았을 때 감독선생님께서 깨워주셔서 계속 학업에 집중할 수 있었다.</v>
@@ -13212,7 +13212,7 @@
         <v>집에서 혼자 모의고사를 풀면 시간이나 방식을 제대로 지키지 않게 된다. 하지만 여기서는 모의고사 환경을 조성해줘 실제 수능을 보는듯한 마음가짐으로 모의고사를 볼 수 있었다. 또 성적이 나와 나의 대략적 위치를 파악하기가 용의했다.</v>
       </c>
       <c r="I354" t="str">
-        <v>힘들때마다 응원해주셔서 감사합니다. 선생님들 덕분에 대학갈 수 있었어요!! 특히 공부하라고 따끔하게 한마디 해주신거 당시엔 너무너무 속상했는데 지금 생각하니 정말 좋은 동기부여였던 것 같아요 사랑합니다!!!</v>
+        <v>힘들 때마다 응원해주셔서 감사합니다. 선생님들 덕분에 대학갈 수 있었어요!! 특히 공부하라고 따끔하게 한마디 해주신거 당시엔 너무너무 속상했는데 지금 생각하니 정말 좋은 동기부여였던 것 같아요 사랑합니다!!!</v>
       </c>
       <c r="J354" t="str">
         <v>실제 수험장과 똑같은 환경으로 관리해 주셔서 실전처럼 매일 공부할 수 있었어요.</v>
@@ -13250,7 +13250,7 @@
 ​엄격한 시간 제한 속에서 OMR 카드 마킹까지 마쳐야 하는 연습을 반복하다 보니, 실제 시험에서 느낄 수 있는 압박감에 익숙해질 수 있었습니다. 특히 고퀄리티의 문항들을 접하며 시간 배분 전략을 스스로 점검하고, 어려운 문제에 직면했을 때의 대처 능력을 기를 수 있었던 점이 만족스러웠습니다.</v>
       </c>
       <c r="I355" t="str">
-        <v>담임 선생님, 실장 선생님 , 사감선생님, 영양사선생님 등등 전부 감사인사를 드립니다. 덕분에 수험생활을 잘 마칠 수 있었습니다. 항상 하는 일마다 행운이 깃들기를 기원하겠습니다!</v>
+        <v>담임 선생님, 실장 선생님 , 사감선생님, 영양사선생님 등등 전부 감사인사를 드립니다. 덕분에 수험 생활을 잘 마칠 수 있었습니다. 항상 하는 일마다 행운이 깃들기를 기원하겠습니다!</v>
       </c>
       <c r="J355" t="str">
         <v>학원에서 제공하는 학습 계획 플래너 관리를 받으면서 공부의 질이 완전히 달라졌었어요.</v>
@@ -13273,7 +13273,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E356" t="str">
-        <v>수험생활을 하며 힘든 포인트에 공부도 있지만, 수험생 본인이 처한 주변환경도 무시할 수 없다고 생각합니다. 그래서 저에겐 일상생활에 생긴 일에 대해 상담해주는 코칭 시스템이 주변환경의 짐을 덜어주고 공부에게만 집중하게 도와주었다고 생각합니다.</v>
+        <v>수험 생활을 하며 힘든 포인트에 공부도 있지만, 수험생 본인이 처한 주변환경도 무시할 수 없다고 생각합니다. 그래서 저에겐 일상생활에 생긴 일에 대해 상담해주는 코칭 시스템이 주변환경의 짐을 덜어주고 공부에게만 집중하게 도와주었다고 생각합니다.</v>
       </c>
       <c r="F356" t="str">
         <v>너무 많은 인강선생님들 속에서 누가 나에게 맞는 인강 선생님일지, 어떤 교재가 나에게 맞을지 감도 안 잡혔는데 나에게 어떤 선생님과 교재가 많을 지 직접 추천해주시니까 공부를 시작하는데에 큰 도움이 됐어요</v>
@@ -13308,19 +13308,19 @@
         <v>N수생</v>
       </c>
       <c r="E357" t="str">
-        <v>긴 n수생활로 생활루틴을 어떻게잡을지도 지쳐있고 매번 정해지지않은 상태로 그날그날에 끌리는 과목만 공부하는정도였는데 이투스247에서 담임선생님과의 일주일에 한번씩 생활루틴을 상담받으면서 점차 제 루틴이 정립되었고 그게쌓이면서 수능때 좋은성적을 받게되었던것같습니다</v>
+        <v>긴 n수생활로 생활루틴을 어떻게잡을지도 지쳐있고 매번 정해지지않은 상태로 그날그날에 끌리는 과목만 공부하는정도였는데 이투스247에서 담임 선생님과의 일주일에 한 번씩 생활루틴을 상담받으면서 점차 제 루틴이 정립되었고 그게쌓이면서 수능때 좋은성적을 받게되었던것같습니다</v>
       </c>
       <c r="F357" t="str">
-        <v>항상 과목시간도 정해놓지않고 끌리는대로만 공부를 하던상황이라 제가 인지하지도 못한 채 성적이 잘나오는 과목만 더 열심히 하게되고, 잘 안나오는 과목은 후순위로 두는 실수를 두게되었는데 담임선생님이 제가 쓴 학습 계획서를 꼼꼼히 봐주면서 지금 제가 어느과목을 회피하고있는지 명확히 알려주시고 해야한다에 그치지않고 그 과목이 부족한이유와 그 수준에맞는 새로운 공부법과 문제집을 계속 추천해주시면서 부족한과목을 놓지않게하여 결국 수능날 전체과목의 평균이 높은상태로 마무리되어 평균자체가 높아 유리한 교대에 합격하게된것같습니다</v>
+        <v>항상 과목시간도 정해놓지않고 끌리는대로만 공부를 하던상황이라 제가 인지하지도 못한 채 성적이 잘나오는 과목만 더 열심히 하게되고, 잘 안나오는 과목은 후순위로 두는 실수를 두게되었는데 담임 선생님이 제가 쓴 학습 계획서를 꼼꼼히 봐주면서 지금 제가 어느과목을 회피하고있는지 명확히 알려주시고 해야한다에 그치지않고 그 과목이 부족한이유와 그 수준에맞는 새로운 공부법과 문제집을 계속 추천해주시면서 부족한과목을 놓지않게하여 결국 수능날 전체과목의 평균이 높은상태로 마무리되어 평균자체가 높아 유리한 교대에 합격하게된것같습니다</v>
       </c>
       <c r="G357" t="str">
-        <v>아무래도 태블릿과 핸드폰이 수험생활에서 제일 큰 방해요인이 아닐까라고 생각이 드는데, 이투스247김포점은 말로만 태블릿과 핸드폰을 하지말라고만 하는게 아니라 방화벽까지 꼼꼼하게 막아두고 재원학생들의 태블릿을 등록시켜놔서 딴짓을 하고있는지 계속 주의하면서 실제로 2분정도 딴짓을 하기위해 이 정도면 모르시겠지하고 인터넷을 들어갔는데 바로 감시중이던 선생님이 인터넷 접속을 원격으로 끊으셔서 오히려 딴짓할까 생각도 하지못하고 오히려 딴짓도 못하는데 공부라도 열심히해야겠다라는 마인드로 바로 바뀌었던것같습니다 그만큼 태블릿관리를 말로만하지않으시고 실제계속된감시와 주의로 학생들이 공부에만 집중할수있게 면학 분위기를 조성시킨게 정말 큰 도움이되었던것같습니다</v>
+        <v>아무래도 태블릿과 핸드폰이 수험 생활에서 제일 큰 방해요인이 아닐까라고 생각이 드는데, 이투스247김포점은 말로만 태블릿과 핸드폰을 하지말라고만 하는게 아니라 방화벽까지 꼼꼼하게 막아두고 재원학생들의 태블릿을 등록시켜놔서 딴짓을 하고있는지 계속 주의하면서 실제로 2분정도 딴짓을 하기위해 이 정도면 모르시겠지하고 인터넷을 들어갔는데 바로 감시중이던 선생님이 인터넷 접속을 원격으로 끊으셔서 오히려 딴짓할까 생각도 하지못하고 오히려 딴짓도 못하는데 공부라도 열심히해야겠다라는 마인드로 바로 바뀌었던것같습니다 그만큼 태블릿관리를 말로만하지않으시고 실제계속된감시와 주의로 학생들이 공부에만 집중할 수있게 면학 분위기를 조성시킨게 정말 큰 도움이되었던것같습니다</v>
       </c>
       <c r="H357" t="str">
         <v>솔직히 이투스모의고사는 사설이라서 그렇게 중요하지않겠지라는 생각으로 이투스모의고사를 생각했었는데 실제 재원생으로 이투스247을 다니면서 이투스모의고사가 제가 수능생활을 유지할수있게하는 큰 도움이 된것같습니다 아무래도 수능생활에서 6월9월모의고사 수능 이렇게 중요한모의고사는 3개라고 볼수있는데 그 사이의 텀이 너무 긴데, 그 사이동안 긴장이 풀어지면서 해아해질수있는 기간을 이투스모의고사가 적절히 그 기간동안 긴장의 끈을 놓지않게 텐션을 유지해주면서 나의 성적대가 지금 어느정도인지 내가 공부하고있는 지금 이 방향이 잘가고있는지 확인할수있게만든 중요한 이정표의 역할이 되었다고 생각합니다 그래서 이투스모의고사를 통해 수능때까지의 긴장의끈을 놓지않고 달리며 수능때좋은성적을 거뒀던것같습니다</v>
       </c>
       <c r="I357" t="str">
-        <v>늦은나이에 공부를 시작하느라 뭐가뭔지도 모르고 수능의기조가 어떤지도 몰랐는데 이튜스선생님들을 만나고 쓴소리와 격려의말을 들으면서 제가부족한점과 지금 고쳐야할점을 회피하지않고 직면하게되면서 지금 이 수험생활에서 중요하게 뭔지 다시금 생각하게 해주셨고, 격려의 말을 통해 나라는 학생도 수능에서의 성공을 꿈꿀수있는사람으로서 다시 생각하게해쥬셨던것같습니다 많이 모자랐는데도 그저 지나가는 학생이 아닌 정말 끌어서 제가원하는 목표를 이루게 하기위해 힘드실텐데도 본인들의 에너지를 써가면서 저를 설득하고 공부하게끔 다시도와주시는 모습을 수능끝나고 뼈저리게 감사한 마음을 느꼈던것같습니다 이투스247김포점에서 선생님들을 만나고 꿈을 이루게 된것에 너무 감사드리고 저를 지나가는 학생이 아니라 진심으로 대해주셔서 정말 감사합니다 덕분에 꿈을 이룬것같습니다 항상 행복하세요 선생님들 !❤️</v>
+        <v>늦은나이에 공부를 시작하느라 뭐가뭔지도 모르고 수능의기조가 어떤지도 몰랐는데 이튜스선생님들을 만나고 쓴소리와 격려의말을 들으면서 제가부족한점과 지금 고쳐야할점을 회피하지않고 직면하게되면서 지금 이 수험 생활에서 중요하게 뭔지 다시금 생각하게 해주셨고, 격려의 말을 통해 나라는 학생도 수능에서의 성공을 꿈꿀수있는사람으로서 다시 생각하게해쥬셨던것같습니다 많이 모자랐는데도 그저 지나가는 학생이 아닌 정말 끌어서 제가원하는 목표를 이루게 하기위해 힘드실텐데도 본인들의 에너지를 써가면서 저를 설득하고 공부하게끔 다시도와주시는 모습을 수능끝나고 뼈저리게 감사한 마음을 느꼈던것같습니다 이투스247김포점에서 선생님들을 만나고 꿈을 이루게 된것에 너무 감사드리고 저를 지나가는 학생이 아니라 진심으로 대해주셔서 정말 감사합니다 덕분에 꿈을 이룬것같습니다 항상 행복하세요 선생님들 !❤️</v>
       </c>
       <c r="J357" t="str">
         <v>담임 선생님께서 부족한 과목을 보완할 수 있는 교재를 추천해 주셨는데 잘 맞았어요!</v>
@@ -13378,13 +13378,13 @@
         <v>반수생</v>
       </c>
       <c r="E359" t="str">
-        <v>반수생이라 조금 다른사람에 비해서 늦게 시작한 감이 있었는데 제 위치와 현재 상황에 맞게  각 과목별로 추천하는 커리어나 학습량 그리고 생활 패턴까지 알려주셔서 좀 더 계획을 현실적으로 잡고 공부에만 집중할수 있었습니다</v>
+        <v>반수생이라 조금 다른사람에 비해서 늦게 시작한 감이 있었는데 제 위치와 현재 상황에 맞게  각 과목별로 추천하는 커리어나 학습량 그리고 생활 패턴까지 알려주셔서 좀 더 계획을 현실적으로 잡고 공부에만 집중할 수 있었습니다</v>
       </c>
       <c r="F359" t="str">
-        <v>혼자 무작정 진도를 나가는 것이 아니라 일정 주기로 얼만큼 학습했는지 확인을 받을수 있어서 공부가 잘되었던 주간이나 잘 안되었던 주간을 직접 확인할수 있어 중간에 흔들리더라도 다시 마음을 잡고 공부할수있는데에 큰 도움이 되었습니다</v>
+        <v>혼자 무작정 진도를 나가는 것이 아니라 일정 주기로 얼만큼 학습했는지 확인을 받을 수 있어서 공부가 잘되었던 주간이나 잘 안되었던 주간을 직접 확인할수 있어 중간에 흔들리더라도 다시 마음을 잡고 공부할 수있는데에 큰 도움이 되었습니다</v>
       </c>
       <c r="G359" t="str">
-        <v>제가 집중을 잘 못해서 초반에는 딴생각 하거나 조는일이 자주 있었는데 그때마다 바로바로 깨워 주셔서 나중에는 오히려 그게 습관이 고쳐져서 후반에는 딴생각이나 조는 일 없이 공부에만 집중할수 있었던거 같습니다</v>
+        <v>제가 집중을 잘 못해서 초반에는 딴생각 하거나 조는일이 자주 있었는데 그때마다 바로바로 깨워 주셔서 나중에는 오히려 그게 습관이 고쳐져서 후반에는 딴생각이나 조는 일 없이 공부에만 집중할 수 있었던거 같습니다</v>
       </c>
       <c r="H359" t="str">
         <v>일정 주기로 모의고사를 보는거 자체가 수능 준비에 큰 도움이 되었고 성적표에서 수능 예상등급까지 따로 분석해 주어서 내 위치를 정확히 파악할수 있어서 좋았고 또 재원생내에서 등수도 알려줘서 은근히 승부욕도 생겨 좋았었습니다</v>
@@ -13448,7 +13448,7 @@
         <v>N수생</v>
       </c>
       <c r="E361" t="str">
-        <v>이투스247을 다니면서 좋았던 점은 담임선생님과의 학습 상담이었습니다. 독학이다 보니까 방향을 잡는 게 어려웠는데, 상담하면서 제 상태를 정확하게 알 수 있어서 도움이 되었습니다.  그냥 열심히 하라고만 하는 게 아니라, 제 성적과 공부 습관을 보고 현실적으로 할 수 있는 계획을 같이 짜주셔서 좋았습니다. 그래서 막막할 때마다 다시 방향을 잡는 데 도움이 되었습니다.  또 분위기도 부담스럽지 않아서 편하게 질문하거나 고민을 말할 수 있었고, 그때마다 바로 피드백을 받을 수 있어서 좋았습니다. 혼자 공부하는데도 혼자 하는 느낌이 덜해서 계속 유지하는 데 도움이 되었습니다. 전체적으로 상담 덕분에 공부 방향이 덜 흔들렸고, 관리받는 느낌이 있어서 만족했습니다. 혼자 수험생활을 보내는 것에 부담이 있다면 이투스 247이 좋은 선택일 것 같습니다.</v>
+        <v>이투스247을 다니면서 좋았던 점은 담임 선생님과의 학습 상담이었습니다. 독학이다 보니까 방향을 잡는 게 어려웠는데, 상담하면서 제 상태를 정확하게 알 수 있어서 도움이 되었습니다.  그냥 열심히 하라고만 하는 게 아니라, 제 성적과 공부 습관을 보고 현실적으로 할 수 있는 계획을 같이 짜주셔서 좋았습니다. 그래서 막막할 때마다 다시 방향을 잡는 데 도움이 되었습니다.  또 분위기도 부담스럽지 않아서 편하게 질문하거나 고민을 말할 수 있었고, 그때마다 바로 피드백을 받을 수 있어서 좋았습니다. 혼자 공부하는데도 혼자 하는 느낌이 덜해서 계속 유지하는 데 도움이 되었습니다. 전체적으로 상담 덕분에 공부 방향이 덜 흔들렸고, 관리받는 느낌이 있어서 만족했습니다. 혼자 수험 생활을 보내는 것에 부담이 있다면 이투스 247이 좋은 선택일 것 같습니다.</v>
       </c>
       <c r="F361" t="str">
         <v>이투스247의 학습 계획이랑 플래너 관리도 도움이 많이 됐습니다. 혼자 하면 계획을 세워도 잘 안 지키게 되는 경우가 많은데, 여기서는 계속 체크를 받으니까 더 신경 쓰게 됐습니다. 처음에 계획을 세울 때도 무리하게 잡는 게 아니라, 실제로 지킬 수 있는 수준으로 맞춰서 짜주셔서 현실적으로 공부할 수 있었습니다. 그래서 중간에 포기하는 일이 줄어든 것 같습니다. 플래너도 그냥 쓰고 끝나는 게 아니라, 매일 점검을 받으니까 제가 얼마나 했는지 바로 확인할 수 있어서 좋았습니다. 계획 대비 얼마나 했는지도 보이니까 스스로 반성도 하게 되고, 다음 날 계획 세우는 데도 도움이 됐습니다. 전체적으로 계획 세우고 실행하는 흐름이 잡혀서, 혼자 공부할 때보다 훨씬 안정적으로 공부할 수 있었습니다. 무엇보다 플래너를 쓰고나서 끝인 게 아니고, 선생님께 확인 받아야한다는 생각에 더욱 잘 지킬 수 있었습니다.</v>
@@ -13460,7 +13460,7 @@
         <v>매일 일정한 시간에 단어 테스트를 보는 것도 좋았던 점이라고 생각합니다. 영어가 약한 편이라 단어를 외우는 게 항상 밀리거나 제대로 안 되는 경우가 많았는데, 매일 정해진 시간에 테스트를 보니까 어쩔 수 없이 계속 보게 되어서 도움이 됐습니다. 그냥 혼자 할 때는 미루게 되는 경우가 많았는데, 테스트가 있으니까 꾸준히 반복하게 되는 점이 좋았습니다.  또 한 번 보고 끝나는 게 아니라 틀린 단어를 다시 복습하게 되면서 자연스럽게 반복 학습이 되었습니다. 계속 같은 단어를 여러 번 보게 되니까 점점 익숙해지고, 예전보다 단어가 덜 부담스럽게 느껴졌습니다.  전체적으로 매일 단어 테스트를 통해 영어 공부를 꾸준히 이어갈 수 있었고, 약했던 부분을 조금씩 보완할 수 있어서 만족스러웠습니다.</v>
       </c>
       <c r="I361" t="str">
-        <v>데스크 선생님과 담임 선생님 모두 항상 웃는 얼굴로 대해주셔서 좋았습니다. 학원에 갈 때마다 밝게 인사해주시고 친절하게 대해주셔서 수험생활 중에 작은 부분이지만 힘이 많이 됐습니다. 혼자 공부하다 보면 지치거나 기분이 다운될 때가 많은데, 그런 분위기 덕분에 조금이나마 편하게 다닐 수 있었던 것 같습니다.  또 중간에 성적이 잘 안 나오거나 공부가 잘 안 풀려서 낙담할 때도 있었는데, 그럴 때마다 항상 응원해주시고 괜찮다고 말해주셔서 다시 마음 잡는 데 도움이 됐습니다. 단순한 관리만 하는 게 아니라 학생 입장에서 이해해주시고 말해주시는 느낌이 들어서 더 의지가 됐습니다.  전체적으로 공부 환경뿐만 아니라 사람적인 부분에서도 도움을 많이 받았고, 그런 점들이 수험생활을 버티는 데 큰 힘이 됐다고 생각합니다.</v>
+        <v>데스크 선생님과 담임 선생님 모두 항상 웃는 얼굴로 대해주셔서 좋았습니다. 학원에 갈 때마다 밝게 인사해주시고 친절하게 대해주셔서 수험 생활 중에 작은 부분이지만 힘이 많이 됐습니다. 혼자 공부하다 보면 지치거나 기분이 다운될 때가 많은데, 그런 분위기 덕분에 조금이나마 편하게 다닐 수 있었던 것 같습니다.  또 중간에 성적이 잘 안 나오거나 공부가 잘 안 풀려서 낙담할 때도 있었는데, 그럴 때마다 항상 응원해주시고 괜찮다고 말해주셔서 다시 마음 잡는 데 도움이 됐습니다. 단순한 관리만 하는 게 아니라 학생 입장에서 이해해주시고 말해주시는 느낌이 들어서 더 의지가 됐습니다.  전체적으로 공부 환경뿐만 아니라 사람적인 부분에서도 도움을 많이 받았고, 그런 점들이 수험 생활을 버티는 데 큰 힘이 됐다고 생각합니다.</v>
       </c>
       <c r="J361" t="str">
         <v>이투스247학원의 학습 계획이랑 플래너 관리도 도움이 많이 됐어요.</v>
@@ -13589,16 +13589,16 @@
         <v>N수생</v>
       </c>
       <c r="E364" t="str">
-        <v>처음 입소 당시 공부를 어디서부터 어떻게 해야하는지 막막했는데 선생님께서 잘 알려주시고 이끌어주셔서 공부 방향을 잡게되고 중간에 흐트러지지 않게 지도해주셔서 성적향상을 이룰 수 있어서 학습코칭 시스템이 유용했다고 생각합니다</v>
+        <v>처음 입소 당시 공부를 어디서부터 어떻게 해야하는지 막막했는데 선생님께서 잘 알려주시고 이끌어주셔서 공부 방향을 잡게되고 중간에 흐트러지지 않게 지도해주셔서 성적 향상을 이룰 수 있어서 학습코칭 시스템이 유용했다고 생각합니다</v>
       </c>
       <c r="F364" t="str">
-        <v>6,9모 학원 모의고사를 정기적으로 보고 지원가능대학 라인을 확인함으로써 적당한 긴장감과 도전의식을 가지며 공부할 수 있었다고 생각해서 이 학습관리 시스템이 유용했다고 생각이 되었습니다</v>
+        <v>6,9모 학원 모의고사를 정기적으로 보고 지원가능대학 라인을 확인함으로써 적당한 긴장감과 도전의식을 가지며 공부할 수 있었다고 생각해서 이 학습 관리 시스템이 유용했다고 생각이 되었습니다</v>
       </c>
       <c r="G364" t="str">
-        <v>휴대폰과 전자기기와의 차단을 통해서 오로지 잡생각 안 하고 학습에만 집중할 수 있어서 단기간에 성적향상도 이루고 멘탈관리도 되어서 전자기기 사용금지 시스템이 유용하다고 생각을 했습니다</v>
+        <v>휴대폰과 전자기기와의 차단을 통해서 오로지 잡생각 안 하고 학습에만 집중할 수 있어서 단기간에 성적 향상도 이루고 멘탈관리도 되어서 전자기기 사용금지 시스템이 유용하다고 생각을 했습니다</v>
       </c>
       <c r="H364" t="str">
-        <v>학원 내 모의고사를 봄으로써 내가 아는 것과 모르는 것 어중간하게 아는 것을 구분을 할 수 있어서 추후 학습 계획을 세우고 오답정리를 할 때 취약점을 빠르게 보완하고 성적향상을 이룰 수 있게 해줘서 원내 모의고사가 좋았습니다</v>
+        <v>학원 내 모의고사를 봄으로써 내가 아는 것과 모르는 것 어중간하게 아는 것을 구분을 할 수 있어서 추후 학습 계획을 세우고 오답정리를 할 때 취약점을 빠르게 보완하고 성적 향상을 이룰 수 있게 해줘서 원내 모의고사가 좋았습니다</v>
       </c>
       <c r="I364" t="str" xml:space="preserve">
         <v xml:space="preserve">2월부터 11월까지 잘 지도해주셔서 감사합니다 전역 후에 입시하느라 되게 막막하고 불안하고 했었는데 여기서 빡세게 공부해서 숭실대 잘 다니고 있어요_x000d_
@@ -13660,7 +13660,7 @@
         <v>반수생</v>
       </c>
       <c r="E366" t="str">
-        <v>제가 현역일 때 잘못된 공부법을 바로잡고 제대로 된 커리큘럼을 탈 수 있어서 좋았던 것 같습니다. 되게 체계적으로 공부한다는 기분이 들었고 어떻게 공부해야할지 막막했는데 딱딱 정해서 이만큼씩 하면 돼! 라고 해주시니까 편하게 커리큘럼에 대한 고민 없이 오로지 공부에만 집중할 수 있었던 것 같습니다.</v>
+        <v>제가 현역일 때 잘못된 공부법을 바로잡고 제대로 된 커리큘럼을 탈 수 있어서 좋았던 것 같습니다. 되게 체계적으로 공부한다는 기분이 들었고 어떻게 공부해야 할지 막막했는데 딱딱 정해서 이만큼씩 하면 돼! 라고 해주시니까 편하게 커리큘럼에 대한 고민 없이 오로지 공부에만 집중할 수 있었던 것 같습니다.</v>
       </c>
       <c r="F366" t="str">
         <v>주기적으로 공부하기 싫어지고 해이해지고 할 때 상담이 잡혀있다는 걸 생각하면 하루라도 미룰 수 없어서 꾸준히 공부하게 되어서 좋았습니다. 미루는 습관이 있었던 면이 없지 않아 있는데 상담을 되게 자주 하다 보니까 하루이틀 미루다 보면 상담 당일에 밀린 양을 감당할 수가 없게 되니까 꾸준히 공부하는 습관을 들일 수 있었던 것 같습니다.</v>
@@ -13696,7 +13696,7 @@
         <v>N수생</v>
       </c>
       <c r="E367" t="str">
-        <v>담임선생님을 배정하여 각자 어떤 방식으로 공부하는지 매주 확인하는 것이 좋은 시스템이었다고 생각합니다. 또한 3월, 6월, 9월 모의고사 뿐 아니라 대성 더프나 여러 사설 모의고사를 자주 실시하여 시험에 최적화된 시간을 계속해서 겪는 것이 좋았습니다.</v>
+        <v>담임 선생님을 배정하여 각자 어떤 방식으로 공부하는지 매주 확인하는 것이 좋은 시스템이었다고 생각합니다. 또한 3월, 6월, 9월 모의고사 뿐 아니라 대성 더프나 여러 사설 모의고사를 자주 실시하여 시험에 최적화된 시간을 계속해서 겪는 것이 좋았습니다.</v>
       </c>
       <c r="F367" t="str">
         <v>미리 선생님과의 질의응답을 예약하여 시간에 맞춰 모르는 부분을 언제든지 질문할 수 있는 부분이 좋았습니다. 또 각 과목마다 수업이 개설되어 나의 부족한 부분을 보충수업을 통해 채워나가는 프로그램이 있다는 것이 좋았습니다.</v>

</xml_diff>

<commit_message>
Apply extensive typo and spacing corrections
</commit_message>
<xml_diff>
--- a/reviews_with_keywords.xlsx
+++ b/reviews_with_keywords.xlsx
@@ -461,7 +461,7 @@
         <v>N수생</v>
       </c>
       <c r="E2" t="str">
-        <v>자신의 현재 점수대(3모,6모,9모 등)에 따라 할 수 있는, 해야하는 공부방법을 컨설팅해주는 것이 좋았다. 또한 목표 점수를 달성하기 위해 어떤 전략(어떤 유형의 문제를 풀 지, 실제 모고나 수능에서 어떻게 문제에 시간배분을 할 건지 등)을 세워 주는 점 또한 유용했다</v>
+        <v>자신의 현재 점수대(3모,6모,9모 등)에 따라 할 수 있는, 해야하는 공부 방법을 컨설팅해주는 것이 좋았다. 또한 목표 점수를 달성하기 위해 어떤 전략(어떤 유형의 문제를 풀 지, 실제 모고나 수능에서 어떻게 문제에 시간배분을 할 건지 등)을 세워 주는 점 또한 유용했다</v>
       </c>
       <c r="F2" t="str">
         <v>자신이 할 수 있는 현실적인 전략을 세워주는 점이 유용했다. 예를 들어, 수학의 경우, 무작정 N를 푸는 것이 아닌, 3점, 쉬운 4점  현실적으로 점수를 올릴 수 있는 전략을 세워주었다. 버릴 문제는 버리고, 챙길 문제는 챙기게 해 주는 점이 효율적이었다.</v>
@@ -714,7 +714,7 @@
         <v>모르는 부분을 바로바로 질문할 수 있어서  시간 낭비를 줄이고 효율적으로 공부할 수 있었던 점이 정말 좋았습니다. 조교 쌤들 다 너무 친절하게 기초부터 설명해주셔서 실력 향상에 정말 많은 도움이 되었습니다!</v>
       </c>
       <c r="G9" t="str">
-        <v>핸드폰 수거로 핸드폰을 확인하여 시간낭비하는 일이 줄어 공부에 더욱 집중 할 수 있어서 좋았습니다! 하루 목표 공부령을 채우는데 큰 도움이 되었고 공부에 집중하는 습관을 기르는데 가장 많은 도움이 된 것 같습니당</v>
+        <v>핸드폰 수거로 핸드폰을 확인하여 시간낭비하는 일이 줄어 공부에 더욱 집중할 수 있어서 좋았습니다! 하루 목표 공부령을 채우는데 큰 도움이 되었고 공부에 집중하는 습관을 기르는데 가장 많은 도움이 된 것 같습니당</v>
       </c>
       <c r="H9" t="str">
         <v>이투스 모의고사를 통해 현재 제 실력을 객관적으로 확인할 수 있어 좋았습니다. 응시하면서 부족한 부분을 체계적으로 파악하고 보완할 수 있어 학습 방향을 잡는 데 큰 도움이 되었고 모의고사 성적을 비롯한 상담을 통해 성적을 향상시킬 수 있었습니다!</v>
@@ -781,7 +781,7 @@
         <v>문제집을 풀면서 모르는 문제가 있을때 매번 답지만 보며 시간을 많이 썼는데 학습 상담을 통해서 시간을 효율적으로 쓸  수 있었고 이해하는데도 도움이 많이 되었습니다. 그리고 공부 커리큘럼을 어떻게 짜야할지 몰랐는데 학습 상담을 통해서 어떻게 공부해야 할지 감을 잡고 공부할 수 있었습니다.</v>
       </c>
       <c r="F11" t="str">
-        <v>보통 문제집을 풀면 강의가 없어 답지를 보고 문제를 혼자 이해했어야하는데 1:1로 질의 응답을 해주셔서 이해하는데 도움이 많이 되었습니다. 제가 모르는 부분을 더 집중적으로 자세하게 설명을 들을 수 있었고 못하는 부분을 보완하기 위해 무엇을 공부 해야하는지도 알 수 있어 좋았습니다.</v>
+        <v>보통 문제집을 풀면 강의가 없어 답지를 보고 문제를 혼자 이해했어야하는데 1:1로 질의 응답을 해주셔서 이해하는데 도움이 많이 되었습니다. 제가 모르는 부분을 더 집중적으로 자세하게 설명을 들을 수 있었고 못하는 부분을 보완하기 위해 무엇을 공부 해야 하는지도 알 수 있어 좋았습니다.</v>
       </c>
       <c r="G11" t="str">
         <v>일단 학원에 있으면 연락 알람 자체도 안오기때문에 공부에 집중하는데 정말 도움이 되었습니다. 또한 인강 사이트 외에는 인터넷이 안되서 강제로 공부할 수 있는 환경을 조성해주셔서 공부 하기에 정말 적합한 환경이였습니다.</v>
@@ -896,7 +896,7 @@
         <v>이투스 인강에서 국어, 사문 등 여러가지 강의를 보면서 도움이 되었던 거 같습니다. 다른 사이트에서 인강도 많이 봤지만 국어, 사문은 이투스 인강에서 더 도움을 많이 받은 거 같습니다.</v>
       </c>
       <c r="I14" t="str">
-        <v>1년 동안 제가 공부에 온전히 집중 할 수 있고, 다른 것에 신경 팔리지 않게 도움을 주셔서 정말 감사했습니다. 그 외에도 제가 힘들면 상담을 해주시고 저에게 방향성을 제시해 주셔서 감사했습니다</v>
+        <v>1년 동안 제가 공부에 온전히 집중할 수 있고, 다른 것에 신경 팔리지 않게 도움을 주셔서 정말 감사했습니다. 그 외에도 제가 힘들면 상담을 해주시고 저에게 방향성을 제시해 주셔서 감사했습니다</v>
       </c>
       <c r="J14" t="str">
         <v>제가 모의고사를 풀거나 공부를 하며 많은 스트레스를 받았을 때 담임 선생님께 상담을 받아 많은 도움이 되었던 거 같아요.</v>
@@ -1132,7 +1132,7 @@
         <v>고등학교 때 생각없이 공부하다가 마음에 들지 않는 대학에 진학하였고, 결국 반수를 결심하게 되었다. 한 학기동안은 홀로 계획을 짜 보고 이것저것 다양한 공부법을 시도해 봤지만 이게 효율적인 방법이 맞는지 알 수 없어 답답했다. 그러다가 이투스에 와서 본격적인 반수를 시작하고,담임 선생님과의 상담을 통해 현재 내가 해야하는 부분, 강점과 부족한 부분, 세세한 모의고사 피드백 등을 알 수 있어 만족스러웠다.</v>
       </c>
       <c r="F21" t="str">
-        <v>독학재수는 쉽지 않다. 이투스 등록 전까진 아무리 플래너를 그럴듯하게 써놔도 막상 달성률은 처참했다. 누군가 옆에서 잡아주고 감시해주는 사람이 없으니, 자기합리화를 계속 하며 미루고 미루다 결국 할 일이 엄청 불어났다. 그러나 학원에 오게 되면, 선생님들이 플래너를 매주 검사하신다. 현재 내가 모든 과목을 균형있게 골고루 공부하고 있는지, 계획이 너무 무리하진 않은지 플래너를 세세히 보시고 하나하나 피드백해 주신다. 덕분에 학원에 온 지 한 달만에 미루는 습관을 교정하게 될 수 있었다.</v>
+        <v>독학재수는 쉽지 않다. 이투스 등록 전까진 아무리 플래너를 그럴듯하게 써놔도 막상 달성률은 처참했다. 누군가 옆에서 잡아주고 감시해주는 사람이 없으니, 자기합리화를 계속 하며 미루고 미루다 결국 할 일이 엄청 불어났다. 그러나 학원에 오게 되면, 선생님들이 플래너를 매주 검사하신다. 현재 내가 모든 과목을 균형있게 고루 공부하고 있는지, 계획이 너무 무리하진 않은지 플래너를 세세히 보시고 하나하나 피드백해 주신다. 덕분에 학원에 온 지 한 달만에 미루는 습관을 교정하게 될 수 있었다.</v>
       </c>
       <c r="G21" t="str" xml:space="preserve">
         <v xml:space="preserve">나는 잠에 정말 약하다. 고3 때 모의고사를 볼 때도 몽롱한 정신으로 풀었고, 아침잠이 너무 많은 탓에 결국 현역 수능 1교시 시작 직전까지 하품을 쩍쩍 하다 결국 처참한 국어 성적을 받았다. 학원에 온 이후로는 선생님들께서 졸음 관리를 해 주셔서 좋았다. 항상 공부를 할 땐 나도 모르는 사이 꾸벅꾸벅 졸곤 했었는데, 그럴 때 마다 감독 선생님들께서 안마봉으로 깨워주셨다._x000d_
@@ -1164,7 +1164,7 @@
 이투스 대구달서점 화이팅~~</v>
       </c>
       <c r="J21" t="str">
-        <v>내가 모든 과목을 균형있게 골고루 공부하고 있는지, 너무 무리하진 않은지 플래너를 세세히 보시고 하나하나 피드백해 주셨어요.</v>
+        <v>내가 모든 과목을 균형있게 고루 공부하고 있는지, 너무 무리하진 않은지 플래너를 세세히 보시고 하나하나 피드백해 주셨어요.</v>
       </c>
       <c r="K21" t="str">
         <v/>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="E28" t="str" xml:space="preserve">
         <v xml:space="preserve">아이에 성향 파악도 원장님 께서 빠르시고 상황에 맞는 최선의 입시 전략을 코칭해 주셔서 좋았습니다._x000d_
-스트레스 없이 아이가 입시 공부에만 집중 할 수 있는 분위기 조성도 잘 해주신것 같습니다.</v>
+스트레스 없이 아이가 입시 공부에만 집중할 수 있는 분위기 조성도 잘 해주신것 같습니다.</v>
       </c>
       <c r="F28" t="str">
         <v>일대일 코칭 선생님께서 부족한 부분을 잘 파악 하시고 점수를 올리기 위해서 추가로 공부 해야 할 부분들을 잘 코칭해 주셨고 실제로 성적 향상이 되었습니다 . 또한 따뜻한 격려의 말씀도 너무 감사하고 도움이 많이 되었습니다</v>
@@ -1439,7 +1439,7 @@
         <v>성적이 낮은 과목이 있었는데 저에게 알맞은  강의를 추천해 주셔서 많이 도움이 되었습니다 모의고사 성적표가 나올때마다 어떤 과목 중심으로 공부해야 효율적일지 같이 고민하고 상담해주셔서 좋았습니다</v>
       </c>
       <c r="F29" t="str">
-        <v>매일 플래너를 쓰니까 계획적으로 학습을 할수 있어서 좋았습니다.  플래너를 쓰지 않았을때보다 더 체계적이고 효율적으로 공부할 수 있었습니다. 매일 플래너를 쓰다보니 습관이 되어서 공부 계획을 잘 세우게되었습니다</v>
+        <v>매일 플래너를 쓰니까 계획적으로 학습을 할수 있어서 좋았습니다.  플래너를 쓰지 않았을 때보다 더 체계적이고 효율적으로 공부할 수 있었습니다. 매일 플래너를 쓰다보니 습관이 되어서 공부 계획을 잘 세우게되었습니다</v>
       </c>
       <c r="G29" t="str">
         <v>혼자 공부하면 5분만 눈을 붙인다는 게 1시간이 되기 일쑤인데 선생님이 주기적으로 순회하며 즉각 깨워주니 흐름이 끊기지 않았습니다. 졸음이 확산되기 전에 차단해주는 강제성이 가장 큰 장점이었습니다</v>
@@ -1451,7 +1451,7 @@
         <v>선생님 1년정도의 기간동안 잘 코칭해주셔서 정말 감사했습니다ㅎㅎ 덕분에 수험기간 잘 버텨낼수 있었어용! 쌤덕분에 수능때 영어도 3등급 받아냈어요~~ 앞으로 행복하세요!! 독서도 열심히 할게요</v>
       </c>
       <c r="J29" t="str">
-        <v>플래너를 쓰지 않았을때보다 더 체계적이고 효율적으로 공부할 수 있었어요.</v>
+        <v>플래너를 쓰지 않았을 때보다 더 체계적이고 효율적으로 공부할 수 있었어요.</v>
       </c>
       <c r="K29" t="str">
         <v/>
@@ -1510,7 +1510,7 @@
         <v>일주일에 한 번씩 상담을 했는데 지금까지 얼마나 진도를 나갔는지 말씀드리고 하루에 이정도는 해야 진도를 다 끝낼수있고 마무리할 수 있다 이렇게 도움을 주셔서 학습에 큰 도움이 됐습니다 하다보니 진도 나가는 시간도 빨라졌고 공부하는 데에 엄청 도움이 됐습니다 또 상담시간 아니여도 질문을 할 수 있는데 평소에도 선생님이 계시고 질문을 많이 할수있어서 학습에 큰 도움이 됐습니다</v>
       </c>
       <c r="F31" t="str">
-        <v>일단 모의고사를 주기적으로 정말 많이 봤습니다 평가원 뿐만 아니라 사설 모의고사도 많이 봤는데 볼 때마다 성적이 어느정도 나오는지 어느 학교가 적정인지 알려주는 그래프와 수치를 맨날 받았습니다 그걸 보고 어떤 과목이 부족했고 더 열심히해야하는지 알 수 있어서 도움이 됐어요</v>
+        <v>일단 모의고사를 주기적으로 정말 많이 봤습니다 평가원 뿐만 아니라 사설 모의고사도 많이 봤는데 볼 때마다 성적이 어느정도 나오는지 어느 학교가 적정인지 알려주는 그래프와 수치를 맨날 받았습니다 그걸 보고 어떤 과목이 부족했고 더 열심히해야 하는지 알 수 있어서 도움이 됐어요</v>
       </c>
       <c r="G31" t="str">
         <v>공부를 하다보면 당연히 딴 짓을 하고 싶은데 선생님들이 주기적으로 돌아다니면서 출석 체크하시고 조는 아이들이 있으면 깨워주시고 이런 분위기 덕분에 더 공부에 집중하려고 노력했던 거 같고 실제로 공부가 잘 되어서 유용했습니다</v>
@@ -1620,7 +1620,7 @@
         <v>신뢰할 수 있는 대학생 멘토쌤과 언제든지 1:1 질의응답을 할 수 있는게 되게 유용했습니다. 문제에 관한 질문뿐만 아니라 학습법, 학습방향, 선택과목 설정 등 공부 고민에 대한 질문도 할 수 있다는게 좋았습니다. 실제로 6모 후 선택과목을 바꿀때 많은 도움이 되었고 그 외 걱정거리 또한 멘토샘들이 친절하게 상담해주셔서 많이 도움 받았습니다. 수험생이라면 1년 동안 공부 고민이 많을텐데 그때 1:1 질의응답을 이용해도 유용할 것 같습니다</v>
       </c>
       <c r="G34" t="str" xml:space="preserve">
-        <v xml:space="preserve">혼자 공부할때 가장 힘든게 핸드폰, 태블릿 사용인데 학원에서 관리해주니 정말 좋았습니다. 공부 할때 내내 감시받는 기분이라 딴짓은 절대 못하고 _x000d_
+        <v xml:space="preserve">혼자 공부할때 가장 힘든게 핸드폰, 태블릿 사용인데 학원에서 관리해주니 정말 좋았습니다. 공부할때 내내 감시받는 기분이라 딴짓은 절대 못하고 _x000d_
 공부에만 몰입할 수 있어 많이 유용하였습니다. 전자기기 사용 욕구 또한 많이 줄어들어 학원이 끝나고도, 일상생활에서도 전자기기에 의존하지 않을 수 있게 되었습니다.</v>
       </c>
       <c r="H34" t="str">
@@ -1651,10 +1651,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E35" t="str">
-        <v>수능과목중 내가 어떤 과목에 강점이 있는지, 내가 어떤 과목이 약점이고 왜 이 과목을 해야하는지에 대하여 상세히 알려주고 공부법을 알려줬었는데 2학년때 모의로 해봤던 것에 비해 등급이 한 두 단계 올라갔고 그 덕분인지 대학에 합격할 수 있었습니다.</v>
+        <v>수능과목중 내가 어떤 과목에 강점이 있는지, 내가 어떤 과목이 약점이고 왜 이 과목을 해야 하는지에 대하여 상세히 알려주고 공부법을 알려줬었는데 2학년때 모의로 해봤던 것에 비해 등급이 한 두 단계 올라갔고 그 덕분인지 대학에 합격할 수 있었습니다.</v>
       </c>
       <c r="F35" t="str">
-        <v>수능 과목이 여러개이기도하고 이곳에 들어오기 전까지 학습방법이나 어떤 과목을 해야하는지 조차도 정해져있지 않았기 때문에 도움이 절실했는데 쥐약이던 수학과 국어를 어떻게 하면 더 효율적으로 성적을 올릴 수 있는지와 공부하는 방법을 제대로 디렉팅하고 그 방향대로 할 수 있게 지도해주셨습니다.</v>
+        <v>수능 과목이 여러개이기도하고 이곳에 들어오기 전까지 학습방법이나 어떤 과목을 해야 하는지 조차도 정해져있지 않았기 때문에 도움이 절실했는데 쥐약이던 수학과 국어를 어떻게 하면 더 효율적으로 성적을 올릴 수 있는지와 공부하는 방법을 제대로 디렉팅하고 그 방향대로 할 수 있게 지도해주셨습니다.</v>
       </c>
       <c r="G35" t="str">
         <v>딴짓 할 생각이 들어도 어차피 못하게 막아놓다 보니깐 처음엔 너무 짜증났었는데 다들 패드나 노트북이 있어도 이 방화벽 때문에 전부 공부를 하고있는데 나 혼자 그냥 적당히 하는 시늉을 하고있으니깐 너무 별로인거 같았습니다. 그래서 더욱 공부에 힘을 썼고 폰이나 인터넷은 하원한 뒤 자기 전에 잠깐하거나 주말에 2시간까지만 했습니다. 솔직히 이런게 없으면 공부할 환경 자체가 만들어지지 않기에 더더욱 좋았던거 같습니다.</v>
@@ -1793,7 +1793,7 @@
         <v>N수생</v>
       </c>
       <c r="E39" t="str">
-        <v>우선 저는 수능이라는 시험을 제대로 준비해본적이 없어서 처음에 많리 힘들었습니다. 계획짜는 방법이나 공부방법을 잘 몰랐어서 힘들었지만 선생님들의 조언과 말씀들 덕분에 공부를 어떻게 해야하는지 알게 되었습니다.</v>
+        <v>우선 저는 수능이라는 시험을 제대로 준비해본적이 없어서 처음에 많리 힘들었습니다. 계획짜는 방법이나 공부 방법을 잘 몰랐어서 힘들었지만 선생님들의 조언과 말씀들 덕분에 공부를 어떻게 해야 하는지 알게 되었습니다.</v>
       </c>
       <c r="F39" t="str">
         <v>앞서 말씀했듯이 저는 계획하는 방법을 모르고 있었습니다. 선생님께서 전과목의 시간 계산이나 과목을 언제 어떻게 하루에 얼마나 해야하는 양과 정확하게 가르쳐주셨습니다. 저는 그걸 피드백으로 생각하고 똑같이 병행해보았습니다.</v>
@@ -1809,7 +1809,7 @@
         <v>안녕하세요 선생님! 이투스 학원을 다니면서 매번 감사했습니다. 형편없는 제 실력을 탓하지 않고 끝까지 응원해주셔서 감사합니다 비록 학교는 좋은 곳, 원하던 곳을 가지 않았지만 수능이라는 것을 제대로 준비해본 적이 없었는데 선생님들 덕분에 좋은 부분들 많이 배워갑니다!  정말 감사했습니다</v>
       </c>
       <c r="J39" t="str">
-        <v>계획 짜는 방법이나 공부 방법을 잘 몰라서 힘들었지만 선생님들의 조언과 말씀들 덕분에 공부를 어떻게 해야하는지 알게 되었어요.</v>
+        <v>계획 짜는 방법이나 공부 방법을 잘 몰라서 힘들었지만 선생님들의 조언과 말씀들 덕분에 공부를 어떻게 해야 하는지 알게 되었어요.</v>
       </c>
       <c r="K39" t="str">
         <v/>
@@ -2043,7 +2043,7 @@
   저 같은 경우는 아쉽게도 끝까지 완수하지 못하였지만 다른 학생들 같은 경우 선생님들 덕분에 힘든 수험 생활을 넘길수도 있는 분도 있을겁니다.</v>
       </c>
       <c r="F46" t="str">
-        <v>수험생의 상태를 성적뿐 아니라 그 이외의 것 들도 수험 생활에 집중 할 수 있도록 상담해주십니다. 건강이 좋지 않아도 한 번은 이투스247학원에서 수험 생활을 노력해볼수 있을 거라고 생각합니다.</v>
+        <v>수험생의 상태를 성적뿐 아니라 그 이외의 것 들도 수험 생활에 집중할 수 있도록 상담해주십니다. 건강이 좋지 않아도 한 번은 이투스247학원에서 수험 생활을 노력해볼수 있을 거라고 생각합니다.</v>
       </c>
       <c r="G46" t="str">
         <v>솔직히 방금 네가지 선택지 다 별로였는데 와이파이 방화벽은 비교적 도움이 돼었지만, 핸드폰 반납같은 경우 혼자서 수험 생활을 준비하는 학생의 경우 꽤 불편합니다.  학원 와서도 핸드폰으로 딴짓 하면 그것은 개인의 의지 문제이고 선생님들이 관리도 하시니 이 부분은 추후에 더 효율적으로 관리되었으면 합니다.</v>
@@ -2055,7 +2055,7 @@
         <v>몸도 마음도 힘들었지만 재원하는동안 사정봐주시고 신경 써주셔서 너무 감사합니다. 저 같은 수험생은 보지않고 싶으실것 같습니다. 그래도 신경써주셔서 그나마 덜 힘들었습니다. 학생 개개인 별로 사정을 파악하고 조치를 취하시는게 어려울것 같습니다만 그렇게 해주셔서 감사합니다</v>
       </c>
       <c r="J46" t="str">
-        <v>성적뿐만 아니라 그 이외의 것 들도 수험 생활에 집중 할 수 있도록 상담해주셨어요.</v>
+        <v>성적뿐만 아니라 그 이외의 것 들도 수험 생활에 집중할 수 있도록 상담해주셨어요.</v>
       </c>
       <c r="K46" t="str">
         <v/>
@@ -2661,7 +2661,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E63" t="str">
-        <v>과목별로 바로바로 질문을 해결할 수 있었으며 과목별 공부방법에 대해 꿀팁을 얻을 수 있다. 모으고사 틀린문제를 직접 분석해주시며 개인별 부족한점과 보완할점을 각각 알려주셔 성적 향상에 큰 도움이 되었다</v>
+        <v>과목별로 바로바로 질문을 해결할 수 있었으며 과목별 공부 방법에 대해 꿀팁을 얻을 수 있다. 모으고사 틀린문제를 직접 분석해주시며 개인별 부족한점과 보완할점을 각각 알려주셔 성적 향상에 큰 도움이 되었다</v>
       </c>
       <c r="F63" t="str">
         <v>취약한 부분에 대해 알 수 있고, 입시라는 현실에 부딪히게 해주어서 과목 편식과 같은 습관들로부터 벗어날 수 있었다 또한 나의 문제점을 바로 확인할 수 있었다. 질문을 바로 해결할 수 있다.</v>
@@ -2837,10 +2837,10 @@
         <v>반수생</v>
       </c>
       <c r="E68" t="str">
-        <v>수능을 다시 준비하면서 내가 가지고 있던 안 좋은 습관이나 공부방법을 상담을 통해 개선시킬 수 있었다. 특히 취침시간과 기상시간에서 문제가 많이 있었는데 이투스 학원을 통해 그러한 단점들을 극복하고 개선시킬 수 있었다. 학생들과 함께 유대감을 쌓으면서 생활측면에서 많은 도움이 되었다.</v>
+        <v>수능을 다시 준비하면서 내가 가지고 있던 안 좋은 습관이나 공부 방법을 상담을 통해 개선시킬 수 있었다. 특히 취침시간과 기상시간에서 문제가 많이 있었는데 이투스 학원을 통해 그러한 단점들을 극복하고 개선시킬 수 있었다. 학생들과 함께 유대감을 쌓으면서 생활측면에서 많은 도움이 되었다.</v>
       </c>
       <c r="F68" t="str">
-        <v>현재 내가 실시하고 있는 공부방법이 나에게 적절한지, 내 생활패턴이 실력향상 및 점수에 좋은 영향이 있는지 분석하여 앞으로의 내가 어떤 식으로 공부하고 생활할지 방향성을 제시받을 수 있었다는 점에서 좋았다. 이런 데이터 분석을 통해 많은 학갱들이 도움받았을 것이다.</v>
+        <v>현재 내가 실시하고 있는 공부 방법이 나에게 적절한지, 내 생활 패턴이 실력향상 및 점수에 좋은 영향이 있는지 분석하여 앞으로의 내가 어떤 식으로 공부하고 생활할지 방향성을 제시받을 수 있었다는 점에서 좋았다. 이런 데이터 분석을 통해 많은 학갱들이 도움받았을 것이다.</v>
       </c>
       <c r="G68" t="str">
         <v>면학 분위기를 체계적으로 조성해 주어 자연스럽게 집중력이 높아졌고, 주변 학생들도 모두 공부에 몰입하고 있어 흐름을 따라가기 쉬웠습니다. 또한 일정한 시간마다 환기를 유도하고, 좌석 관리와 순찰을 통해 졸음을 방지해 주어 장시간 공부에도 효율을 유지할 수 있었습니다. 이런 생활 관리 시스템 덕분에 학습 습관이 규칙적으로 잡히고 성과 향상에 큰 도움이 되었습니다.</v>
@@ -2907,7 +2907,7 @@
         <v>반수생</v>
       </c>
       <c r="E70" t="str">
-        <v>아침 기상 시간을 맞춰 매우 효율적으로 움직일 수 있는 점이 좋았습니다. 6시반에 기상하여 7시50분까지 착석하면 되는 일정이었으나 아침 산책 및 간단한 식사 후 7시까지 자리에 앉아 아침 공부를 하며 루틴을 만들어 생활패턴을 지킬 수 있다는 점이 가장 좋았습니다.</v>
+        <v>아침 기상 시간을 맞춰 매우 효율적으로 움직일 수 있는 점이 좋았습니다. 6시반에 기상하여 7시50분까지 착석하면 되는 일정이었으나 아침 산책 및 간단한 식사 후 7시까지 자리에 앉아 아침 공부를 하며 루틴을 만들어 생활 패턴을 지킬 수 있다는 점이 가장 좋았습니다.</v>
       </c>
       <c r="F70" t="str">
         <v>학습에 관해 고민이 있거나 번아웃이 오면 담임 선생님께 편하게 질문, 상담한 것이 좋았습니다. 기숙이라는 답답할 수 있는 공간에서 털어놓을 수 있어 힘든 순간이 와도 다시 마음을 다잡을 수 있었던 것 같습니다.</v>
@@ -3102,7 +3102,7 @@
         <v>고2 올라가는 겨울방학 때 이투스를 다니면서 도움을 많이 받았습니다. 특히 조교 선생님분들 덕분에 해이해질 수 있는 시기에 동기부여도 받고 두달동안 무너지않았던 것 같습니다. 감사합니다.</v>
       </c>
       <c r="J75" t="str">
-        <v>규치적인 오전 시간 영단어 시험 덕분에 취약했던 영어 실력을 향상시킬 수 있었어요.</v>
+        <v>규칙적인 오전 시간 영단어 시험 덕분에 취약했던 영어 실력을 향상시킬 수 있었어요.</v>
       </c>
       <c r="K75" t="str">
         <v/>
@@ -3198,7 +3198,7 @@
       <c r="E78" t="str" xml:space="preserve">
         <v xml:space="preserve">체계적인 관리와 적극적인 상담시도로_x000d_
 입시생활 기간동안 고민이 발생했을 때 _x000d_
-언제나 부담없이 가서 담임 선생님과 상담할 수 있던 부분이 가장 크게 도움된 것 같아요. 또한 적극적인 관심 덕분에 다른 사설 상담업체 방문이 필요없었고 매상황마다 적절하고 적합한 조언이 크게 도움 됐어요</v>
+언제나 부담 없이 가서 담임 선생님과 상담할 수 있던 부분이 가장 크게 도움된 것 같아요. 또한 적극적인 관심 덕분에 다른 사설 상담업체 방문이 필요없었고 매상황마다 적절하고 적합한 조언이 크게 도움 됐어요</v>
       </c>
       <c r="F78" t="str" xml:space="preserve">
         <v xml:space="preserve">매일매일 내가 학습한 공부량을 확인할 수 있어 좋았고 내가 공부한 부분을 정리함으로써 한번 더 상기된 것 같다_x000d_
@@ -3214,7 +3214,7 @@
         <v>선생님께서 늘 따뜻하게 지도해 주시고, 이해할 때까지 친절하게 설명해 주셔서 감사드립니다. 덕분에 학습에 대한 자신감이 생겼고 성적도 많이 향상되었습니다. 앞으로도 배운 내용을 바탕으로 더욱 노력하겠습니다.</v>
       </c>
       <c r="J78" t="str">
-        <v>언제나 부담없이 가서 담임 선생님과 상담할 수 있던 부분이 가장 크게 도움된 것 같아요.</v>
+        <v>언제나 부담 없이 가서 담임 선생님과 상담할 수 있던 부분이 가장 크게 도움된 것 같아요.</v>
       </c>
       <c r="K78" t="str">
         <v/>
@@ -3506,7 +3506,7 @@
         <v>이투스 모고 꽤나 도움 됐어요. 현장감 유지랑 전략 실현에 좋았어요! 일단 현장감을 지속적으로 유지해볼 수 있어서 달마다 수능 때도 큰 긴장감 없이 잘 볼 수 있게 된 것 같았어요. 그리고 전략을 수정해서 젤 잘 맞는 순서로 문제를  풀 수 있게 되었어요</v>
       </c>
       <c r="I86" t="str">
-        <v>그동안 친절하게 가르쳐주셔서 감사합니다! 덕분에 힘애서 공부 할 수 있었고, 뿌듯한 수능 전 3달을 보낼 수 있었습니다! 그리고 항상 웃음으로 대해주셔서 힘든 반수생 생활이 덕분에 덜 힘들었어요! 감사해요!!!</v>
+        <v>그동안 친절하게 가르쳐주셔서 감사합니다! 덕분에 힘애서 공부할 수 있었고, 뿌듯한 수능 전 3달을 보낼 수 있었습니다! 그리고 항상 웃음으로 대해주셔서 힘든 반수생 생활이 덕분에 덜 힘들었어요! 감사해요!!!</v>
       </c>
       <c r="J86" t="str">
         <v>항상 웃음으로 대해주셔서 힘든 반수생 생활이 덕분에 덜 힘들었어요.</v>
@@ -3758,7 +3758,7 @@
         <v>항상 좋은 말씀 해주서서 감사했습니다. 중간중간에 이벤트도 힘써주셔서 엄청 큰 도움이 되었어요. 또 철저한 출걸관리 덕분에 아침에 지각하는 횟수를 줄일 수 있었습니다. 감사합니다.</v>
       </c>
       <c r="J93" t="str">
-        <v>저도 모르게 한 과목에만 너무 집중하게 되었는데, 선생님의 피드백으로 균형있는 학습을 할 수 있었어요.</v>
+        <v>저도 모르게 한 과목에만 너무 집중하게 되었는데, 선생님의 피드백으로 균형 있는 학습을 할 수 있었어요.</v>
       </c>
       <c r="K93" t="str">
         <v/>
@@ -3828,7 +3828,7 @@
         <v>1년 동안 관리해주셔서 감사합니다 이투스덕분에 많은것을 얻고 가는것 같네요 비록 이번 수능은 실패로 끝났지만 여기서 얻은 경험을 바탕으로 마지막 수험 생활 제대로 끝마치겠습니다 감사합니다</v>
       </c>
       <c r="J95" t="str">
-        <v>담임 선생님께서 수면 시간 조절하는 방법에 도움을 주셔서 생활 리듬을 바로 잡아 공부의 질과 양이 높아졌어요.</v>
+        <v>담임 선생님께서 수면 시간 조절하는 방법에 도움을 주셔서 생활 리듬을 바로잡아 공부의 질과 양이 높아졌어요.</v>
       </c>
       <c r="K95" t="str">
         <v/>
@@ -4107,7 +4107,7 @@
         <v>N수생</v>
       </c>
       <c r="E103" t="str">
-        <v>자기 주도 학습을 위해 자습시간을 어떻게 더 효율적으로 활용할 지 고민이 많았는데 담당 담임 선생님과의 상담을 통해 과목별 시간 배분을 어떻게 할지와 취약 과목에 대한 공부방법 등 전체적인 공부 습관을 형성하는 것에 도움을 많이 받았습니다.</v>
+        <v>자기 주도 학습을 위해 자습시간을 어떻게 더 효율적으로 활용할 지 고민이 많았는데 담당 담임 선생님과의 상담을 통해 과목별 시간 배분을 어떻게 할지와 취약 과목에 대한 공부 방법 등 전체적인 공부 습관을 형성하는 것에 도움을 많이 받았습니다.</v>
       </c>
       <c r="F103" t="str">
         <v>학습 계획 설정과 플래너 관리에서 공부 습관이 형성되어 있지 않을 때에 하루에 어떻게 공부를 하고 어느정도의 양을 소화할 수 있는지 확인하고 앞으로의 학습을 위해 효율적인 계획을 세울 수 있도록 스스로 훈련할 수 있었습니다.</v>
@@ -4122,7 +4122,7 @@
         <v>학습 습관 형성 및 성적 향상을 위한 여러 지도 감사드립니다. 덕분에 전년도와는 다른 공부 습관 및 방법들을 터득하고 이를 통해 성적 향상 뿐만 아니라 앞으로의 공부에 도움이 많이 될만한 것들을 얻어갈 수 있었습니다.</v>
       </c>
       <c r="J103" t="str">
-        <v>학습 습관 형성 및 성적 향상을 위한 여러 지도 감사드립다.</v>
+        <v>학습 습관 형성 및 성적 향상을 위한 여러 지도 감사드립니다.</v>
       </c>
       <c r="K103" t="str">
         <v/>
@@ -4142,7 +4142,7 @@
         <v>N수생</v>
       </c>
       <c r="E104" t="str">
-        <v>어떤 선생님꺼 들어야하는지 어떻게공부해야하는지 혼자 고민을 많이하다가 상담하면 어떤 강의를 들어야하는지 어떻게 공부해야하는지 같이 고민해주시고 꿀팁도주시고 알려주셔서 많은 도움이되었고 유용했음</v>
+        <v>어떤 선생님꺼 들어야하는지 어떻게공부해야 하는지 혼자 고민을 많이하다가 상담하면 어떤 강의를 들어야하는지 어떻게 공부해야 하는지 같이 고민해주시고 꿀팁도주시고 알려주셔서 많은 도움이되었고 유용했음</v>
       </c>
       <c r="F104" t="str">
         <v>공부하다가 해설을 봐도 헷갈리거나 이해가안되거나 모르는 문제가있으면 바로 가져가서 물어보면 친절하게 알려주셔서 빠르고 쉽게 이해할수있고 이해못하면어떡하나 이런 심적 부담감이 없었던게 좋았다</v>
@@ -4180,7 +4180,7 @@
         <v>선생님께서 매일 종례를 하셨는데 그때 학생들의 상태를 확인하시고 항상 명언과 같은 동기부여의 말, 응원의 말을 해주셔서 정신적으로 도움을 받았습니다. 학생들을 정말 진심으로 아끼시는 분이 담임이라 버틸 수 있었습니다.</v>
       </c>
       <c r="F105" t="str">
-        <v>어느 부분을 더 집중적으로 보완해야하는지 콕 찝어서 말씀해주셔서 부족한 점을 채울 수 있었습니다. 혼자서라면 무엇을 해야 할지 막막했을텐데 선생님과 상의할  수 있었다는게 큰 도움이 되었습니다.</v>
+        <v>어느 부분을 더 집중적으로 보완해야 하는지 콕 찝어서 말씀해주셔서 부족한 점을 채울 수 있었습니다. 혼자서라면 무엇을 해야 할지 막막했을텐데 선생님과 상의할  수 있었다는게 큰 도움이 되었습니다.</v>
       </c>
       <c r="G105" t="str">
         <v>기숙학원에선 주변 사람들이 자신의 목표를 위해 열심히 노력하는 모습을 보고 포기하고 싶을 때마다 다시 힘을 낼 수 있었습니다. 혼자하면 쉽게 흐트러졌을거같은데 다 같이 열심히 하는 분위기가 좋았습니다.</v>
@@ -4212,7 +4212,7 @@
         <v>N수생</v>
       </c>
       <c r="E106" t="str" xml:space="preserve">
-        <v xml:space="preserve">담임쌤이랑 매주 한 번씩 공부방법,피드백,고쳐야 할점 등등 학습에 도움되는 이야기를 할 수 있어서 좋았고_x000d_
+        <v xml:space="preserve">담임쌤이랑 매주 한 번씩 공부 방법,피드백, 고쳐야 할 점 등등 학습에 도움되는 이야기를 할 수 있어서 좋았고_x000d_
 큐엔에이도 과목마다 다양한 선생님들이랑 당일날에 바로바로 대면으로 해결할수있어서 좋있습니다</v>
       </c>
       <c r="F106" t="str" xml:space="preserve">
@@ -4233,7 +4233,7 @@
 모두 감사했고 수고하셨습니다</v>
       </c>
       <c r="J106" t="str">
-        <v>담임 선생님과 매주 공부방법,피드백,고쳐야 할점 등 학습에 도움되는 이야기를 할 수 있어서 좋았어요.</v>
+        <v>담임 선생님과 매주 공부 방법,피드백, 고쳐야 할 점 등 학습에 도움되는 이야기를 할 수 있어서 좋았어요.</v>
       </c>
       <c r="K106" t="str">
         <v/>
@@ -4365,7 +4365,7 @@
         <v>어떤 인강이 좋을지 어떤 교재가 좋을지 내 수준에 딱 맞고 지금 나에게 필요한게 무엇인지 처음 공부를 시작할때 무척 막막하였는데 학원 상담을 통해 하나하나 어디서 부터 시작하고 어떤 인강과 교재로 학습을 하면 좋을지 코치받아서 학습의 기본 토대가 만들어져서 유용했습니다.</v>
       </c>
       <c r="G110" t="str">
-        <v>평소에 잠이 많고 집중을 잘 못했었는데, 면학 분위기 감독과 졸음 관리 덕분에 공부에 더 집중 할 수 있었고 그 덕분에 엉덩이 힘도 더 좋아지며 공부하는 습관이 잘 잡혀나간 점에서 매우 유용하였습니다.</v>
+        <v>평소에 잠이 많고 집중을 잘 못했었는데, 면학 분위기 감독과 졸음 관리 덕분에 공부에 더 집중할 수 있었고 그 덕분에 엉덩이 힘도 더 좋아지며 공부하는 습관이 잘 잡혀나간 점에서 매우 유용하였습니다.</v>
       </c>
       <c r="H110" t="str">
         <v>평소에 의지박약으로 단어를 외웠다가 안외웠다가 갈팡질팡 공부했었는데 학원을 다니면서 의무적으로 매일 아침마다 보는 단어시험으로 비몽사몽한 뇌를 깨우는 데에도 매우 도움이되었고 단어도 처음으로 꾸준히 암기 할 수 있었던 부분에서 매우 유용했습니다.</v>
@@ -4609,7 +4609,7 @@
         <v>N수생</v>
       </c>
       <c r="E117" t="str">
-        <v>매주 학습 플래너와 공부 계획을 점검 및 피드백 해주셨고 과목별 고민이나 공부방법, 커리큘럼 추천도 해주셨고 무엇보다 모의고사 응시 후 모의고사 관련 피드백이 매우 유용했던 것 같습니다.</v>
+        <v>매주 학습 플래너와 공부 계획을 점검 및 피드백 해주셨고 과목별 고민이나 공부 방법, 커리큘럼 추천도 해주셨고 무엇보다 모의고사 응시 후 모의고사 관련 피드백이 매우 유용했던 것 같습니다.</v>
       </c>
       <c r="F117" t="str">
         <v>앞서 말했던것 처럼 매주 과목별로 공부량이나 공부 방법등을 피드백 해주시고 과목별 고민이나 모의고사 운영 전략, 시간 관리 등등 실전적인 부분도 도움울 주셨던 점이 많이 도움이 되었던것 같습니다.</v>
@@ -4644,7 +4644,7 @@
         <v>N수생</v>
       </c>
       <c r="E118" t="str">
-        <v>어떻게 공부해야하고 무슨 책을 공부하고 어떤 단계를 해야하는지 인강은 누구를 들어야하는지 혼자 할 때는 잘 몰랐는데 중간중간 상담하면서 잘못된 건 바로 잡아주시고 올바른 공부 방향성을 잡아주셔서 좋았다</v>
+        <v>어떻게 공부해야하고 무슨 책을 공부하고 어떤 단계를 해야 하는지 인강은 누구를 들어야하는지 혼자 할 때는 잘 몰랐는데 중간중간 상담하면서 잘못된 건 바로잡아주시고 올바른 공부 방향성을 잡아주셔서 좋았다</v>
       </c>
       <c r="F118" t="str" xml:space="preserve">
         <v xml:space="preserve">강의마다 수준이 달라서 들을 수 있는 게 있고 없는 게 있는데 혼자 할 때는 잘 몰라서 그냥 1타 강사 것만 찾아서 들었다_x000d_
@@ -4657,7 +4657,7 @@
         <v>이투스 모의고사를 보면서 나의 실력을 체크할 수 있고 어려워하는 부분이나 잘 모르는 부분을 체크할 수 있으며 어느부분이 부족한지 파악하고 그 부분을 중점적으로 공부할 수 있도록 도와준 것 같다</v>
       </c>
       <c r="I118" t="str" xml:space="preserve">
-        <v xml:space="preserve">삭막한 재수 생활에 원장님과 실장님들이 친근하게 말 걸어주셔서 너무 감사했어요 그리고 한 번도 가져본 적 없던 규칙적인 생활패턴이 생겨서 너무 도움됐어요_x000d_
+        <v xml:space="preserve">삭막한 재수 생활에 원장님과 실장님들이 친근하게 말 걸어주셔서 너무 감사했어요 그리고 한 번도 가져본 적 없던 규칙적인 생활 패턴이 생겨서 너무 도움됐어요_x000d_
 뭘 요청하거나 질문을 했을 때 잘 답변해주셔서 감사합니다</v>
       </c>
       <c r="J118" t="str">
@@ -4693,7 +4693,7 @@
         <v>무시하고 놓아버릴 수 있는 영어 단어 학습을 꾸준하게 시켜주는 유일한 시간입니다. 아침에 단어시험지를 받아서 모르는 단어만 골라 뜻을 확인하고 확인한 단어를 따로 모아서 저장해두는 방식으로 사용한다면 효율적으로 공부할 수 있습니다</v>
       </c>
       <c r="I119" t="str">
-        <v>학습에 많은 도움이 되었습니다. 수능 전에는 적당한 긴장분위기를 만들어주어서 큰 부담없이 수능을 볼 수 있었습니다. 식사 관련해서도 크게 문제될 것 없이 적당하게 나와서 불편함은 없었습니다. 또한 인원이 적어서 선생님들이 케어하기 좋다는 것도 장점입니다</v>
+        <v>학습에 많은 도움이 되었습니다. 수능 전에는 적당한 긴장분위기를 만들어주어서 큰 부담 없이 수능을 볼 수 있었습니다. 식사 관련해서도 크게 문제될 것 없이 적당하게 나와서 불편함은 없었습니다. 또한 인원이 적어서 선생님들이 케어하기 좋다는 것도 장점입니다</v>
       </c>
       <c r="J119" t="str">
         <v>개인별 학습 계획과 진행 상황을 점검받고, 과목별 취약점과 개선점을 확인하며 학습 방법을 보완했어요.</v>
@@ -4799,7 +4799,7 @@
         <v>인강 구독권을 무료로 제공해준 점은 확실히 도움이 됐다. 따로 강의를 결제하지 않아도 필요한 과목을 바로 들을 수 있어서 부담이 줄었고, 부족한 부분을 보완하는 데 유용했다. 다만 모든 강의를 다 활용하기보다는, 본인에게 필요한 강의만 선택해서 듣는 게 더 중요하다고 느꼈다. 그래도 기본적인 학습 환경을 갖춰준다는 점에서 충분히 만족스러운 혜택이었다.</v>
       </c>
       <c r="I122" t="str">
-        <v>담임 선생님부터, 생활 관리 선생님들, 기숙 사감 선생님들 덕에 좋은 습관으로 공부 할 수 있었습니다!선생님들께서 항상 친절하게 대해주시고, 필요할 때마다 도움을 주셔서 감사했다. 공부를 하면서 힘들 때도 있었지만, 응원해주시고 방향을 잡아주신 덕분에 끝까지 버틸 수 있었던 것 같다. 과하게 간섭하기보다는 필요한 순간에 도움을 주시는 방식이 오히려 더 편하게 느껴졌고, 그 점이 특히 좋았다. 진심으로 감사드립니다.</v>
+        <v>담임 선생님부터, 생활 관리 선생님들, 기숙 사감 선생님들 덕에 좋은 습관으로 공부할 수 있었습니다!선생님들께서 항상 친절하게 대해주시고, 필요할 때마다 도움을 주셔서 감사했다. 공부를 하면서 힘들 때도 있었지만, 응원해주시고 방향을 잡아주신 덕분에 끝까지 버틸 수 있었던 것 같다. 과하게 간섭하기보다는 필요한 순간에 도움을 주시는 방식이 오히려 더 편하게 느껴졌고, 그 점이 특히 좋았다. 진심으로 감사드립니다.</v>
       </c>
       <c r="J122" t="str">
         <v>일정한 생활 패턴을 유지하고, 공부에만 집중할 수 있는 환경 속에서 자연스럽게 학습 루틴을 잡을 수 있었어요.</v>
@@ -5115,7 +5115,7 @@
         <v>N수생</v>
       </c>
       <c r="E131" t="str">
-        <v>처음 공부시작할때 구체적인 방향성 설정해가면서 주기적으로 점검하면서 공부 할수 있어 좋았고 혼자 계획 설정하고 공부할때에는 밀리거나 놓치는 부분이 있는데 그런 부분 보완해주는 느낌이 좋았습니다.</v>
+        <v>처음 공부시작할때 구체적인 방향성 설정해가면서 주기적으로 점검하면서 공부할수 있어 좋았고 혼자 계획 설정하고 공부할때에는 밀리거나 놓치는 부분이 있는데 그런 부분 보완해주는 느낌이 좋았습니다.</v>
       </c>
       <c r="F131" t="str">
         <v>본인이 혼자 공부하다보면 모르는 부분이 생기기 마련이고 그 부분을 공부하다보면 계속 본인이 아는 방향으로만 풀거나 실수가 쉽사리 보이지 않을때가 많은데 1대1질문으로 평소 시간 써야 할 부분을 줄이고 효율적으로 공부가 가능했습니다.</v>
@@ -5226,7 +5226,7 @@
         <v>원래 수기로 직접 플래너를 쓰면서 공부를 했었는데, 프로그램으로 계획을 작성을 하니까 나의 공부 시간 비중, 패턴을 쉽게 파악할 수 있었다. 그래서 매주 과목 공부 비중을 신경 쓰면서 계획을 짤 수 있었다.</v>
       </c>
       <c r="G134" t="str">
-        <v>공부를 할 때 제일 방해가 되는 것이 핸드폰이다. 집이나 다른 곳에서 공부를 하게 되면 핸드폰을 보게 되어 공부에 집중을 못하는 경우가 종종 발생한다.이투스 학원을 다니면서 핸드폰을 제출함으로써 공부 시간은 물론 쉬는시간에도 핸드폰을 못하니까 순공시간이 늘어나게 되었다.</v>
+        <v>공부를 할 때 제일 방해가 되는 것이 핸드폰이다. 집이나 다른 곳에서 공부를 하게 되면 핸드폰을 보게 되어 공부에 집중을 못하는 경우가 종종 발생한다.이투스 학원을 다니면서 핸드폰을 제출함으로써 공부 시간은 물론 쉬는시간에도 핸드폰을 못하니까 순공 시간이 늘어나게 되었다.</v>
       </c>
       <c r="H134" t="str">
         <v>영어공부 중에서 단어를 외우는 것은 중요하다. 그치만 단어를 스스로 외우는 것은 쉽지 않은 일이다. 학원에서 단어테스트를 진행함으로써 강제적으로 단어를 매일매일 외울 수 있어서 도움이 되었다.</v>
@@ -5255,7 +5255,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E135" t="str">
-        <v>매일 매일 학습 계획을 짤 때 체계적이고 실행가능하게 짤 수 있도록 도와주셔서 도움이 많이 되었다. 또한 어느 부분이 부족하고 어느부분을 더 공략해야하는지 상담을 잘 해주셔서 도움이 많이 되었다</v>
+        <v>매일 매일 학습 계획을 짤 때 체계적이고 실행가능하게 짤 수 있도록 도와주셔서 도움이 많이 되었다. 또한 어느 부분이 부족하고 어느부분을 더 공략해야 하는지 상담을 잘 해주셔서 도움이 많이 되었다</v>
       </c>
       <c r="F135" t="str">
         <v>학습 일정, 계획을 짤 때 도움이 많이 되었고 계획적으로 학습을 할 수 있어서 좋았다. 또한 매일 얼만큼 공부를 했는지 체크할 수 있어서 나의 학습현황도 확인하기에 유용해서 도움이 많이 되었다</v>
@@ -5299,7 +5299,7 @@
         <v>정말 필요한 만큼만 핸드폰 수거하는게 가장 좋았다. 점심시간과 저녁시간에는 핸드폰 사용이 가능해서 다른 학원에 비해 부담이 매우 적었다. 핸드폰 중독이 심한 사람은 핸드폰을 장시간 사용 못하면 불안하여 오히려 집중이 더 안되는데, 딱 필요한 공부 시간만 수거하는게 좋았다</v>
       </c>
       <c r="H136" t="str">
-        <v>학력평가와 평가원 모의고사 뿐만 아니라 이투스 모의고사를 정기적으로 봄으로써 좋은 성적을 긴장을 놓치지 않고 유지 할 수 있었다. 모의고사도 퀄리티가 좋아서 공부 할 때도 매우 도움이 되었다</v>
+        <v>학력평가와 평가원 모의고사 뿐만 아니라 이투스 모의고사를 정기적으로 봄으로써 좋은 성적을 긴장을 놓치지 않고 유지 할 수 있었다. 모의고사도 퀄리티가 좋아서 공부할 때도 매우 도움이 되었다</v>
       </c>
       <c r="I136" t="str">
         <v>학원에서 공부하는데 지루하지 않게 자주 이벤트를 많이 준비해주어 좋았습니다!! 계속 학원에서 공부만 하면 지루한데 유쾌한 분위기로 만들어주어 오히려 집중력 향상에 도움 되었어요!! 감사했습니다!!!</v>
@@ -5705,7 +5705,7 @@
         <v>항상 따뜻한 마음으로 지도해주시고, 공부에 집중할 수 있는 좋은 환경을 만들어주셔서 진심으로 감사드립니다. 선생님들의 세심한 배려와 응원 덕분에 더욱 성실하게 노력할 수 있었습니다.</v>
       </c>
       <c r="J147" t="str">
-        <v>국어가 가장 취약 과목이였는데, 담임 선생님과의 상담을 통해 공부 방법과 글 읽는 방향을 바로 잡아 성적 향상에 큰 도움이 되었어요.</v>
+        <v>국어가 가장 취약 과목이였는데, 담임 선생님과의 상담을 통해 공부 방법과 글 읽는 방향을 바로잡아 성적 향상에 큰 도움이 되었어요.</v>
       </c>
       <c r="K147" t="str">
         <v/>
@@ -5843,13 +5843,13 @@
         <v>아침에 꾸준히 학습 계획을 쓰게 되면서 하루 목표 공부량과 시간을 정확히 알 수 있어서 좋았고 꾸준히 쓰다보니 진도도 안밀리고 부족한부분 보완할점도 같이 알려주셔서 공부하는데 많은 도움을 받았습니다</v>
       </c>
       <c r="G151" t="str">
-        <v>잠이 많아서 정말 자주 졸아서 공부 집중시간도 짧고 순공시간도 짧았는데 계속 돌아다니시면서 깨워주셔서 갈 수록 덜 졸게되고 집중시간도 길어지고 공부도 집중해서 더 잘 할 수 있었던 것 같아 좋았습니다.</v>
+        <v>잠이 많아서 정말 자주 졸아서 공부 집중시간도 짧고 순공 시간도 짧았는데 계속 돌아다니시면서 깨워주셔서 갈 수록 덜 졸게되고 집중시간도 길어지고 공부도 집중해서 더 잘 할 수 있었던 것 같아 좋았습니다.</v>
       </c>
       <c r="H151" t="str">
         <v>혼자공부할때는 영어단어 안외우고 계속 미루게되었는데 이투스247에서는 아침마다 테스트를 보고 통과했어야하기 때문에 꾸준히 외우게되서 전보다 암기량과 암기속도 모두 좋아져서 도움이 되었습니다.</v>
       </c>
       <c r="I151" t="str">
-        <v>현역때 공부를 정말 많이 안했어서 재수를 어떻게 시작해야 할지 공부는 어떻게해야하는지 정말 막막했었는데 공부법이랑 공부관리.상담 잘해주시고 1년 동안 재수하는데 많은 도움주셔서 정말 감사합니다.</v>
+        <v>현역때 공부를 정말 많이 안했어서 재수를 어떻게 시작해야 할지 공부는 어떻게해야 하는지 정말 막막했었는데 공부법이랑 공부관리.상담 잘해주시고 1년 동안 재수하는데 많은 도움주셔서 정말 감사합니다.</v>
       </c>
       <c r="J151" t="str">
         <v>아침마다 영단어 테스트를 보며 꾸준히 암기한 덕분에 암기량과 속도를 함께 높일 수 있었어요.</v>
@@ -5942,12 +5942,12 @@
         <v>N수생</v>
       </c>
       <c r="E154" t="str" xml:space="preserve">
-        <v xml:space="preserve">어떤 전략을 가지고 대학교를 지원해야하는지 친절하게 생명해주심_x000d_
+        <v xml:space="preserve">어떤 전략을 가지고 대학교를 지원해야 하는지 친절하게 생명해주심_x000d_
 덕분에 진학가라는 앱을 유용하게 사용하는법을 알고 정시 카드를 잘 썼다_x000d_
 세세하게 분석하는법을 알려주시는게 정말 인상적이였다고 생각한다</v>
       </c>
       <c r="F154" t="str">
-        <v>내가 어떤 과목이 부족하고 부족한 과목을 어떤식으로 공부하고 얼마나 더 해야하는지 알려주셔서 그 과목에 맞추어서 더 열심히 공부하게 되었던것 같다. 그런식으로 하니 어떻게 공부해야하는지 깨달았다</v>
+        <v>내가 어떤 과목이 부족하고 부족한 과목을 어떤식으로 공부하고 얼마나 더 해야 하는지 알려주셔서 그 과목에 맞추어서 더 열심히 공부하게 되었던것 같다. 그런식으로 하니 어떻게 공부해야 하는지 깨달았다</v>
       </c>
       <c r="G154" t="str">
         <v>원래 아이패드나 핸드폰이 있으면 집중을 잘 하지 못하는 성격인데 그런 것을 다 통제해버리니까 내가 공부하는 시간에 더 집중일 기울여서 했던것 같다 힘들고 지루했지만 인상적인 시간들이였던것 같다</v>
@@ -5983,7 +5983,7 @@
         <v>일단 학습 스케쥴에 방해 되지 않도록 상담일자를 잡아주셔서 좋았다. 그리고 내가 알지 못했던 인강 커리큘럼이나 모의고사 등을 현 수준과 현황에 맞추어 추천해주신 것이 도움이 되었다. 내 학습 진도 상황도 체크해주셔서 더 성실하게 공부를 할 수 있었다.</v>
       </c>
       <c r="F155" t="str">
-        <v>학습 시간에 인강 자료나 커리큘럼을 둘러보고 찾아보는 것이 매우 큰 시간 낭비라고 느꼈는데 선생님께서 현 상황에 알맞는 것들을 추천 해주셔서 시간을 대폭 절약하고 공부에 집중 할 수 있었다</v>
+        <v>학습 시간에 인강 자료나 커리큘럼을 둘러보고 찾아보는 것이 매우 큰 시간 낭비라고 느꼈는데 선생님께서 현 상황에 알맞는 것들을 추천 해주셔서 시간을 대폭 절약하고 공부에 집중할 수 있었다</v>
       </c>
       <c r="G155" t="str">
         <v>여름 기간에 지치거나 아침에 나도 모르게 졸 때가 많았는데 지속적인 순찰로 잠을 깨워주셔서 경각심을 가지며 학습 할 수 있었다. 벌점을 받지 않으려고 잠을 깨기 위해 노력했던것 같다.</v>
@@ -6056,7 +6056,7 @@
         <v>2주마다 담임 선생님과 상담을 했던게 정말 큰 도움이 됐습니다. 만약에 혼자 공부를 했다면 내가 이 방향으로 가는것이 맞는건가? 라는 생각과 불안함이 많이 들었을텐데 계속 옆에서 방향을 잡아주셨었고, 내가 하루에 이정도 공부는 해야한다를 정해주셔서 그걸 나의 페이스대로 성실하게 할 수 있었고 그걸 계속 체크하면서 검사해주셔서 대충하지 않고 열심히 할 수 있었습니다</v>
       </c>
       <c r="G157" t="str">
-        <v>일단 원래 앉는 고정좌석이 있었는데 사실 처음에는 너무 답답하지 않을까 걱정을 많이 했었는데 생활해보니까 오히려 옆자리를 신경 쓰지 않아도 되고 집중이 너무 잘 돼서 일차적으로 그게 좋았습니다. 그리고 리프레쉬 룸이나 밖에도 서서 공부하거나 답답하지 않게 공부 할 수 있능 공간이 있는게 너무 좋았고 다들 집중해서 공부하는 모습을 보고 자극도 많이 받으면서 잘 공부했습니다</v>
+        <v>일단 원래 앉는 고정좌석이 있었는데 사실 처음에는 너무 답답하지 않을까 걱정을 많이 했었는데 생활해보니까 오히려 옆자리를 신경 쓰지 않아도 되고 집중이 너무 잘 돼서 일차적으로 그게 좋았습니다. 그리고 리프레쉬 룸이나 밖에도 서서 공부하거나 답답하지 않게 공부할 수 있능 공간이 있는게 너무 좋았고 다들 집중해서 공부하는 모습을 보고 자극도 많이 받으면서 잘 공부했습니다</v>
       </c>
       <c r="H157" t="str">
         <v>매달 마다 이투스 모의고사를 보면서 나의 위치가 어느정도이고 내가 어느위치인지를 확인 하면서 공부를 하다보니 나의 부족한 점과 채울 부분을 많이 알게 됐다. 그리고 모의고사를 매달 보다보니 모의고사에서 많은 변수를 만나게 됐고 내가 만났던 그런 변수들이 실제 수능에서도 큰 도움이 됐습니다. 그리고 질 좋은 문제들이 매우 많았고 해설지도 양질로 매우 도움이 됐습니다</v>
@@ -6338,7 +6338,7 @@
         <v>모르는 문제가 있으면 이투스 어플에 들어가 바로 상담신청을 하면 조교 선생님께서 문제를 알려주어 당일에 해결을 할수 있었고 중간중간 정신적으로 힘들 때 마다 저의 조교 담당 선생님과 멘탈 관리를 받아서 힘들았던 재수 생활이였지만 버틸수 있었던거 같다</v>
       </c>
       <c r="G165" t="str">
-        <v>다른 지점 같은 경우는 들리는 말로는 몰래 다른 활동을 할수 있다고 들었는데 이투스 247은 와이파이가 막혀있어 다른 사이트가 접속이 안되니 오로지 인강 사이트에 집중 할수 있었던거 같고 집중이 안될때에도 어쩔수 없이 인강만 들을수 있으니 다시 집중하여 들을수 있었던거 같다</v>
+        <v>다른 지점 같은 경우는 들리는 말로는 몰래 다른 활동을 할수 있다고 들었는데 이투스 247은 와이파이가 막혀있어 다른 사이트가 접속이 안되니 오로지 인강 사이트에 집중할수 있었던거 같고 집중이 안될때에도 어쩔수 없이 인강만 들을수 있으니 다시 집중하여 들을수 있었던거 같다</v>
       </c>
       <c r="H165" t="str">
         <v>매일매일 단어 시험만 보는것이 아닌 우리 지점은 주마다 매주 국어 시험과 수학을 시험을 보았는데 영어 단어도 평소에 나였으면 가끔 드문드문 보았을거 같은데 매일 시험을 보게하여 도움이 되었던거 같고 수학 국어시험을 매주보아 감을 잃지 않아 성적유지 및 향상에 도움이 되었다</v>
@@ -6447,7 +6447,7 @@
         <v>카드를 찍으며 왔다갔다 하니까 소속감이 생겼고 출결에 더 신경쓰여 빠지지 않고 매일 매일 등원에 더 신견써서 공부 했던거 같습니다. 또한 카드를 사용하였기에 핸드폰이 없어도 되어 좋았던거 같습니다</v>
       </c>
       <c r="H168" t="str">
-        <v>무료로 이투스 강의를 제공해주어 제가 듣고 싶은 강사님을 들을 수 있어서 좋았습니다 덕분에 경제적 부담없이 성적을 늘리기에 좋았던거 같습니다 저 같은 경우 사탐을 이투스 덕에 올린거 같습니다</v>
+        <v>무료로 이투스 강의를 제공해주어 제가 듣고 싶은 강사님을 들을 수 있어서 좋았습니다 덕분에 경제적 부담 없이 성적을 늘리기에 좋았던거 같습니다 저 같은 경우 사탐을 이투스 덕에 올린거 같습니다</v>
       </c>
       <c r="I168" t="str">
         <v>짧은 시간동안 감사했습니다 만족하는 결과가 나오지는 못 했지만 이건 저의 부족함 때문이였던거 같습니다 분위기가 가족같아서 좋았던거 같습니드 앞으로도 번창하세요 이투스247 일산 서구점 파이팅</v>
@@ -6526,7 +6526,7 @@
         <v xml:space="preserve">학습 관리 시스템 중에서도 출석 관리와 생활 관리 부분이 특히 유용하다고 느꼈습니다😊_x000d_
 매일 출석 날짜를 체계적으로 관리해주셔서 스스로 흐트러지지 않고 꾸준히 학원에 나올 수 있었고, 자연스럽게 규칙적인 생활 습관을 유지하는 데 큰 도움이 되었습니다. 혼자였다면 쉽게 느슨해질 수 있었을 텐데, 이러한 관리 덕분에 끝까지 긴장감을 유지할 수 있었습니다._x000d_
 _x000d_
-또한 선생님들께서 학원을 직접 돌아다니시면서 학생들의 학습 상태를 확인해주신 점도 인상 깊었습니다. 공부하다가 졸거나 집중력이 떨어질 때 바로 잡아주셔서 다시 흐름을 이어갈 수 있었고, 그 덕분에 공부 시간의 밀도가 훨씬 높아졌다고 느꼈습니다💪_x000d_
+또한 선생님들께서 학원을 직접 돌아다니시면서 학생들의 학습 상태를 확인해주신 점도 인상 깊었습니다. 공부하다가 졸거나 집중력이 떨어질 때 바로잡아주셔서 다시 흐름을 이어갈 수 있었고, 그 덕분에 공부 시간의 밀도가 훨씬 높아졌다고 느꼈습니다💪_x000d_
 _x000d_
 이러한 세심한 관리 덕분에 단순히 자리에 앉아 있는 것이 아니라, 실제로 집중해서 공부하는 시간을 늘릴 수 있었고, 스스로를 통제하는 힘도 함께 기를 수 있었습니다. 결과적으로 학습 습관을 잡고 꾸준함을 유지하는 데 큰 도움이 된 시스템이었다고 생각합니다✨</v>
       </c>
@@ -6576,7 +6576,7 @@
         <v>저의 현재 상태와 위치를 알 수 있었고 이를 통해 선생님과 상담 후 저의 방향을 설정할 수 있었고 사람마다 맞는 공부 스타일과 방법이 있으며 좋은 공부 방법과 나쁜 공부 방법은 딱히 없고 본인에게 맞는 학습 방법을 가져가면 되겠다고 생각했습니다</v>
       </c>
       <c r="G171" t="str">
-        <v>평소 저를 포함한 모든 학생들이 휴대폰에 빠져 살고 있지만 휴대폰을 수거함으로써 유혹도 제거되고 온전히 공부에만 집중할 수 있게 되었습니다 휴대폰이 없으니 공부도 더 잘 되고 순공시간도 늘어났습니다! 단순한 억제가 아닌 인내였다고 느꼈습니다</v>
+        <v>평소 저를 포함한 모든 학생들이 휴대폰에 빠져 살고 있지만 휴대폰을 수거함으로써 유혹도 제거되고 온전히 공부에만 집중할 수 있게 되었습니다 휴대폰이 없으니 공부도 더 잘 되고 순공 시간도 늘어났습니다! 단순한 억제가 아닌 인내였다고 느꼈습니다</v>
       </c>
       <c r="H171" t="str">
         <v>이투스에는 훌륭한 인강 강사분들이 계시지만 이투스는 다른 앱과 다르게 구독을 갱신해야한다는 불편함이 있었지만 이투스247독학재수학원을 다니면서 무료로 이투스 인강을 볼 수 있어서 정말 좋았고 구독갱신을 안해도 되어서 너무 편했습니다</v>
@@ -6800,7 +6800,7 @@
         <v>시험을 딱 한 번 봤었고 실수를 제외하면 시험 결과 또한 맘에 들게 나오게 돼서 결과로 별로 위로받지 못했던 나에게 큰 위로와 자신감을 불어넣어줄 수 있었다 온전한 시험의 효과라기보단 개인의 특수성이 포함된거지만 이 시험이 있었기에 그런 경험 또한 이뤄냈다고 생각한다</v>
       </c>
       <c r="I177" t="str">
-        <v>매주, 매일 정해진 크고 작은 루틴들을 큰 문제 없이 균일하고 안정적이게 진행시켜 주셔서 감사합니다 덕분에 변수를 가정하지 않고 온전히 공부에만 집중하여 많은 순공시간을 확보할 수 있었습니다</v>
+        <v>매주, 매일 정해진 크고 작은 루틴들을 큰 문제 없이 균일하고 안정적이게 진행시켜 주셔서 감사합니다 덕분에 변수를 가정하지 않고 온전히 공부에만 집중하여 많은 순공 시간을 확보할 수 있었습니다</v>
       </c>
       <c r="J177" t="str">
         <v>공부를 제대로 계획 세워 해본 적이 없어서 시작도 못할 뻔 했는데, 선생님과 상담하면서 현재 내 위치를 인지하고 시작할 수 있었어요.</v>
@@ -7301,7 +7301,7 @@
       </c>
       <c r="G191" t="str" xml:space="preserve">
         <v xml:space="preserve">생활 관리 측면에서 세심하게 챙겨주신 부분이 특히 좋았습니다. 단순히 공부만 강조하는 것이 아니라, 실제로 공부를 지속할 수 있는 컨디션을 유지하도록 도와주신 점이 인상 깊었습니다. 수험 생활을 하다 보면 졸음이 쏟아지거나 집중력이 떨어지는 순간이 많은데, 그럴 때마다 적절하게 깨워주시고 현재 상태를 체크해주셔서 흐름이 끊기지 않도록 관리해주셨습니다._x000d_
-특히 “괜찮겠지” 하고 그냥 넘어갈 수 있는 부분까지도 수시로 확인해주시면서, 졸거나 집중이 흐트러질 때 바로 잡아주신 점이 도움이 많이 되었습니다. 덕분에 스스로 놓치기 쉬운 생활 리듬이나 집중 상태를 꾸준히 유지할 수 있었고, 혼자였다면 무너졌을 타이밍도 잘 넘길 수 있었습니다._x000d_
+특히 “괜찮겠지” 하고 그냥 넘어갈 수 있는 부분까지도 수시로 확인해주시면서, 졸거나 집중이 흐트러질 때 바로잡아주신 점이 도움이 많이 되었습니다. 덕분에 스스로 놓치기 쉬운 생활 리듬이나 집중 상태를 꾸준히 유지할 수 있었고, 혼자였다면 무너졌을 타이밍도 잘 넘길 수 있었습니다._x000d_
 또한 단순히 깨워주는 데서 끝나는 것이 아니라, 언제 쉬는 게 좋은지, 어떻게 다시 집중을 끌어올려야 하는지까지 함께 지도해주셔서 효율적으로 하루를 운영할 수 있었습니다. 이런 세심한 생활 관리 덕분에 공부 시간의 질 자체가 올라갔다고 느꼈습니다.</v>
       </c>
       <c r="H191" t="str" xml:space="preserve">
@@ -7404,7 +7404,7 @@
         <v>N수생</v>
       </c>
       <c r="E194" t="str">
-        <v>담임 선생님과 성적 고민을 부담없이 나눌 수 있어 좋았고 멘토 선생님과 얘기를 하며 학습 향상에 도움이 되었다. 해야되는 공부량을 일주일에 한 번씩 대면하면서 모의고사나 더프 등 시험볼 때의 팁들을 알아갈 수 있어서 좋았다.</v>
+        <v>담임 선생님과 성적 고민을 부담 없이 나눌 수 있어 좋았고 멘토 선생님과 얘기를 하며 학습 향상에 도움이 되었다. 해야되는 공부량을 일주일에 한 번씩 대면하면서 모의고사나 더프 등 시험볼 때의 팁들을 알아갈 수 있어서 좋았다.</v>
       </c>
       <c r="F194" t="str">
         <v>평소에는 계획을 잘 세우지 않는편이라 공부할 때 방향성을 잡기 쉽지 않았는데 매일 내가 한 학습량과 앞으로 해야 할 것들을 정리하면서 하루하루 성취감도 생기고 공부 계획을 철저하게 세울 수 있어 도움이 되었다.</v>
@@ -7668,7 +7668,7 @@
         <v>계획이 저처럼 있는 학생은 이 계획을 잘 지켰는지 검사를 함으로서 나태해지는 길로 가는 걸 막아주셔서 좋았던 거 같습니다. 감시가 있는 덕분에 스스로와의 타협은 버리고 공부로의 정진을 택해 좋은 결과가 이렇게 나오게 된 거 같아 기분이 좋았습니다.</v>
       </c>
       <c r="G201" t="str">
-        <v>혼자서 반수를 하게 되면 안 그래도 고3 때의 시절과 달리 대학을 다니다 수능을 다시 치르는 거라 그 수험생 때의 생활패턴으로 돌아가기가 힘들텐데 이 독학재수학원에 다니면서 생활패턴을 어느정도 관리할 수 있던 점이 상당히 좋았던 거 같습니다.</v>
+        <v>혼자서 반수를 하게 되면 안 그래도 고3 때의 시절과 달리 대학을 다니다 수능을 다시 치르는 거라 그 수험생 때의 생활 패턴으로 돌아가기가 힘들텐데 이 독학재수학원에 다니면서 생활 패턴을 어느정도 관리할 수 있던 점이 상당히 좋았던 거 같습니다.</v>
       </c>
       <c r="H201" t="str">
         <v>평가원 기출 문제나 교육청 같은 문제도 중요하지만 요즘엔 안 그래도 사설 컨텐츠의 퀄이 상당히 좋습니다. 그렇기 때문에 이러한 점에서 이득을 볼 수 있게 해주어 다양한 유형의 문제를 풀 수 있어 좋았던 거 같습니다.</v>
@@ -7777,15 +7777,15 @@
         <v>N수생</v>
       </c>
       <c r="E204" t="str" xml:space="preserve">
-        <v xml:space="preserve">저희 원주 이투스 247은 사람 한 명 한명에 맞춰서 공부 습관과 성향에 따라 스케쥴을 짜주십니다. 큰 틀인 공부 커리큘럼을 짜주시기도 하셨고, 정말 세세하게 몇 페이지부터 몇 페이지까지 몇 일 몇 시에 해야하는지 까지 짜주십니다. _x000d_
+        <v xml:space="preserve">저희 원주 이투스 247은 사람 한 명 한명에 맞춰서 공부 습관과 성향에 따라 스케쥴을 짜주십니다. 큰 틀인 공부 커리큘럼을 짜주시기도 하셨고, 정말 세세하게 몇 페이지부터 몇 페이지까지 몇 일 몇 시에 해야 하는지 까지 짜주십니다. _x000d_
 그 외에도 어떻게 글을 읽어야 흐름이 이어지는지 어떻게 문제를 풀어야 쉽고 빠르게 풀 수 있는지에 대한 방법도 알려주십니다. _x000d_
 시험을 본 후 오답에 대해서 같이 얘기도 하는데 그 과정에서 나도 모르는 나의 안 좋은 공부 태도 및 공부 방법을 찾을 수 있고, 그 과정에서 한 걸음 성장하는 계기가 될 수 있었던 것 같습니다.</v>
       </c>
       <c r="F204" t="str">
-        <v>사실 재수종합학원에서 관리를 해준다고 해도 100% 내가 뭘하는지 내가 무슨 공부를 어떻게 하는지는 다른 학원에는 모르실겁니다. 하지만 이투스 247 원주에서는 한 명 한 명 타이트한 플래너 검사와 생활지도로 학생을 관리하시는 모든 선생님이 학생 한 명 한 명 공부를 어떻게 하는지 언제 학원 외출을 하는지에 대해 알고 계십니다. 학생 입장에선 이 점이 학원을 믿고 맡길 수 있는 점이라고 생각합니다</v>
+        <v>사실 재수종합학원에서 관리를 해준다고 해도 100% 내가 뭘하는지 내가 무슨 공부를 어떻게 하는지는 다른 학원에는 모르실겁니다. 하지만 이투스 247 원주에서는 한 명 한 명 타이트한 플래너 검사와 생활 지도로 학생을 관리하시는 모든 선생님이 학생 한 명 한 명 공부를 어떻게 하는지 언제 학원 외출을 하는지에 대해 알고 계십니다. 학생 입장에선 이 점이 학원을 믿고 맡길 수 있는 점이라고 생각합니다</v>
       </c>
       <c r="G204" t="str">
-        <v>이투스 247 원주 학원은 학원에 학생이 공부하고 있는 시간엔 통행금지 시간 외엔 10분 이내로 졸음지도, 생활지도를 했습니다. 이 경우 학생들은 지도를 의식하며 더 공부를 열심히 하고 더 깊은 집중을 갖고 공부를 할 수 있는 것 같습니다. 또, 핸드폰 미제출 관리 및 학원 내 정숙을 항상 유지시키기 때문에 불필요한 집중을 깨는 사유들을 없앨 수 있는 것 같습니다.</v>
+        <v>이투스 247 원주 학원은 학원에 학생이 공부하고 있는 시간엔 통행금지 시간 외엔 10분 이내로 졸음 지도, 생활 지도를 했습니다. 이 경우 학생들은 지도를 의식하며 더 공부를 열심히 하고 더 깊은 집중을 갖고 공부를 할 수 있는 것 같습니다. 또, 핸드폰 미제출 관리 및 학원 내 정숙을 항상 유지시키기 때문에 불필요한 집중을 깨는 사유들을 없앨 수 있는 것 같습니다.</v>
       </c>
       <c r="H204" t="str">
         <v>사실 혼자 영어 공부를 한다면 개인적인 의견이지만 80%의 학생들은 단어를 소홀히 여길 것이고, 그럼 당연히 영어 성적은 오르지 않을 것 입니다. 영어의 기본은 독해, 문법, 듣기 모두 중요하지만 그의 기반은 영어 단어가 얼마나 잘 외워졌느냐 부터 시작 할 것 같습니다. 이에 필수적으로 voca를 하기에 학생들이 챙기기 귀찮아하는 영어 단어 외우기를 잘 할 수 있었던 것 같습니다.</v>
@@ -7884,10 +7884,10 @@
         <v>N수생</v>
       </c>
       <c r="E207" t="str">
-        <v>어떤 점이 부족하고 어떻게 공부해야하는지 친절히 알려주셨습니다. 또한 인강 선생님들마다의 특징도 잘 알고 계시고 무슨 교재가 지금 적절할지 조언해주셨습니다. 모의고사가 얼마 남지 않았을땐 어떻게 선택과 집중을 해야하는지, 어떤 단원에 힘을 써야할지도 제 상황에 맞게 알려주시고 지도해주셔서 큰 도움이 되었고 힘이 되었습니다.</v>
+        <v>어떤 점이 부족하고 어떻게 공부해야 하는지 친절히 알려주셨습니다. 또한 인강 선생님들마다의 특징도 잘 알고 계시고 무슨 교재가 지금 적절할지 조언해주셨습니다. 모의고사가 얼마 남지 않았을땐 어떻게 선택과 집중을 해야 하는지, 어떤 단원에 힘을 써야할지도 제 상황에 맞게 알려주시고 지도해주셔서 큰 도움이 되었고 힘이 되었습니다.</v>
       </c>
       <c r="F207" t="str">
-        <v>무엇보다 부담없이 과목별 선생님과 상담할 수 있는 것이 마음에 들었습니다. 인강을 들으면서 학습을 하다 보니 모르거나 궁금한 것이 있을때 바로 의견•조언을 얻기가 힘들어서 고민이었는데, 그럴때마다 바로바로 질문을 드리고 해답을 얻을 수 있는 것이 큰 도움이 되었습니다.</v>
+        <v>무엇보다 부담 없이 과목별 선생님과 상담할 수 있는 것이 마음에 들었습니다. 인강을 들으면서 학습을 하다 보니 모르거나 궁금한 것이 있을때 바로 의견•조언을 얻기가 힘들어서 고민이었는데, 그럴때마다 바로바로 질문을 드리고 해답을 얻을 수 있는 것이 큰 도움이 되었습니다.</v>
       </c>
       <c r="G207" t="str">
         <v>재수학원의 생활 관리 시스템은 규칙적인 생활 습관을 형성하는 데 큰 도움이 되었습니다. 정해진 시간표에 따라 공부와 휴식을 반복하면서 집중력이 높아졌고, 학습 계획을 체계적으로 유지할 수 있어 학업 효율도 자연스럽게 향상되었습니다.</v>
@@ -7989,7 +7989,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E210" t="str">
-        <v>선생님들께서 주기적으로 상담해주시면서 과목별로 자세히 어떻게 공부해야하는지 알려주셨고, 단체로 실전 모의고사를 친 후에 상담했던 것도 도움이 많이 되었고, 학습 뿐만 아니라 마음가짐에 대해서 알려주신 것도 유용했습니다.</v>
+        <v>선생님들께서 주기적으로 상담해주시면서 과목별로 자세히 어떻게 공부해야 하는지 알려주셨고, 단체로 실전 모의고사를 친 후에 상담했던 것도 도움이 많이 되었고, 학습 뿐만 아니라 마음가짐에 대해서 알려주신 것도 유용했습니다.</v>
       </c>
       <c r="F210" t="str">
         <v>일주일 단위로 자세히 학습 계획표를 짜게 하셨는데, 구체적이고 정확한 목표를 정하고 나니까 오늘은 무엇을 하고 어디까지 끝내야 할지가 눈에 보여서 학습량이 늘어나는 데 도움이 되었습니다.</v>
@@ -8171,7 +8171,7 @@
         <v>재수하기 전, 인강을 들을 때 수강율에 집착하고 주변 친구들의 추천을 통해 강의만 마구잡이로 많이 들어 그 해 수능에서 그닥 효과를 보지 못한 경험이 있었다. 이투스 학원에서 제공한 인강 추천 및 수강 관리 시스템으로 나에게 맞는 인강 강사 선생님을 나보다 인강에 대해 잘 아시는 분이 추천해주시니 한 인강 선생님의 커리큘럼을 성실하게 수행해내었다. 또 주마다 수강율 체크로 내가 지금 그 주에 소홀히 하고 있는 과목을 파악하고 이에 맞추어 그 주 인강 계획을 자세하게 수정해주시니 내가 그에 들일 노력을 대신 해주셔서 시간이 절약되는 효과를 누렸다.</v>
       </c>
       <c r="G215" t="str">
-        <v>현역 때, 독서실이나 스터디카페에서는 인강 시청을 위해 패드를 키고 공부를 하는 것이 아닌 패드로 유튜브를 보거나 소셜미디어 앱으로 노는 경향이 있었고 이로 인해 순공시간이 확실히 떨어졌다. 강제성이 부족해 실패를 겪으니, 이투스 학원에서 제공해주는 감독 시스템으로 패드를 통해 딴 짓을 못하게 되니 순공시간이 비약적으로 늘고 공부에만 오로지 집중할 수 있는 환경이 만들어졌다. 또 공부 시간에 잠이 와 졸거나 책상에서 쪽잠을 잘때 감독관 선생님이 와서 깨워주시니 순공시간이 늘어나는 효과와 함께 최대한 졸음을 깨우기 위해 노력하고 긴장감을 가지는 습관을 들게 되었다. 이를 통해 수능에서 현역 때의 수능 보다 좋은 결과를 얻은 것 같아 이투스의 생활 관리 시스템이 유용했다고 생각한다.</v>
+        <v>현역 때, 독서실이나 스터디카페에서는 인강 시청을 위해 패드를 키고 공부를 하는 것이 아닌 패드로 유튜브를 보거나 소셜미디어 앱으로 노는 경향이 있었고 이로 인해 순공 시간이 확실히 떨어졌다. 강제성이 부족해 실패를 겪으니, 이투스 학원에서 제공해주는 감독 시스템으로 패드를 통해 딴 짓을 못하게 되니 순공 시간이 비약적으로 늘고 공부에만 오로지 집중할 수 있는 환경이 만들어졌다. 또 공부 시간에 잠이 와 졸거나 책상에서 쪽잠을 잘때 감독관 선생님이 와서 깨워주시니 순공 시간이 늘어나는 효과와 함께 최대한 졸음을 깨우기 위해 노력하고 긴장감을 가지는 습관을 들게 되었다. 이를 통해 수능에서 현역 때의 수능 보다 좋은 결과를 얻은 것 같아 이투스의 생활 관리 시스템이 유용했다고 생각한다.</v>
       </c>
       <c r="H215" t="str">
         <v>이투스에서 제공해주는 전국 모의고사 시스템으로, 재수하는 동안 전국 재수생 간의 성적 지표를 알 수 있는 기회를 더 프리미엄 모의고사나 평가원 모의고사 외에 하나를 더 제공해주어 좋았다. 시험 후, 성적에 관한 분석 자료와 지금 성적으로 갈 수 있는 대학 등을 알려주어 지금 나의 상태에 대한 평가와 더 높은 성적을 위한 각오를 심어주어 학원을 다니는 동안 나에게 좋은 자극을 주었다. 달마다 모의고사를 정해진 시간에 수능 시스템으로 시험을 치르니, 후에 볼 수능을 연습해 볼 기회가 늘어나 매우 유용했다.</v>
@@ -8235,13 +8235,13 @@
         <v>반수생</v>
       </c>
       <c r="E217" t="str">
-        <v>당시에 고등학교 자퇴후에 제대로 된 확실한 목표없이 그저 사는대로 살아가면서 생활패턴이 완전히 무너져 아침 늦게 일어나고 새벽 넘어서 잠드는 삶을 살다가 이투스 247에 다니게 되면서 아침 일찍 일어나고 비교적 일찍 잠에 들며, 일정한 시간에 식사를 하는등 생활패턴이 7개월동안 일정하게 유지되면서 건강이 좋아진것은 물론이고 스스로도 지금 잘 살아가고 있다는 뿌듯함을 느끼게 되었음</v>
+        <v>당시에 고등학교 자퇴후에 제대로 된 확실한 목표없이 그저 사는대로 살아가면서 생활 패턴이 완전히 무너져 아침 늦게 일어나고 새벽 넘어서 잠드는 삶을 살다가 이투스 247에 다니게 되면서 아침 일찍 일어나고 비교적 일찍 잠에 들며, 일정한 시간에 식사를 하는등 생활 패턴이 7개월동안 일정하게 유지되면서 건강이 좋아진것은 물론이고 스스로도 지금 잘 살아가고 있다는 뿌듯함을 느끼게 되었음</v>
       </c>
       <c r="F217" t="str">
         <v>당시에 했던 쉬운 난이도의  검정고시 공부를 제외하면 중학교때 이후로 공부를 한적이 없어서 혼자 시작해볼려고 해도 어디부터,뭐부터 시작해야 하는지를 몰라 공부가 막막하게 느껴져서 공부를 더더욱 안하게 되는 상황이였으며 수능공부는 더욱 멀게만 느껴졌는데 이투스247에서 선생님들이 내 수준에 맞는 인강,교재등을 추천해주었고 실제로도 잘 맞았으며 자신에게 맞지 않다면 즉각적으로 인강,교제등을 변경하여서 해결하던 점이 유용했다</v>
       </c>
       <c r="G217" t="str">
-        <v>이투스 247학원에 처음 들어갔을때 생활패턴이 완전히 무너진 상태였었기에 아침에 공부할때는 졸면서 1~2시간을 낭비하는게 흔한일이였다. 하지만 이투스 247에서는 졸거나 집중을 제대로 못할때마다 관리감독 선생님께서 매번 도와주시면서 점차 조는 시간이 줄어들었다,정말 많이 졸았는데 포기하지 않으시고 매번 깨워주시며 노력하신점이 유용하다</v>
+        <v>이투스 247학원에 처음 들어갔을때 생활 패턴이 완전히 무너진 상태였었기에 아침에 공부할때는 졸면서 1~2시간을 낭비하는게 흔한일이였다. 하지만 이투스 247에서는 졸거나 집중을 제대로 못할때마다 관리감독 선생님께서 매번 도와주시면서 점차 조는 시간이 줄어들었다,정말 많이 졸았는데 포기하지 않으시고 매번 깨워주시며 노력하신점이 유용하다</v>
       </c>
       <c r="H217" t="str">
         <v>이투스247을 다니기 전까지는 모의고사가 도대체 무슨 효과가 있냐는 생각을 하였다 특히 사설 모의고사는 더,실제로도 초반에는 모의고사를 보고나서는 내 등급을 확인하고 스트레스만 쌓일 뿐이였다 하지만 어느날 모의고사를 보고나서 틀린점들을 분석하면서 복습을 하고 부족했던점들을 다음 모의고사때 적용하고 나서 처음으로 수능 사설 모의고사에서 8등급을 벗어나며 그때부터 실력이 조금씩 상승했기에 이 점이 유용하다 생각한다</v>
@@ -8532,7 +8532,7 @@
 얼마남지 않은 시기에 최고의 효율을 발휘해 예체능임에도 불구하고 2등급이라는 좋은 성적을 받을 수 있었습니다.</v>
       </c>
       <c r="G225" t="str">
-        <v>어떤 일을 하든 항상 스마트폰이 가장 큰 방해요소 중 하나였는데 강제적으로라도 폰을 사용하는 시간이 확 줄어 집중력도 높아지고 순공시간 또한 늘릴 수 있어서 입시에 큰 도움이 되었던것같습니다</v>
+        <v>어떤 일을 하든 항상 스마트폰이 가장 큰 방해요소 중 하나였는데 강제적으로라도 폰을 사용하는 시간이 확 줄어 집중력도 높아지고 순공 시간 또한 늘릴 수 있어서 입시에 큰 도움이 되었던것같습니다</v>
       </c>
       <c r="H225" t="str">
         <v>3,6모의고사를 못 본 저한테는 실전경험이 절실히 필요했습니다. 이투스 모의고사를 통해 수능장과 비슷한 상황에서 연습을 충분히 할 수 있었고 막판에 성적이 오른 가장 큰 요인 중 하나였습니다</v>
@@ -8567,14 +8567,14 @@
         <v>혼자 공부하다가 계속 모르는 문제들을 바로바로 선생님들께 여쭈어 볼 수 있어서 좋았습니다. 질문하는 것에 대해 부담이 있었는데 1:1 질문 시스템 덕분에 궁금한 점을 물어볼 수 있었습니다. 덕분에 문제들을 정확히 알고 넘어갈 수 있었습니다.</v>
       </c>
       <c r="G226" t="str" xml:space="preserve">
-        <v xml:space="preserve">학원의 면학 분위기 조성을 위하여 매 공부 시간마다 선생님들께서 돌아다니시면서 자는 사람들을 깨우고 공부에 집중 할 수 있도록 하셨습니다._x000d_
+        <v xml:space="preserve">학원의 면학 분위기 조성을 위하여 매 공부 시간마다 선생님들께서 돌아다니시면서 자는 사람들을 깨우고 공부에 집중할 수 있도록 하셨습니다._x000d_
 또한 시끄러운 사람이 있어 선생님들께 이야기하면 바로 조치를 취해주셔서 편안하게 조용한 환경에서 공부를 할 수 있었습니다.</v>
       </c>
       <c r="H226" t="str">
         <v>대성 모의고사와 교육청 모의고사, 평가원 모의고사로는 실전 모의고사 연습이 부족했었는데 이투스 모의고사도 봄으로써 더 많은 연습을 할 수 있어서 좋았습니다. 다양한 문제와 친절한 해설을 보면서 더욱 모의고사 푸는 연습을 할 수 있어서 도움이 많이 되었습니다.</v>
       </c>
       <c r="I226" t="str" xml:space="preserve">
-        <v xml:space="preserve">아침마다 이름 불러주시며 밝게 인사해주시고 공부에 집중 할 수 있도록 도와주셔서 감사합니다! 선생님들께서 학생 한명한명  도와주시고 신경써주신 덕분에 좋은 환경에서 열심히 공부 할 수 있었습니다!!_x000d_
+        <v xml:space="preserve">아침마다 이름 불러주시며 밝게 인사해주시고 공부에 집중할 수 있도록 도와주셔서 감사합니다! 선생님들께서 학생 한명한명  도와주시고 신경써주신 덕분에 좋은 환경에서 열심히 공부할 수 있었습니다!!_x000d_
 감사합니다</v>
       </c>
       <c r="J226" t="str">
@@ -8744,7 +8744,7 @@
         <v>스스로 학습 플래너를 쓰고 하면서 놓치거나 빠지는 과목, 부분들이 꽤 많았었는데 학습 관리 시스템을 활용함으로써 내가 빠뜨린 부분이나 조금 더 보완해야 할 부분들에 대해서 자세하게 피드백을 받을 수 있는 점이 유용했다. 또한 과목의 하나의 커리가 끝나게 되면 그에 맞는 다음 커리큘럼을 짜주고 공부 설정 방향을 설정해주는 점에서 많은 도움을 받을 수 있었다.</v>
       </c>
       <c r="G231" t="str">
-        <v>평소 핸드폰을 일상생활에서 분리하지 않고 외부에서 스스로 공부 할 때에는 아무리 핸드폰을 꺼놓아도 규제나 관리가 없었기에 수시로 확인하는 일이 많았다. 하지만 이와 같은 생활 관리 시스템이 이루어짐으로써 공부에 조금 더 집중 할 수 있는 환경이 만들어져서 좋았다.</v>
+        <v>평소 핸드폰을 일상생활에서 분리하지 않고 외부에서 스스로 공부할 때에는 아무리 핸드폰을 꺼놓아도 규제나 관리가 없었기에 수시로 확인하는 일이 많았다. 하지만 이와 같은 생활 관리 시스템이 이루어짐으로써 공부에 조금 더 집중할 수 있는 환경이 만들어져서 좋았다.</v>
       </c>
       <c r="H231" t="str">
         <v>단어는 혼자서 외우다 보면 어느정도 알고 있다는 생각을 가지게 됨으로써 복습하거나 따로 공부하지 않게 되었다. 하지만 보카 시험 콘텐츠가 있기에 매일매일 최소 30개의 단어를 외우고 볼 수 있었던 점이 영어 공부에 생각보다 더 많은 도움이 되었다. 또한 시험이기에 시간이 나거나 집중이 되지 않을 때 틈틈히 외운 것도 도움이 되었다.</v>
@@ -8858,7 +8858,7 @@
         <v>학원에 계시는 모든 분들 정말 진심으로 응원해주시고 관리해주신다는 걸  정말 많이 느꼈습니다. 가끔 쓴소리도 해주시지만 그것또한 다 잘되라고 하시는 거라는 걸 잘 알고 있습니다. 수험기간 동안 수고많이해주셔서 정말 감사했습니다.</v>
       </c>
       <c r="J234" t="str">
-        <v>담임 선생님과 성적 고민을 부담없이 나눌 수 있어 좋았고, 멘토 선생님과 얘기를 하며 학습 향상에 도움이 되었어요.</v>
+        <v>담임 선생님과 성적 고민을 부담 없이 나눌 수 있어 좋았고, 멘토 선생님과 얘기를 하며 학습 향상에 도움이 되었어요.</v>
       </c>
       <c r="K234" t="str">
         <v/>
@@ -9012,7 +9012,7 @@
         <v>감사드립니다. 덕분에 학원 생활을 하면서 큰 부담 없이 지낼 수 있었고, 편안한 분위기 속에서 생활할 수 있었습니다. 학생들을 세심하게 챙겨주시려는 모습도 느껴져서 감사했습니다. 때로는 조금 더 꼼꼼한 관리가 있었으면 좋겠다고 느끼기도 했지만, 전체적으로는 편하게 적응할 수 있게 도와주셔서 고맙게 생각합니다.</v>
       </c>
       <c r="J238" t="str">
-        <v>멘탈 관리와 학습 계획 점검, 생활패턴 관리 덕분에 반수 생활을 끝까지 버티고 좋은 결과를 얻을 수 있었어요.</v>
+        <v>멘탈 관리와 학습 계획 점검, 생활 패턴 관리 덕분에 반수 생활을 끝까지 버티고 좋은 결과를 얻을 수 있었어요.</v>
       </c>
       <c r="K238" t="str">
         <v>학습 계획</v>
@@ -9120,7 +9120,7 @@
 위대한 사람은 되지 못하더라도, 언젠가는 한 명의 어른으로 성장할 수 있도록 앞으로도 열심히 살아가겠습니다 :)</v>
       </c>
       <c r="J241" t="str">
-        <v>세세한 맞춤 학습 계획과 플래너 점검, 생활지도와 단어 테스트 덕분에 믿고 집중하며 공부할 수 있었어요.</v>
+        <v>세세한 맞춤 학습 계획과 플래너 점검, 생활 지도와 단어 테스트 덕분에 믿고 집중하며 공부할 수 있었어요.</v>
       </c>
       <c r="K241" t="str">
         <v>학습 계획</v>
@@ -9143,7 +9143,7 @@
         <v>특정 과목에서 어려운 부분이 있으면 그 부분을 어떻게 해야 잘 풀어낼 수 있는지에 대해 아이디어를 주셔서 좋았습니다. 또한 주기적으로 풀고 있는 교재들을 점검해 주시고 다음으로 풀 교재들을 추천해주신 것도 도움이 많이 되었습니다.</v>
       </c>
       <c r="F242" t="str">
-        <v>어떤 부분이 어려운지를 이야기 하면 멘토분들께서 본인이 풀어보셨던 문제집을 추천해주시기도 하는데 저는 이렇게 접한 교재로 도움을 정말 많이 받았습니다! 그리고 현재 풀고 있는 문제집을 말씀 드리면 어느정도로 교재의 장단점이나 어느정도로 학습해야하는지도 알려주시는 경우가 있어서 좋았어요</v>
+        <v>어떤 부분이 어려운지를 이야기 하면 멘토분들께서 본인이 풀어보셨던 문제집을 추천해주시기도 하는데 저는 이렇게 접한 교재로 도움을 정말 많이 받았습니다! 그리고 현재 풀고 있는 문제집을 말씀 드리면 어느정도로 교재의 장단점이나 어느정도로 학습해야 하는지도 알려주시는 경우가 있어서 좋았어요</v>
       </c>
       <c r="G242" t="str">
         <v>기본적으로 아침에 등원하자마자 핸드폰을 내고 그 이후에는 데스크 안쪽으로 폰 수거함이 들어가 있어서 딱히 핸드폰을 하고 싶다는 생각도 안 듭니다.. 핸드폰을 냈는지 안 냈는지를 크게 검사하는 느낌은 아니지만 본인이 공부를 할 의지가 있다면 핸드폰을 걷어가고 쉽게 핸드폰을 꺼낼 수 없는 환경인 게 도움이 될 수 있어요</v>
@@ -9286,13 +9286,13 @@
         <v>이투스 247 학습 상담은 자신의 현재 학습 수준과 문제점을 객관적으로 파악할 수 있게 해주어 매우 유용했다. 특히 개인별 맞춤 학습 계획을 세워주고, 시간 관리 방법과 과목별 공부 전략을 구체적으로 제시해 주어 학습 효율을 높이는 데 큰 도움이 되었다. 또한 지속적인 피드백을 통해 부족한 부분을 보완할 수 있어 성적 향상에 긍정적인 영향을 주었다. 또한 언제든 질문할 선생님이 있다는 점이 든든했다.</v>
       </c>
       <c r="F246" t="str">
-        <v>1:1 질의응답은 내가 이해하지 못한 부분을 바로 질문하고 해결할 수 있어 매우 유용했다. 수업에서는 놓치기 쉬운 세부 내용까지 자세히 설명을 들을 수 있었고, 나의 수준에 맞춘 설명 덕분에 이해도가 훨씬 높아졌다. 또한 즉각적인 피드백을 통해 잘못 알고 있던 개념을 바로잡을 수 있어 학습의 정확성과 효율성을 높이는 데 큰 도움이 되었다. 부담없이 질문할 수 있어 학습에 큰 도움이 되었다.</v>
+        <v>1:1 질의응답은 내가 이해하지 못한 부분을 바로 질문하고 해결할 수 있어 매우 유용했다. 수업에서는 놓치기 쉬운 세부 내용까지 자세히 설명을 들을 수 있었고, 나의 수준에 맞춘 설명 덕분에 이해도가 훨씬 높아졌다. 또한 즉각적인 피드백을 통해 잘못 알고 있던 개념을 바로잡을 수 있어 학습의 정확성과 효율성을 높이는 데 큰 도움이 되었다. 부담 없이 질문할 수 있어 학습에 큰 도움이 되었다.</v>
       </c>
       <c r="G246" t="str">
         <v>면학 분위기 속에서 감독이 이루어지니 자연스럽게 집중력이 높아지고 공부에 몰입할 수 있어 좋았다. 주변 모두가 학습에 집중하는 환경이라 흐트러지기 어려웠고, 감독이 있어 긴장감과 책임감도 생겨 스스로를 더 잘 통제할 수 있었다. 그 결과 불필요한 시간 낭비가 줄고 학습 효율이 크게 향상되었다. 또한 식사 후 식곤증에 빠지지 않게 관리해주시는게 큰 도움이 되었다.</v>
       </c>
       <c r="H246" t="str">
-        <v>이투스 구독 시스템은 다양한 강의를 한 번에 자유롭게 이용할 수 있어 매우 효율적이었다. 과목별로 필요한 강의를 추가 비용 부담 없이 선택해 들을 수 있어 학습 범위를 넓히는 데 도움이 되었고, 자신의 수준과 목표에 맞게 강의를 유연하게 조합할 수 있었다. 또한 반복 수강이 가능해 부족한 부분을 여러 번 복습하며 이해도를 높일 수 있어 학습 효과를 극대화할 수 있었다. 내가 원하는 부분만 듣고 싶었는데 비용 부담없이 여러 강의를 들을 수 있어서 좋았다.</v>
+        <v>이투스 구독 시스템은 다양한 강의를 한 번에 자유롭게 이용할 수 있어 매우 효율적이었다. 과목별로 필요한 강의를 추가 비용 부담 없이 선택해 들을 수 있어 학습 범위를 넓히는 데 도움이 되었고, 자신의 수준과 목표에 맞게 강의를 유연하게 조합할 수 있었다. 또한 반복 수강이 가능해 부족한 부분을 여러 번 복습하며 이해도를 높일 수 있어 학습 효과를 극대화할 수 있었다. 내가 원하는 부분만 듣고 싶었는데 비용 부담 없이 여러 강의를 들을 수 있어서 좋았다.</v>
       </c>
       <c r="I246" t="str">
         <v>선생님들께 진심으로 감사드립니다. 항상 학생 한 명 한 명에게 관심을 가지고 세심하게 지도해 주셔서 큰 힘이 되었습니다. 이해가 되지 않는 부분도 끝까지 설명해 주시고, 포기하지 않도록 격려해 주신 덕분에 꾸준히 공부할 수 있었습니다. 선생님들의 노력과 진심 덕분에 많이 성장할 수 있었고, 앞으로도 그 가르침을 잊지 않고 최선을 다하겠습니다. 다시 한 번 감사드립니다.</v>
@@ -9473,7 +9473,7 @@
         <v>수능공부를 처음 시작할 땐 막막했지만 천천히 따라가다보니 괜찮은 성과를 거두었다 생각합니다 한번에 이해를 못하고 몇번이고 되물은적도 많았는데 그럴때마다 차분히 다시 알려주셔서 도움이 많이 되었었습니다 감사합니다</v>
       </c>
       <c r="J251" t="str">
-        <v>선생님의 빈틈없는 감독과 졸음 관리 덕분에 순공시간이 늘어났고, 수능에서 현역 때보다 훨씬 만족스러운 결과를 얻었어요.</v>
+        <v>선생님의 빈틈없는 감독과 졸음 관리 덕분에 순공 시간이 늘어났고, 수능에서 현역 때보다 훨씬 만족스러운 결과를 얻었어요.</v>
       </c>
       <c r="K251" t="str">
         <v>졸음 관리</v>
@@ -9699,7 +9699,7 @@
         <v>어떻게 공부를 해야 할 지 모르던 저에게 올바른 방향을 제시해주시고 멘탈이 흔들릴 때나 지칠 때 잡아주시고 따뜻하게 대해주셔서 정말 감사했습니다. 덕분에 긴 수험 생활 잘 버틴 것 같습니다.!!</v>
       </c>
       <c r="J257" t="str">
-        <v>졸음지도 및 관리 덕분에 집중력을 유지하여, 순공시간 확보에 큰 도움이 되었어요.</v>
+        <v>졸음 지도 및 관리 덕분에 집중력을 유지하여, 순공 시간 확보에 큰 도움이 되었어요.</v>
       </c>
       <c r="K257" t="str">
         <v/>
@@ -9804,7 +9804,7 @@
         <v>감사했습니다 덕분에 좋은 대학생활 즐기고있어요 힘든일도이ㅛ았고 좋은일도 있었으나 결국 이겨내어 대학에 오게되었네요 이투스 관리감독 하시느라 힘드셨을텐데 앞으로도 힘내시길바랍니다!!</v>
       </c>
       <c r="J260" t="str">
-        <v>시기별로 상황에 맞춰 학습 방법을 추천해 주시고, 중간중간 점더고 해주셔서 취약 과목의 성적을 올리는데 정말 많은 도움이 됐어요!</v>
+        <v>시기별로 상황에 맞춰 학습 방법을 추천해 주시고, 중간중간 점검도 해주셔서 취약 과목의 성적을 올리는데 정말 많은 도움이 됐어요!</v>
       </c>
       <c r="K260" t="str">
         <v/>
@@ -9865,7 +9865,7 @@
         <v>한 강사의 커리큘럼만 추천하기보단 여러 강사들의 좋은 교재만 발췌해주시며 저의 스타일에 맞는 인강을 추천해주시고 매주 진도를 확인하시며 그때 그때 저에게 필요한 플랜을 짜주신 것이 너무 인상적이었습니다</v>
       </c>
       <c r="G262" t="str">
-        <v>평소 혼자서 공부할 때는 핸드폰 유혹에 넘어가며 순공시간이 길지 않았지만 학원에서 핸드폰을 압수하며 집중력이 흐트러지지 않도록 도와주시고 주변의 소식이나 연락도 잘 받을 수 없어 오로지 공부에만 집중할 수 있었습니다</v>
+        <v>평소 혼자서 공부할 때는 핸드폰 유혹에 넘어가며 순공 시간이 길지 않았지만 학원에서 핸드폰을 압수하며 집중력이 흐트러지지 않도록 도와주시고 주변의 소식이나 연락도 잘 받을 수 없어 오로지 공부에만 집중할 수 있었습니다</v>
       </c>
       <c r="H262" t="str">
         <v>매달 시험을 치르며 풀모의고사를 시간대로 풀 수 있는 시간대가 주어져 실전에서 도전해보지 못한 여러 방법을 적용해보며 모의고사속에서 저만의 스킬을 만들 수 있었고 다른 학생들과 같이 보며 등급과 성적을 볼 수 있어 동기부여가 되었습니다</v>
@@ -10004,7 +10004,7 @@
       <c r="E266" t="str" xml:space="preserve">
         <v xml:space="preserve">독재학원에서의 코칭 시스템은 단순한 학습 관리 수준을 넘어, 수험 생활 전반을 안정적으로 유지할 수 있도록 돕는 장치라는 점에서 특히 유용했습니다. 그중에서도 생활상담 중심의 멘토링은 제가 공부를 지속할 수 있게 만든 핵심 요소였습니다._x000d_
 _x000d_
-우선, 수험 생활은 장기간 이어지기 때문에 집중력이나 의지가 일정하게 유지되기 어렵습니다. 실제로 하루 공부량보다 더 중요한 것은 ‘흐름을 유지하는 것’인데, 생활상담을 통해 이 흐름이 무너지지 않도록 지속적으로 점검받을 수 있었습니다. 예를 들어, 수면 패턴이 흐트러지거나 식사 시간이 불규칙해질 때 이를 바로 잡아주는 피드백을 받을 수 있었고, 이는 곧 학습 효율의 회복으로 이어졌습니다._x000d_
+우선, 수험 생활은 장기간 이어지기 때문에 집중력이나 의지가 일정하게 유지되기 어렵습니다. 실제로 하루 공부량보다 더 중요한 것은 ‘흐름을 유지하는 것’인데, 생활상담을 통해 이 흐름이 무너지지 않도록 지속적으로 점검받을 수 있었습니다. 예를 들어, 수면 패턴이 흐트러지거나 식사 시간이 불규칙해질 때 이를 바로잡아주는 피드백을 받을 수 있었고, 이는 곧 학습 효율의 회복으로 이어졌습니다._x000d_
 _x000d_
 또한, 단순히 공부 계획만을 점검하는 것이 아니라 개인의 상태를 함께 고려해주는 점이 인상적이었습니다. 슬럼프가 오거나 잡생각이 많아질 때, 이를 방치하지 않고 상담을 통해 원인을 짚어주고 해결 방향을 제시해 주었기 때문에 감정적인 소모를 줄일 수 있었습니다. 특히 재수 기간에는 스스로를 객관적으로 바라보기 어려운데, 코치 선생님과의 대화를 통해 현재 상태를 정리하고 다시 집중할 수 있는 계기를 만들 수 있었습니다._x000d_
 _x000d_
@@ -10157,7 +10157,7 @@
         <v>반수생</v>
       </c>
       <c r="E269" t="str">
-        <v>학습 상담을 진행하면서 공부 방향을 정하고 그에 맞춰서 공부하면서 열심히 공부 할 수 있었던것 같다. 당일 할 일을 정하여 그것만큼은 꼭 해결하려한 것이 공부에 큰 도움이 됐다고 생각했다.</v>
+        <v>학습 상담을 진행하면서 공부 방향을 정하고 그에 맞춰서 공부하면서 열심히 공부할 수 있었던것 같다. 당일 할 일을 정하여 그것만큼은 꼭 해결하려한 것이 공부에 큰 도움이 됐다고 생각했다.</v>
       </c>
       <c r="F269" t="str">
         <v>평소에 계획을 세우고 공부하기보다는 그냥 마구잡이로 공부를 하는 성향이 있었다. 하지만 계획을 세우면서 공부하니 좀 더 효과적으로 공부할 수 있었던 것 같다. 계획을 세우는 습관을 들임으로써 앞으로도 나에게 큰 도움이 될 것 같다고 생각이 든다.</v>
@@ -10201,7 +10201,7 @@
         <v>핸드폰을 걷는 것도 몰론 중요하지만 그런 것 보다도 유투브를 상요하지 못 하는 것이 중요 했습니다. 만약 유투브를 사용 할 수 있었으면 헤이해져 공부에 전념하지 못 했을 텐데 사용하지 못하게 막음으로 써 공부에 전념해 좋은 성과를 걷을 수 있었습니다</v>
       </c>
       <c r="H270" t="str">
-        <v>이투스 전국 모의고사의 난이도를 떠나서 모의고사를 매월 침으로 써 나의 현재 실략을 점검하고 못보면 그로인한 자극을 얻고 잘 보면 더 잘해 야 겠다는 자극을 얻으면서 더욱 실력 향상을 위해 객관적으로 공부 할 수 있었습니다</v>
+        <v>이투스 전국 모의고사의 난이도를 떠나서 모의고사를 매월 침으로 써 나의 현재 실략을 점검하고 못보면 그로인한 자극을 얻고 잘 보면 더 잘해 야 겠다는 자극을 얻으면서 더욱 실력 향상을 위해 객관적으로 공부할 수 있었습니다</v>
       </c>
       <c r="I270" t="str">
         <v>배은지 선생님 제가 비록 재수생 같지도 않게 직장인 처럼 빨간날 마다 쉬고 주말에도 잘 나오지 않았지만 포기하지 않고 3주 마다 상담을 나눠 주시며 대회 상대가 돼줬던 것이 저의 재수 생활에 큰 활력이 됐습니다</v>
@@ -10236,7 +10236,7 @@
         <v>앞에서 말했듯이 쉬는시간에 피곤해서 자는 경우가 많은데 스카에서 자게되면 깨워줄 사람의 부재로 너무 오래 잠들까 걱정돼서 맘편히 못자는데 이투스에선 선생님들이 돌아가면서 깨워주셔서 맘편히 깊게 잠들 수 있어요. 또한 수업시간에 졸 때도 깨워주시고 한 번씩 잠 깨라고 사탕도 주셨는데 너무 도움이 많이 됐습니다.</v>
       </c>
       <c r="H271" t="str">
-        <v>정승제 선생님같이 좋은 선생님이신데 이투스를 구독하거나 단일 강의는 듣기엔 돈이 아까워서 못듣는 이투스 강사들을 부담없이 필요한 부분만 들을 수 있는게 좋았고, 그만큼 들을 수 있는 강사가 늘어난거니 그 강사의 모의고사나 엔제 등을 더 잘 접할 수 있게 됐습니다.</v>
+        <v>정승제 선생님같이 좋은 선생님이신데 이투스를 구독하거나 단일 강의는 듣기엔 돈이 아까워서 못듣는 이투스 강사들을 부담 없이 필요한 부분만 들을 수 있는게 좋았고, 그만큼 들을 수 있는 강사가 늘어난거니 그 강사의 모의고사나 엔제 등을 더 잘 접할 수 있게 됐습니다.</v>
       </c>
       <c r="I271" t="str" xml:space="preserve">
         <v xml:space="preserve">선생님들 덕분에 재밌는 대학생활 하고 있고 잊지 못할 추억 가져가는것 같아요. 대치동으로 옮겨서 가면 뭔가 방해될까봐 못갔는데 다음에 시간나면 한번 가볼게요…ㅎ_x000d_
@@ -10298,7 +10298,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E273" t="str">
-        <v>내가 지금 하고 있는 공부법이 효율적인지 같이 고민해주시고 인강 사이트를 활용해서 공부하고 있다면 해당 강사에 대한 구체적인 로드맵도 함께 구상하는 시간을 가져서 도움이 많이 됐어요. 그리고 조교 선생님만의 공부법과 팁들을 많이 전수해주셔서 유익하게 공부방법응 계획할 수 있었어요!</v>
+        <v>내가 지금 하고 있는 공부법이 효율적인지 같이 고민해주시고 인강 사이트를 활용해서 공부하고 있다면 해당 강사에 대한 구체적인 로드맵도 함께 구상하는 시간을 가져서 도움이 많이 됐어요. 그리고 조교 선생님만의 공부법과 팁들을 많이 전수해주셔서 유익하게 공부 방법응 계획할 수 있었어요!</v>
       </c>
       <c r="F273" t="str">
         <v>수학 같은 경우는 해설지를 봐도 이해가 안 됐던 경우가 많았는데, 직접 문제를 함께 살펴보고 차근차근 설명해주신 점이 맘에 들었습니다. 또한 모르는 문제에 대해 바로 알려주는 것이 아니라 어떠한 점에서 막혔고 잘못된 습관이 있지는 않은지 점검해주신 후 능동적으로 문제릉 풀 수 있도록 도와주신 덕분에 스스로 문제를 풀어내는 능력을 기를 수 있었습니다!</v>
@@ -10664,7 +10664,7 @@
         <v>인강과 교재를 선택하면서 이전에는 많은 인강과 교재로 학습을 했다면 멘토 선생님의 도움으로 나에게 알맞은 인강과 교재로, 또한 그 인강과 교재에 맞는 학습 방법으로 학습할 수 있어 도움을 받음.</v>
       </c>
       <c r="G283" t="str">
-        <v>아무래도 인강을 수강하면서 태블릿으로 수강을 하다 보니 당연히 인터넷과 같은 다른 곳으로 빠질 수 있는데, 인터넷 방화벽으로 학습 외 사이트에 접속을 막아 놓아 더욱 학습에 집중 할 수 있었음.</v>
+        <v>아무래도 인강을 수강하면서 태블릿으로 수강을 하다 보니 당연히 인터넷과 같은 다른 곳으로 빠질 수 있는데, 인터넷 방화벽으로 학습 외 사이트에 접속을 막아 놓아 더욱 학습에 집중할 수 있었음.</v>
       </c>
       <c r="H283" t="str">
         <v>수능 영어를 공부하면서 제일 중요한 것은 영어 단어 암기라고 생각하는데 VOCA 테스트로 매일 아침 영단어 테스트로 영어 단어를 얼마나 암기했는지 점검 할 수 있어 지속적인 영어 학습에 큰 도움을 받음.</v>
@@ -10845,7 +10845,7 @@
         <v>저는 학원에 있는 동안, 거의 매일 매리트 문제를 풀었는데, 이것이 가장 큰 힘을 발휘한 것은 영어였습니다. 저는 영어는 학원에서 주는 실모 문제와 매리트만 풀었는데, 매리트는 제가 영어 문제를 푸는 데 감을 잊지 않도록 도와주었습니다. 또한 영어 단어를 와울 때 매리트를 사용하는 것은 매우 유용했습니다.</v>
       </c>
       <c r="I288" t="str">
-        <v>선생님들, 제가 학원에 있는 동안 제게 많은 것들을 알려주셔서 수능을 준비하는데 큰 도움을 주신 것에 진심으로 감사드립다. 학교에 다니지 않았던 저에게 이투스 247학원에서 공부하고 선생님들의 수업을 들었던 시간은 저에게 참 특별한 시간이었습니다. 다시 한 번 더 진심으로 감사드립니다.</v>
+        <v>선생님들, 제가 학원에 있는 동안 제게 많은 것들을 알려주셔서 수능을 준비하는데 큰 도움을 주신 것에 진심으로 감사드립니다. 학교에 다니지 않았던 저에게 이투스 247학원에서 공부하고 선생님들의 수업을 들었던 시간은 저에게 참 특별한 시간이었습니다. 다시 한 번 더 진심으로 감사드립니다.</v>
       </c>
       <c r="J288" t="str">
         <v>학습 슬럼프에 빠질 뻔한 적이 있었는데 그때마다 담임 선생님과 상담을 하며 다시 동기부여를 받고 공부할 수 있었습니다.</v>
@@ -10941,10 +10941,10 @@
         <v>매주 담임 선생님과의 학습 상담을 과목별 맞춤 전략을 세우며 지속적으로 변하는 저의 학습 진행상황에 맞도록 공부할 수 있는 점이 좋았습니다. 또한 자주 치르는 실전 모의고사에서의 피드백도 매번 진행되어 실전적 측면에서의 도움도 많이 받을 수 있었습니다.</v>
       </c>
       <c r="F291" t="str">
-        <v>저는 고3 때 정시를 준비하던 학생이었습니다. 전과목의 성적을 모두 챙기는 것이 중요한 정시 전형에서, 제가 흥미를 느끼는 과목만을 선택적으로 공부하는 저의 학습 패턴은 실패요인이었습니다. 그리고 이투스247 학원을 다니며 이를 매주 진행되는 일주일 간의 학습 일정 조정을 통해 극복할 수 있었고, 모든 과목을 골고루 공부하는데 큰 도움이 되었습니다.</v>
+        <v>저는 고3 때 정시를 준비하던 학생이었습니다. 전과목의 성적을 모두 챙기는 것이 중요한 정시 전형에서, 제가 흥미를 느끼는 과목만을 선택적으로 공부하는 저의 학습 패턴은 실패요인이었습니다. 그리고 이투스247 학원을 다니며 이를 매주 진행되는 일주일 간의 학습 일정 조정을 통해 극복할 수 있었고, 모든 과목을 고루 공부하는데 큰 도움이 되었습니다.</v>
       </c>
       <c r="G291" t="str">
-        <v>아침8시부터 밤12시까지 오랜시간의 공부를 특별한 여가생활 없이 매일 반복해낸다는 것은 저에게 정신적,체력적으로 상당한 부담이 되었습니다. 그렇기에 피로해진 상태의 저는 늘 졸음과 싸우고는 했습니다. 이때 이투스247의 졸음지도 및 관리는 집중력을 유지하여 공부하는 순공부 시간 확보에 큰 도움이 되었습니다.</v>
+        <v>아침8시부터 밤12시까지 오랜시간의 공부를 특별한 여가생활 없이 매일 반복해낸다는 것은 저에게 정신적,체력적으로 상당한 부담이 되었습니다. 그렇기에 피로해진 상태의 저는 늘 졸음과 싸우고는 했습니다. 이때 이투스247의 졸음 지도 및 관리는 집중력을 유지하여 공부하는 순공부 시간 확보에 큰 도움이 되었습니다.</v>
       </c>
       <c r="H291" t="str">
         <v>우선, 매일 등원과 동시에 아침에 풀어야하는 국어 지문 1지문은 평가원 및 교육청 기출을 자주 접할 수 있도록 도와주었을 뿐 아니라 하루의 집중력을 긴 글을 통해 깨워주어 효율적의 학습의 시작을 마련해주었습니다. 그에 더해 매일 치러지는 영단어시험은 수능에 필요한 영단어들을 반복적으로 학습할 수 있도록 해주어 어휘력을 기르는데 큰 도움을 주었습니다.</v>
@@ -11008,10 +11008,10 @@
         <v>반수생</v>
       </c>
       <c r="E293" t="str">
-        <v>나의 상황에 맞는 학습플랜과 필요힌 공부방법을 알려주셨고, 더 구체적으로 강의 수강 진도도 체크해주시고 추천 강의도 알려주셔서 맞춤 공부하기 유용했습니다. 어려운 단원이나 특히 부족한 부분에 대해 보완할 수 있는 점을 정확히 알려주셨습니다.</v>
+        <v>나의 상황에 맞는 학습플랜과 필요힌 공부 방법을 알려주셨고, 더 구체적으로 강의 수강 진도도 체크해주시고 추천 강의도 알려주셔서 맞춤 공부하기 유용했습니다. 어려운 단원이나 특히 부족한 부분에 대해 보완할 수 있는 점을 정확히 알려주셨습니다.</v>
       </c>
       <c r="F293" t="str">
-        <v>나의 성적과 학업 목표에 따라 시간단위로  쪼개서 구체적이고 효율적으로 공부할 수 있도록 지도해주신 점이 좋았습니다. 특히 부족한 공부를 미루고 하고 싶은 공부 위주로 공부하는 습관이 있었는데 학원에서 준 계획표대로 실천하도록 노력했더니 균형있는 공부를 할 수 있었습니다.</v>
+        <v>나의 성적과 학업 목표에 따라 시간단위로  쪼개서 구체적이고 효율적으로 공부할 수 있도록 지도해주신 점이 좋았습니다. 특히 부족한 공부를 미루고 하고 싶은 공부 위주로 공부하는 습관이 있었는데 학원에서 준 계획표대로 실천하도록 노력했더니 균형 있는 공부를 할 수 있었습니다.</v>
       </c>
       <c r="G293" t="str">
         <v>공부를 방해하는 직접적인 요인을 강제적으로 제거함으로써 공부에만 오직 집중할 수 있는 환경이 만들어진 점이 가장 좋았습니다. 스터니카페나 다른 학원에서보다 더 통제적으로 핸드폰과 테블릿 사용을 조절할 수 있어서 공부에 집중하는데 효과적이었습니다.</v>
@@ -11228,7 +11228,7 @@
 기숙학원은 가족, 친구들로부터 떨어져서 혼자 지내야하는 곳이기에 멘탈적인 부분에서도 담임 선생님께 의지를 많이 했습니다.</v>
       </c>
       <c r="G299" t="str" xml:space="preserve">
-        <v xml:space="preserve">스마트폰은 통제하기 어렵고 가장 큰 방해가 되는 요인인데 아예 휴대폰을 제출하였기에 집중도에 큰 도움을 받았습니다. 테블릿 피시도 제한적으로, 정말 공부에 필요할 때만 사용할 수 있었기에 순공시간 확보에 유용했습니다. _x000d_
+        <v xml:space="preserve">스마트폰은 통제하기 어렵고 가장 큰 방해가 되는 요인인데 아예 휴대폰을 제출하였기에 집중도에 큰 도움을 받았습니다. 테블릿 피시도 제한적으로, 정말 공부에 필요할 때만 사용할 수 있었기에 순공 시간 확보에 유용했습니다. _x000d_
 개인적으로 음악 듣기를 포기하기가 어려웠는데 학원에서 제한해주다보니 마음 잡고 공부했던 것 같습니다.</v>
       </c>
       <c r="H299" t="str">
@@ -11652,7 +11652,7 @@
         <v>N수생</v>
       </c>
       <c r="E311" t="str">
-        <v>내가 부족한 과목을 어떻게 얼마나 공부해야하는지 방향을 잡아주셨고 , 정신적으로 힘들 때 응원과 격려의 말씀을 보내주셨습니다. 모의고사 풀이를 보고서 어떤 유형이 취약하고 무슨 문제를 풀어야 보완될지 알려주셨습니다.</v>
+        <v>내가 부족한 과목을 어떻게 얼마나 공부해야 하는지 방향을 잡아주셨고 , 정신적으로 힘들 때 응원과 격려의 말씀을 보내주셨습니다. 모의고사 풀이를 보고서 어떤 유형이 취약하고 무슨 문제를 풀어야 보완될지 알려주셨습니다.</v>
       </c>
       <c r="F311" t="str">
         <v>플래너 관리를 통해 규칙적인 학원 생활을 만들 수 있었고, 모의고사에서 여러 루틴을 시도해 저에게 맞는 루틴을 찾을 수 있었습니다. 또한 , 학습 방향이 맞는지 불안할 때 객관적인 시선으로 바라볼 수 있어서 좋았습니다.</v>
@@ -11728,7 +11728,7 @@
         <v>원래 현역 고3 때 공부할때는 계획 짜는것이 의미 없다고 생각되어서 플래너를 따로 작성하지 않았습니다. 하지만 재수를 하면서 이투스학원에서 플래너를 무상으로 지급을 해주는데 매일 공부를 다하고 집에 가기전에 다음날 무엇을 할지 플래너를 작성해놓으면 다음날 학원에 왔을때 목표치가 설정되어 있어서 좀 더 공부하는데 수월했던것 같습니다.</v>
       </c>
       <c r="G313" t="str">
-        <v>핸드폰이 자기 수중에 있게 되면 공부하다가 연락이 오거나 알람이 떴을 때  어쩔수 없이 보다가 시간을 허비하고 집중력이 깨지는 경우가 많습니다. 이투스에서는 핸드폰을 아침시간 출석과 동시에 걷기때문에 핸드폰의 유혹에서 벗어나 좀 더 유용한 환경에서 공부 할수가 있었습니다.</v>
+        <v>핸드폰이 자기 수중에 있게 되면 공부하다가 연락이 오거나 알람이 떴을 때  어쩔수 없이 보다가 시간을 허비하고 집중력이 깨지는 경우가 많습니다. 이투스에서는 핸드폰을 아침시간 출석과 동시에 걷기때문에 핸드폰의 유혹에서 벗어나 좀 더 유용한 환경에서 공부할수가 있었습니다.</v>
       </c>
       <c r="H313" t="str">
         <v>재수를 하면서 수 많은 기출들과 모의고사들을 풀게 되는데 막판으로 갈수록 양질의 모의고사들을 얻기가 어려워집니다. 1달~2달에 한 번씩 치뤄지는 이투스 모의고사로 자기의 요즘 컨디션과 얼마나 성장했는지 체크도 하고 또 피드백까지 할수 있었던게 굉장한 도움이 되었던거 같습니다. 또 퀄리티 또한 입증이 되있기에 이투스에서 현장감을 느끼며 풀면서 실전성도 높일수가 있습니다.</v>
@@ -11827,7 +11827,7 @@
         <v>반수생</v>
       </c>
       <c r="E316" t="str">
-        <v>과목별로 제 수준에 맞게 공부방법을 알려주신게 도움이 많이 되었습니다 예를 들어 수학과목에서 저는 항상 시험시간이 부족했어서 문제를 읽어보지도 못하고 틀리는 문제가 1,2개씩 있었습니다 이럴때 시험시간을 보다 효율적으로 사용하기 위해선 계산하고 식을 쓰는 시간을 줄이고 문제에 대해 충분히 생각해본 후 필요한 계산만 간략히 하는 전략을 추천해주셨습니다</v>
+        <v>과목별로 제 수준에 맞게 공부 방법을 알려주신게 도움이 많이 되었습니다 예를 들어 수학과목에서 저는 항상 시험시간이 부족했어서 문제를 읽어보지도 못하고 틀리는 문제가 1,2개씩 있었습니다 이럴때 시험시간을 보다 효율적으로 사용하기 위해선 계산하고 식을 쓰는 시간을 줄이고 문제에 대해 충분히 생각해본 후 필요한 계산만 간략히 하는 전략을 추천해주셨습니다</v>
       </c>
       <c r="F316" t="str">
         <v>학원에서 치른 모의고사 점수 1등부터 10등까지는 복도에 게시되고 장학금도 주셨는데 그것이 공부하는것에 큰 동기부여가 되서 더 열심히 공부하고 싶어졌습니다 또 제 성적이 게시되면 저가 지금 공부를 잘하고 있다고 확인받는 느낌이 들어 자신감이 생겼습니다</v>
@@ -11969,7 +11969,7 @@
         <v>반수생</v>
       </c>
       <c r="E320" t="str">
-        <v>이투스247을 다니기 전에는 혼자서 생활 관리가 안돼서 핸드폰을 하루종일 붙잡고 있었고 순공시간이 적었습니다. 생활 관리가 이투스를 통해 된 후부터 순공시간이 늘어났고 성적이 오르기 시작했습니다.</v>
+        <v>이투스247을 다니기 전에는 혼자서 생활 관리가 안돼서 핸드폰을 하루종일 붙잡고 있었고 순공 시간이 적었습니다. 생활 관리가 이투스를 통해 된 후부터 순공 시간이 늘어났고 성적이 오르기 시작했습니다.</v>
       </c>
       <c r="F320" t="str">
         <v>학습 계획을 혼자서 공부할때는 세우지않고 그때그때 원하는대로 공부하다보니 진도가 잘 나가지 않고 하는 과목만 계속하는 문제가 있었습니다. 플래너를 통해 각 과목별로 시간을 정해서 하다보니 모든과목의 성적을 올릴수 있어서 좋았습니다</v>
@@ -11981,7 +11981,7 @@
         <v>재수생특성상 현역때와 다르게 교육청모의고사를 치지 못하고 6,9,수능밖에 없어서 실전경험이 현역에 비해 떨어질수 있다고 생각하는데 이투스모의고사를 통해 현역보다도 많은 모의고사를 치면서 실전감각을 올릴수 있었습니다</v>
       </c>
       <c r="I320" t="str">
-        <v>생활지도선생님과 질의응답선생님 둘다 정말 감사합니다. 이투스247의 체계적인 관리와 편한 질의응답 시스템에 정말 많은 도움을 받았고 덕분에 원하던 의대에 합격해 정말 재밌게 학교생활 하고있습니다!</v>
+        <v>생활 지도선생님과 질의응답선생님 둘다 정말 감사합니다. 이투스247의 체계적인 관리와 편한 질의응답 시스템에 정말 많은 도움을 받았고 덕분에 원하던 의대에 합격해 정말 재밌게 학교생활 하고있습니다!</v>
       </c>
       <c r="J320" t="str">
         <v>평가원 외에도 모의고사를 매달 실시해 실전 경험을 많이 쌓을 수 있어서 수능 당일에도 많은 도움이 됐어요!</v>
@@ -12405,7 +12405,7 @@
         <v>일반 독서실이나 관리형 독서실들과는 다르게 핵심과목인 국어,영어,수학 전공자 선생님들께서 상주하고 계셔서 문제를 풀다가 막힘이 오거나 특정과목에 대한 상담이 필요할때 즉각적인 질의응답을 통한 학습이 가능하다는 점이 가장 큰 장점이였다. 온라인 강의와 사이트를 이용하다보면 강의와 개념, 문제들에 대한 질문을 qna 게시판을 통해서만 질문이 가능한데 이는 시간도 오래걸리고 대면으로 질문하는것이 아니기에 한계가 존재했었다. 또한 이투스 247 목동 졸업생들이 멘토로 근무를 하여 특정 탐구 과목들에 대한 피드백과 질문, 조언들을 얻을 수 있다는 점에서 이투스 247 목동만의 독보적이고 차별적인 시스템이다.</v>
       </c>
       <c r="G332" t="str">
-        <v>공부를 하는 학생 입장에서 독학재수학원을 생각할때 중요시하게 고려하는 요소가 면학 분위기 입니다. 그러한점에서 목동 이투스 247은 다양한 시스템을 통한 최고의 면학 분위기를 제공해주었습니다. 우선 매너타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다같이 집중 할 수 있는 공부 환경을 제공해줍니다. 또한 학생들이 학습중 자지 않도록 상시로 감독 선생님께서 자습실을 비롯한 공용학습 공간까지 꼼꼼히 돌아다니시며 모든 학생이 열심히 공부를 할 수 있게 도와주십니다.</v>
+        <v>공부를 하는 학생 입장에서 독학재수학원을 생각할때 중요시하게 고려하는 요소가 면학 분위기 입니다. 그러한점에서 목동 이투스 247은 다양한 시스템을 통한 최고의 면학 분위기를 제공해주었습니다. 우선 매너타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다같이 집중할 수 있는 공부 환경을 제공해줍니다. 또한 학생들이 학습중 자지 않도록 상시로 감독 선생님께서 자습실을 비롯한 공용학습 공간까지 꼼꼼히 돌아다니시며 모든 학생이 열심히 공부를 할 수 있게 도와주십니다.</v>
       </c>
       <c r="H332" t="str">
         <v>목동 이투스 247점에서는 단어테스트반을 모집하여 매주 영단어 테스트를 봅니다. 학생들이 가장 귀찮아하고 소홀히하는 영단어 외우기를 같은 학생들과 함께 매주 테스트를 보며 매주 빼먹지 않게 외우게된다는 장점이 있습니다.</v>
@@ -12414,7 +12414,7 @@
         <v>항상 입시 스트레스로와 몸 건강으로 인해 학원에게 피해를 많이 끼쳤지만 그럼에도 불구하고 항상 격려해주시고 힘을 내게 도와주셔서 덕분에 끝까지 입시를 마칠 수 있었습니다. 모두 선생님들 덕분입니다. 제 입시에서 이투스 247 선생님들을 만난것이 가장 큰 행운이였습니다 감사합니다..!</v>
       </c>
       <c r="J332" t="str">
-        <v>매너 타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다같이 집중 할 수 있는 공부 환경을 제공해주셨어요.</v>
+        <v>매너 타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다같이 집중할 수 있는 공부 환경을 제공해주셨어요.</v>
       </c>
       <c r="K332" t="str">
         <v/>
@@ -12539,7 +12539,7 @@
         <v>N수생</v>
       </c>
       <c r="E336" t="str">
-        <v>모의고사 시험지 분석을 통해, 자신이 어떤 단원, 무엇이 부족한지를  알려주시며, 자신의 성적에 따라 어떤 것에 집중해야하는지를 알려주셔서 도움이 되었습니다. 또한 상담이 필요할 때 원하는 만큼 상담할 수 있어서 심리적 불안감을 줄일 수 있었습니다.</v>
+        <v>모의고사 시험지 분석을 통해, 자신이 어떤 단원, 무엇이 부족한지를  알려주시며, 자신의 성적에 따라 어떤 것에 집중해야 하는지를 알려주셔서 도움이 되었습니다. 또한 상담이 필요할 때 원하는 만큼 상담할 수 있어서 심리적 불안감을 줄일 수 있었습니다.</v>
       </c>
       <c r="F336" t="str">
         <v>처음 기숙학원에 들어왔을 때 무엇을 할지 몰라서 일단 제가 좋아하는 과목을 위주로 공부를 해 각 과목 점수의 편차가 컸습니다.그러나 선생님께서 플래너를 작성하고 어떻게 활용해야 하는 지를 알려주고 난 후, 과목 불균형을 해소하여 시험을 볼때 대부분 과목들이 비슷한 등급을 받았습니다. 또한 자신이 어디까지 공부했고 어디가 부족한지 표시하여 그다음날 무엇을 더집중적으로 하고, 또 무엇을 보충할지 등 더 체계적으로 공부할 수 있었습니다.</v>
@@ -12548,7 +12548,7 @@
         <v>제가 제일 공부할때 방해되는것이 인터넷 이였습니다. 공부를 하다가도 집중이 안되면 핸드폰을 보며 유튜브를 들어가거나 게임을 하기도 했었습니다. 그러나 이투스 기숙학원에 들어오고나서 핸드폰을 걷고 학원 태블릿을 이용하여 강의만 들을 수 있어서  처음에는 그게 불만이였지만 나중에는 유튜브나 인터넷에 못들어가니 공부에 더 집중할 수 있었습니다.</v>
       </c>
       <c r="H336" t="str">
-        <v>제가 궁금한건 어떻게 공부해야 할지 였습니다. 모의고사를 보고나서 이걸 어떻게 분석해야하는지가 문제였는데 이투스 모의고사를 보고 어디 단원을 공부해야하고 어디가 부족하고 다른사람들은 어느정도 맞췄는지, 그리고 이점수로 어느 대학에 진학할수 있는지를 알려주어서 큰 도움이 되었습니다.</v>
+        <v>제가 궁금한건 어떻게 공부해야 할지 였습니다. 모의고사를 보고나서 이걸 어떻게 분석해야 하는지가 문제였는데 이투스 모의고사를 보고 어디 단원을 공부해야하고 어디가 부족하고 다른사람들은 어느정도 맞췄는지, 그리고 이점수로 어느 대학에 진학할수 있는지를 알려주어서 큰 도움이 되었습니다.</v>
       </c>
       <c r="I336" t="str">
         <v>고3 수능때 평균 5등급 학생이였고, 공부를 포기했습니다. 그러나 기숙학원에 들어오고   점수가 달라졌습니다. 뭐 하나 잘하는게 없는 제가 서서히 점수가 올라가는것이 신기했었습니다. 수능때 국어가 아쉬운 점수가나왔지만, 제가 꿈도 못꾼 대학에 진학하게 도와주셔서 감사합니다!</v>
@@ -12785,7 +12785,7 @@
         <v>N수생</v>
       </c>
       <c r="E343" t="str">
-        <v>어떻게 하면 수능에서 고득점을 받을 수 있을지 구체적인 공부법들을 제안해주셨다. 공부를 하다보면 자칫 객관성을 잃고 잘못된 방향으로 빠질 수도 있는데, 매일 밴드로 적절한 공부방법과 동기부여를 올려주셔서 1년 동안 제대로 된 방향으로 공부할 수 있었다. 또한 수능이라는 시험에 대한 이해도를 높여주셔서 나중에는 스스로 올바른 공부방법을 찾아나갈 수 있었다.</v>
+        <v>어떻게 하면 수능에서 고득점을 받을 수 있을지 구체적인 공부법들을 제안해주셨다. 공부를 하다보면 자칫 객관성을 잃고 잘못된 방향으로 빠질 수도 있는데, 매일 밴드로 적절한 공부 방법과 동기부여를 올려주셔서 1년 동안 제대로 된 방향으로 공부할 수 있었다. 또한 수능이라는 시험에 대한 이해도를 높여주셔서 나중에는 스스로 올바른 공부 방법을 찾아나갈 수 있었다.</v>
       </c>
       <c r="F343" t="str">
         <v>온라인으로 미리 예약한 후 질의응답하는 시스템을 통해 1분 1초가 아까운 수험 생활에서 시간을 허비할 일이 없어서 좋았다. 선생님들 또한 질문을 가지고 가면 열정적으로 답변해주셨으며, 문제 풀이 뿐만 아니라 학습 상담까지 친절하게 해주셨다.</v>
@@ -12828,7 +12828,7 @@
 또한 주기적으로 선생님과 플래너 상담을 진행하며 학습이 계획대로 이루어지고 있는지 점검하고, 진도가 늦어지거나 예상보다 빠른 경우에는 상황에 맞는 추가 학습 솔루션을 제공받을 수 있었습니다. 그 결과 매일 평균 13시간의 순공 시간을 달성할 수 있었고, 그 안에서 저에게 맞는 학습 타임테이블을 구축해 더욱 효율적이고 집중도 높은 공부를 이어갈 수 있었습니다.</v>
       </c>
       <c r="G344" t="str" xml:space="preserve">
-        <v xml:space="preserve">혼자 공부할 때는 집중력이 흐트러지거나 졸음으로 인해 공부를 중단하는 경우가 많았고, 일반 독서실에서는 면학 분위기가 잘 유지되지 않아 어려움을 느끼기도 했습니다. 그러나 이투스247에서는 선생님께서 자습실을 지속적으로 관리하며 면학 분위기를 철저히 유지해주셨고, 졸거나 집중이 흐트러질 때에도 바로 잡아주셔서 다시 공부에 몰입할 수 있었습니다._x000d_
+        <v xml:space="preserve">혼자 공부할 때는 집중력이 흐트러지거나 졸음으로 인해 공부를 중단하는 경우가 많았고, 일반 독서실에서는 면학 분위기가 잘 유지되지 않아 어려움을 느끼기도 했습니다. 그러나 이투스247에서는 선생님께서 자습실을 지속적으로 관리하며 면학 분위기를 철저히 유지해주셨고, 졸거나 집중이 흐트러질 때에도 바로잡아주셔서 다시 공부에 몰입할 수 있었습니다._x000d_
 또한 지정된 개인 좌석뿐만 아니라 오픈존, 스탠딩 책상 등 다양한 학습 공간이 마련되어 있어, 집중이 떨어질 때는 환경을 바꿔가며 효율적으로 공부할 수 있었습니다. 더불어 수능과 동일한 시간표에 맞춰 생활 패턴을 관리할 수 있어 불필요한 시간 낭비 없이 학습에 집중할 수 있었습니다. 이러한 생활 관리 시스템 덕분에 자습실 전체에 열심히 공부하는 분위기가 형성되었고, 그 속에서 저 역시 자연스럽게 동기부여를 받아 더욱 꾸준히 학습할 수 있었습니다.</v>
       </c>
       <c r="H344" t="str" xml:space="preserve">
@@ -12951,7 +12951,7 @@
         <v>독학재수에서의 가장 큰 단점이 자신이 어느정도까지 공부를 했는지, 어느정도에 위치해 있는지, 어떤 점이 잘못되었는지 를 스스로 알아차리기 힘든 것인데, 성적 레포팅과 피드백을 거치면서 내가 어떤 잘못된 공부 방법을 가지고 있는지 내가 이때까지 성장했는지를 제 3자의 눈으로 볼 수 있었다는 점이 가장 좋았습니다.</v>
       </c>
       <c r="G347" t="str">
-        <v>순공시간을 확보하고 높은 집중력을 가지고 공부를 하기 위해서는 어쩔 수 없이 졸음과 싸워야하는데 혼자서는 졸음을 이겨내는데 한계가 있다고 생각해서 졸음관리라 가장 유용했습니다. 선생님들의 시선을 의식해서라도 더 열심히하려하고 더 졸지 않으려고 노력하면서 점차 생활 패턴도 맞춰지고 수험 생활을 보낼수록 졸음을 이겨내는게 쉬워졌기 때문입니다.</v>
+        <v>순공 시간을 확보하고 높은 집중력을 가지고 공부를 하기 위해서는 어쩔 수 없이 졸음과 싸워야하는데 혼자서는 졸음을 이겨내는데 한계가 있다고 생각해서 졸음관리라 가장 유용했습니다. 선생님들의 시선을 의식해서라도 더 열심히하려하고 더 졸지 않으려고 노력하면서 점차 생활 패턴도 맞춰지고 수험 생활을 보낼수록 졸음을 이겨내는게 쉬워졌기 때문입니다.</v>
       </c>
       <c r="H347" t="str">
         <v>영어단어 외우기를 평소에 너무 귀찮아해서 항상 영어단어가 부족했었는데 보카테스트를 정해진 요일에 하면서 귀찮더라도 억지로 암기 습관을 들이며 매주 응시하면서 점차 영어단어에 대한 거부감도 사라지고 매주하다보니 점차 아는 단어가 많아지면서 문제가 잘 풀리다보니 점점 더 영어 공부에 애정을 가지게 되어 재밌게 공부할 수 있었습니다.</v>
@@ -13282,7 +13282,7 @@
         <v>공부하면서 제일 참기 힘든 게 핸드폰이라고 생각하는데 등원할 때 핸드폰을 수거해 가니까 핸드폰이 옆에 있을 때보다 핸드폰에 대한 생각이 줄어들어서 공부에 더 집중할 수 있게 됐어요 그래서 도움이 되었다고 생각합니다</v>
       </c>
       <c r="H356" t="str">
-        <v>인강에 쓰는 돈이 적은 돈도 아니고 부모님께 부탁하기도 미안할 정도의 금액인데 이투스247에 다니면 이투스 구독을 해주니까 학원도 다니면서 인강도 부담없이 들을 수 있어서 많은 도움이 되었다고 생각합니다</v>
+        <v>인강에 쓰는 돈이 적은 돈도 아니고 부모님께 부탁하기도 미안할 정도의 금액인데 이투스247에 다니면 이투스 구독을 해주니까 학원도 다니면서 인강도 부담 없이 들을 수 있어서 많은 도움이 되었다고 생각합니다</v>
       </c>
       <c r="I356" t="str">
         <v>감사합니다 선생님들 덕분에 더 나은 제가 될 수 있었어요. 이투스247에 다니며 선생님들과 함께 생활했던 1년은 공부뿐만 아니라 인생에 대해서도 많은 걸 배울 수 있었던 한 해였습니다. 제 인생에서 절대 잊지 못할 기억이고 은인이십니다. 다시 한 번 진심으로 감사드립니다.</v>
@@ -13589,7 +13589,7 @@
         <v>N수생</v>
       </c>
       <c r="E364" t="str">
-        <v>처음 입소 당시 공부를 어디서부터 어떻게 해야하는지 막막했는데 선생님께서 잘 알려주시고 이끌어주셔서 공부 방향을 잡게되고 중간에 흐트러지지 않게 지도해주셔서 성적 향상을 이룰 수 있어서 학습코칭 시스템이 유용했다고 생각합니다</v>
+        <v>처음 입소 당시 공부를 어디서부터 어떻게 해야 하는지 막막했는데 선생님께서 잘 알려주시고 이끌어주셔서 공부 방향을 잡게되고 중간에 흐트러지지 않게 지도해주셔서 성적 향상을 이룰 수 있어서 학습코칭 시스템이 유용했다고 생각합니다</v>
       </c>
       <c r="F364" t="str">
         <v>6,9모 학원 모의고사를 정기적으로 보고 지원가능대학 라인을 확인함으로써 적당한 긴장감과 도전의식을 가지며 공부할 수 있었다고 생각해서 이 학습 관리 시스템이 유용했다고 생각이 되었습니다</v>

</xml_diff>

<commit_message>
Replace additional typos: 제시해주셔서, 있었던건
</commit_message>
<xml_diff>
--- a/reviews_with_keywords.xlsx
+++ b/reviews_with_keywords.xlsx
@@ -708,7 +708,7 @@
         <v>N수생</v>
       </c>
       <c r="E9" t="str">
-        <v>이투스 개별 맞춤 학습 상담을 통해 제 실력이 현재 어느 정도인지, 그리고 앞으로 어떤 부분을 집중해야 할지 명확하게 알 수 있어서 좋았습니다! 상담 과정에서 꼼꼼하게 제 실력에 맞춰 학습 방향을 제시해주셔서 학습 계획을 세우는 데 큰 도움이 되었습니다! 한달을 되돌아 볼 수 있는 소중한 시간이었습니다!</v>
+        <v>이투스 개별 맞춤 학습 상담을 통해 제 실력이 현재 어느 정도인지, 그리고 앞으로 어떤 부분을 집중해야 할지 명확하게 알 수 있어서 좋았습니다! 상담 과정에서 꼼꼼하게 제 실력에 맞춰 학습 방향을 제시해 주셔서 학습 계획을 세우는 데 큰 도움이 되었습니다! 한달을 되돌아 볼 수 있는 소중한 시간이었습니다!</v>
       </c>
       <c r="F9" t="str">
         <v>모르는 부분을 바로바로 질문할 수 있어서  시간 낭비를 줄이고 효율적으로 공부할 수 있었던 점이 정말 좋았습니다. 조교 쌤들 다 너무 친절하게 기초부터 설명해주셔서 실력 향상에 정말 많은 도움이 되었습니다!</v>
@@ -723,7 +723,7 @@
         <v>1년이 조금 안되눈 시간동안 항상 따뜻하게 지도해주시고 응원해주셔서 감사합니다 선생님들 덕분에 재수 했을 때의 기억이 마냥 힘든 시간으로만 기억되지 않을것 같아요! 진심으로 너무 감사했습니다🩷🩷</v>
       </c>
       <c r="J9" t="str">
-        <v>상담 과정에서 꼼꼼하게 제 실력에 맞춰 학습 방향을 제시해주셔서 학습 계획을 세우는 데 큰 도움이 되었어요.</v>
+        <v>상담 과정에서 꼼꼼하게 제 실력에 맞춰 학습 방향을 제시해 주셔서 학습 계획을 세우는 데 큰 도움이 되었어요.</v>
       </c>
       <c r="K9" t="str">
         <v>학습 계획</v>
@@ -1027,7 +1027,7 @@
         <v>클리닉 수업에서는 ”부족한 점 위주로 보완“ 하는 프로그램이 이루어진다고 느꼈습니다. 단순히 진도를 빼는 수업이 아니라, 학생이 뭐가 부족하고, 어떻게 보완해야 할지를 제시해주셨습니다</v>
       </c>
       <c r="F18" t="str">
-        <v>스스로 해결하기 어려운 질문들을 1:1 질의응답을 통해 해결할 수 있었고, 과목별 공부법이나, 일일테스트 질문까지 가능하여 학습에 유용했습니다. 뿐만 아니라, 질문을 해결하고 어떤걸 추가로 학습하면 좋을지도 제시해주셔서 학습 방향을 올바르게 잡는데도 도움이 돠었습니다</v>
+        <v>스스로 해결하기 어려운 질문들을 1:1 질의응답을 통해 해결할 수 있었고, 과목별 공부법이나, 일일테스트 질문까지 가능하여 학습에 유용했습니다. 뿐만 아니라, 질문을 해결하고 어떤걸 추가로 학습하면 좋을지도 제시해 주셔서 학습 방향을 올바르게 잡는데도 도움이 돠었습니다</v>
       </c>
       <c r="G18" t="str">
         <v>핸드폰이 공부에 가장 큰 방해가 되는건 누구나 그럴 것 같습니다. 원천적으로 차단을 시켜주니 핸드폰에 접근할 생각조차 없어졌었습니다. 재원 기간동안 스마트폰 사용 습관이 많이 잡힌 것 같다고 느꼈습니다</v>
@@ -1758,7 +1758,7 @@
         <v>N수생</v>
       </c>
       <c r="E38" t="str">
-        <v>국어 선생님께서 국어를 어떻기 학습해야 할지 자세히 알려주셔서 좋았습니다. 특히 저는 현대소설이 약했는데, 9월 평가원에서 현대소설이 어렵게 출제되어 오답에 부담을 느끼고 있었는데 담임 선생님께서 오답을 하는 가이드라인을 제시해주셔서 도움을 많이 받았던 기억이 있습니다.</v>
+        <v>국어 선생님께서 국어를 어떻기 학습해야 할지 자세히 알려주셔서 좋았습니다. 특히 저는 현대소설이 약했는데, 9월 평가원에서 현대소설이 어렵게 출제되어 오답에 부담을 느끼고 있었는데 담임 선생님께서 오답을 하는 가이드라인을 제시해 주셔서 도움을 많이 받았던 기억이 있습니다.</v>
       </c>
       <c r="F38" t="str">
         <v>저는 2주에 한 번씩 학습 상담울 받았었는데요, 저는 못하는 과목을 기피하는 성향이 있었는데,특히 영어가 그랬던 것 같습니다. 하지만 선생님께서 영어를 꾸준히 학습할 수 있게끔 단어 테스트를 치게 하는 등으로 도움을 꾸준히 주셔서 영어 공부를 놓치 않고 지속적으로 할 수 있었습니다.</v>
@@ -2145,7 +2145,7 @@
         <v>N수생</v>
       </c>
       <c r="E49" t="str">
-        <v>매월 진행되는 사설 모의고사와 평가원 모의고사의 분석지를 토대로 정확한 수치와 데이터를 기반으로 한 공부 방법 점검과 나아가야할 방향성을 제시해주셔서 좋았다. 또한 상담을 주기적으로 하면서 나의 현재 위치를 알고 계속하여 마음을 다 잡을 수 있었다</v>
+        <v>매월 진행되는 사설 모의고사와 평가원 모의고사의 분석지를 토대로 정확한 수치와 데이터를 기반으로 한 공부 방법 점검과 나아가야할 방향성을 제시해 주셔서 좋았다. 또한 상담을 주기적으로 하면서 나의 현재 위치를 알고 계속하여 마음을 다 잡을 수 있었다</v>
       </c>
       <c r="F49" t="str">
         <v>매일 작성하는 일간 학습 플래너를 토대로 하교시 제출 후, 다음날 바로 바로 피드백을 해주셔서 좋았다. 놓치고 있는 부분을 보완할 수 있도록 바로 바로 체크해주시고 진도나간 부분을 다시 한번 복습할 수 있는 시스템이 좋았다</v>
@@ -3543,7 +3543,7 @@
 영어 단어 테스트를 하는것이 하루의 루틴으로 자리 잡아서 하다보니 강제성이 없어도 스스로 알아서 하게되었습니다.</v>
       </c>
       <c r="I87" t="str">
-        <v>1년 동안 이런저런 고민거리 들어주시고 해결책을 제시해주셔서 감사했고, 불편한점을 해결해주시기 위해서 노력해주셔서 감사했습니다. 덕분에 공부에 집중할 수 있었습니다. 저 때문에 고생도 많이 하셨습니다. 앞으로 건강히 잘지내세요</v>
+        <v>1년 동안 이런저런 고민거리 들어주시고 해결책을 제시해 주셔서 감사했고, 불편한점을 해결해주시기 위해서 노력해주셔서 감사했습니다. 덕분에 공부에 집중할 수 있었습니다. 저 때문에 고생도 많이 하셨습니다. 앞으로 건강히 잘지내세요</v>
       </c>
       <c r="J87" t="str">
         <v>과목별 선생님과 꾸준한 상담으로 재수 생활의 부담을 덜 수 있었고, 어려운 문제도 차근차근 해결할 수 있었어요.</v>
@@ -3710,7 +3710,7 @@
         <v>현재 공부 진행률을 점검하고 앞으로의 공부 진행방향에 대해 생각해볼 수 있는 시간이었습니다. 학습 방향성에 있어서 고민이 되었던 것이나 생각하지 못했던 방법을 개개인 맞춤식으로 고려해 함께 고민하고 제안해주셔서 많은 도움이 되었습니다.</v>
       </c>
       <c r="F92" t="str">
-        <v>성적에 대한 냉정한 판단으로 현실적인 목표를 잡을 수 있게되었고 상담을 통해 성적에 맞는 학습 방향을 제시해주셔서 성적에 알맞는 방법으로 학습을 진행할 수 있다는 점에서 유용했습니다. 또한 가시적으로 성적을 직면하고 성적의 원인을 분석할 수 있어서 좋았습니다.</v>
+        <v>성적에 대한 냉정한 판단으로 현실적인 목표를 잡을 수 있게되었고 상담을 통해 성적에 맞는 학습 방향을 제시해 주셔서 성적에 알맞는 방법으로 학습을 진행할 수 있다는 점에서 유용했습니다. 또한 가시적으로 성적을 직면하고 성적의 원인을 분석할 수 있어서 좋았습니다.</v>
       </c>
       <c r="G92" t="str">
         <v>개인적으로 학원 밖에서 혼자 공부할 때는 전자기기에 학습 외의 앱들의 유혹을 참기가 힘들 때가 있었습니다. 이투스 학원에서 이런 유혹을 캐치해 학습 관련 사이트나 앱에만 접속할 수 있게 제어해줘서 공부할 때 공부에만 집중할 수 있었던 것 같습니다.</v>
@@ -4955,7 +4955,7 @@
 제 멘탈이 무너질 때마다 응원해주시고 붙잡아주셔서, 수능 공부뿐만 아니라 다른 분야에서도 자신감을 얻을 수 있게 되었습니다. 잘 챙겨주셔서 감사합니다.</v>
       </c>
       <c r="J126" t="str">
-        <v>원장님과 선생님들께서 제 학습 상황을 세심하게 파악하고 맞춤 계획을 제시해주셔서 심적으로도 안정감을 얻을 수 있었어요.</v>
+        <v>원장님과 선생님들께서 제 학습 상황을 세심하게 파악하고 맞춤 계획을 제시해 주셔서 심적으로도 안정감을 얻을 수 있었어요.</v>
       </c>
       <c r="K126" t="str">
         <v/>
@@ -5328,7 +5328,7 @@
         <v>여러 비슷한 유형의 학원을 다녀본 결과 이투스247만의 특별한 장점은 대학생 멘토분께서 1:1로 학생들 담당하여 매주 학습 코칭을 해주신다는 것이었습니다. 학생 개개인의 상황에 맞는 적절한 피드백과 공부 계획을 함께 고민해주시고 방향을 잡아주셔서  큰 도움이 되었습니다.</v>
       </c>
       <c r="F137" t="str">
-        <v>어떤 강사의 강의를 듣고, 어떤 유형의 교재를 결정할지는 수능을 준비하는 학생들에게 가장 큰 고민이라는 생각이 드는데, 멘토분께서 저에게 가장 적합한 커리큘럼을 제시해주셔서  좋았습니다. 특히 지금 상황에서 추천하지 않는 강의를 지적해주셔서 제 계획을 수정하는 데에 도움이 되었습니다.</v>
+        <v>어떤 강사의 강의를 듣고, 어떤 유형의 교재를 결정할지는 수능을 준비하는 학생들에게 가장 큰 고민이라는 생각이 드는데, 멘토분께서 저에게 가장 적합한 커리큘럼을 제시해 주셔서  좋았습니다. 특히 지금 상황에서 추천하지 않는 강의를 지적해주셔서 제 계획을 수정하는 데에 도움이 되었습니다.</v>
       </c>
       <c r="G137" t="str">
         <v>독학재수학원을 다닌 가장 큰 이유였습니다. 혼자서 독서실에 가 공부를 했을 때는 빈번하게 폰을 확인하며 공부에 집중하지 못하고 딴 짓을 하는 경우가 많았는데, 이투스247 학원에서는 등원과 함께 폰을 수거해주셔서 오로지 공부에만 집중할 수 있었습니다.</v>
@@ -5364,7 +5364,7 @@
 또한 특강을 많이 깔아주셔서 공부하는데 편리하였다</v>
       </c>
       <c r="F138" t="str">
-        <v>플래너를 하나하나 다 검사하셔서 공부하는데 흐트러짐 없이 공부할 수 있었다.또한 목표를 명확하게 만들어줌으로써 방향성을 제시해주셔서 고민이 없어졌다 또 자기통제력이 강화되어서 미루는 습관이 없어졌다</v>
+        <v>플래너를 하나하나 다 검사하셔서 공부하는데 흐트러짐 없이 공부할 수 있었다.또한 목표를 명확하게 만들어줌으로써 방향성을 제시해 주셔서 고민이 없어졌다 또 자기통제력이 강화되어서 미루는 습관이 없어졌다</v>
       </c>
       <c r="G138" t="str">
         <v>뇌가 한가지 일에 집중할 수 잇어서 깊은상태로 오래 공부를 할 수 있었다.또한 도파민 과부화가 감소하여서 공부에 흥미를 느끼게 되었다. 또한 자기전에 폰 보는 습관이 고쳐져서 깊은 잠을 편안하게 잘 수 잇게 되엇다</v>
@@ -6277,7 +6277,7 @@
         <v>학생 한 명 한 명을 신경 써 주시며 도와주시고 응원해 주신 덕분에 끝까지 포기하지 않고 노력할 수 있었습니다. 올바른 공부 방법과 태도를 배울 수 있어 더욱 의미 있는 시간이었던 것 같습니다. 앞으로도 선생님들께 배운 것을 바탕으로 더 성장할 수 있도록 노력하겠습니다. 진심으로 감사드립니다!</v>
       </c>
       <c r="J163" t="str">
-        <v>고3 때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던건 선생님들의 탁월한 입시전략과 상담, 생활환경 조성 덕분이었어요.</v>
+        <v>고3 때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던 건 선생님들의 탁월한 입시전략과 상담, 생활환경 조성 덕분이었어요.</v>
       </c>
       <c r="K163" t="str">
         <v/>
@@ -7265,7 +7265,7 @@
 고마운 존재였습니다. 결코 쉽지 않은 난이도로 항상 저를 당황시켰는데 오히려 시험준비에 더 열심히 임할 수 있었던 것 같습니다.</v>
       </c>
       <c r="I190" t="str">
-        <v>작년, 걱정과 불안이 가득한 입시상담을 받았던게 새록새록 떠오르는데 저는 지금 그 때의 상담에서 선생님께서 말씀하신 대학의 학과에 입학했습니다! 고3 때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던건 이투스 강서지점 선생님들의 탁월한 입시전략과 상담, 생활환경 조성 덕분이었습니다. 저의 처음이자 마지막 재수를 성공적으로 마치게 해주신 이투스 강서지점 선생님들께 감사를 표합니다!</v>
+        <v>작년, 걱정과 불안이 가득한 입시상담을 받았던게 새록새록 떠오르는데 저는 지금 그 때의 상담에서 선생님께서 말씀하신 대학의 학과에 입학했습니다! 고3 때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던 건 이투스 강서지점 선생님들의 탁월한 입시전략과 상담, 생활환경 조성 덕분이었습니다. 저의 처음이자 마지막 재수를 성공적으로 마치게 해주신 이투스 강서지점 선생님들께 감사를 표합니다!</v>
       </c>
       <c r="J190" t="str">
         <v>생활 상담을 포함한 코칭 시스템은 공부 외적인 부분까지 함께 관리해 준다는 점에서 의미가 있었어요.</v>
@@ -8306,7 +8306,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E219" t="str">
-        <v>현재 내 학습 수준과 남은 시간과 시기 등의 상황을 고려하여 적절한 강의와 커리큘럼을 추천해 주셔서 학습 방향을 보다 명확하게 설정하여 불필요한 시간 낭비 없이 효율적으로 공부할 수 있게 되었고 또한 학습 상담 과정에서 세심하게 제 고민과 부족한 부분을 파악해주시고 현실적인 조언과 구체적인 학습 방법까지 제시해주셔서 신뢰가 갔으며 동기부여에도 큰 도움이 되었습니다.</v>
+        <v>현재 내 학습 수준과 남은 시간과 시기 등의 상황을 고려하여 적절한 강의와 커리큘럼을 추천해 주셔서 학습 방향을 보다 명확하게 설정하여 불필요한 시간 낭비 없이 효율적으로 공부할 수 있게 되었고 또한 학습 상담 과정에서 세심하게 제 고민과 부족한 부분을 파악해주시고 현실적인 조언과 구체적인 학습 방법까지 제시해 주셔서 신뢰가 갔으며 동기부여에도 큰 도움이 되었습니다.</v>
       </c>
       <c r="F219" t="str">
         <v>현재 내 학습 수준과 남은 시간 등을 고려하여 교재와 인강을 체계적으로 추천해 주셔서 무엇부터 어떻게 공부해야 할지 명확하게 알 수 있어 매우 유용했습니다. 특히 개인에게 맞는 강의와 교재를 연결해주어 학습 효율이 높아졌고 시행착오를 줄일 수 있었습니다.</v>
@@ -10368,7 +10368,7 @@
         <v>N수생</v>
       </c>
       <c r="E275" t="str">
-        <v>전반적인 성적, 부족한 과목과 파트를 자세히 파악해주시고 이를 토대로 구체적인 학습 방향을 제시해주셔서 학습 계획 수립에 큰 도움이 되었습니다. 특히 저는 수학과 탐구 과목이 부족하였는데, 제시해주신 학습 방향대로 공부하니 성적 향상을 거둘 수 있었습니다.</v>
+        <v>전반적인 성적, 부족한 과목과 파트를 자세히 파악해주시고 이를 토대로 구체적인 학습 방향을 제시해 주셔서 학습 계획 수립에 큰 도움이 되었습니다. 특히 저는 수학과 탐구 과목이 부족하였는데, 제시해주신 학습 방향대로 공부하니 성적 향상을 거둘 수 있었습니다.</v>
       </c>
       <c r="F275" t="str">
         <v>수많은 콘텐츠가 넘쳐나는 현재 대학 입시 상황에서 무슨 교재와 강의를 선택해야 저의 현재 성적대에 도움이 될지 잘 모르겠어서 힘들었었는데 분석하신 제 성적을 바탕으로 각 과목의 교재와 강의를 꼼꼼히 추천해 주셔서 크게 도움이 되었습니다.</v>
@@ -12472,7 +12472,7 @@
         <v>선생님들이 과목별로 다르게 저한테 맞는 공부법을 알려주셨습니다. 선생님 본인의 수험 생활에서 효과를 보셨던 방법들부터 선배님들의 방법까지 소개해주셔서 도움이 많이 됐습니다. 학습 뿐만아니라 생활부분에서도 힘든 점이나 어려운 점이 있으면 쉽게 말할 수 있는 분위기여서 학원 생활에 있어 큰 어려움은 없었습니다. 선생님들 덕분에 수월한 수험 생활을 한 것 같습니다.</v>
       </c>
       <c r="F334" t="str">
-        <v>매달 정기고사나 모의고사가 끝나면 필수로 해야하는 상담이 있었는데 결과가 좋든 좋지 않든 선생님께서 편안하게 상담을 진행해주셨고, 잘 한 부분은 아낌없는 칭찬과 아쉬운 부분은 어떻게 해결해나가야하는지에 대해 보완점도 제시해주셔서 유용했습니다.</v>
+        <v>매달 정기고사나 모의고사가 끝나면 필수로 해야하는 상담이 있었는데 결과가 좋든 좋지 않든 선생님께서 편안하게 상담을 진행해주셨고, 잘 한 부분은 아낌없는 칭찬과 아쉬운 부분은 어떻게 해결해나가야하는지에 대해 보완점도 제시해 주셔서 유용했습니다.</v>
       </c>
       <c r="G334" t="str">
         <v>너무 피곤한 날이나 체력적으로 피곤 할 때 공부하다 졸면 감독하시면서 지나다니시는 선생님들이 깨워주시거나 리프레쉬할 수 있는 산책시간을 가질 수 있어서 좋았습니다. 이러한 감독 시스템이 있어서 딴짓이나 졸음을 막는 데 유용했던 것 갔습니다.</v>

</xml_diff>

<commit_message>
Apply third batch of text corrections
</commit_message>
<xml_diff>
--- a/reviews_with_keywords.xlsx
+++ b/reviews_with_keywords.xlsx
@@ -606,7 +606,7 @@
         <v>재수하면서 멘탈이 흔들릴때가 많았는데 그때마다 상담하면서 중심을 잡을 수 있었던것 같습니다. 그리고 담당 선생님이 열심히 쪼아주셔서 나태해질때마다 다시 정신 붙잡고 공부할 수 있었고 후반에는 공부를 어떻게 해야되는지 안 것 같은 느낌이었습니다</v>
       </c>
       <c r="F6" t="str">
-        <v>앞서 말한것과 비슷하게 개인적인 성향이 혼자둬도 공부 엔간히 하지만 옆에 두고 관리해주실때 공부 효율이 더 나는 사람이라 플래너라든지 공부 방향 관리해주신게 좋았습니다! 효율적으로 공부하게 되는 느낌이었어여</v>
+        <v>앞서 말한 것과 비슷하게 개인적인 성향이 혼자둬도 공부 엔간히 하지만 옆에 두고 관리해주실때 공부 효율이 더 나는 사람이라 플래너라든지 공부 방향 관리해주신게 좋았습니다! 효율적으로 공부하게 되는 느낌이었어여</v>
       </c>
       <c r="G6" t="str">
         <v>다른건 막 좋지는 않았는데 그냥 그랬어여 그나마 나은게 출결이었음. 그냥 빨리 일어나니까 생활 습관 잡히고 아침에 뇌가 깨어 있는 느낌? 좋았습니다. 근데 다른건 개선 할게 좀 있어여</v>
@@ -787,7 +787,7 @@
         <v>일단 학원에 있으면 연락 알람 자체도 안오기때문에 공부에 집중하는데 정말 도움이 되었습니다. 또한 인강 사이트 외에는 인터넷이 안되서 강제로 공부할 수 있는 환경을 조성해주셔서 공부 하기에 정말 적합한 환경이였습니다.</v>
       </c>
       <c r="H11" t="str">
-        <v>공부하는데 제일 중요한것은 감을 잃지 않는 것인데 모의고사를 통해서 수능을 볼때의 감을 잃지 않을 수 있었고 지금 제가 어느정도의 실력을 갖고 있는지 정검할 수 있어서 더 부족하다고 생각하는 과목의 공부를 하는데 도움이 되었습니다.</v>
+        <v>공부하는데 제일 중요한 것은 감을 잃지 않는 것인데 모의고사를 통해서 수능을 볼때의 감을 잃지 않을 수 있었고 지금 제가 어느정도의 실력을 갖고 있는지 정검할 수 있어서 더 부족하다고 생각하는 과목의 공부를 하는데 도움이 되었습니다.</v>
       </c>
       <c r="I11" t="str">
         <v>이투스247에 다니는 동안 상담과 출결 관리까지 꼼꼼히 신경 써주셔서 감사합니다. 공부하기 좋은 환경과 힘들게 공부할 때 많이 챙겨 주셔서 재수 생활을 버티는데 도움이 많이 되었습니다. 선생님들의 덕분에 공부에 도움이 많이 되었고, 좋은 결과로 이어질 수 있었습니다. 감사합니다</v>
@@ -1293,7 +1293,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E25" t="str">
-        <v>헉습에 집중할 수있더록 멘탈관리를 잘해주셨습니다 주기적인 상담을 해주셨고 멘탈이 떨어질때 여러방법으로 상담을 주셔서 이갸낼수있었습니다 모의고사를 보고나면 과목별 학습 상담이 도움이 되었습니다</v>
+        <v>헉습에 집중할 수있더록 멘탈 관리를 잘해주셨습니다 주기적인 상담을 해주셨고 멘탈이 떨어질때 여러방법으로 상담을 주셔서 이갸낼수있었습니다 모의고사를 보고나면 과목별 학습 상담이 도움이 되었습니다</v>
       </c>
       <c r="F25" t="str">
         <v>과목별 성적변화에 대한 상담이 도움이되었고 그에따른 과목별 시간배분과 교재선정및 학습 계획에 대해 도움을 받았습니다 어떤과목에 현재 더 시간을 쏟아야할지 가이드라인을 해주셨습니다 한과목에 치중하지않도록 시건배분에대한 계획에 도움을 받았습니다</v>
@@ -1340,10 +1340,10 @@
         <v>모의고사의 양이 절대적으로 중요한 학생들에게 이투스 모의고사라는 자체적인 컨텐츠를 제공하는 점이 좋았습니다. 또 그 컨텐츠가 단순히 기출을 짜깁기한 것이 아니라 새롭고 퀄리티 있는 시험지라는 점에서 너무나도 큰 도움이 되었습니다.</v>
       </c>
       <c r="I26" t="str">
-        <v>재학 기간 동안 많은 건강적인 문제가 있었는데 많은 편의를 봐주셔서 오랫동안 공부하며 꾸준히 노력할 수 있었습니다 감사합니다. 또 지칠 때 응원해주시며 동기부여해주시는게 수험 생활의 소소한 낙이었습니다. 감사드립니다</v>
+        <v>재학 기간 동안 많은 건강적인 문제가 있었는데 많은 편의를 봐주셔서 오랫동안 공부하며 꾸준히 노력할 수 있었습니다 감사합니다. 또 지칠 때 응원해주시며 동기부여해주시는 게 수험 생활의 소소한 낙이었습니다. 감사드립니다</v>
       </c>
       <c r="J26" t="str">
-        <v>지칠 때 응원해주시며 동기부여해주시는게 수험 생활의 소소한 낙이었어요.</v>
+        <v>지칠 때 응원해주시며 동기부여해주시는 게 수험 생활의 소소한 낙이었어요.</v>
       </c>
       <c r="K26" t="str">
         <v/>
@@ -1838,10 +1838,10 @@
         <v>물론 방화벽을 뚫는 학생들도 보았습니다. 하지만 저는 막아둔 것에 의미가 있다고 생각하여 틀안에서 벗어나지 않으려했는데요, 인터넷에 노출되지않아 잡생각과 유혹등에 현혹되지않을수 있어서 좋았던 것 같습니다.</v>
       </c>
       <c r="H40" t="str">
-        <v>자칫하면 타 과목을 공부하느라 단어를 놓치기 일수라고 생각합니다. 그런데 다같이 단어를 시험보면서 강제성과 의무가 부여되니 자연스럽게 단어를 외우고 부담이 줄어들어 좋았습니다. 그리고 반복해서 단어시험을 치기때문에 독해력에도 도움이 된것같습니다.</v>
+        <v>자칫하면 타 과목을 공부하느라 단어를 놓치기 일수라고 생각합니다. 그런데 다 같이 단어를 시험보면서 강제성과 의무가 부여되니 자연스럽게 단어를 외우고 부담이 줄어들어 좋았습니다. 그리고 반복해서 단어시험을 치기때문에 독해력에도 도움이 된것같습니다.</v>
       </c>
       <c r="I40" t="str">
-        <v>비록 수능날에 긴장을 너무많이해서 실력발휘를 못한것이 너무나 아쉽긴하지만, 실력은 확실히 늘었음을 체감할 수 있었습니다. 약 일년간 지도해주시느라 수고많으셨고 현역때의 아쉬움을 해결하고 넘어갈수있어서 좋았습니다. 서포트해주셔서 감사합니다.</v>
+        <v>비록 수능날에 긴장을 너무많이해서 실력발휘를 못한 것이 너무나 아쉽긴하지만, 실력은 확실히 늘었음을 체감할 수 있었습니다. 약 일년간 지도해주시느라 수고많으셨고 현역때의 아쉬움을 해결하고 넘어갈수있어서 좋았습니다. 서포트해주셔서 감사합니다.</v>
       </c>
       <c r="J40" t="str">
         <v>각 과목별로 담당 선생님께 질의응답을 신청하여 문제를 해결할 수 있었던 점이 좋았어요.</v>
@@ -2251,7 +2251,7 @@
         <v>반수생</v>
       </c>
       <c r="E52" t="str" xml:space="preserve">
-        <v xml:space="preserve">국어가 맨날 5~6등급이었지만 국어 멘토링덕분에 2,3,4등급은 안정적으로 받을 수있는 수준으로 발전하였다_x000d_
+        <v xml:space="preserve">국어가 맨날 5~6등급이었지만 국어 멘토링덕분에 2,3,4등급은 안정적으로 받을 수 있는 수준으로 발전하였다_x000d_
 또한 탐구를 담임 선생님께서 잘 체크해주셔서 빠뜨리지 않고 잘 공부할 수있었다</v>
       </c>
       <c r="F52" t="str" xml:space="preserve">
@@ -2268,7 +2268,7 @@
         <v>모든 선생님들 지도해주셔서 감사했습니다 특히 태민선생님 상담 잘해주시고 피드백 잘해주셔서 감사했습니다 찾아뵙고싶었는데 못찾아뵈었네요 죄송합니다 다음에 기회가 된다면 꼭 찾아뵙고싶습니다</v>
       </c>
       <c r="J52" t="str">
-        <v>6등급이었지만 국어 멘토링덕분에 2,3,4등급은 안정적으로 받을 수있는 수준으로 발전하였어요.</v>
+        <v>6등급이었지만 국어 멘토링덕분에 2,3,4등급은 안정적으로 받을 수 있는 수준으로 발전하였어요.</v>
       </c>
       <c r="K52" t="str">
         <v/>
@@ -2297,7 +2297,7 @@
         <v>면학 분위기가 잘 유지된다는 점에서 집중하는 데 큰 도움이 됐다. 주변 학생들도 다들 조용히 공부하는 분위기라 자연스럽게 흐름을 따라가게 됐고, 졸음 관리도 중간중간 체크해주거나 환기할 수 있게 도와줘서 흐트러지지 않고 공부를 이어갈 수 있었다. 혼자 집에서 할 때보다 훨씬 덜 나태해지고, 규칙적인 생활을 유지하는 데 도움이 됐다는 점이 좋았다.</v>
       </c>
       <c r="H53" t="str">
-        <v>보카 테스트 콘텐츠는 꾸준히 단어를 외우도록 습관을 만들어준다는 점에서 유용했다. 정해진 분량을 반복적으로 테스트하다 보니 자연스럽게 복습이 되고, 틀린 단어를 다시 체크하면서 암기 효율도 높일 수 있었다. 혼자 하면 미루기 쉬운 단어 공부를 꾸준히 유지하게 해준다는 점이 특히 도움이 됐다.</v>
+        <v>단어 테스트 콘텐츠는 꾸준히 단어를 외우도록 습관을 만들어준다는 점에서 유용했다. 정해진 분량을 반복적으로 테스트하다 보니 자연스럽게 복습이 되고, 틀린 단어를 다시 체크하면서 암기 효율도 높일 수 있었다. 혼자 하면 미루기 쉬운 단어 공부를 꾸준히 유지하게 해준다는 점이 특히 도움이 됐다.</v>
       </c>
       <c r="I53" t="str">
         <v>선생님들께 감사드립니다. 작년 한 해 동안 혼자 공부하면서 흔들릴 때도 많았는데, 그때마다 상담과 관리로 방향을 잡아주셔서 끝까지 버틸 수 있었습니다. 단순히 공부만이 아니라 생활 습관이나 멘탈까지 챙겨주신 점이 특히 기억에 남습니다. 덕분에 이전보다 훨씬 더 꾸준하게 공부할 수 있었고, 스스로에 대한 믿음도 조금은 생긴 것 같습니다. 진심으로 감사합니다.</v>
@@ -2393,7 +2393,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E56" t="str">
-        <v>독학공부를 하다보니 학습방향성에 대해 자주 불안했었는데 친절하신 담당과목 선생님들과의 상담이 자유로워 불안을 즉시 해결할 수 있었음. 더 나아가 장기적으로 보았을 때 수험생 멘탈관리 부분에서도 효과적이었던 것 같음.</v>
+        <v>독학공부를 하다보니 학습방향성에 대해 자주 불안했었는데 친절하신 담당과목 선생님들과의 상담이 자유로워 불안을 즉시 해결할 수 있었음. 더 나아가 장기적으로 보았을 때 수험생 멘탈 관리 부분에서도 효과적이었던 것 같음.</v>
       </c>
       <c r="F56" t="str">
         <v>혼자 공부를 하다보면 나태해져 과목편식이 심해졌었는데 관리를 받으니 하기 싫은 과목도 꾸준히 하게 되는 점이 좋았다. 플래너 쓰기 귀찮아서 대충 썼었는데 플래너 검사를 통해 해야 되는 것을 가시화하는 습관을 만들게 되어 수험 생활에 큰 도움이 되었음.</v>
@@ -2402,7 +2402,7 @@
         <v>일반 독서실에 가면 아무리 휴대폰을 안 보려 해도 자꾸만 손이 가는게 스트레스였는데 강제로 휴대폰을 수거해 가서 공부에 집중할 수 있다는 점이 좋았음. 점심,저녁시간에도 휴대폰을 못 쓰니 자연스럽게 휴대폰 의존도가  낮아져 평소 집중력도 올라건 것 같음.</v>
       </c>
       <c r="H56" t="str">
-        <v>영단어 외우는 건 항상 뒤로 미뤄 스트레스를 받았었는데 의무적으로 보는 보카 테스트 덕분에 꾸준히 영단어를 학습하게 된 것이 마음에 들었음. 영어성적 향상에 직접적인 영향을 주어 만족스러웠음.</v>
+        <v>영단어 외우는 건 항상 뒤로 미뤄 스트레스를 받았었는데 의무적으로 보는 단어 테스트 덕분에 꾸준히 영단어를 학습하게 된 것이 마음에 들었음. 영어성적 향상에 직접적인 영향을 주어 만족스러웠음.</v>
       </c>
       <c r="I56" t="str">
         <v>이투스 선생님들 좋은 면학 분위기를 위해 노력해주시고 훌륭한 지도 해주셔서 감사합니다. 덕분에 성적 향상과 좋은 습관을 얻은 것 같습니다. 후배들이나 다시 도전하는 친구들에게 좋을 말 많이 전할게요</v>
@@ -2634,7 +2634,7 @@
 환경 자체가 공부에 맞춰져 있어 스스로 통제하기 어려운 부분을 보완해준다는 점에서 큰 도움이 되었습니다</v>
       </c>
       <c r="H62" t="str" xml:space="preserve">
-        <v xml:space="preserve">보카 테스트를 꾸준히 보면서 단어 암기를 미루지 않고 반복할 수 있었던 점이 좋았습니다. 정기적으로 시험을 보니 자연스럽게 복습이 이루어졌고, 부족한 단어를 바로 확인하며 보완할 수 있었습니다_x000d_
+        <v xml:space="preserve">단어 테스트를 꾸준히 보면서 단어 암기를 미루지 않고 반복할 수 있었던 점이 좋았습니다. 정기적으로 시험을 보니 자연스럽게 복습이 이루어졌고, 부족한 단어를 바로 확인하며 보완할 수 있었습니다_x000d_
 꾸준한 테스트 덕분에 암기 효율이 높아지고, 영어 실력 향상에도 큰 도움이 되었습니다</v>
       </c>
       <c r="I62" t="str">
@@ -2767,7 +2767,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E66" t="str">
-        <v>과목 별 선생님분들께서 친절히 수준에 맞게 앞으로의 학습방향에 대해 달 코칭해주시고 모르는것에 대한 질문들을 잘 설명해주셨습니다.    또한 학습할때의 불편한것이 있는지 항상 확인해주시고 계속 신경써주셔서 편한 환경에서 공부를 할 수 있었습니다</v>
+        <v>과목 별 선생님분들께서 친절히 수준에 맞게 앞으로의 학습방향에 대해 달 코칭해주시고 모르는것에 대한 질문들을 잘 설명해주셨습니다.    또한 학습할때의 불편한 것이 있는지 항상 확인해주시고 계속 신경써주셔서 편한 환경에서 공부를 할 수 있었습니다</v>
       </c>
       <c r="F66" t="str">
         <v>베이스가 없는상태에서 시작했는데 이투스뿐만 아니라 다른 사이트 강사 선생님들을 저의 성향에 맞게 추천해주셨던것 같습니다.                                  .</v>
@@ -2808,7 +2808,7 @@
         <v>혼자서 하면 모르는것을 질문하기 어렵습니다. 인강의 QnA질문을 해도 빨라도 하루는 걸리는 질의응답을 실시간으로 궁굼한 점이 생기면 바로바로 질문하고 답변받을 수 있어서 좋았습니다.</v>
       </c>
       <c r="G67" t="str">
-        <v>먼저 핸드폰을 수거해서 좋았습니다. 또 핸드폰이 없어도 패드로도 딴 짓을 할 수있는데 와이파이 방화벽으로 그것도 관리할 수 있어서 좋았습니다. 또 선생님께서 주기적으로 돌아다니시면서 졸거나 그럴때 깨워주시고 면학 분위기 유지하기위해 노력해주셔서 좋았습니다</v>
+        <v>먼저 핸드폰을 수거해서 좋았습니다. 또 핸드폰이 없어도 패드로도 딴 짓을 할 수 있는데 와이파이 방화벽으로 그것도 관리할 수 있어서 좋았습니다. 또 선생님께서 주기적으로 돌아다니시면서 졸거나 그럴때 깨워주시고 면학 분위기 유지하기위해 노력해주셔서 좋았습니다</v>
       </c>
       <c r="H67" t="str">
         <v>이투스에 듣고싶은 강사가 있었는데 한분만 듣고싶어서  구독하기에는 부담이 되는 상황이였습니다 그런데 이투스247를 다니면 이투스구독 서비스가 제공되어서 강의를 듣게 되어서 좋았습니다.</v>
@@ -3234,7 +3234,7 @@
         <v>N수생</v>
       </c>
       <c r="E79" t="str" xml:space="preserve">
-        <v xml:space="preserve">재수 생활을 시작하며 막막했던 제게 학습코칭은 단순한 스케줄 관리를 넘어선 '터닝 포인트'였습니다. 이전에는 무작정 문제집만 풀며 양치기에 집착했다면, 코칭을 통해 저의 취약점을 객관적으로 분석하고 이를 보완할 수 있는 구체적인 학습 전략을 세울 수 있었습니다._x000d_
+        <v xml:space="preserve">재수 생활을 시작하며 막막했던 제게 학습 코칭은 단순한 스케줄 관리를 넘어선 '터닝 포인트'였습니다. 이전에는 무작정 문제집만 풀며 양치기에 집착했다면, 코칭을 통해 저의 취약점을 객관적으로 분석하고 이를 보완할 수 있는 구체적인 학습 전략을 세울 수 있었습니다._x000d_
 ​특히 매주 진행되는 상담을 통해 흐트러진 멘탈을 잡고, 저에게 최적화된 시간 배분법을 익히면서 공부 효율이 눈에 띄게 좋아졌습니다. 전문가의 피드백 덕분에 '내가 잘하고 있나?'라는 불안감 대신 '오늘도 계획대로 해냈다'는 성취감을 느끼며 공부할 수 있게 되었습니다. 성적 향상은 물론 올바른 공부 습관까지 잡고 싶은 후배들에게 적극 추천합니다!</v>
       </c>
       <c r="F79" t="str" xml:space="preserve">
@@ -3253,7 +3253,7 @@
         <v>​"막막했던 재수 생활의 시작부터 지금까지, 늘 곁에서 든든한 페이스메이커가 되어주신 선생님들과 학원 관계자분들께 진심으로 감사드립니다. 단순히 지식만 배우는 곳이 아니라 저의 가능성을 믿어주신 덕분에 끝까지 완주할 수 있었습니다. 이곳에서 배운 성실함과 자신감을 바탕으로 더 멋진 미래를 만들어 나가겠습니다. 정말 감사합니다!"</v>
       </c>
       <c r="J79" t="str">
-        <v>재수 생활을 시작하며 막막했던 제게 학습코칭은 단순한 스케줄 관리를 넘어선 '터닝 포인트'였어요.</v>
+        <v>재수 생활을 시작하며 막막했던 제게 학습 코칭은 단순한 스케줄 관리를 넘어선 '터닝 포인트'였어요.</v>
       </c>
       <c r="K79" t="str">
         <v/>
@@ -3396,7 +3396,7 @@
         <v>면학 분위기가 잘 조성되어 있어 자연스럽게 공부에 집중할 수 있었고 흐트러지지 않고 학습을 이어갈 수 있었다. 특히 졸음 관리를 위해 하루에 20분씩 두 번 짧게 휴식을 취할 수 있었던게  피로를 효과적으로 해소할 수 있었고 그 덕분에 공부할 때 잠오고 집중이 안되는 상태로 억지로 이어나가는 것이 아닌  더 또렷한 상태로 집중력을 유지할 수 있었다</v>
       </c>
       <c r="H83" t="str">
-        <v>영어가 절대평가다보니 공부 시간이 다른 과목에 비해 적었고 특히 고3이 되니 영단어에 소홀해져서 스스로 외우는 시간이 줄어들어 독해를 할 때 종종 어려움을 겪었었는데 보카 테스트를 통해 매일 꾸준히 단어를 점검할 수 있었고 반복 학습이 자연스럽게 이루어져 암기 효율이 높아졌다.</v>
+        <v>영어가 절대평가다보니 공부 시간이 다른 과목에 비해 적었고 특히 고3이 되니 영단어에 소홀해져서 스스로 외우는 시간이 줄어들어 독해를 할 때 종종 어려움을 겪었었는데 단어 테스트를 통해 매일 꾸준히 단어를 점검할 수 있었고 반복 학습이 자연스럽게 이루어져 암기 효율이 높아졌다.</v>
       </c>
       <c r="I83" t="str">
         <v>학습과 생활 전반을 꼼꼼히 챙겨 주셔서 진심으로 감사드립니다. 고3 재학생인지라 학교에서 수시를 쓰고 공부하지 않는 친구들도 많았는데 덕분에 흔들리지 않고 꾸준히 공부할 수 있었습니다. 수능공부릉 한번도 해보지 않았던 제가 공부를 하다가 흔들릴때도 스스로에 대한 믿음을 가질 수 있었습니다. 앞으로도 배운 점을 바탕으로 더 성실하게 노력하겠습니다.</v>
@@ -3434,10 +3434,10 @@
         <v>메가스터디와 이투스 패스를 둘다 사용한 저로써 대표적으로 이투스의 국어박광일 강사의 강의가 매우 도움이많이됐고, 다른 타과목의 강사진들 또한 경쟁력있으신분들이 많아서 좋았던것같습니다</v>
       </c>
       <c r="I84" t="str">
-        <v>Tm반 담임 송상윤 선생님 1년 동안 열정과 관심으로 저희 tm반 신경쓰고 관리해주셔서 감사했습니다. 종례때마다 해주시는 덕담과 조언이 재수 생활 많은 도움이 됐던것 같습니다. 뿐만 아니라 주간,야간,타반 전략 담임 선생님분들 모두 1년 동안 감사했습니다</v>
+        <v>Tm반 담임 송상윤 선생님 1년 동안 열정과 관심으로 저희 tm반 신경쓰고 관리해주셔서 감사했습니다. 종례때마다 해주시는 덕담과 조언이 재수 생활 많은 도움이 됐던 것 같습니다. 뿐만 아니라 주간,야간,타반 전략 담임 선생님분들 모두 1년 동안 감사했습니다</v>
       </c>
       <c r="J84" t="str">
-        <v>종례 때마다 해주시는 덕담과 조언이 재수 생활에 많은 도움이 됐던것 같아요.</v>
+        <v>종례 때마다 해주시는 덕담과 조언이 재수 생활에 많은 도움이 됐던 것 같아요.</v>
       </c>
       <c r="K84" t="str">
         <v/>
@@ -3787,7 +3787,7 @@
         <v>출석 시 진행되는 핸드폰 수거 시스템 덕분에 학습 시간 동안 오로지 공부에만 몰입할 수 있는 환경이 조성되어 매우 만족스러웠습니다. 스스로 통제하기 힘든 디지털 기기 유혹을 원천적으로 차단해주어 순공 시간을 확보하는 데 큰 도움이 되었습니다.</v>
       </c>
       <c r="H94" t="str">
-        <v>매일 진행되는 영단어 보카 테스트 덕분에 자칫 소홀해질 수 있는 기초 어휘력을 체계적으로 쌓을 수 있었습니다. 혼자 공부할 때는 암기량을 유지하기가 쉽지 않았는데, 학원의 강제성 있는 테스트 시스템이 꾸준한 학습 습관을 만드는 데 큰 역할을 했습니다.</v>
+        <v>매일 진행되는 영단어 단어 테스트 덕분에 자칫 소홀해질 수 있는 기초 어휘력을 체계적으로 쌓을 수 있었습니다. 혼자 공부할 때는 암기량을 유지하기가 쉽지 않았는데, 학원의 강제성 있는 테스트 시스템이 꾸준한 학습 습관을 만드는 데 큰 역할을 했습니다.</v>
       </c>
       <c r="I94" t="str">
         <v>수능을 5개월 앞두고 입학해 약 3개월 동안 이곳에서 공부하며 정말 많은 도움을 받았습니다. 비록 수능 2개월을 남겨두고 논술 준비를 위해 학원을 그만두게 되었지만, 짧다면 짧은 그 시간 동안 선생님들께서 보여주신 진심 어린 정성은 제 수험 생활의 큰 버팀목이었습니다. 특히 코치님께서 등원할 때마다 항상 밝은 미소로 인사를 건네주시고, 현실적인 조언으로 멘탈을 잡아주셔서 정말 든든했습니다. 무엇보다 제가 핸드폰을 사용하다 걸렸을 때도 모른 척해주시며 믿고 기회를 주셨던 배려에 진심으로 감사드립니다. 그 따뜻한 배려 덕분에 제 행동을 반성하고 남은 기간 더 집중할 수 있었습니다. 짧은 인연이었지만 저를 한 명의 제자로 소중히 아껴주신 마음 잊지 않겠습니다. 선생님들 덕분에 이투스에서 기분 좋게 공부하고 나갑니다. 정말 감사합니다!</v>
@@ -4046,7 +4046,7 @@
         <v>저는 수험생 때, 같은 자습실이나 교실을 쓰는 친구들이 자고 있는 분위기 속에서는 공부 의지가 떨어지는 듯한 느낌을 받았습니다. 한두명이 졸고 있어도 신경이 쓰였습니다. 같은 방의 경쟁자들까지 졸지 않고 공부하는 ’간절한 분위기‘ 속에서 공부하고 싶었기 때문입니다. 이투스247에서는 적어도 30분에 한 번씩은 감독관이나 선생님들께서 돌아다니며 졸고 있는 아이들을 깨워주셨습니다. 그 덕분에 모든 친구들이 공부에만 열중할 수 있었던 것 같고, 그 점이 참 마음에 들었습니다.</v>
       </c>
       <c r="H101" t="str">
-        <v>모의고사 퀄리티가 괜찮았었기 때문에 실력 점검을 위한 테스트로 좋았습니다~ 하지만 수학은 너무 어려웠습니다…🥹🥹 국어 영어 시험지 퀄리티는 정말 마음에 들었었던 것으로 기억해요! 혼자서 보는 모의고사와  학원에서 단체로 보는 모의고사는 느낌이 천차만별이기 때문에 다같이 으쌰으쌰하는 분위기 속에서 시험 보는 게 넘 좋았네용</v>
+        <v>모의고사 퀄리티가 괜찮았었기 때문에 실력 점검을 위한 테스트로 좋았습니다~ 하지만 수학은 너무 어려웠습니다…🥹🥹 국어 영어 시험지 퀄리티는 정말 마음에 들었었던 것으로 기억해요! 혼자서 보는 모의고사와  학원에서 단체로 보는 모의고사는 느낌이 천차만별이기 때문에 다 같이 으쌰으쌰하는 분위기 속에서 시험 보는 게 넘 좋았네용</v>
       </c>
       <c r="I101" t="str">
         <v>선생님들 감사합니다❤️ 덕분에 재수가 좋은 기억으로 남아있어요 항상 건강하시고 주변에 이투스247 홍보 엄청 하고 있습니다ㅎㅎ 강북이투스 짱이었어요🤩🤩🤩🤩🤩🤩🤩🤩🤩🤩🤩🤩🤩🤩🤩🤩🤩🤩🤩🤩</v>
@@ -4151,7 +4151,7 @@
         <v>집에서 하거나 스터기카페에서 혼자 공부를 하면 핸드폰을 습관처럼 계속 보고 신경이 쓰여서 집중을 잘 못하는데 핸드폰을 제출하니까 핸드폰 샹각이나도 폰이없으니 하지않게되어서 공부에 집중하는데에 좋았다</v>
       </c>
       <c r="H104" t="str">
-        <v>요일마다 다른과목들을 매일 테스트보니까 까먹을것도 안까먹게되고 알아가는것도 생기고 테스트를 보기위해서 단어도 외우게되고 공부를 하게되어서 스스로 열심히하게만드는 수단이되었던것같아서 유용한것같다</v>
+        <v>요일마다 다른과목들을 매일 테스트보니까 까먹을것도 안까먹게되고 알아가는것도 생기고 테스트를 보기위해서 단어도 외우게되고 공부를 하게되어서 스스로 열심히하게만드는 수단이되었던것같아서 유용한 것같다</v>
       </c>
       <c r="I104" t="str">
         <v>재수 처음할때 답답하고 되게 막막했는데 많은 도움들 주셔서 덕분에 잘 할 수 있었오요 ! 항상 친절하게대해주시고 딸처럼 걱정해주시고 챙겨주셨어서 짱 감사합니다...!!!! ❤️❤️</v>
@@ -4833,7 +4833,7 @@
         <v>집에서서는 시간관리를 못하고 핸드폰하느라 공부에 집중을 못할때가 다수였는대 핸드폰을 제출하고 공부하니까 자습시간이 늘고 공부에 더 집중할 수 있었어요 효율적인 시간관리가 가능했습니다</v>
       </c>
       <c r="H123" t="str">
-        <v>매일 보카테스트를 시행해서 단어 암기의 필요성을 느끼고 꾸준하게 학습할수있는 습관을 만들게 되었습니다.영어가 절대평가다 보니 안하고 미루는 경향이 있는데 이를 고치고 조금이라도 학습하게끔 해줬습니다</v>
+        <v>매일 보카테스트를 시행해서 단어 암기의 필요성을 느끼고 꾸준하게 학습할수 있는 습관을 만들게 되었습니다.영어가 절대평가다 보니 안하고 미루는 경향이 있는데 이를 고치고 조금이라도 학습하게끔 해줬습니다</v>
       </c>
       <c r="I123" t="str">
         <v>감사합니다ㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅜㅏㅏㅏㅏㅏㅏㅏㅏㅏㅓㅏㅏㅏㅏㅓㅓㅏㅓㅓㅓㅏㅏㅏㅏㅏㅏㅏㅘㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅡㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏㅏ</v>
@@ -4910,11 +4910,11 @@
       </c>
       <c r="I125" t="str" xml:space="preserve">
         <v xml:space="preserve">감사했습니다_x000d_
-힘들 때도 많았지만 잘 다잡아주셔서 수험 생활 잘 마무리 한것 같습니다_x000d_
+힘들 때도 많았지만 잘 다잡아주셔서 수험 생활 잘 마무리 한 것 같습니다_x000d_
 학습 선생님과 카윤터에 계신 선생님들 모두 정말 감사했습니다 항상 친절하게 대해주시고 잘 잡아주셔서 너무 좋았습니다</v>
       </c>
       <c r="J125" t="str">
-        <v>힘들 때도 많았지만 잘 다잡아주셔서 수험 생활 잘 마무리 한것 같아요.</v>
+        <v>힘들 때도 많았지만 잘 다잡아주셔서 수험 생활 잘 마무리 한 것 같아요.</v>
       </c>
       <c r="K125" t="str">
         <v/>
@@ -4984,7 +4984,7 @@
         <v>저는 옛날부터 핸드폰같은 노는것에 대한 자제력이 좋지 못해, 고등학교 3학년때 수업시간에 공부를 하다가도 폰을 하기도 했습니다. 그런데 재수를 시작하고 여기 독서실에서 핸드폰 수거를 하니 핸드폰을 못하게되여 많이 집중할 수 있게, 성장할수 있게된거같습니더 ㅣ</v>
       </c>
       <c r="H127" t="str">
-        <v>고등학교 3학년때에는 학교에서 시행된 모의고사만 치뤘었는데 n수생이 빠진 표본이라 저의 실력을 가늠하기 어령웠습니다 하지만 이쿠스 전국모의고사라는 컨텐츠를 통해 재수생을 포함한 표본을 알수있게됬고 성적에 맞는 대학을 확인 할수있는거도 좋았습니다</v>
+        <v>고등학교 3학년때에는 학교에서 시행된 모의고사만 치뤘었는데 n수생이 빠진 표본이라 저의 실력을 가늠하기 어령웠습니다 하지만 이쿠스 전국모의고사라는 컨텐츠를 통해 재수생을 포함한 표본을 알수있게됬고 성적에 맞는 대학을 확인 할수 있는거도 좋았습니다</v>
       </c>
       <c r="I127" t="str">
         <v>8개월정도동안 정말 감사했습니다!! 평생 기억에 남을정도로 힘든적도 많았지만, 선생님들이 도와주신덕에 8개월동안 버틸수 있었던고 같습니다!!! 선생님분들 하는일 다 잘되시고 좋은일 가득하시기를 기도하겠습니다!!</v>
@@ -5616,7 +5616,7 @@
         <v>평소에 쉽게 접하기 힘들고 학교 선생님들과의 상담으로는 만족하기 어려웠던 입시상담을 전문적인 선생님들 , 조교님들과 자세하게 알아볼 수 있어 좋았다. 수능이 끝난 이후에도 찾아가서 입시 상담을 할 수 있다는 점이 정말 큰 장점이라고 생각하고 이투스 247 입시상담 덕분에 대학에 합격할 수 있었다고 생각한다.</v>
       </c>
       <c r="F145" t="str">
-        <v>학습 계획을 짜며 여러가지 고려할 점이 많아 혼자하기 어렵다고 생각하여 계획없이 공부하였는데 이투스 247에 와서 전문적인 선생님들이 계획을 짜주니 걱정없이 할 수 있었다. 인강에 진도나 개인의 취향 , 성격까지 고려하여 시간표를 짜주는 모습에 정말 감동받았고 이로 인해 성적을 정말 많이 향상시킬 수 있었다.</v>
+        <v>학습 계획을 짜며 여러가지 고려할 점이 많아 혼자하기 어렵다고 생각하여 계획없이 공부하였는데 이투스 247에 와서 전문적인 선생님들이 계획을 짜주니 걱정 없이 할 수 있었다. 인강에 진도나 개인의 취향 , 성격까지 고려하여 시간표를 짜주는 모습에 정말 감동받았고 이로 인해 성적을 정말 많이 향상시킬 수 있었다.</v>
       </c>
       <c r="G145" t="str">
         <v>공부하며 졸리거나 피곤할때는 반드시 온다. 그러나 옆에서 깨워주는 사람이 있으면 다시 정신차리고 공부할 수 있다고 생각한다. 피곤하거나 졸 때 한 번씩 다독여주며 응원해주는 모습이 나에게는 정말 감동이었고 공부를 할 수 있는 원동력이 되었다. 그냥 깨워주는 것이 아니라 응원해주는 조교님들 모습에서 많은 감동을 받았다.</v>
@@ -5767,7 +5767,7 @@
         <v>N수생</v>
       </c>
       <c r="E149" t="str">
-        <v>제가 어떻게 학습을 시작해야 할지 막막했는데 한 가지 방법만 조언해주시는게 아닌, 과목별로 방향성을 잡아주셔서 저의 기존 방법과 선생님이 조언해주신 방법들이 적절히 섞일 수 있었던 점이 가장 좋았습니다!</v>
+        <v>제가 어떻게 학습을 시작해야 할지 막막했는데 한 가지 방법만 조언해주시는 게 아닌, 과목별로 방향성을 잡아주셔서 저의 기존 방법과 선생님이 조언해주신 방법들이 적절히 섞일 수 있었던 점이 가장 좋았습니다!</v>
       </c>
       <c r="F149" t="str">
         <v>가장 좋았던 코칭 시스템과 연관된 내용으로 여러 방향 중에서 각각 방향에 맞는 인강이나 교재 혹은 문제 하나하나 마저도 알려주셨던게 가장 도움이 되고, 특히 문제 추천은 제가 부족한 부분을 집중적으로 채울 수 있어서 가장 유용했습니다.</v>
@@ -5922,7 +5922,7 @@
         <v>윈터스쿨때 다니며 저의 공부 습관을 잡을 수 있었던 것 같습니다. 주기적인 학습 관리와 조언을 해주시고, 학습에 방해가 되지 않도록 휴대폰 관리, 학습 관리에 있어서 도와주신 선생님들께 감사합니다.</v>
       </c>
       <c r="J153" t="str">
-        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는것과 공부하는 것을 관리, 감독해주시는게 도움이 많이 됐어요.</v>
+        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는것과 공부하는 것을 관리, 감독해주시는 게 도움이 많이 됐어요.</v>
       </c>
       <c r="K153" t="str">
         <v/>
@@ -6126,7 +6126,7 @@
         <v>원래 플래너를 적지 않았었는데, 이투스를 다니면서 학습 플래너나 학습 일기를 통해서 본인 스스로 오늘 했던 공부나 보완할 점들을 생각할 수 있었고, 어떤 과목을 앞으로 얼마큼 공부하고, 또 어떻게 공부할지에 관해서 윤곽을 쉽게 잡을 수 있었고, 전반적인 공부의 방향을 정할 수 있어서 좋았습니다.</v>
       </c>
       <c r="G159" t="str">
-        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는것과 공부하는 것을 관리, 감독해주시는게 도움이 많이 됐습니다. 또한 혼자 독서실을 가면 핸드폰을 보거나 공부 이외의 딴짓을 자주 하는데 핸드폰을 제출하고 독서실에 들어가고, 지속적으로 감시를 해주시는것이 무척 좋았습니다.</v>
+        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는것과 공부하는 것을 관리, 감독해주시는 게 도움이 많이 됐습니다. 또한 혼자 독서실을 가면 핸드폰을 보거나 공부 이외의 딴짓을 자주 하는데 핸드폰을 제출하고 독서실에 들어가고, 지속적으로 감시를 해주시는것이 무척 좋았습니다.</v>
       </c>
       <c r="H159" t="str">
         <v>결국 수능에서의 실전 감각이 매우 중요하다고 생각하는데 저는 고3현역이여서 학원에서 다 같이 시험을 보지는 못하였지만 담당 선생님이 모의고사를 챙겨주셔서 주말에 모의고사를 풀 수 있었고, 이러한 실전 경험들이 쌓여서 매우 큰 성적 향상을 이뤄낼 수 있었다고 생각합니다. 또한 문제의 퀄리티 역시 매우 뛰어나고, EBS 반영까지 잘 되어 있어서 실전 연습을 하기에 적합하다고 생각합니다.</v>
@@ -6190,7 +6190,7 @@
         <v>N수생</v>
       </c>
       <c r="E161" t="str">
-        <v>현재 내 상황에서 알맞는 강의 및 문제집을 추천해주시는게 굉장히 맘에 들았습니다. 솔직히 처음 공부를 시작할 때는 뭐부터 해야 할지 감을 잡기 어려웠는데 덕분에 수월하게 진도를 나간 것 같아요</v>
+        <v>현재 내 상황에서 알맞는 강의 및 문제집을 추천해주시는 게 굉장히 맘에 들았습니다. 솔직히 처음 공부를 시작할 때는 뭐부터 해야 할지 감을 잡기 어려웠는데 덕분에 수월하게 진도를 나간 것 같아요</v>
       </c>
       <c r="F161" t="str">
         <v>제 MBTI가 P성향인지라 계획 세우기를 엄청 어려워 했었는데, 선생님이 플래너 작성과 계획 세우기를 코칭해주시고,적극적으로 조언을 해주셔서 체계적인 학습을 수행하는데 아주 큰 도움이 되었습니다.</v>
@@ -6205,7 +6205,7 @@
         <v>재수를 하는 과정이 정말 쉽지 않은 길이었고, 몸도 마음도 정말 많이 지쳤었는데 선생님들의 적극적인 지원과 응원에 참 감동 많이 받았습니다. 2025 한 해 동안 도와주셔서 정말 감사했습니다.</v>
       </c>
       <c r="J161" t="str">
-        <v>강압적이고 딱딱한 분위기가 아니라 다같이 힘내서 공부하는 따뜻한 분위기여서 훨씬 공부에 집중할 수 있었고, 스트레스 관리도 용이했어요.</v>
+        <v>강압적이고 딱딱한 분위기가 아니라 다 같이 힘내서 공부하는 따뜻한 분위기여서 훨씬 공부에 집중할 수 있었고, 스트레스 관리도 용이했어요.</v>
       </c>
       <c r="K161" t="str">
         <v/>
@@ -6277,7 +6277,7 @@
         <v>학생 한 명 한 명을 신경 써 주시며 도와주시고 응원해 주신 덕분에 끝까지 포기하지 않고 노력할 수 있었습니다. 올바른 공부 방법과 태도를 배울 수 있어 더욱 의미 있는 시간이었던 것 같습니다. 앞으로도 선생님들께 배운 것을 바탕으로 더 성장할 수 있도록 노력하겠습니다. 진심으로 감사드립니다!</v>
       </c>
       <c r="J163" t="str">
-        <v>고3 때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던 건 선생님들의 탁월한 입시전략과 상담, 생활환경 조성 덕분이었어요.</v>
+        <v>고3 때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던 건 선생님들의 탁월한 입시 전략과 상담, 생활 환경 조성 덕분이었어요.</v>
       </c>
       <c r="K163" t="str">
         <v/>
@@ -6312,7 +6312,7 @@
         <v>낯선 기숙학원 생활에 적응하느라 몸도 마음도 힘들 때 곁에서 잡아주신 선생님들 덕분에 포기하지 않고 끝까지 완주할 수 있었습니다. 이른 새벽부터 늦은 밤까지 학생들의 사소한 고민까지 귀 기울여 주시던 그 정성 덕분에, 불안했던 수험 공부가 확신으로 바뀔 수 있었다고 생각합니다. 혼자였다면 절대 버티지 못했을 이 길을 함께 걸어주시고, 공부에만 전념할 수 있는 최고의 환경을 만들어주신 선생님들께 진심으로 깊은 감사의 인사를 전하고 싶습니다.</v>
       </c>
       <c r="J164" t="str">
-        <v>휴대폰이 공부하는 데에 가장 방해되는 요인인데 입실할때 휴대폰 내고 나갈때 받을 수 있도록 철저하게 관리해주시니 정말 오직 공부에만 집중할 수 있었어요.</v>
+        <v>휴대폰이 공부하는 데에 가장 방해되는 요인인데 입실할 때 휴대폰 내고 나갈 때 받을 수 있도록 철저하게 관리해주시니 정말 오직 공부에만 집중할 수 있었어요.</v>
       </c>
       <c r="K164" t="str">
         <v/>
@@ -6383,7 +6383,7 @@
 감사합니다감사합니다감사합니다감사합니다 감사합니다. 감사합니다.</v>
       </c>
       <c r="J166" t="str">
-        <v>학습하는 분위기가 조성되어있는 것이 가장 큰 도움이 되었어요.</v>
+        <v>학습하는 분위기가 조성되어 있는 것이 가장 큰 도움이 되었어요.</v>
       </c>
       <c r="K166" t="str">
         <v/>
@@ -6476,7 +6476,7 @@
         <v>담임 선생님과 함께 본인에 맞는 커리큘럼을 짜며 소통할수있어 좋았고 달별로 점검 받으며 부족한 과목의 공부량을 더 늘리거나 하는등의 즉각적인 학습 계획수정이 용이했음,또한 자주 특강을 개설하여 선택학생에게  공부중 부족한 부분을 추가로 공부할 수 있도록 하게해서 좋았음.</v>
       </c>
       <c r="F169" t="str">
-        <v>2주마다 학습멘토와 함께 공부를 점검하며 한무동안 소홀하거나 잘했던 부분을 확인하고 다음주의 공부게획을 점검하는 점이좋았고,학습매니저에게 공부를 점검받아야하므로 공부를 계속 하게되서 좋았고,학습 매니저에게 모르는 부분을 물어보면서 공부할 수있는점도 좋았다</v>
+        <v>2주마다 학습멘토와 함께 공부를 점검하며 한무동안 소홀하거나 잘했던 부분을 확인하고 다음주의 공부게획을 점검하는 점이좋았고,학습매니저에게 공부를 점검받아야하므로 공부를 계속 하게되서 좋았고,학습 매니저에게 모르는 부분을 물어보면서 공부할 수 있는점도 좋았다</v>
       </c>
       <c r="G169" t="str">
         <v>출석할때 핸드폰을 수거해서 공부외에 사소하고 잡다한 다른 요소들을 배제할수 있어 공부에 더 집중할 수있도록 환경을 만들어준 점이 좋았고,저녁에 핸드폰을 가져가면서 학원에서 공부가 끝나고 집갈때  핸드폰을 보며 마음편하게 쉴수있었던것같다</v>
@@ -6490,7 +6490,7 @@
 작년에 재수할때 기억이 지금도 계속 생각이 나네요.작년에 다사다난한 일이있었지만 지나고 보니 다 해프닝일 뿐이네요 작년에 보냈던 기억은 계속 생각날것같아요.좋은 추억을 함께 보낼수있어서 감사했습니다.</v>
       </c>
       <c r="J169" t="str">
-        <v>1대1로 선생님께서 상담을 해주시는게 좋았어요.</v>
+        <v>1대1로 선생님께서 상담을 해주시는 게 좋았어요.</v>
       </c>
       <c r="K169" t="str">
         <v/>
@@ -6683,7 +6683,7 @@
       </c>
       <c r="G174" t="str" xml:space="preserve">
         <v xml:space="preserve">야간 취침시간  관리며  아침 점심  다  통제시간도 철저했으며  식사 외  간식 제안  라면등   특식으로  제공되겠음 해주셔서  보기좋았습니다._x000d_
-아이들이  좋아하는것만 해줄 수있는데  적당히 잘 통제되어서  만족했습니다</v>
+아이들이  좋아하는것만 해줄 수 있는데  적당히 잘 통제되어서  만족했습니다</v>
       </c>
       <c r="H174" t="str" xml:space="preserve">
         <v xml:space="preserve">학생들이  정기적으로 시험을 보면서  자기 위치를  알 수 있어서  좋았습니다._x000d_
@@ -7008,7 +7008,7 @@
         <v>스스로 강의를 보고 교재를 풀면서 공부해야 하는 시스템이기 때문에 강의에서 해결하기 어려운 개념이나 문제가 생겼을 때, 각 학원에 상주하고 계신 담당 과목 선생님께 그때마다 여쭤볼 수 있어서 공부하는데 큰 도움이 되었습니다.</v>
       </c>
       <c r="G183" t="str">
-        <v>강압적이고 딱딱한 분위기가 아니라 다같이 힘내서 공부하는 따뜻한 분위기여서 훨씬 공부에 집중할 수 있었고, 스트레스 관리도 용이했습니다. 특히 중간에 공부하다가 졸았을 때, 한번 씩 깨워주시는데 바로 흔들어서 깨워주시는게 아니라 토닥이듯이 깨워주셔서 위로 받는 느낌이 컸고 다시 마음을 다잡고 공부할 수 있었습니다.</v>
+        <v>강압적이고 딱딱한 분위기가 아니라 다 같이 힘내서 공부하는 따뜻한 분위기여서 훨씬 공부에 집중할 수 있었고, 스트레스 관리도 용이했습니다. 특히 중간에 공부하다가 졸았을 때, 한번 씩 깨워주시는데 바로 흔들어서 깨워주시는게 아니라 토닥이듯이 깨워주셔서 위로 받는 느낌이 컸고 다시 마음을 다잡고 공부할 수 있었습니다.</v>
       </c>
       <c r="H183" t="str">
         <v>평가원 모의고사와 조금 다르긴 하지만 이투스 모의고사가 거의 매달 치뤄졌기 때문에 시간 관리와 개념 및 문제 풀이에 큰 도움을 받았습니다. 특히 3월, 6월 모의고사 같은 중요한 시험을 보는데 있어서 감을 유지하는데도 이점이 있었습니다. 또한 시험 이후 진행하는 오답노트를 통해 나의 부족한 점을 채울 수 있다는 점도 효율적인 학습을 진행하는데 도움이 되었습니다.</v>
@@ -7178,7 +7178,7 @@
         <v>N수생</v>
       </c>
       <c r="E188" t="str" xml:space="preserve">
-        <v xml:space="preserve">학습적인 면 뿐만아니라 멘탈관리도 해주시고 고민상담도 해주시고 공부잘하는 친구같은 느낌으로 학생들이 가장 선호하는 형식의 멘토였음_x000d_
+        <v xml:space="preserve">학습적인 면 뿐만아니라 멘탈 관리도 해주시고 고민상담도 해주시고 공부잘하는 친구같은 느낌으로 학생들이 가장 선호하는 형식의 멘토였음_x000d_
 학습적인 부분에서는 어디서도 듣지못한 공부법을 여럿 들었고 실제로 도움이 되었음</v>
       </c>
       <c r="F188" t="str">
@@ -7265,7 +7265,7 @@
 고마운 존재였습니다. 결코 쉽지 않은 난이도로 항상 저를 당황시켰는데 오히려 시험준비에 더 열심히 임할 수 있었던 것 같습니다.</v>
       </c>
       <c r="I190" t="str">
-        <v>작년, 걱정과 불안이 가득한 입시상담을 받았던게 새록새록 떠오르는데 저는 지금 그 때의 상담에서 선생님께서 말씀하신 대학의 학과에 입학했습니다! 고3 때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던 건 이투스 강서지점 선생님들의 탁월한 입시전략과 상담, 생활환경 조성 덕분이었습니다. 저의 처음이자 마지막 재수를 성공적으로 마치게 해주신 이투스 강서지점 선생님들께 감사를 표합니다!</v>
+        <v>작년, 걱정과 불안이 가득한 입시상담을 받았던게 새록새록 떠오르는데 저는 지금 그 때의 상담에서 선생님께서 말씀하신 대학의 학과에 입학했습니다! 고3 때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던 건 이투스 강서지점 선생님들의 탁월한 입시 전략과 상담, 생활 환경 조성 덕분이었습니다. 저의 처음이자 마지막 재수를 성공적으로 마치게 해주신 이투스 강서지점 선생님들께 감사를 표합니다!</v>
       </c>
       <c r="J190" t="str">
         <v>생활 상담을 포함한 코칭 시스템은 공부 외적인 부분까지 함께 관리해 준다는 점에서 의미가 있었어요.</v>
@@ -7482,7 +7482,7 @@
         <v>자신에게 맞는 인강 선생님을 고르는게 수험 공부에 있어 중요한 부분을 차지한다고 생각하는데 그런 점에 있어서 많은 도움을 받았던거 같습니다. 꾸준히 진도 체크해주면서 인강 수강을 하니 좋은 결과를 얻을 수 있었습니다.</v>
       </c>
       <c r="G196" t="str">
-        <v>휴대폰이 공부하는 데에 가장 방해되는 요인인데 입실할때 휴대폰 내고 나갈때 받을 수 있도록 철저하게 관리해주시니 정말 오직 공부에만 집중할 수 있었습니다. 특히 식사시간에 휴대폰을 보지 않고 차라리 산책을 갔다오니 멘탈적으로 많은 도움이 됐습니다.</v>
+        <v>휴대폰이 공부하는 데에 가장 방해되는 요인인데 입실할 때 휴대폰 내고 나갈 때 받을 수 있도록 철저하게 관리해주시니 정말 오직 공부에만 집중할 수 있었습니다. 특히 식사시간에 휴대폰을 보지 않고 차라리 산책을 갔다오니 멘탈적으로 많은 도움이 됐습니다.</v>
       </c>
       <c r="H196" t="str">
         <v>수능이 다가오다보면 영어에 소홀해지기 마련인데 게속 단어 테스트 보면서 영어 감을 익히고 단어도 외우다보니까 영어에서 이익을 볼 수 있었습니다. 특히 올해같이 어려웠던 영어 수능에서 많은 도움이 되었습니다.</v>
@@ -7571,7 +7571,7 @@
         <v>재수라는 길고 외로운 싸움을 하는 동안 곁에서 아낌없이 도움을 주신 선생님께 진심으로 감사드립니다. 공부 습관을 잡을 수 있도록 세심하게 지도해 주시고, 힘들고 지칠 때마다 다시 일어설 수 있도록 따뜻하게 격려해 주신 덕분에 포기하지 않고 끝까지 나아갈 수 있었습니다. 저 혼자였다면 방향을 잃고 쉽게 흔들렸겠지만, 선생님의 꾸준한 관심이 있었기에 흔들릴 때마다 다시 중심을 잡을 수 있었습니다. 재수 생활의 크고 작은 순간마다 함께해 주셔서 진심으로 감사드리고, 선생님의 가르침을 발판 삼아 진학한 대학에서 열심히 하며 최선을 다하겠습니다.</v>
       </c>
       <c r="J198" t="str">
-        <v>멘탈적인 부분의 영향력을 무시할 수 없는데, 그 멘탈관리 부분에서 큰 도움이 되었어요.</v>
+        <v>멘탈적인 부분의 영향력을 무시할 수 없는데, 그 멘탈 관리 부분에서 큰 도움이 되었어요.</v>
       </c>
       <c r="K198" t="str">
         <v/>
@@ -7633,7 +7633,7 @@
         <v>인강에 대한 경험이 없어 어떤 강의를 수강하면 좋을지에 대한 고민이 있었습니다. 현재 학습 수준 및 목표에 따른 인강강사 및 교재 추천을 받고 고민을 해결하여 시간을 절약하고 효율적으로 학습할 수 있었습니다.</v>
       </c>
       <c r="G200" t="str">
-        <v>학습하는 분위기가 조성되어있는 것이 가장 큰 도움이 되었습니다. 또한 학습시간에 실수로 조는 경우가 종종 있었는데, 찾아와 직접 깨워주셨던 것이 학습의 흐름 유지와 학습태도 향상에 큰 도움이 되었습니다.</v>
+        <v>학습하는 분위기가 조성되어 있는 것이 가장 큰 도움이 되었습니다. 또한 학습시간에 실수로 조는 경우가 종종 있었는데, 찾아와 직접 깨워주셨던 것이 학습의 흐름 유지와 학습태도 향상에 큰 도움이 되었습니다.</v>
       </c>
       <c r="H200" t="str">
         <v>주기적으로 전국 모의고사를 볼 수 있었던 점이 실제 수능 시험장에 대한 적응을 크게 도왔습니다. 구체적 시간 관리 등 수능 시험에 대한 실전같은 연습이 실제 수능 시험에서 많은 도움이 되었습니다.</v>
@@ -7829,7 +7829,7 @@
         <v>여태껏 제대로 공부해본적 없던 제가 태어나서 가장 오랜기간 열심히 준비했던 재수기간이였습니다. 약 9개월간 다니며 큰 불편함 없었고 여러 선생님들의 케어와 격려를 받으며 끝까지 포기하지않고 잘 마무리했었던 것 같습니다.</v>
       </c>
       <c r="J205" t="str">
-        <v>학습 상담으로 맞춤 인강·교재를 선택하고, 방화벽과 보카 테스트로 집중력을 높였어요.</v>
+        <v>학습 상담으로 맞춤 인강·교재를 선택하고, 방화벽과 단어 테스트로 집중력을 높였어요.</v>
       </c>
       <c r="K205" t="str">
         <v>학습 관리, 방화벽</v>
@@ -7919,7 +7919,7 @@
         <v>N수생</v>
       </c>
       <c r="E208" t="str">
-        <v>1대1로 선생님께서 상담을 해주시는게 좋았습니다. 담당하는 학생이 많았지만 상담할때 어떤 방향으로 원서접수를 해야 좋을지, 나에게 맞는 학습 방법과 진도를 하나부터 열까지 도와주셨습니다. 이것은 관리형독서실이나 스카에서는 없는 이투스에서만 경험 가능한 시스템이라 좋았습니다</v>
+        <v>1대1로 선생님께서 상담을 해주시는 게 좋았습니다. 담당하는 학생이 많았지만 상담할때 어떤 방향으로 원서접수를 해야 좋을지, 나에게 맞는 학습 방법과 진도를 하나부터 열까지 도와주셨습니다. 이것은 관리형독서실이나 스카에서는 없는 이투스에서만 경험 가능한 시스템이라 좋았습니다</v>
       </c>
       <c r="F208" t="str">
         <v>질문을 원하는 학생이 많아 질문이 있을때 바로 질문 신청을 하고 몇시간 혹은 며칠을 기다리면 질의응답을 받을 수 있었습니다. 그래도 담당 과목 선생님을 직접 고를 수 있으며 이해가 갈 때까지 차근차근 설명해주셨습니다. 덕분에 정말 어려웠던 과목을 수능에서 좋은 성적을 받을 수 있었습니다. 또한 같은 선생님께 질문을 계속하다보면 어느정도의 유대감이 쌓이고 질문 하는 것이 정말 편해지고 이해도 더 잘되는 것 같았습니다.</v>
@@ -7960,7 +7960,7 @@
         <v>평소 계획을 세우고 공부하지 않고 그때그때 하고싶은 공부를 하여 공부 비중이 고르지않았다. 근데 주단위로 하루에 무엇을 얼만큼 공부할지 계획을 같이 세우고 피드백해주셔서 고르게 공부할 수 있었다.</v>
       </c>
       <c r="G209" t="str">
-        <v>잠이 많은 편이라 공부할 때 많이 졸았는데 학습코칭 선생님께서 졸음 관리를 확실하게 지도해주셔서 많은 도움이 되었다. 졸릴 때는 자리에서 벗어나 밖에 서서 공부하라고 해주시는게 도움됐다.</v>
+        <v>잠이 많은 편이라 공부할 때 많이 졸았는데 학습 코칭 선생님께서 졸음 관리를 확실하게 지도해주셔서 많은 도움이 되었다. 졸릴 때는 자리에서 벗어나 밖에 서서 공부하라고 해주시는 게 도움됐다.</v>
       </c>
       <c r="H209" t="str">
         <v>실전처럼 모의고사를 볼 수 있는 환경이 마련되어 있어 실제 시험을 대비하는 데 큰 도움이 되었다. 시험 분위기를 미리 경험할 수 있어서 긴장감 조절에도 좋았고 문제 풀이 감각을 익히는 데 유익했다. 그리고 콘텐츠를 신청할 수 있는 방식이 가까워서 번거롭지 않고 편리하게 이용할 수 있었던 점도 좋았다.</v>
@@ -8379,7 +8379,7 @@
         <v>수시원서를 쓰기전에 한 명씩 친절하게 상담을 해주십니다. 각자의 모의고사와 실모, 내신 성적을 기반으로 같은 성적이여도 최선의 선택이 될 수 있게 같이 고민해주십니다. 입시전형요강에 댜해 빠삭하게 알고 있고 관련 설명도 자주 진행합니다.</v>
       </c>
       <c r="F221" t="str">
-        <v>일요일마다 모의고사를 보고 며칠 뒤에 성적표를 나눠준다. 더프처럼 다같이 보는 모의고사가 아니더라도 학원내에서 평균과 컷을 산출하여 알려주는 점이 매 모의고사에 진심으로 임하게 되는 것 같다.</v>
+        <v>일요일마다 모의고사를 보고 며칠 뒤에 성적표를 나눠준다. 더프처럼 다 같이 보는 모의고사가 아니더라도 학원내에서 평균과 컷을 산출하여 알려주는 점이 매 모의고사에 진심으로 임하게 되는 것 같다.</v>
       </c>
       <c r="G221" t="str">
         <v>기숙의 가장 큰 장점이 외부와 차단되는 것이라고 생각하는데 정말 방화벽이 잘 되어있어서 태블릿으로 딴짓할 수 없고 그만큼 그 시간들이 공부 시간으로 이어지기 때문에 가장 공부에 도움이 된다</v>
@@ -8703,7 +8703,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E230" t="str">
-        <v>자주 학습 상태를 체크해주시고 상담도 여러번이 있어서 좋았습니다. 그리고 매주마다 수학과 국어 테스트를 보고 수학은 해설까지 해주시는게 정말 도움 많이 된 것 같습니다. 주마다 하는 테스트 덕분에 더 열심히 공부한 것 같습니다.</v>
+        <v>자주 학습 상태를 체크해주시고 상담도 여러번이 있어서 좋았습니다. 그리고 매주마다 수학과 국어 테스트를 보고 수학은 해설까지 해주시는 게 정말 도움 많이 된 것 같습니다. 주마다 하는 테스트 덕분에 더 열심히 공부한 것 같습니다.</v>
       </c>
       <c r="F230" t="str">
         <v>제가 원래 꼼꼼하게 계획을 세워서 공부하는 스타일이 아니라 그때 그때 하고 싶은 과목만 공부를 쭉 하다가 또 다른 과목이 하고 싶으면 그 과목만 해서 공부 시간의 격차가 너무 심했었는데 플래너를 작성하면서 그날 무슨 공부를 할지 고민하지 않았던게 좋았습니다</v>
@@ -9289,7 +9289,7 @@
         <v>1:1 질의응답은 내가 이해하지 못한 부분을 바로 질문하고 해결할 수 있어 매우 유용했다. 수업에서는 놓치기 쉬운 세부 내용까지 자세히 설명을 들을 수 있었고, 나의 수준에 맞춘 설명 덕분에 이해도가 훨씬 높아졌다. 또한 즉각적인 피드백을 통해 잘못 알고 있던 개념을 바로잡을 수 있어 학습의 정확성과 효율성을 높이는 데 큰 도움이 되었다. 부담 없이 질문할 수 있어 학습에 큰 도움이 되었다.</v>
       </c>
       <c r="G246" t="str">
-        <v>면학 분위기 속에서 감독이 이루어지니 자연스럽게 집중력이 높아지고 공부에 몰입할 수 있어 좋았다. 주변 모두가 학습에 집중하는 환경이라 흐트러지기 어려웠고, 감독이 있어 긴장감과 책임감도 생겨 스스로를 더 잘 통제할 수 있었다. 그 결과 불필요한 시간 낭비가 줄고 학습 효율이 크게 향상되었다. 또한 식사 후 식곤증에 빠지지 않게 관리해주시는게 큰 도움이 되었다.</v>
+        <v>면학 분위기 속에서 감독이 이루어지니 자연스럽게 집중력이 높아지고 공부에 몰입할 수 있어 좋았다. 주변 모두가 학습에 집중하는 환경이라 흐트러지기 어려웠고, 감독이 있어 긴장감과 책임감도 생겨 스스로를 더 잘 통제할 수 있었다. 그 결과 불필요한 시간 낭비가 줄고 학습 효율이 크게 향상되었다. 또한 식사 후 식곤증에 빠지지 않게 관리해주시는 게 큰 도움이 되었다.</v>
       </c>
       <c r="H246" t="str">
         <v>이투스 구독 시스템은 다양한 강의를 한 번에 자유롭게 이용할 수 있어 매우 효율적이었다. 과목별로 필요한 강의를 추가 비용 부담 없이 선택해 들을 수 있어 학습 범위를 넓히는 데 도움이 되었고, 자신의 수준과 목표에 맞게 강의를 유연하게 조합할 수 있었다. 또한 반복 수강이 가능해 부족한 부분을 여러 번 복습하며 이해도를 높일 수 있어 학습 효과를 극대화할 수 있었다. 내가 원하는 부분만 듣고 싶었는데 비용 부담 없이 여러 강의를 들을 수 있어서 좋았다.</v>
@@ -9725,7 +9725,7 @@
         <v>출석체크를 통한 규칙적인 생활의 강제성, 꾸준함 그리고 만약 혼자 공부했더라면 전자기기 케어를 못하고 유튜브만 봤을 텐데 누군가가 날 지켜보고 있다고 생각하니 딴 짓을 안 하게 됨</v>
       </c>
       <c r="G258" t="str">
-        <v>다들 열심히 하는 학습 분위기 속에서 같이 열심히 공부할 수 있었음 만약 다같이 은근히 노는 분위기였다면 나도 휩쓸려갔을 듯 또 잡담도 거의 나누지 않는 분위기였던 게 특히 좋았음</v>
+        <v>다들 열심히 하는 학습 분위기 속에서 같이 열심히 공부할 수 있었음 만약 다 같이 은근히 노는 분위기였다면 나도 휩쓸려갔을 듯 또 잡담도 거의 나누지 않는 분위기였던 게 특히 좋았음</v>
       </c>
       <c r="H258" t="str">
         <v>사이트 들어가서 영어듣기 평가를 자주 했었다 솔직히 영어듣기는 따로 종이책 사기는 부담스러운데 그냥 간편하게 패드로 답 체크하고 들을 수 있어서 편했다 특히 학원에서 이용하니 다른 sns에 안 들어가고 바로 사이트&gt;영듣 들어가서 할 수 있었다</v>
@@ -10377,7 +10377,7 @@
         <v>아무래도 수험 생활의 가장 큰 적은 인터넷으로 즐길 수 있는 오락거리와 미디어라고 생각합니다. 하지만 이투스 247에서는 와이파이 방화벽을 통해 애초에 접속 가능성을 막고 학습사이트만 들어갈 수 있게 설계되어있어 스스로 자제력이 부족해 인터넷 사용시간이 많았던 저에게 도움이 되었습니다.</v>
       </c>
       <c r="H275" t="str">
-        <v>영어가 현재 수능 체제에서 절대평가 과목이기도 해서 영어를 소홀히 하는 경향도 있었고 특히나 단어같은 경우는 귀찮아서 안 외우는 경우가 많았습니다. 단어를 선별해서 자료를 주신 덕에 외우기도 편리했고 다같이 시험을 봐 강제성이 생긴 덕분에 꾸준히 단어를 외울 수 있었습니다.</v>
+        <v>영어가 현재 수능 체제에서 절대평가 과목이기도 해서 영어를 소홀히 하는 경향도 있었고 특히나 단어같은 경우는 귀찮아서 안 외우는 경우가 많았습니다. 단어를 선별해서 자료를 주신 덕에 외우기도 편리했고 다 같이 시험을 봐 강제성이 생긴 덕분에 꾸준히 단어를 외울 수 있었습니다.</v>
       </c>
       <c r="I275" t="str">
         <v>힘들었던 재수 생활이었지만 독학기숙에서 시간을 보낼 수 있었기에 큰 힘이 되었던 것 같습니다. 힘들 때 상담해주시고, 방향성을 잡아주신 덕에 수월하게 공부했던 것 같습니다. 선생님들 덕분에 2026 입시를 마무리할 수 있었습니다. 감사합니다!</v>
@@ -10635,7 +10635,7 @@
         <v>영단어를 소홀히 하기 쉬운데 그 점을 아주 잘 바로잡아준거같다. 영단어는 꾸준히 매일 조금씩 반복학습으로 하는게 중요한데 그 중요지점을 잘 파고든 시스템같다. 그 지점에서 아주 유용하다고 생각한다</v>
       </c>
       <c r="I282" t="str">
-        <v>감사합니다. 항상 수고 많으십니다. 재수라는게 사람마다 정도는 다르겠지만 멘탈적인 부분의 영향력을 무시할 수 없어서 그 멘탈관리에 조금이나마 도움이 되지 않았나 싶다. 수능공부는 결과만 남는게 절대 아니고 과정 속에서도 얻어가는 점이 분명히 있기에 이런 독학재수학원의 경험이 개인적으로 기억에 깊게 남아있다.</v>
+        <v>감사합니다. 항상 수고 많으십니다. 재수라는게 사람마다 정도는 다르겠지만 멘탈적인 부분의 영향력을 무시할 수 없어서 그 멘탈 관리에 조금이나마 도움이 되지 않았나 싶다. 수능공부는 결과만 남는게 절대 아니고 과정 속에서도 얻어가는 점이 분명히 있기에 이런 독학재수학원의 경험이 개인적으로 기억에 깊게 남아있다.</v>
       </c>
       <c r="J282" t="str">
         <v>학습 슬럼프를 겪을 때 선생님이 지속적으로 상담을 통해 저에게 맞는 공부 방법을 찾아주셔서 계속 공부할 수 있었습니다.</v>
@@ -10973,7 +10973,7 @@
         <v>N수생</v>
       </c>
       <c r="E292" t="str">
-        <v>학습코칭이 가장 유용했습니다. 국어, 영어, 수학 과목별로 담당 선생님들이 한 분씩 계셔서 모르는 문제를 질문하거나 세부 학습플랜을 세우는 데에 큰 도움을 받았습니다. 담임 선생님께 입시상담을 하고, 과목별 담당 선생님들께 코칭을 받은 덕에 성적을 빨리 향상시킬 수 있었습니다.</v>
+        <v>학습 코칭이 가장 유용했습니다. 국어, 영어, 수학 과목별로 담당 선생님들이 한 분씩 계셔서 모르는 문제를 질문하거나 세부 학습플랜을 세우는 데에 큰 도움을 받았습니다. 담임 선생님께 입시상담을 하고, 과목별 담당 선생님들께 코칭을 받은 덕에 성적을 빨리 향상시킬 수 있었습니다.</v>
       </c>
       <c r="F292" t="str">
         <v>성적 리포팅 및 관리가 도움이 되었습니다. 모의고사 응시 성적과 수능 예상 점수까지 리포팅되어 직관적으로 저의 위치를 알 수 있었고, 과목 간의 밸런스를 맞추기에도 수월했습니다. 월별로 성적 추이를 비교하며 공부하니 동기부여가 되어 더 열심히 공부했던 거 같습니다.</v>
@@ -11341,7 +11341,7 @@
       </c>
       <c r="I302" t="str" xml:space="preserve">
         <v xml:space="preserve">1년 동안 저를 지도해주신 모든 선생님들께 정말 감사합니다 덕분에 지금 제가 대학생이 되어 캠퍼스 생활도 하고 즐겁게 지낼 수 있다고 생각합니다_x000d_
-특히 멘탈관리에 많은 도움을 주신 em반 담임 선생님 정은숙 선생님, 항상 맛있는 밥을 만들어주셨던 동원홈푸드 영양사님께 감사합니다!</v>
+특히 멘탈 관리에 많은 도움을 주신 em반 담임 선생님 정은숙 선생님, 항상 맛있는 밥을 만들어주셨던 동원홈푸드 영양사님께 감사합니다!</v>
       </c>
       <c r="J302" t="str">
         <v>하루 일정을 체계적으로 관리해 주셔서 자연스럽게 규칙적인 생활 습관을 만들 수 있어 좋았습니다.</v>
@@ -11696,10 +11696,10 @@
         <v>면학 분위기가 조용해서 공부에 집중하기 좋은 환경이었으며 선생님들께서 돌아다니면서 졸고 있는 학생을 깨운다거나 시끄러운 학생들에게 주의를 주는 등 면학 분위기에 매우 신경써주셨습니다.</v>
       </c>
       <c r="H312" t="str">
-        <v>수능을 앞두고 모의고사 문제를 푸는 것이 실전감각을 키우는데 매우 중요하다고 생각하는데 이투스 모의고사는 실제 모의고사와 비슷한 형태이며 학원에서 다같이 보기 때문에 수능을 준비하는데 도움이 되었습니다.</v>
+        <v>수능을 앞두고 모의고사 문제를 푸는 것이 실전감각을 키우는데 매우 중요하다고 생각하는데 이투스 모의고사는 실제 모의고사와 비슷한 형태이며 학원에서 다 같이 보기 때문에 수능을 준비하는데 도움이 되었습니다.</v>
       </c>
       <c r="I312" t="str">
-        <v>1년 동안 학생들의 학습코칭뿐만 아니라 멘탈관리와 지친 학생들을 위한 간식 이벤트 등 많은 도움을 주셔서 매우 감사합니다! 덕분에 1년을 포기하지 않고  끝까지 잘 버틸 수 있었습니다.</v>
+        <v>1년 동안 학생들의 학습 코칭뿐만 아니라 멘탈 관리와 지친 학생들을 위한 간식 이벤트 등 많은 도움을 주셔서 매우 감사합니다! 덕분에 1년을 포기하지 않고  끝까지 잘 버틸 수 있었습니다.</v>
       </c>
       <c r="J312" t="str">
         <v>학습 코칭뿐만 아니라 지친 학생들을 위해 다양한 이벤트도 진행해 주시고, 심리 상담도 해주셔서 끝까지 해낼 수 있었어요.</v>
@@ -12298,7 +12298,7 @@
         <v>생활 관리 시스템은 규칙적인 생활 습관을 형성할 수 있도록 도와주어 일상 전반의 균형을 유지하는 데 유용했습니다. 정해진 시간에 맞춰 생활하도록 지도해 주어 생활 리듬이 안정되었고, 타 학생들과 함께 생활하면서 서로에게 피해를 주지 않도록 책임감도 기를 수 있었습니다. 또한 어려움이 있을 때에는 상담을 통해 도움을 받을 수 있어 보다 안정적인 생활을 이어가는 데 큰 도움이 되었습니다.</v>
       </c>
       <c r="H329" t="str">
-        <v>제공된 콘텐츠 중에서는 단어 보카 테스트와 이투스 모의고사가 특히 유용했습니다. 보카 테스트를 통해 어휘를 반복적으로 점검하며 암기 효과를 높일 수 있었고, 이투스 모의고사를 통해 실제 시험과 유사한 환경에서 자신의 실력을 확인하고 부족한 부분을 파악할 수 있었습니다. 이러한 콘텐츠들이 학습의 방향을 잡고 실력을 향상시키는 데 큰 도움이 되었습니다.</v>
+        <v>제공된 콘텐츠 중에서는 단어 단어 테스트와 이투스 모의고사가 특히 유용했습니다. 단어 테스트를 통해 어휘를 반복적으로 점검하며 암기 효과를 높일 수 있었고, 이투스 모의고사를 통해 실제 시험과 유사한 환경에서 자신의 실력을 확인하고 부족한 부분을 파악할 수 있었습니다. 이러한 콘텐츠들이 학습의 방향을 잡고 실력을 향상시키는 데 큰 도움이 되었습니다.</v>
       </c>
       <c r="I329" t="str">
         <v>이투스247학원 선생님들께 진심으로 감사의 말씀을 전해드립니다. 항상 학생들의 학습과 생활을 세심하게 살펴주시고, 힘들 때마다 따뜻하게 상담해 주셔서 큰 힘이 되었습니다. 덕분에 흔들리지 않고 꾸준히 공부할 수 있었으며, 스스로를 관리하는 능력도 많이 성장할 수 있었습니다. 앞으로도 선생님들께서 해주신 지도와 응원을 잊지 않고 더욱 노력하겠습니다. 진심으로 감사합니다.</v>
@@ -12405,7 +12405,7 @@
         <v>일반 독서실이나 관리형 독서실들과는 다르게 핵심과목인 국어,영어,수학 전공자 선생님들께서 상주하고 계셔서 문제를 풀다가 막힘이 오거나 특정과목에 대한 상담이 필요할때 즉각적인 질의응답을 통한 학습이 가능하다는 점이 가장 큰 장점이였다. 온라인 강의와 사이트를 이용하다보면 강의와 개념, 문제들에 대한 질문을 qna 게시판을 통해서만 질문이 가능한데 이는 시간도 오래걸리고 대면으로 질문하는것이 아니기에 한계가 존재했었다. 또한 이투스 247 목동 졸업생들이 멘토로 근무를 하여 특정 탐구 과목들에 대한 피드백과 질문, 조언들을 얻을 수 있다는 점에서 이투스 247 목동만의 독보적이고 차별적인 시스템이다.</v>
       </c>
       <c r="G332" t="str">
-        <v>공부를 하는 학생 입장에서 독학재수학원을 생각할때 중요시하게 고려하는 요소가 면학 분위기 입니다. 그러한점에서 목동 이투스 247은 다양한 시스템을 통한 최고의 면학 분위기를 제공해주었습니다. 우선 매너타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다같이 집중할 수 있는 공부 환경을 제공해줍니다. 또한 학생들이 학습중 자지 않도록 상시로 감독 선생님께서 자습실을 비롯한 공용학습 공간까지 꼼꼼히 돌아다니시며 모든 학생이 열심히 공부를 할 수 있게 도와주십니다.</v>
+        <v>공부를 하는 학생 입장에서 독학재수학원을 생각할때 중요시하게 고려하는 요소가 면학 분위기 입니다. 그러한점에서 목동 이투스 247은 다양한 시스템을 통한 최고의 면학 분위기를 제공해주었습니다. 우선 매너타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다 같이 집중할 수 있는 공부 환경을 제공해줍니다. 또한 학생들이 학습중 자지 않도록 상시로 감독 선생님께서 자습실을 비롯한 공용학습 공간까지 꼼꼼히 돌아다니시며 모든 학생이 열심히 공부를 할 수 있게 도와주십니다.</v>
       </c>
       <c r="H332" t="str">
         <v>목동 이투스 247점에서는 단어테스트반을 모집하여 매주 영단어 테스트를 봅니다. 학생들이 가장 귀찮아하고 소홀히하는 영단어 외우기를 같은 학생들과 함께 매주 테스트를 보며 매주 빼먹지 않게 외우게된다는 장점이 있습니다.</v>
@@ -12414,7 +12414,7 @@
         <v>항상 입시 스트레스로와 몸 건강으로 인해 학원에게 피해를 많이 끼쳤지만 그럼에도 불구하고 항상 격려해주시고 힘을 내게 도와주셔서 덕분에 끝까지 입시를 마칠 수 있었습니다. 모두 선생님들 덕분입니다. 제 입시에서 이투스 247 선생님들을 만난것이 가장 큰 행운이였습니다 감사합니다..!</v>
       </c>
       <c r="J332" t="str">
-        <v>매너 타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다같이 집중할 수 있는 공부 환경을 제공해주셨어요.</v>
+        <v>매너 타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다 같이 집중할 수 있는 공부 환경을 제공해주셨어요.</v>
       </c>
       <c r="K332" t="str">
         <v/>
@@ -12580,7 +12580,7 @@
         <v>인터넷강의의 가장 큰 단점은 커리가 너무 많다는점인데 선생님과 상담후 나에게 딱 맞는 강의를 수강하는데 도움이 많이 되었습니다.반수생이었던 저는 시간이 부족해 선택과 집중이 되게 중요했는데 선생님의 도움이 없었더라면 혼자 방황했을꺼 같습니다.</v>
       </c>
       <c r="G337" t="str">
-        <v>현역때의 수능실패 원인을 되돌아보자면 휴대폰이었습니다.공부를 하러 도서관애 갔어도 휴대폰만 하고 돌아오던 시간이 대부분이었습니다.휴대폰을 등교때 제출함으로써 집중력 분산도 안되고 온전히 공부에만 집중할 수있는 환경이 만들어졌습니다.</v>
+        <v>현역때의 수능실패 원인을 되돌아보자면 휴대폰이었습니다.공부를 하러 도서관애 갔어도 휴대폰만 하고 돌아오던 시간이 대부분이었습니다.휴대폰을 등교 때 제출함으로써 집중력 분산도 안되고 온전히 공부에만 집중할 수 있는 환경이 만들어졌습니다.</v>
       </c>
       <c r="H337" t="str">
         <v>유명하신 선생님들의 강의를 무료로 수강할수있어서 좋았습니다.특히 국어영역의 김민경 선생님의 강의중 ebs 연계에 대한 강의를 자투리 시간에 수강함으로써 ebs 독서 연계에 대해 대비를 더욱 철저히 하게 될 수 있었습니다.</v>
@@ -12589,7 +12589,7 @@
         <v>5개월 동안 성적을 끌어올랄수 았었던건 이투스 247 선생님분들이 있었기에 가능했습니다.혼자였다면 백분위 10이 절대로 상승하지 못했을것입니다.5개월 동안 신경써주셔서 정말 감사했습니다</v>
       </c>
       <c r="J337" t="str">
-        <v>휴대폰을 등교때 제출함으로써 집중력 분산도 안되고 온전히 공부에만 집중할 수있는 환경이 만들어졌었어요.</v>
+        <v>휴대폰을 등교 때 제출함으로써 집중력 분산도 안되고 온전히 공부에만 집중할 수 있는 환경이 만들어졌었어요.</v>
       </c>
       <c r="K337" t="str">
         <v/>
@@ -12714,7 +12714,7 @@
         <v>반수생</v>
       </c>
       <c r="E341" t="str">
-        <v>매주 학습 계획표를 짜서 학습 하는 과정이 수월했습니다. 계획을 짜는 과정에서 부족한 부분과 필요하지 않은 학습에 대해 인지하는 시간을 가질 수 있었습니다. 또한 수준에 맞는 교재와 실모를 추천 받을 수 있어서 좋았습니다.</v>
+        <v>매주 학습 계획표를 짜서 학습하는 과정이 수월했습니다. 계획을 짜는 과정에서 부족한 부분과 필요하지 않은 학습에 대해 인지하는 시간을 가질 수 있었습니다. 또한 수준에 맞는 교재와 실모를 추천 받을 수 있어서 좋았습니다.</v>
       </c>
       <c r="F341" t="str">
         <v>본인 수준에 맞는 인강과 교재를 통해 무리하지 않은 학습을 할 수 있었습니다. 그덕에 문풀 실력과 성적이 한단계씩 오르는 경험을 하였습니다. 학업 성취를 느끼는 기회가 되었습니다.</v>
@@ -12729,7 +12729,7 @@
         <v>얼마 안되는 기간동안 좌절에 빠지는 시간도 종종 있었는데 닦달않고 북돋아주셔서 감사했습니다. 덕분에 반수기간 동안 학습적인 부분을 제외하고도 심리적으로도 도움을 많이 받았습니다. 감사인사를 전할 기회가 이렇게 생겨서 다행입니다.</v>
       </c>
       <c r="J341" t="str">
-        <v>매주 학습 계획표를 짜서 학습 하는 과정이 수월했어요.</v>
+        <v>매주 학습 계획표를 짜서 학습하는 과정이 수월했어요.</v>
       </c>
       <c r="K341" t="str">
         <v>학습 계획</v>
@@ -13200,7 +13200,7 @@
         <v>N수생</v>
       </c>
       <c r="E354" t="str">
-        <v>가나다군의 입시전략을 세우는 데에 유용했다. 진학사 칸수만으로는 알기 힘든 정보로 좀 더 현실적인 전략을 세워주셨다. 지난 학생들의 정보를 통해 몇칸정도 채워지면 어느정도 가능성이 있는지 알려주셨고 그대로 들어맞아 결국 원하는 대학에 합격할 수 있었다.</v>
+        <v>가나다군의 입시 전략을 세우는 데에 유용했다. 진학사 칸수만으로는 알기 힘든 정보로 좀 더 현실적인 전략을 세워주셨다. 지난 학생들의 정보를 통해 몇칸정도 채워지면 어느정도 가능성이 있는지 알려주셨고 그대로 들어맞아 결국 원하는 대학에 합격할 수 있었다.</v>
       </c>
       <c r="F354" t="str">
         <v>문제를 풀다보면 인강이나 답지만으로는 해결할 수 없는 경우가 종종 있다. 이때 혼자서 해결하려고 했으면 막막했을텐데 담당 선생님께 여쭈어 바로바로 해결할 수 있어 학습이 원활했다. 또 다양한 풀이방법을 선생님과 함께 고민할 수 있어 학업능력이 향상되었다</v>
@@ -13317,10 +13317,10 @@
         <v>아무래도 태블릿과 핸드폰이 수험 생활에서 제일 큰 방해요인이 아닐까라고 생각이 드는데, 이투스247김포점은 말로만 태블릿과 핸드폰을 하지말라고만 하는게 아니라 방화벽까지 꼼꼼하게 막아두고 재원학생들의 태블릿을 등록시켜놔서 딴짓을 하고있는지 계속 주의하면서 실제로 2분정도 딴짓을 하기위해 이 정도면 모르시겠지하고 인터넷을 들어갔는데 바로 감시중이던 선생님이 인터넷 접속을 원격으로 끊으셔서 오히려 딴짓할까 생각도 하지못하고 오히려 딴짓도 못하는데 공부라도 열심히해야겠다라는 마인드로 바로 바뀌었던것같습니다 그만큼 태블릿관리를 말로만하지않으시고 실제계속된감시와 주의로 학생들이 공부에만 집중할 수있게 면학 분위기를 조성시킨게 정말 큰 도움이되었던것같습니다</v>
       </c>
       <c r="H357" t="str">
-        <v>솔직히 이투스모의고사는 사설이라서 그렇게 중요하지않겠지라는 생각으로 이투스모의고사를 생각했었는데 실제 재원생으로 이투스247을 다니면서 이투스모의고사가 제가 수능생활을 유지할수있게하는 큰 도움이 된것같습니다 아무래도 수능생활에서 6월9월모의고사 수능 이렇게 중요한모의고사는 3개라고 볼수있는데 그 사이의 텀이 너무 긴데, 그 사이동안 긴장이 풀어지면서 해아해질수있는 기간을 이투스모의고사가 적절히 그 기간동안 긴장의 끈을 놓지않게 텐션을 유지해주면서 나의 성적대가 지금 어느정도인지 내가 공부하고있는 지금 이 방향이 잘가고있는지 확인할수있게만든 중요한 이정표의 역할이 되었다고 생각합니다 그래서 이투스모의고사를 통해 수능때까지의 긴장의끈을 놓지않고 달리며 수능때좋은성적을 거뒀던것같습니다</v>
+        <v>솔직히 이투스모의고사는 사설이라서 그렇게 중요하지않겠지라는 생각으로 이투스모의고사를 생각했었는데 실제 재원생으로 이투스247을 다니면서 이투스모의고사가 제가 수능생활을 유지할수있게하는 큰 도움이 된것같습니다 아무래도 수능생활에서 6월9월모의고사 수능 이렇게 중요한모의고사는 3개라고 볼수 있는데 그 사이의 텀이 너무 긴데, 그 사이동안 긴장이 풀어지면서 해아해질수 있는 기간을 이투스모의고사가 적절히 그 기간동안 긴장의 끈을 놓지않게 텐션을 유지해주면서 나의 성적대가 지금 어느정도인지 내가 공부하고있는 지금 이 방향이 잘가고있는지 확인할수있게만든 중요한 이정표의 역할이 되었다고 생각합니다 그래서 이투스모의고사를 통해 수능때까지의 긴장의끈을 놓지않고 달리며 수능때좋은성적을 거뒀던것같습니다</v>
       </c>
       <c r="I357" t="str">
-        <v>늦은나이에 공부를 시작하느라 뭐가뭔지도 모르고 수능의기조가 어떤지도 몰랐는데 이튜스선생님들을 만나고 쓴소리와 격려의말을 들으면서 제가부족한점과 지금 고쳐야할점을 회피하지않고 직면하게되면서 지금 이 수험 생활에서 중요하게 뭔지 다시금 생각하게 해주셨고, 격려의 말을 통해 나라는 학생도 수능에서의 성공을 꿈꿀수있는사람으로서 다시 생각하게해쥬셨던것같습니다 많이 모자랐는데도 그저 지나가는 학생이 아닌 정말 끌어서 제가원하는 목표를 이루게 하기위해 힘드실텐데도 본인들의 에너지를 써가면서 저를 설득하고 공부하게끔 다시도와주시는 모습을 수능끝나고 뼈저리게 감사한 마음을 느꼈던것같습니다 이투스247김포점에서 선생님들을 만나고 꿈을 이루게 된것에 너무 감사드리고 저를 지나가는 학생이 아니라 진심으로 대해주셔서 정말 감사합니다 덕분에 꿈을 이룬것같습니다 항상 행복하세요 선생님들 !❤️</v>
+        <v>늦은나이에 공부를 시작하느라 뭐가뭔지도 모르고 수능의기조가 어떤지도 몰랐는데 이튜스선생님들을 만나고 쓴소리와 격려의말을 들으면서 제가부족한점과 지금 고쳐야할점을 회피하지않고 직면하게되면서 지금 이 수험 생활에서 중요하게 뭔지 다시금 생각하게 해주셨고, 격려의 말을 통해 나라는 학생도 수능에서의 성공을 꿈꿀수 있는사람으로서 다시 생각하게해쥬셨던것같습니다 많이 모자랐는데도 그저 지나가는 학생이 아닌 정말 끌어서 제가원하는 목표를 이루게 하기위해 힘드실텐데도 본인들의 에너지를 써가면서 저를 설득하고 공부하게끔 다시도와주시는 모습을 수능끝나고 뼈저리게 감사한 마음을 느꼈던것같습니다 이투스247김포점에서 선생님들을 만나고 꿈을 이루게 된것에 너무 감사드리고 저를 지나가는 학생이 아니라 진심으로 대해주셔서 정말 감사합니다 덕분에 꿈을 이룬것같습니다 항상 행복하세요 선생님들 !❤️</v>
       </c>
       <c r="J357" t="str">
         <v>담임 선생님께서 부족한 과목을 보완할 수 있는 교재를 추천해 주셨는데 잘 맞았어요!</v>
@@ -13381,7 +13381,7 @@
         <v>반수생이라 조금 다른사람에 비해서 늦게 시작한 감이 있었는데 제 위치와 현재 상황에 맞게  각 과목별로 추천하는 커리어나 학습량 그리고 생활 패턴까지 알려주셔서 좀 더 계획을 현실적으로 잡고 공부에만 집중할 수 있었습니다</v>
       </c>
       <c r="F359" t="str">
-        <v>혼자 무작정 진도를 나가는 것이 아니라 일정 주기로 얼만큼 학습했는지 확인을 받을 수 있어서 공부가 잘되었던 주간이나 잘 안되었던 주간을 직접 확인할수 있어 중간에 흔들리더라도 다시 마음을 잡고 공부할 수있는데에 큰 도움이 되었습니다</v>
+        <v>혼자 무작정 진도를 나가는 것이 아니라 일정 주기로 얼만큼 학습했는지 확인을 받을 수 있어서 공부가 잘되었던 주간이나 잘 안되었던 주간을 직접 확인할수 있어 중간에 흔들리더라도 다시 마음을 잡고 공부할 수 있는데에 큰 도움이 되었습니다</v>
       </c>
       <c r="G359" t="str">
         <v>제가 집중을 잘 못해서 초반에는 딴생각 하거나 조는일이 자주 있었는데 그때마다 바로바로 깨워 주셔서 나중에는 오히려 그게 습관이 고쳐져서 후반에는 딴생각이나 조는 일 없이 공부에만 집중할 수 있었던거 같습니다</v>
@@ -13393,7 +13393,7 @@
         <v>반년간 빠짐없이 출석확인과 공부태도들을 점검해주시느라 고생 많으셨고 또 덕분에 공부 진짜 안했던 제가 이런 학교에 와볼수 있다는게 꿈만 같습니다.대학교 다니면서도 이때 시간이 마냥 즐겁기만 한건 아니였지만 하나의 추억으로 오래동안 남을것 같습니다 정말 감사했었습니다</v>
       </c>
       <c r="J359" t="str">
-        <v>반수생이라 마음이 조급했는데 제 상황에 맞춰 커리큘럼을 같이 세워주셔서 걱정없이 공부했어요!</v>
+        <v>반수생이라 마음이 조급했는데 제 상황에 맞춰 커리큘럼을 같이 세워주셔서 걱정 없이 공부했어요!</v>
       </c>
       <c r="K359" t="str">
         <v/>
@@ -13589,13 +13589,13 @@
         <v>N수생</v>
       </c>
       <c r="E364" t="str">
-        <v>처음 입소 당시 공부를 어디서부터 어떻게 해야 하는지 막막했는데 선생님께서 잘 알려주시고 이끌어주셔서 공부 방향을 잡게되고 중간에 흐트러지지 않게 지도해주셔서 성적 향상을 이룰 수 있어서 학습코칭 시스템이 유용했다고 생각합니다</v>
+        <v>처음 입소 당시 공부를 어디서부터 어떻게 해야 하는지 막막했는데 선생님께서 잘 알려주시고 이끌어주셔서 공부 방향을 잡게되고 중간에 흐트러지지 않게 지도해주셔서 성적 향상을 이룰 수 있어서 학습 코칭 시스템이 유용했다고 생각합니다</v>
       </c>
       <c r="F364" t="str">
         <v>6,9모 학원 모의고사를 정기적으로 보고 지원가능대학 라인을 확인함으로써 적당한 긴장감과 도전의식을 가지며 공부할 수 있었다고 생각해서 이 학습 관리 시스템이 유용했다고 생각이 되었습니다</v>
       </c>
       <c r="G364" t="str">
-        <v>휴대폰과 전자기기와의 차단을 통해서 오로지 잡생각 안 하고 학습에만 집중할 수 있어서 단기간에 성적 향상도 이루고 멘탈관리도 되어서 전자기기 사용금지 시스템이 유용하다고 생각을 했습니다</v>
+        <v>휴대폰과 전자기기와의 차단을 통해서 오로지 잡생각 안 하고 학습에만 집중할 수 있어서 단기간에 성적 향상도 이루고 멘탈 관리도 되어서 전자기기 사용금지 시스템이 유용하다고 생각을 했습니다</v>
       </c>
       <c r="H364" t="str">
         <v>학원 내 모의고사를 봄으로써 내가 아는 것과 모르는 것 어중간하게 아는 것을 구분을 할 수 있어서 추후 학습 계획을 세우고 오답정리를 할 때 취약점을 빠르게 보완하고 성적 향상을 이룰 수 있게 해줘서 원내 모의고사가 좋았습니다</v>

</xml_diff>

<commit_message>
Replace typo: 상담울 -> 상담을
</commit_message>
<xml_diff>
--- a/reviews_with_keywords.xlsx
+++ b/reviews_with_keywords.xlsx
@@ -1761,7 +1761,7 @@
         <v>국어 선생님께서 국어를 어떻기 학습해야 할지 자세히 알려주셔서 좋았습니다. 특히 저는 현대소설이 약했는데, 9월 평가원에서 현대소설이 어렵게 출제되어 오답에 부담을 느끼고 있었는데 담임 선생님께서 오답을 하는 가이드라인을 제시해 주셔서 도움을 많이 받았던 기억이 있습니다.</v>
       </c>
       <c r="F38" t="str">
-        <v>저는 2주에 한 번씩 학습 상담울 받았었는데요, 저는 못하는 과목을 기피하는 성향이 있었는데,특히 영어가 그랬던 것 같습니다. 하지만 선생님께서 영어를 꾸준히 학습할 수 있게끔 단어 테스트를 치게 하는 등으로 도움을 꾸준히 주셔서 영어 공부를 놓치 않고 지속적으로 할 수 있었습니다.</v>
+        <v>저는 2주에 한 번씩 학습 상담을 받았었는데요, 저는 못하는 과목을 기피하는 성향이 있었는데,특히 영어가 그랬던 것 같습니다. 하지만 선생님께서 영어를 꾸준히 학습할 수 있게끔 단어 테스트를 치게 하는 등으로 도움을 꾸준히 주셔서 영어 공부를 놓치 않고 지속적으로 할 수 있었습니다.</v>
       </c>
       <c r="G38" t="str">
         <v>저희 학원에서는 순찰을 자주 도셨는데요, 한 자리에 오래 앉아있다 보면 자세도 흐트러지고 집중력도 떨어지고, 졸음도 오기 마련인데 선생님들께서 순찰을 자주 돌아주셔서 어느정도 긴장감을 꾸준히 유지하면서 집중해서 공부를 할 수 있었던 것 같습니다.</v>
@@ -1773,7 +1773,7 @@
         <v>언제나 진심으로 최선을 다해서 학생들을 관리해주셔서 감사합니다. 덕분에 알찬 일년을 보낼 수 있었던 것 같습니다. 만약 주변에서 독학재수학원을 고민하는 지인이 있다면, 저는 고민없이 이투스247을 추천랄 것 같습니다.</v>
       </c>
       <c r="J38" t="str">
-        <v>저는 2주에 한 번씩 학습 상담울 받았었는데요, 상담을 받으면서 기피하는 과목을 가까이 하는 방법에 대해 많은 조언을 해주셨어요.</v>
+        <v>저는 2주에 한 번씩 학습 상담을 받았었는데요, 상담을 받으면서 기피하는 과목을 가까이 하는 방법에 대해 많은 조언을 해주셨어요.</v>
       </c>
       <c r="K38" t="str">
         <v>학습 관리</v>

</xml_diff>

<commit_message>
Apply fourth batch of typo corrections
</commit_message>
<xml_diff>
--- a/reviews_with_keywords.xlsx
+++ b/reviews_with_keywords.xlsx
@@ -477,7 +477,7 @@
 지난 한 해 동안 정말 감사하였습니다. 다른 학원생들도 좋은 결과가 있으면 좋겠습니다.</v>
       </c>
       <c r="J2" t="str">
-        <v>선생님들께서 좋은 면학 분위기가 조성해주셔서 자연스럽게 졸지 않으려고 노력하게 되었어요.</v>
+        <v>선생님들께서 좋은 면학 분위기를 조성해주셔서 자연스럽게 졸지 않으려고 노력하게 되었어요.</v>
       </c>
       <c r="K2" t="str">
         <v>면학 분위기</v>
@@ -571,7 +571,7 @@
         <v>제가 일반전형이 아니라 기회균등 전형 농어촌 학생이여서 관련 자료가 부족 했음에도 불구하고 저의 전형에 맞추어서 저의 성적에 맞추어서 세심하게 입시 상담을 진행해 주셔서 진심으로 감사했습니다.</v>
       </c>
       <c r="F5" t="str">
-        <v>제가 현역일때에 공부할 때 태어나서 한 번도 플레너를 써 본 적이 없었는데 하남 이투스 247  재수 학원을 다니면서 플레너 쓰는 법을 배우고 익히면서 올바린 공부의 방향과 계획이 잡힐 수 있었던 것 같습니다</v>
+        <v>제가 현역일때에 공부할 때 태어나서 한 번도 플래너를 써 본 적이 없었는데 하남 이투스 247  재수 학원을 다니면서 플래너 쓰는 법을 배우고 익히면서 올바린 공부의 방향과 계획이 잡힐 수 있었던 것 같습니다</v>
       </c>
       <c r="G5" t="str">
         <v>제가 공부를 못하서 현역때 대학교 3광탈을 하고 재수를 할 수 밖에 없었던 이유가 항상 핸드폰이나 유튜브로 딴 짓을 해서 인데요 와이파이 방화벽으로 인해서 인강 아니면 아무데도 들어 갈 수 없었기 때문에 온전히 공부에 집중할 수 있었던 것 같습니다.</v>
@@ -580,13 +580,13 @@
         <v>현역때에는 학교에서 보는 교육청과 전국연합 평가원 모의고사가 전부였는데 이투스 전용 모의사를 통해서 새로운 유형의 문제들을 접해보면서 새로운 문제에 대한 두려움이 사라지고 모의고사에 적응이 되면서 수능날에 긴장감이 줄어들었던 것 같습니다.</v>
       </c>
       <c r="I5" t="str">
-        <v>원장 선생님과 출결 관리를 해주셨던 선생님 그리고 플레너 관리를 해주셨던 선생님 정말 감사합니다!!!!!항상 건강하실 바라겠습니다!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!</v>
+        <v>원장 선생님과 출결 관리를 해주셨던 선생님 그리고 플래너 관리를 해주셨던 선생님 정말 감사합니다!!!!!항상 건강하실 바라겠습니다!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!</v>
       </c>
       <c r="J5" t="str">
-        <v>원장 선생님과 출결 관리를 해주셨던 선생님 그리고 플레너 관리를 해주셨던 선생님 정말 감사했어요.</v>
+        <v>원장 선생님과 출결 관리를 해주셨던 선생님 그리고 플래너 관리를 해주셨던 선생님 정말 감사했어요.</v>
       </c>
       <c r="K5" t="str">
-        <v/>
+        <v>플래너 관리</v>
       </c>
     </row>
     <row r="6">
@@ -814,7 +814,7 @@
       </c>
       <c r="E12" t="str" xml:space="preserve">
         <v xml:space="preserve">이것 저것 다 해야 할 것 같은 조급함에 이러지도 저러지도 못하고 있을때 담임 선생님과의 학습 상담을 통해서 저와 맞는 학습 계획을 세우고 저만의 템포로 공부할 수 있어서 좋았습니다_x000d_
-또한, 저는 맞는 인강쌤을 찾기 힘들어 많이 왔다갔다 거리는 인강 유목민이었습니다. 인강이 없으면 안된다고 생각했는데 학습 상담을 통해 인강이 맞지 않는 과목의 경우여도 독학으로 좋은 성적을 받을 수 있음을 알게되었습니다. 머리가 복잡한 수험생을 옳은 길로 잘 이끌어주셨습니다</v>
+또한, 저는 맞는 인강쌤을 찾기 힘들어 많이 왔다갔다 거리는 인강 유목민이었습니다. 인강이 없으면 안 된다고 생각했는데 학습 상담을 통해 인강이 맞지 않는 과목의 경우여도 독학으로 좋은 성적을 받을 수 있음을 알게되었습니다. 머리가 복잡한 수험생을 옳은 길로 잘 이끌어주셨습니다</v>
       </c>
       <c r="F12" t="str">
         <v>앞서 언급했듯 다양한 방면으로 공부법을 제시해주시고, 결정하게 해주셔서 좋았습니다. 사람마다 맞는 공부법이 다르기에 그것을 찾아 정착하는데에는 꽤 오랜 시간이 걸린다고 생각합니다. 이투스 담임 선생님과의 꾸준한 소통과 학습 관리 시스템을 통해 시간낭비를 줄일 수 있었던 것 같습니다</v>
@@ -829,7 +829,7 @@
         <v>여러모로 학생만큼 고생하셨을텐데 길다면 긴, 짧다면 짧은 기간동안 감사했습니다! 선생님들의 격려와 응원, 도움이 없었다면 힘든 수험 생활 진작에 무너졌을 것 같아요,, 제 수험 생활에 함께해주셔서 감사합니다</v>
       </c>
       <c r="J12" t="str">
-        <v>수업이 없으면 안된다고 생각했는데 학습 상담을 통해 저에게 맞는 공부법을 알려주셔서 좋은 성적을 받을 수 있었어요.</v>
+        <v>수업이 없으면 안 된다고 생각했는데 학습 상담을 통해 저에게 맞는 공부법을 알려주셔서 좋은 성적을 받을 수 있었어요.</v>
       </c>
       <c r="K12" t="str">
         <v>학습 관리</v>
@@ -969,7 +969,7 @@
         <v>수고 많으셨습니다. 그리고 제 까다롭고 예민하고 어떨 때는 또 유별난 성격을 잘 아실 것입니다. 제가 어떤 면에서는 다소간 피곤하다고 느끼셨을지도 모르겠으나, 그만큼 도움 많이 받아갔습니다. 감사합니다.</v>
       </c>
       <c r="J16" t="str">
-        <v>담임 선생님과 함께 공부 계획을 작성하고, 그에 따른 성취 여부를 하나 한 기록하다보니 좋은 성적을 얻을 수 있었어요.</v>
+        <v>담임 선생님과 함께 공부 계획을 작성하고, 그에 따른 성취 여부를 하나하나 기록하다 보니 좋은 성적을 얻을 수 있었어요.</v>
       </c>
       <c r="K16" t="str">
         <v/>
@@ -1132,7 +1132,7 @@
         <v>고등학교 때 생각없이 공부하다가 마음에 들지 않는 대학에 진학하였고, 결국 반수를 결심하게 되었다. 한 학기동안은 홀로 계획을 짜 보고 이것저것 다양한 공부법을 시도해 봤지만 이게 효율적인 방법이 맞는지 알 수 없어 답답했다. 그러다가 이투스에 와서 본격적인 반수를 시작하고,담임 선생님과의 상담을 통해 현재 내가 해야하는 부분, 강점과 부족한 부분, 세세한 모의고사 피드백 등을 알 수 있어 만족스러웠다.</v>
       </c>
       <c r="F21" t="str">
-        <v>독학재수는 쉽지 않다. 이투스 등록 전까진 아무리 플래너를 그럴듯하게 써놔도 막상 달성률은 처참했다. 누군가 옆에서 잡아주고 감시해주는 사람이 없으니, 자기합리화를 계속 하며 미루고 미루다 결국 할 일이 엄청 불어났다. 그러나 학원에 오게 되면, 선생님들이 플래너를 매주 검사하신다. 현재 내가 모든 과목을 균형있게 고루 공부하고 있는지, 계획이 너무 무리하진 않은지 플래너를 세세히 보시고 하나하나 피드백해 주신다. 덕분에 학원에 온 지 한 달만에 미루는 습관을 교정하게 될 수 있었다.</v>
+        <v>독학재수는 쉽지 않다. 이투스 등록 전까진 아무리 플래너를 그럴듯하게 써놔도 막상 달성률은 처참했다. 누군가 옆에서 잡아주고 감시해주는 사람이 없으니, 자기합리화를 계속 하며 미루고 미루다 결국 할 일이 엄청 불어났다. 그러나 학원에 오게 되면, 선생님들이 플래너를 매주 검사하신다. 현재 내가 모든 과목을 균형 있게 고루 공부하고 있는지, 계획이 너무 무리하진 않은지 플래너를 세세히 보시고 하나하나 피드백해 주신다. 덕분에 학원에 온 지 한 달만에 미루는 습관을 교정하게 될 수 있었다.</v>
       </c>
       <c r="G21" t="str" xml:space="preserve">
         <v xml:space="preserve">나는 잠에 정말 약하다. 고3 때 모의고사를 볼 때도 몽롱한 정신으로 풀었고, 아침잠이 너무 많은 탓에 결국 현역 수능 1교시 시작 직전까지 하품을 쩍쩍 하다 결국 처참한 국어 성적을 받았다. 학원에 온 이후로는 선생님들께서 졸음 관리를 해 주셔서 좋았다. 항상 공부를 할 땐 나도 모르는 사이 꾸벅꾸벅 졸곤 했었는데, 그럴 때 마다 감독 선생님들께서 안마봉으로 깨워주셨다._x000d_
@@ -1164,7 +1164,7 @@
 이투스 대구달서점 화이팅~~</v>
       </c>
       <c r="J21" t="str">
-        <v>내가 모든 과목을 균형있게 고루 공부하고 있는지, 너무 무리하진 않은지 플래너를 세세히 보시고 하나하나 피드백해 주셨어요.</v>
+        <v>내가 모든 과목을 균형 있게 고루 공부하고 있는지, 너무 무리하진 않은지 플래너를 세세히 보시고 하나하나 피드백해 주셨어요.</v>
       </c>
       <c r="K21" t="str">
         <v/>
@@ -2043,7 +2043,7 @@
   저 같은 경우는 아쉽게도 끝까지 완수하지 못하였지만 다른 학생들 같은 경우 선생님들 덕분에 힘든 수험 생활을 넘길수도 있는 분도 있을겁니다.</v>
       </c>
       <c r="F46" t="str">
-        <v>수험생의 상태를 성적뿐 아니라 그 이외의 것 들도 수험 생활에 집중할 수 있도록 상담해주십니다. 건강이 좋지 않아도 한 번은 이투스247학원에서 수험 생활을 노력해볼수 있을 거라고 생각합니다.</v>
+        <v>수험생의 상태를 성적뿐 아니라 그 이외의 것들도 수험 생활에 집중할 수 있도록 상담해주십니다. 건강이 좋지 않아도 한 번은 이투스247학원에서 수험 생활을 노력해볼수 있을 거라고 생각합니다.</v>
       </c>
       <c r="G46" t="str">
         <v>솔직히 방금 네가지 선택지 다 별로였는데 와이파이 방화벽은 비교적 도움이 돼었지만, 핸드폰 반납같은 경우 혼자서 수험 생활을 준비하는 학생의 경우 꽤 불편합니다.  학원 와서도 핸드폰으로 딴짓 하면 그것은 개인의 의지 문제이고 선생님들이 관리도 하시니 이 부분은 추후에 더 효율적으로 관리되었으면 합니다.</v>
@@ -2055,7 +2055,7 @@
         <v>몸도 마음도 힘들었지만 재원하는동안 사정봐주시고 신경 써주셔서 너무 감사합니다. 저 같은 수험생은 보지않고 싶으실것 같습니다. 그래도 신경써주셔서 그나마 덜 힘들었습니다. 학생 개개인 별로 사정을 파악하고 조치를 취하시는게 어려울것 같습니다만 그렇게 해주셔서 감사합니다</v>
       </c>
       <c r="J46" t="str">
-        <v>성적뿐만 아니라 그 이외의 것 들도 수험 생활에 집중할 수 있도록 상담해주셨어요.</v>
+        <v>성적뿐만 아니라 그 이외의 것들도 수험 생활에 집중할 수 있도록 상담해주셨어요.</v>
       </c>
       <c r="K46" t="str">
         <v/>
@@ -2251,7 +2251,7 @@
         <v>반수생</v>
       </c>
       <c r="E52" t="str" xml:space="preserve">
-        <v xml:space="preserve">국어가 맨날 5~6등급이었지만 국어 멘토링덕분에 2,3,4등급은 안정적으로 받을 수 있는 수준으로 발전하였다_x000d_
+        <v xml:space="preserve">국어가 맨날 5~6등급이었지만 국어 멘토링 덕분에 2,3,4등급은 안정적으로 받을 수 있는 수준으로 발전하였다_x000d_
 또한 탐구를 담임 선생님께서 잘 체크해주셔서 빠뜨리지 않고 잘 공부할 수있었다</v>
       </c>
       <c r="F52" t="str" xml:space="preserve">
@@ -2268,7 +2268,7 @@
         <v>모든 선생님들 지도해주셔서 감사했습니다 특히 태민선생님 상담 잘해주시고 피드백 잘해주셔서 감사했습니다 찾아뵙고싶었는데 못찾아뵈었네요 죄송합니다 다음에 기회가 된다면 꼭 찾아뵙고싶습니다</v>
       </c>
       <c r="J52" t="str">
-        <v>6등급이었지만 국어 멘토링덕분에 2,3,4등급은 안정적으로 받을 수 있는 수준으로 발전하였어요.</v>
+        <v>6등급이었지만 국어 멘토링 덕분에 2,3,4등급은 안정적으로 받을 수 있는 수준으로 발전하였어요.</v>
       </c>
       <c r="K52" t="str">
         <v/>
@@ -2872,10 +2872,10 @@
         <v>N수생</v>
       </c>
       <c r="E69" t="str">
-        <v>입시에 대해서 많이 무지한 편이었는데 도움을 많이 주셔서 입시 시스템이 어떻게 돌아가는지 정확하게 파악하는 걸 수월하게 할 수 있었고, 심리적으로도 대학 입시와 수능 공부 방향을 어떻게 해야 할 지도 알려주셔서 많이 도움되었던 것 같았습니다.</v>
+        <v>입시에 대해서 많이 무지한 편이었는데 도움을 많이 주셔서 입시 시스템이 어떻게 돌아가는지 정확하게 파악하는 걸 수월하게 할 수 있었고, 심리적으로도 대학 입시와 수능 공부 방향을 어떻게 해야 할지도 알려주셔서 많이 도움되었던 것 같았습니다.</v>
       </c>
       <c r="F69" t="str">
-        <v>자기가 무슨 인강을 들어야할 지 처음엔 감이 안잡힐 때가 많은데 제 성적과 학습 수준에 따라서 어떤 교재와 인강을 들어야할 지 추천해 주셔서 좋았습니다. 방향을 잡는데 많이 도움되었다고 생각해요</v>
+        <v>자기가 무슨 인강을 들어야할지 처음엔 감이 안잡힐 때가 많은데 제 성적과 학습 수준에 따라서 어떤 교재와 인강을 들어야할지 추천해 주셔서 좋았습니다. 방향을 잡는데 많이 도움되었다고 생각해요</v>
       </c>
       <c r="G69" t="str">
         <v>핸드폰이 진짜 수능 준비에 가장 방해가 많이 되는 물품이라고 생각하는데, 이렇게 확실하게 강제성을 주니까 공부에만 집중하게 될 수 있는 환경이 만들어져서 정말 좋았습니다. 졸음도 가끔 들어오셔서 돌아다니시면서 깨워주시는데 그것 덕에 졸음도 깨고 공부 집중에 도움이 되었습니다.</v>
@@ -3351,7 +3351,7 @@
         <v>N수생</v>
       </c>
       <c r="E82" t="str">
-        <v>매달 치르는 모의고사 성적표로 개인 상담을 진행했을때 과목별로 현재 부족한 점과 보완할 점을 자세히 알려주셨습니다. 뿐만아니라 모르는 문제가 생기거나 고민이 있을때마다 언제든 상담실로 내려가서 국/영/수 선생님께 질문할 수 있었던 점이 매우 좋았습니다.</v>
+        <v>매달 치르는 모의고사 성적표로 개인 상담을 진행했을 때 과목별로 현재 부족한 점과 보완할 점을 자세히 알려주셨습니다. 뿐만아니라 모르는 문제가 생기거나 고민이 있을때마다 언제든 상담실로 내려가서 국/영/수 선생님께 질문할 수 있었던 점이 매우 좋았습니다.</v>
       </c>
       <c r="F82" t="str">
         <v>저는 수학선생님께 가장 많이 질문했지만 국어,영어,지구과학 선생님도 학원에 계셨기에 언제든 1:1로 질의응답이 가능했습니다. 혼자 공부하다가 모르는 문제가 생기면 편하게 질문할 수 있어서 좋았고 학원을 다니지않고 혼자 개인적으로 공부하기보다 선생님께 질문하면서 배워나가는 과정이 중요하다고 생각하기때문에 유용했습니다.</v>
@@ -3366,7 +3366,7 @@
         <v>항상 제 터무니없는 질문들도 너그럽게 받아주셔서 너무 감사했습니다. 특히 수학선생님의 수학 특강이 정말 많은 도움이 되었고 실제로 수능장에서도 써먹은 것이 정말 많았습니다!! 덕분에 행복한 대학생활 하고있는것 같아요 ㅎ감사합니다</v>
       </c>
       <c r="J82" t="str">
-        <v>매달 치르는 모의고사 성적표로 개인 상담을 진행했을때 과목별로 현재 부족한 점과 보완할 점을 자세히 알려주셨어요.</v>
+        <v>매달 치르는 모의고사 성적표로 개인 상담을 진행했을 때 과목별로 현재 부족한 점과 보완할 점을 자세히 알려주셨어요.</v>
       </c>
       <c r="K82" t="str">
         <v>모의고사</v>
@@ -4107,7 +4107,7 @@
         <v>N수생</v>
       </c>
       <c r="E103" t="str">
-        <v>자기 주도 학습을 위해 자습시간을 어떻게 더 효율적으로 활용할 지 고민이 많았는데 담당 담임 선생님과의 상담을 통해 과목별 시간 배분을 어떻게 할지와 취약 과목에 대한 공부 방법 등 전체적인 공부 습관을 형성하는 것에 도움을 많이 받았습니다.</v>
+        <v>자기 주도 학습을 위해 자습시간을 어떻게 더 효율적으로 활용할지 고민이 많았는데 담당 담임 선생님과의 상담을 통해 과목별 시간 배분을 어떻게 할지와 취약 과목에 대한 공부 방법 등 전체적인 공부 습관을 형성하는 것에 도움을 많이 받았습니다.</v>
       </c>
       <c r="F103" t="str">
         <v>학습 계획 설정과 플래너 관리에서 공부 습관이 형성되어 있지 않을 때에 하루에 어떻게 공부를 하고 어느정도의 양을 소화할 수 있는지 확인하고 앞으로의 학습을 위해 효율적인 계획을 세울 수 있도록 스스로 훈련할 수 있었습니다.</v>
@@ -4212,7 +4212,7 @@
         <v>N수생</v>
       </c>
       <c r="E106" t="str" xml:space="preserve">
-        <v xml:space="preserve">담임쌤이랑 매주 한 번씩 공부 방법,피드백, 고쳐야 할 점 등등 학습에 도움되는 이야기를 할 수 있어서 좋았고_x000d_
+        <v xml:space="preserve">담임쌤이랑 매주 한 번씩 공부 방법, 피드백, 고쳐야 할 점 등등 학습에 도움되는 이야기를 할 수 있어서 좋았고_x000d_
 큐엔에이도 과목마다 다양한 선생님들이랑 당일날에 바로바로 대면으로 해결할수있어서 좋있습니다</v>
       </c>
       <c r="F106" t="str" xml:space="preserve">
@@ -4233,7 +4233,7 @@
 모두 감사했고 수고하셨습니다</v>
       </c>
       <c r="J106" t="str">
-        <v>담임 선생님과 매주 공부 방법,피드백, 고쳐야 할 점 등 학습에 도움되는 이야기를 할 수 있어서 좋았어요.</v>
+        <v>담임 선생님과 매주 공부 방법, 피드백, 고쳐야 할 점 등 학습에 도움되는 이야기를 할 수 있어서 좋았어요.</v>
       </c>
       <c r="K106" t="str">
         <v/>
@@ -4822,7 +4822,7 @@
         <v>N수생</v>
       </c>
       <c r="E123" t="str" xml:space="preserve">
-        <v xml:space="preserve">6월 모의고사 성적과 9월 모의고사 성적을 바탕으로 선생님께서 수시원서상담을 친절하게 진행해주셔서 도움이 많이 됐어 제 성적대에 맞는 대학을 추천해 주셔서 감사했습니다 과도한 상향원서 작성이_x000d_
+        <v xml:space="preserve">6월 모의고사 성적과 9월 모의고사 성적을 바탕으로 선생님께서 수시 원서상담을 친절하게 진행해주셔서 도움이 많이 됐어 제 성적대에 맞는 대학을 추천해 주셔서 감사했습니다 과도한 상향원서 작성이_x000d_
 아닌 현실적으로 가능한 원서를 작성하게끔 해주셔서 안정적으로 입시를 마무리했습니다</v>
       </c>
       <c r="F123" t="str" xml:space="preserve">
@@ -4859,7 +4859,7 @@
         <v>반수생</v>
       </c>
       <c r="E124" t="str">
-        <v>모의고사 점수를 비교 분석하여 이전보다 무엇이 부족했고, 어떤 점이 늘었는지를 보다 객관적으로 알 수 있었다. 또한 평소에도 어떻게 공부할 지에 대해 상담이 가능한 점이 도움이 되었다.</v>
+        <v>모의고사 점수를 비교 분석하여 이전보다 무엇이 부족했고, 어떤 점이 늘었는지를 보다 객관적으로 알 수 있었다. 또한 평소에도 어떻게 공부할지에 대해 상담이 가능한 점이 도움이 되었다.</v>
       </c>
       <c r="F124" t="str">
         <v>모르는 문제나 헷갈리는 개념에 대해서 1대1 질의 응답이 가능한 점이 마음에 들었다. 자세히 물어봐도 친절하게 답해주시고 더불어 학습 팁도 알려주셔서 공부하는 방향을 잡기에 도움이 되었다.</v>
@@ -4914,7 +4914,7 @@
 학습 선생님과 카윤터에 계신 선생님들 모두 정말 감사했습니다 항상 친절하게 대해주시고 잘 잡아주셔서 너무 좋았습니다</v>
       </c>
       <c r="J125" t="str">
-        <v>힘들 때도 많았지만 잘 다잡아주셔서 수험 생활 잘 마무리 한 것 같아요.</v>
+        <v>힘들 때도 많았지만 잘 다잡아주셔서 수험 생활을 잘 마무리한 것 같아요.</v>
       </c>
       <c r="K125" t="str">
         <v/>
@@ -5705,7 +5705,7 @@
         <v>항상 따뜻한 마음으로 지도해주시고, 공부에 집중할 수 있는 좋은 환경을 만들어주셔서 진심으로 감사드립니다. 선생님들의 세심한 배려와 응원 덕분에 더욱 성실하게 노력할 수 있었습니다.</v>
       </c>
       <c r="J147" t="str">
-        <v>국어가 가장 취약 과목이였는데, 담임 선생님과의 상담을 통해 공부 방법과 글 읽는 방향을 바로잡아 성적 향상에 큰 도움이 되었어요.</v>
+        <v>국어가 가장 취약 과목이었는데, 담임 선생님과의 상담을 통해 공부 방법과 글 읽는 방향을 바로잡아 성적 향상에 큰 도움이 되었어요.</v>
       </c>
       <c r="K147" t="str">
         <v/>
@@ -5734,7 +5734,7 @@
         <v>출석 시 전자기기를 제출 함으로써 공부에 가장 방해되는 요소인 핸드폰을 제거해서 긴 시간동안 학원에 머무르는데도 불구하고 집중력을 유지할 수 있게 된거 같습니다 또 휴식시간에도 핸드폰을 주지 않으셔서 온전하게 휴식을 하게 되어서 쉬는 시간 후 공부를 할 때 큰 도움을 받았던거 같습니다</v>
       </c>
       <c r="H148" t="str">
-        <v>제가 영어가 가장 취약한 과목이였는데 고3에는 매일 단어를 외우지 않았습니다 하지만 이투스 247학원에 오면서 매일 의무적으로 단어를 40개씩 외우게 해주셔서 영어 실력의 기본기가 갖춰지게 된거 같습니다 또 일일테스트 뿐만 아니라 토요일에 실행하는 단어 총정리 테스트를 통해 복습을 꾸준하게 진행할 수 있어서 좋았습니다</v>
+        <v>제가 영어가 가장 취약한 과목이었는데 고3에는 매일 단어를 외우지 않았습니다 하지만 이투스 247학원에 오면서 매일 의무적으로 단어를 40개씩 외우게 해주셔서 영어 실력의 기본기가 갖춰지게 된거 같습니다 또 일일테스트 뿐만 아니라 토요일에 실행하는 단어 총정리 테스트를 통해 복습을 꾸준하게 진행할 수 있어서 좋았습니다</v>
       </c>
       <c r="I148" t="str" xml:space="preserve">
         <v xml:space="preserve">재수 생활 함께 해주셔서 감사합니다_x000d_
@@ -5922,7 +5922,7 @@
         <v>윈터스쿨때 다니며 저의 공부 습관을 잡을 수 있었던 것 같습니다. 주기적인 학습 관리와 조언을 해주시고, 학습에 방해가 되지 않도록 휴대폰 관리, 학습 관리에 있어서 도와주신 선생님들께 감사합니다.</v>
       </c>
       <c r="J153" t="str">
-        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는것과 공부하는 것을 관리, 감독해주시는 게 도움이 많이 됐어요.</v>
+        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는 것과 공부하는 것을 관리, 감독해주시는 게 도움이 많이 됐어요.</v>
       </c>
       <c r="K153" t="str">
         <v/>
@@ -5960,7 +5960,7 @@
         <v>감사합니다!!올해도 열심히 할게요 덕분에 공부하는 방법을 깨달아서 스스로 더 열심히 해서 더 좋은 대학에 진학할수 있도록 노력하겠습니다 앞으로도 좋은 학원으로 남아주셨으면 좋겠습니다</v>
       </c>
       <c r="J154" t="str">
-        <v>면학 분위기를 위해 지켜야 할 규칙이 명확하고,담임 선생님이 면학 분위기 조성을 위해 충고를 아끼지 않으셔서 더욱 분위기가 잘 잡힌것 같아요.</v>
+        <v>면학 분위기를 위해 지켜야 할 규칙이 명확하고,담임 선생님이 면학 분위기 조성을 위해 충고를 아끼지 않으셔서 더욱 분위기가 잘 잡힌 것 같아요.</v>
       </c>
       <c r="K154" t="str">
         <v>면학 분위기</v>
@@ -6126,7 +6126,7 @@
         <v>원래 플래너를 적지 않았었는데, 이투스를 다니면서 학습 플래너나 학습 일기를 통해서 본인 스스로 오늘 했던 공부나 보완할 점들을 생각할 수 있었고, 어떤 과목을 앞으로 얼마큼 공부하고, 또 어떻게 공부할지에 관해서 윤곽을 쉽게 잡을 수 있었고, 전반적인 공부의 방향을 정할 수 있어서 좋았습니다.</v>
       </c>
       <c r="G159" t="str">
-        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는것과 공부하는 것을 관리, 감독해주시는 게 도움이 많이 됐습니다. 또한 혼자 독서실을 가면 핸드폰을 보거나 공부 이외의 딴짓을 자주 하는데 핸드폰을 제출하고 독서실에 들어가고, 지속적으로 감시를 해주시는것이 무척 좋았습니다.</v>
+        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는 것과 공부하는 것을 관리, 감독해주시는 게 도움이 많이 됐습니다. 또한 혼자 독서실을 가면 핸드폰을 보거나 공부 이외의 딴짓을 자주 하는데 핸드폰을 제출하고 독서실에 들어가고, 지속적으로 감시를 해주시는것이 무척 좋았습니다.</v>
       </c>
       <c r="H159" t="str">
         <v>결국 수능에서의 실전 감각이 매우 중요하다고 생각하는데 저는 고3현역이여서 학원에서 다 같이 시험을 보지는 못하였지만 담당 선생님이 모의고사를 챙겨주셔서 주말에 모의고사를 풀 수 있었고, 이러한 실전 경험들이 쌓여서 매우 큰 성적 향상을 이뤄낼 수 있었다고 생각합니다. 또한 문제의 퀄리티 역시 매우 뛰어나고, EBS 반영까지 잘 되어 있어서 실전 연습을 하기에 적합하다고 생각합니다.</v>
@@ -6196,7 +6196,7 @@
         <v>제 MBTI가 P성향인지라 계획 세우기를 엄청 어려워 했었는데, 선생님이 플래너 작성과 계획 세우기를 코칭해주시고,적극적으로 조언을 해주셔서 체계적인 학습을 수행하는데 아주 큰 도움이 되었습니다.</v>
       </c>
       <c r="G161" t="str">
-        <v>공부를 하다보면 나도 모르게 졸게 되는 경우도 많은데, 감독 선생님이 와서 깨워주시면 졸음도 가시고,리프레쉬를 할 수 있게 되어서 좋았어요. 또한 면학 분위기를 위해 지켜야 할 규칙이 명확하고,담임 선생님이 면학 분위기 조성을 위해 충고를 아끼지 않으셔서 더욱 분위기가 잘 잡힌것 같아요.</v>
+        <v>공부를 하다보면 나도 모르게 졸게 되는 경우도 많은데, 감독 선생님이 와서 깨워주시면 졸음도 가시고,리프레쉬를 할 수 있게 되어서 좋았어요. 또한 면학 분위기를 위해 지켜야 할 규칙이 명확하고,담임 선생님이 면학 분위기 조성을 위해 충고를 아끼지 않으셔서 더욱 분위기가 잘 잡힌 것 같아요.</v>
       </c>
       <c r="H161" t="str">
         <v>매일매일 반복적으로 진행되는 영어 단어 테스트 덕분에 꾸준히 일정량 이상의 영어 단어 암기가 가능하였고, 그동안 외운 영어 단어를 복기하는데에도 효과적이라 영어 모의고사 성적을 유지하는데 큰 도움이 된 것 같아 마음에 들었어요.</v>
@@ -6277,7 +6277,7 @@
         <v>학생 한 명 한 명을 신경 써 주시며 도와주시고 응원해 주신 덕분에 끝까지 포기하지 않고 노력할 수 있었습니다. 올바른 공부 방법과 태도를 배울 수 있어 더욱 의미 있는 시간이었던 것 같습니다. 앞으로도 선생님들께 배운 것을 바탕으로 더 성장할 수 있도록 노력하겠습니다. 진심으로 감사드립니다!</v>
       </c>
       <c r="J163" t="str">
-        <v>고3 때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던 건 선생님들의 탁월한 입시 전략과 상담, 생활 환경 조성 덕분이었어요.</v>
+        <v>고3 때까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던 건 선생님들의 탁월한 입시 전략과 상담, 생활 환경 조성 덕분이었어요.</v>
       </c>
       <c r="K163" t="str">
         <v/>
@@ -6585,7 +6585,7 @@
         <v>원장님이랑 실장님이랑 경쌤! 25년 한 해 동안 정말 신세 많이 졌습니다 대학가서 재밋게 지내고 있어요! 곧 인사 차 방문드릴게요 ㅎㅎ 제 학습 방향 설정해주셔서 감사했고 멘탈도 케어해주셔서 정말 감사했습니다!</v>
       </c>
       <c r="J171" t="str">
-        <v>확실이 휴대폰이 없으니 공부에 집중이 더 잘 되고 성취감도 있어서 생활 관리에 유용했어요.</v>
+        <v>확실히 휴대폰이 없으니 공부에 집중이 더 잘 되고 성취감도 있어서 생활 관리에 유용했어요.</v>
       </c>
       <c r="K171" t="str">
         <v>생활 관리</v>
@@ -6620,7 +6620,7 @@
         <v>약 1년 동안 많은 학생들을 케어하기 힘드셨을텐데 그럼에도 항상 질문에 대해 친절하게 답변해주시고 성적이 잘 나오지 않아 답답해서 힘들어 할 때도 격려해주셔서 끝까지 포기하지 않고 꾸준히 1년을 달릴 수 있었던 것 같아서 감사합니다.</v>
       </c>
       <c r="J172" t="str">
-        <v>수시원서를 쓰기전에 한 명씩 친절하게 상담을 해주셨어요.</v>
+        <v>수시 원서를 쓰기 전에 한 명씩 친절하게 상담을 해주셨어요.</v>
       </c>
       <c r="K172" t="str">
         <v/>
@@ -7265,7 +7265,7 @@
 고마운 존재였습니다. 결코 쉽지 않은 난이도로 항상 저를 당황시켰는데 오히려 시험준비에 더 열심히 임할 수 있었던 것 같습니다.</v>
       </c>
       <c r="I190" t="str">
-        <v>작년, 걱정과 불안이 가득한 입시상담을 받았던게 새록새록 떠오르는데 저는 지금 그 때의 상담에서 선생님께서 말씀하신 대학의 학과에 입학했습니다! 고3 때 까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던 건 이투스 강서지점 선생님들의 탁월한 입시 전략과 상담, 생활 환경 조성 덕분이었습니다. 저의 처음이자 마지막 재수를 성공적으로 마치게 해주신 이투스 강서지점 선생님들께 감사를 표합니다!</v>
+        <v>작년, 걱정과 불안이 가득한 입시상담을 받았던게 새록새록 떠오르는데 저는 지금 그 때의 상담에서 선생님께서 말씀하신 대학의 학과에 입학했습니다! 고3 때까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던 건 이투스 강서지점 선생님들의 탁월한 입시 전략과 상담, 생활 환경 조성 덕분이었습니다. 저의 처음이자 마지막 재수를 성공적으로 마치게 해주신 이투스 강서지점 선생님들께 감사를 표합니다!</v>
       </c>
       <c r="J190" t="str">
         <v>생활 상담을 포함한 코칭 시스템은 공부 외적인 부분까지 함께 관리해 준다는 점에서 의미가 있었어요.</v>
@@ -8206,7 +8206,7 @@
         <v>저는 인강을 들으면서도 내가 내 수준에 맞게 잘 듣고 있는 게 맞을까?라는 의문이 계속 들었습니다. 특히 국어와 수학이 약해서 고민도 많고 걱정도 많았었는데, 선생님께서 조언을 잘 해주셔서 제 커리에 맞게 차근차근 해 나갈 수 있었습니다.</v>
       </c>
       <c r="G216" t="str">
-        <v>저는 휴대폰이 근처에 있으면 공부 효율이 현저히 떨어지는 스타일이라 일부러 휴대폰을 걷는 곳으로 학원을 선택했었습니다. 확실이 휴대폰이 없으니 공부에 집중이 더 잘 되고 성취감도 있어서 생활 관리에 유용했습니다.</v>
+        <v>저는 휴대폰이 근처에 있으면 공부 효율이 현저히 떨어지는 스타일이라 일부러 휴대폰을 걷는 곳으로 학원을 선택했었습니다. 확실히 휴대폰이 없으니 공부에 집중이 더 잘 되고 성취감도 있어서 생활 관리에 유용했습니다.</v>
       </c>
       <c r="H216" t="str">
         <v>혼자 공부하다 보면 영어 단어 암기의 중요성을 간과하게 되는 느낌이 있습니다. 저도 독학을 시작한 후로 영어 단어 암기에 소홀했는데 이투스에서 매일 단어 시험지를 나누어 주니 억지로라도 했던 것이 도움이 되었습니다.</v>
@@ -8376,7 +8376,7 @@
         <v>반수생</v>
       </c>
       <c r="E221" t="str">
-        <v>수시원서를 쓰기전에 한 명씩 친절하게 상담을 해주십니다. 각자의 모의고사와 실모, 내신 성적을 기반으로 같은 성적이여도 최선의 선택이 될 수 있게 같이 고민해주십니다. 입시전형요강에 댜해 빠삭하게 알고 있고 관련 설명도 자주 진행합니다.</v>
+        <v>수시 원서를 쓰기 전에 한 명씩 친절하게 상담을 해주십니다. 각자의 모의고사와 실모, 내신 성적을 기반으로 같은 성적이여도 최선의 선택이 될 수 있게 같이 고민해주십니다. 입시전형요강에 댜해 빠삭하게 알고 있고 관련 설명도 자주 진행합니다.</v>
       </c>
       <c r="F221" t="str">
         <v>일요일마다 모의고사를 보고 며칠 뒤에 성적표를 나눠준다. 더프처럼 다 같이 보는 모의고사가 아니더라도 학원내에서 평균과 컷을 산출하여 알려주는 점이 매 모의고사에 진심으로 임하게 되는 것 같다.</v>
@@ -9070,7 +9070,7 @@
         <v>처음에 시작할 때 아무 방향 없이 시작 했었는데, 개별 학습 데이터를 바탕으로 취약점과 공부 방향에 개인의 방향을 알려주어 좋았다. 특히 점수대 별에 맞춰, 시기별로 어떤 전략으로 공부하며 좋을지 알려주어서, 혼자서 공부할 때의 막막함을 해소 할 수 있어서 좋았다.</v>
       </c>
       <c r="F240" t="str">
-        <v>나는 원래 공부할 때 학습 계획은 대략적으로 만 세우고, 플레너는 쓰지도 않았었다. 하지만 이투스247에서 제공하는 프로그램으로 학습 계획과 플레너를 쓰면서, 객관적인 공부 시간을 시각적으로 파악하며, 따로 큰 힘을 들이지 않아도 공부 계획을 세울 수 있었다. 그리고 완료한 항목에 체크 표시를 해 나가면서 성취감도 얻을 수 있었고, 나의 기록을 보며 특정과목에만 치우치지 않게 공부양을 조절하며, 매일 기록을 복기하며 어려웠던 부분을 마스터 할 수 있었다.</v>
+        <v>나는 원래 공부할 때 학습 계획은 대략적으로 만 세우고, 플래너는 쓰지도 않았었다. 하지만 이투스247에서 제공하는 프로그램으로 학습 계획과 플래너를 쓰면서, 객관적인 공부 시간을 시각적으로 파악하며, 따로 큰 힘을 들이지 않아도 공부 계획을 세울 수 있었다. 그리고 완료한 항목에 체크 표시를 해 나가면서 성취감도 얻을 수 있었고, 나의 기록을 보며 특정과목에만 치우치지 않게 공부양을 조절하며, 매일 기록을 복기하며 어려웠던 부분을 마스터 할 수 있었다.</v>
       </c>
       <c r="G240" t="str" xml:space="preserve">
         <v xml:space="preserve">나의 공부에서 가장 큰 문제는 공부 시간을 제대로 활용하지 못하고 딴 짓을 한다는 것이었다. 그런데 와이파이 장벽은 스스로 자기 통제가 어려운 수험 생활 초반에 올바른 공부 습관을 형성하는데 큰 도움을 주었다. _x000d_
@@ -9557,7 +9557,7 @@
 앞으로도 선생님들께 배운 점을 바탕으로 더 노력하는 모습 보여드리겠습니다. 다시 한 번 진심으로 감사드립니다</v>
       </c>
       <c r="J253" t="str">
-        <v>학원에서 처음으로 저의 학습 성향을 알게 되면서 어떻게 공부를 해야 할 지 습관을 바로 잡을 수 있어서 좋았습니다.</v>
+        <v>학원에서 처음으로 저의 학습 성향을 알게 되면서 어떻게 공부를 해야 할지 습관을 바로 잡을 수 있어서 좋았습니다.</v>
       </c>
       <c r="K253" t="str">
         <v/>
@@ -9684,7 +9684,7 @@
         <v>N수생</v>
       </c>
       <c r="E257" t="str">
-        <v>공부를 시작할 때 어떤 걸 해야 할 지 모르겠는 막막함과 두려움이 있었습니다. 하지만 이투스 코칭 시스템을 통해 올바른 방향으로 공부를 할 수 있어서 심리적으로 안정감도 들고 도움이 많이 되었습니다.</v>
+        <v>공부를 시작할 때 어떤 걸 해야 할지 모르겠는 막막함과 두려움이 있었습니다. 하지만 이투스 코칭 시스템을 통해 올바른 방향으로 공부를 할 수 있어서 심리적으로 안정감도 들고 도움이 많이 되었습니다.</v>
       </c>
       <c r="F257" t="str">
         <v>인강 콘텐츠들이 넘쳐나는 요즘 시대에서 나한테 맞고 좋은 선생님들 찾는데 시간이 많이 걸리고 지치는 일이 많았습니다. 하지만 이투스학원에서 추천해주시고 알려주시는 덕분에 스트레스 받는 일도 덜 했고 효과적이었습니다.</v>
@@ -9696,7 +9696,7 @@
         <v>각 인강 사이트마다 자신한테 맞는 선생들이 계시기 때문에 여러 패스를 끊어서 맞는 분을 찾는게 제일이지만 패스를 끊는 것도 비용이 들기 때문에 부담이 컸습니다. 그러나 이투스 247을 다니면 이투스 패스를 주어서 인강 선생님들 뵐 수 있다는 것이 비용적으로 부담이 줄었고 좋았습니다.</v>
       </c>
       <c r="I257" t="str">
-        <v>어떻게 공부를 해야 할 지 모르던 저에게 올바른 방향을 제시해주시고 멘탈이 흔들릴 때나 지칠 때 잡아주시고 따뜻하게 대해주셔서 정말 감사했습니다. 덕분에 긴 수험 생활 잘 버틴 것 같습니다.!!</v>
+        <v>어떻게 공부를 해야 할지 모르던 저에게 올바른 방향을 제시해주시고 멘탈이 흔들릴 때나 지칠 때 잡아주시고 따뜻하게 대해주셔서 정말 감사했습니다. 덕분에 긴 수험 생활 잘 버틴 것 같습니다.!!</v>
       </c>
       <c r="J257" t="str">
         <v>졸음 지도 및 관리 덕분에 집중력을 유지하여, 순공 시간 확보에 큰 도움이 되었어요.</v>
@@ -9970,7 +9970,7 @@
         <v>반수하고 6월에 기숙학원에 들어와서 어떤 선생님에 수업을 들어야할지 고민하던 중 이투스 이천 기숙학원에 계시는 담당 선생님의 학습 상담을 통해 빠르게 공부의 방향을 잡고 진도를 나갈 수 있었습니다.</v>
       </c>
       <c r="F265" t="str">
-        <v>이투스 이천 247 기숙학원에 계시는 담당 선생님께서 매주 상담을 진행하시며 플레너에 계획한 계획을 잘 지켰는지 매주 검사하고 방향성을 정하는 시간을 가졌는데요. 이 덕분에 학습 분량 조절을 원활히 할 수 있었습니다</v>
+        <v>이투스 이천 247 기숙학원에 계시는 담당 선생님께서 매주 상담을 진행하시며 플래너에 계획한 계획을 잘 지켰는지 매주 검사하고 방향성을 정하는 시간을 가졌는데요. 이 덕분에 학습 분량 조절을 원활히 할 수 있었습니다</v>
       </c>
       <c r="G265" t="str">
         <v>독서실에 있으면 다른 생각이 들기 마련인데, 와이파이 방화벽이 정말 잘 되어있어 공부에만 집중할 수 있었습니다. 그 덕분에 이투스247 기숙학원에 있는 동안에는 공부에만 몰두하여 좋은 성적을 거둘 수 있었던 거 같습니다.</v>
@@ -10836,7 +10836,7 @@
         <v>학습을 하면서 잘 모르는 것들을 물어볼 수 있다는 것이 가장 유용했다고 할 수 있는데, 학습을 하는 데 잘 몰랐던 개념들이 분명해지는 계기가 되었습니다. 국어, 수학, 영어에서 문제를 풀 때 실질적으로 유용한 풀이 방법들도 알려주셔서 수능을 준비하는 데 도움이 되었습니다.</v>
       </c>
       <c r="F288" t="str">
-        <v>공부를 하는 데 있어서 가장 중요한 것 중 하나가 시간관리입니다. 이투스 247에서 제공하는 플래너 관리는 제가 학원에 있는 동안 시간관리를 하는 데 있어서 큰 도움이 되었는데, 제가 어느 과목을 얼만큼 공부하는지를 실질적으로 보여주었고 이를 반영해서 어느 과목에 시간을 투자해야 할 지를 알 수 있게 해주었습니다.</v>
+        <v>공부를 하는 데 있어서 가장 중요한 것 중 하나가 시간관리입니다. 이투스 247에서 제공하는 플래너 관리는 제가 학원에 있는 동안 시간관리를 하는 데 있어서 큰 도움이 되었는데, 제가 어느 과목을 얼만큼 공부하는지를 실질적으로 보여주었고 이를 반영해서 어느 과목에 시간을 투자해야 할지를 알 수 있게 해주었습니다.</v>
       </c>
       <c r="G288" t="str">
         <v>요즘에 학습을 하는 데 있어서 가장 큰 방해물 중 하나가 스마트폰이라고 할 수 있습니다. 학습하는 동안에 스마트폰이 있으면 스마트폰에 집중이 분산되어서 학습에 온전히 집중할 수 없는데, 이러한 방해물에 대한 사전의 차단은 학습 시간을 밀도있게 하는 데 매우 유용했습니다.</v>
@@ -11617,7 +11617,7 @@
         <v>반수생</v>
       </c>
       <c r="E310" t="str">
-        <v>다양한 대학교와 목표하는 대학교의 입결과 대학별로 더 중요치를 두는 과목 등에 대해서 자세하게 설명해주셔서 어느부분의 공부에 더욱 집중하여 학습해야 할 지 알 수 있어서 많은 도움이 되았습니다!</v>
+        <v>다양한 대학교와 목표하는 대학교의 입결과 대학별로 더 중요치를 두는 과목 등에 대해서 자세하게 설명해주셔서 어느부분의 공부에 더욱 집중하여 학습해야 할지 알 수 있어서 많은 도움이 되았습니다!</v>
       </c>
       <c r="F310" t="str">
         <v>매주 보는 개인 모의고사라던지, 평가원 모의고사, 달마다 학원에서 전체시행하는 더프모의고사같은 모의고사를 보고 나서 혼자서 사고하기 어려웠던 부분들에 대해 여쭈어보면 친절하게 알려주시고 그렇게 배운 부분이 하나의 자양분이 되어서 좋은 성적의 발판이 되었다고 생각합니다!</v>
@@ -12125,7 +12125,7 @@
         <v>1년 동안 옆에서 꼼꼼하게 챙겨주신 선생님들께 정말 감사드립니다. 힘들고 지칠 때마다 따뜻하게 격려해주신 덕분에 끝까지 포기하지 않고 버틸 수 있었어요. 덕분에 좋은 결과를 얻을 수 있었습니다. 감사합니다!​​​​​​​​​​​​​​​​</v>
       </c>
       <c r="J324" t="str">
-        <v>시기별로 인강 추천을 해주셔서 어떤 것을 들어야 할 지 찾는 시간을 아껴 공부할 수 있었어요.</v>
+        <v>시기별로 인강 추천을 해주셔서 어떤 것을 들어야 할지 찾는 시간을 아껴 공부할 수 있었어요.</v>
       </c>
       <c r="K324" t="str">
         <v>인강 추천</v>
@@ -12983,7 +12983,7 @@
         <v>담임 선생님께서 상담하실 때 마다 각 과목 별 공부가 어떻게 진행되고 있는지 구체적으로 상담해주시고(예를 들면 어떤 인강을 듣고 있는지, 또는 어떤 문제집을 풀고 있는지) 해당 내용이 끝난 다음에는 어떤 커리큘럼을 밟으면 좋은지 상담해주시는 등 구체적인 공부방향 설정에 큰 도움을 주셨습니다.</v>
       </c>
       <c r="F348" t="str">
-        <v>플래너를 주기적으로 검사함을 통해 하루에 몇 시간 정도 공부하는지 또 과목별로 균형있게 학습하고 있는 지를 확인해 주시고 그에 따라 학습 피드백을 해주시는 것이 좋았습니다. 또 상담을 통해 또는 스스로 세운 계획을 얼마나 잘 지키고 있는지 점검함을 통해 학습 관리를 잘 해주신 부분이 좋았습니다.</v>
+        <v>플래너를 주기적으로 검사함을 통해 하루에 몇 시간 정도 공부하는지 또 과목별로 균형 있게 학습하고 있는 지를 확인해 주시고 그에 따라 학습 피드백을 해주시는 것이 좋았습니다. 또 상담을 통해 또는 스스로 세운 계획을 얼마나 잘 지키고 있는지 점검함을 통해 학습 관리를 잘 해주신 부분이 좋았습니다.</v>
       </c>
       <c r="G348" t="str">
         <v>담임 선생님들이 주기적으로 면학 분위기 조성에 힘쓰시는 것이 느껴졌습니다. 일단 오전, 오후마다 선생님들이 졸고 있는 학생들을 깨우셨고 휴가 전후로 전체적으로 분위기가 헤이해지면 더 강하게 면학 분위기 관리에 힘을 쓰셨습니다. 덕분에 분위기에 휩쓸리지 않고 공부할 수 있어서 좋았습니다.</v>
@@ -13766,7 +13766,7 @@
         <v>N수생</v>
       </c>
       <c r="E369" t="str">
-        <v>수시원서 접수 상담 과정에서 다양한 자료를 제공받아 대학을 대학선택에 큰 도움을 받았고, 세 차례의 상담을 통해  학생에게 더 적합한 대학을 구체적으로 판단해주셔서 원서 접수를 보다 수월하게 진행할 수 있었습니다.</v>
+        <v>수시 원서 접수 상담 과정에서 다양한 자료를 제공받아 대학을 대학선택에 큰 도움을 받았고, 세 차례의 상담을 통해  학생에게 더 적합한 대학을 구체적으로 판단해주셔서 원서 접수를 보다 수월하게 진행할 수 있었습니다.</v>
       </c>
       <c r="F369" t="str">
         <v>매달 한 번씩 진행된 상담을 통해 학습 과정에서의 고민을 해소할 수 있어 도움이 되었으며, 지속적인 상담으로 체계적인 케어를 받는다는 느낌을 받았습니다. 또한 플래너 관리를 통해 부족한 부분을 보완할 수 있었습니다.</v>

</xml_diff>

<commit_message>
Apply fifth batch of typo corrections
</commit_message>
<xml_diff>
--- a/reviews_with_keywords.xlsx
+++ b/reviews_with_keywords.xlsx
@@ -497,7 +497,7 @@
         <v>N수생</v>
       </c>
       <c r="E3" t="str">
-        <v>학생별 맞춤 진도 상담을 통해 부족한 부분을 정확히 파악할 수 있었고, 모의고사 이후 구체적인 공부 방향을 제시해주어 큰 도움이 되었습니다. 특히 막히는 부분에 대한 친절한 질의응답 덕분에 학습 효율이 높아져 매우 만족스럽습니다</v>
+        <v>학생별 맞춤 진도 상담을 통해 부족한 부분을 정확히 파악할 수 있었고, 모의고사 이후 구체적인 공부 방향을 제시해 주어 큰 도움이 되었습니다. 특히 막히는 부분에 대한 친절한 질의응답 덕분에 학습 효율이 높아져 매우 만족스럽습니다</v>
       </c>
       <c r="F3" t="str">
         <v>학습 플래너를 꼼꼼히 확인하며 진도를 체크해 주신 점이 좋았습니다. 특히 제 취약 부분을 정확히 짚어내고, 앞으로의 학습 방향과 구체적인 보완 방법을 세밀하게 코칭해 주셔서 큰 확신을 가지고 공부에 매진할 수 있었습니다</v>
@@ -512,7 +512,7 @@
         <v>철저한 출결 관리와 졸음 방지 등 학원의 전반적인 분위기를 세심하게 잡아주신 선생님께 진심으로 감사드립니다! 선생님의 지도 덕분에 나태해지지 않고 수험 생활을 끝까지 완주할 수 있었습니다. 덕분에 재수하여 현재 대학 생활을 즐겁게 하고 있습니다. 제 공부 습관을 바로잡아 주시고 대학 입학까지 잘 이끌어 주셔서 정말 감사합니다</v>
       </c>
       <c r="J3" t="str">
-        <v>학생별 맞춤 진도 상담을 통해 부족한 부분을 정확히 파악할 수 있었고, 모의고사 이후 구체적인 공부 방향을 제시해주어 큰 도움이 되었어요.</v>
+        <v>학생별 맞춤 진도 상담을 통해 부족한 부분을 정확히 파악할 수 있었고, 모의고사 이후 구체적인 공부 방향을 제시해 주어 큰 도움이 되었어요.</v>
       </c>
       <c r="K3" t="str">
         <v>모의고사</v>
@@ -758,7 +758,7 @@
         <v>재수하면서 선생님들을 정말 귀찮게 많이 했는데.. 불편한 기색없이 질문도 정말 정성스럽게 답변해주시고 고민들도 같이 들어주고, 고민하고, 도움을 주셨던 부분들이 정말 감사했습니다.</v>
       </c>
       <c r="J10" t="str">
-        <v>정말 나에게 맞는 공부를 추천해주시고, 관리도 잘해주셔서 성적이 오를 수 있었어요.</v>
+        <v>정말 나에게 맞는 공부를 추천해 주시고, 관리도 잘해주셔서 성적이 오를 수 있었어요.</v>
       </c>
       <c r="K10" t="str">
         <v/>
@@ -934,7 +934,7 @@
         <v>선생님 따로 연락은 제대로 못 드렸지만 언제나 학원에서 인사해주시고 공부잘되어가는지 힘든건 없는지 여쭤봐주셔서 감사했어요. 길고 긴 수험 생활이었지만 이투스 덕분에 저에게 과분한 대학에 오게된 것 같아 아직도 감사합니다. ㅎㅎ</v>
       </c>
       <c r="J15" t="str">
-        <v>원장 선생님께서 재원생 한 명, 한 명을 기억하시고, 마주치실 때마다 공부는 잘 되는지 항상 체크해주셨어요.</v>
+        <v>원장 선생님께서 재원생 한 명, 한 명을 기억하시고, 마주치실 때마다 공부는 잘 되는지 항상 체크해 주셨어요.</v>
       </c>
       <c r="K15" t="str">
         <v/>
@@ -1036,10 +1036,10 @@
         <v>특히 국어의 경우, 실제 모의고사 형태로 되어있어서 일일테스트를 통해 부족한 부분을 발견하고, 점검할 수 있었습니다. 실제로 일일테스트를 통해 독서에서의 부족한 점을 찾고 보완한 바 있습니다. 또한 영어 단어, 듣기까지 등한시하지 않고 매일 테스트를 보니 감을 잃지 않을 수 있었습니다</v>
       </c>
       <c r="I18" t="str">
-        <v>윈터스쿨 2달동안 생활, 학습 전반적인 부분에서 밀도있게 관리해주셔서 현재 따로 관리형을 다니지 않아도 그때의 습관이 그대로 남아있는것 같습니다. 또, 정말 중요한 영어 과목에서 늘 3등급이 나오던게 속상했었는데 클리닉을 받고, 독해, 단어에서 부족한 점을 2달동안 바로잡은 덕분에 이번 3월 모의고사에서 85점이라는 점수를 받을 수 있었습니다. 학습 상담, 생활 상담, 입시 상담까지 모두 윈터스쿨에서 그치는게 아니라 개학 후에까지 긍정적인 영향을 주고 있다고 생각합니다. 썸머스쿨, 2학기기간에 다시 복귀해서도 열심히 다니겠습니다. 감사합니다</v>
+        <v>윈터스쿨 2달동안 생활, 학습 전반적인 부분에서 밀도있게 관리해 주셔서 현재 따로 관리형을 다니지 않아도 그때의 습관이 그대로 남아있는것 같습니다. 또, 정말 중요한 영어 과목에서 늘 3등급이 나오던게 속상했었는데 클리닉을 받고, 독해, 단어에서 부족한 점을 2달동안 바로잡은 덕분에 이번 3월 모의고사에서 85점이라는 점수를 받을 수 있었습니다. 학습 상담, 생활 상담, 입시 상담까지 모두 윈터스쿨에서 그치는 게 아니라 개학 후에까지 긍정적인 영향을 주고 있다고 생각합니다. 썸머스쿨, 2학기기간에 다시 복귀해서도 열심히 다니겠습니다. 감사합니다</v>
       </c>
       <c r="J18" t="str">
-        <v>학습 상담, 생활 상담, 입시 상담까지 모두 윈터스쿨에서 그치는게 아니라 개학 후에까지 긍정적인 영향을 주고 있다고 생각했어요.</v>
+        <v>학습 상담, 생활 상담, 입시 상담까지 모두 윈터스쿨에서 그치는 게 아니라 개학 후에까지 긍정적인 영향을 주고 있다고 생각했어요.</v>
       </c>
       <c r="K18" t="str">
         <v>학습 관리, 입시 관리, 생활 관리</v>
@@ -1071,7 +1071,7 @@
         <v>전국적인 본인의 위치를 알기 좋습니다. 통계적으로 각 과목별로 나와 있어서 상당히 보기가 좋습니다. 공부에 대한 경쟁의식을 자극하기도 하여 좋았습니다. 공부를 몰입할 수 있었습니다.</v>
       </c>
       <c r="I19" t="str">
-        <v>감사합니다. 특히 급식을 해주셨던 영양사분께 특별히 엄청난 감사를 전합니다. 재수학원 다니면서 제일 행복할때가 밥을 섭취할 때였으며 충분히 배부르게 먹을 수 있었습니다. 영양사분들께 너무나도 감사드립니다.</v>
+        <v>감사합니다. 특히 급식을 해주셨던 영양사분께 특별히 엄청난 감사를 전합니다. 재수 학원 다니면서 제일 행복할때가 밥을 섭취할 때였으며 충분히 배부르게 먹을 수 있었습니다. 영양사분들께 너무나도 감사드립니다.</v>
       </c>
       <c r="J19" t="str">
         <v>잠 관리가 잘 안되는 편이였는데 생활 담임 선생님들이 아침에 깨워주셔서 규칙적인 학습 루틴을 유지할 수 있었어요.</v>
@@ -1187,7 +1187,7 @@
         <v>예전에는 시간에만 쫓기다가 제대로된 학습을 못했는데 이투스247에 다니면서 어떻게 공부해야 효율적으로 학습할 수 있는지 배울 수 있었습니다. 6모 전까지 어디까지 끝내야 하는지, 9모 전까지 어디까지 끝내야 하는지, N제는 어떤 교재가 좋은지 등 자세한 코칭 시스템 덕분에 계획적으로 공부할 수 있었습니다.</v>
       </c>
       <c r="F22" t="str">
-        <v>무조건 유명한 강사 뿐만이 아니라 학생 개인에게 맞는 인강과 강사를 추천해주시고 성적에 따라 단계적으로 수준에 맞는 강의를 추천해 주셔서 유용했습니다. 기출이나 N제 또한 진도와 성적에 맞는 교재로 추천해 주셔서 성적 향상에 더 큰 도움을 받을 수 있었습니다.</v>
+        <v>무조건 유명한 강사 뿐만이 아니라 학생 개인에게 맞는 인강과 강사를 추천해 주시고 성적에 따라 단계적으로 수준에 맞는 강의를 추천해 주셔서 유용했습니다. 기출이나 N제 또한 진도와 성적에 맞는 교재로 추천해 주셔서 성적 향상에 더 큰 도움을 받을 수 있었습니다.</v>
       </c>
       <c r="G22" t="str">
         <v>면학 분위기가 굉장히 좋았습니다. 자습실도 책상마다 칸막이가 설치되어있어서 더 공부에 몰입할 수 있었고 강의실 또한 쾌적했습니다. 가끔 피곤해서 졸리기도 했지만 감독 선생님들께서 친절하게 깨워주셔서 다시 정신을 차릴 수 있었습니다.</v>
@@ -1219,25 +1219,25 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E23" t="str">
-        <v>재수학원에서 받은 학습 상담은 나의 학습 방향을 구체적으로 설정하는 데 큰 도움이 되었다. 특히 상담을 통해 모든 과목을 동일하게 끌어올리기보다는, 부족한 과목은 기본 점수를 확보하는 수준으로 관리하고 자신 있는 과목은 최대한 점수를 끌어올리는 전략이 효과적이라는 점을 배웠다. 이에 따라 취약 과목은 핵심 개념 위주로 최소한의 점수를 확보하는 데 집중하고, 강점 과목에는 더 많은 시간을 투자해 고득점을 목표로 학습 계획을 세웠다. 이러한 전략적 접근 덕분에 전체적인 성적 균형을 유지하면서도 총점을 효율적으로 높일 수 있었고, 학습에 대한 부담도 줄일 수 있었다.</v>
+        <v>재수 학원에서 받은 학습 상담은 나의 학습 방향을 구체적으로 설정하는 데 큰 도움이 되었다. 특히 상담을 통해 모든 과목을 동일하게 끌어올리기보다는, 부족한 과목은 기본 점수를 확보하는 수준으로 관리하고 자신 있는 과목은 최대한 점수를 끌어올리는 전략이 효과적이라는 점을 배웠다. 이에 따라 취약 과목은 핵심 개념 위주로 최소한의 점수를 확보하는 데 집중하고, 강점 과목에는 더 많은 시간을 투자해 고득점을 목표로 학습 계획을 세웠다. 이러한 전략적 접근 덕분에 전체적인 성적 균형을 유지하면서도 총점을 효율적으로 높일 수 있었고, 학습에 대한 부담도 줄일 수 있었다.</v>
       </c>
       <c r="F23" t="str">
-        <v>재수학원의 1대1 질의응답 시스템은 모르는 문제를 단순히 해결하는 것을 넘어, 문제를 접근하는 방법 자체를 배우는 데 유용했다. 특히 모의고사 이후 틀린 문제를 질문하면 단순한 해설이 아니라 문제를 푸는 과정과 공략법을 단계적으로 설명해 주어, 같은 유형의 문제를 다시 만났을 때 스스로 해결할 수 있는 능력을 기를 수 있었다. 또한 과목별로 효율적인 풀이 순서와 시간 배분 방법 등 구체적인 학습방법까지 제시해 주어, 실전에서의 문제 해결 능력을 높이는 데 도움이 되었다. 이를 통해 단순 암기 중심의 공부에서 벗어나 전략적으로 문제를 해결하는 학습 습관을 형성할 수 있었다.</v>
+        <v>재수 학원의 1대1 질의응답 시스템은 모르는 문제를 단순히 해결하는 것을 넘어, 문제를 접근하는 방법 자체를 배우는 데 유용했다. 특히 모의고사 이후 틀린 문제를 질문하면 단순한 해설이 아니라 문제를 푸는 과정과 공략법을 단계적으로 설명해 주어, 같은 유형의 문제를 다시 만났을 때 스스로 해결할 수 있는 능력을 기를 수 있었다. 또한 과목별로 효율적인 풀이 순서와 시간 배분 방법 등 구체적인 학습방법까지 제시해 주어, 실전에서의 문제 해결 능력을 높이는 데 도움이 되었다. 이를 통해 단순 암기 중심의 공부에서 벗어나 전략적으로 문제를 해결하는 학습 습관을 형성할 수 있었다.</v>
       </c>
       <c r="G23" t="str" xml:space="preserve">
-        <v xml:space="preserve">재수학원의 생활 관리 시스템 중에서 특히 면학 분위기 감독과 졸음 관리는 실제로 공부하는 데 있어 정말 많은 도움이 됐다._x000d_
+        <v xml:space="preserve">재수 학원의 생활 관리 시스템 중에서 특히 면학 분위기 감독과 졸음 관리는 실제로 공부하는 데 있어 정말 많은 도움이 됐다._x000d_
 면학 분위기 감독의 경우, 처음에는 감시받는 느낌이 좀 불편하게 느껴질 수도 있는데 막상 생활해보면 오히려 고맙게 느껴지는 부분이 많았다. 혼자 집에서 공부할 때는 핸드폰을 한 번만 보려 했다가 어느새 한 시간이 훌쩍 지나있는 경우가 다반사였는데, 학원에서는 그런 유혹 자체가 차단되다 보니 자연스럽게 공부에만 집중할 수 있었다. 또 주변 친구들이 모두 묵묵히 공부하고 있는 모습을 보면 나도 모르게 자극을 받게 되고, 괜히 혼자 딴짓을 하기가 민망해지는 분위기가 만들어졌다. 억지로 집중하려 애쓰지 않아도 환경 자체가 집중하게 만들어준다는 게 가장 큰 장점이었다._x000d_
 졸음 관리도 생각보다 훨씬 유용했다. 재수를 하다 보면 마음이 무겁고 무기력해지는 날이 많아서 자꾸 늦게 자고 늦게 일어나는 패턴이 생기기 쉬운데, 학원의 규칙적인 기상과 취침 시간 덕분에 생활 리듬을 잡을 수 있었다. 특히 수능 시험 시간대에 맞춰 뇌가 활발하게 돌아가는 습관이 만들어진다는 점은 장기적으로 정말 중요한 부분이었다. 오후에 졸음이 몰려올 때 잠깐의 낮잠 시간을 허용해주는 것도 좋았는데, 억지로 버티다가 결국 책상에 엎드려 한 시간을 자는 것보다 짧게 자고 개운하게 다시 시작하는 편이 훨씬 효율적이었다. 졸음이 심할 때 선생님과 개별적으로 이야기를 나누며 원인을 찾아볼 수 있었던 것도 단순한 졸음 관리를 넘어 전반적인 컨디션을 챙겨준다는 느낌이 들어서 꽤 든든했다._x000d_
 돌이켜보면 이 두 가지 시스템이 잘 갖춰져 있었기 때문에 흔들리기 쉬운 재수 생활을 버텨낼 수 있었던 것 같다. 스스로를 통제하는 게 어려울 때 환경이 그 역할을 대신해준다는 게 얼마나 큰 힘이 되는지, 직접 경험하고 나서야 비로소 알게 됐다.</v>
       </c>
       <c r="H23" t="str">
-        <v>재수학원의 모의고사 시스템은 나의 현재 학습 수준을 객관적으로 파악하는 데 큰 도움이 되었다. 이전에는 모의고사를 충분히 경험해보지 못해 실전 감각과 위치를 정확히 알기 어려웠지만, 정기적인 모의고사를 통해 나의 성적과 등급을 구체적으로 확인할 수 있었다. 특히 과목별 점수와 취약 단원을 분석하면서 어떤 부분을 보완해야 하는지 명확히 알게 되었고, 이를 바탕으로 학습 방향을 설정할 수 있었다. 그 결과 막연하게 공부하는 것이 아니라 목표와 전략을 가지고 효율적으로 학습할 수 있게 되었다.</v>
+        <v>재수 학원의 모의고사 시스템은 나의 현재 학습 수준을 객관적으로 파악하는 데 큰 도움이 되었다. 이전에는 모의고사를 충분히 경험해보지 못해 실전 감각과 위치를 정확히 알기 어려웠지만, 정기적인 모의고사를 통해 나의 성적과 등급을 구체적으로 확인할 수 있었다. 특히 과목별 점수와 취약 단원을 분석하면서 어떤 부분을 보완해야 하는지 명확히 알게 되었고, 이를 바탕으로 학습 방향을 설정할 수 있었다. 그 결과 막연하게 공부하는 것이 아니라 목표와 전략을 가지고 효율적으로 학습할 수 있게 되었다.</v>
       </c>
       <c r="I23" t="str">
         <v>이투스 247 선생님들께 진심으로 감사드립니다. 공부가 힘들고 지칠 때마다 흔들리던 저의 마음을 바로잡아 주시고, 다시 학습에 집중할 수 있도록 도와주신 점이 가장 큰 힘이 되었습니다. 특히 피로감이 쌓여 집중력이 떨어질 때마다 적절한 조언과 격려를 통해 다시 공부 흐름을 이어갈 수 있게 해주신 덕분에 끝까지 포기하지 않고 학습을 이어갈 수 있었습니다. 선생님들의 세심한 지도와 관심이 있었기에 지금까지 꾸준히 노력할 수 있었다고 생각합니다. 진심으로 감사드립니다.</v>
       </c>
       <c r="J23" t="str">
-        <v>재수학원의 생활 관리 시스템 중에서 특히 면학 분위기 감독과 졸음 관리는 실제로 공부하는 데 있어 정말 많은 도움이 됐어요.</v>
+        <v>재수 학원의 생활 관리 시스템 중에서 특히 면학 분위기 감독과 졸음 관리는 실제로 공부하는 데 있어 정말 많은 도움이 됐어요.</v>
       </c>
       <c r="K23" t="str">
         <v>생활 관리, 면학 분위기, 졸음 관리</v>
@@ -1340,10 +1340,10 @@
         <v>모의고사의 양이 절대적으로 중요한 학생들에게 이투스 모의고사라는 자체적인 컨텐츠를 제공하는 점이 좋았습니다. 또 그 컨텐츠가 단순히 기출을 짜깁기한 것이 아니라 새롭고 퀄리티 있는 시험지라는 점에서 너무나도 큰 도움이 되었습니다.</v>
       </c>
       <c r="I26" t="str">
-        <v>재학 기간 동안 많은 건강적인 문제가 있었는데 많은 편의를 봐주셔서 오랫동안 공부하며 꾸준히 노력할 수 있었습니다 감사합니다. 또 지칠 때 응원해주시며 동기부여해주시는 게 수험 생활의 소소한 낙이었습니다. 감사드립니다</v>
+        <v>재학 기간 동안 많은 건강적인 문제가 있었는데 많은 편의를 봐주셔서 오랫동안 공부하며 꾸준히 노력할 수 있었습니다 감사합니다. 또 지칠 때 응원해주시며 동기부여해 주시는 게 수험 생활의 소소한 낙이었습니다. 감사드립니다</v>
       </c>
       <c r="J26" t="str">
-        <v>지칠 때 응원해주시며 동기부여해주시는 게 수험 생활의 소소한 낙이었어요.</v>
+        <v>지칠 때 응원해주시며 동기부여해 주시는 게 수험 생활의 소소한 낙이었어요.</v>
       </c>
       <c r="K26" t="str">
         <v/>
@@ -1666,7 +1666,7 @@
         <v>진짜 너무 고맙습니다. 여기 안들어갔으면 엄마 등골 빨아먹으면서 집에 눌러앉은 백수가 되거나 재수를 하면서 더 많은 비용을 내거나 둘 중 하나가 돨뻔했는데 대학 들어가니깐 너무 고맙더라고요. 특히 부원장님, 국어 수업 너무 좋았어요.</v>
       </c>
       <c r="J35" t="str">
-        <v>이투스247학원이 없었다면 공부할 환경 자체가 만들어지지 않았을 거에요.</v>
+        <v>이투스247학원이 없었다면 공부할 환경 자체가 만들어지지 않았을 거예요.</v>
       </c>
       <c r="K35" t="str">
         <v/>
@@ -1722,7 +1722,7 @@
         <v>반수생</v>
       </c>
       <c r="E37" t="str">
-        <v>반수를 시작했을 때는 이미 늦었다는 생각이 들어 불안했지만, 이투스247재수학원에서 체계적인 관리와 상담을 받으며 더 빠르게 방향을 잡을 수 있었던 것 같다. 학습 상담을 통해 현재 실력을 정확히 파악하고 효율적인 공부 방법을 제시받아 시간 낭비를 줄일 수 있었고, 생활상담을 통해 흐트러지기 쉬운 생활 패턴도 안정적으로 유지할 수 있었다. 또한 입시상담에서는 현실적인 조언과 전략을 통해 목표를 구체화할 수 있어 막연했던 불안이 많이 해소되었다. 전반적으로 늦게 시작했음에도 불구하고 빠르게 중심을 잡고 끝까지 버틸 수 있도록 큰 도움을 받은 만족스러운 경험이었다.</v>
+        <v>반수를 시작했을 때는 이미 늦었다는 생각이 들어 불안했지만, 이투스247재수 학원에서 체계적인 관리와 상담을 받으며 더 빠르게 방향을 잡을 수 있었던 것 같다. 학습 상담을 통해 현재 실력을 정확히 파악하고 효율적인 공부 방법을 제시받아 시간 낭비를 줄일 수 있었고, 생활상담을 통해 흐트러지기 쉬운 생활 패턴도 안정적으로 유지할 수 있었다. 또한 입시상담에서는 현실적인 조언과 전략을 통해 목표를 구체화할 수 있어 막연했던 불안이 많이 해소되었다. 전반적으로 늦게 시작했음에도 불구하고 빠르게 중심을 잡고 끝까지 버틸 수 있도록 큰 도움을 받은 만족스러운 경험이었다.</v>
       </c>
       <c r="F37" t="str">
         <v>인강 추천이 체계적이고 수준에 맞게 이루어져서 공부 효율이 크게 올라갔다. 과목별로 필요한 강의를 정확히 짚어주어 불필요한 선택 고민이 줄었고, 덕분에 시간 낭비 없이 핵심 내용에 집중할 수 있어 전체적인 학습 만족도가 높았다.</v>
@@ -1770,7 +1770,7 @@
         <v>저는 영어 공부를 하기 정말 싫어했는데요, 이투스 voca 덕분에 꾸준히 조금씩이라도 영단어 학습을 해서 성적을 유지할 수 있었던 것 같습니다. 특히 저는 점심,저녁 먹고 자투리 시간을 활용해서 영단어를 틈틈히 외웠던게 수능 때 도움이 되었던 것 같습니다.</v>
       </c>
       <c r="I38" t="str">
-        <v>언제나 진심으로 최선을 다해서 학생들을 관리해주셔서 감사합니다. 덕분에 알찬 일년을 보낼 수 있었던 것 같습니다. 만약 주변에서 독학재수학원을 고민하는 지인이 있다면, 저는 고민없이 이투스247을 추천랄 것 같습니다.</v>
+        <v>언제나 진심으로 최선을 다해서 학생들을 관리해 주셔서 감사합니다. 덕분에 알찬 일년을 보낼 수 있었던 것 같습니다. 만약 주변에서 독학재수 학원을 고민하는 지인이 있다면, 저는 고민없이 이투스247을 추천랄 것 같습니다.</v>
       </c>
       <c r="J38" t="str">
         <v>저는 2주에 한 번씩 학습 상담을 받았었는데요, 상담을 받으면서 기피하는 과목을 가까이 하는 방법에 대해 많은 조언을 해주셨어요.</v>
@@ -1899,7 +1899,7 @@
         <v>N수생</v>
       </c>
       <c r="E42" t="str">
-        <v>지점마다 차이가 있겠지만 다른 독학재수학원에 비해 학생당 선생님 수가 많아서 디테일한 상담이 가능했고 이로 하여금 담임 선생님께서 잘하고 있는 점부터 약한 과목에 대한 보충방법까지 잘 설명해주셨다.</v>
+        <v>지점마다 차이가 있겠지만 다른 독학재수 학원에 비해 학생당 선생님 수가 많아서 디테일한 상담이 가능했고 이로 하여금 담임 선생님께서 잘하고 있는 점부터 약한 과목에 대한 보충방법까지 잘 설명해주셨다.</v>
       </c>
       <c r="F42" t="str">
         <v>주기적으로 일정기간동안 작성한 플래너를 검사받으면서 담임 선생님과 어떤 교재나 강의 그리고 공부 계획등을 언제까지 끝낼지, 또 그 계획이 잘 이루어졌는지를 확인할 수 있어 좋았다. 이로 하여금 계획을 잘 마치겠다는 생각이 계속 공부를 열심히 하게 된 계기가 되었다.</v>
@@ -1911,7 +1911,7 @@
         <v>특정 지점에서는 이투스 인강 패스를 재원기간 내에 한정하여 무료로 증정하는데, 처음 공부를 시작하거나 인강을 처음 들어보는 수험생들이 인강에 적응할 수 있게, 또 좋은 선생님의 강의를 듣게 해주었다.</v>
       </c>
       <c r="I42" t="str">
-        <v>다른 독학재수학원과 차별화된 점이 많았고 이를 실행하는 데에 있어서 선생님들이 엄청나게 열정적이셔서 감사했고 또한 모두 친절하셔서 감사했습니다. 이투스 247 화이팅~~~~~!!!!!</v>
+        <v>다른 독학재수 학원과 차별화된 점이 많았고 이를 실행하는 데에 있어서 선생님들이 엄청나게 열정적이셔서 감사했고 또한 모두 친절하셔서 감사했습니다. 이투스 247 화이팅~~~~~!!!!!</v>
       </c>
       <c r="J42" t="str">
         <v>선생님과 함께 저와 맞는 계획을 세워서 계속 공부를 열심히 할 수 있었어요.</v>
@@ -1969,7 +1969,7 @@
         <v>N수생</v>
       </c>
       <c r="E44" t="str">
-        <v>재수학원에서 담임 선생님이 1:1로 꾸준히 상담을 진행해주셔서 학습적인 부분뿐만 아니라 정신적으로도 큰 위로와 도움을 받을 수 있었습니다. 막연하게 느껴졌던 목표를 현실적으로 다시 설정할 수 있었고, 저의 부족한 부분을 구체적으로 짚어주셔서 하나씩 개선해 나갈 수 있었습니다. 덕분에 공부에 대한 방향성이 분명해지고 자신감도 많이 생겼습니다.</v>
+        <v>재수 학원에서 담임 선생님이 1:1로 꾸준히 상담을 진행해주셔서 학습적인 부분뿐만 아니라 정신적으로도 큰 위로와 도움을 받을 수 있었습니다. 막연하게 느껴졌던 목표를 현실적으로 다시 설정할 수 있었고, 저의 부족한 부분을 구체적으로 짚어주셔서 하나씩 개선해 나갈 수 있었습니다. 덕분에 공부에 대한 방향성이 분명해지고 자신감도 많이 생겼습니다.</v>
       </c>
       <c r="F44" t="str">
         <v>모르는 문제를 질문하면 바로바로 해결할 수 있어 학습의 흐름이 끊기지 않아 좋았습니다. 단순히 정답만 알려주는 것이 아니라 풀이 과정과 개념까지 꼼꼼하게 설명해주셔서 이해도를 높일 수 있었습니다. 덕분에 비슷한 유형의 문제에도 스스로 적용할 수 있는 힘이 길러졌고, 공부에 대한 자신감도 함께 생겼습니다.</v>
@@ -1981,7 +1981,7 @@
         <v>영어단어를 꾸준히 외우는게 생각보다 쉽지 않은데 학원에서 프린트물+테스트를 봐야해서 꾸준히 외울 수 있었던 거 같습니다. 또 중요단어들을 계속 볼 수 있어서 좋았습니다! 단어 외우는 습관을 잡을 수 있는게 가장 좋았어요</v>
       </c>
       <c r="I44" t="str">
-        <v>항상 친절하게 답해주시고 응원해주셔서 넘 감사했어용. 가끔 지칠 때도 있었는데 그때마다 진지하게 함께 고민해주시고 위로도 해주셨고 성적 올리는데도 많은 도움 주셨습니다. 공부습관 잡는데 큰 도움 됐어요</v>
+        <v>항상 친절하게 답해주시고 응원해주셔서 넘 감사했어용. 가끔 지칠 때도 있었는데 그때마다 진지하게 함께 고민해주시고 위로도 해주셨고 성적 올리는 데도 많은 도움 주셨습니다. 공부습관 잡는데 큰 도움 됐어요</v>
       </c>
       <c r="J44" t="str">
         <v>규칙적인 생활 습관도 함께 잡을 수 있었고 집중하는 시간도 점점 늘어서 학습에 도움이 많이 됐어요.</v>
@@ -2075,10 +2075,10 @@
         <v>N수생</v>
       </c>
       <c r="E47" t="str">
-        <v>재수학원의 코칭 시스템은 단순한 관리가 아니라 방향을 잡아주는 나침반 같은 존재다. 학습 습관부터 시간 관리, 취약 과목 분석까지 체계적으로 점검해주기 때문에 혼자 공부할 때 놓치기 쉬운 부분을 보완해준다. 덕분에 불안은 줄이고 효율은 높이며, 목표에 더 빠르고 정확하게 다가갈 수 있을 것 같다!</v>
+        <v>재수 학원의 코칭 시스템은 단순한 관리가 아니라 방향을 잡아주는 나침반 같은 존재다. 학습 습관부터 시간 관리, 취약 과목 분석까지 체계적으로 점검해주기 때문에 혼자 공부할 때 놓치기 쉬운 부분을 보완해준다. 덕분에 불안은 줄이고 효율은 높이며, 목표에 더 빠르고 정확하게 다가갈 수 있을 것 같다!</v>
       </c>
       <c r="F47" t="str">
-        <v>재수학원의 코칭 시스템은 모르는 문제를 그냥 넘기지 않게 만드는 점에서 특히 유용한 것 같다. 막힌 문제를 어떻게 접근해야 하는지 풀이 방향과 사고 과정을 짚어주고, 문제 풀이 팁까지 함께 알려주기 때문에 같은 유형을 다시 만났을 때 스스로 해결할 힘이 생긴다. 단순한 정답 암기가 아니라 ‘푸는 방법’을 배우게 해준다는 점에서 큰 도움이 된다.</v>
+        <v>재수 학원의 코칭 시스템은 모르는 문제를 그냥 넘기지 않게 만드는 점에서 특히 유용한 것 같다. 막힌 문제를 어떻게 접근해야 하는지 풀이 방향과 사고 과정을 짚어주고, 문제 풀이 팁까지 함께 알려주기 때문에 같은 유형을 다시 만났을 때 스스로 해결할 힘이 생긴다. 단순한 정답 암기가 아니라 ‘푸는 방법’을 배우게 해준다는 점에서 큰 도움이 된다.</v>
       </c>
       <c r="G47" t="str">
         <v>졸음 관리와 생활 습관 교정에도 큰 도움을 준다. 규칙적인 수면 시간과 학습 리듬을 잡아주고, 집중력이 떨어질 때는 쉬는 타이밍과 방법까지 코칭해줘 효율을 높인다. 덕분에 무작정 버티는 공부가 아니라, 컨디션을 유지하며 꾸준히 몰입할 수 있는 환경을 만들어준다.</v>
@@ -2251,7 +2251,7 @@
         <v>반수생</v>
       </c>
       <c r="E52" t="str" xml:space="preserve">
-        <v xml:space="preserve">국어가 맨날 5~6등급이었지만 국어 멘토링 덕분에 2,3,4등급은 안정적으로 받을 수 있는 수준으로 발전하였다_x000d_
+        <v xml:space="preserve">국어가 맨날 5~6등급이었지만 국어 멘토링 덕분에 2~4등급은 안정적으로 받을 수 있는 수준으로 발전하였다_x000d_
 또한 탐구를 담임 선생님께서 잘 체크해주셔서 빠뜨리지 않고 잘 공부할 수있었다</v>
       </c>
       <c r="F52" t="str" xml:space="preserve">
@@ -2268,7 +2268,7 @@
         <v>모든 선생님들 지도해주셔서 감사했습니다 특히 태민선생님 상담 잘해주시고 피드백 잘해주셔서 감사했습니다 찾아뵙고싶었는데 못찾아뵈었네요 죄송합니다 다음에 기회가 된다면 꼭 찾아뵙고싶습니다</v>
       </c>
       <c r="J52" t="str">
-        <v>6등급이었지만 국어 멘토링 덕분에 2,3,4등급은 안정적으로 받을 수 있는 수준으로 발전하였어요.</v>
+        <v>6등급이었지만 국어 멘토링 덕분에 2~4등급은 안정적으로 받을 수 있는 수준으로 발전하였어요.</v>
       </c>
       <c r="K52" t="str">
         <v/>
@@ -2329,7 +2329,7 @@
         <v>요즘 인강과 같이 컨텐츠적으로 부족함이 없다고 생각이 들 정도로 포화 상태라고 생각이 들지만 궁금한 부분을 해결하는것에 있어서 아직은 온라인 강의가 부족하다고 생각이 들었는데 학원 1대1 질의응답 시스템은 단순히 문제를 풀어주시는 것이 아닌 제가 제 질문 과정에 있어서 선생님들이 저의 어떤것들을 잘못 하고 어떤것을 잘했는지 꼼꼼히 설명 해주시고 앞으로의 방향까지 설정해주시니 인강으로만 공부했을때 부족한 부분을 해결해줘서 저는 가장 만족하는 컨텐츠라고 생각합니다</v>
       </c>
       <c r="G54" t="str">
-        <v>오전 오후 하루 두 번 20분 수면 관리는 매우 인상적이였습니다 다른곳은 정해진 시간에 잘 수 있는 시간이 있다고 하는데 이는 사실 효율적이라고 생각하지 않습니다 자기가 정말 필요로 할 때 이용할 수 있는 유연한 제도가 좋았고 면학 분위기 관리에 있어서 실장님도 유연하게 학생들을 관리해주셔서 좋았습니다</v>
+        <v>오전 오후 하루 두 번 20분 수면 관리는 매우 인상적이였습니다 다른곳은 정해진 시간에 잘 수 있는 시간이 있다고 하는데 이는 사실 효율적이라고 생각하지 않습니다 자기가 정말 필요로 할 때 이용할 수 있는 유연한 제도가 좋았고 면학 분위기 관리에 있어서 실장님도 유연하게 학생들을 관리해 주셔서 좋았습니다</v>
       </c>
       <c r="H54" t="str">
         <v>6월 9월 전국 모의고사만으로는 자신의 위치를 확인하기에 어려운 부분이 있었는데 매달 시행했던 사설 모의고사 진행은 좋은 컨텐츠의 문제를 통해 자신의 위치를 확인할 수 있는 좋은 컨텐츠였고 여러번의 모의고사를 통해 수능때 나올 수 있는 여러 상황을 대비하는것에 있어서 굉장히 만족했습니다</v>
@@ -2370,7 +2370,7 @@
         <v>매일 정해진 분량의 단어를 강제적으로 암기하고 테스트하는 시스템 덕분에, 수험 생활에서 가장 소홀해지기 쉬운 어휘력을 탄탄하게 다질 수 있었습니다. 혼자 외울 때는 자칫 뒤로 미루거나 대충 확인하고 넘어가기 쉬운데, 체계적인 테스트를 통해 나의 암기 상태를 객관적으로 점검할 수 있다는 점이 매우 유용했습니다.</v>
       </c>
       <c r="I55" t="str">
-        <v>수험 생활을 하다 보면 불안하고 막막한 순간이 참 많았는데, 그때마다 따뜻한 조언과 현실적인 격려로 제 마음을 다잡아주셔서 큰 힘이 되었습니다. 무심한 듯 툭 던져주시는 응원 한마디가 저에게는 다시 책상 앞에 앉을 수 있는 원동력이 되었습니다.</v>
+        <v>수험 생활을 하다 보면 불안하고 막막한 순간이 참 많았는데, 그때마다 따뜻한 조언과 현실적인 격려로 제 마음을 다잡아 주셔서 큰 힘이 되었습니다. 무심한 듯 툭 던져주시는 응원 한마디가 저에게는 다시 책상 앞에 앉을 수 있는 원동력이 되었습니다.</v>
       </c>
       <c r="J55" t="str">
         <v>체계적인 플래너 관리와 엄격한 생활 관리 덕분에 자습 시간을 더 효율적으로 활용할 수 있었어요.</v>
@@ -2428,7 +2428,7 @@
         <v>N수생</v>
       </c>
       <c r="E57" t="str">
-        <v>매달 담당 선생님이 직접 찾아오셔서 부르셔서 학습 과제 학습 진행 상태 등을 직접 점검해주시고 직접 과목마다 인터넷강의 강사와 교재등을 추천해주시고 가끔 간식같은것도 챙겨주시고 덕담,응원의 말들을 많이 해주셔서 많이 힘이 됐습니다.</v>
+        <v>매달 담당 선생님이 직접 찾아오셔서 부르셔서 학습 과제 학습 진행 상태 등을 직접 점검해주시고 직접 과목마다 인터넷강의 강사와 교재등을 추천해 주시고 가끔 간식같은것도 챙겨주시고 덕담,응원의 말들을 많이 해주셔서 많이 힘이 됐습니다.</v>
       </c>
       <c r="F57" t="str">
         <v>학습 관리를 담당 선생님이 세심하게 해주시고 모의고사 끝날때마다 4층으로 부르셔서 각 과목 담당 선생님이 시험난이도나 등급컷 어려운 문제 해설 등등을 해주셔서 도움이 많이 되었습니다. 그리고 제가 졸거나 집중 못하고있을때 확인하셔서 깨워주시는게 도움되었습니다.</v>
@@ -2526,13 +2526,13 @@
       </c>
       <c r="I59" t="str" xml:space="preserve">
         <v xml:space="preserve">한명한명 학생들에게 친절하게 대해주시고 언제나 필요한 부분이 있다면 최대한 도와주시려는 모습들 모두 감사했습니다_x000d_
-선생님들의 관리가 없었다면 아마 헤이해지는 순간들이 더 많았을거 같습니다_x000d_
+선생님들의 관리가 없었다면 아마 해이해지는 순간들이 더 많았을거 같습니다_x000d_
 선생님들도 아침부터 밤까지 일하시면서 피곤하실때도 있고 쉬고 싶을때도 있을테지만 저희 학생들을 위해서 매일매일 관리해주시는 모습들은 아직 기억이 날 정도로 감사했습니다_x000d_
 수능을 위해 같이 달려온 날들이 결코 짧지 않았고 그만큼 선생님들에게 감사한 마음은 작지 않습니다_x000d_
 앞으로 행복하고 좋은 일만 가득했으면 좋겠습니다!!</v>
       </c>
       <c r="J59" t="str">
-        <v>선생님들의 관리가 없었다면 아마 헤이해지는 순간들이 더 많았을거 같아요.</v>
+        <v>선생님들의 관리가 없었다면 아마 해이해지는 순간들이 더 많았을거 같아요.</v>
       </c>
       <c r="K59" t="str">
         <v/>
@@ -3434,7 +3434,7 @@
         <v>메가스터디와 이투스 패스를 둘다 사용한 저로써 대표적으로 이투스의 국어박광일 강사의 강의가 매우 도움이많이됐고, 다른 타과목의 강사진들 또한 경쟁력있으신분들이 많아서 좋았던것같습니다</v>
       </c>
       <c r="I84" t="str">
-        <v>Tm반 담임 송상윤 선생님 1년 동안 열정과 관심으로 저희 tm반 신경쓰고 관리해주셔서 감사했습니다. 종례때마다 해주시는 덕담과 조언이 재수 생활 많은 도움이 됐던 것 같습니다. 뿐만 아니라 주간,야간,타반 전략 담임 선생님분들 모두 1년 동안 감사했습니다</v>
+        <v>Tm반 담임 송상윤 선생님 1년 동안 열정과 관심으로 저희 tm반 신경쓰고 관리해 주셔서 감사했습니다. 종례때마다 해주시는 덕담과 조언이 재수 생활 많은 도움이 됐던 것 같습니다. 뿐만 아니라 주간,야간,타반 전략 담임 선생님분들 모두 1년 동안 감사했습니다</v>
       </c>
       <c r="J84" t="str">
         <v>종례 때마다 해주시는 덕담과 조언이 재수 생활에 많은 도움이 됐던 것 같아요.</v>
@@ -3825,7 +3825,7 @@
         <v>나머지 3가지 컨텐츠는 진행하지 못하여 이를 선택함 하지만 모의고사를 볼때 시험장 분위기와 실전적 진행을 역설적이게도 적절한 자유도의 조화가 완벽했다는점이 칭찬할만한 범이 아닌가 싶음</v>
       </c>
       <c r="I95" t="str">
-        <v>1년 동안 관리해주셔서 감사합니다 이투스덕분에 많은것을 얻고 가는것 같네요 비록 이번 수능은 실패로 끝났지만 여기서 얻은 경험을 바탕으로 마지막 수험 생활 제대로 끝마치겠습니다 감사합니다</v>
+        <v>1년 동안 관리해 주셔서 감사합니다 이투스덕분에 많은것을 얻고 가는것 같네요 비록 이번 수능은 실패로 끝났지만 여기서 얻은 경험을 바탕으로 마지막 수험 생활 제대로 끝마치겠습니다 감사합니다</v>
       </c>
       <c r="J95" t="str">
         <v>담임 선생님께서 수면 시간 조절하는 방법에 도움을 주셔서 생활 리듬을 바로잡아 공부의 질과 양이 높아졌어요.</v>
@@ -3848,7 +3848,7 @@
         <v>N수생</v>
       </c>
       <c r="E96" t="str">
-        <v>일단 내가 부족한 점을 알게되어서 좋았고 시간을 유용하게 사용할 수 있게되어서 효율적인 학습을 할 수 있었다. 또한 학습환경 학습 분위기 등을 잡아주셔서 도움이 되었다. 그리고 심적인 부분에서 힘들 때마다 상담을 통해 쉽고 편안하게 해결 할 수 있었다</v>
+        <v>일단 내가 부족한 점을 알게되어서 좋았고 시간을 유용하게 사용할 수 있게되어서 효율적인 학습을 할 수 있었다. 또한 학습 환경과 학습 분위기 등을 잡아주셔서 도움이 되었다. 그리고 심적인 부분에서 힘들 때마다 상담을 통해 쉽고 편안하게 해결 할 수 있었다</v>
       </c>
       <c r="F96" t="str">
         <v>내가 계획을 잘 못짜서 항상 공부를 할 때 부족함을 느꼈는데 플래너를 통해 학습량과 공부방향을 정해 공부를 할 수 있어서 능률이 올라갔고 효율적으로 공부할 수 있었다. 그리고 플래너를 통해서 점차 많은 목표를 이루어 갔을 때 성취감을 느껴서 좋았다</v>
@@ -3863,7 +3863,7 @@
         <v>지난 일년동안 지도해주셔서 감사했습니다. 덕분에 수능도 현역때보다 더 잘 보게 되었고 기숙학원에 있는동안 힘든 점도 많았지만 선생님들 덕분에 행복한 기억도 많았던 거 같습니다. 앞으로 인생을 살면서 이런 경험을 할 수 있을지는 모르지만 힘들면서 행복한 한 해가 되었습니다</v>
       </c>
       <c r="J96" t="str">
-        <v>학습환경 학습 분위기 등을 잡아주셔서 도움이 되었어요.</v>
+        <v>학습 환경과 학습 분위기 등을 잡아주셔서 도움이 되었어요.</v>
       </c>
       <c r="K96" t="str">
         <v/>
@@ -3924,7 +3924,7 @@
         <v>재수 학원을 다니는 가장 큰 이유가 꾸준함과 성실함이 부족하면 일관된 생활 패턴과 적절한 학습량을 만들 수 없기 때문인데, 플래너를 통해 스스로 학습 계획을 세우고 적절한 계획인지 확인받아가며 저만의 공부 루틴을 세울 수 있었습니다.</v>
       </c>
       <c r="G98" t="str">
-        <v>학습 중 집중력이 흐트러지거나 피곤해서 깜빡 조는 경우가 종종 있기 마련인데, 주기적으로 선생님들께서 감독하며 집중해 공부할 수 있게 도와주셨습니다. 또한 학습 환경이 적절한지 체크하며 관리해주셔서 편하게 공부할 수 있었습니다.</v>
+        <v>학습 중 집중력이 흐트러지거나 피곤해서 깜빡 조는 경우가 종종 있기 마련인데, 주기적으로 선생님들께서 감독하며 집중해 공부할 수 있게 도와주셨습니다. 또한 학습 환경이 적절한지 체크하며 관리해 주셔서 편하게 공부할 수 있었습니다.</v>
       </c>
       <c r="H98" t="str">
         <v>평소 영어 단어를 따로 암기하는 데 어려움이 있었는데, 매 주 정해진 분량만큼 암기해 테스트를 보게 하는 시스템 덕분에 단어를 꾸준히 암기할 수 있었습니다. 암기가 부족했던 단어도 테스트를 통해 다시 확인할 수 있어 좋았습니다.</v>
@@ -3933,7 +3933,7 @@
         <v>항상 세세한 부분까지 꼼꼼하게 신경써주셔서 편안한 마음가짐으로 열심히 공부에 집중할 수 있었습니다. 선생님들 덕분에 수능 결과도 목표한 대로 잘 받을 있었던 것 같습니다 감사합니다!</v>
       </c>
       <c r="J98" t="str">
-        <v>학습 환경이 적절한지 체크하며 관리해주셔서 편하게 공부할 수 있었어요.</v>
+        <v>학습 환경이 적절한지 체크하며 관리해 주셔서 편하게 공부할 수 있었어요.</v>
       </c>
       <c r="K98" t="str">
         <v/>
@@ -3998,7 +3998,7 @@
       </c>
       <c r="G100" t="str" xml:space="preserve">
         <v xml:space="preserve">몰랐는데 핸드폰 수거하는 거 자체가 되게 공부에 도움이 많이되더라구요_x000d_
-진짜 공부할거면 재수학원 보내는 게 맞는 것 같아요_x000d_
+진짜 공부할거면 재수 학원 보내는 게 맞는 것 같아요_x000d_
 점점 집중력도 올라가고, 실제로 앉아있는 시간도 길어졌어툐</v>
       </c>
       <c r="H100" t="str" xml:space="preserve">
@@ -4037,7 +4037,7 @@
         <v>N수생</v>
       </c>
       <c r="E101" t="str">
-        <v>이투스 247 독학재수학원을 다니며, 국어선생님께 도움을 많이 받았던 것 같습니다. 계속 봐도 이해가 되지 않았던 국어 문제가 있으면 선생님께서 개념부터 찬찬히 알려주셔서 끝으로 제 힘으로 문제를 사고하는 능력을 키워주셨던 것 같습니다!  개인적으로 국어 과외는 별로 선호하지 않는 편이었고, 헷갈리고 이해 안 가는 몇몇 문제들만 누군가 도와주셨으면 좋겠다 하는 입장이었어서 이투스의 코칭 시스템이 맘에 들었습니다.</v>
+        <v>이투스 247 독학재수 학원을 다니며, 국어선생님께 도움을 많이 받았던 것 같습니다. 계속 봐도 이해가 되지 않았던 국어 문제가 있으면 선생님께서 개념부터 찬찬히 알려주셔서 끝으로 제 힘으로 문제를 사고하는 능력을 키워주셨던 것 같습니다!  개인적으로 국어 과외는 별로 선호하지 않는 편이었고, 헷갈리고 이해 안 가는 몇몇 문제들만 누군가 도와주셨으면 좋겠다 하는 입장이었어서 이투스의 코칭 시스템이 맘에 들었습니다.</v>
       </c>
       <c r="F101" t="str">
         <v>앞에서 작성한 바와 같이 국영수 중심의 코칭 시스템이 특히 마음에 들었습니다. 또한 학습 보조 및 관리 측면에서는 제 성적을 누군가 지속적으로 점검해준다는 점에서 항상 긴장감을 유지하며 시험에 임할 수 있어 도움이 되었습니다. 매달 모의고사를 통해 성적을 확인하는 시간을 담임 선생님과 가질 때면 떨리기도 하고, 앞으로 더 열심히 공부해야겠다는 다짐을 할 수 있는 기회가 되었어서 좋았습니다.</v>
@@ -4253,7 +4253,7 @@
         <v>N수생</v>
       </c>
       <c r="E107" t="str">
-        <v>같은 학원에서 좋은 성적을 받고 대학에 입학하신 멘토님께서 제 고민을 같이 고민해주시면서 제 수준에 필요한 좋은 교재도 추천해주시고, 방황할 때 이대로 쭉 해도 좋겠다고 격려해주신 점이 너무 좋았습니다.</v>
+        <v>같은 학원에서 좋은 성적을 받고 대학에 입학하신 멘토님께서 제 고민을 같이 고민해주시면서 제 수준에 필요한 좋은 교재도 추천해 주시고, 방황할 때 이대로 쭉 해도 좋겠다고 격려해주신 점이 너무 좋았습니다.</v>
       </c>
       <c r="F107" t="str">
         <v>다른 친구들은 방심하다가 놓칠 수도 있는 평가원 모의고사나 유명한 사설 모의고사, 학원에서만 받을 수 있는 간쓸개 같은 프로그램을 시즌마다 복도에 붙여 놓치는 일 없도록 도와주신 점이 학습에 차질이 생기지 않게 해주셨다고 생각합니다</v>
@@ -4615,7 +4615,7 @@
         <v>앞서 말했던것 처럼 매주 과목별로 공부량이나 공부 방법등을 피드백 해주시고 과목별 고민이나 모의고사 운영 전략, 시간 관리 등등 실전적인 부분도 도움울 주셨던 점이 많이 도움이 되었던것 같습니다.</v>
       </c>
       <c r="G117" t="str">
-        <v>핸드폰 수거는 재수학원에서 무엇보다 필수적인 요소라고 생각하는데 공부에 방해가 되기때문에 매일 등원할때 마다 제출 할 수 있도록 해서 학습에 방해가 되지않아서 매우 좋았습니다. 점심시간 및 저녁시간에는 사용 가능했고 복귀시 다시 제출해야 했습니다.</v>
+        <v>핸드폰 수거는 재수 학원에서 무엇보다 필수적인 요소라고 생각하는데 공부에 방해가 되기때문에 매일 등원할때 마다 제출 할 수 있도록 해서 학습에 방해가 되지않아서 매우 좋았습니다. 점심시간 및 저녁시간에는 사용 가능했고 복귀시 다시 제출해야 했습니다.</v>
       </c>
       <c r="H117" t="str">
         <v>이투스247 학원을 다니면서 가장 가성비 좋고 효과적으로 학습에 도움을 주었던 것은 무엇보다 매월 구독료를 내고 수강해야했던 이투스 패스를 무료로 제공하여 영빌의 강의를 무료로 수강할 수 있었던 것이 매우 좋았던것 같습니다.</v>
@@ -4910,11 +4910,11 @@
       </c>
       <c r="I125" t="str" xml:space="preserve">
         <v xml:space="preserve">감사했습니다_x000d_
-힘들 때도 많았지만 잘 다잡아주셔서 수험 생활 잘 마무리 한 것 같습니다_x000d_
+힘들 때도 많았지만 잘 다잡아 주셔서 수험 생활 잘 마무리 한 것 같습니다_x000d_
 학습 선생님과 카윤터에 계신 선생님들 모두 정말 감사했습니다 항상 친절하게 대해주시고 잘 잡아주셔서 너무 좋았습니다</v>
       </c>
       <c r="J125" t="str">
-        <v>힘들 때도 많았지만 잘 다잡아주셔서 수험 생활을 잘 마무리한 것 같아요.</v>
+        <v>힘들 때도 많았지만 잘 다잡아 주셔서 수험 생활을 잘 마무리한 것 같아요.</v>
       </c>
       <c r="K125" t="str">
         <v/>
@@ -5092,7 +5092,7 @@
         <v>단어는 스스로 외우려고 해도 채점답안이 저에게 있기 때문에 순전히 저의 양심에만 맡겨야하고, 매일매일 규칙적으로 하기는 어렵습니다. 그런데 그 점을 모두 이투스에서 관리해주어 저는 단어만 외우면 되고, 매일매일 외울 수 있게 되어 좋았습니다. 또 재시도 철저하게 하고 이름을 게시함으로써 스스로 부끄럼을 느껴 더 열심히 하게 되었습니다.</v>
       </c>
       <c r="I130" t="str">
-        <v>추운 겨울방학 내내 따뜻하게 웃으며 맞이해주시고 학습이 지속적으로 이루어질 수 있도록 관리해주셔서 감사합니다! 또 멘토 선생님들 덕분에 많이 배우고 성장할 수 있었어요. 항상 신경 써주시고 도와주셔서 진심으로 감사합니다!</v>
+        <v>추운 겨울방학 내내 따뜻하게 웃으며 맞이해주시고 학습이 지속적으로 이루어질 수 있도록 관리해 주셔서 감사합니다! 또 멘토 선생님들 덕분에 많이 배우고 성장할 수 있었어요. 항상 신경 써주시고 도와주셔서 진심으로 감사합니다!</v>
       </c>
       <c r="J130" t="str">
         <v>상담을 통해 제게 맞는 인강 커리큘럼을 함께 구성하고, 주기적인 플래너 점검으로 학습 방향에 대한 확신을 얻을 수 있었어요.</v>
@@ -5156,7 +5156,7 @@
         <v>힘들고 지칠 때마다 마음을 다잡을 수 있도록 도와주셨던 상담이 정말 큰 힘이 되었습니다. 선생님들께서 해주신 진심 어린 조언과 따뜻한 공감 덕분에 흔들리던 제 자신을 다시 바로 세울 수 있었고, 학습 플래너 관리까지 체계적으로 도와주셔서 공부 방향을 잃지 않고 꾸준히 나아갈 수 있었습니다.</v>
       </c>
       <c r="G132" t="str">
-        <v>힘들고 지칠 때마다 마음을 다잡을 수 있도록 도와주셨던 상담이 정말 큰 힘이 되었습니다. 선생님들께서 해주신 진심 어린 조언과 따뜻한 공감 덕분에 흔들리던 제 자신을 다시 바로 세울 수 있었고, 학습 플래너 관리까지 체계적으로 도와주셔서 공부 방향을 잃지 않고 꾸준히 나아갈 수 있었습니다. 또한 출석 시 휴대폰을 관리해주셔서 불필요한 사용을 줄이고, 공부에 더욱 집중할 수 있는 환경이 만들어진 점도 큰 도움이 되었습니다.</v>
+        <v>힘들고 지칠 때마다 마음을 다잡을 수 있도록 도와주셨던 상담이 정말 큰 힘이 되었습니다. 선생님들께서 해주신 진심 어린 조언과 따뜻한 공감 덕분에 흔들리던 제 자신을 다시 바로 세울 수 있었고, 학습 플래너 관리까지 체계적으로 도와주셔서 공부 방향을 잃지 않고 꾸준히 나아갈 수 있었습니다. 또한 출석 시 휴대폰을 관리해 주셔서 불필요한 사용을 줄이고, 공부에 더욱 집중할 수 있는 환경이 만들어진 점도 큰 도움이 되었습니다.</v>
       </c>
       <c r="H132" t="str">
         <v>이투스 모의고사를 통해 실전과 같은 환경에서 문제를 풀어볼 수 있어 큰 도움이 되었습니다. 다양한 유형의 문제를 경험하며 약점을 파악할 수 있었고, 성적 분석을 통해 부족한 부분을 보완할 수 있었습니다. 꾸준한 모의고사 응시로 시간 관리 능력과 실전 감각을 키울 수 있었던 점이 가장 좋았습니다.</v>
@@ -5165,7 +5165,7 @@
         <v>선생님들께 항상 진심으로 감사드립니다. 힘들고 지칠 때마다 따뜻한 말 한마디와 진심 어린 조언으로 다시 일어설 수 있게 도와주셔서 큰 힘이 되었습니다. 늘 학생 한 명 한 명을 세심하게 챙겨주시고, 끝까지 포기하지 않도록 이끌어주신 덕분에 여기까지 올 수 있었습니다. 앞으로도 이 마음 잊지 않고 더 열심히 하겠습니다. 감사합니다.</v>
       </c>
       <c r="J132" t="str">
-        <v>출석 시 휴대폰을 관리해주셔서 불필요한 사용을 줄이고, 공부에 더욱 집중할 수 있는 환경이 만들어진 점이 큰 도움이 되었어요.</v>
+        <v>출석 시 휴대폰을 관리해 주셔서 불필요한 사용을 줄이고, 공부에 더욱 집중할 수 있는 환경이 만들어진 점이 큰 도움이 되었어요.</v>
       </c>
       <c r="K132" t="str">
         <v/>
@@ -5235,7 +5235,7 @@
         <v>등원할 때, 하원할 때 항상 밝은 얼굴로 인사해주셔서 감사했어요. 짧은 인사지만 덕분에 저도 웃으면서 학원에 들어오고 나올 수 있었어요! 그리고 매번 모의고사 볼 때마다 꼼꼼하게 신경써주셔서 감사합니다.</v>
       </c>
       <c r="J134" t="str">
-        <v>MY 247에서 온라인으로 계획을 작성을 하니까 나의 공부 시간 비중, 패턴을 쉽게 파악할 수 있었어요.</v>
+        <v>MY247에서 온라인으로 계획을 작성을 하니까 나의 공부 시간 비중, 패턴을 쉽게 파악할 수 있었어요.</v>
       </c>
       <c r="K134" t="str">
         <v/>
@@ -5331,7 +5331,7 @@
         <v>어떤 강사의 강의를 듣고, 어떤 유형의 교재를 결정할지는 수능을 준비하는 학생들에게 가장 큰 고민이라는 생각이 드는데, 멘토분께서 저에게 가장 적합한 커리큘럼을 제시해 주셔서  좋았습니다. 특히 지금 상황에서 추천하지 않는 강의를 지적해주셔서 제 계획을 수정하는 데에 도움이 되었습니다.</v>
       </c>
       <c r="G137" t="str">
-        <v>독학재수학원을 다닌 가장 큰 이유였습니다. 혼자서 독서실에 가 공부를 했을 때는 빈번하게 폰을 확인하며 공부에 집중하지 못하고 딴 짓을 하는 경우가 많았는데, 이투스247 학원에서는 등원과 함께 폰을 수거해주셔서 오로지 공부에만 집중할 수 있었습니다.</v>
+        <v>독학재수 학원을 다닌 가장 큰 이유였습니다. 혼자서 독서실에 가 공부를 했을 때는 빈번하게 폰을 확인하며 공부에 집중하지 못하고 딴 짓을 하는 경우가 많았는데, 이투스247 학원에서는 등원과 함께 폰을 수거해주셔서 오로지 공부에만 집중할 수 있었습니다.</v>
       </c>
       <c r="H137" t="str">
         <v>영어가 가장 취약한 과목이었어서 단어 암기가 가장 필요했었는데, 혼자서 단어장을 가지고 외우기엔 규칙적인 학습과 복습을 하지 못했습니다. 이투스247에서는 매일 점심시간 학원의 계획표에 따라 정해진 범위의 단어 테스트를 제공해주셔서, 단어 암기에 정말 큰 도움이 되었습니다.</v>
@@ -5443,7 +5443,7 @@
         <v>1:1로 진행하여 질문을 받아주시는 선생님이 온전히 나에게 집중할 수 있고, 나 또한 모르는 것을 바로바로 해결할 수 있어서 좋았다. 그리고 눈치보지 않고 편하게 질문할 수 있는 것이 장점이 되었고, 선생님께서 중간중간에 문제푸는 팁이나 스킬들을 알려주셔서 좋았다. 그리고 여러 선생님들이 계셔서 나에게 맞는 선생님을 골라 질문할 수 있었다는 것이 큰 장점으로 작용했다</v>
       </c>
       <c r="G140" t="str">
-        <v>재수학원에서 휴대폰을 걷는 제도는 공부 집중력을 높이는 데 큰 도움이 됐다. 평소에는 무의식적으로 SNS나 메신저를 확인하며 시간을 낭비하기 쉬운데, 휴대폰이 없으니 그런 방해 요소가 사라졌다. 그 덕분에 자연스럽게 공부에 몰입하는 시간이 늘었고, 학습 효율도 훨씬 좋아졌다. 또한 다른 학생들도 같은 환경이라 분위기가 흐트러지지 않고, 전체적으로 집중하기 좋은 환경이 만들어졌다는 점도 유용했다.</v>
+        <v>재수 학원에서 휴대폰을 걷는 제도는 공부 집중력을 높이는 데 큰 도움이 됐다. 평소에는 무의식적으로 SNS나 메신저를 확인하며 시간을 낭비하기 쉬운데, 휴대폰이 없으니 그런 방해 요소가 사라졌다. 그 덕분에 자연스럽게 공부에 몰입하는 시간이 늘었고, 학습 효율도 훨씬 좋아졌다. 또한 다른 학생들도 같은 환경이라 분위기가 흐트러지지 않고, 전체적으로 집중하기 좋은 환경이 만들어졌다는 점도 유용했다.</v>
       </c>
       <c r="H140" t="str">
         <v>단어를 외우는 과정은 학습의 기초를 다지는 데 매우 유용했다. 특히 영어 지문을 읽을 때 모르는 단어가 줄어들어 해석 속도가 빨라졌고, 문제 풀이 시간도 단축되었다. 또한 반복적으로 단어를 암기하면서 기억력이 향상되고, 유사한 단어들까지 함께 익힐 수 있어 어휘력이 전반적으로 늘어났다. 이러한 변화는 독해뿐만 아니라 듣기와 쓰기에도 긍정적인 영향을 주었다.</v>
@@ -5484,7 +5484,7 @@
         <v>이투스 모의고사 및 따른 모의고사 일정을 벽에 붙여주셨는데요. 초반에는 강제성을 띄우고 학생들에게 모의고사를 참여하도록하였는데요. 후반에는 초반에 학생들이 참여했던 모의고사를 바탕으로 그 중요성을 깨닫고 많은 학생들이 자발적으로 모의고사를 신청했습니다. 저또한 그부분에서 실전감각을 깨우칠 수 있었던것 같습니다</v>
       </c>
       <c r="I141" t="str">
-        <v>선생님들 안녕하세요 이재용입니다 작년 6월에 학원에 들어가게 되었는데요 짧은 기간동안 신경 많이 써주시고 잘 관리해주셔서 감사합니다. 반수기간을 떠올리면 저는 오히려 재밌었고 추억할만한 시간이였다고 생각이 드네요!!</v>
+        <v>선생님들 안녕하세요 이재용입니다 작년 6월에 학원에 들어가게 되었는데요 짧은 기간동안 신경 많이 써주시고 잘 관리해 주셔서 감사합니다. 반수기간을 떠올리면 저는 오히려 재밌었고 추억할만한 시간이였다고 생각이 드네요!!</v>
       </c>
       <c r="J141" t="str">
         <v>저에게 맞는 좋은 인강들을 추천받을 수 있어서 만족스러웠고, 선생님들의 세심한 관리 덕분에 안정적으로 공부할 수 있었어요.</v>
@@ -5555,10 +5555,10 @@
         <v>인강을 시청하고 매일 문제를 풀어도 불안했었는데 이투스 모의고사를 자주 풀면서 감을 익히고 실전에서 어떻게 행동할지 등을 자꾸만 연습해보고 생각할 수 있어서 너무 좋았다.   모의고사를 풀면서 계속 나만의  루틴을 만들고 계속 적용하면서 실제 수능 현장에서도 너무 당황하지않고 나아갈 수 있었던 것 같다.</v>
       </c>
       <c r="I143" t="str">
-        <v>인사도 제대로 못하고 그만두게 되어 너무 죄송했었어요. 근데 이투스 다니면서 정말 많이 배운것 같아요! 1층에 계신 선생님들, 담임쌤들, 태은쌤,원장쌤까지 이투스 학생들이 잘되길 바라고 사랑하는 따듯한 마음도 항상 느꼈어요!! 이투스 다니면서 만약에 1학년 때 부터 이런 좋은 환경에서 공부했으면 내신 성적도 많이 달라졌을 것 같다고 생각도 했었어요 ㅎㅎ 글고 이투스에서 상담했던 것들, 매주 모의고사 봤던거 , 모의수능 프로그램 등 등 너무 도움이 많이 됐습니다!! 선생님들, 원장님 모두 감사해요!</v>
+        <v>인사도 제대로 못하고 그만두게 되어 너무 죄송했었어요. 근데 이투스 다니면서 정말 많이 배운것 같아요! 1층에 계신 선생님들, 담임쌤들, 태은쌤,원장쌤까지 이투스 학생들이 잘되길 바라고 사랑하는 따뜻한 마음도 항상 느꼈어요!! 이투스 다니면서 만약에 1학년 때 부터 이런 좋은 환경에서 공부했으면 내신 성적도 많이 달라졌을 것 같다고 생각도 했었어요 ㅎㅎ 글고 이투스에서 상담했던 것들, 매주 모의고사 봤던거 , 모의수능 프로그램 등 등 너무 도움이 많이 됐습니다!! 선생님들, 원장님 모두 감사해요!</v>
       </c>
       <c r="J143" t="str">
-        <v>선생님들께서 항상 학생들이 잘되길 바라고, 학생들을 사랑하는 따듯한 마음을 느낄 수 있었어요.</v>
+        <v>선생님들께서 항상 학생들이 잘되길 바라고, 학생들을 사랑하는 따뜻한 마음을 느낄 수 있었어요.</v>
       </c>
       <c r="K143" t="str">
         <v/>
@@ -5767,7 +5767,7 @@
         <v>N수생</v>
       </c>
       <c r="E149" t="str">
-        <v>제가 어떻게 학습을 시작해야 할지 막막했는데 한 가지 방법만 조언해주시는 게 아닌, 과목별로 방향성을 잡아주셔서 저의 기존 방법과 선생님이 조언해주신 방법들이 적절히 섞일 수 있었던 점이 가장 좋았습니다!</v>
+        <v>제가 어떻게 학습을 시작해야 할지 막막했는데 한 가지 방법만 조언해 주시는 게 아닌, 과목별로 방향성을 잡아주셔서 저의 기존 방법과 선생님이 조언해주신 방법들이 적절히 섞일 수 있었던 점이 가장 좋았습니다!</v>
       </c>
       <c r="F149" t="str">
         <v>가장 좋았던 코칭 시스템과 연관된 내용으로 여러 방향 중에서 각각 방향에 맞는 인강이나 교재 혹은 문제 하나하나 마저도 알려주셨던게 가장 도움이 되고, 특히 문제 추천은 제가 부족한 부분을 집중적으로 채울 수 있어서 가장 유용했습니다.</v>
@@ -5922,7 +5922,7 @@
         <v>윈터스쿨때 다니며 저의 공부 습관을 잡을 수 있었던 것 같습니다. 주기적인 학습 관리와 조언을 해주시고, 학습에 방해가 되지 않도록 휴대폰 관리, 학습 관리에 있어서 도와주신 선생님들께 감사합니다.</v>
       </c>
       <c r="J153" t="str">
-        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는 것과 공부하는 것을 관리, 감독해주시는 게 도움이 많이 됐어요.</v>
+        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는 것과 공부하는 것을 관리, 감독해 주시는 게 도움이 많이 됐어요.</v>
       </c>
       <c r="K153" t="str">
         <v/>
@@ -6126,7 +6126,7 @@
         <v>원래 플래너를 적지 않았었는데, 이투스를 다니면서 학습 플래너나 학습 일기를 통해서 본인 스스로 오늘 했던 공부나 보완할 점들을 생각할 수 있었고, 어떤 과목을 앞으로 얼마큼 공부하고, 또 어떻게 공부할지에 관해서 윤곽을 쉽게 잡을 수 있었고, 전반적인 공부의 방향을 정할 수 있어서 좋았습니다.</v>
       </c>
       <c r="G159" t="str">
-        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는 것과 공부하는 것을 관리, 감독해주시는 게 도움이 많이 됐습니다. 또한 혼자 독서실을 가면 핸드폰을 보거나 공부 이외의 딴짓을 자주 하는데 핸드폰을 제출하고 독서실에 들어가고, 지속적으로 감시를 해주시는것이 무척 좋았습니다.</v>
+        <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는 것과 공부하는 것을 관리, 감독해 주시는 게 도움이 많이 됐습니다. 또한 혼자 독서실을 가면 핸드폰을 보거나 공부 이외의 딴짓을 자주 하는데 핸드폰을 제출하고 독서실에 들어가고, 지속적으로 감시를 해주시는것이 무척 좋았습니다.</v>
       </c>
       <c r="H159" t="str">
         <v>결국 수능에서의 실전 감각이 매우 중요하다고 생각하는데 저는 고3현역이여서 학원에서 다 같이 시험을 보지는 못하였지만 담당 선생님이 모의고사를 챙겨주셔서 주말에 모의고사를 풀 수 있었고, 이러한 실전 경험들이 쌓여서 매우 큰 성적 향상을 이뤄낼 수 있었다고 생각합니다. 또한 문제의 퀄리티 역시 매우 뛰어나고, EBS 반영까지 잘 되어 있어서 실전 연습을 하기에 적합하다고 생각합니다.</v>
@@ -6190,7 +6190,7 @@
         <v>N수생</v>
       </c>
       <c r="E161" t="str">
-        <v>현재 내 상황에서 알맞는 강의 및 문제집을 추천해주시는 게 굉장히 맘에 들았습니다. 솔직히 처음 공부를 시작할 때는 뭐부터 해야 할지 감을 잡기 어려웠는데 덕분에 수월하게 진도를 나간 것 같아요</v>
+        <v>현재 내 상황에서 알맞는 강의 및 문제집을 추천해 주시는 게 굉장히 맘에 들았습니다. 솔직히 처음 공부를 시작할 때는 뭐부터 해야 할지 감을 잡기 어려웠는데 덕분에 수월하게 진도를 나간 것 같아요</v>
       </c>
       <c r="F161" t="str">
         <v>제 MBTI가 P성향인지라 계획 세우기를 엄청 어려워 했었는데, 선생님이 플래너 작성과 계획 세우기를 코칭해주시고,적극적으로 조언을 해주셔서 체계적인 학습을 수행하는데 아주 큰 도움이 되었습니다.</v>
@@ -6490,7 +6490,7 @@
 작년에 재수할때 기억이 지금도 계속 생각이 나네요.작년에 다사다난한 일이있었지만 지나고 보니 다 해프닝일 뿐이네요 작년에 보냈던 기억은 계속 생각날것같아요.좋은 추억을 함께 보낼수있어서 감사했습니다.</v>
       </c>
       <c r="J169" t="str">
-        <v>1대1로 선생님께서 상담을 해주시는 게 좋았어요.</v>
+        <v>1대1로 선생님께서 상담을 해 주시는 게 좋았어요.</v>
       </c>
       <c r="K169" t="str">
         <v/>
@@ -6510,7 +6510,7 @@
         <v>N수생</v>
       </c>
       <c r="E170" t="str" xml:space="preserve">
-        <v xml:space="preserve">재수학원을 다니면서 제일 좋았던 건 진짜 학습 상담이었던 것 같아요🥹_x000d_
+        <v xml:space="preserve">재수 학원을 다니면서 제일 좋았던 건 진짜 학습 상담이었던 것 같아요🥹_x000d_
 그냥 성적만 확인하고 끝나는 게 아니라, 제 공부 상태를 같이 진지하게 돌아봐주고 앞으로 어떻게 해야 할지 방향을 잡아주셔서 너무 든든했어요. 혼자 공부할 때는 ‘이게 맞나…?’ 싶을 때가 진짜 많았는데, 상담을 받으면서 “아 내가 잘 가고 있구나” 하는 확신이 생겨서 마음이 훨씬 편해졌습니다✨_x000d_
 특히 좋았던 건 과목별로 부족한 부분을 엄청 구체적으로 짚어주신 거였어요. 그냥 “더 열심히 해라” 이런 게 아니라, 문제를 어떻게 풀어야 하는지, 개념을 어떤 식으로 다시 정리해야 하는지까지 알려주셔서 바로 공부에 적용할 수 있었습니다! 그래서 전보다 훨씬 효율적으로 공부할 수 있었던 것 같아요📚 그리고 상담이 한 번으로 끝나는 게 아니라, 이전에 세운 계획을 계속 체크해 주시고 피드백을 주신 것도 진짜 도움이 많이 됐어요. 잘했을 때는 칭찬해주시고, 부족한 부분은 다시 방향 잡아주셔서 자연스럽게 꾸준히 공부하는 습관도 생겼습니다. 이 과정에서 스스로를 관리하는 힘도 많이 길러졌다고 느꼈어요💪 학원 분위기도 진짜 좋았습니다. 전체적으로 조용하고 집중 잘 되는 환경이라 공부에 몰입하기 너무 좋았고, 주변 친구들도 다 열심히 하는 분위기라 저도 자연스럽게 더 열심히 하게 되더라고요🔥 약간 긴장감 있으면서도 서로 자극되는 느낌…? 그래서 힘들 때도 쉽게 포기하지 않게 잡아주는 분위기였습니다. 선생님들도 단순히 관리만 하는 게 아니라 진짜 학생들 잘되길 바라는 게 느껴져서 더 믿고 따라갈 수 있었던 것 같아요🥺 그래서 학원이 그냥 공부만 하는 곳이 아니라, 같이 성장하는 공간처럼 느껴졌습니다.</v>
       </c>
@@ -6524,7 +6524,7 @@
       </c>
       <c r="G170" t="str" xml:space="preserve">
         <v xml:space="preserve">학습 관리 시스템 중에서도 출석 관리와 생활 관리 부분이 특히 유용하다고 느꼈습니다😊_x000d_
-매일 출석 날짜를 체계적으로 관리해주셔서 스스로 흐트러지지 않고 꾸준히 학원에 나올 수 있었고, 자연스럽게 규칙적인 생활 습관을 유지하는 데 큰 도움이 되었습니다. 혼자였다면 쉽게 느슨해질 수 있었을 텐데, 이러한 관리 덕분에 끝까지 긴장감을 유지할 수 있었습니다._x000d_
+매일 출석 날짜를 체계적으로 관리해 주셔서 스스로 흐트러지지 않고 꾸준히 학원에 나올 수 있었고, 자연스럽게 규칙적인 생활 습관을 유지하는 데 큰 도움이 되었습니다. 혼자였다면 쉽게 느슨해질 수 있었을 텐데, 이러한 관리 덕분에 끝까지 긴장감을 유지할 수 있었습니다._x000d_
 _x000d_
 또한 선생님들께서 학원을 직접 돌아다니시면서 학생들의 학습 상태를 확인해주신 점도 인상 깊었습니다. 공부하다가 졸거나 집중력이 떨어질 때 바로잡아주셔서 다시 흐름을 이어갈 수 있었고, 그 덕분에 공부 시간의 밀도가 훨씬 높아졌다고 느꼈습니다💪_x000d_
 _x000d_
@@ -6579,7 +6579,7 @@
         <v>평소 저를 포함한 모든 학생들이 휴대폰에 빠져 살고 있지만 휴대폰을 수거함으로써 유혹도 제거되고 온전히 공부에만 집중할 수 있게 되었습니다 휴대폰이 없으니 공부도 더 잘 되고 순공 시간도 늘어났습니다! 단순한 억제가 아닌 인내였다고 느꼈습니다</v>
       </c>
       <c r="H171" t="str">
-        <v>이투스에는 훌륭한 인강 강사분들이 계시지만 이투스는 다른 앱과 다르게 구독을 갱신해야한다는 불편함이 있었지만 이투스247독학재수학원을 다니면서 무료로 이투스 인강을 볼 수 있어서 정말 좋았고 구독갱신을 안해도 되어서 너무 편했습니다</v>
+        <v>이투스에는 훌륭한 인강 강사분들이 계시지만 이투스는 다른 앱과 다르게 구독을 갱신해야한다는 불편함이 있었지만 이투스247독학재수 학원을 다니면서 무료로 이투스 인강을 볼 수 있어서 정말 좋았고 구독갱신을 안해도 되어서 너무 편했습니다</v>
       </c>
       <c r="I171" t="str">
         <v>원장님이랑 실장님이랑 경쌤! 25년 한 해 동안 정말 신세 많이 졌습니다 대학가서 재밋게 지내고 있어요! 곧 인사 차 방문드릴게요 ㅎㅎ 제 학습 방향 설정해주셔서 감사했고 멘탈도 케어해주셔서 정말 감사했습니다!</v>
@@ -7250,7 +7250,7 @@
       </c>
       <c r="E190" t="str" xml:space="preserve">
         <v xml:space="preserve">안녕하세요! 저는 작년 6월에 반수를 시작하여 2026 수능을 보고 현재 원하는 학과에 입학하여 즐거운 대학생활 중인 대학생입니다! _x000d_
- 제가 휴학한 후, 가장 먼저 한 일은 학원을 고르는 것이었습니다. 저에게 있어 고등학생 신분을 벗어난 입시생활은 처음이었기 때문에 첫 재수학원을 고르는 것은 매우 중요한 일이었는데요. 여러 후기들과 집 과의 거리, 생활 환경 등을 종목적으로 따진 결과 여기, 이투스 서울강서 지점으로 결정하게 되었습니다!_x000d_
+ 제가 휴학한 후, 가장 먼저 한 일은 학원을 고르는 것이었습니다. 저에게 있어 고등학생 신분을 벗어난 입시생활은 처음이었기 때문에 첫 재수 학원을 고르는 것은 매우 중요한 일이었는데요. 여러 후기들과 집 과의 거리, 생활 환경 등을 종목적으로 따진 결과 여기, 이투스 서울강서 지점으로 결정하게 되었습니다!_x000d_
  이투스 서울강서 지점의 코칭 시스템 증 가장 마음에 들었던 것은 입시 코칭 부분이었는데, 가고 싶은 학과가 명확했던 제게 선생님께선 제 성적으로 갈 수 있는 대학을 객관적인 지표와 현실적인 조언으로 설명해 주셨습니다. 그 말씀을 토대로 학습전략을 설정하고 내 페이스에 맞게 공부하며 결국 원하는 학과에 입학하게 되었습니다. 모의고사를 보며 흔들릴 때 마다 해낼 수 있다는 자신감과 힘을 심어주신 덕분에 이렇게 원하는 대학생활을 할 수 있던게 아닐까 싶습니다!</v>
       </c>
       <c r="F190" t="str" xml:space="preserve">
@@ -7346,7 +7346,7 @@
         <v>단어량이 자동으로 많이 늘어서 영어 등급 향상에 많은 도움이 되었던 것 같습니다. 저는 강제성이 없이 자발적으로 공부하는 편이었어서 단어가 항상 뒤로 밀렸는데 억지로라도 계속 테스트를 보니까 어휘력이 늘어서 등급이 두달만에 3등급 상승했습니다.</v>
       </c>
       <c r="I192" t="str">
-        <v>제 고3시절 중 가장 행복했던 시간은 이투스에서 였습니다.. 항상 학원 갈 때 올 때 수고한다고 말해주시고 등하교 찍을 때도 힘들지~ 이런 말 해주시는 게 항상 힘이 되었습니다. 집중도 가장 잘 되었고 환경도 너무 쾌적해서 저는 인생에서 이투스에 있을 때 공부를 제일 효율적으로, 또 많이 했습니다. 선생님들의 많은 격려와 칭찬이 저를 동기부여 했던 것 같습니다. 지금도 이투스를 생각하면 기분이 좋습니다. 이투스 아니었으면 저 대학 못갔습니다 감사합니다~</v>
+        <v>제 고3시절 중 가장 행복했던 시간은 이투스에서 였습니다.. 항상 학원 갈 때 올 때 수고한다고 말해주시고 등하교 찍을 때도 힘들지~ 이런 말 해 주시는 게 항상 힘이 되었습니다. 집중도 가장 잘 되었고 환경도 너무 쾌적해서 저는 인생에서 이투스에 있을 때 공부를 제일 효율적으로, 또 많이 했습니다. 선생님들의 많은 격려와 칭찬이 저를 동기부여 했던 것 같습니다. 지금도 이투스를 생각하면 기분이 좋습니다. 이투스 아니었으면 저 대학 못갔습니다 감사합니다~</v>
       </c>
       <c r="J192" t="str">
         <v>고민 상담, 멘탈 관리, 공부 팁 등도 자주 알려주셔서 큰 도움이 되었어요.</v>
@@ -7410,7 +7410,7 @@
         <v>평소에는 계획을 잘 세우지 않는편이라 공부할 때 방향성을 잡기 쉽지 않았는데 매일 내가 한 학습량과 앞으로 해야 할 것들을 정리하면서 하루하루 성취감도 생기고 공부 계획을 철저하게 세울 수 있어 도움이 되었다.</v>
       </c>
       <c r="G194" t="str">
-        <v>한 자리에서 계속 공부를 하면 지치거나 졸릴때도 있어 체력적으로 힘든데 학습 분위기를 조교 선생님들이 관리해주셔서 더 편안했다. 집중을 잘 할 수 있는 분위기를 만들어주셔서 믿고 온전히 공부에만 집중할 수 있었다.</v>
+        <v>한 자리에서 계속 공부를 하면 지치거나 졸릴때도 있어 체력적으로 힘든데 학습 분위기를 조교 선생님들이 관리해 주셔서 더 편안했다. 집중을 잘 할 수 있는 분위기를 만들어주셔서 믿고 온전히 공부에만 집중할 수 있었다.</v>
       </c>
       <c r="H194" t="str">
         <v>수능 입시를 준비하다보면 평가원 모의고사 뿐만이 아니라 많은 사설 모의고사들도 풀어보며 시험 볼 때의 태도를 많이 연습할 수 있는데 이투스 모의고사를 의무로 봄으로써 학원에서 강제적으로라도 나의 시험 태도를 확인할 수 있어서 좋았다.</v>
@@ -7668,7 +7668,7 @@
         <v>계획이 저처럼 있는 학생은 이 계획을 잘 지켰는지 검사를 함으로서 나태해지는 길로 가는 걸 막아주셔서 좋았던 거 같습니다. 감시가 있는 덕분에 스스로와의 타협은 버리고 공부로의 정진을 택해 좋은 결과가 이렇게 나오게 된 거 같아 기분이 좋았습니다.</v>
       </c>
       <c r="G201" t="str">
-        <v>혼자서 반수를 하게 되면 안 그래도 고3 때의 시절과 달리 대학을 다니다 수능을 다시 치르는 거라 그 수험생 때의 생활 패턴으로 돌아가기가 힘들텐데 이 독학재수학원에 다니면서 생활 패턴을 어느정도 관리할 수 있던 점이 상당히 좋았던 거 같습니다.</v>
+        <v>혼자서 반수를 하게 되면 안 그래도 고3 때의 시절과 달리 대학을 다니다 수능을 다시 치르는 거라 그 수험생 때의 생활 패턴으로 돌아가기가 힘들텐데 이 독학재수 학원에 다니면서 생활 패턴을 어느정도 관리할 수 있던 점이 상당히 좋았던 거 같습니다.</v>
       </c>
       <c r="H201" t="str">
         <v>평가원 기출 문제나 교육청 같은 문제도 중요하지만 요즘엔 안 그래도 사설 컨텐츠의 퀄이 상당히 좋습니다. 그렇기 때문에 이러한 점에서 이득을 볼 수 있게 해주어 다양한 유형의 문제를 풀 수 있어 좋았던 거 같습니다.</v>
@@ -7707,13 +7707,13 @@
         <v>혼자서는 꾸준히 규칙적으로 계속 공부하는걸 이어나가는게 힘든데 학습 관리 시스템 덕분에 도움을 많이 받았습니다 세세한 부분까지 관리받을 수 있어서 딴생각 안하고 공부만 잘 할수 있었던거같아요</v>
       </c>
       <c r="G202" t="str">
-        <v>선생님이 직접 돌아다니면서 관리해주셔서 좋았어요 무작정 깨우지도 않고 너무 힘들 때는 어느정도 잘수 있게도 해주셔서 감사햇습니다 자주 돌아다니면서 면학 분위기 관리를 해주셔서 분위기 안좋았던 적이 거의 없었던거같아요 방해 안돼서 좋았습미다</v>
+        <v>선생님이 직접 돌아다니면서 관리해 주셔서 좋았어요 무작정 깨우지도 않고 너무 힘들 때는 어느정도 잘수 있게도 해주셔서 감사햇습니다 자주 돌아다니면서 면학 분위기 관리를 해주셔서 분위기 안좋았던 적이 거의 없었던거같아요 방해 안돼서 좋았습미다</v>
       </c>
       <c r="H202" t="str">
         <v>이투스 구독을 무료로 할 수 있어서 구독 갱신 같은 거 신경 안쓰고 학습 효율을 크게 높일수있었습니다! 이투스 안에 다양한 강의가 있어서 듣고싶은 거 제약없이 다 들을 수 있어서 좋았어요 무엇보다!!! 학원비에 구독비를 추가로 낼 필요가 없으니까 별도의 비용 부담 없이 이투스 강의를 들을수 있어서 경제적인 측면에서도 매우 좋앗습니다 ㅎㅎ</v>
       </c>
       <c r="I202" t="str">
-        <v>이투스에서 항상 저를 위해 신경써주셧던 선생님들께 진심으로 감사드립니다 !! 힘들고 지칠 때마다 따뜻한 말도 해주시고 현실적인 말도 해주셔서 다시 마음을 다잡고 할수있었어요 늘 묵묵히 응원도 해주시고 세심하게 관리해주셔서 큰 힘이 되었습니다! 덕분에 학원에서 열심히 공부할 수있었어요</v>
+        <v>이투스에서 항상 저를 위해 신경써주셧던 선생님들께 진심으로 감사드립니다 !! 힘들고 지칠 때마다 따뜻한 말도 해주시고 현실적인 말도 해주셔서 다시 마음을 다잡고 할수있었어요 늘 묵묵히 응원도 해주시고 세심하게 관리해 주셔서 큰 힘이 되었습니다! 덕분에 학원에서 열심히 공부할 수있었어요</v>
       </c>
       <c r="J202" t="str">
         <v>매번 학습일지를 작성하고 주기적인 피드백을 받으며 공부 계획을 잡아 원동력을 잃지 않고 공부할 수 있었어요.</v>
@@ -7890,13 +7890,13 @@
         <v>무엇보다 부담 없이 과목별 선생님과 상담할 수 있는 것이 마음에 들었습니다. 인강을 들으면서 학습을 하다 보니 모르거나 궁금한 것이 있을때 바로 의견•조언을 얻기가 힘들어서 고민이었는데, 그럴때마다 바로바로 질문을 드리고 해답을 얻을 수 있는 것이 큰 도움이 되었습니다.</v>
       </c>
       <c r="G207" t="str">
-        <v>재수학원의 생활 관리 시스템은 규칙적인 생활 습관을 형성하는 데 큰 도움이 되었습니다. 정해진 시간표에 따라 공부와 휴식을 반복하면서 집중력이 높아졌고, 학습 계획을 체계적으로 유지할 수 있어 학업 효율도 자연스럽게 향상되었습니다.</v>
+        <v>재수 학원의 생활 관리 시스템은 규칙적인 생활 습관을 형성하는 데 큰 도움이 되었습니다. 정해진 시간표에 따라 공부와 휴식을 반복하면서 집중력이 높아졌고, 학습 계획을 체계적으로 유지할 수 있어 학업 효율도 자연스럽게 향상되었습니다.</v>
       </c>
       <c r="H207" t="str">
         <v>여러 단어들을 자주 시험치게 되니 어떤 단어를 내가 모르고, 헷갈리는 것이 무엇인지 주기적으로 체크하고 보완할 수 있었습니다. 이 덕분에 영단어 실력이 크게 상승되고 유지할 수 있었습니다.</v>
       </c>
       <c r="I207" t="str">
-        <v>재원하는 동안 항상 친절하게 관리해주셔서 정말 감사했습니다. 덕분에 힘든 수험 생활을 그나마 재밌고 쾌적하게 할 수 있었습니다! 항상 파이팅하시고 좋은 일들만 있으시길 기원합니다😊</v>
+        <v>재원하는 동안 항상 친절하게 관리해 주셔서 정말 감사했습니다. 덕분에 힘든 수험 생활을 그나마 재밌고 쾌적하게 할 수 있었습니다! 항상 파이팅하시고 좋은 일들만 있으시길 기원합니다😊</v>
       </c>
       <c r="J207" t="str">
         <v>제 수준에 맞는 강의와 커리큘럼을 추천받고, 질의응답을 통해 못 푼 문제를 다시 풀어보며 부족한 부분을 채울 수 있었어요.</v>
@@ -7919,7 +7919,7 @@
         <v>N수생</v>
       </c>
       <c r="E208" t="str">
-        <v>1대1로 선생님께서 상담을 해주시는 게 좋았습니다. 담당하는 학생이 많았지만 상담할때 어떤 방향으로 원서접수를 해야 좋을지, 나에게 맞는 학습 방법과 진도를 하나부터 열까지 도와주셨습니다. 이것은 관리형독서실이나 스카에서는 없는 이투스에서만 경험 가능한 시스템이라 좋았습니다</v>
+        <v>1대1로 선생님께서 상담을 해 주시는 게 좋았습니다. 담당하는 학생이 많았지만 상담할때 어떤 방향으로 원서접수를 해야 좋을지, 나에게 맞는 학습 방법과 진도를 하나부터 열까지 도와주셨습니다. 이것은 관리형독서실이나 스카에서는 없는 이투스에서만 경험 가능한 시스템이라 좋았습니다</v>
       </c>
       <c r="F208" t="str">
         <v>질문을 원하는 학생이 많아 질문이 있을때 바로 질문 신청을 하고 몇시간 혹은 며칠을 기다리면 질의응답을 받을 수 있었습니다. 그래도 담당 과목 선생님을 직접 고를 수 있으며 이해가 갈 때까지 차근차근 설명해주셨습니다. 덕분에 정말 어려웠던 과목을 수능에서 좋은 성적을 받을 수 있었습니다. 또한 같은 선생님께 질문을 계속하다보면 어느정도의 유대감이 쌓이고 질문 하는 것이 정말 편해지고 이해도 더 잘되는 것 같았습니다.</v>
@@ -7960,7 +7960,7 @@
         <v>평소 계획을 세우고 공부하지 않고 그때그때 하고싶은 공부를 하여 공부 비중이 고르지않았다. 근데 주단위로 하루에 무엇을 얼만큼 공부할지 계획을 같이 세우고 피드백해주셔서 고르게 공부할 수 있었다.</v>
       </c>
       <c r="G209" t="str">
-        <v>잠이 많은 편이라 공부할 때 많이 졸았는데 학습 코칭 선생님께서 졸음 관리를 확실하게 지도해주셔서 많은 도움이 되었다. 졸릴 때는 자리에서 벗어나 밖에 서서 공부하라고 해주시는 게 도움됐다.</v>
+        <v>잠이 많은 편이라 공부할 때 많이 졸았는데 학습 코칭 선생님께서 졸음 관리를 확실하게 지도해주셔서 많은 도움이 되었다. 졸릴 때는 자리에서 벗어나 밖에 서서 공부하라고 해 주시는 게 도움됐다.</v>
       </c>
       <c r="H209" t="str">
         <v>실전처럼 모의고사를 볼 수 있는 환경이 마련되어 있어 실제 시험을 대비하는 데 큰 도움이 되었다. 시험 분위기를 미리 경험할 수 있어서 긴장감 조절에도 좋았고 문제 풀이 감각을 익히는 데 유익했다. 그리고 콘텐츠를 신청할 수 있는 방식이 가까워서 번거롭지 않고 편리하게 이용할 수 있었던 점도 좋았다.</v>
@@ -8247,7 +8247,7 @@
         <v>이투스247을 다니기 전까지는 모의고사가 도대체 무슨 효과가 있냐는 생각을 하였다 특히 사설 모의고사는 더,실제로도 초반에는 모의고사를 보고나서는 내 등급을 확인하고 스트레스만 쌓일 뿐이였다 하지만 어느날 모의고사를 보고나서 틀린점들을 분석하면서 복습을 하고 부족했던점들을 다음 모의고사때 적용하고 나서 처음으로 수능 사설 모의고사에서 8등급을 벗어나며 그때부터 실력이 조금씩 상승했기에 이 점이 유용하다 생각한다</v>
       </c>
       <c r="I217" t="str">
-        <v>당시에 재수학원등은 그냥 폰뺐고 돈만 많이 드는 일반 스터디카페라는 인식이 박혀있었는데 직접 다녀보면서 성적은 물론이고 생활 습관이 굉장히 많이 개선이 되며 다니던 예체능 실기에서도 도움이 많이 되었습니다 감사합니다</v>
+        <v>당시에 재수 학원등은 그냥 폰뺐고 돈만 많이 드는 일반 스터디카페라는 인식이 박혀있었는데 직접 다녀보면서 성적은 물론이고 생활 습관이 굉장히 많이 개선이 되며 다니던 예체능 실기에서도 도움이 많이 되었습니다 감사합니다</v>
       </c>
       <c r="J217" t="str">
         <v>최적의 학습 환경과 선생님의 세심한 관리로 끝까지 집중하며 긍정적인 변화와 함께 재수 성공을 이뤄내어 뿌듯해요.</v>
@@ -8447,7 +8447,7 @@
         <v>N수생</v>
       </c>
       <c r="E223" t="str">
-        <v>이투스 독학재수학원의 생활상담시스템은 학습뿐 아니라 생활 전반을 관리해준다는 점에서 매우 유용했습니다. 규칙적인 출결 관리와 학습 계획 점검을 통해 스스로 나태해지지 않도록 도와주었고, 상담을 통해 스트레스나 슬럼프를 조기에 해소할 수 있었습니다. 또한 개인 상황에 맞춘 피드백을 제공해 학습 효율을 높이는 데 큰 도움이 되었습니다.</v>
+        <v>이투스 독학재수 학원의 생활상담시스템은 학습뿐 아니라 생활 전반을 관리해준다는 점에서 매우 유용했습니다. 규칙적인 출결 관리와 학습 계획 점검을 통해 스스로 나태해지지 않도록 도와주었고, 상담을 통해 스트레스나 슬럼프를 조기에 해소할 수 있었습니다. 또한 개인 상황에 맞춘 피드백을 제공해 학습 효율을 높이는 데 큰 도움이 되었습니다.</v>
       </c>
       <c r="F223" t="str">
         <v>이투스의 일대일 학습 관리 시스템은 모르는 과목이나 문제를 바로 질문하고 해결할 수 있다는 점에서 매우 유용했습니다. 혼자 공부할 때 생길 수 있는 개념 공백을 즉시 메울 수 있었고, 이해가 부족한 부분을 개인 수준에 맞게 설명받아 학습 효율이 높아졌습니다. 또한 반복적인 피드백을 통해 약점을 빠르게 보완할 수 있어 성적 향상에 큰 도움이 되었습니다.</v>
@@ -8703,7 +8703,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E230" t="str">
-        <v>자주 학습 상태를 체크해 주시고 상담도 여러번이 있어서 좋았습니다. 그리고 매주마다 수학과 국어 테스트를 보고 수학은 해설까지 해주시는 게 정말 도움 많이 된 것 같습니다. 주마다 하는 테스트 덕분에 더 열심히 공부한 것 같습니다.</v>
+        <v>자주 학습 상태를 체크해 주시고 상담도 여러번이 있어서 좋았습니다. 그리고 매주마다 수학과 국어 테스트를 보고 수학은 해설까지 해 주시는 게 정말 도움 많이 된 것 같습니다. 주마다 하는 테스트 덕분에 더 열심히 공부한 것 같습니다.</v>
       </c>
       <c r="F230" t="str">
         <v>제가 원래 꼼꼼하게 계획을 세워서 공부하는 스타일이 아니라 그때 그때 하고 싶은 과목만 공부를 쭉 하다가 또 다른 과목이 하고 싶으면 그 과목만 해서 공부 시간의 격차가 너무 심했었는데 플래너를 작성하면서 그날 무슨 공부를 할지 고민하지 않았던게 좋았습니다</v>
@@ -8846,7 +8846,7 @@
         <v>가장 좋았던 건 물어보고 싶을 때 언제든지 물어볼 수 있는 것이었습니다. 항상 멘토, 선생님들이 상주해계시고 할때마다 친절하고 자세히 알려주셔서 정말 좋았습니다. 또 한분한분 진심으로 알게해주려고 하셔서 감사했습니다. 단순한 문재풀이 뿐만 아니라 접근방법도 상세히 알려주십니다.</v>
       </c>
       <c r="F234" t="str">
-        <v>독학재수학원이기 때문에 자기관리가 힘들 수 있습니다. 하지만 과목별로 주기적인 상담을 통해 본인 진도에 맞춰서 알맞은 계획을 세워주십니다. 저는 학습 계획을 세우는 것에 있어서 어려움을 느꼈는데 학습 관리 시스템 덕분에 계획 짜는 법에 도움을 많이 받았습니다.</v>
+        <v>독학재수 학원이기 때문에 자기관리가 힘들 수 있습니다. 하지만 과목별로 주기적인 상담을 통해 본인 진도에 맞춰서 알맞은 계획을 세워주십니다. 저는 학습 계획을 세우는 것에 있어서 어려움을 느꼈는데 학습 관리 시스템 덕분에 계획 짜는 법에 도움을 많이 받았습니다.</v>
       </c>
       <c r="G234" t="str">
         <v>수험 생활 중 굉장히 힘든 점 중 하나가 스마트폰 관리라고 생각합니다. 이투스 247에서는 강제적으로라도 휴대폰을 수거해서 처음에는 조금 힘들 수 있지만 결국에는 많은 도움을 받았던 것 같습니다.</v>
@@ -8878,12 +8878,12 @@
         <v>N수생</v>
       </c>
       <c r="E235" t="str" xml:space="preserve">
-        <v xml:space="preserve">이투스 독학재수학원을 다니면서 가장 크게 만족했던 부분은 ‘학습 코칭’이었습니다. 혼자 공부하는 시간이 많은 독재 학원의 특성상 방향을 잡는 것이 중요한데, 이곳의 학습 코칭은 그 부분을 확실하게 채워주었습니다._x000d_
+        <v xml:space="preserve">이투스 독학재수 학원을 다니면서 가장 크게 만족했던 부분은 ‘학습 코칭’이었습니다. 혼자 공부하는 시간이 많은 독재 학원의 특성상 방향을 잡는 것이 중요한데, 이곳의 학습 코칭은 그 부분을 확실하게 채워주었습니다._x000d_
 공부를 하다가 막히는 개념이나 문제가 생겼을 때 단순히 답만 알려주는 것이 아니라, 이해가 될 때까지 자세하게 설명해주고 비슷한 유형의 문제를 추가로 제공해주셨습니다. 덕분에 한 번 헷갈렸던 부분을 제대로 정리하고 넘어갈 수 있었고, 같은 유형의 문제에 대한 자신감도 자연스럽게 생겼습니다. 또한 학습 코칭을 통해 제 공부 상태를 객관적으로 점검할 수 있었던 점도 매우 좋았습니다. 혼자 공부하다 보면 내가 잘하고 있는지, 방향이 맞는지 불안해질 때가 많은데, 코칭을 통해 부족한 부분을 정확히 짚어주고 보완할 수 있어서 훨씬 효율적으로 공부할 수 있었습니다._x000d_
 단순히 질문을 받아주는 수준을 넘어서, 학습의 방향성과 문제 해결 능력을 함께 키워준다는 점에서 이투스 독재의 학습 코칭은 큰 장점이라고 생각합니다. 혼자서는 채우기 어려운 부분을 확실하게 보완해준 덕분에 끝까지 흔들리지 않고 공부를 이어갈 수 있었습니다. 실제로 많은 성적 향상을 이루었고 제가 만족할 수 있는 대학교에 오게 되었습니다.</v>
       </c>
       <c r="F235" t="str" xml:space="preserve">
-        <v xml:space="preserve">이투스 독학재수학원을 다니면서 좋았던 점 중 하나는 인강이나 교재 추천 시스템이 정말 체계적이었다는 점입니다. 저는 검정고시를 보고 수능을 준비한 케이스라서, 어떤 교재를 써야 하는지, 어떤 인강을 들어야 하는지에 대한 기준이 거의 없는 상태였습니다. 혼자였다면 수준에 맞지 않는 교재를 선택하거나, 방향 없이 이것저것 건드리다가 시간만 낭비했을 가능성이 컸다고 생각합니다. 그런데 학습 코칭을 통해 현재 제 실력에 맞는 교재와 인강을 추천해 주셔서 공부 방향을 잡는 데 큰 도움이 되었습니다. 특히 단순히 유명한 교재를 추천하는 것이 아니라, 제 수준에 맞는 단계별 교재를 골라주셨던 점이 인상적이었습니다. 실제로 학습에서는 자신의 수준에 맞는 교재 선택이 굉장히 중요한데, 난이도가 맞지 않으면 학습 효율이 떨어질 수 있다는 점에서도 이런 추천이 큰 도움이 되었습니다. _x000d_
+        <v xml:space="preserve">이투스 독학재수 학원을 다니면서 좋았던 점 중 하나는 인강이나 교재 추천 시스템이 정말 체계적이었다는 점입니다. 저는 검정고시를 보고 수능을 준비한 케이스라서, 어떤 교재를 써야 하는지, 어떤 인강을 들어야 하는지에 대한 기준이 거의 없는 상태였습니다. 혼자였다면 수준에 맞지 않는 교재를 선택하거나, 방향 없이 이것저것 건드리다가 시간만 낭비했을 가능성이 컸다고 생각합니다. 그런데 학습 코칭을 통해 현재 제 실력에 맞는 교재와 인강을 추천해 주셔서 공부 방향을 잡는 데 큰 도움이 되었습니다. 특히 단순히 유명한 교재를 추천하는 것이 아니라, 제 수준에 맞는 단계별 교재를 골라주셨던 점이 인상적이었습니다. 실제로 학습에서는 자신의 수준에 맞는 교재 선택이 굉장히 중요한데, 난이도가 맞지 않으면 학습 효율이 떨어질 수 있다는 점에서도 이런 추천이 큰 도움이 되었습니다. _x000d_
 또한 교재와 인강이 서로 연계되도록 추천해 주셔서, 개념 이해 → 문제 적용 → 복습까지 자연스럽게 이어지는 학습 흐름을 만들 수 있었습니다. 덕분에 막연하게 공부하는 느낌이 아니라, 체계적으로 실력이 쌓여가는 느낌을 받을 수 있었습니다._x000d_
 특히 저처럼 기초가 부족한 상태에서 시작한 경우에는 무엇을 먼저 해야 할지 몰라서 방황하기 쉬운데, 이런 부분을 잡아주고 학습 로드맵을 제시해준 점이 가장 큰 장점이라고 느꼈습니다. 혼자 했다면 절대 만들기 어려웠을 공부 방향을 잡아줬다는 점에서 매우 만족스러웠습니다.</v>
       </c>
@@ -9289,7 +9289,7 @@
         <v>1:1 질의응답은 내가 이해하지 못한 부분을 바로 질문하고 해결할 수 있어 매우 유용했다. 수업에서는 놓치기 쉬운 세부 내용까지 자세히 설명을 들을 수 있었고, 나의 수준에 맞춘 설명 덕분에 이해도가 훨씬 높아졌다. 또한 즉각적인 피드백을 통해 잘못 알고 있던 개념을 바로잡을 수 있어 학습의 정확성과 효율성을 높이는 데 큰 도움이 되었다. 부담 없이 질문할 수 있어 학습에 큰 도움이 되었다.</v>
       </c>
       <c r="G246" t="str">
-        <v>면학 분위기 속에서 감독이 이루어지니 자연스럽게 집중력이 높아지고 공부에 몰입할 수 있어 좋았다. 주변 모두가 학습에 집중하는 환경이라 흐트러지기 어려웠고, 감독이 있어 긴장감과 책임감도 생겨 스스로를 더 잘 통제할 수 있었다. 그 결과 불필요한 시간 낭비가 줄고 학습 효율이 크게 향상되었다. 또한 식사 후 식곤증에 빠지지 않게 관리해주시는 게 큰 도움이 되었다.</v>
+        <v>면학 분위기 속에서 감독이 이루어지니 자연스럽게 집중력이 높아지고 공부에 몰입할 수 있어 좋았다. 주변 모두가 학습에 집중하는 환경이라 흐트러지기 어려웠고, 감독이 있어 긴장감과 책임감도 생겨 스스로를 더 잘 통제할 수 있었다. 그 결과 불필요한 시간 낭비가 줄고 학습 효율이 크게 향상되었다. 또한 식사 후 식곤증에 빠지지 않게 관리해 주시는 게 큰 도움이 되었다.</v>
       </c>
       <c r="H246" t="str">
         <v>이투스 구독 시스템은 다양한 강의를 한 번에 자유롭게 이용할 수 있어 매우 효율적이었다. 과목별로 필요한 강의를 추가 비용 부담 없이 선택해 들을 수 있어 학습 범위를 넓히는 데 도움이 되었고, 자신의 수준과 목표에 맞게 강의를 유연하게 조합할 수 있었다. 또한 반복 수강이 가능해 부족한 부분을 여러 번 복습하며 이해도를 높일 수 있어 학습 효과를 극대화할 수 있었다. 내가 원하는 부분만 듣고 싶었는데 비용 부담 없이 여러 강의를 들을 수 있어서 좋았다.</v>
@@ -9365,7 +9365,7 @@
         <v>인강사이트를 결제하는데에 꽤 부담이 되는 금액이 필요한데, 이투스를 사용할 수 있어 좋았다. 나는 타 인강사이트 하나와 이투스를 사용해 독학재수 내내 공부했다. 가끔 나눠주신 이투스 인강강사의 교재도 도움이 되었다.</v>
       </c>
       <c r="I248" t="str">
-        <v>학원의 면학 분위기와 따듯한 관심 덕분에 이투스에서 두번째 수능을 마무리할 수 있었습니다. 재원기간동안 매주 상담을 해주신 담임 선생님, 아침마다 인사해주시던 선생님들, 졸 때마다 깨워주신 선생님 감사합니다.</v>
+        <v>학원의 면학 분위기와 따뜻한 관심 덕분에 이투스에서 두번째 수능을 마무리할 수 있었습니다. 재원기간동안 매주 상담을 해주신 담임 선생님, 아침마다 인사해주시던 선생님들, 졸 때마다 깨워주신 선생님 감사합니다.</v>
       </c>
       <c r="J248" t="str">
         <v>조용하고 긴장감 있는 분위기 속에서 졸음 관리까지 확실히 받아, 장시간 안정적인 페이스로 공부에 온전히 집중할 수 있었어요.</v>
@@ -9528,7 +9528,7 @@
         <v>반수생</v>
       </c>
       <c r="E253" t="str" xml:space="preserve">
-        <v xml:space="preserve">재수학원에서 진행된 학습 상담은 단순히 공부 방법을 듣는 것을 넘어서, 제 공부 습관과 문제점을 객관적으로 돌아볼 수 있는 계기가 되었습니다. 특히 스스로는 잘 인지하지 못했던 시간 관리의 비효율성과 과목별 학습 편차를 구체적으로 짚어주어 학습 방향을 다시 설정하는 데 큰 도움이 되었습니다._x000d_
+        <v xml:space="preserve">재수 학원에서 진행된 학습 상담은 단순히 공부 방법을 듣는 것을 넘어서, 제 공부 습관과 문제점을 객관적으로 돌아볼 수 있는 계기가 되었습니다. 특히 스스로는 잘 인지하지 못했던 시간 관리의 비효율성과 과목별 학습 편차를 구체적으로 짚어주어 학습 방향을 다시 설정하는 데 큰 도움이 되었습니다._x000d_
 또한 상담을 통해 과목별로 자주 틀리는 문제 유형을 분석하고, 이에 맞는 보완 방법을 제시받을 수 있었습니다. 예를 들어 오답노트 정리 방식이나 문제 풀이 순서를 조정하는 방법 등을 적용하면서, 단순히 문제를 많이 푸는 것이 아니라 틀린 이유를 이해하는 데 집중하게 되었습니다. 그 결과 학습의 효율이 높아졌다고 느꼈습니다._x000d_
 더불어 멘탈 관리 측면에서도 많은 도움이 되었습니다. 재수 과정에서 생기는 불안감이나 슬럼프에 대해 현실적인 조언을 들을 수 있었고, 이를 바탕으로 꾸준히 공부를 이어갈 수 있는 루틴을 만들 수 있었습니다._x000d_
 이처럼 학습 상담은 제게 맞는 공부 방법을 찾고 이를 지속할 수 있도록 도와준 중요한 경험이었다고 생각합니다.</v>
@@ -9687,7 +9687,7 @@
         <v>공부를 시작할 때 어떤 걸 해야 할지 모르겠는 막막함과 두려움이 있었습니다. 하지만 이투스 코칭 시스템을 통해 올바른 방향으로 공부를 할 수 있어서 심리적으로 안정감도 들고 도움이 많이 되었습니다.</v>
       </c>
       <c r="F257" t="str">
-        <v>인강 콘텐츠들이 넘쳐나는 요즘 시대에서 나한테 맞고 좋은 선생님들 찾는데 시간이 많이 걸리고 지치는 일이 많았습니다. 하지만 이투스학원에서 추천해주시고 알려주시는 덕분에 스트레스 받는 일도 덜 했고 효과적이었습니다.</v>
+        <v>인강 콘텐츠들이 넘쳐나는 요즘 시대에서 나한테 맞고 좋은 선생님들 찾는데 시간이 많이 걸리고 지치는 일이 많았습니다. 하지만 이투스학원에서 추천해 주시고 알려주시는 덕분에 스트레스 받는 일도 덜 했고 효과적이었습니다.</v>
       </c>
       <c r="G257" t="str">
         <v>카드로 찍는 출결 시스템 덕분에 부모님께 문자가 자동으로 가서  걱정을 덜어드리는데 도움이 많이 되었습니다. 또한 기계로 하기 때문에 실수가 적어 체계적이여서 너무너무 좋았습니다.</v>
@@ -9804,7 +9804,7 @@
         <v>감사했습니다 덕분에 좋은 대학생활 즐기고있어요 힘든일도이ㅛ았고 좋은일도 있었으나 결국 이겨내어 대학에 오게되었네요 이투스 관리감독 하시느라 힘드셨을텐데 앞으로도 힘내시길바랍니다!!</v>
       </c>
       <c r="J260" t="str">
-        <v>시기별로 상황에 맞춰 학습 방법을 추천해 주시고, 중간중간 점검도 해주셔서 취약 과목의 성적을 올리는데 정말 많은 도움이 됐어요!</v>
+        <v>시기별로 상황에 맞춰 학습 방법을 추천해 주시고, 중간중간 점검도 해주셔서 취약 과목의 성적을 올리는 데 정말 많은 도움이 됐어요!</v>
       </c>
       <c r="K260" t="str">
         <v/>
@@ -9862,7 +9862,7 @@
         <v>수능을 망쳐서 원하는 대학을 가기에는 어려운 성적을 받았지만 선생님들께서 성적만 보고 판단하시지 않고 경쟁률 보시며 같이 상담해주시고 원서를 써서 원하는 대학에 붙을 수 있었습니다</v>
       </c>
       <c r="F262" t="str">
-        <v>한 강사의 커리큘럼만 추천하기보단 여러 강사들의 좋은 교재만 발췌해주시며 저의 스타일에 맞는 인강을 추천해주시고 매주 진도를 확인하시며 그때 그때 저에게 필요한 플랜을 짜주신 것이 너무 인상적이었습니다</v>
+        <v>한 강사의 커리큘럼만 추천하기보단 여러 강사들의 좋은 교재만 발췌해주시며 저의 스타일에 맞는 인강을 추천해 주시고 매주 진도를 확인하시며 그때 그때 저에게 필요한 플랜을 짜주신 것이 너무 인상적이었습니다</v>
       </c>
       <c r="G262" t="str">
         <v>평소 혼자서 공부할 때는 핸드폰 유혹에 넘어가며 순공 시간이 길지 않았지만 학원에서 핸드폰을 압수하며 집중력이 흐트러지지 않도록 도와주시고 주변의 소식이나 연락도 잘 받을 수 없어 오로지 공부에만 집중할 수 있었습니다</v>
@@ -9900,7 +9900,7 @@
         <v>혼자 재수할땐 그런 부분은 다 알수가 없고 전문가가 아니어서 정보를 다른곳에서 하나하나 얻어야 해서 힘들었는데 학원을 통해 필요한 정보만 알 수 있어서 좋았습니다. 꼭 n수를 안하더라도 고등학생이 다니기도 좋을 것 같습니다</v>
       </c>
       <c r="G263" t="str">
-        <v>전 잠도 많고 집중력도 안좋아서 다 잡아주시는게 좋았습니다. 1년 동안 다니면서 학습 습관이 정말 좋아졌습니다. 딴짓하거나 졸어나 집중력이 흐트러질때 잘 잡아주셔서 감사했습니다. 재수학원이어서 추천하겠다는 말이 욕처럼 들릴진 모르겠지만 그냥 공부 습관 잡는겸 다니는것도 나쁘지 않을것같습니다</v>
+        <v>전 잠도 많고 집중력도 안좋아서 다 잡아주시는게 좋았습니다. 1년 동안 다니면서 학습 습관이 정말 좋아졌습니다. 딴짓하거나 졸어나 집중력이 흐트러질때 잘 잡아주셔서 감사했습니다. 재수 학원이어서 추천하겠다는 말이 욕처럼 들릴진 모르겠지만 그냥 공부 습관 잡는겸 다니는것도 나쁘지 않을것같습니다</v>
       </c>
       <c r="H263" t="str">
         <v>모의고사를 매주 보기때문에 미리 연습하는겸 준비해볼수 있어서 좋았습니다. 전 긴장을 정말 많이 하는 사람이기때문에 모의고사를 많이 푸는 것 많으로 마음에 준비를 할 수 있었습니다.</v>
@@ -9979,7 +9979,7 @@
         <v>이투스 전국모의고사를 매달 보는 것이 좋았습니다. 이투스 전국모의고사를 통해 다른 친구들과 나의 실력을 비교하는 기회를 제공받을 수 있었고, 무엇이 부족한지 파악할 수 있었습니다.</v>
       </c>
       <c r="I265" t="str">
-        <v>기숙학원에 있는동안 잘 케어해주셔서 감사합니다. 담임 선생님의 철저한 학습 관리와 멘토링 덕분에 반수에 성공해서 더 좋은 대학에 다닐 수 있게 되었습니다. 이투스247 기숙학원에서 관리해주셔서 감사합니다.</v>
+        <v>기숙학원에 있는동안 잘 케어해주셔서 감사합니다. 담임 선생님의 철저한 학습 관리와 멘토링 덕분에 반수에 성공해서 더 좋은 대학에 다닐 수 있게 되었습니다. 이투스247 기숙학원에서 관리해 주셔서 감사합니다.</v>
       </c>
       <c r="J265" t="str">
         <v>사소한 부분까지 함께 의견을 나누며 의지할 수 있는 선생님이 계셨다는 점이 수험 생활의 작은 힘이 되었어요.</v>
@@ -10163,7 +10163,7 @@
         <v>평소에 계획을 세우고 공부하기보다는 그냥 마구잡이로 공부를 하는 성향이 있었다. 하지만 계획을 세우면서 공부하니 좀 더 효과적으로 공부할 수 있었던 것 같다. 계획을 세우는 습관을 들임으로써 앞으로도 나에게 큰 도움이 될 것 같다고 생각이 든다.</v>
       </c>
       <c r="G269" t="str">
-        <v>공부할때 나에게 가장 방해가 된다고 생각이 든것은 전자기기였다. 혼자 스카에서 공부하는게 아닌 독학재수학원을 선택한 이유 역시 이러한 전자기기로부터 떨어져서 온전히 공부에만 집중하고 싶어서였다. 덕분에 공부에 집중할 수 잇는 환경이 나에게 큰 도움이 되었다.</v>
+        <v>공부할때 나에게 가장 방해가 된다고 생각이 든것은 전자기기였다. 혼자 스카에서 공부하는게 아닌 독학재수 학원을 선택한 이유 역시 이러한 전자기기로부터 떨어져서 온전히 공부에만 집중하고 싶어서였다. 덕분에 공부에 집중할 수 잇는 환경이 나에게 큰 도움이 되었다.</v>
       </c>
       <c r="H269" t="str">
         <v>이투스 패스를 가장 우선으로 활용한 것은 아니었지만 몇가지 괜찮은 강의들이 있어 그것을 활용하기 위해 패스를 구독했다. 패스값을 학원에서 지원해주어서 원하는 강의를 추가적으로 들을 수 있어고 그것이 나에게 도움이 되었다.</v>
@@ -10591,7 +10591,7 @@
 ​이때 상담 선생님께서 제 모의고사 성적과 학습 성향을 분석하여, 부족한 개념을 채워줄 최적의 강의와 교재를 딱 맞게 골라주셨습니다. 덕분에 교재 선택에 들어가는 고민과 시간을 획기적으로 줄일 수 있었고, 검증된 콘텐츠로 학습한 결과 성적 향상에도 큰 효과를 보았습니다. 본인에게 가장 효율적인 학습 경로를 찾고 싶은 학생들에게 이 시스템이 정말 유용할 것이라고 생각합니다.</v>
       </c>
       <c r="G281" t="str" xml:space="preserve">
-        <v xml:space="preserve">독학재수학원을 선택할 때 가장 걱정했던 부분이 자제력이었는데, 이투스247의 철저한 면학 분위기 조성과 졸음 관리 덕분에 흐트러짐 없이 공부에만 몰입할 수 있었습니다. 조용한 환경이 항상 유지되도록 선생님들께서 수시로 복도를 돌며 관리해 주시는 점이 인상적이었습니다._x000d_
+        <v xml:space="preserve">독학재수 학원을 선택할 때 가장 걱정했던 부분이 자제력이었는데, 이투스247의 철저한 면학 분위기 조성과 졸음 관리 덕분에 흐트러짐 없이 공부에만 몰입할 수 있었습니다. 조용한 환경이 항상 유지되도록 선생님들께서 수시로 복도를 돌며 관리해 주시는 점이 인상적이었습니다._x000d_
 ​특히 공부하다가 나도 모르게 졸음이 쏟아질 때면, 선생님께서 즉각적으로 깨워주시거나 스탠딩 책상 이용을 권장해 주시는 등 세심하게 관리해 주셔서 큰 도움이 되었습니다. 혼자라면 쉽게 나태해질 수 있는 시간들을 학원의 체계적인 생활 관리 시스템이 잡아준 덕분에 하루 목표 공부량을 꾸준히 채울 수 있었습니다. 타이트한 분위기 속에서 집중력을 극대화하고 싶은 학생들에게 최적의 환경이라고 생각합니다.</v>
       </c>
       <c r="H281" t="str" xml:space="preserve">
@@ -10635,7 +10635,7 @@
         <v>영단어를 소홀히 하기 쉬운데 그 점을 아주 잘 바로잡아준거같다. 영단어는 꾸준히 매일 조금씩 반복학습으로 하는게 중요한데 그 중요지점을 잘 파고든 시스템같다. 그 지점에서 아주 유용하다고 생각한다</v>
       </c>
       <c r="I282" t="str">
-        <v>감사합니다. 항상 수고 많으십니다. 재수라는게 사람마다 정도는 다르겠지만 멘탈적인 부분의 영향력을 무시할 수 없어서 그 멘탈 관리에 조금이나마 도움이 되지 않았나 싶다. 수능공부는 결과만 남는게 절대 아니고 과정 속에서도 얻어가는 점이 분명히 있기에 이런 독학재수학원의 경험이 개인적으로 기억에 깊게 남아있다.</v>
+        <v>감사합니다. 항상 수고 많으십니다. 재수라는게 사람마다 정도는 다르겠지만 멘탈적인 부분의 영향력을 무시할 수 없어서 그 멘탈 관리에 조금이나마 도움이 되지 않았나 싶다. 수능공부는 결과만 남는게 절대 아니고 과정 속에서도 얻어가는 점이 분명히 있기에 이런 독학재수 학원의 경험이 개인적으로 기억에 깊게 남아있다.</v>
       </c>
       <c r="J282" t="str">
         <v>학습 슬럼프를 겪을 때 선생님이 지속적으로 상담을 통해 저에게 맞는 공부 방법을 찾아주셔서 계속 공부할 수 있었습니다.</v>
@@ -10798,7 +10798,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E287" t="str">
-        <v>이투스 재수학원의 코칭 시스템은 단순히 공부 계획을 세워주는 데서 끝나는 것이 아니라, 개인의 학습 습관과 약점을 정확하게 분석해 맞춤형으로 관리해준다는 점이 특히 유용했습니다. 정기적인 상담을 통해 현재 공부 방향이 맞는지 점검받을 수 있었고, 성적 변화에 따라 계획을 유연하게 수정해 주어 효율적으로 공부할 수 있었습니다. 또한 동기 부여가 떨어질 때마다 코치 선생님이 지속적으로 피드백을 주셔서 끝까지 꾸준히 공부하는 데 큰 도움이 되었습니다.</v>
+        <v>이투스 재수 학원의 코칭 시스템은 단순히 공부 계획을 세워주는 데서 끝나는 것이 아니라, 개인의 학습 습관과 약점을 정확하게 분석해 맞춤형으로 관리해준다는 점이 특히 유용했습니다. 정기적인 상담을 통해 현재 공부 방향이 맞는지 점검받을 수 있었고, 성적 변화에 따라 계획을 유연하게 수정해 주어 효율적으로 공부할 수 있었습니다. 또한 동기 부여가 떨어질 때마다 코치 선생님이 지속적으로 피드백을 주셔서 끝까지 꾸준히 공부하는 데 큰 도움이 되었습니다.</v>
       </c>
       <c r="F287" t="str">
         <v>학습 관리 시스템은 하루 공부량과 과목별 학습 시간을 체계적으로 기록하고 확인할 수 있어 자기 관리에 큰 도움이 되었습니다. 계획 대비 실제 공부 시간을 비교하면서 부족한 부분을 바로 파악할 수 있었고, 이를 통해 비효율적인 공부 습관을 개선할 수 있었습니다. 또한 누적 데이터로 자신의 학습 패턴을 한눈에 볼 수 있어 장기적인 공부 방향을 잡는 데에도 매우 유용했습니다.</v>
@@ -11539,7 +11539,7 @@
         <v>N수생</v>
       </c>
       <c r="E308" t="str">
-        <v>인강이나 문제집을 찾을 시간이 많이 없었는데 어떤 걸 풀면 좋을지 추천해주시고 진도 체크를 매주 해주셔서 도움이 되었다. 모의고사를 푼 이후에 틀린 문제를 기반으로 무엇을 보충하면 좋을지도 추천해주셨다.</v>
+        <v>인강이나 문제집을 찾을 시간이 많이 없었는데 어떤 걸 풀면 좋을지 추천해 주시고 진도 체크를 매주 해주셔서 도움이 되었다. 모의고사를 푼 이후에 틀린 문제를 기반으로 무엇을 보충하면 좋을지도 추천해주셨다.</v>
       </c>
       <c r="F308" t="str">
         <v>수학 문제를 풀면서 도저히 접근이 안되는 문제를 자주 질문했는데 이해를 할 수 있을 때까지 계속 설명해주셔서 풀 수 있는 문제가 는 것 같다. 해설지가 제대로 제공되지 않는 문제도 많아서 그 때 도움을 많이 받았다.</v>
@@ -11574,17 +11574,17 @@
         <v>반수생</v>
       </c>
       <c r="E309" t="str" xml:space="preserve">
-        <v xml:space="preserve">이투스 재수학원의 생활 지도는학습 몰입을 방해하는 요소를 원천 차단한다는 점에서 매우 효과적이었습니다._x000d_
+        <v xml:space="preserve">이투스 재수 학원의 생활 지도는학습 몰입을 방해하는 요소를 원천 차단한다는 점에서 매우 효과적이었습니다._x000d_
 무엇보다 엄격한 휴대폰 관리와 인터넷 강의 외 사이트 차단 시스템 덕분에 딴짓을 하고 싶은 유혹을 물리치고 오로지 공부에만 전념할 수 있었습니다. 또한, 졸음이나 학습 태도를 상시 점검하는 관리 선생님들이 계셔서 자칫 느슨해질 수 있는 오후 시간에도 긴장감을 유지할 수 있었던 점이 좋았습니다._x000d_
 단순히 통제만 하는 것이 아니라, 전략 담임 선생님과의 정기적인 상담을 통해 멘탈 관리와 학습 방향성을 함께 잡아주어 수험 생활 내내 심리적인 안정감을 느낄 수 있었던 점이 큰 장점입니다.</v>
       </c>
       <c r="F309" t="str" xml:space="preserve">
-        <v xml:space="preserve">이투스 재수학원의 학습 플래너 관리는 나태해지기 쉬운 수험 생활에서 공부의 중심을 잡아주는 역할을 했습니다._x000d_
+        <v xml:space="preserve">이투스 재수 학원의 학습 플래너 관리는 나태해지기 쉬운 수험 생활에서 공부의 중심을 잡아주는 역할을 했습니다._x000d_
 가장 좋았던 점은 담임 선생님이 내 플래너를 직접 확인하며 과목별 밸런스를 짚어주신다는 것이었습니다. 혼자 공부하다 보면 좋아하는 과목만 파고들게 되는데, 선생님의 피드백 덕분에 부족한 과목에 시간을 더 할당하는 객관적인 시각을 가질 수 있었습니다._x000d_
 또한, 매일 아침 목표를 세우고 밤에 피드백을 하는 과정이 습관이 되면서 막연한 불안감이 사라지고 '오늘 해야 할 일'에만 집중할 수 있었습니다. 단순히 기록하는 것을 넘어, 내가 제대로 가고 있는지 실시간으로 점검받는 느낌이라 끝까지 지치지 않고 완주할 수 있었던 것 같습니다.</v>
       </c>
       <c r="G309" t="str" xml:space="preserve">
-        <v xml:space="preserve">이투스 재수학원의 전자출결 시스템은 수험생 입장에서 **'강제성 섞인 안정감'**을 주는 장치였습니다._x000d_
+        <v xml:space="preserve">이투스 재수 학원의 전자출결 시스템은 수험생 입장에서 **'강제성 섞인 안정감'**을 주는 장치였습니다._x000d_
 우선, 등원과 하원 시간이 찍히자마자 부모님께 바로 알림이 가기 때문에 딴길로 새거나 늦잠을 자는 등의 나태함을 부릴 틈이 없었습니다. 처음에는 조금 타이트하게 느껴졌지만, 오히려 이런 규칙적인 생활이 몸에 배면서 수능 당일 컨디션에 맞춘 **'새벽형 생체 리듬'**을 만드는 데 큰 도움이 되었습니다._x000d_
 특히 단순 출결뿐만 아니라 외출이나 조퇴도 엄격하게 데이터로 관리되다 보니, 학원 안의 전반적인 분위기가 면학에만 집중할 수 있도록 차분하게 유지되는 점이 만족스러웠습니다. 내 출결 현황을 숫자로 확인하며 스스로 성실함을 증명받는 기분이 들어, 슬럼프가 올 때도 마음을 다잡는 계기가 되었습니다.</v>
       </c>
@@ -11632,7 +11632,7 @@
         <v>감사합니다! 항상 신경써주시고 잘 챙겨주시고 공부환경에 대해서 많이 배려해주셔서 감사해요. 제가 좀 까탈스러운편인데 배려해주신 부분이 너무 감사했습니다.. 항상 좋은 나날 되시길 부탁드려요!.!!</v>
       </c>
       <c r="J310" t="str">
-        <v>모르는 문제를 여쭤볼 때 세세하게 풀이 방법을 알려주셔서 성적을 올리는데 정말 많은 도움이 됐습니다!</v>
+        <v>모르는 문제를 여쭤볼 때 세세하게 풀이 방법을 알려주셔서 성적을 올리는 데 정말 많은 도움이 됐습니다!</v>
       </c>
       <c r="K310" t="str">
         <v/>
@@ -11839,7 +11839,7 @@
         <v>모의고사를 푸는 것 자체로 실전경험을 기를 수 있어서 좋다고 생각하고 모의고사를 다 풀고 틀린문제를 오답하는 과정에서 몰랐던 것을 알게 되거나 자주 하는 실수를 발견할 수 있어서 실력향상에 큰 도움이 되었습니다 이런 모의고사를 주기적으로 학원에서 시행하니 실력이 늘 수밖에 없었습니다</v>
       </c>
       <c r="I316" t="str">
-        <v>작년 저의 공부를 도와주시고 관리해주셔서 정말 감사합니다 선생님들 덕분에 대학에 합격할 수 있었습니다 모의고사 성적이 나오면 제 성적을 분석해 주시고 상담해주신 선생님들 다시 한번 감사드립니다</v>
+        <v>작년 저의 공부를 도와주시고 관리해 주셔서 정말 감사합니다 선생님들 덕분에 대학에 합격할 수 있었습니다 모의고사 성적이 나오면 제 성적을 분석해 주시고 상담해주신 선생님들 다시 한번 감사드립니다</v>
       </c>
       <c r="J316" t="str">
         <v>모의고사 등급을 잘 받아 학원에서 장학금을 주셨는데 공부하면서 많은 동기부여를 얻을 수 있었습니다!</v>
@@ -11900,7 +11900,7 @@
         <v>매주 담임 선생님과 함께 전 과목의 교재 진도를 계획하고, 일주일 후 그 계획을 실제로 수행했는지 선생님과 함께 교재를 통해 점검받을 수 있었다. 혼자 계획을 세우고 공부할 때보다 지속적인 피드백을 받을 수 있어 학습에 대한 긴장감을 유지할 수 있었고, 그 덕분에 끈기를 잃지 않고 꾸준히 공부할 수 있었다.</v>
       </c>
       <c r="F318" t="str">
-        <v>담임 선생님께서 다양한 과목의 인터넷 강의에 대한 이해도가 높아, 나의 수준과 현재 상황에 맞는 강의와 교재를 적절하게 추천해주신 점이 가장 유용했다. 덕분에 혼자서 선택에 시간을 낭비하지 않고 효율적으로 학습할 수 있었으며, 수강 진도까지 함께 관리해주셔서 꾸준히 공부를 이어가는 데 큰 도움이 되었다.</v>
+        <v>담임 선생님께서 다양한 과목의 인터넷 강의에 대한 이해도가 높아, 나의 수준과 현재 상황에 맞는 강의와 교재를 적절하게 추천해주신 점이 가장 유용했다. 덕분에 혼자서 선택에 시간을 낭비하지 않고 효율적으로 학습할 수 있었으며, 수강 진도까지 함께 관리해 주셔서 꾸준히 공부를 이어가는 데 큰 도움이 되었다.</v>
       </c>
       <c r="G318" t="str">
         <v>수능 공부와 관련된 앱/사이트에만 접속이 가능하니 학습에만 집중할 수 있었던 점이 가장 유용했다. 스스로 통제하기 어려운 상황에서도 외부적인 관리가 이루어지니 흐트러짐을 줄일 수 있었다.</v>
@@ -12405,7 +12405,7 @@
         <v>일반 독서실이나 관리형 독서실들과는 다르게 핵심과목인 국어,영어,수학 전공자 선생님들께서 상주하고 계셔서 문제를 풀다가 막힘이 오거나 특정과목에 대한 상담이 필요할때 즉각적인 질의응답을 통한 학습이 가능하다는 점이 가장 큰 장점이였다. 온라인 강의와 사이트를 이용하다보면 강의와 개념, 문제들에 대한 질문을 qna 게시판을 통해서만 질문이 가능한데 이는 시간도 오래걸리고 대면으로 질문하는것이 아니기에 한계가 존재했었다. 또한 이투스 247 목동 졸업생들이 멘토로 근무를 하여 특정 탐구 과목들에 대한 피드백과 질문, 조언들을 얻을 수 있다는 점에서 이투스 247 목동만의 독보적이고 차별적인 시스템이다.</v>
       </c>
       <c r="G332" t="str">
-        <v>공부를 하는 학생 입장에서 독학재수학원을 생각할때 중요시하게 고려하는 요소가 면학 분위기 입니다. 그러한점에서 목동 이투스 247은 다양한 시스템을 통한 최고의 면학 분위기를 제공해주었습니다. 우선 매너타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다 같이 집중할 수 있는 공부 환경을 제공해줍니다. 또한 학생들이 학습중 자지 않도록 상시로 감독 선생님께서 자습실을 비롯한 공용학습 공간까지 꼼꼼히 돌아다니시며 모든 학생이 열심히 공부를 할 수 있게 도와주십니다.</v>
+        <v>공부를 하는 학생 입장에서 독학재수 학원을 생각할때 중요시하게 고려하는 요소가 면학 분위기 입니다. 그러한점에서 목동 이투스 247은 다양한 시스템을 통한 최고의 면학 분위기를 제공해주었습니다. 우선 매너타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다 같이 집중할 수 있는 공부 환경을 제공해줍니다. 또한 학생들이 학습중 자지 않도록 상시로 감독 선생님께서 자습실을 비롯한 공용학습 공간까지 꼼꼼히 돌아다니시며 모든 학생이 열심히 공부를 할 수 있게 도와주십니다.</v>
       </c>
       <c r="H332" t="str">
         <v>목동 이투스 247점에서는 단어테스트반을 모집하여 매주 영단어 테스트를 봅니다. 학생들이 가장 귀찮아하고 소홀히하는 영단어 외우기를 같은 학생들과 함께 매주 테스트를 보며 매주 빼먹지 않게 외우게된다는 장점이 있습니다.</v>
@@ -12685,7 +12685,7 @@
         <v>수업을 듣다가 모르는 부분이 있거나 공부할 때 궁금증이 생기면 각 과목별 선생님께 1:1로 질문할 수 있다는 점이 좋았다. 1:1로 하니 불편하지 않고 선생님께 모르는 부분을 다 터놓고 이야기할 수 있어 궁금증을 해소하는데 큰 도움이 되었다.</v>
       </c>
       <c r="G340" t="str">
-        <v>아무리 마음을 다잡고 열심히 공부하려고 들어왔더라도 가끔 졸리거나 할 때가 분명 있는데, 이를 감독 선생님께서 돌아다니며 관리해주셔서 더 마음을 굳건히 먹고 공부할 수 있었다. 또한 면학 분위기 조성으로 학원에 있는 동안에는 공부에만 집중할 수 있었다.</v>
+        <v>아무리 마음을 다잡고 열심히 공부하려고 들어왔더라도 가끔 졸리거나 할 때가 분명 있는데, 이를 감독 선생님께서 돌아다니며 관리해 주셔서 더 마음을 굳건히 먹고 공부할 수 있었다. 또한 면학 분위기 조성으로 학원에 있는 동안에는 공부에만 집중할 수 있었다.</v>
       </c>
       <c r="H340" t="str">
         <v>혼자서 단어를 외우려고 하다보면 의지 부족으로 루틴이 꾸준히 이어지지 못하는데, 학원에서는 일괄적으로 단어 시험을 봐서 단어를 외우는 습관을 들일 수 있었다. 매일 영단어를 외우고 시험보고, 또 반복하다 보니 확실하게 영단어를 습득할 수 있었다.</v>
@@ -12861,7 +12861,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E345" t="str" xml:space="preserve">
-        <v xml:space="preserve">고등학교 3년 동안 이투스 247 재수학원을 다니면서 가장 도움이 됐던 부분은 선생님과의 학습 상담이었다. 단순히 공부를 열심히 하라고 하는 것이 아니라, 스케줄링 상담을 통해 하루 단위, 주 단위로 어떻게 시간을 써야 하는지 구체적으로 계획을 세울 수 있었다._x000d_
+        <v xml:space="preserve">고등학교 3년 동안 이투스 247 재수 학원을 다니면서 가장 도움이 됐던 부분은 선생님과의 학습 상담이었다. 단순히 공부를 열심히 하라고 하는 것이 아니라, 스케줄링 상담을 통해 하루 단위, 주 단위로 어떻게 시간을 써야 하는지 구체적으로 계획을 세울 수 있었다._x000d_
 _x000d_
 특히 내가 어느 과목에 시간을 더 투자해야 하는지, 지금 시기에 무엇을 우선적으로 해야 하는지에 대해 명확하게 방향을 제시해 주신 점이 인상 깊었다. 혼자 공부할 때는 막연하게 느껴졌던 부분들이 상담을 통해 정리되면서, ‘지금 내가 제대로 가고 있는지’에 대한 확신을 가질 수 있었다._x000d_
 _x000d_

</xml_diff>

<commit_message>
Apply sixth batch of typo corrections
</commit_message>
<xml_diff>
--- a/reviews_with_keywords.xlsx
+++ b/reviews_with_keywords.xlsx
@@ -477,7 +477,7 @@
 지난 한 해 동안 정말 감사하였습니다. 다른 학원생들도 좋은 결과가 있으면 좋겠습니다.</v>
       </c>
       <c r="J2" t="str">
-        <v>선생님들께서 좋은 면학 분위기를 조성해주셔서 자연스럽게 졸지 않으려고 노력하게 되었어요.</v>
+        <v>선생님들께서 좋은 면학 분위기를 조성해 주셔서 자연스럽게 졸지 않으려고 노력하게 되었어요.</v>
       </c>
       <c r="K2" t="str">
         <v>면학 분위기</v>
@@ -606,7 +606,7 @@
         <v>재수하면서 멘탈이 흔들릴때가 많았는데 그때마다 상담하면서 중심을 잡을 수 있었던것 같습니다. 그리고 담당 선생님이 열심히 쪼아주셔서 나태해질때마다 다시 정신 붙잡고 공부할 수 있었고 후반에는 공부를 어떻게 해야되는지 안 것 같은 느낌이었습니다</v>
       </c>
       <c r="F6" t="str">
-        <v>앞서 말한 것과 비슷하게 개인적인 성향이 혼자둬도 공부 엔간히 하지만 옆에 두고 관리해주실때 공부 효율이 더 나는 사람이라 플래너라든지 공부 방향 관리해주신게 좋았습니다! 효율적으로 공부하게 되는 느낌이었어여</v>
+        <v>앞서 말한 것과 비슷하게 개인적인 성향이 혼자둬도 공부 엔간히 하지만 옆에 두고 관리해주실때 공부 효율이 더 나는 사람이라 플래너라든지 공부 방향 관리해 주신게 좋았습니다! 효율적으로 공부하게 되는 느낌이었어여</v>
       </c>
       <c r="G6" t="str">
         <v>다른건 막 좋지는 않았는데 그냥 그랬어여 그나마 나은게 출결이었음. 그냥 빨리 일어나니까 생활 습관 잡히고 아침에 뇌가 깨어 있는 느낌? 좋았습니다. 근데 다른건 개선 할게 좀 있어여</v>
@@ -638,10 +638,10 @@
         <v>반수생</v>
       </c>
       <c r="E7" t="str">
-        <v>매주 하루 정해서 상담을 해주셨는데, 현재 공부 상태 확인과 스스로가 계획을 잘 세워서 이행하고 있는지를 꼼꼼하게 확인해주셨다. 그리고 어느 부분을 일주일동안 공부해왔으며 과목별로 공부 진행을 어떻게 하고 있는지 확인하고 공부량 조언해주신 것이 도움이 되었다.</v>
+        <v>매주 하루 정해서 상담을 해주셨는데, 현재 공부 상태 확인과 스스로가 계획을 잘 세워서 이행하고 있는지를 꼼꼼하게 확인해주셨다. 그리고 어느 부분을 일주일동안 공부해왔으며 과목별로 공부 진행을 어떻게 하고 있는지 확인하고 공부량 조언해 주신 것이 도움이 되었다.</v>
       </c>
       <c r="F7" t="str">
-        <v>평소에 플래너를 쓰는 습관이 없었는데, 플래너를 쓰는 것을 처음부터 도와주셨다. 그리고 매주 확인을 해주신 덕분에 매일매일 밀리지 않고 하루의 계획을 철저히 세워서 이행할 수 있었다.</v>
+        <v>평소에 플래너를 쓰는 습관이 없었는데, 플래너를 쓰는 것을 처음부터 도와주셨다. 그리고 매주 확인을 해 주신 덕분에 매일매일 밀리지 않고 하루의 계획을 철저히 세워서 이행할 수 있었다.</v>
       </c>
       <c r="G7" t="str">
         <v>같이 공부하는 환경에서 자고 있는 학생이 있으면 깨워주시고 시간별로 돌아다니시면서 학습 분위기를 잡아주어 도움이 되었다. 그리고 시끄러운 학생이 있으면 자리를 옮기게 해주는 등 도움을 주셨다.</v>
@@ -711,7 +711,7 @@
         <v>이투스 개별 맞춤 학습 상담을 통해 제 실력이 현재 어느 정도인지, 그리고 앞으로 어떤 부분을 집중해야 할지 명확하게 알 수 있어서 좋았습니다! 상담 과정에서 꼼꼼하게 제 실력에 맞춰 학습 방향을 제시해 주셔서 학습 계획을 세우는 데 큰 도움이 되었습니다! 한달을 되돌아 볼 수 있는 소중한 시간이었습니다!</v>
       </c>
       <c r="F9" t="str">
-        <v>모르는 부분을 바로바로 질문할 수 있어서  시간 낭비를 줄이고 효율적으로 공부할 수 있었던 점이 정말 좋았습니다. 조교 쌤들 다 너무 친절하게 기초부터 설명해주셔서 실력 향상에 정말 많은 도움이 되었습니다!</v>
+        <v>모르는 부분을 바로바로 질문할 수 있어서  시간 낭비를 줄이고 효율적으로 공부할 수 있었던 점이 정말 좋았습니다. 조교 쌤들 다 너무 친절하게 기초부터 설명해 주셔서 실력 향상에 정말 많은 도움이 되었습니다!</v>
       </c>
       <c r="G9" t="str">
         <v>핸드폰 수거로 핸드폰을 확인하여 시간낭비하는 일이 줄어 공부에 더욱 집중할 수 있어서 좋았습니다! 하루 목표 공부령을 채우는데 큰 도움이 되었고 공부에 집중하는 습관을 기르는데 가장 많은 도움이 된 것 같습니당</v>
@@ -720,7 +720,7 @@
         <v>이투스 모의고사를 통해 현재 제 실력을 객관적으로 확인할 수 있어 좋았습니다. 응시하면서 부족한 부분을 체계적으로 파악하고 보완할 수 있어 학습 방향을 잡는 데 큰 도움이 되었고 모의고사 성적을 비롯한 상담을 통해 성적을 향상시킬 수 있었습니다!</v>
       </c>
       <c r="I9" t="str">
-        <v>1년이 조금 안되눈 시간동안 항상 따뜻하게 지도해주시고 응원해주셔서 감사합니다 선생님들 덕분에 재수 했을 때의 기억이 마냥 힘든 시간으로만 기억되지 않을것 같아요! 진심으로 너무 감사했습니다🩷🩷</v>
+        <v>1년이 조금 안되눈 시간동안 항상 따뜻하게 지도해 주시고 응원해 주셔서 감사합니다 선생님들 덕분에 재수 했을 때의 기억이 마냥 힘든 시간으로만 기억되지 않을것 같아요! 진심으로 너무 감사했습니다🩷🩷</v>
       </c>
       <c r="J9" t="str">
         <v>상담 과정에서 꼼꼼하게 제 실력에 맞춰 학습 방향을 제시해 주셔서 학습 계획을 세우는 데 큰 도움이 되었어요.</v>
@@ -746,7 +746,7 @@
         <v>요즘같이 수 많은 컨텐츠가 쏟아지는 시기에 나한테 맞는 커리큘럼은 무엇인지, 등등 정확하게 현재 내게 필요한 공부만 할 수 있었습니다. 또한 성적이 나오지 않아 전전긍긍할 때에도 객관적으로 나를 평가해 올바른 방법으로 공부할 수 있도록 꾸준히 이끌어주었습니다.</v>
       </c>
       <c r="F10" t="str">
-        <v>저는 인강을 많이 듣지 않고 스스로 공부하는 것을 좋아하였는데 이때 자칫 공부량이 너무 적어질 수 있는 문제가 있었습니다. 그러나 이러한 부분들을 관리해주시고 정말 나에게 맞는 공부를 추천해 주셔서 잘 할 수 있었습니다.</v>
+        <v>저는 인강을 많이 듣지 않고 스스로 공부하는 것을 좋아하였는데 이때 자칫 공부량이 너무 적어질 수 있는 문제가 있었습니다. 그러나 이러한 부분들을 관리해 주시고 정말 나에게 맞는 공부를 추천해 주셔서 잘 할 수 있었습니다.</v>
       </c>
       <c r="G10" t="str">
         <v>저는 집중력이 좋지 않아 스터디카페에서는 한 문제 풀고 핸드폰 보고 하는 등의 문제가 있었는데 이러한 부분들을 핸드폰 제출로 해결할 수 있었습니다. 또한 SNS를 잘 보지 않게 돼 남들과 저를 비교하지 못하는 것도 좋았습니다.</v>
@@ -755,10 +755,10 @@
         <v>인터넷 강의는 이투스도 그렇고 타 회사도 그렇고 너무 비싸서 듣기에 부담스러웠는데 이투스247을 다니니 질 좋은 강의를 무료로 수강할 수 있어서 부담 없이 잘 들었던 것 같습니다. 노베이스였던 제가 공부에 발을 들이기 좋은 선생님들이 너무 많았습니다.</v>
       </c>
       <c r="I10" t="str">
-        <v>재수하면서 선생님들을 정말 귀찮게 많이 했는데.. 불편한 기색없이 질문도 정말 정성스럽게 답변해주시고 고민들도 같이 들어주고, 고민하고, 도움을 주셨던 부분들이 정말 감사했습니다.</v>
+        <v>재수하면서 선생님들을 정말 귀찮게 많이 했는데.. 불편한 기색없이 질문도 정말 정성스럽게 답변해 주시고 고민들도 같이 들어주고, 고민하고, 도움을 주셨던 부분들이 정말 감사했습니다.</v>
       </c>
       <c r="J10" t="str">
-        <v>정말 나에게 맞는 공부를 추천해 주시고, 관리도 잘해주셔서 성적이 오를 수 있었어요.</v>
+        <v>정말 나에게 맞는 공부를 추천해 주시고, 관리도 잘해 주셔서 성적이 오를 수 있었어요.</v>
       </c>
       <c r="K10" t="str">
         <v/>
@@ -781,10 +781,10 @@
         <v>문제집을 풀면서 모르는 문제가 있을때 매번 답지만 보며 시간을 많이 썼는데 학습 상담을 통해서 시간을 효율적으로 쓸  수 있었고 이해하는데도 도움이 많이 되었습니다. 그리고 공부 커리큘럼을 어떻게 짜야할지 몰랐는데 학습 상담을 통해서 어떻게 공부해야 할지 감을 잡고 공부할 수 있었습니다.</v>
       </c>
       <c r="F11" t="str">
-        <v>보통 문제집을 풀면 강의가 없어 답지를 보고 문제를 혼자 이해했어야하는데 1:1로 질의 응답을 해주셔서 이해하는데 도움이 많이 되었습니다. 제가 모르는 부분을 더 집중적으로 자세하게 설명을 들을 수 있었고 못하는 부분을 보완하기 위해 무엇을 공부 해야 하는지도 알 수 있어 좋았습니다.</v>
+        <v>보통 문제집을 풀면 강의가 없어 답지를 보고 문제를 혼자 이해했어야하는데 1:1로 질의 응답을 해 주셔서 이해하는데 도움이 많이 되었습니다. 제가 모르는 부분을 더 집중적으로 자세하게 설명을 들을 수 있었고 못하는 부분을 보완하기 위해 무엇을 공부 해야 하는지도 알 수 있어 좋았습니다.</v>
       </c>
       <c r="G11" t="str">
-        <v>일단 학원에 있으면 연락 알람 자체도 안오기때문에 공부에 집중하는데 정말 도움이 되었습니다. 또한 인강 사이트 외에는 인터넷이 안되서 강제로 공부할 수 있는 환경을 조성해주셔서 공부 하기에 정말 적합한 환경이였습니다.</v>
+        <v>일단 학원에 있으면 연락 알람 자체도 안오기때문에 공부에 집중하는데 정말 도움이 되었습니다. 또한 인강 사이트 외에는 인터넷이 안되서 강제로 공부할 수 있는 환경을 조성해 주셔서 공부 하기에 정말 적합한 환경이였습니다.</v>
       </c>
       <c r="H11" t="str">
         <v>공부하는데 제일 중요한 것은 감을 잃지 않는 것인데 모의고사를 통해서 수능을 볼때의 감을 잃지 않을 수 있었고 지금 제가 어느정도의 실력을 갖고 있는지 정검할 수 있어서 더 부족하다고 생각하는 과목의 공부를 하는데 도움이 되었습니다.</v>
@@ -817,7 +817,7 @@
 또한, 저는 맞는 인강쌤을 찾기 힘들어 많이 왔다갔다 거리는 인강 유목민이었습니다. 인강이 없으면 안 된다고 생각했는데 학습 상담을 통해 인강이 맞지 않는 과목의 경우여도 독학으로 좋은 성적을 받을 수 있음을 알게되었습니다. 머리가 복잡한 수험생을 옳은 길로 잘 이끌어주셨습니다</v>
       </c>
       <c r="F12" t="str">
-        <v>앞서 언급했듯 다양한 방면으로 공부법을 제시해주시고, 결정하게 해주셔서 좋았습니다. 사람마다 맞는 공부법이 다르기에 그것을 찾아 정착하는데에는 꽤 오랜 시간이 걸린다고 생각합니다. 이투스 담임 선생님과의 꾸준한 소통과 학습 관리 시스템을 통해 시간낭비를 줄일 수 있었던 것 같습니다</v>
+        <v>앞서 언급했듯 다양한 방면으로 공부법을 제시해 주시고, 결정하게 해 주셔서 좋았습니다. 사람마다 맞는 공부법이 다르기에 그것을 찾아 정착하는데에는 꽤 오랜 시간이 걸린다고 생각합니다. 이투스 담임 선생님과의 꾸준한 소통과 학습 관리 시스템을 통해 시간낭비를 줄일 수 있었던 것 같습니다</v>
       </c>
       <c r="G12" t="str">
         <v>사실 휴대폰과 태블릿의 유혹에 수험생이 가장 취약하다고 생각하는데요. 하지만 이런 유혹은 수험 생활을 쉽게 망치기 일쑤입니다. 이투스 학원을 다니며 이러한 유혹에 견딜 수 있는데에 와이파이 방화벽이 큰 기여를 했다고 생각합니다</v>
@@ -826,7 +826,7 @@
         <v>저는 메가패스와 대성패스만 보유하고 있었는데요. 연계공부를 압축적으로 해야하는 상황이었는데 이투스 패스 덕분에 김민정쌤을 들을 수 있었습니다. 그때 들었던 작품들이 운이 좋게도 전부 수능에 나와 문학을 다 맞을 수 있었습니다!!</v>
       </c>
       <c r="I12" t="str">
-        <v>여러모로 학생만큼 고생하셨을텐데 길다면 긴, 짧다면 짧은 기간동안 감사했습니다! 선생님들의 격려와 응원, 도움이 없었다면 힘든 수험 생활 진작에 무너졌을 것 같아요,, 제 수험 생활에 함께해주셔서 감사합니다</v>
+        <v>여러모로 학생만큼 고생하셨을텐데 길다면 긴, 짧다면 짧은 기간동안 감사했습니다! 선생님들의 격려와 응원, 도움이 없었다면 힘든 수험 생활 진작에 무너졌을 것 같아요,, 제 수험 생활에 함께해 주셔서 감사합니다</v>
       </c>
       <c r="J12" t="str">
         <v>수업이 없으면 안 된다고 생각했는데 학습 상담을 통해 저에게 맞는 공부법을 알려주셔서 좋은 성적을 받을 수 있었어요.</v>
@@ -861,7 +861,7 @@
         <v>영어 단어는 항상 시간 내서 공부하기 애매한 부분이라 생각했다. VOCA 테스트 프로그램을 통해 아침마다 영어 단어 테스트를 보면서 간단하게 오답을 하며 점점 아는 단어가 쌓일 수 있었다. 또 점심엔 영어 듣기 연습이 가능해서 영어 공부에 대한 접근이 쉬워 좋았다.</v>
       </c>
       <c r="I13" t="str">
-        <v>학생 한명한명 봐주시느라 힘드셨을텐데 항상 좋은말씀으로 응원해주시고 잘못된 방향으로 가지 않도록 열심히 지도해주셔서 감사했습니다! 선생님들 덕분에 포기하지 않을 수 있었던 것 같아요!</v>
+        <v>학생 한명한명 봐주시느라 힘드셨을텐데 항상 좋은말씀으로 응원해 주시고 잘못된 방향으로 가지 않도록 열심히 지도해 주셔서 감사했습니다! 선생님들 덕분에 포기하지 않을 수 있었던 것 같아요!</v>
       </c>
       <c r="J13" t="str">
         <v>각 과목의 세세한 공부 방법과 멘탈 관리에 대한 상담을 받을 수 있었어요.</v>
@@ -896,7 +896,7 @@
         <v>이투스 인강에서 국어, 사문 등 여러가지 강의를 보면서 도움이 되었던 거 같습니다. 다른 사이트에서 인강도 많이 봤지만 국어, 사문은 이투스 인강에서 더 도움을 많이 받은 거 같습니다.</v>
       </c>
       <c r="I14" t="str">
-        <v>1년 동안 제가 공부에 온전히 집중할 수 있고, 다른 것에 신경 팔리지 않게 도움을 주셔서 정말 감사했습니다. 그 외에도 제가 힘들면 상담을 해주시고 저에게 방향성을 제시해 주셔서 감사했습니다</v>
+        <v>1년 동안 제가 공부에 온전히 집중할 수 있고, 다른 것에 신경 팔리지 않게 도움을 주셔서 정말 감사했습니다. 그 외에도 제가 힘들면 상담을 해 주시고 저에게 방향성을 제시해 주셔서 감사했습니다</v>
       </c>
       <c r="J14" t="str">
         <v>제가 모의고사를 풀거나 공부를 하며 많은 스트레스를 받았을 때 담임 선생님께 상담을 받아 많은 도움이 되었던 거 같아요.</v>
@@ -919,10 +919,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E15" t="str">
-        <v>원장 선생님께서 재원생 한명한명을 기억하시고, 마주치실때마다 공부잘되어가는지 여쭤봐주십니다. 또한 원장 선생님, 부원장 선생님을 비롯한 선생님들께서 정말 언제든 시간을 내어 적극적으로 상담해주셔서 좋았어요</v>
+        <v>원장 선생님께서 재원생 한명한명을 기억하시고, 마주치실때마다 공부잘되어가는지 여쭤봐주십니다. 또한 원장 선생님, 부원장 선생님을 비롯한 선생님들께서 정말 언제든 시간을 내어 적극적으로 상담해 주셔서 좋았어요</v>
       </c>
       <c r="F15" t="str">
-        <v>부원장 선생님과 국어 상담을 몇 번 진행했는데, 타 인강 강사 선생님들의 세부적인 특징들을 모두 말해주시면서 저와 가장 잘 맞아보이는 선생님을 추천해주셨어요. 다른 학원 선생님들과도 많이 상담해봤지만 정말 친절하다는게 느껴질 정도였고, 아직도 감사한 기억으로 남습니다</v>
+        <v>부원장 선생님과 국어 상담을 몇 번 진행했는데, 타 인강 강사 선생님들의 세부적인 특징들을 모두 말해주시면서 저와 가장 잘 맞아보이는 선생님을 추천해 주셨어요. 다른 학원 선생님들과도 많이 상담해봤지만 정말 친절하다는게 느껴질 정도였고, 아직도 감사한 기억으로 남습니다</v>
       </c>
       <c r="G15" t="str">
         <v>고3시절 아무리 공부를 해야한다는 압박감에도 불구하고 학습용 아이패드로 sns를 들어가보는게 습관이되었습니다. 하지만 이투스 방화벽시스템으로 아예 들어가는것 자체가 불가하니까sns생각이 안나서 너무 좋았어요</v>
@@ -931,7 +931,7 @@
         <v>매달 치르는 다양한 사설 모의고사들로 굳은살 배기듯이 익숙해져서 수능 당시는 정말 긴장을 안했어요 11월 모의고사를 치르는 심정으로 편하게 시험칠 수 있었어요! 다른 친구들에게 모의고사 시스템 하나는 정말 강력 추천하고싶어요</v>
       </c>
       <c r="I15" t="str">
-        <v>선생님 따로 연락은 제대로 못 드렸지만 언제나 학원에서 인사해주시고 공부잘되어가는지 힘든건 없는지 여쭤봐주셔서 감사했어요. 길고 긴 수험 생활이었지만 이투스 덕분에 저에게 과분한 대학에 오게된 것 같아 아직도 감사합니다. ㅎㅎ</v>
+        <v>선생님 따로 연락은 제대로 못 드렸지만 언제나 학원에서 인사해 주시고 공부잘되어가는지 힘든건 없는지 여쭤봐주셔서 감사했어요. 길고 긴 수험 생활이었지만 이투스 덕분에 저에게 과분한 대학에 오게된 것 같아 아직도 감사합니다. ㅎㅎ</v>
       </c>
       <c r="J15" t="str">
         <v>원장 선생님께서 재원생 한 명, 한 명을 기억하시고, 마주치실 때마다 공부는 잘 되는지 항상 체크해 주셨어요.</v>
@@ -989,7 +989,7 @@
         <v>N수생</v>
       </c>
       <c r="E17" t="str">
-        <v>저는 3월부터 재수를 했기 때문에 다른 재수생 친구들보다 살짝 뒤처진 편 이었습니다. 그래서 불안감이 있었고, 완전한 노베 상태도 아니었기 때문에 학습 계획과 생활 패턴을 혼자서 짜기 어려웠습니다. 이런 저에게 담임쌤과 국어, 수학 담당 원장님들이 재수 생활에 대한 전반적인 조언을 해주신 덕분에 안정적으로 수험 생활을 할 수 있었던 것 같습니다.</v>
+        <v>저는 3월부터 재수를 했기 때문에 다른 재수생 친구들보다 살짝 뒤처진 편 이었습니다. 그래서 불안감이 있었고, 완전한 노베 상태도 아니었기 때문에 학습 계획과 생활 패턴을 혼자서 짜기 어려웠습니다. 이런 저에게 담임쌤과 국어, 수학 담당 원장님들이 재수 생활에 대한 전반적인 조언을 해 주신 덕분에 안정적으로 수험 생활을 할 수 있었던 것 같습니다.</v>
       </c>
       <c r="F17" t="str">
         <v>주요 과목인 국어, 영어, 수학의 질의응답을 해주시는 전문적인 선생님들이 계셔서 정말 마음이 놓였습니다! 1대1 질의 응답 시스템에서는 단순히 모르는 문제의 풀이뿐만 아니라 해당 과목에 대한 전체적인 공부 방법 등도 조언 받는 게 가능했기 때문에 매우 유용했습니다!</v>
@@ -1004,7 +1004,7 @@
         <v>선생님들 덕에 경희대 입학했습니다. 감사합니다 :) 너무너무너무너무너무너무너무너무너무너무너무너무너무너무너무 좋은 1년이었습니다. 번창하세요!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!!</v>
       </c>
       <c r="J17" t="str">
-        <v>담임 선생님과 국어, 수학 담당 선생님들께서 재수 생활에 대한 전반적인 조언을 해주신 덕분에 안정적으로 수험 생활을 할 수 있었던 것 같아요.</v>
+        <v>담임 선생님과 국어, 수학 담당 선생님들께서 재수 생활에 대한 전반적인 조언을 해 주신 덕분에 안정적으로 수험 생활을 할 수 있었던 것 같아요.</v>
       </c>
       <c r="K17" t="str">
         <v/>
@@ -1094,10 +1094,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E20" t="str">
-        <v>학습 계획이나 모의고사 계획을 어떻기 세워야할지 막막했는데 담당 선생님께서 이에 대해 코칭해주시고 같이 내 일정에 맞게 계획을 세워주셔서 도움이 많이 되었다. 내가 들으면 좋을 만한 인강도 추천해 주셔서 실제로도 영어 성적이 많이 올랐다. 항상 무계획으로 공부했던 시절과 다르게 학습 습관이 잡혀서 계획적으로 공부를 해나갈 수 있었다.</v>
+        <v>학습 계획이나 모의고사 계획을 어떻기 세워야할지 막막했는데 담당 선생님께서 이에 대해 코칭해 주시고 같이 내 일정에 맞게 계획을 세워주셔서 도움이 많이 되었다. 내가 들으면 좋을 만한 인강도 추천해 주셔서 실제로도 영어 성적이 많이 올랐다. 항상 무계획으로 공부했던 시절과 다르게 학습 습관이 잡혀서 계획적으로 공부를 해나갈 수 있었다.</v>
       </c>
       <c r="F20" t="str">
-        <v>솔직히 학교 선생님 제외 모르는 문제를 물어볼 사람이 마땅히 없었는데 학원 선생님께 물어보니 친절히 답변해주셔서 좋았다. 다들 학력이 높으셔서 그런지 설명도 잘 하시고 수학같은 경우엔 효율적인 문제 풀이 방법을 알려주셔서 이 점도 많은 도움이 됐었다.</v>
+        <v>솔직히 학교 선생님 제외 모르는 문제를 물어볼 사람이 마땅히 없었는데 학원 선생님께 물어보니 친절히 답변해 주셔서 좋았다. 다들 학력이 높으셔서 그런지 설명도 잘 하시고 수학같은 경우엔 효율적인 문제 풀이 방법을 알려주셔서 이 점도 많은 도움이 됐었다.</v>
       </c>
       <c r="G20" t="str">
         <v>나의 공부 방해 요소 중 하나가 전자기기였다. 그래서 휴대폰을 누군가 강제적으로 제출하게 해야 공부에 집중할 수 있었는데 이투스에서 그런 시스템을 가지고 관리를 해주어서 공부에 집중할 수 있었다. 학원을 다니는 동안 휴대폰 사용 시간이 많이 줄어서 좋았다.</v>
@@ -1109,7 +1109,7 @@
         <v>솔직히 모의고사 공부를 제대로 시작한게 고3 때라 너무 막막했는데 같이 계획도 세워주시고 무엇보다 모르는것을 친절하게 알려주셔서 많은 도움이 되었습니다. 물론 수시로 대학에 갔지만 수능 공부하면서도 많은것을 얻을 수 있었어요! 내년에 한번 찾아뵐게요(이유는 그때가서 말씀드릴게요) 감사합니다!!</v>
       </c>
       <c r="J20" t="str">
-        <v>휴대폰을 제출하여 공부에 집중할 수 있었고, 뿐만 아니라 다른 생활 관리 시스템으로 관리를 해주셔서 공부에 집중할 수 있었어요.</v>
+        <v>휴대폰을 제출하여 공부에 집중할 수 있었고, 뿐만 아니라 다른 생활 관리 시스템으로 관리를 해 주셔서 공부에 집중할 수 있었어요.</v>
       </c>
       <c r="K20" t="str">
         <v>생활 관리</v>
@@ -1159,7 +1159,7 @@
 _x000d_
 사실 이투스에 처음 왔을때는 조금 걱정됐습니다. 고등학교 3학년 때는 담임 선생님이랑 트러블이 엄청 심했었고, 그거 때문에 스트레스도 엄청 받았어요. 하지만 이투스 선생님들은 너무 친절하고 따뜻해서 좋았습니다..돌이켜 보면, 현역때는 학교 가기 싫다는 생각을 수도없이 했었는데,막상 반수를 할 때는 학원 가기 싫다는 생각은 거의 하지 않은 것 같아요_x000d_
 _x000d_
-옆에서 지켜봐주시고 코칭해주신 선생님들께 정말 감사하다는 말씀을 드리고 싶습니다.. 각박한 반수생활 속에서 따뜻한 선생님들 덕분에 힘든 시기를 잘 보낼 수 있었어요_x000d_
+옆에서 지켜봐주시고 코칭해 주신 선생님들께 정말 감사하다는 말씀을 드리고 싶습니다.. 각박한 반수생활 속에서 따뜻한 선생님들 덕분에 힘든 시기를 잘 보낼 수 있었어요_x000d_
 _x000d_
 이투스 대구달서점 화이팅~~</v>
       </c>
@@ -1234,7 +1234,7 @@
         <v>재수 학원의 모의고사 시스템은 나의 현재 학습 수준을 객관적으로 파악하는 데 큰 도움이 되었다. 이전에는 모의고사를 충분히 경험해보지 못해 실전 감각과 위치를 정확히 알기 어려웠지만, 정기적인 모의고사를 통해 나의 성적과 등급을 구체적으로 확인할 수 있었다. 특히 과목별 점수와 취약 단원을 분석하면서 어떤 부분을 보완해야 하는지 명확히 알게 되었고, 이를 바탕으로 학습 방향을 설정할 수 있었다. 그 결과 막연하게 공부하는 것이 아니라 목표와 전략을 가지고 효율적으로 학습할 수 있게 되었다.</v>
       </c>
       <c r="I23" t="str">
-        <v>이투스 247 선생님들께 진심으로 감사드립니다. 공부가 힘들고 지칠 때마다 흔들리던 저의 마음을 바로잡아 주시고, 다시 학습에 집중할 수 있도록 도와주신 점이 가장 큰 힘이 되었습니다. 특히 피로감이 쌓여 집중력이 떨어질 때마다 적절한 조언과 격려를 통해 다시 공부 흐름을 이어갈 수 있게 해주신 덕분에 끝까지 포기하지 않고 학습을 이어갈 수 있었습니다. 선생님들의 세심한 지도와 관심이 있었기에 지금까지 꾸준히 노력할 수 있었다고 생각합니다. 진심으로 감사드립니다.</v>
+        <v>이투스 247 선생님들께 진심으로 감사드립니다. 공부가 힘들고 지칠 때마다 흔들리던 저의 마음을 바로잡아 주시고, 다시 학습에 집중할 수 있도록 도와주신 점이 가장 큰 힘이 되었습니다. 특히 피로감이 쌓여 집중력이 떨어질 때마다 적절한 조언과 격려를 통해 다시 공부 흐름을 이어갈 수 있게 해 주신 덕분에 끝까지 포기하지 않고 학습을 이어갈 수 있었습니다. 선생님들의 세심한 지도와 관심이 있었기에 지금까지 꾸준히 노력할 수 있었다고 생각합니다. 진심으로 감사드립니다.</v>
       </c>
       <c r="J23" t="str">
         <v>재수 학원의 생활 관리 시스템 중에서 특히 면학 분위기 감독과 졸음 관리는 실제로 공부하는 데 있어 정말 많은 도움이 됐어요.</v>
@@ -1257,7 +1257,7 @@
         <v>N수생</v>
       </c>
       <c r="E24" t="str">
-        <v>작년에 이투스 남구점을 다니면서 가장 만족했던 점은 학습 코칭이었습니다. 생명과학을 처음 시작하면서 막막했고, 절대평가인 영어 과목과 약점이었던 국어 공부 방향에 대해 고민이 많았는데, 제 성향에 맞게 공부 계획을 세워주고 인강까지 추천해 주셔서 큰 도움이 되었습니다. 단순한 관리가 아니라 개인 맞춤형 코칭을 받을 수 있어 좋았습니다. 그리고 질의응답 조교님들도 너무 친절하게 모르는 것을 설명해주셔서 실력향상에 큰 도움이 되었습니다.</v>
+        <v>작년에 이투스 남구점을 다니면서 가장 만족했던 점은 학습 코칭이었습니다. 생명과학을 처음 시작하면서 막막했고, 절대평가인 영어 과목과 약점이었던 국어 공부 방향에 대해 고민이 많았는데, 제 성향에 맞게 공부 계획을 세워주고 인강까지 추천해 주셔서 큰 도움이 되었습니다. 단순한 관리가 아니라 개인 맞춤형 코칭을 받을 수 있어 좋았습니다. 그리고 질의응답 조교님들도 너무 친절하게 모르는 것을 설명해 주셔서 실력향상에 큰 도움이 되었습니다.</v>
       </c>
       <c r="F24" t="str" xml:space="preserve">
         <v xml:space="preserve">생명과학 개념에서 헷갈리는 부분이나 어려운 문제를 질문하면 단순히 답만 알려주는 것이 아니라, 어떤 방향으로 접근해야 하는지까지 자세히 설명해 주셔서 이해가 훨씬 잘 됐습니다. 이투스 모의고사를 보고 틀린 문제들도 함께 점검해 주면서 앞으로 어떻게 공부해야 할지 구체적인 방향을 잡아주신 점이 큰 도움이 되었습니다. 수학도 고난이도 문제를 질문을 많이했는데 항상 친절하게 풀어줬습니다. 풀어주실 때는 풀이 과정을 이해하기 쉽게 설명해 주셔서 실력 향상에 많은 도움이 됐습니다. 국어 또한 제가 공부하고 있는 방식이 맞는지 실제 수험생 사례를 들어 설명해 주셔서 불안함을 덜 수 있었습니다._x000d_
@@ -1305,7 +1305,7 @@
         <v>평가원 모의고사외에 이투스를 통해 중간중간 내성적을 알수있어서 도움되었습니다 모의고사를 자주 보다보니 그날은 더 집중해서 임핤 있고 그 결과에  따라 학습수준을 가늠할수있어서 도움받았습니다</v>
       </c>
       <c r="I25" t="str">
-        <v>크게 부담을 주지않으시면서도 늘 관심을 가져주시고 컨디션이 저하될때 불러서 상담 해주시고 도와주시려 마음싸주신 덕분에 이투스에서의 생활에 늘 의지가 되었습니다  진심으로 감사드립니다</v>
+        <v>크게 부담을 주지않으시면서도 늘 관심을 가져주시고 컨디션이 저하될때 불러서 상담 해 주시고 도와주시려 마음싸주신 덕분에 이투스에서의 생활에 늘 의지가 되었습니다  진심으로 감사드립니다</v>
       </c>
       <c r="J25" t="str">
         <v>매일 플래너를 점검받고 피드백을 얻으면서 완벽한 학습 루틴을 만들 수 있었어요.</v>
@@ -1366,7 +1366,7 @@
         <v>입시 상담을 통해 막막하게 느껴지던 진로와 전형 선택에 대해 구체적인 방향을 잡을 수 있었습니다. 특히 현재 성적과 상황을 바탕으로 가능한 전형들을 꼼꼼히 살펴봐 주셔서 현실적인 선택을 할 수 있었고, 공부하는 과정에서도 무엇을 목표로 해야 하는지 분명한 이정표가 되어주어 큰 도움이 되었습니다.</v>
       </c>
       <c r="F27" t="str">
-        <v>원장 선생님께서 수학 과목에 대해 학생들이 이해하기 어려워하는 부분까지도 하나하나 세심하게 짚어주시며, 질문할 때마다 친절하고 쉽게 설명해주셔서 큰 도움을 받았습니다. 덕분에 수학에 대한 부담감이 줄어들었고, 학습에 대한 자신감도 점차 생길 수 있었습니다.</v>
+        <v>원장 선생님께서 수학 과목에 대해 학생들이 이해하기 어려워하는 부분까지도 하나하나 세심하게 짚어주시며, 질문할 때마다 친절하고 쉽게 설명해 주셔서 큰 도움을 받았습니다. 덕분에 수학에 대한 부담감이 줄어들었고, 학습에 대한 자신감도 점차 생길 수 있었습니다.</v>
       </c>
       <c r="G27" t="str">
         <v>학원의 면학 분위기가 매우 잘 조성되어 있어 공부에 집중하기에 좋은 환경이었습니다. 생활 전반에서도 학생들이 공부에 방해를 받지 않도록 세심하게 신경 써주셔서 자연스럽게 학습에 몰입할 수 있었고, 규칙적인 생활 습관을 유지하는 데에도 큰 도움이 되었습니다.</v>
@@ -1375,7 +1375,7 @@
         <v>이투스 학원에 다니면서 모든 강의를 무료로 구독할 수 있어 학습에 큰 도움이 되었습니다. 필요한 과목이나 부족한 부분을 언제든지 반복해서 들을 수 있었고, 시간과 장소에 구애받지 않고 효율적으로 공부할 수 있어 학습의 폭과 깊이를 넓히는 데 유익했습니다.</v>
       </c>
       <c r="I27" t="str">
-        <v>학원 선생님들께서 늘 친절하게 대해주시고, 공부하는 데 불편함이 없도록 세심하게 배려해 주셔서 큰 도움을 받았습니다. 학생들의 상황을 이해하며 편의를 많이 봐주신 덕분에 보다 편안한 마음으로 학습에 집중할 수 있었고, 감사한 마음이 큽니다.</v>
+        <v>학원 선생님들께서 늘 친절하게 대해 주시고, 공부하는 데 불편함이 없도록 세심하게 배려해 주셔서 큰 도움을 받았습니다. 학생들의 상황을 이해하며 편의를 많이 봐주신 덕분에 보다 편안한 마음으로 학습에 집중할 수 있었고, 감사한 마음이 큽니다.</v>
       </c>
       <c r="J27" t="str">
         <v>학원의 면학 분위기가 매우 잘 조성되어 있어 공부에 집중하기에 좋은 환경이었어요.</v>
@@ -1399,7 +1399,7 @@
       </c>
       <c r="E28" t="str" xml:space="preserve">
         <v xml:space="preserve">아이에 성향 파악도 원장님 께서 빠르시고 상황에 맞는 최선의 입시 전략을 코칭해 주셔서 좋았습니다._x000d_
-스트레스 없이 아이가 입시 공부에만 집중할 수 있는 분위기 조성도 잘 해주신것 같습니다.</v>
+스트레스 없이 아이가 입시 공부에만 집중할 수 있는 분위기 조성도 잘 해 주신것 같습니다.</v>
       </c>
       <c r="F28" t="str">
         <v>일대일 코칭 선생님께서 부족한 부분을 잘 파악 하시고 점수를 올리기 위해서 추가로 공부 해야 할 부분들을 잘 코칭해 주셨고 실제로 성적 향상이 되었습니다 . 또한 따뜻한 격려의 말씀도 너무 감사하고 도움이 많이 되었습니다</v>
@@ -1413,10 +1413,10 @@
       <c r="I28" t="str" xml:space="preserve">
         <v xml:space="preserve">모든 선생님 한분 한분께 이렇게라도 감사인사를 전하게 되어 감사합니다._x000d_
 정말 감사 드립니다. _x000d_
- 누군가에겐 의미없는 말 한마디가 힘이 되기도 하고 상처가 되기도 합니다. 항상 힘이 되는 말을 해주신 선생님들께 감사드립니다.</v>
+ 누군가에겐 의미없는 말 한마디가 힘이 되기도 하고 상처가 되기도 합니다. 항상 힘이 되는 말을 해 주신 선생님들께 감사드립니다.</v>
       </c>
       <c r="J28" t="str">
-        <v>스트레스 없이 공부에만 집중할 수 있는 분위기를 조성해주셔서 감사했어요.</v>
+        <v>스트레스 없이 공부에만 집중할 수 있는 분위기를 조성해 주셔서 감사했어요.</v>
       </c>
       <c r="K28" t="str">
         <v/>
@@ -1436,7 +1436,7 @@
         <v>반수생</v>
       </c>
       <c r="E29" t="str">
-        <v>성적이 낮은 과목이 있었는데 저에게 알맞은  강의를 추천해 주셔서 많이 도움이 되었습니다 모의고사 성적표가 나올때마다 어떤 과목 중심으로 공부해야 효율적일지 같이 고민하고 상담해주셔서 좋았습니다</v>
+        <v>성적이 낮은 과목이 있었는데 저에게 알맞은  강의를 추천해 주셔서 많이 도움이 되었습니다 모의고사 성적표가 나올때마다 어떤 과목 중심으로 공부해야 효율적일지 같이 고민하고 상담해 주셔서 좋았습니다</v>
       </c>
       <c r="F29" t="str">
         <v>매일 플래너를 쓰니까 계획적으로 학습을 할수 있어서 좋았습니다.  플래너를 쓰지 않았을 때보다 더 체계적이고 효율적으로 공부할 수 있었습니다. 매일 플래너를 쓰다보니 습관이 되어서 공부 계획을 잘 세우게되었습니다</v>
@@ -1448,7 +1448,7 @@
         <v>독재는 자칫 자기 객관화가 부족해질 수 있는데 정기적인 모의고사를 통해 전국의 수험생 사이에서 내 현재 위치와 성적 추이를 정확히 분석하고 학습 방향을 수정할 수 있어 효율적이었습니다</v>
       </c>
       <c r="I29" t="str">
-        <v>선생님 1년정도의 기간동안 잘 코칭해주셔서 정말 감사했습니다ㅎㅎ 덕분에 수험기간 잘 버텨낼수 있었어용! 쌤덕분에 수능때 영어도 3등급 받아냈어요~~ 앞으로 행복하세요!! 독서도 열심히 할게요</v>
+        <v>선생님 1년정도의 기간동안 잘 코칭해 주셔서 정말 감사했습니다ㅎㅎ 덕분에 수험기간 잘 버텨낼수 있었어용! 쌤덕분에 수능때 영어도 3등급 받아냈어요~~ 앞으로 행복하세요!! 독서도 열심히 할게요</v>
       </c>
       <c r="J29" t="str">
         <v>플래너를 쓰지 않았을 때보다 더 체계적이고 효율적으로 공부할 수 있었어요.</v>
@@ -1519,7 +1519,7 @@
         <v>영단어는 수능영어를 위해선 빼먹을 수 없다고 생각하는데 이투스에선 매일매일 단어 테스트와 듣기 둘 다 테스트하여 실전에서도 많은 도움이 됐습니다 집에서 했다면 하루는 건너뛰었을 거 같은데 학원에서 매일 시험을 보니 영단어와 듣기평가가 익숙해져서 도움이 됐어요</v>
       </c>
       <c r="I31" t="str">
-        <v>처음에 갔을 땐 공부가 너무 힘들고 집중하기도 힘들었는데 좋은 말 해주셔서 감사했습니다 그리고 항상 친절하게 말해주시고 인사해주셔서 매일 기분이 좋았고 덕분에 공부도 잘 됐던 거 같아요 감사드립니다</v>
+        <v>처음에 갔을 땐 공부가 너무 힘들고 집중하기도 힘들었는데 좋은 말 해 주셔서 감사했습니다 그리고 항상 친절하게 말해 주시고 인사해 주셔서 매일 기분이 좋았고 덕분에 공부도 잘 됐던 거 같아요 감사드립니다</v>
       </c>
       <c r="J31" t="str">
         <v>철저한 출결 및 생활 관리 시스템 덕분에 나태해지지 않고 꾸준히 원하는 순공 시간을 달성했어요.</v>
@@ -1542,13 +1542,13 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E32" t="str">
-        <v>멘토샘들이 멘탈 관리를 잘 해주시고, 학습 피드백도 꼼꼼하게 해주셔서 부족한 부분을 정확히 알 수 있었습니다. 또 1년 동안 입시를 함께 준비하는 느낌이 들어서 심적으로도 많이 의지할 수 있었고 전반적으로 만족스러웠습니다.</v>
+        <v>멘토샘들이 멘탈 관리를 잘 해 주시고, 학습 피드백도 꼼꼼하게 해 주셔서 부족한 부분을 정확히 알 수 있었습니다. 또 1년 동안 입시를 함께 준비하는 느낌이 들어서 심적으로도 많이 의지할 수 있었고 전반적으로 만족스러웠습니다.</v>
       </c>
       <c r="F32" t="str">
         <v>1:1 질의응답 시간에 멘토 선생님들께서 항상 친절하게 응대해 주셔서 부담 없이 질문할 수 있었습니다. 이해가 안 되는 부분도 끝까지 자세히 설명해 주시고, 추가 질문에도 성의 있게 답해 주셔서 학습에 큰 도움이 되었고 만족도가 높았습니다.</v>
       </c>
       <c r="G32" t="str">
-        <v>면학 분위기 관리와 감독이 잘 이루어져서 학습에 집중하기 좋은 환경이었습니다. 특히 졸음 관리도 꼼꼼하게 해주셔서 흐트러지지 않고 공부할 수 있었고, 규칙적인 생활 습관을 유지하는 데에도 큰 도움이 되어 전반적으로 만족스러웠습니다.</v>
+        <v>면학 분위기 관리와 감독이 잘 이루어져서 학습에 집중하기 좋은 환경이었습니다. 특히 졸음 관리도 꼼꼼하게 해 주셔서 흐트러지지 않고 공부할 수 있었고, 규칙적인 생활 습관을 유지하는 데에도 큰 도움이 되어 전반적으로 만족스러웠습니다.</v>
       </c>
       <c r="H32" t="str">
         <v>이투스 구독 서비스를 무료로 이용할 수 있어서 경제적인 부담 없이 다양한 강의를 들을 수 있었던 점이 좋았습니다. 필요한 과목을 자유롭게 선택해 학습할 수 있었고, 자기주도적으로 공부할 수 있는 환경이 마련되어 있어 전반적인 학습 효율도 높아졌다고 느꼈습니다.</v>
@@ -1589,7 +1589,7 @@
         <v>특정 선생님 강의만 듣고 싶어서 따로 인강을 구매하기에는 부담이 있었는데, 학원에서 제공되는 이투스 인강 구독을 통해 추가 비용 없이 이용할 수 있어 좋았다. 덕분에 필요한 강의만 효율적으로 들을 수 있었고, 비용 부담 없이 학습에 집중할 수 있었다.</v>
       </c>
       <c r="I33" t="str">
-        <v>항상 세심하게 지도해주신 선생님들께 감사드립니다. 힘들 때마다 방향을 잡아주시고 꾸준히 격려해주신 덕분에 끝까지 포기하지 않고 공부할 수 있었습니다. 앞으로도 배운 것들을 바탕으로 더 노력하겠습니다.</v>
+        <v>항상 세심하게 지도해 주신 선생님들께 감사드립니다. 힘들 때마다 방향을 잡아주시고 꾸준히 격려해 주신 덕분에 끝까지 포기하지 않고 공부할 수 있었습니다. 앞으로도 배운 것들을 바탕으로 더 노력하겠습니다.</v>
       </c>
       <c r="J33" t="str">
         <v>감독 시스템이 있어 집중력을 유지하는 데 큰 도움이 되었어요.</v>
@@ -1617,7 +1617,7 @@
 그리고 매일 영단어 시험, 영어 듣기 테스트, 문제 질문첨삭 상담 등 코칭 시스템이 다양하고 풍부하여 유용하게 활용하였습니다</v>
       </c>
       <c r="F34" t="str">
-        <v>신뢰할 수 있는 대학생 멘토쌤과 언제든지 1:1 질의응답을 할 수 있는게 되게 유용했습니다. 문제에 관한 질문뿐만 아니라 학습법, 학습방향, 선택과목 설정 등 공부 고민에 대한 질문도 할 수 있다는게 좋았습니다. 실제로 6모 후 선택과목을 바꿀때 많은 도움이 되었고 그 외 걱정거리 또한 멘토샘들이 친절하게 상담해주셔서 많이 도움 받았습니다. 수험생이라면 1년 동안 공부 고민이 많을텐데 그때 1:1 질의응답을 이용해도 유용할 것 같습니다</v>
+        <v>신뢰할 수 있는 대학생 멘토쌤과 언제든지 1:1 질의응답을 할 수 있는게 되게 유용했습니다. 문제에 관한 질문뿐만 아니라 학습법, 학습방향, 선택과목 설정 등 공부 고민에 대한 질문도 할 수 있다는게 좋았습니다. 실제로 6모 후 선택과목을 바꿀때 많은 도움이 되었고 그 외 걱정거리 또한 멘토샘들이 친절하게 상담해 주셔서 많이 도움 받았습니다. 수험생이라면 1년 동안 공부 고민이 많을텐데 그때 1:1 질의응답을 이용해도 유용할 것 같습니다</v>
       </c>
       <c r="G34" t="str" xml:space="preserve">
         <v xml:space="preserve">혼자 공부할때 가장 힘든게 핸드폰, 태블릿 사용인데 학원에서 관리해주니 정말 좋았습니다. 공부할때 내내 감시받는 기분이라 딴짓은 절대 못하고 _x000d_
@@ -1627,11 +1627,11 @@
         <v>저같은 경우에는 영어단어 외우기가 굉장히 귀찮았고 실제로 영어 공부 시간 또한 현저히 적었습니다. 그러나 이투스247을 다니고나선 매일 VOCA 테스트를 보니깐 강제로 영어단어를 외우게 되어 좋았습니다. 매일 보는 단어테스트가 누적되어 수능날이 되면 결코 무시하지 못할 양의 단어를 외운 셈이고 또한 한권을 몇바퀴 돌리고 다음 단어책으로 넘어가 복습까지 자동으로 되었습니다.</v>
       </c>
       <c r="I34" t="str" xml:space="preserve">
-        <v xml:space="preserve">선생님들 모두모두 친절하게 대해주시고 생활 관리도 잘해주셔서 정말 감사했습니다.  덕분에 윈터스쿨, 썸머스쿨동안 공부 열심히 할 수 있었던 것 같습니다.  _x000d_
+        <v xml:space="preserve">선생님들 모두모두 친절하게 대해 주시고 생활 관리도 잘해 주셔서 정말 감사했습니다.  덕분에 윈터스쿨, 썸머스쿨동안 공부 열심히 할 수 있었던 것 같습니다.  _x000d_
 또한 인사도 잘 받아주시고 아침마다 반겨주시는 선생님들 덕분에 하루를 밝고 긍정적이게 시작할 수 있었습니다. 매일 똑같은 곳에서 똑같은 시간에 똑같이 공부하지만 친근하게 대해주시는 선생님들 덕분에 힘들지 않았던 것 같습니다. 감사합니다</v>
       </c>
       <c r="J34" t="str">
-        <v>선생님들 모두 친절하게 대해주시고 생활 관리도 잘해주셔서 정말 감사했어요.</v>
+        <v>선생님들 모두 친절하게 대해 주시고 생활 관리도 잘해 주셔서 정말 감사했어요.</v>
       </c>
       <c r="K34" t="str">
         <v>생활 관리</v>
@@ -1735,7 +1735,7 @@
       </c>
       <c r="I37" t="str" xml:space="preserve">
         <v xml:space="preserve">선생님께,_x000d_
-항상 제 학습 방향을 잘 잡아주시고 세심하게 지도해주셔서 정말 감사드립니다. 공부를 하면서 불안하고 흔들릴 때마다 진심으로 상담해주시고 따뜻하게 이끌어주셔서 큰 힘이 되었습니다. 덕분에 포기하지 않고 끝까지 해낼 수 있었습니다. 선생님의 응원과 조언 오래 기억하겠습니다. 진심으로 감사드립니다.</v>
+항상 제 학습 방향을 잘 잡아주시고 세심하게 지도해 주셔서 정말 감사드립니다. 공부를 하면서 불안하고 흔들릴 때마다 진심으로 상담해 주시고 따뜻하게 이끌어주셔서 큰 힘이 되었습니다. 덕분에 포기하지 않고 끝까지 해낼 수 있었습니다. 선생님의 응원과 조언 오래 기억하겠습니다. 진심으로 감사드립니다.</v>
       </c>
       <c r="J37" t="str">
         <v>면학 분위기가 잘 조성되어 있어 자연스럽게 집중할 수 있었어요.</v>
@@ -1773,7 +1773,7 @@
         <v>언제나 진심으로 최선을 다해서 학생들을 관리해 주셔서 감사합니다. 덕분에 알찬 일년을 보낼 수 있었던 것 같습니다. 만약 주변에서 독학재수 학원을 고민하는 지인이 있다면, 저는 고민없이 이투스247을 추천랄 것 같습니다.</v>
       </c>
       <c r="J38" t="str">
-        <v>저는 2주에 한 번씩 학습 상담을 받았었는데요, 상담을 받으면서 기피하는 과목을 가까이 하는 방법에 대해 많은 조언을 해주셨어요.</v>
+        <v>저는 2주에 한 번씩 학습 상담을 받았었는데요, 상담을 받으면서 기피하는 과목을 가까이 하는 방법에 대해 많은 조언을 해 주셨어요.</v>
       </c>
       <c r="K38" t="str">
         <v>학습 관리</v>
@@ -1806,7 +1806,7 @@
 두개씩 인강 패스를 끊기 많이 부담스러웠기 때문에 정말 좋았습니다.</v>
       </c>
       <c r="I39" t="str">
-        <v>안녕하세요 선생님! 이투스 학원을 다니면서 매번 감사했습니다. 형편없는 제 실력을 탓하지 않고 끝까지 응원해주셔서 감사합니다 비록 학교는 좋은 곳, 원하던 곳을 가지 않았지만 수능이라는 것을 제대로 준비해본 적이 없었는데 선생님들 덕분에 좋은 부분들 많이 배워갑니다!  정말 감사했습니다</v>
+        <v>안녕하세요 선생님! 이투스 학원을 다니면서 매번 감사했습니다. 형편없는 제 실력을 탓하지 않고 끝까지 응원해 주셔서 감사합니다 비록 학교는 좋은 곳, 원하던 곳을 가지 않았지만 수능이라는 것을 제대로 준비해본 적이 없었는데 선생님들 덕분에 좋은 부분들 많이 배워갑니다!  정말 감사했습니다</v>
       </c>
       <c r="J39" t="str">
         <v>계획 짜는 방법이나 공부 방법을 잘 몰라서 힘들었지만 선생님들의 조언과 말씀들 덕분에 공부를 어떻게 해야 하는지 알게 되었어요.</v>
@@ -1832,7 +1832,7 @@
         <v>기숙이라 여러모로 불편한 점이 많았는데 상담을 통해 격려와 응원을 받았고 시설 문제가 생겼을 때 대처해주려 노력하시는 부분이 좋았습니다…또한 타 학생의 방해행동에 대해 서로 불편하지 않는 선에서 해결해주셨습니다..</v>
       </c>
       <c r="F40" t="str">
-        <v>각 과목별로 담당 선생님께 질의응답을 신청하여 문제를 해결할 수 있었던 점이 좋았습니다. 특히 수학같은경우 담당 선생님께서 시간이 오버되면 또 다른 시간을 잡아서라도 끝까지 설명해주셔서 감사했습니다.</v>
+        <v>각 과목별로 담당 선생님께 질의응답을 신청하여 문제를 해결할 수 있었던 점이 좋았습니다. 특히 수학같은경우 담당 선생님께서 시간이 오버되면 또 다른 시간을 잡아서라도 끝까지 설명해 주셔서 감사했습니다.</v>
       </c>
       <c r="G40" t="str">
         <v>물론 방화벽을 뚫는 학생들도 보았습니다. 하지만 저는 막아둔 것에 의미가 있다고 생각하여 틀안에서 벗어나지 않으려했는데요, 인터넷에 노출되지않아 잡생각과 유혹등에 현혹되지않을수 있어서 좋았던 것 같습니다.</v>
@@ -1841,7 +1841,7 @@
         <v>자칫하면 타 과목을 공부하느라 단어를 놓치기 일수라고 생각합니다. 그런데 다 같이 단어를 시험보면서 강제성과 의무가 부여되니 자연스럽게 단어를 외우고 부담이 줄어들어 좋았습니다. 그리고 반복해서 단어시험을 치기때문에 독해력에도 도움이 된것같습니다.</v>
       </c>
       <c r="I40" t="str">
-        <v>비록 수능날에 긴장을 너무많이해서 실력발휘를 못한 것이 너무나 아쉽긴하지만, 실력은 확실히 늘었음을 체감할 수 있었습니다. 약 일년간 지도해주시느라 수고많으셨고 현역때의 아쉬움을 해결하고 넘어갈수있어서 좋았습니다. 서포트해주셔서 감사합니다.</v>
+        <v>비록 수능날에 긴장을 너무많이해서 실력발휘를 못한 것이 너무나 아쉽긴하지만, 실력은 확실히 늘었음을 체감할 수 있었습니다. 약 일년간 지도해주시느라 수고많으셨고 현역때의 아쉬움을 해결하고 넘어갈수있어서 좋았습니다. 서포트해 주셔서 감사합니다.</v>
       </c>
       <c r="J40" t="str">
         <v>각 과목별로 담당 선생님께 질의응답을 신청하여 문제를 해결할 수 있었던 점이 좋았어요.</v>
@@ -1864,10 +1864,10 @@
         <v>반수생</v>
       </c>
       <c r="E41" t="str">
-        <v>각 과목에서 어떤 인강이나 어떤 책을 풀어야하는지 자세하게 상담해주셔서 좋았어요 특히 영어 과목이 많이 부족했는데 수능특강 영어독해연습을 풀어보라고 하셔서 수능특강 위주로 학습을 했었고 지구과학도 실전 모의고사 추천 해주셔서 학습하는데 도움이 됐습니다</v>
+        <v>각 과목에서 어떤 인강이나 어떤 책을 풀어야하는지 자세하게 상담해 주셔서 좋았어요 특히 영어 과목이 많이 부족했는데 수능특강 영어독해연습을 풀어보라고 하셔서 수능특강 위주로 학습을 했었고 지구과학도 실전 모의고사 추천 해 주셔서 학습하는데 도움이 됐습니다</v>
       </c>
       <c r="F41" t="str">
-        <v>1주일에 한 번 씩 상담 선생님이랑 상담을 했었는데 부족한 점이나 잘하고 있는게 어떤건지 명확하게 설명해주셔서 좋았어요. 상담 간격도 텀이 길지 않고 1주일에 한 번이라서 좋았어요.</v>
+        <v>1주일에 한 번 씩 상담 선생님이랑 상담을 했었는데 부족한 점이나 잘하고 있는게 어떤건지 명확하게 설명해 주셔서 좋았어요. 상담 간격도 텀이 길지 않고 1주일에 한 번이라서 좋았어요.</v>
       </c>
       <c r="G41" t="str">
         <v>주변에 시끄러운 친구가 있을 때 피드백 반영이 빠르게 됐고 감독을 자주 하러 오셔서 졸지 않고 더 집중해서 공부할 수 있었어요. 거의 30분 간격으로 오셔서 자는 친구 있어도 바로바로 깨워주셔서 좋았어요.</v>
@@ -1876,7 +1876,7 @@
         <v>원래 구독했던 다른 인강 서비스가 있어서 이투스까지 구독하기엔 돈이 부족했는데 재원생이라 이투스패스를 들을 수 있었어요. 국어 김민정쌤의 ebs 정리집을 수능 2주 전부터 들었는데 깔끔하게 내용 정리할 수 있어서 좋았어요.</v>
       </c>
       <c r="I41" t="str">
-        <v>감독하러 여러번 오셔서 관리해주신 점이 가장 마음에 들어요. 그리고 시끄러운 친구들 컴플레인 넣으면 바로바로 해결해주시는 거 같아서 감사했습니다. 질문이나 조퇴할 때도 항상 나긋나긋한 말투로 말씀해주셔서 너무 감사했어요.</v>
+        <v>감독하러 여러번 오셔서 관리해 주신 점이 가장 마음에 들어요. 그리고 시끄러운 친구들 컴플레인 넣으면 바로바로 해결해주시는 거 같아서 감사했습니다. 질문이나 조퇴할 때도 항상 나긋나긋한 말투로 말씀해 주셔서 너무 감사했어요.</v>
       </c>
       <c r="J41" t="str">
         <v>주변에 시끄러운 친구가 있을 때 피드백 반영이 빠르게 됐고 감독을 자주 하러 오셔서 졸지 않고 더 집중해서 공부할 수 있었어요.</v>
@@ -1946,7 +1946,7 @@
         <v>솔직히 요즘 인강 가격대가 장난이 아닌데, 학원비까지 생각하면 정말 힘듭니다. 그래도 이투스에서 인강 구독을 지원해주니 조금이나마 마음 편하게 공부했습니다! 좋은 시스템이라고 생각합니다!</v>
       </c>
       <c r="I43" t="str">
-        <v>정말 감사했습니다!!!!!!!! 무리한 목표에도 현실적인 전략도 세워주시고, 항상 편안하고 재밌게 대해주셔서 정말 즐겁게 학원생활 했습니다! 다시 한 번 감사드립니다!!!!!!!!!!</v>
+        <v>정말 감사했습니다!!!!!!!! 무리한 목표에도 현실적인 전략도 세워주시고, 항상 편안하고 재밌게 대해 주셔서 정말 즐겁게 학원생활 했습니다! 다시 한 번 감사드립니다!!!!!!!!!!</v>
       </c>
       <c r="J43" t="str">
         <v>학생 개개인의 성적과 목표에 맞는 전략을 정말 구체적으로 세워주셨어요.</v>
@@ -1969,10 +1969,10 @@
         <v>N수생</v>
       </c>
       <c r="E44" t="str">
-        <v>재수 학원에서 담임 선생님이 1:1로 꾸준히 상담을 진행해주셔서 학습적인 부분뿐만 아니라 정신적으로도 큰 위로와 도움을 받을 수 있었습니다. 막연하게 느껴졌던 목표를 현실적으로 다시 설정할 수 있었고, 저의 부족한 부분을 구체적으로 짚어주셔서 하나씩 개선해 나갈 수 있었습니다. 덕분에 공부에 대한 방향성이 분명해지고 자신감도 많이 생겼습니다.</v>
+        <v>재수 학원에서 담임 선생님이 1:1로 꾸준히 상담을 진행해 주셔서 학습적인 부분뿐만 아니라 정신적으로도 큰 위로와 도움을 받을 수 있었습니다. 막연하게 느껴졌던 목표를 현실적으로 다시 설정할 수 있었고, 저의 부족한 부분을 구체적으로 짚어주셔서 하나씩 개선해 나갈 수 있었습니다. 덕분에 공부에 대한 방향성이 분명해지고 자신감도 많이 생겼습니다.</v>
       </c>
       <c r="F44" t="str">
-        <v>모르는 문제를 질문하면 바로바로 해결할 수 있어 학습의 흐름이 끊기지 않아 좋았습니다. 단순히 정답만 알려주는 것이 아니라 풀이 과정과 개념까지 꼼꼼하게 설명해주셔서 이해도를 높일 수 있었습니다. 덕분에 비슷한 유형의 문제에도 스스로 적용할 수 있는 힘이 길러졌고, 공부에 대한 자신감도 함께 생겼습니다.</v>
+        <v>모르는 문제를 질문하면 바로바로 해결할 수 있어 학습의 흐름이 끊기지 않아 좋았습니다. 단순히 정답만 알려주는 것이 아니라 풀이 과정과 개념까지 꼼꼼하게 설명해 주셔서 이해도를 높일 수 있었습니다. 덕분에 비슷한 유형의 문제에도 스스로 적용할 수 있는 힘이 길러졌고, 공부에 대한 자신감도 함께 생겼습니다.</v>
       </c>
       <c r="G44" t="str">
         <v>시간대별로 꾸준히 잠을 깨워주셔서 흐트러지지 않고 학습에 집중할 수 있었습니다. 덕분에 규칙적인 생활 습관도 함께 잡을 수 있었고 집중하는 시간도 점점 늘어서 학습에 도움이 많이 됐습니다.</v>
@@ -1981,7 +1981,7 @@
         <v>영어단어를 꾸준히 외우는게 생각보다 쉽지 않은데 학원에서 프린트물+테스트를 봐야해서 꾸준히 외울 수 있었던 거 같습니다. 또 중요단어들을 계속 볼 수 있어서 좋았습니다! 단어 외우는 습관을 잡을 수 있는게 가장 좋았어요</v>
       </c>
       <c r="I44" t="str">
-        <v>항상 친절하게 답해주시고 응원해주셔서 넘 감사했어용. 가끔 지칠 때도 있었는데 그때마다 진지하게 함께 고민해주시고 위로도 해주셨고 성적 올리는 데도 많은 도움 주셨습니다. 공부습관 잡는데 큰 도움 됐어요</v>
+        <v>항상 친절하게 답해 주시고 응원해 주셔서 넘 감사했어용. 가끔 지칠 때도 있었는데 그때마다 진지하게 함께 고민해 주시고 위로도 해주셨고 성적 올리는 데도 많은 도움 주셨습니다. 공부습관 잡는데 큰 도움 됐어요</v>
       </c>
       <c r="J44" t="str">
         <v>규칙적인 생활 습관도 함께 잡을 수 있었고 집중하는 시간도 점점 늘어서 학습에 도움이 많이 됐어요.</v>
@@ -2010,7 +2010,7 @@
         <v>일단 인강을 들어본 적이 없었지만 이투스에 있는 정승제,이지영 선생님들의 커리를 따라서 공부하다보니 성적을 올리는 데 수월했으며 선생님들께서 매 시간마다의 과제들을 다 알려주시다보니 따라가면 알아서 성적이 올랐던 것 같습니다</v>
       </c>
       <c r="G45" t="str">
-        <v>핸드폰을 수거함으로써 일단 자기주도학습과 집중력면에서 가장 성과를 많이 본 것 같은데 집중력이 제가 정말 안 좋은 편이였지만 핸드폰을 수거하고 선생님들이 학생들을 다 감시해주셔서 저도 혼자 공부하는 것보다 훨씬 높은 효율로 공부할 수 있었던 것 같습니다</v>
+        <v>핸드폰을 수거함으로써 일단 자기주도학습과 집중력면에서 가장 성과를 많이 본 것 같은데 집중력이 제가 정말 안 좋은 편이였지만 핸드폰을 수거하고 선생님들이 학생들을 다 감시해 주셔서 저도 혼자 공부하는 것보다 훨씬 높은 효율로 공부할 수 있었던 것 같습니다</v>
       </c>
       <c r="H45" t="str">
         <v>일단 이투스에 있는 모든 강좌를 무제한으로 볼 수 있었기에 정말 좋았고 또, 이투스는 다른 타사와는 달리 정말 싼 가격에 일타 강사 선생님들의 강의를 모두 수강할 수 있다는 점이 매우 좋다고 생각이 들어서 이투스 학원을 다니지 않을 때에도 계속 구독을 하였습니다</v>
@@ -2052,10 +2052,10 @@
         <v>수능까지 아직 시간이 많이 남은 경우이 한가지 과목만 공부하는 날이 많은데,  그런 날 다른과목을 최소한으로라도 학습량을 챙길수 있어서 감각이 떨어지지 않거나 덜 떨어트릴 수 있는 콘텐츠라고 생각합니다.</v>
       </c>
       <c r="I46" t="str">
-        <v>몸도 마음도 힘들었지만 재원하는동안 사정봐주시고 신경 써주셔서 너무 감사합니다. 저 같은 수험생은 보지않고 싶으실것 같습니다. 그래도 신경써주셔서 그나마 덜 힘들었습니다. 학생 개개인 별로 사정을 파악하고 조치를 취하시는게 어려울것 같습니다만 그렇게 해주셔서 감사합니다</v>
+        <v>몸도 마음도 힘들었지만 재원하는동안 사정봐주시고 신경 써주셔서 너무 감사합니다. 저 같은 수험생은 보지않고 싶으실것 같습니다. 그래도 신경써주셔서 그나마 덜 힘들었습니다. 학생 개개인 별로 사정을 파악하고 조치를 취하시는게 어려울것 같습니다만 그렇게 해 주셔서 감사합니다</v>
       </c>
       <c r="J46" t="str">
-        <v>성적뿐만 아니라 그 이외의 것들도 수험 생활에 집중할 수 있도록 상담해주셨어요.</v>
+        <v>성적뿐만 아니라 그 이외의 것들도 수험 생활에 집중할 수 있도록 상담해 주셨어요.</v>
       </c>
       <c r="K46" t="str">
         <v/>
@@ -2087,7 +2087,7 @@
         <v>이투스 패스를 제공해 인강 활용까지 가능하게 해준다. 다양한 강의를 자유롭게 들으며 부족한 과목을 보완할 수 있고, 현장 수업과 온라인 학습을 병행해 시너지 효과를 낼 수 있다. 덕분에 학습 선택의 폭이 넓어지고, 자기에게 맞는 방식으로 효율적인 공부가 가능해진다.</v>
       </c>
       <c r="I47" t="str">
-        <v>코칭과 세심한 관리 덕분에 흔들릴 때마다 다시 방향을 잡을 수 있었습니다. 늘 학생 입장에서 고민해주시고 도움 주셔서 진심으로 감사드립니다. 앞으로도 배운 습관과 방법을 잘 이어가 좋은 결과로 보답하겠습니다.</v>
+        <v>코칭과 세심한 관리 덕분에 흔들릴 때마다 다시 방향을 잡을 수 있었습니다. 늘 학생 입장에서 고민해 주시고 도움 주셔서 진심으로 감사드립니다. 앞으로도 배운 습관과 방법을 잘 이어가 좋은 결과로 보답하겠습니다.</v>
       </c>
       <c r="J47" t="str">
         <v>졸음 관리와 생활 습관 교정에도 큰 도움을 주었어요.</v>
@@ -2122,7 +2122,7 @@
         <v>아무리 현장 강의보다 인터넷 강의가 더 싸다고 하지만 과목이 엄청 많은 만큼 타 인강 사이트 선생님들도 듣게 되는데 이투스 247을 다니면 이투스 인강사이트를 무료로 이용할 수 있다는 점에서 너무 좋았습니다</v>
       </c>
       <c r="I48" t="str">
-        <v>그동안에 좀 바보 같은 질문을 많이 했던거 같은데 그때마다 잘 알려주셔서 정말 감사했습니다. 이투스  247 다니면서 학습방법과 지금은 퇴보했지만 집중력을 높일 수 있었고 너무 친절하고 친근하게 대해주셔서 잘 다닐 수 있었던 것 같습니다</v>
+        <v>그동안에 좀 바보 같은 질문을 많이 했던거 같은데 그때마다 잘 알려주셔서 정말 감사했습니다. 이투스  247 다니면서 학습방법과 지금은 퇴보했지만 집중력을 높일 수 있었고 너무 친절하고 친근하게 대해 주셔서 잘 다닐 수 있었던 것 같습니다</v>
       </c>
       <c r="J48" t="str">
         <v>학습 상담뿐만 아니라 졸음을 느낄 때, 집중력이 흐려질 때 등 생활 상담으로 해답을 주셔서 좋았어요.</v>
@@ -2148,7 +2148,7 @@
         <v>매월 진행되는 사설 모의고사와 평가원 모의고사의 분석지를 토대로 정확한 수치와 데이터를 기반으로 한 공부 방법 점검과 나아가야할 방향성을 제시해 주셔서 좋았다. 또한 상담을 주기적으로 하면서 나의 현재 위치를 알고 계속하여 마음을 다 잡을 수 있었다</v>
       </c>
       <c r="F49" t="str">
-        <v>매일 작성하는 일간 학습 플래너를 토대로 하교시 제출 후, 다음날 바로 바로 피드백을 해주셔서 좋았다. 놓치고 있는 부분을 보완할 수 있도록 바로 바로 체크해 주시고 진도나간 부분을 다시 한번 복습할 수 있는 시스템이 좋았다</v>
+        <v>매일 작성하는 일간 학습 플래너를 토대로 하교시 제출 후, 다음날 바로 바로 피드백을 해 주셔서 좋았다. 놓치고 있는 부분을 보완할 수 있도록 바로 바로 체크해 주시고 진도나간 부분을 다시 한번 복습할 수 있는 시스템이 좋았다</v>
       </c>
       <c r="G49" t="str">
         <v>매 시간 선생님들께서 돌아다니시면서 조는 친구들을 깨워주시니 자연스럽게 면학 분위기도 잡혀서 좋았다. 또한 와이파이 방화벽 시스템을 통해, 자칫 자제하기 힘들뻔한 인터넷 사용을 강제적으로 막아주어 마음을 다잡고 재수 생활을 보낼 수 있었다</v>
@@ -2158,10 +2158,10 @@
       </c>
       <c r="I49" t="str" xml:space="preserve">
         <v xml:space="preserve">의지가 부족했던 저를 앞으로 나아갈 수 있도록 이끌어주셔서 감사합니다. _x000d_
-어려움이 있어서 찾아갔을 때에도 저와 함께 최선의 방법으로 갈 수 있도록 진심을 다해 상담해주셔서 많은 용기 얻을 수 있었습니다. 재수뿐만 아니라 인생에서도 지치지 않고 나아갈 수 있는 방법을 배운 한 해 였습니다 :)</v>
+어려움이 있어서 찾아갔을 때에도 저와 함께 최선의 방법으로 갈 수 있도록 진심을 다해 상담해 주셔서 많은 용기 얻을 수 있었습니다. 재수뿐만 아니라 인생에서도 지치지 않고 나아갈 수 있는 방법을 배운 한 해 였습니다 :)</v>
       </c>
       <c r="J49" t="str">
-        <v>어려움이 있어서 찾아갔을 때에도 최선의 방법으로, 진심을 다해 상담해주셔서 많은 용기를 얻을 수 있었어요.</v>
+        <v>어려움이 있어서 찾아갔을 때에도 최선의 방법으로, 진심을 다해 상담해 주셔서 많은 용기를 얻을 수 있었어요.</v>
       </c>
       <c r="K49" t="str">
         <v/>
@@ -2193,7 +2193,7 @@
         <v>이투스 패스가 지원되어 인강 선택의 폭이 넓어 자신에게 맞는 수업 스타일을 가진 인강 선생님을 찾는데 도움이 되어 인강 수강과 자기주도 학습의 밸런스를 완벽하게 맞출 수 있었습니다. 친절한 상담과 확실한 관리, 좋은 혜택까지 모두 만족스럽습니다</v>
       </c>
       <c r="I50" t="str">
-        <v>선생님들 항상 친절하게 격려해주셔서 정말 감사했습니다. 덕분에 걱정이 줄고 공부에 더 집중할 수 있게 되었던 거 같아요. 세심한 상담 덕분에 수험 생활의 중심을 잘 잡게 되었습니다. 체계적인 관리와 분위기 너무 좋았습니다. 그동안 정말 감사했습니다~</v>
+        <v>선생님들 항상 친절하게 격려해 주셔서 정말 감사했습니다. 덕분에 걱정이 줄고 공부에 더 집중할 수 있게 되었던 거 같아요. 세심한 상담 덕분에 수험 생활의 중심을 잘 잡게 되었습니다. 체계적인 관리와 분위기 너무 좋았습니다. 그동안 정말 감사했습니다~</v>
       </c>
       <c r="J50" t="str">
         <v>친절한 상담으로 멘탈을 잡아주시면서도, 공부할 때는 확실하게 관리해 주시는 시스템 덕분에 효율적으로 성적을 올릴 수 있었어요.</v>
@@ -2252,20 +2252,20 @@
       </c>
       <c r="E52" t="str" xml:space="preserve">
         <v xml:space="preserve">국어가 맨날 5~6등급이었지만 국어 멘토링 덕분에 2~4등급은 안정적으로 받을 수 있는 수준으로 발전하였다_x000d_
-또한 탐구를 담임 선생님께서 잘 체크해주셔서 빠뜨리지 않고 잘 공부할 수있었다</v>
+또한 탐구를 담임 선생님께서 잘 체크해 주셔서 빠뜨리지 않고 잘 공부할 수있었다</v>
       </c>
       <c r="F52" t="str" xml:space="preserve">
         <v xml:space="preserve">오늘 할일을 처음 아침에 앉아 생각해볼수있었고 그것을 실천하여_x000d_
 최대한의 효율과 무리를 하지않고 공부할 수있었던것 같다 또한 공부끝나고 오늘 한일을 체크하고 피드백하는과정에서 부족한부분도 체크할수있어서 좋았다</v>
       </c>
       <c r="G52" t="str">
-        <v>개인적으로 잠이 많고 졸음이 많은데 선생님께서 졸지말라고 잘 깨워주셨고 다른 좌석에서 친구들이 잘때소리나는 코고는소리 숨소리를 모두 체크해주셔서 면학 분위기에 좋은 영향을 끼칠수있었던것 같다</v>
+        <v>개인적으로 잠이 많고 졸음이 많은데 선생님께서 졸지말라고 잘 깨워주셨고 다른 좌석에서 친구들이 잘때소리나는 코고는소리 숨소리를 모두 체크해 주셔서 면학 분위기에 좋은 영향을 끼칠수있었던것 같다</v>
       </c>
       <c r="H52" t="str">
         <v>개인적으로 영어란과목에서 단어 암기가 좀 많이 부족하고 듣기평가를 볼때도 항상 1,2개씩틀렸다 절대평가인 영어란 과목특이상 듣기를 틀린다는것은 1,2등급에 굉장한 영향을 끼칠수있기때문에 아침에 계속 테스트를 거르지않고 본결과 26수능 듣기를 다맞을수있었다</v>
       </c>
       <c r="I52" t="str">
-        <v>모든 선생님들 지도해주셔서 감사했습니다 특히 태민선생님 상담 잘해주시고 피드백 잘해주셔서 감사했습니다 찾아뵙고싶었는데 못찾아뵈었네요 죄송합니다 다음에 기회가 된다면 꼭 찾아뵙고싶습니다</v>
+        <v>모든 선생님들 지도해 주셔서 감사했습니다 특히 태민선생님 상담 잘해 주시고 피드백 잘해 주셔서 감사했습니다 찾아뵙고싶었는데 못찾아뵈었네요 죄송합니다 다음에 기회가 된다면 꼭 찾아뵙고싶습니다</v>
       </c>
       <c r="J52" t="str">
         <v>6등급이었지만 국어 멘토링 덕분에 2~4등급은 안정적으로 받을 수 있는 수준으로 발전하였어요.</v>
@@ -2326,7 +2326,7 @@
         <v>단순히 출석 확인만 하고 생활적 부분에만 관리를 했다면 학교 등록에 있어서 고민을 좀 했을 거 같습니다 하지만 일주일에 한 번씩 저의 그동안의 학습 방향에 있어서 올바른 지도와 멘탈적 관리 그리고 컨텐츠적으로 여러가지 선택지를 제시해 주시니 제가 그동안 잘못 공부하고 있던 것들을 효율적으로 교정하는 것에 있어서 여러 도움을 받았습니다</v>
       </c>
       <c r="F54" t="str">
-        <v>요즘 인강과 같이 컨텐츠적으로 부족함이 없다고 생각이 들 정도로 포화 상태라고 생각이 들지만 궁금한 부분을 해결하는것에 있어서 아직은 온라인 강의가 부족하다고 생각이 들었는데 학원 1대1 질의응답 시스템은 단순히 문제를 풀어주시는 것이 아닌 제가 제 질문 과정에 있어서 선생님들이 저의 어떤것들을 잘못 하고 어떤것을 잘했는지 꼼꼼히 설명 해주시고 앞으로의 방향까지 설정해주시니 인강으로만 공부했을때 부족한 부분을 해결해줘서 저는 가장 만족하는 컨텐츠라고 생각합니다</v>
+        <v>요즘 인강과 같이 컨텐츠적으로 부족함이 없다고 생각이 들 정도로 포화 상태라고 생각이 들지만 궁금한 부분을 해결하는것에 있어서 아직은 온라인 강의가 부족하다고 생각이 들었는데 학원 1대1 질의응답 시스템은 단순히 문제를 풀어주시는 것이 아닌 제가 제 질문 과정에 있어서 선생님들이 저의 어떤것들을 잘못 하고 어떤것을 잘했는지 꼼꼼히 설명 해 주시고 앞으로의 방향까지 설정해주시니 인강으로만 공부했을때 부족한 부분을 해결해줘서 저는 가장 만족하는 컨텐츠라고 생각합니다</v>
       </c>
       <c r="G54" t="str">
         <v>오전 오후 하루 두 번 20분 수면 관리는 매우 인상적이였습니다 다른곳은 정해진 시간에 잘 수 있는 시간이 있다고 하는데 이는 사실 효율적이라고 생각하지 않습니다 자기가 정말 필요로 할 때 이용할 수 있는 유연한 제도가 좋았고 면학 분위기 관리에 있어서 실장님도 유연하게 학생들을 관리해 주셔서 좋았습니다</v>
@@ -2405,7 +2405,7 @@
         <v>영단어 외우는 건 항상 뒤로 미뤄 스트레스를 받았었는데 의무적으로 보는 단어 테스트 덕분에 꾸준히 영단어를 학습하게 된 것이 마음에 들었음. 영어성적 향상에 직접적인 영향을 주어 만족스러웠음.</v>
       </c>
       <c r="I56" t="str">
-        <v>이투스 선생님들 좋은 면학 분위기를 위해 노력해주시고 훌륭한 지도 해주셔서 감사합니다. 덕분에 성적 향상과 좋은 습관을 얻은 것 같습니다. 후배들이나 다시 도전하는 친구들에게 좋을 말 많이 전할게요</v>
+        <v>이투스 선생님들 좋은 면학 분위기를 위해 노력해 주시고 훌륭한 지도 해 주셔서 감사합니다. 덕분에 성적 향상과 좋은 습관을 얻은 것 같습니다. 후배들이나 다시 도전하는 친구들에게 좋을 말 많이 전할게요</v>
       </c>
       <c r="J56" t="str">
         <v>플래너 점검을 통해 해야 할 일을 한눈에 정리하는 습관이 생겨 수험 생활에 큰 도움이 되었어요.</v>
@@ -2428,10 +2428,10 @@
         <v>N수생</v>
       </c>
       <c r="E57" t="str">
-        <v>매달 담당 선생님이 직접 찾아오셔서 부르셔서 학습 과제 학습 진행 상태 등을 직접 점검해주시고 직접 과목마다 인터넷강의 강사와 교재등을 추천해 주시고 가끔 간식같은것도 챙겨주시고 덕담,응원의 말들을 많이 해주셔서 많이 힘이 됐습니다.</v>
+        <v>매달 담당 선생님이 직접 찾아오셔서 부르셔서 학습 과제 학습 진행 상태 등을 직접 점검해 주시고 직접 과목마다 인터넷강의 강사와 교재등을 추천해 주시고 가끔 간식같은것도 챙겨주시고 덕담,응원의 말들을 많이 해 주셔서 많이 힘이 됐습니다.</v>
       </c>
       <c r="F57" t="str">
-        <v>학습 관리를 담당 선생님이 세심하게 해주시고 모의고사 끝날때마다 4층으로 부르셔서 각 과목 담당 선생님이 시험난이도나 등급컷 어려운 문제 해설 등등을 해주셔서 도움이 많이 되었습니다. 그리고 제가 졸거나 집중 못하고있을때 확인하셔서 깨워주시는게 도움되었습니다.</v>
+        <v>학습 관리를 담당 선생님이 세심하게 해 주시고 모의고사 끝날때마다 4층으로 부르셔서 각 과목 담당 선생님이 시험난이도나 등급컷 어려운 문제 해설 등등을 해 주셔서 도움이 많이 되었습니다. 그리고 제가 졸거나 집중 못하고있을때 확인하셔서 깨워주시는게 도움되었습니다.</v>
       </c>
       <c r="G57" t="str">
         <v>생활 관리 시스템중에서 특히 유용했던점은 전자출결 시스템을 이용해서 일일이 확인하는일이 없어 서로 번거로운일 없이 출석체크가 가능합니다. 그리고 외출하거나 조퇴하는 일이 있을때 일일이 담당 선생님께 말씀드리고 확인받고 갈 필요없이 전자출결로 조회를 해놓으면 되니 매우 편리하고 도움이 많이되는 시스템이었다고 생각되었습니다.</v>
@@ -2440,7 +2440,7 @@
         <v>교육청,평가원에서 실시하는 전국 모의고사 뿐만이 아니라 이투스 학원에서 제공하는 이투스 모의고사를 추가로 풀고 답을 확인하고 해설을 들으니 더 철저히 수능을 준비할수 있었고 모르는 개념도 추가로 확인하고 얻어갈수있었고 시험을 여러번 보다보니 수능 당일날 크게 긴장하지 않는 마인드셋을 가질수있었던것 같습니다.</v>
       </c>
       <c r="I57" t="str">
-        <v>학원에 있는동안 친절하게 도와주시고 응원해주셔서 감사합니다! 국어 선생님은 항상 친절하게 문학,독서 관련 팁들을 알려주셔서 도움이 많이 되었고 수학 선생님은 본인도 n수 경험이 있다며 현실적인 경험담과 조언을 많이 해주셨고 영어 선생님은 제 담임 선생님으로써 많이 케어해주셨습니다 모두 도움이 많이 되었습니다 늘 감사합니다!</v>
+        <v>학원에 있는동안 친절하게 도와주시고 응원해 주셔서 감사합니다! 국어 선생님은 항상 친절하게 문학,독서 관련 팁들을 알려주셔서 도움이 많이 되었고 수학 선생님은 본인도 n수 경험이 있다며 현실적인 경험담과 조언을 많이 해주셨고 영어 선생님은 제 담임 선생님으로써 많이 케어해주셨습니다 모두 도움이 많이 되었습니다 늘 감사합니다!</v>
       </c>
       <c r="J57" t="str">
         <v>전자출결 시스템 덕분에 번거로운 확인 과정 없이 편하게 출석 체크를 할 수 있었어요.</v>
@@ -2525,7 +2525,7 @@
 또한 외운 단어가 실제로 지문에 나왔을때 기분도 좋고 해석이 원활히 되는걸 보고 더 열심히 하게 돼 좋은 학습 콘텐츠라고 생각합니다</v>
       </c>
       <c r="I59" t="str" xml:space="preserve">
-        <v xml:space="preserve">한명한명 학생들에게 친절하게 대해주시고 언제나 필요한 부분이 있다면 최대한 도와주시려는 모습들 모두 감사했습니다_x000d_
+        <v xml:space="preserve">한명한명 학생들에게 친절하게 대해 주시고 언제나 필요한 부분이 있다면 최대한 도와주시려는 모습들 모두 감사했습니다_x000d_
 선생님들의 관리가 없었다면 아마 해이해지는 순간들이 더 많았을거 같습니다_x000d_
 선생님들도 아침부터 밤까지 일하시면서 피곤하실때도 있고 쉬고 싶을때도 있을테지만 저희 학생들을 위해서 매일매일 관리해주시는 모습들은 아직 기억이 날 정도로 감사했습니다_x000d_
 수능을 위해 같이 달려온 날들이 결코 짧지 않았고 그만큼 선생님들에게 감사한 마음은 작지 않습니다_x000d_
@@ -2564,7 +2564,7 @@
         <v>너무 어려운 문제들도 아니고 개념을 이해하고 풀기에 좋다고 생각해서 개념 이해에 대한 확인 용도로 풀기에 좋았다 또 해설도 제공해주어서 완벽하게 이해한 후에 넘어갈 수 있어서 도움이 되었다</v>
       </c>
       <c r="I60" t="str">
-        <v>저희의 학업능력 증진을 위해 노력해주셔서 감사합니다 사소한 부분들이 모여서 정말 큰 도움이 되었고 공부습관을 고칠 수 있어 더 효율적이게 공부할 수 있었던 것 같습니다 그리 긴 시간은 아니었지만 이투스에서 공부할 때 제일 집중도 잘 되었던 것 같습니다</v>
+        <v>저희의 학업능력 증진을 위해 노력해 주셔서 감사합니다 사소한 부분들이 모여서 정말 큰 도움이 되었고 공부습관을 고칠 수 있어 더 효율적이게 공부할 수 있었던 것 같습니다 그리 긴 시간은 아니었지만 이투스에서 공부할 때 제일 집중도 잘 되었던 것 같습니다</v>
       </c>
       <c r="J60" t="str">
         <v>1:1 상담과 스케줄 관리, 태블릿 제한 덕분에 효율적인 공부 습관을 만들 수 있었어요.</v>
@@ -2594,16 +2594,16 @@
 수학또한 강사님을 먼저 골라주시고 거기서 저의 수준에 맞게 강의를 골라주셔서 그나마 더 나은 성적이 나오게 되었습니다.</v>
       </c>
       <c r="G61" t="str">
-        <v>제가 핸드폰을 많이 보는데 핸드폰을 수거해감으로서 다른 불필요한 요소등을 제거해주셔서 그나마 공부에 더 집중을 할 수 있게 해주셔서 핸드폰 수거가 좋다고 느꼈습니다. 잠을 많이 조는 편인데 잠도 깨워주셔서 그나마 더 공부를 했습니다.</v>
+        <v>제가 핸드폰을 많이 보는데 핸드폰을 수거해감으로서 다른 불필요한 요소등을 제거해 주셔서 그나마 공부에 더 집중을 할 수 있게 해 주셔서 핸드폰 수거가 좋다고 느꼈습니다. 잠을 많이 조는 편인데 잠도 깨워주셔서 그나마 더 공부를 했습니다.</v>
       </c>
       <c r="H61" t="str">
-        <v>달마다 시험을 봄으로써 자신의 수준이 어느정도인지 깨닫게 해주시고 공부 방향을 다시 잡게 해주는 졸은 경험이었던 것 같습니다. 그걸 통해서 사설로 새로운 경향을 문제로 풀어보고 복습해보는 좋은 시럼이었습니다.</v>
+        <v>달마다 시험을 봄으로써 자신의 수준이 어느정도인지 깨닫게 해 주시고 공부 방향을 다시 잡게 해주는 졸은 경험이었던 것 같습니다. 그걸 통해서 사설로 새로운 경향을 문제로 풀어보고 복습해보는 좋은 시럼이었습니다.</v>
       </c>
       <c r="I61" t="str">
         <v>잠을 너무 많이 졸았는데 항상 깨워주셔서 감사했습니다.. 그덕에 한 과목이라도 1등급이 나왔습니다. 그리고 한국지리 알려주신 선생님 너무 감사합니다. 선생님 덕에 1등급이 나왔습니다!!</v>
       </c>
       <c r="J61" t="str">
-        <v>수준에 맞는 수학 강의 추천을 해주셔서 성적 향상에 도움을 받았어요.</v>
+        <v>수준에 맞는 수학 강의 추천을 해 주셔서 성적 향상에 도움을 받았어요.</v>
       </c>
       <c r="K61" t="str">
         <v/>
@@ -2638,7 +2638,7 @@
 꾸준한 테스트 덕분에 암기 효율이 높아지고, 영어 실력 향상에도 큰 도움이 되었습니다</v>
       </c>
       <c r="I62" t="str">
-        <v>항상 세심하게 지도해주시고 올바른 방향을 잡아주셔서 진심으로 감사드립니다. 덕분에 공부에 대한 이해도가 높아지고, 학습에 더욱 집중할 수 있게 되었습니다. 또한 꾸준히 노력할 수 있는 습관도 기를 수 있어 전반적인 실력 향상에 큰 도움이 되었습니다!</v>
+        <v>항상 세심하게 지도해 주시고 올바른 방향을 잡아주셔서 진심으로 감사드립니다. 덕분에 공부에 대한 이해도가 높아지고, 학습에 더욱 집중할 수 있게 되었습니다. 또한 꾸준히 노력할 수 있는 습관도 기를 수 있어 전반적인 실력 향상에 큰 도움이 되었습니다!</v>
       </c>
       <c r="J62" t="str">
         <v>학습 상담을 받으면서 제 상태를 객관적으로 돌아볼 수 있었고, 멘탈을 정리하는 데 큰 도움이 되었어요.</v>
@@ -2673,10 +2673,10 @@
         <v>이투스에서 단어 관리를 받았을때 처음에는 이게 맞나 싶었지만 6모를 보고 9모를 보면서 아는 영단어도 다른 의미를 알 수 있게 되며 이로 인해 영어 실력을 향상 시킬 수 있었다. 또한 검사를 받기 때문에 대충할 위험도 없다</v>
       </c>
       <c r="I63" t="str">
-        <v>할수 있다고, 갈수 있다고, 수고했다고 항상 응원해주시고 다독여주셔서 감사합니다!  옆에서 도움받지 않고서는 절대 혼자 못했을 결과받게 해주셔서 감사합니다. 비록 원하는 결과는 아니지만  앞으로의 인생에서 도움이 될 값진 경험이었습니다!</v>
+        <v>할수 있다고, 갈수 있다고, 수고했다고 항상 응원해 주시고 다독여주셔서 감사합니다!  옆에서 도움받지 않고서는 절대 혼자 못했을 결과받게 해 주셔서 감사합니다. 비록 원하는 결과는 아니지만  앞으로의 인생에서 도움이 될 값진 경험이었습니다!</v>
       </c>
       <c r="J63" t="str">
-        <v>옆에서 도움받지 않고서는 절대 혼자 못했을 결과를 받게 해주셔서 감사해요.</v>
+        <v>옆에서 도움받지 않고서는 절대 혼자 못했을 결과를 받게 해 주셔서 감사해요.</v>
       </c>
       <c r="K63" t="str">
         <v/>
@@ -2709,7 +2709,7 @@
         <v>이투스 전국모의고사라는 모의고사를 통해 현재 나의 실력을 객관적으로 확인할 수 있었고, 부족한 부분이 무엇인지 구체적으로 파악할 수 있었습니다. 특히 실제 시험과 유사한 환경에서 문제를 풀어보면서 시간 관리 능력과 문제 해결 전략을 점검할 수 있었고, 이후 학습 방향을 설정하는 데에도 큰 도움이 되었습니다.</v>
       </c>
       <c r="I64" t="str">
-        <v>감사합니다선생님께 진심으로 감사드립니다. 항상 세심하게 지도해주시고, 공부 방향을 잡을 수 있도록 도와주신 덕분에 혼자서도 흔들리지 않고 꾸준히 공부할 수 있었습니다. 부족한 부분을 정확하게 짚어주시고 응원해주신 덕분에 큰 힘이 되었고, 앞으로도 더 열심히 해서 좋은 결과로 보답하겠습니다.</v>
+        <v>감사합니다선생님께 진심으로 감사드립니다. 항상 세심하게 지도해 주시고, 공부 방향을 잡을 수 있도록 도와주신 덕분에 혼자서도 흔들리지 않고 꾸준히 공부할 수 있었습니다. 부족한 부분을 정확하게 짚어주시고 응원해 주신 덕분에 큰 힘이 되었고, 앞으로도 더 열심히 해서 좋은 결과로 보답하겠습니다.</v>
       </c>
       <c r="J64" t="str">
         <v>학습 기록과 계획 확인을 반복하면서 스스로를 관리하는 힘이 생겼고, 공부 흐름을 꾸준히 유지할 수 있었어요.</v>
@@ -2767,7 +2767,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E66" t="str">
-        <v>과목 별 선생님분들께서 친절히 수준에 맞게 앞으로의 학습방향에 대해 달 코칭해주시고 모르는것에 대한 질문들을 잘 설명해주셨습니다.    또한 학습할때의 불편한 것이 있는지 항상 확인해주시고 계속 신경써주셔서 편한 환경에서 공부를 할 수 있었습니다</v>
+        <v>과목 별 선생님분들께서 친절히 수준에 맞게 앞으로의 학습방향에 대해 달 코칭해 주시고 모르는것에 대한 질문들을 잘 설명해주셨습니다.    또한 학습할때의 불편한 것이 있는지 항상 확인해 주시고 계속 신경써주셔서 편한 환경에서 공부를 할 수 있었습니다</v>
       </c>
       <c r="F66" t="str">
         <v>베이스가 없는상태에서 시작했는데 이투스뿐만 아니라 다른 사이트 강사 선생님들을 저의 성향에 맞게 추천해주셨던것 같습니다.                                  .</v>
@@ -2808,13 +2808,13 @@
         <v>혼자서 하면 모르는것을 질문하기 어렵습니다. 인강의 QnA질문을 해도 빨라도 하루는 걸리는 질의응답을 실시간으로 궁굼한 점이 생기면 바로바로 질문하고 답변받을 수 있어서 좋았습니다.</v>
       </c>
       <c r="G67" t="str">
-        <v>먼저 핸드폰을 수거해서 좋았습니다. 또 핸드폰이 없어도 패드로도 딴 짓을 할 수 있는데 와이파이 방화벽으로 그것도 관리할 수 있어서 좋았습니다. 또 선생님께서 주기적으로 돌아다니시면서 졸거나 그럴때 깨워주시고 면학 분위기 유지하기위해 노력해주셔서 좋았습니다</v>
+        <v>먼저 핸드폰을 수거해서 좋았습니다. 또 핸드폰이 없어도 패드로도 딴 짓을 할 수 있는데 와이파이 방화벽으로 그것도 관리할 수 있어서 좋았습니다. 또 선생님께서 주기적으로 돌아다니시면서 졸거나 그럴때 깨워주시고 면학 분위기 유지하기위해 노력해 주셔서 좋았습니다</v>
       </c>
       <c r="H67" t="str">
         <v>이투스에 듣고싶은 강사가 있었는데 한분만 듣고싶어서  구독하기에는 부담이 되는 상황이였습니다 그런데 이투스247를 다니면 이투스구독 서비스가 제공되어서 강의를 듣게 되어서 좋았습니다.</v>
       </c>
       <c r="I67" t="str">
-        <v>1년 동안 감사했습니다. 출결 관리도 해주시고 졸거나 집중안될 때 도와주시고 면학 분위기 조성해주셔서 감사했습니다. 이것저것 도움되라고 간식등 챙겨주신것도 감사합니다. 일상에서 간간히 대화했던 것도 힘들지않고 공부하는데 도움많이됐습니다 감사합니다!</v>
+        <v>1년 동안 감사했습니다. 출결 관리도 해 주시고 졸거나 집중안될 때 도와주시고 면학 분위기 조성해 주셔서 감사했습니다. 이것저것 도움되라고 간식등 챙겨주신것도 감사합니다. 일상에서 간간히 대화했던 것도 힘들지않고 공부하는데 도움많이됐습니다 감사합니다!</v>
       </c>
       <c r="J67" t="str">
         <v>졸리거나 집중력이 흐트러질 때 도와주셔서 좋은 면학 분위기 속에서 공부할 수 있었어요.</v>
@@ -2878,7 +2878,7 @@
         <v>자기가 무슨 인강을 들어야할지 처음엔 감이 안잡힐 때가 많은데 제 성적과 학습 수준에 따라서 어떤 교재와 인강을 들어야할지 추천해 주셔서 좋았습니다. 방향을 잡는데 많이 도움되었다고 생각해요</v>
       </c>
       <c r="G69" t="str">
-        <v>핸드폰이 진짜 수능 준비에 가장 방해가 많이 되는 물품이라고 생각하는데, 이렇게 확실하게 강제성을 주니까 공부에만 집중하게 될 수 있는 환경이 만들어져서 정말 좋았습니다. 졸음도 가끔 들어오셔서 돌아다니시면서 깨워주시는데 그것 덕에 졸음도 깨고 공부 집중에 도움이 되었습니다.</v>
+        <v>핸드폰이 진짜 수능 준비에 가장 방해가 많이 되는 물품이라고 생각하는데, 이렇게 확실하게 강제성을 주니까 공부에만 집중하게 될 수 있는 환경이 만들어져서 정말 좋았습니다. 졸음도 가끔 들어오셔서 돌아다니시면서 깨워주시는데 그 덕분에 졸음도 깨고 공부 집중에 도움이 되었습니다.</v>
       </c>
       <c r="H69" t="str">
         <v>아무래도 모의고사이다 보니까 실전 연습을 자주하게 되어서 수능 시험에 많이 익숙해지도록 하게 되었던 것 같습니다. 물론 학원 내, 자기 자리에서 하는 시험이다보니 실질적으로 수능 시험장에서의 긴장감만큼 긴장이 되진 않지만, 실전 연습이라는 점에서 메리트가 상당하다고 생각합니다.</v>
@@ -2887,7 +2887,7 @@
         <v>1년 동안 수능 공부 도와주시고 학원 생활 잘하게끔 많이 이끌어주시고 도와주셔서 감사하다고 말씀 드리고 싶어요. 대학에 지금은 합격해서 다니고 있고, 적응 잘해서 졸업까지 무사히 달려가 앞으로 열심히 인생 살아가보겠습니다. 1년 동안 감사했습니다.</v>
       </c>
       <c r="J69" t="str">
-        <v>돌아다니시면서 깨워주시는데 그것 덕에 졸음도 깨고 공부 집중에 도움이 되었어요.</v>
+        <v>돌아다니시면서 깨워주시는데 그 덕분에 졸음도 깨고 공부에 집중하는 데 도움이 되었어요.</v>
       </c>
       <c r="K69" t="str">
         <v/>
@@ -2916,7 +2916,7 @@
         <v>학습 시간 도중 딴짓을 하지 못하게 방화벽으로 외부 사이트가 차단되어있었으나 일부 막히지않은 사이트, 또는 개인적으로 집중력이 너무 흐려져서 딴짓을 하게된 순간이 몇 번 있었는데 선생님들이 교시마다 돌아다니며 학생들을 점검한 점이 매우 좋았습니다. 또한 식곤증이나 아침잠이 왔을 때도 졸지 않게 깨워주셔서 잘 공부할 수 있었던 것 같습니다. 복도의 스탠딩 책상을 이용할 수 있는 점도 좋았습니다.</v>
       </c>
       <c r="H70" t="str">
-        <v>6,9월 모의고사만으로는 수능 시험장을 체감하기에 너무 적은 횟수이기에 실모를 한달에 한번은 풀로 봐야한다고 생각해서 이투스전국모고가 유용했습니다. 모의고사의 퀄리티와 별개로 하루를 통으로 써서 모의고사를 볼 수 있다는 점 자체로 아주 큰 메리트가 되었던 것 같습니다. 또한 그 성적을 바탕으로 상담도 해주셔서 앞으로 해나갈 공부 방향을 잘 잡을 수 있었습니다.</v>
+        <v>6,9월 모의고사만으로는 수능 시험장을 체감하기에 너무 적은 횟수이기에 실모를 한달에 한번은 풀로 봐야한다고 생각해서 이투스전국모고가 유용했습니다. 모의고사의 퀄리티와 별개로 하루를 통으로 써서 모의고사를 볼 수 있다는 점 자체로 아주 큰 메리트가 되었던 것 같습니다. 또한 그 성적을 바탕으로 상담도 해 주셔서 앞으로 해나갈 공부 방향을 잘 잡을 수 있었습니다.</v>
       </c>
       <c r="I70" t="str">
         <v>반년동안 새로운, 그리고 힘들었던 시간이었는데, 다시 생각해보면 그 안에서 선생님들 덕분에 이겨낼 수 있었던 순간이 꽤나 있었던 것 같습니다.  다른 핑계 없이 나 자신에게 부끄럽지 않게 살아가라는 담임 선생님 말씀이 아직까지 기억에 남는데 앞으로도 기숙학원에서만큼 열심히 살진 못하더라도, 그 경험을 바탕으로 부끄럽지 않게 살도록 노력해보겠습니다. 감사합니다!</v>
@@ -2942,7 +2942,7 @@
         <v>N수생</v>
       </c>
       <c r="E71" t="str">
-        <v>선생님께서 특화된 입시 프로그램을 이용하여 전문적으로 입시 상담을 해주신다. 뿐만 아니라 보통 1년 동안 담당 해주실 담임 선생님이 정해지기 때문에 계속 같은 데이터와 정보를 가지고 상담 해주신다.</v>
+        <v>선생님께서 특화된 입시 프로그램을 이용하여 전문적으로 입시 상담을 해 주신다. 뿐만 아니라 보통 1년 동안 담당해 주실 담임 선생님이 정해지기 때문에 계속 같은 데이터와 정보를 가지고 상담 해 주신다.</v>
       </c>
       <c r="F71" t="str">
         <v>내가 직접 시험 점수를 분석하지 않아도 다양하고 많은 표본을 가지고 내 성적을 분석해준다. 한눈에 보기 편하다. 나의 위치가 어느정도인지 직관적으로, 객관적으로 알 수 있다. 때문에 공부를 위한 원동력이 되기도 한다.</v>
@@ -2957,7 +2957,7 @@
         <v>민호쌤 짱 민호쌤 술 끊으시고 담배 끊으시고 오래오래 건강하시고 맨날 속썩여서 죄송하고 아이스크림 많이 사주셔서 감사합니다 사실 선생님이 제일 좋았어요^^ 과정이 어떻게 됐든 덕분에 완주할 수 있었습니다</v>
       </c>
       <c r="J71" t="str">
-        <v>1년 동안 담당 해주실 담임 선생님이 정해지기 때문에 계속 같은 데이터와 정보를 가지고 상담 해주셨어요.</v>
+        <v>1년 동안 담당해 주실 담임 선생님이 정해지기 때문에 계속 같은 데이터와 정보를 가지고 상담 해 주셨어요.</v>
       </c>
       <c r="K71" t="str">
         <v/>
@@ -2977,7 +2977,7 @@
         <v>N수생</v>
       </c>
       <c r="E72" t="str">
-        <v>멘탈이 흔들릴 때마다 좋은 말씀들로 위로해주셔서 힘든 생활을 버틸 수 있었던 것 같습니다. 또한 한주동안 헷갈렸던 문제들을 모아 한꺼번에 질문을 드릴 수 있어 편리했습니다. 학습수준에 맞춰 쉽게 설명해주셔서 이해하기도 용이했습니다.</v>
+        <v>멘탈이 흔들릴 때마다 좋은 말씀들로 위로해 주셔서 힘든 생활을 버틸 수 있었던 것 같습니다. 또한 한주동안 헷갈렸던 문제들을 모아 한꺼번에 질문을 드릴 수 있어 편리했습니다. 학습수준에 맞춰 쉽게 설명해 주셔서 이해하기도 용이했습니다.</v>
       </c>
       <c r="F72" t="str">
         <v>온라인을 통해 플래너를 작성하여 쉽고 빠르고 편리하게 하루를 시작할 수 있었습니다. 아떤 과목에 시간을 투자하는지 한눈에 볼 수 있어 계획을 바꾸는 것도 쉽게 할 수 있었습니다. 또 멘토링시간에 온라인을 통해 학습교정도 할 수 있었습니다.</v>
@@ -2992,7 +2992,7 @@
         <v>원장쌤, 제가 많이 부족했지만 잘 챙겨주셔서 감사했습니다. 가끔 쌤이 생각납니다. 한번 놀러갈게요~! 그리구 영어쌤께도 진짜 감사합니다. 항상 웃으며 좋은 얘기해주셨던 기억이 나요. 처음 48점 받았을 땐 정말 영어가 막막했는데 이젠 아무리 못 봐도 82점 이상 나오는 수준까지 올렸어요! 전부 선생님 덕분입니다 사랑합니다~!</v>
       </c>
       <c r="J72" t="str">
-        <v>멘탈이 흔들릴 때마다 좋은 말씀들로 위로해주셔서 힘든 생활을 버틸 수 있었던 것 같아요.</v>
+        <v>멘탈이 흔들릴 때마다 좋은 말씀들로 위로해 주셔서 힘든 생활을 버틸 수 있었던 것 같아요.</v>
       </c>
       <c r="K72" t="str">
         <v/>
@@ -3013,7 +3013,7 @@
       </c>
       <c r="E73" t="str" xml:space="preserve">
         <v xml:space="preserve">진도 체크와, 유형 별 인강 추천, 또 얼마나 이해 되었는지 특정 문제를 qna하며 제가 얼마나 학습률을 가져가는지를 알 수 있게 해주셨습니다._x000d_
-또 커리큘럼을 따라가다가 막히면 선생님께 여쭤보고, 다른 방법을 떠올릴 수 있게 해주시고 특정 공식을 변환하여 떠올릴 수 있도록 지도 해 주셨습니다.</v>
+또 커리큘럼을 따라가다가 막히면 선생님께 여쭤보고, 다른 방법을 떠올릴 수 있게 해 주시고 특정 공식을 변환하여 떠올릴 수 있도록 지도 해 주셨습니다.</v>
       </c>
       <c r="F73" t="str">
         <v>1:1 질의 응답과정에서는 단순 답지를 보고 이해하는 것이 아닌 계속 문제에 집중하며 어느 부분에서 제가 뭐를 모르는지 효율적으로 알 수 있었던 장점이 있던 것 같습니다. 그렇게 시간을 아끼고 더 나아가 다른 케이스나/관련 개념을 탄탄히 할 수 있었다는 점에서 정말 1:1 질의응답이 좋았습니다.</v>
@@ -3032,7 +3032,7 @@
 꿈을 향해 달려나가겠습니다.</v>
       </c>
       <c r="J73" t="str">
-        <v>졸음 관리를 해주셔서 스스로 더 절제할 수 있었고, 집중할 수 있는 분위기가 되었어요.</v>
+        <v>졸음 관리를 해 주셔서 스스로 더 절제할 수 있었고, 집중할 수 있는 분위기가 되었어요.</v>
       </c>
       <c r="K73" t="str">
         <v>졸음 관리</v>
@@ -3052,7 +3052,7 @@
         <v>반수생</v>
       </c>
       <c r="E74" t="str">
-        <v>과목별 담당 선생님이 계시고 제일 취약한 과목 선생님을 담임 선생님으로 배정해주셔서 매주 담임 선생님과 학습 진도 확인을 할 수 있다는 점이 좋았습니다. 추가로 필요할 때마다 질문을 할 수 있는 점이 좋았습니다.</v>
+        <v>과목별 담당 선생님이 계시고 제일 취약한 과목 선생님을 담임 선생님으로 배정해 주셔서 매주 담임 선생님과 학습 진도 확인을 할 수 있다는 점이 좋았습니다. 추가로 필요할 때마다 질문을 할 수 있는 점이 좋았습니다.</v>
       </c>
       <c r="F74" t="str">
         <v>질문이나 학습고민이 생겼을 때 질문 대기자 명단에 이름을 작성하면 따로 불러서 봐주신다는 점이 좋았습니다. 또 대학생 선생님이 아니라 경력이 있으신 분들이 계셔서 더 믿음이 갔던 것 같습니다</v>
@@ -3087,7 +3087,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E75" t="str">
-        <v>수능을 준비하는 학생의 경우 하루에 전과목을 어떻게 나누어 공부할 것인지가 관건인데, 하루 일과를 계획한 플래너를 기반으로 과목별 밸런스를 피드백해주셔서 이를 바탕으로 효율적으로 공부할 수 있었다.</v>
+        <v>수능을 준비하는 학생의 경우 하루에 전과목을 어떻게 나누어 공부할 것인지가 관건인데, 하루 일과를 계획한 플래너를 기반으로 과목별 밸런스를 피드백해 주셔서 이를 바탕으로 효율적으로 공부할 수 있었다.</v>
       </c>
       <c r="F75" t="str">
         <v>나와 맞는 인강을 듣고 학습하는 것이 중요하다고 생각하는데, 나의 성적 대의 수준과 맞는 인강을 골라주시거나 내가 선호하는 선생님의 커리 중 나의 수준에 맞는 인강을 골라주셔서 시행착오없이 학습을 시작할 수 있었다</v>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="I76" t="str" xml:space="preserve">
         <v xml:space="preserve">수험 생활이라는 긴 터널을 지나는 동안, 선생님들의 세심한 지도와 관리 덕분에 길을 잃지 않고 여기까지 올 수 있었습니다. 특히 국어 멘토링을 통해 제 부족한 점을 날카롭게 짚어주시고, 1대1 플래너 상담으로 막막했던 학습 방향을 잡아주신 덕분에 큰 힘이 되었습니다._x000d_
-때로는 엄격한 감독으로 긴장감을 유지해주시고, 졸음이 쏟아질 때마다 10분 벨로 저를 깨워주시던 그 정성 어린 마음들을 잊지 않겠습니다. 단순한 지식 전달을 넘어 멘탈까지 세심히 챙겨주신 모든 선생님들께 진심으로 감사의 인사를 올립니다. 보내주신 응원에 보답할 수 있도록, 앞으로의 대학 생활도 성실히 해나가겠습니다!</v>
+때로는 엄격한 감독으로 긴장감을 유지해 주시고, 졸음이 쏟아질 때마다 10분 벨로 저를 깨워주시던 그 정성 어린 마음들을 잊지 않겠습니다. 단순한 지식 전달을 넘어 멘탈까지 세심히 챙겨주신 모든 선생님들께 진심으로 감사의 인사를 올립니다. 보내주신 응원에 보답할 수 있도록, 앞으로의 대학 생활도 성실히 해나가겠습니다!</v>
       </c>
       <c r="J76" t="str">
         <v>국어 멘토링을 통해 제 부족한 점을 날카롭게 짚어주시고, 1대1 플래너 상담으로 막막했던 학습 방향을 잡아주신 덕분에 큰 힘이 되었어요.</v>
@@ -3173,7 +3173,7 @@
         <v>영어단어를 혼자 테스트없이 외우게되면 동기가 없고 의욕도 안생겨서 미루게되는데 강제적으로 테스트를 보게돼서 억지로라도 단어를 외운 것이 매우 좋았습니다 그래서 예전에는 단어책 하나 끝내기도 어려웠는데 이투스를 다니는 동안 매우 많은 단어를 외우게 되었습니다</v>
       </c>
       <c r="I77" t="str">
-        <v>수험 생활을 하면서 힘든 점이 많긴해도 응원해주시고 최대한 공부에 집중할 수 있는 환경을 만들어주실려고 노력해주신 선생님들께 매우 감사합니다 앞으로 대학에서도 좋은 결과를 내보겠습니다</v>
+        <v>수험 생활을 하면서 힘든 점이 많긴해도 응원해 주시고 최대한 공부에 집중할 수 있는 환경을 만들어주실려고 노력해 주신 선생님들께 매우 감사합니다 앞으로 대학에서도 좋은 결과를 내보겠습니다</v>
       </c>
       <c r="J77" t="str">
         <v>과목별 상담과 질문 해결, 와이파이 방화벽 덕분에 집보다 훨씬 집중도 높은 공부가 가능했어요.</v>
@@ -3285,7 +3285,7 @@
         <v>혼자서는 테스트하듯 단어를 암기하여도 실제 학원에서 시험을 보는듯한 효과는 가지지 못한다고 생각합니다. 꾸준하게 영어단어책을 매일매일 암기하고 시험 보는 것이 단어암기에 좋았습니다.</v>
       </c>
       <c r="I80" t="str">
-        <v>이투스 학원을 재원 하며 많은 선생님들께 도움을 받았습니다. 등원하고 하원할 때마다 반갑게 맞아주시는 카운터 선생님들 감사를 드리고 상담도 잘해주시고 항상 학생들 예뻐해 주시는 원장 선생님께도 감사드립니다. 또 이투스 학원 재원 중 제 담임 선생님이셨던 모든 선생님들께 정말 감사하다고 말씀드리고 싶습니다. 시험을 망쳐 하루종일이 우울했던 날 저에게 힘을 북돋아주시고 다시 공부할 수 있게 일으켜주셨던 준태선생님께 정말 감사했다고 전하고 싶습니다.</v>
+        <v>이투스 학원을 재원 하며 많은 선생님들께 도움을 받았습니다. 등원하고 하원할 때마다 반갑게 맞아주시는 카운터 선생님들 감사를 드리고 상담도 잘해 주시고 항상 학생들 예뻐해 주시는 원장 선생님께도 감사드립니다. 또 이투스 학원 재원 중 제 담임 선생님이셨던 모든 선생님들께 정말 감사하다고 말씀드리고 싶습니다. 시험을 망쳐 하루종일이 우울했던 날 저에게 힘을 북돋아주시고 다시 공부할 수 있게 일으켜주셨던 준태선생님께 정말 감사했다고 전하고 싶습니다.</v>
       </c>
       <c r="J80" t="str">
         <v>늘 반갑게 맞아주시는 선생님들과 따뜻하게 상담해주시는 원장 선생님 덕분에 수험 생활에 큰 힘을 얻었어요.</v>
@@ -3323,7 +3323,7 @@
       </c>
       <c r="I81" t="str" xml:space="preserve">
         <v xml:space="preserve">선생님들! 어쩌면 가장 힘든 수험 생활_x000d_
-학생들을 위해 최선을 다해주셔서 감사합니다._x000d_
+학생들을 위해 최선을 다해 주셔서 감사합니다._x000d_
 세심한 관리때문에 성장할수있었고_x000d_
 힘들었던 순간마다 선생님들의 한마디가 큰 힘이 되어 버틸수있었습니다_x000d_
  진심으로 감사드립니다._x000d_
@@ -3422,10 +3422,10 @@
         <v>N수생</v>
       </c>
       <c r="E84" t="str">
-        <v>예를 들어 제 약점과목이었던 국어의 경우 담임 선생님과의 상담을 통해 어떤강사의 인강을추천해주시는지를 현재 제 상태에 맞게 알려주시고 타과목들또한 제 당시수준에 맞추어 학습설계를 해주신점이 좋았습니다</v>
+        <v>예를 들어 제 약점과목이었던 국어의 경우 담임 선생님과의 상담을 통해 어떤강사의 인강을추천해주시는지를 현재 제 상태에 맞게 알려주시고 타과목들또한 제 당시수준에 맞추어 학습설계를 해 주신점이 좋았습니다</v>
       </c>
       <c r="F84" t="str">
-        <v>모의고사 시행직후 담임 선생님과의 상담을 통해 현재 학습수준을 판단하고 이를 토대로 수준에 맞게 인강강사와 커리큘럼을 구체적으로 과목별로 상담해주셔서 좋았고, 추천뿐만 아니라 모의고사전까지 들었던 강의들에대한 진단? 상담?도 해주셔서 좋았습니다</v>
+        <v>모의고사 시행직후 담임 선생님과의 상담을 통해 현재 학습수준을 판단하고 이를 토대로 수준에 맞게 인강강사와 커리큘럼을 구체적으로 과목별로 상담해 주셔서 좋았고, 추천뿐만 아니라 모의고사전까지 들었던 강의들에대한 진단? 상담?도 해 주셔서 좋았습니다</v>
       </c>
       <c r="G84" t="str">
         <v>기본적으로 매달 정기휴가를 제외하고는 대입실에 휴대폰을 보관하도록하니 이게 기숙학원의 큰장점이라고 느꼈고, 휴대폰 사용 적발시 바로 퇴원조치라는 강한 규정이 있어서 더욱 공부에 집중할 수있었던것 같습니다</v>
@@ -3471,7 +3471,7 @@
         <v>아침마다 영어 단어 테스트를 시행하는 것이 영어 공부에 큰 도움이 되었습니다. 다른 과목보다 영어는 시간 할애가 어려운데 정해진 시간마다 단어 시험을 봐서 따로 시간을 내지 않고도 효율적으로 공부할 수 있었습니다.</v>
       </c>
       <c r="I85" t="str">
-        <v>예상치도 못한 재수 생활이었지만 이투스를 다니면서 공부 습관을 기를 수 있었습니다. 평소에 제대로 공부를 해본 적이 없어서 막막한 상황 속에서 시작했는데, 선생님들께서 관리도 잘해주시고 꾸준히 신경 써주셔서 끝까지 포기하지 않고 공부할 수 있었던 것 같습니다. 공부적인 부분뿐만 아니라 생활적인 부분에서도 도움을 많이 받아서 감사했습니다.</v>
+        <v>예상치도 못한 재수 생활이었지만 이투스를 다니면서 공부 습관을 기를 수 있었습니다. 평소에 제대로 공부를 해본 적이 없어서 막막한 상황 속에서 시작했는데, 선생님들께서 관리도 잘해 주시고 꾸준히 신경 써주셔서 끝까지 포기하지 않고 공부할 수 있었던 것 같습니다. 공부적인 부분뿐만 아니라 생활적인 부분에서도 도움을 많이 받아서 감사했습니다.</v>
       </c>
       <c r="J85" t="str">
         <v>중요하게 생각했던 면학 분위기와 졸음 관리가 매우 철저하게 이루어져 공부에 큰 도움이 되었어요.</v>
@@ -3494,7 +3494,7 @@
         <v>반수생</v>
       </c>
       <c r="E86" t="str">
-        <v>일단 모르는 과목 물어볼 수 있는게 너무 좋았어요! 다 너무 친절하시고 성심성의껏 답변해주시고, 언제나 열정적으로 도와주셔서 좋았어요!! 그리고 과목마다 전담 선생님이 계셔서 더 자세하고 쉽게 배울 수 있어서 좋았어요!!</v>
+        <v>일단 모르는 과목 물어볼 수 있는게 너무 좋았어요! 다 너무 친절하시고 성심성의껏 답변해 주시고, 언제나 열정적으로 도와주셔서 좋았어요!! 그리고 과목마다 전담 선생님이 계셔서 더 자세하고 쉽게 배울 수 있어서 좋았어요!!</v>
       </c>
       <c r="F86" t="str">
         <v>뒤에 다른 학생 없으면 쭉 봐주셔서 모르는 질문 쌓인 채로 방치될 일 없고, 몰라도 그때 그때 해결되고, 자세하고 친절하게 알려주셔서 독학의 한줄기 빛과 같아서 좋았어요. 그리고 공부뿐만 아니라 공부법도 알려주셔서 좋았어요</v>
@@ -3506,10 +3506,10 @@
         <v>이투스 모고 꽤나 도움 됐어요. 현장감 유지랑 전략 실현에 좋았어요! 일단 현장감을 지속적으로 유지해볼 수 있어서 달마다 수능 때도 큰 긴장감 없이 잘 볼 수 있게 된 것 같았어요. 그리고 전략을 수정해서 젤 잘 맞는 순서로 문제를  풀 수 있게 되었어요</v>
       </c>
       <c r="I86" t="str">
-        <v>그동안 친절하게 가르쳐주셔서 감사합니다! 덕분에 힘애서 공부할 수 있었고, 뿌듯한 수능 전 3달을 보낼 수 있었습니다! 그리고 항상 웃음으로 대해주셔서 힘든 반수생 생활이 덕분에 덜 힘들었어요! 감사해요!!!</v>
+        <v>그동안 친절하게 가르쳐주셔서 감사합니다! 덕분에 힘애서 공부할 수 있었고, 뿌듯한 수능 전 3달을 보낼 수 있었습니다! 그리고 항상 웃음으로 대해 주셔서 힘든 반수생 생활이 덕분에 덜 힘들었어요! 감사해요!!!</v>
       </c>
       <c r="J86" t="str">
-        <v>항상 웃음으로 대해주셔서 힘든 반수생 생활이 덕분에 덜 힘들었어요.</v>
+        <v>항상 웃음으로 대해 주셔서 힘든 반수생 생활이 덕분에 덜 힘들었어요.</v>
       </c>
       <c r="K86" t="str">
         <v/>
@@ -3529,7 +3529,7 @@
         <v>N수생</v>
       </c>
       <c r="E87" t="str">
-        <v>멘토선생님들께서 거의다 재수 생활을 하셨던 경험이 있으셔서 제가 들려리는 학습에 관한 고민들에대해서 공감해주시고 명쾌한 해결책들을 제시해 주셔서 학습에 관한 고민들에 대해서 해결해 주셨었습니다. 또한 생활에대한 문제들이나 집중력에대한 문제들 또한 좋은 해결책들을 제안해주셔서 너무 유용했습니다</v>
+        <v>멘토선생님들께서 거의다 재수 생활을 하셨던 경험이 있으셔서 제가 들려리는 학습에 관한 고민들에대해서 공감해 주시고 명쾌한 해결책들을 제시해 주셔서 학습에 관한 고민들에 대해서 해결해 주셨었습니다. 또한 생활에대한 문제들이나 집중력에대한 문제들 또한 좋은 해결책들을 제안해 주셔서 너무 유용했습니다</v>
       </c>
       <c r="F87" t="str" xml:space="preserve">
         <v xml:space="preserve">매주 멘토선생님께서 상담을 해주시면서 생활에 관해 답답하거나 잘모르겠는 부분들을 상담해주셨었습니다. 또한 친절하고 친근하게 대해 주셔서 재수 생활동안 받았던 압박들을 해소해주셨습니다. _x000d_
@@ -3543,7 +3543,7 @@
 영어 단어 테스트를 하는것이 하루의 루틴으로 자리 잡아서 하다보니 강제성이 없어도 스스로 알아서 하게되었습니다.</v>
       </c>
       <c r="I87" t="str">
-        <v>1년 동안 이런저런 고민거리 들어주시고 해결책을 제시해 주셔서 감사했고, 불편한점을 해결해주시기 위해서 노력해주셔서 감사했습니다. 덕분에 공부에 집중할 수 있었습니다. 저 때문에 고생도 많이 하셨습니다. 앞으로 건강히 잘지내세요</v>
+        <v>1년 동안 이런저런 고민거리 들어주시고 해결책을 제시해 주셔서 감사했고, 불편한점을 해결해주시기 위해서 노력해 주셔서 감사했습니다. 덕분에 공부에 집중할 수 있었습니다. 저 때문에 고생도 많이 하셨습니다. 앞으로 건강히 잘지내세요</v>
       </c>
       <c r="J87" t="str">
         <v>과목별 선생님과 꾸준한 상담으로 재수 생활의 부담을 덜 수 있었고, 어려운 문제도 차근차근 해결할 수 있었어요.</v>
@@ -3601,7 +3601,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E89" t="str">
-        <v>수능이 얼마 남지 않은 시점에서 경각심을 갖게 하는 말씀을 해주신 것이 유용했다고 생각합니다. 수능 전까지 시간을 잘 쓸 수 있는 방법, 각 과목별로 공부법을 간략하게 설명해주신게 도움이 많이 된 것 같습니다.</v>
+        <v>수능이 얼마 남지 않은 시점에서 경각심을 갖게 하는 말씀을 해 주신 것이 유용했다고 생각합니다. 수능 전까지 시간을 잘 쓸 수 있는 방법, 각 과목별로 공부법을 간략하게 설명해 주신게 도움이 많이 된 것 같습니다.</v>
       </c>
       <c r="F89" t="str">
         <v>하루 루틴이 정해져 있어 특정 시간에 어떤 과목을 공부하고 그 후에 어떤 과목을 공부할지 정하는 과정에서 유용했다고 생각합니다. 틀이 정해져 있으니 그 속에서는 재량것 공부를 할 수 있었다고 생각합니다.</v>
@@ -3613,7 +3613,7 @@
         <v>이투스 학원에 머물고 있다보니 이투스 프로그램에 쉽게 접할 수 있었던 게 유용했다고 생각합니다. 추가적인 정보를 얻을 수 있었고 공부를 할 루트가 추가적으로 생긴것이니 유용했습니다.</v>
       </c>
       <c r="I89" t="str">
-        <v>비록 오랜시간 머물진 않았지만 이투스 학원의 시설이 좋았고 맛있는 밥을 매일 제공해주시는 조리사님들께 감사인사를 드리고 싶습니다. 수험생에게 행복이 되는 끼니를 제공해주셨습니다. 수업을 듣진 않았지만 원장님께서 여러 말씀 해주신게 기억에 남습니다.</v>
+        <v>비록 오랜시간 머물진 않았지만 이투스 학원의 시설이 좋았고 맛있는 밥을 매일 제공해주시는 조리사님들께 감사인사를 드리고 싶습니다. 수험생에게 행복이 되는 끼니를 제공해주셨습니다. 수업을 듣진 않았지만 원장님께서 여러 말씀 해 주신게 기억에 남습니다.</v>
       </c>
       <c r="J89" t="str">
         <v>선생님이 직접 관리하는 환경 덕분에 스스로 더 긴장감을 갖고 학습에 집중할 수 있었어요.</v>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="F90" t="str" xml:space="preserve">
         <v xml:space="preserve">각 과목별 질문을 받아주시는 선생님이 계셔서 문제가 잘 풀리지 않거나 어려울때 답답함이 많이 해소되었습니다 _x000d_
-또 질의응답과 같이 그 과목에 대한 조언들도 해주셔서 조언을 통해 공부하는 방향이 많이 잡힌 것 같습니다</v>
+또 질의응답과 같이 그 과목에 대한 조언들도 해 주셔서 조언을 통해 공부하는 방향이 많이 잡힌 것 같습니다</v>
       </c>
       <c r="G90" t="str">
         <v>너무 피곤해서 잠을 자고싶을때 이야기를 하면 10분 뒤에 깨워주는 것이 정말 좋았습니다 오히려 잠을 덜 자며 공부하는 것보다 조금 자고 일어나 공부하는 것이 더 효율적이었던 것 같습니다 또 계속 출석을 체크해서 중간 중간 나가는 학생이 없어서 공부 흐름이 깨지지 않아 좋았습니다</v>
@@ -3707,7 +3707,7 @@
         <v>N수생</v>
       </c>
       <c r="E92" t="str">
-        <v>현재 공부 진행률을 점검하고 앞으로의 공부 진행방향에 대해 생각해볼 수 있는 시간이었습니다. 학습 방향성에 있어서 고민이 되었던 것이나 생각하지 못했던 방법을 개개인 맞춤식으로 고려해 함께 고민하고 제안해주셔서 많은 도움이 되었습니다.</v>
+        <v>현재 공부 진행률을 점검하고 앞으로의 공부 진행방향에 대해 생각해볼 수 있는 시간이었습니다. 학습 방향성에 있어서 고민이 되었던 것이나 생각하지 못했던 방법을 개개인 맞춤식으로 고려해 함께 고민하고 제안해 주셔서 많은 도움이 되었습니다.</v>
       </c>
       <c r="F92" t="str">
         <v>성적에 대한 냉정한 판단으로 현실적인 목표를 잡을 수 있게되었고 상담을 통해 성적에 맞는 학습 방향을 제시해 주셔서 성적에 알맞는 방법으로 학습을 진행할 수 있다는 점에서 유용했습니다. 또한 가시적으로 성적을 직면하고 성적의 원인을 분석할 수 있어서 좋았습니다.</v>
@@ -3719,8 +3719,8 @@
         <v>학습을 하다보면 강사가 본인과 맞지 않거나 선택과목이 본인과 맞지 않아 변경하게 될 때도 있을 수 있습니다. 이투스 학원에서는 이투스 구독 컨텐츠를 제공하여 앞서 언급한 경우가 발생하였을 때 비교적 자유롭게 강사나 선택과목 변경할 수 있는 여건을 제공하여 학습에 도움이됩니다.</v>
       </c>
       <c r="I92" t="str" xml:space="preserve">
-        <v xml:space="preserve">제 학습과정을 함께 하며 고민도 들어주시고 방향성도 제공해주시고 무엇보다 많은 격려의 말씀 해주셔서 정말 감사드립니다._x000d_
-덕분에 학습과정에서 막막했던 부분들이 많이 해결되었습니다. 그 외에도 좋은 학습 분위기를 제공해주셔서 감사드립니다.</v>
+        <v xml:space="preserve">제 학습과정을 함께 하며 고민도 들어주시고 방향성도 제공해 주시고 무엇보다 많은 격려의 말씀 해 주셔서 정말 감사드립니다._x000d_
+덕분에 학습과정에서 막막했던 부분들이 많이 해결되었습니다. 그 외에도 좋은 학습 분위기를 제공해 주셔서 감사드립니다.</v>
       </c>
       <c r="J92" t="str">
         <v>객관적인 성적 분석과 상담을 통해 현실적인 목표를 세우고, 제 성적에 맞는 학습 방향을 잡을 수 있었어요.</v>
@@ -3749,7 +3749,7 @@
         <v>평소에 플래너 쓰는 것을 소홀히 하는 편이였는데 검사를 무조건한다고 해서 해야한다는 의무감이 생겼고 그로 인해 성취감도 생겨 공부에 큰 도움이 되었던 것 같습니다. 그리고 한 과목에만 집중하면 다른 과목으로 넘어가라는 피드백도 받을 수 있었습니다.</v>
       </c>
       <c r="G93" t="str">
-        <v>밥을 먹고 나면 어쩔 수 없이 졸음과 싸워야하는데 그때 선생님들께서 돌아다니시면서 너무 졸리면 밖에 나와서 공부를 하던지 잠깐 화장실에 갔다오라는지 등의 말씀을 해주셔서 도움이 되었습니다.</v>
+        <v>밥을 먹고 나면 어쩔 수 없이 졸음과 싸워야하는데 그때 선생님들께서 돌아다니시면서 너무 졸리면 밖에 나와서 공부를 하던지 잠깐 화장실에 갔다오라는지 등의 말씀을 해 주셔서 도움이 되었습니다.</v>
       </c>
       <c r="H93" t="str">
         <v>모의고사를 보지 않으면 뭔가 불안했었는데 이투스 모의고사 날에 자리도 랜덤으로 배치하고 실제 모의고사 분위기를 조성해서 시험을 치르는 것이 실전연습을 하는데 큰 도움이 되었습니다.</v>
@@ -3854,13 +3854,13 @@
         <v>내가 계획을 잘 못짜서 항상 공부를 할 때 부족함을 느꼈는데 플래너를 통해 학습량과 공부방향을 정해 공부를 할 수 있어서 능률이 올라갔고 효율적으로 공부할 수 있었다. 그리고 플래너를 통해서 점차 많은 목표를 이루어 갔을 때 성취감을 느껴서 좋았다</v>
       </c>
       <c r="G96" t="str">
-        <v>면학 분위기와 졸음등등을 선생님들이 매일 매시간 관리를 해주셔서 학습을 하는데 있어 많은 도움을 받았다 . 또한 내가 집중이 안될때 공부 하는 장소를 바꾸어 면학 분위기와 졸음 등등을 쉽고 빠르게 문제를 해결 할 수 있게 해주었다</v>
+        <v>면학 분위기와 졸음등등을 선생님들이 매일 매시간 관리를 해 주셔서 학습을 하는데 있어 많은 도움을 받았다 . 또한 내가 집중이 안될때 공부 하는 장소를 바꾸어 면학 분위기와 졸음 등등을 쉽고 빠르게 문제를 해결 할 수 있게 해주었다</v>
       </c>
       <c r="H96" t="str">
         <v>시중에 나와있는 모의고사 평가원 교육청 등등 많은 모의고사를 풀었고 학원에서 매월 나의 성적을 확인 할 수 있는 계기가 되어 좋았다. 또한 매번 기출을 보면 답도 기억나고 과정도 생각이 났는데 이투스 모의고사를 보면서 신유형과 처음 보는 낯선 문제들을 볼 수 있어 좋았다</v>
       </c>
       <c r="I96" t="str">
-        <v>지난 일년동안 지도해주셔서 감사했습니다. 덕분에 수능도 현역때보다 더 잘 보게 되었고 기숙학원에 있는동안 힘든 점도 많았지만 선생님들 덕분에 행복한 기억도 많았던 거 같습니다. 앞으로 인생을 살면서 이런 경험을 할 수 있을지는 모르지만 힘들면서 행복한 한 해가 되었습니다</v>
+        <v>지난 일년동안 지도해 주셔서 감사했습니다. 덕분에 수능도 현역때보다 더 잘 보게 되었고 기숙학원에 있는동안 힘든 점도 많았지만 선생님들 덕분에 행복한 기억도 많았던 거 같습니다. 앞으로 인생을 살면서 이런 경험을 할 수 있을지는 모르지만 힘들면서 행복한 한 해가 되었습니다</v>
       </c>
       <c r="J96" t="str">
         <v>학습 환경과 학습 분위기 등을 잡아주셔서 도움이 되었어요.</v>
@@ -3883,10 +3883,10 @@
         <v>N수생</v>
       </c>
       <c r="E97" t="str">
-        <v>학원 다닐 때 너무 스트레스를 많이 받았는데 담임 선생님과 상담을 받으면서 많이 극복했습니다. 입시가 길어지면서 많이 쳐지기도 했고 스스로도 많이 늘어지고 지친 느낌을 받아서 많이 힘들었습니다. 선생님께서 많이 힘이 되는 말씀을 해주셔서 도움이 많이 되었습니다.</v>
+        <v>학원 다닐 때 너무 스트레스를 많이 받았는데 담임 선생님과 상담을 받으면서 많이 극복했습니다. 입시가 길어지면서 많이 쳐지기도 했고 스스로도 많이 늘어지고 지친 느낌을 받아서 많이 힘들었습니다. 선생님께서 많이 힘이 되는 말씀을 해 주셔서 도움이 많이 되었습니다.</v>
       </c>
       <c r="F97" t="str">
-        <v>혼자 공부할 때는 인강 어떤 강의가 좋고 어떤 커리가 좋은지를 잘 몰랐는데 선생님께서 많이 알려주셔서 컨텐츠적인 방면에서 많은 도움을 받았습니다. 방향을 제시해주시고 스텝도 정해 주셔서 많은 도움이 되었습니더.</v>
+        <v>혼자 공부할 때는 인강 어떤 강의가 좋고 어떤 커리가 좋은지를 잘 몰랐는데 선생님께서 많이 알려주셔서 컨텐츠적인 방면에서 많은 도움을 받았습니다. 방향을 제시해 주시고 스텝도 정해 주셔서 많은 도움이 되었습니더.</v>
       </c>
       <c r="G97" t="str">
         <v>처음에 진짜 많이 졸았는데 많이 깨워주셔서 생활 관리가 잘 되고 많이 습관이 잡힌 것 같습니다. 원래 졸음이 많은 편이라 감독하는 분이 안 계시면 꿈나라에 빠지는 경우가 많은데 졸고 있으면 깨워주셔서 너무 도움이 되었습니다.</v>
@@ -3918,7 +3918,7 @@
         <v>N수생</v>
       </c>
       <c r="E98" t="str">
-        <v>혼자 정하기 어려운 과목 별 분량이나 공부 시간, 현재 나에게 필요한 학습 방법 등을 상세하게 확인해주시고 주기적으로 피드백 받을 수 있었습니다. 저의 경우 수학을 노베이스 상태로 시작했기 때문에 수학과 관련해서 학습 코칭이 큰 도움이 되었습니다.</v>
+        <v>혼자 정하기 어려운 과목 별 분량이나 공부 시간, 현재 나에게 필요한 학습 방법 등을 상세하게 확인해 주시고 주기적으로 피드백 받을 수 있었습니다. 저의 경우 수학을 노베이스 상태로 시작했기 때문에 수학과 관련해서 학습 코칭이 큰 도움이 되었습니다.</v>
       </c>
       <c r="F98" t="str">
         <v>재수 학원을 다니는 가장 큰 이유가 꾸준함과 성실함이 부족하면 일관된 생활 패턴과 적절한 학습량을 만들 수 없기 때문인데, 플래너를 통해 스스로 학습 계획을 세우고 적절한 계획인지 확인받아가며 저만의 공부 루틴을 세울 수 있었습니다.</v>
@@ -3953,22 +3953,22 @@
         <v>N수생</v>
       </c>
       <c r="E99" t="str">
-        <v>어려운 문제가 있을 때 온라인이나 오프라인으로 상담 신청을 하면 바로 답변을 해주셔서 더 편리하게 공부할 수 있었습니다. 특히 국어의 경우 온라인 상담을 많이 이용했는데 너무 지엽적인 질문들이더라도 친절하고 세세히 답변해 주셨습니다. 특히 언어(국어 문법) 영역에서 크게 도움을 받았습니다. 또 대학생 선생님들의 경험에서 녹아든 코칭 또한 실전 감각을 익히고 공부 방향을 재설정 하는 데 유용했습니다.</v>
+        <v>어려운 문제가 있을 때 온라인이나 오프라인으로 상담 신청을 하면 바로 답변을 해 주셔서 더 편리하게 공부할 수 있었습니다. 특히 국어의 경우 온라인 상담을 많이 이용했는데 너무 지엽적인 질문들이더라도 친절하고 세세히 답변해 주셨습니다. 특히 언어(국어 문법) 영역에서 크게 도움을 받았습니다. 또 대학생 선생님들의 경험에서 녹아든 코칭 또한 실전 감각을 익히고 공부 방향을 재설정 하는 데 유용했습니다.</v>
       </c>
       <c r="F99" t="str">
-        <v>대학생 선생님들의 실전 코칭이 가장 좋았던 것 같습니다. 구체적으로 시간 배분하여 일정을 짜주신 부분이 계획형인 저의 성향에도 잘 맞았던 것 같습니다. 또 시기에 맞게 유동적으로 코치해주셔서 불안하지 않고 공부에만 집중할 수 있었던 것 같습니다.</v>
+        <v>대학생 선생님들의 실전 코칭이 가장 좋았던 것 같습니다. 구체적으로 시간 배분하여 일정을 짜주신 부분이 계획형인 저의 성향에도 잘 맞았던 것 같습니다. 또 시기에 맞게 유동적으로 코치해 주셔서 불안하지 않고 공부에만 집중할 수 있었던 것 같습니다.</v>
       </c>
       <c r="G99" t="str">
-        <v>봄이 되어 졸릴 때가 많았는데 학생들이 졸 때마다 수시로 깨우러 오시는 감독 선생님들 덕분에 정신차리고 공부에 집중할 수 있었습니다. 또 학생들 모두 열심히 하는 분위기여서 저도 덩달아 게을러지지 않고 마음을 다잡을 수 있었던 것 같습니다. 또한 학생들이 더워하거나 추워하면 즉각적으로 온도도 개선해주셔서 공부 환경도 무척 만족스러웠습니다.</v>
+        <v>봄이 되어 졸릴 때가 많았는데 학생들이 졸 때마다 수시로 깨우러 오시는 감독 선생님들 덕분에 정신차리고 공부에 집중할 수 있었습니다. 또 학생들 모두 열심히 하는 분위기여서 저도 덩달아 게을러지지 않고 마음을 다잡을 수 있었던 것 같습니다. 또한 학생들이 더워하거나 추워하면 즉각적으로 온도도 개선해 주셔서 공부 환경도 무척 만족스러웠습니다.</v>
       </c>
       <c r="H99" t="str">
         <v>원래 하던 공부책 외에 일일테스트가 있어 수학의 경우 복습용으로 이용하다보니 더 효율적으로 공부했다고 생각합니다. 특히 확률과 통계의 경우 수학1과 수학2에 비해 조금 소홀히 할 수도 있었지만 일일테스트 덕분에 감을 잃지 않고 시험 대비를 할 수 있었습니다.</v>
       </c>
       <c r="I99" t="str">
-        <v>그동안 많이 챙겨주시고 응원해주셔서 감사합니다. 모든 학생들을 관리 감독하는 일이 쉽지 않으셨을텐데 선생님들이 신경써주시는 모습을 보고 기대에 만족시켜드리고자 더 열심히 공부했던 것 같습니다. 선생님들 덕분에 나쁘지 않은 성과를 얻었던 것 같아요!</v>
+        <v>그동안 많이 챙겨주시고 응원해 주셔서 감사합니다. 모든 학생들을 관리 감독하는 일이 쉽지 않으셨을텐데 선생님들이 신경써주시는 모습을 보고 기대에 만족시켜드리고자 더 열심히 공부했던 것 같습니다. 선생님들 덕분에 나쁘지 않은 성과를 얻었던 것 같아요!</v>
       </c>
       <c r="J99" t="str">
-        <v>과목별 질문을 빠르게 해결할 수 있었고 실전 코칭까지 해주셔서 공부 방향을 잡을 수 있었어요.</v>
+        <v>과목별 질문을 빠르게 해결할 수 있었고 실전 코칭까지 해 주셔서 학습 방향을 잡을 수 있었어요.</v>
       </c>
       <c r="K99" t="str">
         <v/>
@@ -4142,7 +4142,7 @@
         <v>N수생</v>
       </c>
       <c r="E104" t="str">
-        <v>어떤 선생님꺼 들어야하는지 어떻게공부해야 하는지 혼자 고민을 많이하다가 상담하면 어떤 강의를 들어야하는지 어떻게 공부해야 하는지 같이 고민해주시고 꿀팁도주시고 알려주셔서 많은 도움이되었고 유용했음</v>
+        <v>어떤 선생님꺼 들어야하는지 어떻게공부해야 하는지 혼자 고민을 많이하다가 상담하면 어떤 강의를 들어야하는지 어떻게 공부해야 하는지 같이 고민해 주시고 꿀팁도주시고 알려주셔서 많은 도움이되었고 유용했음</v>
       </c>
       <c r="F104" t="str">
         <v>공부하다가 해설을 봐도 헷갈리거나 이해가안되거나 모르는 문제가있으면 바로 가져가서 물어보면 친절하게 알려주셔서 빠르고 쉽게 이해할수있고 이해못하면어떡하나 이런 심적 부담감이 없었던게 좋았다</v>
@@ -4154,7 +4154,7 @@
         <v>요일마다 다른과목들을 매일 테스트보니까 까먹을것도 안까먹게되고 알아가는것도 생기고 테스트를 보기위해서 단어도 외우게되고 공부를 하게되어서 스스로 열심히하게만드는 수단이되었던것같아서 유용한 것같다</v>
       </c>
       <c r="I104" t="str">
-        <v>재수 처음할때 답답하고 되게 막막했는데 많은 도움들 주셔서 덕분에 잘 할 수 있었오요 ! 항상 친절하게대해주시고 딸처럼 걱정해주시고 챙겨주셨어서 짱 감사합니다...!!!! ❤️❤️</v>
+        <v>재수 처음할때 답답하고 되게 막막했는데 많은 도움들 주셔서 덕분에 잘 할 수 있었오요 ! 항상 친절하게대해 주시고 딸처럼 걱정해 주시고 챙겨주셨어서 짱 감사합니다...!!!! ❤️❤️</v>
       </c>
       <c r="J104" t="str">
         <v>막막했던 재수 생활에서 상담과 질문 해결, 생활 관리 덕분에 안정적으로 공부할 수 있었어요.</v>
@@ -4177,10 +4177,10 @@
         <v>N수생</v>
       </c>
       <c r="E105" t="str">
-        <v>선생님께서 매일 종례를 하셨는데 그때 학생들의 상태를 확인하시고 항상 명언과 같은 동기부여의 말, 응원의 말을 해주셔서 정신적으로 도움을 받았습니다. 학생들을 정말 진심으로 아끼시는 분이 담임이라 버틸 수 있었습니다.</v>
+        <v>선생님께서 매일 종례를 하셨는데 그때 학생들의 상태를 확인하시고 항상 명언과 같은 동기부여의 말, 응원의 말을 해 주셔서 정신적으로 도움을 받았습니다. 학생들을 정말 진심으로 아끼시는 분이 담임이라 버틸 수 있었습니다.</v>
       </c>
       <c r="F105" t="str">
-        <v>어느 부분을 더 집중적으로 보완해야 하는지 콕 찝어서 말씀해주셔서 부족한 점을 채울 수 있었습니다. 혼자서라면 무엇을 해야 할지 막막했을텐데 선생님과 상의할  수 있었다는게 큰 도움이 되었습니다.</v>
+        <v>어느 부분을 더 집중적으로 보완해야 하는지 콕 찝어서 말씀해 주셔서 부족한 점을 채울 수 있었습니다. 혼자서라면 무엇을 해야 할지 막막했을텐데 선생님과 상의할  수 있었다는게 큰 도움이 되었습니다.</v>
       </c>
       <c r="G105" t="str">
         <v>기숙학원에선 주변 사람들이 자신의 목표를 위해 열심히 노력하는 모습을 보고 포기하고 싶을 때마다 다시 힘을 낼 수 있었습니다. 혼자하면 쉽게 흐트러졌을거같은데 다 같이 열심히 하는 분위기가 좋았습니다.</v>
@@ -4189,7 +4189,7 @@
         <v>이투스는 솔직히 메가나 대성보다 밀리는 느낌이라 수강할 생각을 못했는데 기숙에서 준 수강권을 받아 한 번 시도해볼 수 있어좋았습니다. 이투스에 생각보다 좋은 강사님들이 많이 계셔서 많은 도움을 받았습니다.</v>
       </c>
       <c r="I105" t="str">
-        <v>항상 학생들을 아끼시는 마음으로 관리 해주셔서 큰 힘이 되었습니다. 번거로울 수 있는데도 매일 종례 해주시고 문제가 생기면 바로 해결해주셨던 상헌쌤께 특히 감사드립니다. 진짜 제 인생 통틀어 최고의 담임 선생님이셨습니다.</v>
+        <v>항상 학생들을 아끼시는 마음으로 관리 해 주셔서 큰 힘이 되었습니다. 번거로울 수 있는데도 매일 종례 해 주시고 문제가 생기면 바로 해결해주셨던 상헌쌤께 특히 감사드립니다. 진짜 제 인생 통틀어 최고의 담임 선생님이셨습니다.</v>
       </c>
       <c r="J105" t="str">
         <v>학생들을 정말 진심으로 아끼시는 분이 담임 선생님이라 버틸 수 있었어요.</v>
@@ -4212,12 +4212,12 @@
         <v>N수생</v>
       </c>
       <c r="E106" t="str" xml:space="preserve">
-        <v xml:space="preserve">담임쌤이랑 매주 한 번씩 공부 방법, 피드백, 고쳐야 할 점 등등 학습에 도움되는 이야기를 할 수 있어서 좋았고_x000d_
+        <v xml:space="preserve">담임쌤이랑 매주 한 번씩 공부 방법, 피드백, 고쳐야 할 점 등등 학습에 도움 되는 이야기를 할 수 있어서 좋았고_x000d_
 큐엔에이도 과목마다 다양한 선생님들이랑 당일날에 바로바로 대면으로 해결할수있어서 좋있습니다</v>
       </c>
       <c r="F106" t="str" xml:space="preserve">
         <v xml:space="preserve">매주 부족한 과목은 무엇인지 모의고사를 치고 부족한 부분은 무엇인지 상담을 통해 _x000d_
-학습량과 커리큘럼을 조정할수있어서 좋았습니다 또한 선생님들의 경험을 토대로 추천해주신 인강을 듣고 부족했던 부분을 선생님이 채워주시기도 하셔서 좋았습니다</v>
+학습량과 커리큘럼을 조정할수있어서 좋았습니다 또한 선생님들의 경험을 토대로 추천해 주신 인강을 듣고 부족했던 부분을 선생님이 채워주시기도 하셔서 좋았습니다</v>
       </c>
       <c r="G106" t="str">
         <v>고등학생때 생각해보면 스카에서나 학교에서나 휴대폰 본다고 공부 시간을 날리고 집중도 못하고 그랬었는데 관리형 독재학원을 다니니 이런 부분에서 강제적으로 제한이 되니 환경적 부분에서 공부하시가 훨씬 좋아졌습니다</v>
@@ -4233,7 +4233,7 @@
 모두 감사했고 수고하셨습니다</v>
       </c>
       <c r="J106" t="str">
-        <v>담임 선생님과 매주 공부 방법, 피드백, 고쳐야 할 점 등 학습에 도움되는 이야기를 할 수 있어서 좋았어요.</v>
+        <v>담임 선생님과 매주 공부 방법, 피드백, 고쳐야 할 점 등 학습에 도움 되는 이야기를 할 수 있어서 좋았어요.</v>
       </c>
       <c r="K106" t="str">
         <v/>
@@ -4253,7 +4253,7 @@
         <v>N수생</v>
       </c>
       <c r="E107" t="str">
-        <v>같은 학원에서 좋은 성적을 받고 대학에 입학하신 멘토님께서 제 고민을 같이 고민해주시면서 제 수준에 필요한 좋은 교재도 추천해 주시고, 방황할 때 이대로 쭉 해도 좋겠다고 격려해주신 점이 너무 좋았습니다.</v>
+        <v>같은 학원에서 좋은 성적을 받고 대학에 입학하신 멘토님께서 제 고민을 같이 고민해주시면서 제 수준에 필요한 좋은 교재도 추천해 주시고, 방황할 때 이대로 쭉 해도 좋겠다고 격려해 주신 점이 너무 좋았습니다.</v>
       </c>
       <c r="F107" t="str">
         <v>다른 친구들은 방심하다가 놓칠 수도 있는 평가원 모의고사나 유명한 사설 모의고사, 학원에서만 받을 수 있는 간쓸개 같은 프로그램을 시즌마다 복도에 붙여 놓치는 일 없도록 도와주신 점이 학습에 차질이 생기지 않게 해주셨다고 생각합니다</v>
@@ -4265,7 +4265,7 @@
         <v>단어시험은 강제성이 부여되지 않으면 하루하루 꾸준히 하기 힘든데 점심시간에 나갔다 오면 자리에 놓여있는 시험지때문에 하기싫은 날이라도 외워서 시험을 보는 것이 꾸준함에 도움이 됐습니다</v>
       </c>
       <c r="I107" t="str">
-        <v>학원 처음와서 여기저기 방황할 때 친절하게 상담해주시고, 공부하기 좋은 환경을 만들어주셔서 감사합니다! 그리고 이후 공부에 필요한 자료들을 요청드렸을때도 절차를 친절하게 설명해주셔서 감사합니다</v>
+        <v>학원 처음와서 여기저기 방황할 때 친절하게 상담해 주시고, 공부하기 좋은 환경을 만들어주셔서 감사합니다! 그리고 이후 공부에 필요한 자료들을 요청드렸을때도 절차를 친절하게 설명해 주셔서 감사합니다</v>
       </c>
       <c r="J107" t="str">
         <v>선생님께서 현실적인 조언과 교재 추천을, 학원에서는 시즌별 모의고사 및 학습 일정을 안내해 주셔서 학습 흐름을 놓치지 않을 수 있었어요.</v>
@@ -4300,7 +4300,7 @@
         <v>이투스247학원에서 제공하는 구독 서비스를 무료로 이용할 수 있다는 점은 경제적인 부담을 줄여준다는 점에서 매우 유용했습니다. 다양한 인강과 학습 자료를 추가 비용 없이 활용할 수 있어 학습 선택의 폭이 넓어졌고, 필요한 강의를 바로 수강할 수 있어 시간 낭비도 줄일 수 있었습니다. 이를 통해 보다 효율적으로 공부에 집중할 수 있었습니다.</v>
       </c>
       <c r="I108" t="str">
-        <v>이투스247학원 선생님들께 항상 세심하게 지도해주시고, 학습 방향에 대해 진심으로 고민해주셔서 진심으로 감사드립니다. 덕분에 흔들릴 때마다 다시 중심을 잡을 수 있었고, 끝까지 포기하지 않고 공부를 이어갈 수 있었습니다. 앞으로도 배운 것들을 바탕으로 더 성장할 수 있도록 노력하겠습니다. 정말 감사합니다.</v>
+        <v>이투스247학원 선생님들께 항상 세심하게 지도해 주시고, 학습 방향에 대해 진심으로 고민해 주셔서 진심으로 감사드립니다. 덕분에 흔들릴 때마다 다시 중심을 잡을 수 있었고, 끝까지 포기하지 않고 공부를 이어갈 수 있었습니다. 앞으로도 배운 것들을 바탕으로 더 성장할 수 있도록 노력하겠습니다. 정말 감사합니다.</v>
       </c>
       <c r="J108" t="str">
         <v>하루 공부량을 체계적으로 관리할 수 있었고, 생활 패턴도 규칙적으로 유지하는 데 도움이 되었어요.</v>
@@ -4371,7 +4371,7 @@
         <v>평소에 의지박약으로 단어를 외웠다가 안외웠다가 갈팡질팡 공부했었는데 학원을 다니면서 의무적으로 매일 아침마다 보는 단어시험으로 비몽사몽한 뇌를 깨우는 데에도 매우 도움이되었고 단어도 처음으로 꾸준히 암기 할 수 있었던 부분에서 매우 유용했습니다.</v>
       </c>
       <c r="I110" t="str">
-        <v>평소에 몸이 자주 안 좋아 아팠었는데 그럼에도 불구하고, 그런 저를 수험 생활 끝까지 다정하게 잘 관리해주시고 이끌어주시고 감독해주셔서 입시의 끝을 합격으로 만들어주셔서 정말 감사합니다!</v>
+        <v>평소에 몸이 자주 안 좋아 아팠었는데 그럼에도 불구하고, 그런 저를 수험 생활 끝까지 다정하게 잘 관리해 주시고 이끌어주시고 감독해 주셔서 입시의 끝을 합격으로 만들어주셔서 정말 감사합니다!</v>
       </c>
       <c r="J110" t="str">
         <v>생활 관리와 맞춤 학습 코칭 덕분에 올바른 공부 습관이 생기고 집중력이 올라가서 합격까지 이어졌어요.</v>
@@ -4406,7 +4406,7 @@
         <v>영어가 약했었는데 그 중 큰 이유가 단어를 많이 모른다는 것이었습니다 근데 매일 지정시간마다 단어 시험을 보고 채점을 하게 되니까 단어를 많이 알게되어 영어 성적 상승에 큰 도움을 받은 것 같습니다.</v>
       </c>
       <c r="I111" t="str">
-        <v>그 동안 많은 도움주셔서 감사합니다. 하루에 잠자는 시간말고는 거의 학원에 있었는데 학습 분위기도 좋고 상담도 잘 해주셔서 불편하지 않게 공부 열심히 잘 한 것 같습니다 감사합니다 !</v>
+        <v>그 동안 많은 도움주셔서 감사합니다. 하루에 잠자는 시간말고는 거의 학원에 있었는데 학습 분위기도 좋고 상담도 잘 해 주셔서 불편하지 않게 공부 열심히 잘 한 것 같습니다 감사합니다 !</v>
       </c>
       <c r="J111" t="str">
         <v>좋은 학습 분위기와 세심한 상담 덕분에 오랜 시간 학원에 머물면서도 편하게 공부에 집중할 수 있었어요.</v>
@@ -4476,7 +4476,7 @@
         <v>이투스 무료 구독권을 통해서 듣고 싶었던 강의를 마음 편히 들을 수 있었습니다. 이투스 패스를 사기에는 부담스러웠는데, 학원에서 제공해 주어서 좋았습니다. 덕분에 부족한 점을 메꿀 수 있었고, 실력이 향상되었습니다.</v>
       </c>
       <c r="I113" t="str">
-        <v>1년 동안 변함없이 응원해주시고, 코칭해주신 선생님들 감사합니다! 불편한 부분들을 말씀드리면 곧바로 해결해주셔서 생활의 질이 높은 수험 생활이 되었던 것 같습니다. 부족한 부분들에 대해 함께 의논해 주시고, 격려해 주셔서 감사합니다.</v>
+        <v>1년 동안 변함없이 응원해 주시고, 코칭해 주신 선생님들 감사합니다! 불편한 부분들을 말씀드리면 곧바로 해결해 주셔서 생활의 질이 높은 수험 생활이 되었던 것 같습니다. 부족한 부분들에 대해 함께 의논해 주시고, 격려해 주셔서 감사합니다.</v>
       </c>
       <c r="J113" t="str">
         <v>휴대폰 수거와 와이파이 방화벽 시스템으로 학습 맞춤 환경 덕분에 온전히 공부에만 집중할 수 있었어요.</v>
@@ -4499,7 +4499,7 @@
         <v>반수생</v>
       </c>
       <c r="E114" t="str">
-        <v>원서를 어디에 써야하는지 몰라서 헤매고 있을 때 상담을 성적에 맞게 잘 해주셔서 너무 좋았습니다. 생각지도 못한 방법을 제시해주신 부분도 있어서 안심할 수 있었습니다. 모르는 부분도 잘 알려주시고, 앞으로의 방향성도 계속 잡아주셔서 좋았습니다.</v>
+        <v>원서를 어디에 써야하는지 몰라서 헤매고 있을 때 상담을 성적에 맞게 잘 해 주셔서 너무 좋았습니다. 생각지도 못한 방법을 제시해 주신 부분도 있어서 안심할 수 있었습니다. 모르는 부분도 잘 알려주시고, 앞으로의 방향성도 계속 잡아주셔서 좋았습니다.</v>
       </c>
       <c r="F114" t="str">
         <v>일주일마다 한 번씩 상담 해주셨습니다. 제가 쓴 플래너를 보시고 공부를 잘 하고 있는지 미흡한 부분은 어디인지 알려주셔서 좋았습니다. 제가 저번주에 공부한 부분도 가끔 물어보셔서 그 질문에 답할려고 자동적으로 복습까지 하게 되어서 좋았습니다.</v>
@@ -4511,7 +4511,7 @@
         <v>매일매일 아침마다 단어테스트를 해서 영어단어 공부를 할수 있어서 좋았습니다. 전날에 다음날 시험보는 영어단어를 공부하면 학습 효율이 두배로 올라가는 느낌이 들어서 더 좋았습니다. 또 틀린거 모아 볼 수 있어서 좋았습니다</v>
       </c>
       <c r="I114" t="str">
-        <v>감사합니다. 상담 해주셔서 감사합니다. 학습태도 관리 해주셔서 감사합니다. 좋은 학습 분위기 조성해주셔서 감사합니다. 친절하게 대해주셔서 감사합니다. 청소도 매번 해주셔서 감사합니다.</v>
+        <v>감사합니다. 상담 해 주셔서 감사합니다. 학습태도 관리 해 주셔서 감사합니다. 좋은 학습 분위기 조성해 주셔서 감사합니다. 친절하게 대해 주셔서 감사합니다. 청소도 매번 해 주셔서 감사합니다.</v>
       </c>
       <c r="J114" t="str">
         <v>성적에 맞는 원서 상담과 현실적인 방향 제시 덕분에 안심하고 입시를 준비할 수 있었어요.</v>
@@ -4539,7 +4539,7 @@
       </c>
       <c r="F115" t="str" xml:space="preserve">
         <v xml:space="preserve">궁금하거나 어려운 문제 또는 개념에 대해서 편하게 여쭈어볼 수 있고 혼자서 하는 공부보다 밀도 높은 이해를 할 수 있고 심화 수준까지 꿰뚫어볼 수 있게 됨_x000d_
-친절하게 이해할 수 있을 때까지 설명해주신다</v>
+친절하게 이해할 수 있을 때까지 설명해 주신다</v>
       </c>
       <c r="G115" t="str" xml:space="preserve">
         <v xml:space="preserve">매일매일 규칙적인 생활 패턴을 반복하여 몸에 익히게 해주고 덕분에 아침시간부터 효율적이고 시간에 맞는 공부를 할 수 있음_x000d_
@@ -4549,7 +4549,7 @@
         <v>이투스 강사분들의 강좌를 금액 신경 쓰지 않고 마음껏 볼 수 있고 과목마다 필요한 개념이나 문제풀이 부분만 꼽아서 볼 수도 있고 추후에 교재를 구매하는 쪽으로 잘맞는 강좌를 찾기에도 좋다</v>
       </c>
       <c r="I115" t="str" xml:space="preserve">
-        <v xml:space="preserve">매일 지도해주고 밝은 모습으로 맞아주시고 대해주셔서 이끌어주셔서 감사합니다_x000d_
+        <v xml:space="preserve">매일 지도해주고 밝은 모습으로 맞아주시고 대해 주셔서 이끌어주셔서 감사합니다_x000d_
 학원 시스템에 적응하기 힘들었지만_x000d_
 선생님분들은 편했습니다 학생이 힘들 것을 깊히 헤아려주시는 것같은 느낌이 들 정도로 감사합니다</v>
       </c>
@@ -4612,7 +4612,7 @@
         <v>매주 학습 플래너와 공부 계획을 점검 및 피드백 해주셨고 과목별 고민이나 공부 방법, 커리큘럼 추천도 해주셨고 무엇보다 모의고사 응시 후 모의고사 관련 피드백이 매우 유용했던 것 같습니다.</v>
       </c>
       <c r="F117" t="str">
-        <v>앞서 말했던것 처럼 매주 과목별로 공부량이나 공부 방법등을 피드백 해주시고 과목별 고민이나 모의고사 운영 전략, 시간 관리 등등 실전적인 부분도 도움울 주셨던 점이 많이 도움이 되었던것 같습니다.</v>
+        <v>앞서 말했던것 처럼 매주 과목별로 공부량이나 공부 방법등을 피드백 해 주시고 과목별 고민이나 모의고사 운영 전략, 시간 관리 등등 실전적인 부분도 도움울 주셨던 점이 많이 도움이 되었던것 같습니다.</v>
       </c>
       <c r="G117" t="str">
         <v>핸드폰 수거는 재수 학원에서 무엇보다 필수적인 요소라고 생각하는데 공부에 방해가 되기때문에 매일 등원할때 마다 제출 할 수 있도록 해서 학습에 방해가 되지않아서 매우 좋았습니다. 점심시간 및 저녁시간에는 사용 가능했고 복귀시 다시 제출해야 했습니다.</v>
@@ -4658,7 +4658,7 @@
       </c>
       <c r="I118" t="str" xml:space="preserve">
         <v xml:space="preserve">삭막한 재수 생활에 원장님과 실장님들이 친근하게 말 걸어주셔서 너무 감사했어요 그리고 한 번도 가져본 적 없던 규칙적인 생활 패턴이 생겨서 너무 도움됐어요_x000d_
-뭘 요청하거나 질문을 했을 때 잘 답변해주셔서 감사합니다</v>
+뭘 요청하거나 질문을 했을 때 잘 답변해 주셔서 감사합니다</v>
       </c>
       <c r="J118" t="str">
         <v>내 수준에 맞는 강의와 공부 방향을 잡아주고, 규칙적인 생활 습관 형성에 큰 도움이 됐어요.</v>
@@ -4728,7 +4728,7 @@
         <v>영어가 절대평가로 바뀌면서 영어 과목에 대한 중요도가 많이 떨어졌고 제 체감 상으로도 공부량이 부족하다 느꼈습니다 하지만 감이 중요한 과목인 만큼 매일 꾸준히 할 수 있는 콘텐츠가 필요했는데 제게 그것이 이투스 voca 였습니다 매일 영어단어 시험을 보면서 영어 텍스트에 대한 이해도가 높아진 것 같습니다</v>
       </c>
       <c r="I120" t="str" xml:space="preserve">
-        <v xml:space="preserve">목표했던 학교에 가지는 못했지만 후회되지 않는 시간이었습니다 이 시간을 보낼 수 있었던 건 선생님들의 도움이 컸던 것 같습니다 늘 친절하게 맞이해주시고 청결하게 관리해주시고 제 공부에 관심을 갖고 같이 고민해주셔서 감사했습니다 항상 건강하시고 행복하셨으면 좋겠습니다 _x000d_
+        <v xml:space="preserve">목표했던 학교에 가지는 못했지만 후회되지 않는 시간이었습니다 이 시간을 보낼 수 있었던 건 선생님들의 도움이 컸던 것 같습니다 늘 친절하게 맞이해 주시고 청결하게 관리해 주시고 제 공부에 관심을 갖고 같이 고민해 주셔서 감사했습니다 항상 건강하시고 행복하셨으면 좋겠습니다 _x000d_
 앞으로의 삶에 밑바탕이 될 시간을 만들어주셔서 감사합니다</v>
       </c>
       <c r="J120" t="str">
@@ -4799,7 +4799,7 @@
         <v>인강 구독권을 무료로 제공해준 점은 확실히 도움이 됐다. 따로 강의를 결제하지 않아도 필요한 과목을 바로 들을 수 있어서 부담이 줄었고, 부족한 부분을 보완하는 데 유용했다. 다만 모든 강의를 다 활용하기보다는, 본인에게 필요한 강의만 선택해서 듣는 게 더 중요하다고 느꼈다. 그래도 기본적인 학습 환경을 갖춰준다는 점에서 충분히 만족스러운 혜택이었다.</v>
       </c>
       <c r="I122" t="str">
-        <v>담임 선생님부터, 생활 관리 선생님들, 기숙 사감 선생님들 덕에 좋은 습관으로 공부할 수 있었습니다!선생님들께서 항상 친절하게 대해주시고, 필요할 때마다 도움을 주셔서 감사했다. 공부를 하면서 힘들 때도 있었지만, 응원해주시고 방향을 잡아주신 덕분에 끝까지 버틸 수 있었던 것 같다. 과하게 간섭하기보다는 필요한 순간에 도움을 주시는 방식이 오히려 더 편하게 느껴졌고, 그 점이 특히 좋았다. 진심으로 감사드립니다.</v>
+        <v>담임 선생님부터, 생활 관리 선생님들, 기숙 사감 선생님들 덕에 좋은 습관으로 공부할 수 있었습니다!선생님들께서 항상 친절하게 대해 주시고, 필요할 때마다 도움을 주셔서 감사했다. 공부를 하면서 힘들 때도 있었지만, 응원해 주시고 방향을 잡아주신 덕분에 끝까지 버틸 수 있었던 것 같다. 과하게 간섭하기보다는 필요한 순간에 도움을 주시는 방식이 오히려 더 편하게 느껴졌고, 그 점이 특히 좋았다. 진심으로 감사드립니다.</v>
       </c>
       <c r="J122" t="str">
         <v>일정한 생활 패턴을 유지하고, 공부에만 집중할 수 있는 환경 속에서 자연스럽게 학습 루틴을 잡을 수 있었어요.</v>
@@ -4822,11 +4822,11 @@
         <v>N수생</v>
       </c>
       <c r="E123" t="str" xml:space="preserve">
-        <v xml:space="preserve">6월 모의고사 성적과 9월 모의고사 성적을 바탕으로 선생님께서 수시 원서상담을 친절하게 진행해주셔서 도움이 많이 됐어 제 성적대에 맞는 대학을 추천해 주셔서 감사했습니다 과도한 상향원서 작성이_x000d_
-아닌 현실적으로 가능한 원서를 작성하게끔 해주셔서 안정적으로 입시를 마무리했습니다</v>
+        <v xml:space="preserve">6월 모의고사 성적과 9월 모의고사 성적을 바탕으로 선생님께서 수시 원서상담을 친절하게 진행해 주셔서 도움이 많이 됐어 제 성적대에 맞는 대학을 추천해 주셔서 감사했습니다 과도한 상향원서 작성이_x000d_
+아닌 현실적으로 가능한 원서를 작성하게끔 해 주셔서 안정적으로 입시를 마무리했습니다</v>
       </c>
       <c r="F123" t="str" xml:space="preserve">
-        <v xml:space="preserve">따로 과외나 학원을 다니기에는 학원비가 부담스럽고 시간적 여유도 없는데 과목에 대해 잘 알고있고 스킬이 있는 선생님들께서 1:1 시간제한없이 질의응답해주셔서 도움이 많이 됐습니다 _x000d_
+        <v xml:space="preserve">따로 과외나 학원을 다니기에는 학원비가 부담스럽고 시간적 여유도 없는데 과목에 대해 잘 알고있고 스킬이 있는 선생님들께서 1:1 시간제한없이 질의응답해 주셔서 도움이 많이 됐습니다 _x000d_
 친절하세요</v>
       </c>
       <c r="G123" t="str">
@@ -4862,7 +4862,7 @@
         <v>모의고사 점수를 비교 분석하여 이전보다 무엇이 부족했고, 어떤 점이 늘었는지를 보다 객관적으로 알 수 있었다. 또한 평소에도 어떻게 공부할지에 대해 상담이 가능한 점이 도움이 되었다.</v>
       </c>
       <c r="F124" t="str">
-        <v>모르는 문제나 헷갈리는 개념에 대해서 1대1 질의 응답이 가능한 점이 마음에 들었다. 자세히 물어봐도 친절하게 답해주시고 더불어 학습 팁도 알려주셔서 공부하는 방향을 잡기에 도움이 되었다.</v>
+        <v>모르는 문제나 헷갈리는 개념에 대해서 1대1 질의 응답이 가능한 점이 마음에 들었다. 자세히 물어봐도 친절하게 답해 주시고 더불어 학습 팁도 알려주셔서 공부하는 방향을 잡기에 도움이 되었다.</v>
       </c>
       <c r="G124" t="str">
         <v>아침부터 학원에 와야 하기에 전자 출결 제도를 이용하면 반강제적으로라도 학원에 늦지 않게 올 수 있게 된다. 또한 출석 알림이 부모님께 가기 때문에 더더욱 늦지 않으려고 일찍 일어났다.</v>
@@ -4871,7 +4871,7 @@
         <v>학원에 다니게 되면 조건 없이 이투스 구독권을 제공하는데 비용적 측면에서 매우 도움이 되었다. 또한 패드도 대여가 가능하다고 해서 온라인 강의를 들으며 독학으로 공부하기에 안성맞춤이었다.</v>
       </c>
       <c r="I124" t="str">
-        <v>공부를 하면서 많이 불안하거나 확신이 들지 않을 때도 있었는데 선생님들과 상담하면서 그러한 고민들이 해소되었고 계획한 대로 공부를 잘 마무리할 수 있었습니다! 잘 지도해주셔서 감사합니다!</v>
+        <v>공부를 하면서 많이 불안하거나 확신이 들지 않을 때도 있었는데 선생님들과 상담하면서 그러한 고민들이 해소되었고 계획한 대로 공부를 잘 마무리할 수 있었습니다! 잘 지도해 주셔서 감사합니다!</v>
       </c>
       <c r="J124" t="str">
         <v>모의고사 성적 분석으로 부족한 부분을 객관적으로 파악하고, 1:1 질의응답을 통해 모르는 개념을 정확히 이해할 수 있었어요.</v>
@@ -4894,7 +4894,7 @@
         <v>N수생</v>
       </c>
       <c r="E125" t="str" xml:space="preserve">
-        <v xml:space="preserve">코칭해주시는 선생님이 전과목의 진행상태와 학습 수준에 대해 꼼꼼히 파악하시고 모르는 부분에 대해서도 설명해주셔서 너무 좋았던 것 같다._x000d_
+        <v xml:space="preserve">코칭해주시는 선생님이 전과목의 진행상태와 학습 수준에 대해 꼼꼼히 파악하시고 모르는 부분에 대해서도 설명해 주셔서 너무 좋았던 것 같다._x000d_
 각 과목별로 전문가 선생님들이 계셨던것도 너무 좋았다</v>
       </c>
       <c r="F125" t="str">
@@ -4911,7 +4911,7 @@
       <c r="I125" t="str" xml:space="preserve">
         <v xml:space="preserve">감사했습니다_x000d_
 힘들 때도 많았지만 잘 다잡아 주셔서 수험 생활 잘 마무리 한 것 같습니다_x000d_
-학습 선생님과 카윤터에 계신 선생님들 모두 정말 감사했습니다 항상 친절하게 대해주시고 잘 잡아주셔서 너무 좋았습니다</v>
+학습 선생님과 카윤터에 계신 선생님들 모두 정말 감사했습니다 항상 친절하게 대해 주시고 잘 잡아주셔서 너무 좋았습니다</v>
       </c>
       <c r="J125" t="str">
         <v>힘들 때도 많았지만 잘 다잡아 주셔서 수험 생활을 잘 마무리한 것 같아요.</v>
@@ -4939,7 +4939,7 @@
 선생님들께서 저라는 사람 자체를 존중해주는 기분이 들었고 제게 맞는 도움을 주셔서 심적으로도 안정이 되었었습니다.</v>
       </c>
       <c r="F126" t="str" xml:space="preserve">
-        <v xml:space="preserve">선생님들이 직접 저 한 명의 상황을 봐 주시고 피드백을 제공해주셔서 좋았습니다._x000d_
+        <v xml:space="preserve">선생님들이 직접 저 한 명의 상황을 봐 주시고 피드백을 제공해 주셔서 좋았습니다._x000d_
 인강을 고르며 어려움을 겪고 있을 때도, 저를 개인적으로 불러 다양한 인강들을 추천해주시며 도움을 주셨습니다.</v>
       </c>
       <c r="G126" t="str">
@@ -4952,7 +4952,7 @@
       </c>
       <c r="I126" t="str" xml:space="preserve">
         <v xml:space="preserve">덕분에 제 불안했던 반수 생활을 잘 견뎌낼 수 있었습니다. 감사합니다._x000d_
-제 멘탈이 무너질 때마다 응원해주시고 붙잡아주셔서, 수능 공부뿐만 아니라 다른 분야에서도 자신감을 얻을 수 있게 되었습니다. 잘 챙겨주셔서 감사합니다.</v>
+제 멘탈이 무너질 때마다 응원해 주시고 붙잡아주셔서, 수능 공부뿐만 아니라 다른 분야에서도 자신감을 얻을 수 있게 되었습니다. 잘 챙겨주셔서 감사합니다.</v>
       </c>
       <c r="J126" t="str">
         <v>원장님과 선생님들께서 제 학습 상황을 세심하게 파악하고 맞춤 계획을 제시해 주셔서 심적으로도 안정감을 얻을 수 있었어요.</v>
@@ -5022,7 +5022,7 @@
         <v>매일 요일마다 다른 과목으로  수능특강이나 수능완성 등 수능에서 보는 시험과 관련된 교재로 테스트를 보는것이 사실상 가장 큰 메리트 였다고 본다. 학교에서는 딱히 수능을 위한 시험이 많이 없어서 아쉬웠지만 이투스에서는 시험형태로 보기 때문에 도움이 되었다고 생각한다</v>
       </c>
       <c r="I128" t="str">
-        <v>초반에는 자리가 불편하진 않는지 전체적인 방 분위기가 괜찮은지 계속 여쭤봐주시고 쉬는시간이나 점심시간에 계속 힘내라고 말씀해주신 덕분에 지치지 않고 수험 생활을 잘 보낼 수 있었습니다 감사합니다</v>
+        <v>초반에는 자리가 불편하진 않는지 전체적인 방 분위기가 괜찮은지 계속 여쭤봐주시고 쉬는시간이나 점심시간에 계속 힘내라고 말씀해 주신 덕분에 지치지 않고 수험 생활을 잘 보낼 수 있었습니다 감사합니다</v>
       </c>
       <c r="J128" t="str">
         <v>나만의 시간표와 교재·학습 방법 안내 덕분에 공부를 시작하는 방향을 잡고, 꾸준한 학습 습관까지 만들 수 있었어요.</v>
@@ -5080,7 +5080,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E130" t="str">
-        <v>선생님들의 학습 경험에 기반한 진짜 도움되는 꿀팁들을 상담을 통해 많이 얻었어요. 특히 고3이 되면서 인강을 처음 듣기 시작했는데, 커리큘럼도 진지하게 함께 고민해주시고 저에게 맞는 학습 커리큘럼을 구성해주셔서 맞지 않는 강의 들으며 버리는 시간이 없어서 좋았습니다. 특히 플래너를 주기적으로 검사하고 코멘트를 적어주셔서 저의 학습방향이 맞는지에 대한 조언을 듣고 커리큘럼에 대한 확신이 생겼었습니다!</v>
+        <v>선생님들의 학습 경험에 기반한 진짜 도움되는 꿀팁들을 상담을 통해 많이 얻었어요. 특히 고3이 되면서 인강을 처음 듣기 시작했는데, 커리큘럼도 진지하게 함께 고민해 주시고 저에게 맞는 학습 커리큘럼을 구성해 주셔서 맞지 않는 강의 들으며 버리는 시간이 없어서 좋았습니다. 특히 플래너를 주기적으로 검사하고 코멘트를 적어주셔서 저의 학습방향이 맞는지에 대한 조언을 듣고 커리큘럼에 대한 확신이 생겼었습니다!</v>
       </c>
       <c r="F130" t="str">
         <v>스스로 자주적인 공부를 처음 시작할 때 가장 막막한 것이 계획세우기인데, 계획의 전체적인 방향성과 흐름을 1차적으로 잡아주고 계속해서 피드백하며 저에게 맞게 커리큘럼을 구성할 수 있도록 하는 컨설팅의 방식이 추후 학습에도 큰 도움이 됐었습니다.</v>
@@ -5092,7 +5092,7 @@
         <v>단어는 스스로 외우려고 해도 채점답안이 저에게 있기 때문에 순전히 저의 양심에만 맡겨야하고, 매일매일 규칙적으로 하기는 어렵습니다. 그런데 그 점을 모두 이투스에서 관리해주어 저는 단어만 외우면 되고, 매일매일 외울 수 있게 되어 좋았습니다. 또 재시도 철저하게 하고 이름을 게시함으로써 스스로 부끄럼을 느껴 더 열심히 하게 되었습니다.</v>
       </c>
       <c r="I130" t="str">
-        <v>추운 겨울방학 내내 따뜻하게 웃으며 맞이해주시고 학습이 지속적으로 이루어질 수 있도록 관리해 주셔서 감사합니다! 또 멘토 선생님들 덕분에 많이 배우고 성장할 수 있었어요. 항상 신경 써주시고 도와주셔서 진심으로 감사합니다!</v>
+        <v>추운 겨울방학 내내 따뜻하게 웃으며 맞이해 주시고 학습이 지속적으로 이루어질 수 있도록 관리해 주셔서 감사합니다! 또 멘토 선생님들 덕분에 많이 배우고 성장할 수 있었어요. 항상 신경 써주시고 도와주셔서 진심으로 감사합니다!</v>
       </c>
       <c r="J130" t="str">
         <v>상담을 통해 제게 맞는 인강 커리큘럼을 함께 구성하고, 주기적인 플래너 점검으로 학습 방향에 대한 확신을 얻을 수 있었어요.</v>
@@ -5150,13 +5150,13 @@
         <v>N수생</v>
       </c>
       <c r="E132" t="str">
-        <v>힘들고 지칠 때마다 마음을 다잡을 수 있도록 도와주셨던 상담이 정말 큰 힘이 되었습니다. 선생님들께서 해주신 진심 어린 조언과 따뜻한 공감 덕분에 흔들리던 제 자신을 다시 바로 세울 수 있었고, 그 과정에서 정신적으로 큰 위로와 용기를 얻을 수 있었습니다.</v>
+        <v>힘들고 지칠 때마다 마음을 다잡을 수 있도록 도와주셨던 상담이 정말 큰 힘이 되었습니다. 선생님들께서 해 주신 진심 어린 조언과 따뜻한 공감 덕분에 흔들리던 제 자신을 다시 바로 세울 수 있었고, 그 과정에서 정신적으로 큰 위로와 용기를 얻을 수 있었습니다.</v>
       </c>
       <c r="F132" t="str">
-        <v>힘들고 지칠 때마다 마음을 다잡을 수 있도록 도와주셨던 상담이 정말 큰 힘이 되었습니다. 선생님들께서 해주신 진심 어린 조언과 따뜻한 공감 덕분에 흔들리던 제 자신을 다시 바로 세울 수 있었고, 학습 플래너 관리까지 체계적으로 도와주셔서 공부 방향을 잃지 않고 꾸준히 나아갈 수 있었습니다.</v>
+        <v>힘들고 지칠 때마다 마음을 다잡을 수 있도록 도와주셨던 상담이 정말 큰 힘이 되었습니다. 선생님들께서 해 주신 진심 어린 조언과 따뜻한 공감 덕분에 흔들리던 제 자신을 다시 바로 세울 수 있었고, 학습 플래너 관리까지 체계적으로 도와주셔서 공부 방향을 잃지 않고 꾸준히 나아갈 수 있었습니다.</v>
       </c>
       <c r="G132" t="str">
-        <v>힘들고 지칠 때마다 마음을 다잡을 수 있도록 도와주셨던 상담이 정말 큰 힘이 되었습니다. 선생님들께서 해주신 진심 어린 조언과 따뜻한 공감 덕분에 흔들리던 제 자신을 다시 바로 세울 수 있었고, 학습 플래너 관리까지 체계적으로 도와주셔서 공부 방향을 잃지 않고 꾸준히 나아갈 수 있었습니다. 또한 출석 시 휴대폰을 관리해 주셔서 불필요한 사용을 줄이고, 공부에 더욱 집중할 수 있는 환경이 만들어진 점도 큰 도움이 되었습니다.</v>
+        <v>힘들고 지칠 때마다 마음을 다잡을 수 있도록 도와주셨던 상담이 정말 큰 힘이 되었습니다. 선생님들께서 해 주신 진심 어린 조언과 따뜻한 공감 덕분에 흔들리던 제 자신을 다시 바로 세울 수 있었고, 학습 플래너 관리까지 체계적으로 도와주셔서 공부 방향을 잃지 않고 꾸준히 나아갈 수 있었습니다. 또한 출석 시 휴대폰을 관리해 주셔서 불필요한 사용을 줄이고, 공부에 더욱 집중할 수 있는 환경이 만들어진 점도 큰 도움이 되었습니다.</v>
       </c>
       <c r="H132" t="str">
         <v>이투스 모의고사를 통해 실전과 같은 환경에서 문제를 풀어볼 수 있어 큰 도움이 되었습니다. 다양한 유형의 문제를 경험하며 약점을 파악할 수 있었고, 성적 분석을 통해 부족한 부분을 보완할 수 있었습니다. 꾸준한 모의고사 응시로 시간 관리 능력과 실전 감각을 키울 수 있었던 점이 가장 좋았습니다.</v>
@@ -5197,7 +5197,7 @@
         <v>따로 영어 단어 공부를 많이 하지 않아도 정리 해 주신 수능 특강, 수능 완성 영어 단어집을 바탕으로한 저녁 식사 후 보는 테스트를 통해 실력을 많이 향상 할 수 있어 좋은 컨텐츠였다고 생각합니다.</v>
       </c>
       <c r="I133" t="str">
-        <v>혼자 공부하는 것 보다 실력이 더욱 향상되었다고 생각하고 출결 관리나 졸음 방지 등 여러 관리들 또한 도움이 되었습니다. 또한 항상 친절하고 도움이 되는 말만 해주신 선생님들께 감사하다고 말하고 싶습니다.</v>
+        <v>혼자 공부하는 것 보다 실력이 더욱 향상되었다고 생각하고 출결 관리나 졸음 방지 등 여러 관리들 또한 도움이 되었습니다. 또한 항상 친절하고 도움이 되는 말만 해 주신 선생님들께 감사하다고 말하고 싶습니다.</v>
       </c>
       <c r="J133" t="str">
         <v>모의고사를 보고 성적을 기록해 주시며 상담해 주는 것이 좋았어요.</v>
@@ -5232,7 +5232,7 @@
         <v>영어공부 중에서 단어를 외우는 것은 중요하다. 그치만 단어를 스스로 외우는 것은 쉽지 않은 일이다. 학원에서 단어테스트를 진행함으로써 강제적으로 단어를 매일매일 외울 수 있어서 도움이 되었다.</v>
       </c>
       <c r="I134" t="str">
-        <v>등원할 때, 하원할 때 항상 밝은 얼굴로 인사해주셔서 감사했어요. 짧은 인사지만 덕분에 저도 웃으면서 학원에 들어오고 나올 수 있었어요! 그리고 매번 모의고사 볼 때마다 꼼꼼하게 신경써주셔서 감사합니다.</v>
+        <v>등원할 때, 하원할 때 항상 밝은 얼굴로 인사해 주셔서 감사했어요. 짧은 인사지만 덕분에 저도 웃으면서 학원에 들어오고 나올 수 있었어요! 그리고 매번 모의고사 볼 때마다 꼼꼼하게 신경써주셔서 감사합니다.</v>
       </c>
       <c r="J134" t="str">
         <v>MY247에서 온라인으로 계획을 작성을 하니까 나의 공부 시간 비중, 패턴을 쉽게 파악할 수 있었어요.</v>
@@ -5255,7 +5255,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E135" t="str">
-        <v>매일 매일 학습 계획을 짤 때 체계적이고 실행가능하게 짤 수 있도록 도와주셔서 도움이 많이 되었다. 또한 어느 부분이 부족하고 어느부분을 더 공략해야 하는지 상담을 잘 해주셔서 도움이 많이 되었다</v>
+        <v>매일 매일 학습 계획을 짤 때 체계적이고 실행가능하게 짤 수 있도록 도와주셔서 도움이 많이 되었다. 또한 어느 부분이 부족하고 어느부분을 더 공략해야 하는지 상담을 잘 해 주셔서 도움이 많이 되었다</v>
       </c>
       <c r="F135" t="str">
         <v>학습 일정, 계획을 짤 때 도움이 많이 되었고 계획적으로 학습을 할 수 있어서 좋았다. 또한 매일 얼만큼 공부를 했는지 체크할 수 있어서 나의 학습현황도 확인하기에 유용해서 도움이 많이 되었다</v>
@@ -5267,7 +5267,7 @@
         <v>이투스 강의를 무료로 들을 수 있다는 것이 가장 큰 메리트였다. 가성비있게 들을 수 있고 이투스 온라인 강의를 통해 1타강사들의 강의를 들으며 나의 학습능력을 더 키울 수 있어 도움이 많이 되었다</v>
       </c>
       <c r="I135" t="str">
-        <v>이투스 다니는 동안 너무 잘 챙겨주시고 상담도 잘 해주셔서 너무 감사했어요. 항상 웃으면서 반겨주시고 배웅해주시던 것이 가장 기억에많이 남는 것 같아요ㅎㅎ 입시상담도 도움마니됐어요 너무 감사했습니다!!!</v>
+        <v>이투스 다니는 동안 너무 잘 챙겨주시고 상담도 잘 해 주셔서 너무 감사했어요. 항상 웃으면서 반겨주시고 배웅해주시던 것이 가장 기억에많이 남는 것 같아요ㅎㅎ 입시상담도 도움마니됐어요 너무 감사했습니다!!!</v>
       </c>
       <c r="J135" t="str">
         <v>학습 계획을 짤 때 체계적이고 실행 가능하게 짤 수 있도록 도와주셔서 도움이 많이 되었어요.</v>
@@ -5325,16 +5325,16 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E137" t="str">
-        <v>여러 비슷한 유형의 학원을 다녀본 결과 이투스247만의 특별한 장점은 대학생 멘토분께서 1:1로 학생들 담당하여 매주 학습 코칭을 해주신다는 것이었습니다. 학생 개개인의 상황에 맞는 적절한 피드백과 공부 계획을 함께 고민해주시고 방향을 잡아주셔서  큰 도움이 되었습니다.</v>
+        <v>여러 비슷한 유형의 학원을 다녀본 결과 이투스247만의 특별한 장점은 대학생 멘토분께서 1:1로 학생들 담당하여 매주 학습 코칭을 해 주신다는 것이었습니다. 학생 개개인의 상황에 맞는 적절한 피드백과 공부 계획을 함께 고민해 주시고 방향을 잡아주셔서  큰 도움이 되었습니다.</v>
       </c>
       <c r="F137" t="str">
-        <v>어떤 강사의 강의를 듣고, 어떤 유형의 교재를 결정할지는 수능을 준비하는 학생들에게 가장 큰 고민이라는 생각이 드는데, 멘토분께서 저에게 가장 적합한 커리큘럼을 제시해 주셔서  좋았습니다. 특히 지금 상황에서 추천하지 않는 강의를 지적해주셔서 제 계획을 수정하는 데에 도움이 되었습니다.</v>
+        <v>어떤 강사의 강의를 듣고, 어떤 유형의 교재를 결정할지는 수능을 준비하는 학생들에게 가장 큰 고민이라는 생각이 드는데, 멘토분께서 저에게 가장 적합한 커리큘럼을 제시해 주셔서  좋았습니다. 특히 지금 상황에서 추천하지 않는 강의를 지적해 주셔서 제 계획을 수정하는 데에 도움이 되었습니다.</v>
       </c>
       <c r="G137" t="str">
-        <v>독학재수 학원을 다닌 가장 큰 이유였습니다. 혼자서 독서실에 가 공부를 했을 때는 빈번하게 폰을 확인하며 공부에 집중하지 못하고 딴 짓을 하는 경우가 많았는데, 이투스247 학원에서는 등원과 함께 폰을 수거해주셔서 오로지 공부에만 집중할 수 있었습니다.</v>
+        <v>독학재수 학원을 다닌 가장 큰 이유였습니다. 혼자서 독서실에 가 공부를 했을 때는 빈번하게 폰을 확인하며 공부에 집중하지 못하고 딴 짓을 하는 경우가 많았는데, 이투스247 학원에서는 등원과 함께 폰을 수거해 주셔서 오로지 공부에만 집중할 수 있었습니다.</v>
       </c>
       <c r="H137" t="str">
-        <v>영어가 가장 취약한 과목이었어서 단어 암기가 가장 필요했었는데, 혼자서 단어장을 가지고 외우기엔 규칙적인 학습과 복습을 하지 못했습니다. 이투스247에서는 매일 점심시간 학원의 계획표에 따라 정해진 범위의 단어 테스트를 제공해주셔서, 단어 암기에 정말 큰 도움이 되었습니다.</v>
+        <v>영어가 가장 취약한 과목이었어서 단어 암기가 가장 필요했었는데, 혼자서 단어장을 가지고 외우기엔 규칙적인 학습과 복습을 하지 못했습니다. 이투스247에서는 매일 점심시간 학원의 계획표에 따라 정해진 범위의 단어 테스트를 제공해 주셔서, 단어 암기에 정말 큰 도움이 되었습니다.</v>
       </c>
       <c r="I137" t="str">
         <v>2학기 도중 수시 전형으로 입시를 결정하게 되어 일찍 학원에서 퇴원하게 되었지만, 매일 밝게 인사해주시는 원장님과 졸고 있을 때마다 와서 깨워주시는 조교선생님분들 덕분에 고3 동안 열심히 공부할 수 있었습니다. 감사합니다!</v>
@@ -5511,7 +5511,7 @@
       </c>
       <c r="F142" t="str" xml:space="preserve">
         <v xml:space="preserve">보통 혼자 공부하다보면 자기가 잘하는 과목에 더 몰입하게되고 이러면서 규칙적이고 꾸준히해서 감각을 잃으면 안되는 국,영,수 과목에서 감을 잃을 수 있는 단점이 있는데 자신의_x000d_
-플래너를 확인하시고 저의 학습방향을 확인해주시고 진도량도 확인해주시니까 내가 느리구나 잘하고 있구나 이런 것들을 객관적으로 확인할 수 있으니까 항상 나를 돌아보고 다시 잘해보자라는 마음가짐을 다시 다잡을 수 있었던 것 같아요</v>
+플래너를 확인하시고 저의 학습방향을 확인해 주시고 진도량도 확인해주시니까 내가 느리구나 잘하고 있구나 이런 것들을 객관적으로 확인할 수 있으니까 항상 나를 돌아보고 다시 잘해보자라는 마음가짐을 다시 다잡을 수 있었던 것 같아요</v>
       </c>
       <c r="G142" t="str">
         <v>졸고 있으면 깨워주시는 경우도 많고 다른 친구들이 딴짓하면 분위기 따라서 잘못되게 나도 딴짓을 하거나 시끄러운 환경을 만들 수 있는데 단체활동이다 보니까 학원 내 규정을 통해 제대로 관리해주시니까 나는 절대 저러지 말아야지라는 책임감이 생기는 것 같아요. 또한 진짜 힘들하는 부분에 있어서는 세세하게 챙겨주시기때문에 혼자 학습하는 것과는 다르게 나의 최대를 해내기 위해서 더 노력하게 된다는 점? 이런 게 되게 좋은 것 같습니다</v>
@@ -5520,7 +5520,7 @@
         <v>자기실력을 객관화해서 알아보는 게 중요한 게 달마다 이투스 모의고사를 치뤄주니까 나의 실력의 객관적위치도 확인하고 내가 어디서 약점이 드러나고 강점이 드러나는 지 알 수 있으니까 이를 토대로 이후 학습 계획을 짜는 것에도 굉장히 도움됨. 그리고 성적이 낮을때는 맘적으로 힘든 것도 있지만 굉장히 다음날부터 동기부여되는 부분도 있고 잘볼 경우에는 더 잘보고 싶다는 동기부여가 생기기때문에 이는 되게 좋은 정기 모의고사의 장점이 아닐까 싶습니다</v>
       </c>
       <c r="I142" t="str">
-        <v>항상 따듯하게 맞이해주시고 항상 응원해주는 혼내시더라고 저희를 위한 것이라는 게 느껴져서 항상 감사했습니다. 강압적인 분위기라는 게 너무 힘들었지만 모든게 저희를 위한 것이라는 것들을 돌아보면서 감사한 마음밖에 안듭니다. 제 인생에 큰도움이 된 것 같아여 감사합니다</v>
+        <v>항상 따듯하게 맞이해 주시고 항상 응원해주는 혼내시더라고 저희를 위한 것이라는 게 느껴져서 항상 감사했습니다. 강압적인 분위기라는 게 너무 힘들었지만 모든게 저희를 위한 것이라는 것들을 돌아보면서 감사한 마음밖에 안듭니다. 제 인생에 큰도움이 된 것 같아여 감사합니다</v>
       </c>
       <c r="J142" t="str">
         <v>정기적으로 실전 모의고사를 보며 제 실력을 객관적으로 확인하고 다음 학습 계획을 세울 수 있었어요.</v>
@@ -5543,7 +5543,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E143" t="str">
-        <v>항상 내신 공부에만 집중했어서 수능공부를 제대로 해본적이 없었다. 그 고3 여름방학에 수능공부를 하려는데 막막한 부분이 정말 많았다. 그러나 일주일에 한 두번씩 담당 선생님과 상담을 하면서 과목 별 어떻게 공부하면 더 효과적인지를 알 수 있었다. 특히 국어 과목을 너무 못했어서 고민이 많았는데 담당 선생님께서 어떤 순서로 풀지, 어떻게 글을 읽는게 나에게 더 효과적일지 등을 직접적으로 설명해주셔서 정말 도움이 많이 되었고 그렇게 코칭을 받고 실제로 한 두등급 성적이 향상 되었다</v>
+        <v>항상 내신 공부에만 집중했어서 수능공부를 제대로 해본적이 없었다. 그 고3 여름방학에 수능공부를 하려는데 막막한 부분이 정말 많았다. 그러나 일주일에 한 두번씩 담당 선생님과 상담을 하면서 과목 별 어떻게 공부하면 더 효과적인지를 알 수 있었다. 특히 국어 과목을 너무 못했어서 고민이 많았는데 담당 선생님께서 어떤 순서로 풀지, 어떻게 글을 읽는게 나에게 더 효과적일지 등을 직접적으로 설명해 주셔서 정말 도움이 많이 되었고 그렇게 코칭을 받고 실제로 한 두등급 성적이 향상 되었다</v>
       </c>
       <c r="F143" t="str">
         <v>담당 선생님께서 내가 풀었던 시험지를 직접 보시고 어떤점을 어떻게 풀었고 왜이렇게 생각했는지 등 자세히 물어보면서 내 약점은 무엇이고 항상 하는 실수는 왜 하게 되는지를 같이 찾아봐주시면서 내가 가장 부족한 부분이 뭔지 잘 알려주셨다. 또한 담당 선생님의 노하우도 알려주시면서 그 부족한 점을 메꾸어나가게 지속적인 티칭을 하셨고 그러한 점이 성적 향상에 보탬이 됐다고 생각한다.</v>
@@ -5661,7 +5661,7 @@
       </c>
       <c r="I146" t="str" xml:space="preserve">
         <v xml:space="preserve">원장쌤, 태은쌤 덕분에 모자란 제가 지거국에라도 합격 할 수 있었습니다_x000d_
-졸려고 하면 바로 깨워주시고 딴 짓 하려고 하면 바로 방해해주시고 모든 쌤들이 도와주셔서 제가 대학에 갈 수 있었습니다_x000d_
+졸려고 하면 바로 깨워주시고 딴 짓 하려고 하면 바로 방해해 주시고 모든 쌤들이 도와주셔서 제가 대학에 갈 수 있었습니다_x000d_
 감사합니다. 군대 가기전에 찾아뵙겠습니다._x000d_
 원주 이투스 화이팅_x000d_
 _x000d_
@@ -5702,7 +5702,7 @@
         <v>학력평가를 매달 보지 않아서 모의고사에 대한 감이 부족했는데 이투스 모의고사를 매달 봐서 모의고사에 대한 감을 키우고 유지할 수 있었음. 또한 트렌드에 맞게 문제를 출제하고 수능특강과 적절하게 연계한 문제를 내서 복습도 할 수 있었음.</v>
       </c>
       <c r="I147" t="str">
-        <v>항상 따뜻한 마음으로 지도해주시고, 공부에 집중할 수 있는 좋은 환경을 만들어주셔서 진심으로 감사드립니다. 선생님들의 세심한 배려와 응원 덕분에 더욱 성실하게 노력할 수 있었습니다.</v>
+        <v>항상 따뜻한 마음으로 지도해 주시고, 공부에 집중할 수 있는 좋은 환경을 만들어주셔서 진심으로 감사드립니다. 선생님들의 세심한 배려와 응원 덕분에 더욱 성실하게 노력할 수 있었습니다.</v>
       </c>
       <c r="J147" t="str">
         <v>국어가 가장 취약 과목이었는데, 담임 선생님과의 상담을 통해 공부 방법과 글 읽는 방향을 바로잡아 성적 향상에 큰 도움이 되었어요.</v>
@@ -5734,17 +5734,17 @@
         <v>출석 시 전자기기를 제출 함으로써 공부에 가장 방해되는 요소인 핸드폰을 제거해서 긴 시간동안 학원에 머무르는데도 불구하고 집중력을 유지할 수 있게 된거 같습니다 또 휴식시간에도 핸드폰을 주지 않으셔서 온전하게 휴식을 하게 되어서 쉬는 시간 후 공부를 할 때 큰 도움을 받았던거 같습니다</v>
       </c>
       <c r="H148" t="str">
-        <v>제가 영어가 가장 취약한 과목이었는데 고3에는 매일 단어를 외우지 않았습니다 하지만 이투스 247학원에 오면서 매일 의무적으로 단어를 40개씩 외우게 해주셔서 영어 실력의 기본기가 갖춰지게 된거 같습니다 또 일일테스트 뿐만 아니라 토요일에 실행하는 단어 총정리 테스트를 통해 복습을 꾸준하게 진행할 수 있어서 좋았습니다</v>
+        <v>제가 영어가 가장 취약한 과목이었는데 고3에는 매일 단어를 외우지 않았습니다 하지만 이투스 247학원에 오면서 매일 의무적으로 단어를 40개씩 외우게 해 주셔서 영어 실력의 기본기가 갖춰지게 된거 같습니다 또 일일테스트 뿐만 아니라 토요일에 실행하는 단어 총정리 테스트를 통해 복습을 꾸준하게 진행할 수 있어서 좋았습니다</v>
       </c>
       <c r="I148" t="str" xml:space="preserve">
-        <v xml:space="preserve">재수 생활 함께 해주셔서 감사합니다_x000d_
-재수 생활 함께 해주셔서 감사합니다_x000d_
-재수 생활 함께 해주셔서 감사합니다_x000d_
-재수 생활 함께 해주셔서 감사합니다_x000d_
-재수 생활 함께 해주셔서 감사합니다_x000d_
-재수 생활 함께 해주셔서 감사합니다_x000d_
-재수 생활 함께 해주셔서 감사합니다_x000d_
-재수 생활 함께 해주셔서 감사합니다</v>
+        <v xml:space="preserve">재수 생활 함께 해 주셔서 감사합니다_x000d_
+재수 생활 함께 해 주셔서 감사합니다_x000d_
+재수 생활 함께 해 주셔서 감사합니다_x000d_
+재수 생활 함께 해 주셔서 감사합니다_x000d_
+재수 생활 함께 해 주셔서 감사합니다_x000d_
+재수 생활 함께 해 주셔서 감사합니다_x000d_
+재수 생활 함께 해 주셔서 감사합니다_x000d_
+재수 생활 함께 해 주셔서 감사합니다</v>
       </c>
       <c r="J148" t="str">
         <v>모의고사 후 바로 피드백을 받고, 궁금한 문제도 빠르게 질문하며 해결할 수 있어 공부 흐름을 이어가기 좋았어요.</v>
@@ -5767,7 +5767,7 @@
         <v>N수생</v>
       </c>
       <c r="E149" t="str">
-        <v>제가 어떻게 학습을 시작해야 할지 막막했는데 한 가지 방법만 조언해 주시는 게 아닌, 과목별로 방향성을 잡아주셔서 저의 기존 방법과 선생님이 조언해주신 방법들이 적절히 섞일 수 있었던 점이 가장 좋았습니다!</v>
+        <v>제가 어떻게 학습을 시작해야 할지 막막했는데 한 가지 방법만 조언해 주시는 게 아닌, 과목별로 방향성을 잡아주셔서 저의 기존 방법과 선생님이 조언해 주신 방법들이 적절히 섞일 수 있었던 점이 가장 좋았습니다!</v>
       </c>
       <c r="F149" t="str">
         <v>가장 좋았던 코칭 시스템과 연관된 내용으로 여러 방향 중에서 각각 방향에 맞는 인강이나 교재 혹은 문제 하나하나 마저도 알려주셨던게 가장 도움이 되고, 특히 문제 추천은 제가 부족한 부분을 집중적으로 채울 수 있어서 가장 유용했습니다.</v>
@@ -5837,7 +5837,7 @@
         <v>N수생</v>
       </c>
       <c r="E151" t="str">
-        <v>국어 공부가 가장하기도 어렵고 어떻게 해야 할지 막막했는데 저한테 맞춰서 정말 세세하게 신경써주시면서 코핑해주셔서 좋았습니다. 코칭 할때마다 국어 공부는 어떤지 어떤부분이 잘안되는지 물어봐주셔서 공부하는데 많은 도움이 되었습니다</v>
+        <v>국어 공부가 가장하기도 어렵고 어떻게 해야 할지 막막했는데 저한테 맞춰서 정말 세세하게 신경써주시면서 코핑해 주셔서 좋았습니다. 코칭 할때마다 국어 공부는 어떤지 어떤부분이 잘안되는지 물어봐주셔서 공부하는데 많은 도움이 되었습니다</v>
       </c>
       <c r="F151" t="str">
         <v>아침에 꾸준히 학습 계획을 쓰게 되면서 하루 목표 공부량과 시간을 정확히 알 수 있어서 좋았고 꾸준히 쓰다보니 진도도 안밀리고 부족한부분 보완할점도 같이 알려주셔서 공부하는데 많은 도움을 받았습니다</v>
@@ -5849,7 +5849,7 @@
         <v>혼자공부할때는 영어단어 안외우고 계속 미루게되었는데 이투스247에서는 아침마다 테스트를 보고 통과했어야하기 때문에 꾸준히 외우게되서 전보다 암기량과 암기속도 모두 좋아져서 도움이 되었습니다.</v>
       </c>
       <c r="I151" t="str">
-        <v>현역때 공부를 정말 많이 안했어서 재수를 어떻게 시작해야 할지 공부는 어떻게해야 하는지 정말 막막했었는데 공부법이랑 공부관리.상담 잘해주시고 1년 동안 재수하는데 많은 도움주셔서 정말 감사합니다.</v>
+        <v>현역때 공부를 정말 많이 안했어서 재수를 어떻게 시작해야 할지 공부는 어떻게해야 하는지 정말 막막했었는데 공부법이랑 공부관리.상담 잘해 주시고 1년 동안 재수하는데 많은 도움주셔서 정말 감사합니다.</v>
       </c>
       <c r="J151" t="str">
         <v>아침마다 영단어 테스트를 보며 꾸준히 암기한 덕분에 암기량과 속도를 함께 높일 수 있었어요.</v>
@@ -5884,7 +5884,7 @@
         <v>모의고사가 이투스 자체 모의고사를 제외하고는 따로 풀 기회가 먾이 없습니다. 그렇기에 매번 이투스 모의고사를 보고 싶었는데요. 문제는 현역이라 따로 시험지를 받고 혼자 풀어봐야 한다는 점이 좀 아쉬웠지만 그래도 나름 잘 활용해서 많아 풀어보고 계속 배워나갈 수 있는 부분이였던 것 같습니다!</v>
       </c>
       <c r="I152" t="str">
-        <v>항상 질문도 많고 계속 따라다니며 여쭤보고 그러느라 좀 정신 얎으셨을텐데 끝까지 제 질문 받아주시고 끝까지 앞을 향해 나아갈 수 있게 해주셔서 너무 감사했습니다. 비록 정시가 아닌 수시로 대학을 갔지만 정시에서 성적이 잘 나왔기에 후회는 없는 것 같아요. 덕분에 12년 공부 생활을 잘 마무리하고 새로운 공부 생활을 할 수 있게 도와주셔서 감사합니다!!</v>
+        <v>항상 질문도 많고 계속 따라다니며 여쭤보고 그러느라 좀 정신 얎으셨을텐데 끝까지 제 질문 받아주시고 끝까지 앞을 향해 나아갈 수 있게 해 주셔서 너무 감사했습니다. 비록 정시가 아닌 수시로 대학을 갔지만 정시에서 성적이 잘 나왔기에 후회는 없는 것 같아요. 덕분에 12년 공부 생활을 잘 마무리하고 새로운 공부 생활을 할 수 있게 도와주셔서 감사합니다!!</v>
       </c>
       <c r="J152" t="str">
         <v>학원 선생님께서 매일매일 플래너를 검사하셨고, 피드백도 자주 남겨주셔서 도움이 되었어요.</v>
@@ -5919,7 +5919,7 @@
         <v>영어에 있어서 특히 도움을 많이 받았던 것 같습니다. 영어 단어를 꾸준히 외우는 것에 있어서 어려움을 겪었었는데 단어 시험을 주기적으로 시행하여 꾸준한 학습을 할 수 있었습니다. 혼자 하는 것과 다르게 테스트를 하니 몰랐던 단어와 헷갈렸던 단어를 확실히 알게 되었습니다.</v>
       </c>
       <c r="I153" t="str">
-        <v>윈터스쿨때 다니며 저의 공부 습관을 잡을 수 있었던 것 같습니다. 주기적인 학습 관리와 조언을 해주시고, 학습에 방해가 되지 않도록 휴대폰 관리, 학습 관리에 있어서 도와주신 선생님들께 감사합니다.</v>
+        <v>윈터스쿨때 다니며 저의 공부 습관을 잡을 수 있었던 것 같습니다. 주기적인 학습 관리와 조언을 해 주시고, 학습에 방해가 되지 않도록 휴대폰 관리, 학습 관리에 있어서 도와주신 선생님들께 감사합니다.</v>
       </c>
       <c r="J153" t="str">
         <v>저는 공부하다가 많이 조는 유형인데 졸 때마다 깨워주시는 것과 공부하는 것을 관리, 감독해 주시는 게 도움이 많이 됐어요.</v>
@@ -5980,10 +5980,10 @@
         <v>N수생</v>
       </c>
       <c r="E155" t="str">
-        <v>일단 학습 스케쥴에 방해 되지 않도록 상담일자를 잡아주셔서 좋았다. 그리고 내가 알지 못했던 인강 커리큘럼이나 모의고사 등을 현 수준과 현황에 맞추어 추천해주신 것이 도움이 되었다. 내 학습 진도 상황도 체크해주셔서 더 성실하게 공부를 할 수 있었다.</v>
+        <v>일단 학습 스케쥴에 방해 되지 않도록 상담일자를 잡아주셔서 좋았다. 그리고 내가 알지 못했던 인강 커리큘럼이나 모의고사 등을 현 수준과 현황에 맞추어 추천해 주신 것이 도움이 되었다. 내 학습 진도 상황도 체크해 주셔서 더 성실하게 공부를 할 수 있었다.</v>
       </c>
       <c r="F155" t="str">
-        <v>학습 시간에 인강 자료나 커리큘럼을 둘러보고 찾아보는 것이 매우 큰 시간 낭비라고 느꼈는데 선생님께서 현 상황에 알맞는 것들을 추천 해주셔서 시간을 대폭 절약하고 공부에 집중할 수 있었다</v>
+        <v>학습 시간에 인강 자료나 커리큘럼을 둘러보고 찾아보는 것이 매우 큰 시간 낭비라고 느꼈는데 선생님께서 현 상황에 알맞는 것들을 추천 해 주셔서 시간을 대폭 절약하고 공부에 집중할 수 있었다</v>
       </c>
       <c r="G155" t="str">
         <v>여름 기간에 지치거나 아침에 나도 모르게 졸 때가 많았는데 지속적인 순찰로 잠을 깨워주셔서 경각심을 가지며 학습 할 수 있었다. 벌점을 받지 않으려고 잠을 깨기 위해 노력했던것 같다.</v>
@@ -6053,7 +6053,7 @@
         <v>국어 담당 선생님이신 장유지쌤이 담임을 해주셨는데 공부 계획부터 방향성까지 아주 철저하게 이끌어주셨고 앞에서 문제도 풀면서 즉각적으로 피드백도 받고 혼자 할때는 공부를 이상한 방향으로 할 수도 있었을텐데 선생님이 계셔서 계속 방향을 잡아주셨던게 정말 좋았습니다</v>
       </c>
       <c r="F157" t="str">
-        <v>2주마다 담임 선생님과 상담을 했던게 정말 큰 도움이 됐습니다. 만약에 혼자 공부를 했다면 내가 이 방향으로 가는것이 맞는건가? 라는 생각과 불안함이 많이 들었을텐데 계속 옆에서 방향을 잡아주셨었고, 내가 하루에 이정도 공부는 해야한다를 정해주셔서 그걸 나의 페이스대로 성실하게 할 수 있었고 그걸 계속 체크하면서 검사해주셔서 대충하지 않고 열심히 할 수 있었습니다</v>
+        <v>2주마다 담임 선생님과 상담을 했던게 정말 큰 도움이 됐습니다. 만약에 혼자 공부를 했다면 내가 이 방향으로 가는것이 맞는건가? 라는 생각과 불안함이 많이 들었을텐데 계속 옆에서 방향을 잡아주셨었고, 내가 하루에 이정도 공부는 해야한다를 정해 주셔서 그걸 나의 페이스대로 성실하게 할 수 있었고 그걸 계속 체크하면서 검사해 주셔서 대충하지 않고 열심히 할 수 있었습니다</v>
       </c>
       <c r="G157" t="str">
         <v>일단 원래 앉는 고정좌석이 있었는데 사실 처음에는 너무 답답하지 않을까 걱정을 많이 했었는데 생활해보니까 오히려 옆자리를 신경 쓰지 않아도 되고 집중이 너무 잘 돼서 일차적으로 그게 좋았습니다. 그리고 리프레쉬 룸이나 밖에도 서서 공부하거나 답답하지 않게 공부할 수 있능 공간이 있는게 너무 좋았고 다들 집중해서 공부하는 모습을 보고 자극도 많이 받으면서 잘 공부했습니다</v>
@@ -6065,7 +6065,7 @@
         <v>일단 국어, 수학 담당 선생님들 너무 질문도 잘 받아주시고 제 사고의 능력을 향상시켜주셨고 다른 데스크 쌤들도 너무 친절하셨습니다. 가장 감사한건 담임 선생님이셨고 많은 시간을 대화하면서 어떻게 해야 더 성적을 올릴 수 있었을까를 고민했던 시간이 꽤나 즐거웠고 기억에 남는 경험이지 않았나 싶고 너무 감사합니디</v>
       </c>
       <c r="J157" t="str">
-        <v>학습 관리 시스템을 통해 제 성적과 학습 상태를 바탕으로 필요한 강의를 추천해주신 점이 큰 도움이 되었어요.</v>
+        <v>학습 관리 시스템을 통해 제 성적과 학습 상태를 바탕으로 필요한 강의를 추천해 주신 점이 큰 도움이 되었어요.</v>
       </c>
       <c r="K157" t="str">
         <v>학습 관리</v>
@@ -6120,7 +6120,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E159" t="str">
-        <v>계속 공부만 하다가는 쉽게 지칠 수 있는데 생활상담을 통해서 머리를 리프레쉬 할 수 있었고, 입시생활에서 어떤 과목을 어떻게 공부하고 얼마나 할지, 과목당 공부 시간배분 등 많은 부분에서 궁금하거나 의견을 묻고 싶을때 명확하게 답변을 해주셔서 도움이 많이 되었습니다.</v>
+        <v>계속 공부만 하다가는 쉽게 지칠 수 있는데 생활상담을 통해서 머리를 리프레쉬 할 수 있었고, 입시생활에서 어떤 과목을 어떻게 공부하고 얼마나 할지, 과목당 공부 시간배분 등 많은 부분에서 궁금하거나 의견을 묻고 싶을때 명확하게 답변을 해 주셔서 도움이 많이 되었습니다.</v>
       </c>
       <c r="F159" t="str">
         <v>원래 플래너를 적지 않았었는데, 이투스를 다니면서 학습 플래너나 학습 일기를 통해서 본인 스스로 오늘 했던 공부나 보완할 점들을 생각할 수 있었고, 어떤 과목을 앞으로 얼마큼 공부하고, 또 어떻게 공부할지에 관해서 윤곽을 쉽게 잡을 수 있었고, 전반적인 공부의 방향을 정할 수 있어서 좋았습니다.</v>
@@ -6132,7 +6132,7 @@
         <v>결국 수능에서의 실전 감각이 매우 중요하다고 생각하는데 저는 고3현역이여서 학원에서 다 같이 시험을 보지는 못하였지만 담당 선생님이 모의고사를 챙겨주셔서 주말에 모의고사를 풀 수 있었고, 이러한 실전 경험들이 쌓여서 매우 큰 성적 향상을 이뤄낼 수 있었다고 생각합니다. 또한 문제의 퀄리티 역시 매우 뛰어나고, EBS 반영까지 잘 되어 있어서 실전 연습을 하기에 적합하다고 생각합니다.</v>
       </c>
       <c r="I159" t="str">
-        <v>2월부터 다니기 시작해서 거의 9-10달을 다녔는데 고된 수험기간동안 항상 밝고 친절하게 대해주셔서 감사합니다 덕분에 힘든 수험 생활을 잘 지낼 수 있었습니다 만약 이투스를 다니지 않았더라면 성적이 이렇게 많이 오를수도 없었다고 생각합니다. 지금 대학을 다니면서 항상 바로 앞 지하철역을 지날때마다 이투스 247 독서실과 계시던 선생님들이 생각납니다! 오히러 그때가 더 좋았었던거 같기도…..  그동안 정말 감사했습니다!!</v>
+        <v>2월부터 다니기 시작해서 거의 9-10달을 다녔는데 고된 수험기간동안 항상 밝고 친절하게 대해 주셔서 감사합니다 덕분에 힘든 수험 생활을 잘 지낼 수 있었습니다 만약 이투스를 다니지 않았더라면 성적이 이렇게 많이 오를수도 없었다고 생각합니다. 지금 대학을 다니면서 항상 바로 앞 지하철역을 지날때마다 이투스 247 독서실과 계시던 선생님들이 생각납니다! 오히러 그때가 더 좋았었던거 같기도…..  그동안 정말 감사했습니다!!</v>
       </c>
       <c r="J159" t="str">
         <v>학습 상태를 꾸준히 점검해주고 안정적인 루틴을 만들어줘 공부에만 집중할 수 있었어요.</v>
@@ -6167,7 +6167,7 @@
         <v>다른 과목들에 비해서 영어 반영 비율이 적기 때문에 영어에 시간 투자를 상대적으로 덜 하게 된다. 단어 시험 덕분에 의식적으로 더 단어를 외우게 되면서 공부량이 적어졌더라도 해석을 좀 더 수월하게 할 수 있었고 한 단어장을 여러 번 반복하면서 제대로 암기할 수 있어서 큰 도움이 되었다.</v>
       </c>
       <c r="I160" t="str">
-        <v>고3생활 1년 동안 불안한 적도 많았고 고민도 되게 많았었는데 항상 상담을 통해 잘 들어주시고 좋은 해결책들도 많이 주셨어서 큰 도움을 받았습니다. 자주 돌아다녀주시면서 졸릴 때 깨워주시고 분위기도 좋게 유지해주셔서 편하게 다녔던 것 같습니다. 그리고 항상 밝게 인사해주시고 응원해주셔서 하루하루 열심히 다닐 수 있었습니다. 감사합니다!</v>
+        <v>고3생활 1년 동안 불안한 적도 많았고 고민도 되게 많았었는데 항상 상담을 통해 잘 들어주시고 좋은 해결책들도 많이 주셨어서 큰 도움을 받았습니다. 자주 돌아다녀주시면서 졸릴 때 깨워주시고 분위기도 좋게 유지해 주셔서 편하게 다녔던 것 같습니다. 그리고 항상 밝게 인사해 주시고 응원해 주셔서 하루하루 열심히 다닐 수 있었습니다. 감사합니다!</v>
       </c>
       <c r="J160" t="str">
         <v>공부 계획 짜는 법을 자세히 알려주시고, 매주 점검해 주셨어요.</v>
@@ -6193,7 +6193,7 @@
         <v>현재 내 상황에서 알맞는 강의 및 문제집을 추천해 주시는 게 굉장히 맘에 들았습니다. 솔직히 처음 공부를 시작할 때는 뭐부터 해야 할지 감을 잡기 어려웠는데 덕분에 수월하게 진도를 나간 것 같아요</v>
       </c>
       <c r="F161" t="str">
-        <v>제 MBTI가 P성향인지라 계획 세우기를 엄청 어려워 했었는데, 선생님이 플래너 작성과 계획 세우기를 코칭해주시고,적극적으로 조언을 해주셔서 체계적인 학습을 수행하는데 아주 큰 도움이 되었습니다.</v>
+        <v>제 MBTI가 P성향인지라 계획 세우기를 엄청 어려워 했었는데, 선생님이 플래너 작성과 계획 세우기를 코칭해 주시고,적극적으로 조언을 해 주셔서 체계적인 학습을 수행하는데 아주 큰 도움이 되었습니다.</v>
       </c>
       <c r="G161" t="str">
         <v>공부를 하다보면 나도 모르게 졸게 되는 경우도 많은데, 감독 선생님이 와서 깨워주시면 졸음도 가시고,리프레쉬를 할 수 있게 되어서 좋았어요. 또한 면학 분위기를 위해 지켜야 할 규칙이 명확하고,담임 선생님이 면학 분위기 조성을 위해 충고를 아끼지 않으셔서 더욱 분위기가 잘 잡힌 것 같아요.</v>
@@ -6238,7 +6238,7 @@
         <v>더프리미엄과 서바이벌 프로와 같이 매번 모의고사를 쳐야하는데 비용이 만만치가 않다. 하지만 이투스247 재원생이라면 이투스 모의고사를 달마다 한 번씩 무료로 칠수 있어 돈도 절약 할 슈 있고 퀄리티도 나쁘지 않아서 좋았다</v>
       </c>
       <c r="I162" t="str">
-        <v>한덕원 수학선생님 감사합니다. 또 저의 전반적인 생활을 관리해주시고 각종 다양한 샹활을 관리해주는 태민티처 감사합니다. 솔찍히 몇몇 선생님들은 조금 마음에 안들었지만 다들 열심히 한거라 그래도 감사합니다</v>
+        <v>한덕원 수학선생님 감사합니다. 또 저의 전반적인 생활을 관리해 주시고 각종 다양한 샹활을 관리해주는 태민티처 감사합니다. 솔찍히 몇몇 선생님들은 조금 마음에 안들었지만 다들 열심히 한거라 그래도 감사합니다</v>
       </c>
       <c r="J162" t="str">
         <v>학원에서 제공하는 멘토링 시스템이 좋았어요.</v>
@@ -6332,7 +6332,7 @@
         <v>N수생</v>
       </c>
       <c r="E165" t="str">
-        <v>3월부터 이투스247에 다니게 되었는데 수능 전까지 거의 감시가 널널했던적이 없이 졸고 있으면 바로 깨워주시고 웬만한 시간에 자주 학습실에 들어와 관리를 해주시고 상담 일정도 주기적으로 매칭을 해주어 좋았다</v>
+        <v>3월부터 이투스247에 다니게 되었는데 수능 전까지 거의 감시가 널널했던적이 없이 졸고 있으면 바로 깨워주시고 웬만한 시간에 자주 학습실에 들어와 관리를 해 주시고 상담 일정도 주기적으로 매칭을 해주어 좋았다</v>
       </c>
       <c r="F165" t="str">
         <v>모르는 문제가 있으면 이투스 어플에 들어가 바로 상담신청을 하면 조교 선생님께서 문제를 알려주어 당일에 해결을 할수 있었고 중간중간 정신적으로 힘들 때 마다 저의 조교 담당 선생님과 멘탈 관리를 받아서 힘들았던 재수 생활이였지만 버틸수 있었던거 같다</v>
@@ -6415,7 +6415,7 @@
         <v>이투스 모의고사는 실제 수능과 비슷한 난이도와 문제 유형으로 구성되어 있어 실전 감각을 기르는 데 도움이 되었다. 또한 상세한 해설과 성적 분석을 통해 내 약점을 정확히 파악하고 보완할 수 있었던 점이 가장 좋았다.</v>
       </c>
       <c r="I167" t="str">
-        <v>선생님 덕분에 힘들 때마다 다시 마음을 다잡고 끝까지 포기하지 않을 수 있었습니다. 늘 세심하게 지도해주시고 진심으로 응원해주셔서 큰 힘이 되었고, 그 덕분에 한 걸음씩 성장할 수 있었습니다. 정말 진심으로 감사드립니다.</v>
+        <v>선생님 덕분에 힘들 때마다 다시 마음을 다잡고 끝까지 포기하지 않을 수 있었습니다. 늘 세심하게 지도해 주시고 진심으로 응원해 주셔서 큰 힘이 되었고, 그 덕분에 한 걸음씩 성장할 수 있었습니다. 정말 진심으로 감사드립니다.</v>
       </c>
       <c r="J167" t="str">
         <v>이투스247학원 덕분에 성실한 학습 자세를 만들 수 있었고 그것이 성적 향상까지 이어졌던 거 같아요.</v>
@@ -6453,7 +6453,7 @@
         <v>짧은 시간동안 감사했습니다 만족하는 결과가 나오지는 못 했지만 이건 저의 부족함 때문이였던거 같습니다 분위기가 가족같아서 좋았던거 같습니드 앞으로도 번창하세요 이투스247 일산 서구점 파이팅</v>
       </c>
       <c r="J168" t="str">
-        <v>모의고사 성적관리도 꼼꼼히 해주시고 부족한 부분들을 보완해주시려고 많은 도움을 주셨어요.</v>
+        <v>모의고사 성적관리도 꼼꼼히 해 주시고 부족한 부분들을 보완해주시려고 많은 도움을 주셨어요.</v>
       </c>
       <c r="K168" t="str">
         <v>모의고사</v>
@@ -6512,13 +6512,13 @@
       <c r="E170" t="str" xml:space="preserve">
         <v xml:space="preserve">재수 학원을 다니면서 제일 좋았던 건 진짜 학습 상담이었던 것 같아요🥹_x000d_
 그냥 성적만 확인하고 끝나는 게 아니라, 제 공부 상태를 같이 진지하게 돌아봐주고 앞으로 어떻게 해야 할지 방향을 잡아주셔서 너무 든든했어요. 혼자 공부할 때는 ‘이게 맞나…?’ 싶을 때가 진짜 많았는데, 상담을 받으면서 “아 내가 잘 가고 있구나” 하는 확신이 생겨서 마음이 훨씬 편해졌습니다✨_x000d_
-특히 좋았던 건 과목별로 부족한 부분을 엄청 구체적으로 짚어주신 거였어요. 그냥 “더 열심히 해라” 이런 게 아니라, 문제를 어떻게 풀어야 하는지, 개념을 어떤 식으로 다시 정리해야 하는지까지 알려주셔서 바로 공부에 적용할 수 있었습니다! 그래서 전보다 훨씬 효율적으로 공부할 수 있었던 것 같아요📚 그리고 상담이 한 번으로 끝나는 게 아니라, 이전에 세운 계획을 계속 체크해 주시고 피드백을 주신 것도 진짜 도움이 많이 됐어요. 잘했을 때는 칭찬해주시고, 부족한 부분은 다시 방향 잡아주셔서 자연스럽게 꾸준히 공부하는 습관도 생겼습니다. 이 과정에서 스스로를 관리하는 힘도 많이 길러졌다고 느꼈어요💪 학원 분위기도 진짜 좋았습니다. 전체적으로 조용하고 집중 잘 되는 환경이라 공부에 몰입하기 너무 좋았고, 주변 친구들도 다 열심히 하는 분위기라 저도 자연스럽게 더 열심히 하게 되더라고요🔥 약간 긴장감 있으면서도 서로 자극되는 느낌…? 그래서 힘들 때도 쉽게 포기하지 않게 잡아주는 분위기였습니다. 선생님들도 단순히 관리만 하는 게 아니라 진짜 학생들 잘되길 바라는 게 느껴져서 더 믿고 따라갈 수 있었던 것 같아요🥺 그래서 학원이 그냥 공부만 하는 곳이 아니라, 같이 성장하는 공간처럼 느껴졌습니다.</v>
+특히 좋았던 건 과목별로 부족한 부분을 엄청 구체적으로 짚어주신 거였어요. 그냥 “더 열심히 해라” 이런 게 아니라, 문제를 어떻게 풀어야 하는지, 개념을 어떤 식으로 다시 정리해야 하는지까지 알려주셔서 바로 공부에 적용할 수 있었습니다! 그래서 전보다 훨씬 효율적으로 공부할 수 있었던 것 같아요📚 그리고 상담이 한 번으로 끝나는 게 아니라, 이전에 세운 계획을 계속 체크해 주시고 피드백을 주신 것도 진짜 도움이 많이 됐어요. 잘했을 때는 칭찬해 주시고, 부족한 부분은 다시 방향 잡아주셔서 자연스럽게 꾸준히 공부하는 습관도 생겼습니다. 이 과정에서 스스로를 관리하는 힘도 많이 길러졌다고 느꼈어요💪 학원 분위기도 진짜 좋았습니다. 전체적으로 조용하고 집중 잘 되는 환경이라 공부에 몰입하기 너무 좋았고, 주변 친구들도 다 열심히 하는 분위기라 저도 자연스럽게 더 열심히 하게 되더라고요🔥 약간 긴장감 있으면서도 서로 자극되는 느낌…? 그래서 힘들 때도 쉽게 포기하지 않게 잡아주는 분위기였습니다. 선생님들도 단순히 관리만 하는 게 아니라 진짜 학생들 잘되길 바라는 게 느껴져서 더 믿고 따라갈 수 있었던 것 같아요🥺 그래서 학원이 그냥 공부만 하는 곳이 아니라, 같이 성장하는 공간처럼 느껴졌습니다.</v>
       </c>
       <c r="F170" t="str" xml:space="preserve">
         <v xml:space="preserve">학습 관리 시스템 중에서 가장 유용하다고 느꼈던 점은 1대1 맞춤 강의 추천이었습니다😊_x000d_
-이투스에는 다양한 강의가 있어서 선택의 폭이 넓다는 장점이 있지만, 그만큼 어떤 강의를 들어야 할지 스스로 판단하기가 쉽지 않았습니다. 이런 상황에서 학습 관리 시스템을 통해 제 성적과 학습 상태를 바탕으로 필요한 강의를 추천해주신 점이 큰 도움이 되었습니다._x000d_
+이투스에는 다양한 강의가 있어서 선택의 폭이 넓다는 장점이 있지만, 그만큼 어떤 강의를 들어야 할지 스스로 판단하기가 쉽지 않았습니다. 이런 상황에서 학습 관리 시스템을 통해 제 성적과 학습 상태를 바탕으로 필요한 강의를 추천해 주신 점이 큰 도움이 되었습니다._x000d_
 _x000d_
-특히 단순히 인기 있는 강의를 추천하는 것이 아니라, 제 약점이나 부족한 개념을 보완할 수 있는 강의를 중심으로 안내해주셔서 더욱 효율적으로 공부할 수 있었습니다. 덕분에 불필요하게 여러 강의를 듣기보다는 꼭 필요한 강의에 집중할 수 있었고, 시간 관리 측면에서도 큰 도움이 되었습니다⏰_x000d_
+특히 단순히 인기 있는 강의를 추천하는 것이 아니라, 제 약점이나 부족한 개념을 보완할 수 있는 강의를 중심으로 안내해 주셔서 더욱 효율적으로 공부할 수 있었습니다. 덕분에 불필요하게 여러 강의를 듣기보다는 꼭 필요한 강의에 집중할 수 있었고, 시간 관리 측면에서도 큰 도움이 되었습니다⏰_x000d_
 _x000d_
 또한 1대1로 맞춰진 추천이다 보니, 현재 제 수준에 맞는 난이도의 강의를 선택할 수 있었고, 그 과정에서 학습에 대한 부담도 줄어들었습니다. 스스로 강의를 찾느라 고민하는 시간이 줄어들고, 바로 학습에 집중할 수 있었다는 점에서 학습 흐름을 유지하는 데에도 긍정적인 영향을 주었습니다📚 공부의 방향을 명확하게 잡아주고 효율성을 높여주는 중요한 역할을 했다고 생각합니다✨</v>
       </c>
@@ -6526,7 +6526,7 @@
         <v xml:space="preserve">학습 관리 시스템 중에서도 출석 관리와 생활 관리 부분이 특히 유용하다고 느꼈습니다😊_x000d_
 매일 출석 날짜를 체계적으로 관리해 주셔서 스스로 흐트러지지 않고 꾸준히 학원에 나올 수 있었고, 자연스럽게 규칙적인 생활 습관을 유지하는 데 큰 도움이 되었습니다. 혼자였다면 쉽게 느슨해질 수 있었을 텐데, 이러한 관리 덕분에 끝까지 긴장감을 유지할 수 있었습니다._x000d_
 _x000d_
-또한 선생님들께서 학원을 직접 돌아다니시면서 학생들의 학습 상태를 확인해주신 점도 인상 깊었습니다. 공부하다가 졸거나 집중력이 떨어질 때 바로잡아주셔서 다시 흐름을 이어갈 수 있었고, 그 덕분에 공부 시간의 밀도가 훨씬 높아졌다고 느꼈습니다💪_x000d_
+또한 선생님들께서 학원을 직접 돌아다니시면서 학생들의 학습 상태를 확인해 주신 점도 인상 깊었습니다. 공부하다가 졸거나 집중력이 떨어질 때 바로잡아주셔서 다시 흐름을 이어갈 수 있었고, 그 덕분에 공부 시간의 밀도가 훨씬 높아졌다고 느꼈습니다💪_x000d_
 _x000d_
 이러한 세심한 관리 덕분에 단순히 자리에 앉아 있는 것이 아니라, 실제로 집중해서 공부하는 시간을 늘릴 수 있었고, 스스로를 통제하는 힘도 함께 기를 수 있었습니다. 결과적으로 학습 습관을 잡고 꾸준함을 유지하는 데 큰 도움이 된 시스템이었다고 생각합니다✨</v>
       </c>
@@ -6541,11 +6541,11 @@
 이처럼 이투스 전국모의고사는 실전 대비뿐만 아니라, 자신의 위치를 점검하고 학습 방향을 잡는 데에도 큰 도움을 준 유용한 시스템이었다고 생각합니다✨</v>
       </c>
       <c r="I170" t="str" xml:space="preserve">
-        <v xml:space="preserve">재수 기간 동안 옆에서 함께해주신 조교 선생님들과 원장 선생님께 진심으로 감사의 마음을 전하고 싶습니다_x000d_
+        <v xml:space="preserve">재수 기간 동안 옆에서 함께해 주신 조교 선생님들과 원장 선생님께 진심으로 감사의 마음을 전하고 싶습니다_x000d_
 _x000d_
 조교 선생님들께서는 항상 가까이에서 학생들을 세심하게 살펴봐 주시고, 작은 부분까지 신경 써주셔서 학원 생활을 더욱 안정적으로 이어갈 수 있었습니다. 공부하다가 지치거나 힘들 때마다 따뜻하게 말 한마디 건네주시고, 필요한 부분을 바로 도와주셔서 큰 힘이 되었습니다. 그 덕분에 끝까지 포기하지 않고 버틸 수 있었다고 생각합니다🥹_x000d_
 _x000d_
-또한 원장 선생님께서도 학생 한 명 한 명을 진심으로 생각해주시고, 학원의 전체적인 방향과 분위기를 잘 이끌어주셔서 더욱 믿고 따라갈 수 있었습니다. 항상 학생들의 입장에서 고민해주시고 응원해주신 덕분에, 학원이 단순한 공부 공간이 아니라 의지할 수 있는 곳처럼 느껴졌습니다._x000d_
+또한 원장 선생님께서도 학생 한 명 한 명을 진심으로 생각해 주시고, 학원의 전체적인 방향과 분위기를 잘 이끌어주셔서 더욱 믿고 따라갈 수 있었습니다. 항상 학생들의 입장에서 고민해 주시고 응원해 주신 덕분에, 학원이 단순한 공부 공간이 아니라 의지할 수 있는 곳처럼 느껴졌습니다._x000d_
 _x000d_
 이렇게 많은 도움과 응원을 받으면서 공부할 수 있었던 시간은 저에게 정말 소중한 경험이었습니다. 앞으로도 이곳에서 배운 태도와 마음가짐을 잊지 않고 더 성장해 나가겠습니다. 진심으로 감사드립니다💛</v>
       </c>
@@ -6582,7 +6582,7 @@
         <v>이투스에는 훌륭한 인강 강사분들이 계시지만 이투스는 다른 앱과 다르게 구독을 갱신해야한다는 불편함이 있었지만 이투스247독학재수 학원을 다니면서 무료로 이투스 인강을 볼 수 있어서 정말 좋았고 구독갱신을 안해도 되어서 너무 편했습니다</v>
       </c>
       <c r="I171" t="str">
-        <v>원장님이랑 실장님이랑 경쌤! 25년 한 해 동안 정말 신세 많이 졌습니다 대학가서 재밋게 지내고 있어요! 곧 인사 차 방문드릴게요 ㅎㅎ 제 학습 방향 설정해주셔서 감사했고 멘탈도 케어해주셔서 정말 감사했습니다!</v>
+        <v>원장님이랑 실장님이랑 경쌤! 25년 한 해 동안 정말 신세 많이 졌습니다 대학가서 재밋게 지내고 있어요! 곧 인사 차 방문드릴게요 ㅎㅎ 제 학습 방향 설정해 주셔서 감사했고 멘탈도 케어해 주셔서 정말 감사했습니다!</v>
       </c>
       <c r="J171" t="str">
         <v>확실히 휴대폰이 없으니 공부에 집중이 더 잘 되고 성취감도 있어서 생활 관리에 유용했어요.</v>
@@ -6617,10 +6617,10 @@
         <v>사실 단어가 혼자 외우려면 일정한 양을 매일 꾸준하게 외우고 그것을 확인하는게 쉽지 않은데 학원에서 단어 테스트를 보니까 억지로라도 외우게 되고 그게 쌓이다 보니 재수 후반에 영어를 공부할 때 단어에 대한 문제는 딱히 없었던 것 같아서 단어 테스트는 영어 성적에 있어서 많은 도움이 된 것 같습니다.</v>
       </c>
       <c r="I172" t="str">
-        <v>약 1년 동안 많은 학생들을 케어하기 힘드셨을텐데 그럼에도 항상 질문에 대해 친절하게 답변해주시고 성적이 잘 나오지 않아 답답해서 힘들어 할 때도 격려해주셔서 끝까지 포기하지 않고 꾸준히 1년을 달릴 수 있었던 것 같아서 감사합니다.</v>
+        <v>약 1년 동안 많은 학생들을 케어하기 힘드셨을텐데 그럼에도 항상 질문에 대해 친절하게 답변해 주시고 성적이 잘 나오지 않아 답답해서 힘들어 할 때도 격려해 주셔서 끝까지 포기하지 않고 꾸준히 1년을 달릴 수 있었던 것 같아서 감사합니다.</v>
       </c>
       <c r="J172" t="str">
-        <v>수시 원서를 쓰기 전에 한 명씩 친절하게 상담을 해주셨어요.</v>
+        <v>수시 원서를 쓰기 전에 한 명씩 친절하게 상담을 해 주셨어요.</v>
       </c>
       <c r="K172" t="str">
         <v/>
@@ -6640,7 +6640,7 @@
         <v>N수생</v>
       </c>
       <c r="E173" t="str">
-        <v>여러 사설 모의고사와 평가원 모의고사 등을 보았을 때 나의 수준이 어느정도인지, 취약한 과목이 무엇인지 등을 분석해주시고 어떤식으로 공부방향을 잡아야 할지를 알려주셨던게 매우 유용하였다</v>
+        <v>여러 사설 모의고사와 평가원 모의고사 등을 보았을 때 나의 수준이 어느정도인지, 취약한 과목이 무엇인지 등을 분석해 주시고 어떤식으로 공부방향을 잡아야 할지를 알려주셨던게 매우 유용하였다</v>
       </c>
       <c r="F173" t="str">
         <v>중간중간에 무엇을 해야 할지 몰라 막막했던 상황이 꽤 있었는데 무엇을 하면 좋을지 명확하게 알려주셔서 낭비하는 시간 없이 재수하는 1년을 꽉꽉 채워 보낼 수 있었던 것 같아 유용했다.</v>
@@ -6652,7 +6652,7 @@
         <v>안그래도 영어가 가장 취약하고 싫어하는 과목이었어서 영어 공부를 항상 소홀히 하였었는데 매일 아침마다 보는 단어테스트 덕분에 영어 공부에 조금이라도 시간을 더 쓰게 되어 유용하였던 것 같다.</v>
       </c>
       <c r="I173" t="str">
-        <v>선생님들께서 항상 한결같이 친절하게 대해주시고 올바르게 지도해주셔서 작년보다 좋은 결과 낼 수 있었던 것 같아요. 모두 선생님들 덕분입니다. 정말 감사드리고 이투스 선생님들 항상 파이팅입니다!!</v>
+        <v>선생님들께서 항상 한결같이 친절하게 대해 주시고 올바르게 지도해 주셔서 작년보다 좋은 결과 낼 수 있었던 것 같아요. 모두 선생님들 덕분입니다. 정말 감사드리고 이투스 선생님들 항상 파이팅입니다!!</v>
       </c>
       <c r="J173" t="str">
         <v>이투스247학원의 스마트 관리는 학습뿐 아니라 생활 전반을 관리해준다는 점에서 매우 유용했어요.</v>
@@ -6682,7 +6682,7 @@
 또  담임과 통화하면서  학생에게  동기부여 함으로  자극을 주며, 또한 남녀가 확실히 분리되어  또한  관리도  철저하게 관리되는것을  학생으로 충분히  설명받음</v>
       </c>
       <c r="G174" t="str" xml:space="preserve">
-        <v xml:space="preserve">야간 취침시간  관리며  아침 점심  다  통제시간도 철저했으며  식사 외  간식 제안  라면등   특식으로  제공되겠음 해주셔서  보기좋았습니다._x000d_
+        <v xml:space="preserve">야간 취침시간  관리며  아침 점심  다  통제시간도 철저했으며  식사 외  간식 제안  라면등   특식으로  제공되겠음 해 주셔서  보기좋았습니다._x000d_
 아이들이  좋아하는것만 해줄 수 있는데  적당히 잘 통제되어서  만족했습니다</v>
       </c>
       <c r="H174" t="str" xml:space="preserve">
@@ -6716,7 +6716,7 @@
         <v>N수생</v>
       </c>
       <c r="E175" t="str">
-        <v>매주 정해진 선생님과 학업상담뿐만 아니라 내가 지금 어떤 상황에 처해있고 어떤것 때문에 스트레스를 받는지 상담을 할수 있어 좋았다 예를 들면 학업상담에선 내가 부족한 부분을 찾아주시고 그거에 맞는 책 추천을 통해 발전할수있게 해주셔서 수능에선 그 부분은 안 틀리고 넘어갈수있었다 일상생활에서 받는 스트레스도 같이 공감해주시고 조언을 해주셔서 정신적으로도 도움이 많이 되었다</v>
+        <v>매주 정해진 선생님과 학업상담뿐만 아니라 내가 지금 어떤 상황에 처해있고 어떤것 때문에 스트레스를 받는지 상담을 할수 있어 좋았다 예를 들면 학업상담에선 내가 부족한 부분을 찾아주시고 그거에 맞는 책 추천을 통해 발전할수있게 해 주셔서 수능에선 그 부분은 안 틀리고 넘어갈수있었다 일상생활에서 받는 스트레스도 같이 공감해 주시고 조언을 해 주셔서 정신적으로도 도움이 많이 되었다</v>
       </c>
       <c r="F175" t="str" xml:space="preserve">
         <v xml:space="preserve">수강 관리를 같이 하니까 공부를 미루지 않게 되는 점이 제일 좋았다.현역때는 항상 미루게 되고 누가 검사를 안하니까 안하게 되었는데 여기서는 다 관리를 해주시니까 미루지않고 그때그때 다 하게된거같아 좋았다 그리고 _x000d_
@@ -6753,7 +6753,7 @@
         <v>N수생</v>
       </c>
       <c r="E176" t="str">
-        <v>공부했던 것을 써서 매일 선생님께 제출했다.  선생님께서 매일 나의 학습시간과 과목별 공부량을 확인 하시며 좀 더 공부량을 늘려야하는 과목을 알려주시고 진도가 계속 나가고 있는지 점검해주셔서 느슨해지지 않고 열심히 진도를 나갈 수 있었다.</v>
+        <v>공부했던 것을 써서 매일 선생님께 제출했다.  선생님께서 매일 나의 학습시간과 과목별 공부량을 확인 하시며 좀 더 공부량을 늘려야하는 과목을 알려주시고 진도가 계속 나가고 있는지 점검해 주셔서 느슨해지지 않고 열심히 진도를 나갈 수 있었다.</v>
       </c>
       <c r="F176" t="str">
         <v>해당 과목을 전공하신 선생님께서 각각 계셔서 더 질적인 답변을 받을 수 있었고 질문이 들때마다 바로바로 답을 받을 수 있고 선생님께서도 정말 친절하게 답변을 해주셨어서 1:1 질의응답 서비스가 정말 유용했던 것 같다.</v>
@@ -6765,10 +6765,10 @@
         <v>모의고사를 많이 볼 기회가 없었는데 이투스 모의고사가 있어서 양질의 실전 연습을 중간중간마다 할 수 있어서 실전 감각을 기르고 내 위치를 점검하고 약점을 발견하며 크게 실력이 늘을 수 있게 된 것 같다.</v>
       </c>
       <c r="I176" t="str">
-        <v>선생님께서 질문도 받아주시고 마주칠 때마다 좋은 말씀 많이 해주시고 밥 먹을 때마다 맛있게 먹으라고 따뜻하게 말해주시고 등원, 하원 할 때마다 따뜻하게 인사로 맞이해주셔서 힘든 수험 생활에 큰 힘이 되었던 것 같습니다. 정말 감사드립니다!</v>
+        <v>선생님께서 질문도 받아주시고 마주칠 때마다 좋은 말씀 많이 해 주시고 밥 먹을 때마다 맛있게 먹으라고 따뜻하게 말해 주시고 등원, 하원 할 때마다 따뜻하게 인사로 맞이해 주셔서 힘든 수험 생활에 큰 힘이 되었던 것 같습니다. 정말 감사드립니다!</v>
       </c>
       <c r="J176" t="str">
-        <v>면학 분위기에 대한 관리도 세심하게 해주셔서 집중해서 공부할 수 있었어요.</v>
+        <v>면학 분위기에 대한 관리도 세심하게 해 주셔서 집중해서 공부할 수 있었어요.</v>
       </c>
       <c r="K176" t="str">
         <v>면학 분위기</v>
@@ -6823,7 +6823,7 @@
         <v>N수생</v>
       </c>
       <c r="E178" t="str">
-        <v>이투스247 학원에 다니면서 가장 좋았던 점은 엘리트 선생님들이 직접 멘토 역할을 해주시며 세심하게 지도해주신다는 것이었습니다. 단순히 수업만 하는 것이 아니라 성적 관리부터 학습 계획까지 함께 고민해주시고 방향을 잡아주셔서 공부에 대한 부담이 훨씬 줄었습니다. 또한 지각 관리 시스템도 체계적으로 운영되어 스스로 생활 습관을 잡는 데 큰 도움이 되었고, 전반적으로 학습 분위기가 잘 형성되어 있어 꾸준히 집중할 수 있었습니다.</v>
+        <v>이투스247 학원에 다니면서 가장 좋았던 점은 엘리트 선생님들이 직접 멘토 역할을 해주시며 세심하게 지도해 주신다는 것이었습니다. 단순히 수업만 하는 것이 아니라 성적 관리부터 학습 계획까지 함께 고민해 주시고 방향을 잡아주셔서 공부에 대한 부담이 훨씬 줄었습니다. 또한 지각 관리 시스템도 체계적으로 운영되어 스스로 생활 습관을 잡는 데 큰 도움이 되었고, 전반적으로 학습 분위기가 잘 형성되어 있어 꾸준히 집중할 수 있었습니다.</v>
       </c>
       <c r="F178" t="str">
         <v>학습 관리시스템이 매우 체계적으로 운영되어 공부의 흐름을 꾸준히 유지하는 데 큰 도움이 되었습니다. 출결과 지각 관리가 엄격하게 이루어져 자연스럽게 생활 습관이 잡혔고, 개인별 학습 계획과 성적까지 꼼꼼하게 관리해주어 스스로 부족한 부분을 정확히 파악하고 보완할 수 있었습니다. 덕분에 학습 방향을 잃지 않고 꾸준히 목표를 향해 나아갈 수 있었습니다.</v>
@@ -6838,7 +6838,7 @@
         <v>이투스247 선생님들께 진심으로 감사드립니다. 항상 학생 한 명 한 명에게 관심을 가지고 세심하게 지도해주시며, 학습뿐만 아니라 생활 전반까지 챙겨주셔서 큰 힘이 되었습니다. 덕분에 흔들리지 않고 꾸준히 공부할 수 있었고, 힘들 때마다 따뜻한 조언으로 방향을 잡아주셔서 끝까지 포기하지 않을 수 있었습니다. 정말 감사드립니다.</v>
       </c>
       <c r="J178" t="str">
-        <v>항상 학습 진행 상황을 체크해 주시고 상담도 자주 해주셔서 좋았어요.</v>
+        <v>항상 학습 진행 상황을 체크해 주시고 상담도 자주 해 주셔서 좋았어요.</v>
       </c>
       <c r="K178" t="str">
         <v/>
@@ -6932,7 +6932,7 @@
         <v>N수생</v>
       </c>
       <c r="E181" t="str">
-        <v>대학생 코칭선생님과 일주일에 한 번씩 만나서 현재 진도를 체크하고, 다음 상담까지의 진도 등을 자세히 얘기나눴어요. 상담 외에도 공부하다가 질문할 점이 있으면 과목별로 본인 이름을 쓰고 질문 드릴 수 있었던 게 좋았어요. 수능이 얼마 남지 않았을 때 자신 있는 영어가 80점대 후반이 나와서 불안해져서 상담했을 때도 잘 볼 거라고 확신을 주시고, 독서 읽는 법을 몇 번이나 반복해서 여쭤봤는데 친절히 대답해주신 제 코칭선생님께 감사드립니다 ㅎㅎ</v>
+        <v>대학생 코칭선생님과 일주일에 한 번씩 만나서 현재 진도를 체크하고, 다음 상담까지의 진도 등을 자세히 얘기나눴어요. 상담 외에도 공부하다가 질문할 점이 있으면 과목별로 본인 이름을 쓰고 질문 드릴 수 있었던 게 좋았어요. 수능이 얼마 남지 않았을 때 자신 있는 영어가 80점대 후반이 나와서 불안해져서 상담했을 때도 잘 볼 거라고 확신을 주시고, 독서 읽는 법을 몇 번이나 반복해서 여쭤봤는데 친절히 대답해 주신 제 코칭선생님께 감사드립니다 ㅎㅎ</v>
       </c>
       <c r="F181" t="str">
         <v>앞서 작성한 것처럼 매주 진도를 체크받고 다음에는 어디까지 학습할지 관리를 받았는데, 계획적이지 못하고 설령 계획을 세워도 중도포기하기 일쑤인 저에게 누군가 이끌어주는 것이 큰 도움이 되었습니다. 공부 플래너를 그렇게 연속해서 오랫동안 작성하고 실제로 지킨 게 그때가 처음이었어요.</v>
@@ -6944,7 +6944,7 @@
         <v>수능이 다가올수록 모의고사의 필요성을 점점 더 크게 느껴 주기적으로 이투스 모의고사를 비롯한 사설 모의고사를 신청해 풀곤 했다. 영어 시간에는 듣기평가를 할 때 스피커의 음량이 크게 나와서 좋았고, 수학은 여느 사설 모의고사처럼 상위권 대상이 아니라 실제 수능과 비슷한 난이도로 나와서 좋았다. 또 이투스 구독도 도움이 되었는데, 이투스학원에 다니면 이투스 구독권을 무료로 제공해준다. 그래서 정승제와 김민정, 주혜연 같은 강사의 강의를 저렴한 가격에 들을 수 있어 도움이 되었다. 다만 내가 원래보다 며칠 빨리 퇴원했는데 그때 구독권을 딱 끊어버려서 그건 조금 아쉬움이 남았다.</v>
       </c>
       <c r="I181" t="str">
-        <v>이른 아침부터 데스크에서 학생들을 맞아주시던 인자하신 어르신 직원분과 다른 직원분들 너무 감사합니다 ㅎㅎ 덕분에 여름에는 시원하고 겨울에는 따뜻한 환경에서 공부할 수 있었어요. 쾌적한 공부환경을 제공해 공부 외에는 신경쓰지 않아도 되게 해주셔서 감사했습니다. 그리고 대학생 코칭선생님에게도 학습 관련한 도움도 많이 받았고, 대학생같은 옷을 입고 다니시는 걸 보며 나도 올해 꼭 합격해서 대학 다녀야지 라고 결심하는 계기가 되었어요 ㅎㅎ 매일 맛있는 급식 제공해주신 급식업체 직원분들께도 감사드려요!</v>
+        <v>이른 아침부터 데스크에서 학생들을 맞아주시던 인자하신 어르신 직원분과 다른 직원분들 너무 감사합니다 ㅎㅎ 덕분에 여름에는 시원하고 겨울에는 따뜻한 환경에서 공부할 수 있었어요. 쾌적한 공부환경을 제공해 공부 외에는 신경쓰지 않아도 되게 해 주셔서 감사했습니다. 그리고 대학생 코칭선생님에게도 학습 관련한 도움도 많이 받았고, 대학생같은 옷을 입고 다니시는 걸 보며 나도 올해 꼭 합격해서 대학 다녀야지 라고 결심하는 계기가 되었어요 ㅎㅎ 매일 맛있는 급식 제공해 주신 급식업체 직원분들께도 감사드려요!</v>
       </c>
       <c r="J181" t="str">
         <v>이투스247학원의 학습 관리는 진짜 체계적이라 놀라웠었어요.</v>
@@ -6979,7 +6979,7 @@
         <v>혼자서 단어를 외우면 하기 싫은 날도 있고 작심삼일이 되었을 수도 있는데 매일 일정한 양을 외우고 시험 보는 게 좋았고 잘 외우지 못했을 땐 재시험을 보며 제대로 학습할 수 있어 유용했습니다</v>
       </c>
       <c r="I182" t="str">
-        <v>이투스247에서 함께해주신 선생님들께 진심으로 감사드립니다. 항상 따뜻하게 응원해주시고, 함께 방향을 잡아주셔서 끝까지 포기하지 않을 수 있었습니다. 세심한 상담과 진심 어린 조언 덕분에 한층 더 성장할 수 있었고, 그 과정이 큰 힘이 되었습니다. 1년 동안 학습에 집중할 수 있도록 힘써주셔서 감사합니다.</v>
+        <v>이투스247에서 함께해 주신 선생님들께 진심으로 감사드립니다. 항상 따뜻하게 응원해 주시고, 함께 방향을 잡아주셔서 끝까지 포기하지 않을 수 있었습니다. 세심한 상담과 진심 어린 조언 덕분에 한층 더 성장할 수 있었고, 그 과정이 큰 힘이 되었습니다. 1년 동안 학습에 집중할 수 있도록 힘써주셔서 감사합니다.</v>
       </c>
       <c r="J182" t="str">
         <v>공부에 집중할 수 있는 환경을 만드는 데 큰 도움이 되었어요.</v>
@@ -7002,7 +7002,7 @@
         <v>N수생</v>
       </c>
       <c r="E183" t="str">
-        <v>수시 접수와 정시 접수 모두 상담을 해주셨는데, 수시 접수 때는 생기부까지 봐주시며 코칭해주셔서 원서 접수에 큰 도움이 되었습니다. 또한 정시 접수 때는 진학사을 이용하여 경쟁력을 파악하고, 대안을 여러가지 만들어 만약을 대비할 수 있었습니다. 1차 상담에서 끝나지 않고 3차 대면 상담까지 지속적으로 이어졌으며, 접수 팁까지 알려주셔서 이 부분에서 큰 도움을 얻었습니다.</v>
+        <v>수시 접수와 정시 접수 모두 상담을 해주셨는데, 수시 접수 때는 생기부까지 봐주시며 코칭해 주셔서 원서 접수에 큰 도움이 되었습니다. 또한 정시 접수 때는 진학사을 이용하여 경쟁력을 파악하고, 대안을 여러가지 만들어 만약을 대비할 수 있었습니다. 1차 상담에서 끝나지 않고 3차 대면 상담까지 지속적으로 이어졌으며, 접수 팁까지 알려주셔서 이 부분에서 큰 도움을 얻었습니다.</v>
       </c>
       <c r="F183" t="str">
         <v>스스로 강의를 보고 교재를 풀면서 공부해야 하는 시스템이기 때문에 강의에서 해결하기 어려운 개념이나 문제가 생겼을 때, 각 학원에 상주하고 계신 담당 과목 선생님께 그때마다 여쭤볼 수 있어서 공부하는데 큰 도움이 되었습니다.</v>
@@ -7014,7 +7014,7 @@
         <v>평가원 모의고사와 조금 다르긴 하지만 이투스 모의고사가 거의 매달 치뤄졌기 때문에 시간 관리와 개념 및 문제 풀이에 큰 도움을 받았습니다. 특히 3월, 6월 모의고사 같은 중요한 시험을 보는데 있어서 감을 유지하는데도 이점이 있었습니다. 또한 시험 이후 진행하는 오답노트를 통해 나의 부족한 점을 채울 수 있다는 점도 효율적인 학습을 진행하는데 도움이 되었습니다.</v>
       </c>
       <c r="I183" t="str">
-        <v>항상 등원하고 하원할 때 따뜻한 인사 한마디씩 건네주셔서 큰 힘이 되었습니다. 특히 가끔 학원 내부에서 마주쳤을 때 소소한 이야기를 건네주실 때마다 학생들에게 관심을 가지고 대해주신다는 느낌이 들었고, 반복되는 일상도 덜 지루하게 느끼며 생활할 수 있었습니다! 또 마지막 교시에 종이 울릴 때, 수험생 입장에서 위로가 되거나 힘이 되는 음악을 선생님들께서 직접 골라서 틀어주시는 점도 작지만 큰 위안이 되었던 것 같습니다!! 항상 감사했습니다.</v>
+        <v>항상 등원하고 하원할 때 따뜻한 인사 한마디씩 건네주셔서 큰 힘이 되었습니다. 특히 가끔 학원 내부에서 마주쳤을 때 소소한 이야기를 건네주실 때마다 학생들에게 관심을 가지고 대해 주신다는 느낌이 들었고, 반복되는 일상도 덜 지루하게 느끼며 생활할 수 있었습니다! 또 마지막 교시에 종이 울릴 때, 수험생 입장에서 위로가 되거나 힘이 되는 음악을 선생님들께서 직접 골라서 틀어주시는 점도 작지만 큰 위안이 되었던 것 같습니다!! 항상 감사했습니다.</v>
       </c>
       <c r="J183" t="str">
         <v>상담을 통해 지난 성적과 비교해가며 전략을 짜는 것이 가장 좋았어요.</v>
@@ -7037,7 +7037,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E184" t="str">
-        <v>자기주도학습이 부족한 저에게 꼼꼼한 피드백을 해주시고 공부 시간도 짜주셨습니다 코칭으로 몰랐던 부분을 채워가며 더 나은 학습환경이 만들어졌습니다 모르는 부분을 친절하게 답해주는 것도 좋았습니다</v>
+        <v>자기주도학습이 부족한 저에게 꼼꼼한 피드백을 해 주시고 공부 시간도 짜주셨습니다 코칭으로 몰랐던 부분을 채워가며 더 나은 학습환경이 만들어졌습니다 모르는 부분을 친절하게 답해주는 것도 좋았습니다</v>
       </c>
       <c r="F184" t="str">
         <v>나에게 맞는 학습전략을 세워주며 더 효율적으로 공부할 수 있는 방법을 제공해주셨습니다 또 언제든 상담을 받을 수 있어 고민이 생기면 물어볼 수 있어서 좋았습니다 항상 친절하게 답변해주셨습니다</v>
@@ -7049,7 +7049,7 @@
         <v>인강사이트를 무료로 사용할 수 있는것이 좋았고 이투스 모의고사도 칠 수 있어서 좋았습니다 사설이라 어렵긴 해도 내 위치가 어느정도인지 파악할 수 있어서 좋았습니다 또 이투스구독으로 다양한 수업을 들을 수 있는것도 좋았습니다</v>
       </c>
       <c r="I184" t="str">
-        <v>항상 밝은 미소로 데스크에서 인사해주신 대표님이랑 실장님도 감사합니다 또 항상 제 고민을 들어주신 국어썀도 감사하고 수포자인 저를 가르쳐주신 수학쌤도 감사합니다 또 영어쌤도 항상 저를 반겨주셔서 감사합니다</v>
+        <v>항상 밝은 미소로 데스크에서 인사해 주신 대표님이랑 실장님도 감사합니다 또 항상 제 고민을 들어주신 국어썀도 감사하고 수포자인 저를 가르쳐주신 수학쌤도 감사합니다 또 영어쌤도 항상 저를 반겨주셔서 감사합니다</v>
       </c>
       <c r="J184" t="str">
         <v>지속적인 피드백을 통해 부족한 부분을 보완할 수 있어 성적 향상에 긍정적인 영향을 주었어요.</v>
@@ -7072,14 +7072,14 @@
         <v>반수생</v>
       </c>
       <c r="E185" t="str">
-        <v>이투스 학원에서 제공하는 멘토링 시스템이 좋았습니다. 모르는 문제가 있거나 어떻게 공부해야 할지 모를때 멘토 분들이 하나하나 알려주시고 모르는 문제에 대한 해답이 바로 납득가기 쉽게 설명해주셔서 이부분이 가장 좋았던 것 같습니다</v>
+        <v>이투스 학원에서 제공하는 멘토링 시스템이 좋았습니다. 모르는 문제가 있거나 어떻게 공부해야 할지 모를때 멘토 분들이 하나하나 알려주시고 모르는 문제에 대한 해답이 바로 납득가기 쉽게 설명해 주셔서 이부분이 가장 좋았던 것 같습니다</v>
       </c>
       <c r="F185" t="str" xml:space="preserve">
         <v xml:space="preserve">1:1질의응답에서 몰랐던 부분의 개념이나 활용방법 등등 알지 못했던 부분을 채워주셔서 더욱 더 배움에 있어 단단해 졌던 것 같습니다. 그리고 앞으로 공부를 어떻게 해야 할지도 알려주셔서 맘편하게_x000d_
 다녔던 것 같습니다</v>
       </c>
       <c r="G185" t="str">
-        <v>학생들이 화장실에서 떠들거나 휴개실에사 떠들면 지도를 해주시고 졸거나 하면 깨워주셔서 수능시간 때 졸거나 피곤하지 않게 잘 관리해주신 것 같아 좋았습니다. 또 마음에 들지 않는 점이 있다면 잘 들어주셨습니다</v>
+        <v>학생들이 화장실에서 떠들거나 휴개실에사 떠들면 지도를 해 주시고 졸거나 하면 깨워주셔서 수능시간 때 졸거나 피곤하지 않게 잘 관리해 주신 것 같아 좋았습니다. 또 마음에 들지 않는 점이 있다면 잘 들어주셨습니다</v>
       </c>
       <c r="H185" t="str">
         <v>이투스 전국모의고사를 지원해줘서 한달에 한 번씩 감을 찾을 수 있었고 어느 부분이 부족한지 지표로 나오고 내가 지금 이 성적으로 어디를 갈 수 있는지 알 수 있어서 공부 의욕을 향상하는데 좋았던 것 같고</v>
@@ -7120,7 +7120,7 @@
         <v>단어 테스트는 영어 학습의 기초를 다지는 데 매우 유용했다. 정기적으로 단어를 점검하면서 암기한 내용을 확인할 수 있었고, 부족한 어휘를 반복 학습하는 데 도움이 되었다. 또한 꾸준한 테스트를 통해 어휘력이 향상되었고, 독해나 문제 풀이 시 이해도가 높아지는 효과를 느낄 수 있었다.</v>
       </c>
       <c r="I186" t="str">
-        <v>재수 기간 동안 항상 세심하게 지도해 주시고 격려해 주신 선생님들께 진심으로 감사드립니다. 학습적인 부분뿐만 아니라 힘들 때마다 따뜻한 조언과 응원을 해주셔서 끝까지 포기하지 않고 노력할 수 있었습니다. 선생님들 덕분에 올바른 방향으로 공부할 수 있었고, 좋은 결과를 향해 나아갈 수 있었습니다. 다시 한 번 깊이 감사드립니다.</v>
+        <v>재수 기간 동안 항상 세심하게 지도해 주시고 격려해 주신 선생님들께 진심으로 감사드립니다. 학습적인 부분뿐만 아니라 힘들 때마다 따뜻한 조언과 응원을 해 주셔서 끝까지 포기하지 않고 노력할 수 있었습니다. 선생님들 덕분에 올바른 방향으로 공부할 수 있었고, 좋은 결과를 향해 나아갈 수 있었습니다. 다시 한 번 깊이 감사드립니다.</v>
       </c>
       <c r="J186" t="str">
         <v>담임 선생님께서 성적 정보를 바탕으로 학습 상태를 꼼꼼하게 점검해 주셨어요.</v>
@@ -7146,7 +7146,7 @@
         <v>사실 입시 때는 공부를 열심히 하는건 기본이고 누가 얼마나 어떻게 하느냐가 중요한 것 같습니다. 근데 이 어떻게를 알려주는게 이투스에서 해주니까 전 믿고 할 수 있었던 것 같아요. 학습 상담 뿐만 아니라 또 입시상담 같은것ㄷㅎ 같이 해주니까 좋았구요</v>
       </c>
       <c r="F187" t="str">
-        <v>전 제가 모르는걸 바로바로 물어보고 해결하도록 하는게 중요하다고 생각합니다. 믿을만한 선생님들이 계속 붙어서 질문을 봐주니까 좋았고 또 야러가지 방식으로 풀이해주시고. 개인 과외를 받는 느낌이었습니다.</v>
+        <v>전 제가 모르는걸 바로바로 물어보고 해결하도록 하는게 중요하다고 생각합니다. 믿을만한 선생님들이 계속 붙어서 질문을 봐주니까 좋았고 또 야러가지 방식으로 풀이해 주시고. 개인 과외를 받는 느낌이었습니다.</v>
       </c>
       <c r="G187" t="str">
         <v>면학 분위기를 감독하는 것은 관리형 독서실에서 필수적인 시스템입니다. 근데 이덜 너무 과도하게 잡거나 계속 돌아다니는건 오히려 공부에 방해가 됩니다. 이투스에서는 과도한 방해ㅜ없이 적당한 수준에서 감독을 진행하니 매우 도움이 되었던 것 같습니다.</v>
@@ -7178,7 +7178,7 @@
         <v>N수생</v>
       </c>
       <c r="E188" t="str" xml:space="preserve">
-        <v xml:space="preserve">학습적인 면 뿐만아니라 멘탈 관리도 해주시고 고민상담도 해주시고 공부잘하는 친구같은 느낌으로 학생들이 가장 선호하는 형식의 멘토였음_x000d_
+        <v xml:space="preserve">학습적인 면 뿐만아니라 멘탈 관리도 해 주시고 고민상담도 해 주시고 공부잘하는 친구같은 느낌으로 학생들이 가장 선호하는 형식의 멘토였음_x000d_
 학습적인 부분에서는 어디서도 듣지못한 공부법을 여럿 들었고 실제로 도움이 되었음</v>
       </c>
       <c r="F188" t="str">
@@ -7191,7 +7191,7 @@
         <v>본인이 다닌 지점에서는 구독권이 있지는 않았지만 있었더라면 독학 학원인 만큼 인강의 도움이 크게 필요하고 이투스의 구독권을 통해 부족한 부분의 인강을 듣고 학습을 해 나갈 수 있었을거 같고 성적 향상에 크게 도움이 되었을 것 같음.</v>
       </c>
       <c r="I188" t="str">
-        <v>항상 친절하시고 응원해주시고 너그럽게 이해해주시고 여러면에서 감동도 많이 받고 위로도 많이 받았습니다. 선생님들 덕분에 좋은 결과 있을 수 있었고 힘들었던 입시를 마무리하게되어 너무 감사드립니다!</v>
+        <v>항상 친절하시고 응원해 주시고 너그럽게 이해해 주시고 여러면에서 감동도 많이 받고 위로도 많이 받았습니다. 선생님들 덕분에 좋은 결과 있을 수 있었고 힘들었던 입시를 마무리하게되어 너무 감사드립니다!</v>
       </c>
       <c r="J188" t="str">
         <v>스마트하게 관리가 이루어져서 체계적이라고 느껴졌어요.</v>
@@ -7265,7 +7265,7 @@
 고마운 존재였습니다. 결코 쉽지 않은 난이도로 항상 저를 당황시켰는데 오히려 시험준비에 더 열심히 임할 수 있었던 것 같습니다.</v>
       </c>
       <c r="I190" t="str">
-        <v>작년, 걱정과 불안이 가득한 입시상담을 받았던게 새록새록 떠오르는데 저는 지금 그 때의 상담에서 선생님께서 말씀하신 대학의 학과에 입학했습니다! 고3 때까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던 건 이투스 강서지점 선생님들의 탁월한 입시 전략과 상담, 생활 환경 조성 덕분이었습니다. 저의 처음이자 마지막 재수를 성공적으로 마치게 해주신 이투스 강서지점 선생님들께 감사를 표합니다!</v>
+        <v>작년, 걱정과 불안이 가득한 입시상담을 받았던게 새록새록 떠오르는데 저는 지금 그 때의 상담에서 선생님께서 말씀하신 대학의 학과에 입학했습니다! 고3 때까지 쳐다도 보지 못한 곳을 이렇게 오게 될 수 있었던 건 이투스 강서지점 선생님들의 탁월한 입시 전략과 상담, 생활 환경 조성 덕분이었습니다. 저의 처음이자 마지막 재수를 성공적으로 마치게 해 주신 이투스 강서지점 선생님들께 감사를 표합니다!</v>
       </c>
       <c r="J190" t="str">
         <v>생활 상담을 포함한 코칭 시스템은 공부 외적인 부분까지 함께 관리해 준다는 점에서 의미가 있었어요.</v>
@@ -7288,21 +7288,21 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E191" t="str" xml:space="preserve">
-        <v xml:space="preserve">생활 상담이 가장 인상 깊었습니다. 단순히 공부 시간만 관리하는 것이 아니라, 수험 생활 전반을 어떻게 유지해야 하는지에 대해 구체적이고 현실적으로 지도해주셔서 큰 도움이 되었습니다. 수면 시간, 식사 습관, 휴식 타이밍 같은 기본적인 생활 패턴부터 집중력이 떨어질 때 대처하는 방법까지 세세하게 알려주셔서 스스로를 관리하는 기준이 생겼습니다._x000d_
-특히 좋았던 점은 실천 가능한 수준으로 디테일하게 설명해주셨다는 점입니다. 하루 루틴을 어떻게 짜야 하는지, 쉬는 시간은 어느 정도가 적절한지, 컨디션이 무너질 때는 어떻게 회복해야 하는지 등 실제 상황을 고려한 조언을 해주셔서 바로 적용할 수 있었습니다._x000d_
-또한 단순히 규칙을 제시하는 데서 끝나는 것이 아니라, 왜 그렇게 해야 하는지 이유까지 설명해주셔서 납득하면서 생활 습관을 바꿀 수 있었습니다. 덕분에 억지로 버티는 느낌이 아니라 스스로 조절하면서 안정적으로 공부할 수 있게 되었습니다._x000d_
+        <v xml:space="preserve">생활 상담이 가장 인상 깊었습니다. 단순히 공부 시간만 관리하는 것이 아니라, 수험 생활 전반을 어떻게 유지해야 하는지에 대해 구체적이고 현실적으로 지도해 주셔서 큰 도움이 되었습니다. 수면 시간, 식사 습관, 휴식 타이밍 같은 기본적인 생활 패턴부터 집중력이 떨어질 때 대처하는 방법까지 세세하게 알려주셔서 스스로를 관리하는 기준이 생겼습니다._x000d_
+특히 좋았던 점은 실천 가능한 수준으로 디테일하게 설명해주셨다는 점입니다. 하루 루틴을 어떻게 짜야 하는지, 쉬는 시간은 어느 정도가 적절한지, 컨디션이 무너질 때는 어떻게 회복해야 하는지 등 실제 상황을 고려한 조언을 해 주셔서 바로 적용할 수 있었습니다._x000d_
+또한 단순히 규칙을 제시하는 데서 끝나는 것이 아니라, 왜 그렇게 해야 하는지 이유까지 설명해 주셔서 납득하면서 생활 습관을 바꿀 수 있었습니다. 덕분에 억지로 버티는 느낌이 아니라 스스로 조절하면서 안정적으로 공부할 수 있게 되었습니다._x000d_
 전체적으로 생활 상담을 통해 공부 외적인 부분까지 체계적으로 관리할 수 있게 되었고, 그 덕분에 장기적으로 흔들리지 않고 공부를 이어갈 수 있는 힘을 얻었다고 느꼈습니다.</v>
       </c>
       <c r="F191" t="str" xml:space="preserve">
         <v xml:space="preserve">단순히 “열심히 해라” 식이 아니라, 제 현재 성적과 약점을 기준으로 굉장히 구체적이고 현실적인 계획을 세워주셔서 방향 잡는 데 큰 도움이 됐습니다. 하루 공부 시간 배분부터 과목별 우선순위까지 꼼꼼하게 짜주셔서, 막막했던 재수 생활을 훨씬 체계적으로 시작할 수 있었어요._x000d_
-특히 좋았던 점은 과목별로 어떤 인강을 들으면 좋은지, 어떤 선생님이 제 스타일에 맞는지까지 세세하게 추천해주신 부분이에요. 단순히 유명한 강의를 추천하는 게 아니라 제 수준과 목표에 맞춰 단계별로 커리큘럼을 구성해주셔서 그대로 따라가기만 해도 공부 흐름이 자연스럽게 이어졌습니다._x000d_
-또한 문제집이나 학습 콘텐츠도 구체적으로 알려주셔서 좋았습니다. “이 시기에는 이 문제집을 풀고, 이 단원은 이런 유형 위주로 연습해라”처럼 바로 실행할 수 있는 조언을 해주셔서 시간 낭비 없이 효율적으로 공부할 수 있었습니다. 혼자였다면 자료 선택에 많은 시간을 썼을 텐데, 그런 고민을 줄여줘서 큰 도움이 됐습니다._x000d_
+특히 좋았던 점은 과목별로 어떤 인강을 들으면 좋은지, 어떤 선생님이 제 스타일에 맞는지까지 세세하게 추천해 주신 부분이에요. 단순히 유명한 강의를 추천하는 게 아니라 제 수준과 목표에 맞춰 단계별로 커리큘럼을 구성해 주셔서 그대로 따라가기만 해도 공부 흐름이 자연스럽게 이어졌습니다._x000d_
+또한 문제집이나 학습 콘텐츠도 구체적으로 알려주셔서 좋았습니다. “이 시기에는 이 문제집을 풀고, 이 단원은 이런 유형 위주로 연습해라”처럼 바로 실행할 수 있는 조언을 해 주셔서 시간 낭비 없이 효율적으로 공부할 수 있었습니다. 혼자였다면 자료 선택에 많은 시간을 썼을 텐데, 그런 고민을 줄여줘서 큰 도움이 됐습니다._x000d_
 전체적으로 학습 관리 시스템이 단순한 조언이 아니라, 실제 성적 향상으로 이어질 수 있는 맞춤형 전략이라는 느낌을 받아서 매우 만족했습니다.</v>
       </c>
       <c r="G191" t="str" xml:space="preserve">
-        <v xml:space="preserve">생활 관리 측면에서 세심하게 챙겨주신 부분이 특히 좋았습니다. 단순히 공부만 강조하는 것이 아니라, 실제로 공부를 지속할 수 있는 컨디션을 유지하도록 도와주신 점이 인상 깊었습니다. 수험 생활을 하다 보면 졸음이 쏟아지거나 집중력이 떨어지는 순간이 많은데, 그럴 때마다 적절하게 깨워주시고 현재 상태를 체크해주셔서 흐름이 끊기지 않도록 관리해주셨습니다._x000d_
+        <v xml:space="preserve">생활 관리 측면에서 세심하게 챙겨주신 부분이 특히 좋았습니다. 단순히 공부만 강조하는 것이 아니라, 실제로 공부를 지속할 수 있는 컨디션을 유지하도록 도와주신 점이 인상 깊었습니다. 수험 생활을 하다 보면 졸음이 쏟아지거나 집중력이 떨어지는 순간이 많은데, 그럴 때마다 적절하게 깨워주시고 현재 상태를 체크해 주셔서 흐름이 끊기지 않도록 관리해주셨습니다._x000d_
 특히 “괜찮겠지” 하고 그냥 넘어갈 수 있는 부분까지도 수시로 확인해주시면서, 졸거나 집중이 흐트러질 때 바로잡아주신 점이 도움이 많이 되었습니다. 덕분에 스스로 놓치기 쉬운 생활 리듬이나 집중 상태를 꾸준히 유지할 수 있었고, 혼자였다면 무너졌을 타이밍도 잘 넘길 수 있었습니다._x000d_
-또한 단순히 깨워주는 데서 끝나는 것이 아니라, 언제 쉬는 게 좋은지, 어떻게 다시 집중을 끌어올려야 하는지까지 함께 지도해주셔서 효율적으로 하루를 운영할 수 있었습니다. 이런 세심한 생활 관리 덕분에 공부 시간의 질 자체가 올라갔다고 느꼈습니다.</v>
+또한 단순히 깨워주는 데서 끝나는 것이 아니라, 언제 쉬는 게 좋은지, 어떻게 다시 집중을 끌어올려야 하는지까지 함께 지도해 주셔서 효율적으로 하루를 운영할 수 있었습니다. 이런 세심한 생활 관리 덕분에 공부 시간의 질 자체가 올라갔다고 느꼈습니다.</v>
       </c>
       <c r="H191" t="str" xml:space="preserve">
         <v xml:space="preserve">매일 진행되는 수능특강 영어 단어 테스트가 정말 도움이 많이 되었습니다. 혼자 공부할 때는 단어 암기를 꾸준히 이어가는 것이 쉽지 않은데, 매일 정해진 시간에 테스트를 보게 되니 자연스럽게 반복 학습이 이루어졌습니다. 덕분에 단어를 미루지 않고 꾸준히 외울 수 있었고, 장기적으로 기억에도 더 잘 남는 느낌이었습니다._x000d_
@@ -7310,8 +7310,8 @@
 또한 매일 꾸준히 쌓이는 방식이라 부담스럽지 않으면서도 학습량이 자연스럽게 누적되는 점이 인상적이었습니다. 이런 시스템 덕분에 영어 단어에 대한 기본기가 탄탄해졌고, 독해를 할 때도 훨씬 수월해졌다고 느꼈습니다.</v>
       </c>
       <c r="I191" t="str" xml:space="preserve">
-        <v xml:space="preserve">수험 생활 동안 단순히 공부만 도와주신 것이 아니라, 방향을 잃지 않도록 계속해서 이끌어주시고 세심하게 관리해주신 덕분에 끝까지 버틸 수 있었습니다. 항상 학생 한 명 한 명의 상태를 신경 써주시고, 필요한 부분을 놓치지 않고 챙겨주시는 모습이 정말 인상 깊었습니다._x000d_
-공부뿐만 아니라 생활적인 부분까지 꼼꼼하게 지도해주셔서 안정적으로 수험 생활을 이어갈 수 있었고, 힘들 때마다 해주신 말 한마디, 작은 관심 하나가 큰 힘이 되었습니다. 덕분에 포기하지 않고 계속 나아갈 수 있었던 것 같습니다.</v>
+        <v xml:space="preserve">수험 생활 동안 단순히 공부만 도와주신 것이 아니라, 방향을 잃지 않도록 계속해서 이끌어주시고 세심하게 관리해 주신 덕분에 끝까지 버틸 수 있었습니다. 항상 학생 한 명 한 명의 상태를 신경 써주시고, 필요한 부분을 놓치지 않고 챙겨주시는 모습이 정말 인상 깊었습니다._x000d_
+공부뿐만 아니라 생활적인 부분까지 꼼꼼하게 지도해 주셔서 안정적으로 수험 생활을 이어갈 수 있었고, 힘들 때마다 해 주신 말 한마디, 작은 관심 하나가 큰 힘이 되었습니다. 덕분에 포기하지 않고 계속 나아갈 수 있었던 것 같습니다.</v>
       </c>
       <c r="J191" t="str">
         <v>혼자 공부했으면 하루를 어떻게 보내야 할지 효율적으로 계획하는 것이 힘들었을 텐데 일주일 단위로 공부해야 할 것을 계획할 수 있어서 좋았어요.</v>
@@ -7334,19 +7334,19 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E192" t="str">
-        <v>원장 선생님과 상담할 때 정말 평소 쌓였던 고민들과 걱정이 모두 뻥 사라지는 느낌이었습니다. 수시와 정시를 둘 다 챙기는 게 맞을 지, 과학 공부 방법과 등급 상승 방법 등등 혼자 끙끙 앓던 것들을 질문하니까 정말 명료하게 해결해주셨던 기억이 납니다. 잘하고 있다고 항상 응원해주시고 격려 많이해주셔서 학원 상담이 기다려졌던 것 같네요!</v>
+        <v>원장 선생님과 상담할 때 정말 평소 쌓였던 고민들과 걱정이 모두 뻥 사라지는 느낌이었습니다. 수시와 정시를 둘 다 챙기는 게 맞을 지, 과학 공부 방법과 등급 상승 방법 등등 혼자 끙끙 앓던 것들을 질문하니까 정말 명료하게 해결해주셨던 기억이 납니다. 잘하고 있다고 항상 응원해 주시고 격려 많이해 주셔서 학원 상담이 기다려졌던 것 같네요!</v>
       </c>
       <c r="F192" t="str">
         <v>평소 궁금했던 것을 해결할 수 있는 점이 좋았고 팁 주신 것들을 다음주에 다시 여쭤보시니까 더 열심히 지키려고 노력했던 것 같습니다. 개인적으로 봐주시는 시간이 있어서 성적 상승과 동기부여에 좋은 영향을 미쳤던 것 같습니다.</v>
       </c>
       <c r="G192" t="str">
-        <v>선생님들이 계속 돌아다니시고 감독하시니까 졸려도 쉬는 시간까지 참고 공부하고 한 타임동안 억지로라도 집중하려 하다보니 집중력이 많이 늘었던 것 같습니다. 그리고 항상 집중하고 있으니 선생님들이 칭찬도 해주셔서 뿌듯했고 기분이 좋았습니다..</v>
+        <v>선생님들이 계속 돌아다니시고 감독하시니까 졸려도 쉬는 시간까지 참고 공부하고 한 타임동안 억지로라도 집중하려 하다보니 집중력이 많이 늘었던 것 같습니다. 그리고 항상 집중하고 있으니 선생님들이 칭찬도 해 주셔서 뿌듯했고 기분이 좋았습니다..</v>
       </c>
       <c r="H192" t="str">
         <v>단어량이 자동으로 많이 늘어서 영어 등급 향상에 많은 도움이 되었던 것 같습니다. 저는 강제성이 없이 자발적으로 공부하는 편이었어서 단어가 항상 뒤로 밀렸는데 억지로라도 계속 테스트를 보니까 어휘력이 늘어서 등급이 두달만에 3등급 상승했습니다.</v>
       </c>
       <c r="I192" t="str">
-        <v>제 고3시절 중 가장 행복했던 시간은 이투스에서 였습니다.. 항상 학원 갈 때 올 때 수고한다고 말해주시고 등하교 찍을 때도 힘들지~ 이런 말 해 주시는 게 항상 힘이 되었습니다. 집중도 가장 잘 되었고 환경도 너무 쾌적해서 저는 인생에서 이투스에 있을 때 공부를 제일 효율적으로, 또 많이 했습니다. 선생님들의 많은 격려와 칭찬이 저를 동기부여 했던 것 같습니다. 지금도 이투스를 생각하면 기분이 좋습니다. 이투스 아니었으면 저 대학 못갔습니다 감사합니다~</v>
+        <v>제 고3시절 중 가장 행복했던 시간은 이투스에서 였습니다.. 항상 학원 갈 때 올 때 수고한다고 말해 주시고 등하교 찍을 때도 힘들지~ 이런 말 해 주시는 게 항상 힘이 되었습니다. 집중도 가장 잘 되었고 환경도 너무 쾌적해서 저는 인생에서 이투스에 있을 때 공부를 제일 효율적으로, 또 많이 했습니다. 선생님들의 많은 격려와 칭찬이 저를 동기부여 했던 것 같습니다. 지금도 이투스를 생각하면 기분이 좋습니다. 이투스 아니었으면 저 대학 못갔습니다 감사합니다~</v>
       </c>
       <c r="J192" t="str">
         <v>고민 상담, 멘탈 관리, 공부 팁 등도 자주 알려주셔서 큰 도움이 되었어요.</v>
@@ -7416,7 +7416,7 @@
         <v>수능 입시를 준비하다보면 평가원 모의고사 뿐만이 아니라 많은 사설 모의고사들도 풀어보며 시험 볼 때의 태도를 많이 연습할 수 있는데 이투스 모의고사를 의무로 봄으로써 학원에서 강제적으로라도 나의 시험 태도를 확인할 수 있어서 좋았다.</v>
       </c>
       <c r="I194" t="str">
-        <v>항상 아침에 웃는 얼굴로 인사해주시고 대학 상담이나 여쭙고 싶은게 있을 때 언제든지 환영해주셔서 감사했습니다. 수능 후 논술 대비까지 응원해주셔서 덕분에 좋은 재수 생활을 하고 합격할 수 있었던 것 같아요. 감사합니다!</v>
+        <v>항상 아침에 웃는 얼굴로 인사해 주시고 대학 상담이나 여쭙고 싶은게 있을 때 언제든지 환영해 주셔서 감사했습니다. 수능 후 논술 대비까지 응원해 주셔서 덕분에 좋은 재수 생활을 하고 합격할 수 있었던 것 같아요. 감사합니다!</v>
       </c>
       <c r="J194" t="str">
         <v>취약 유형을 담임 선생님과 상담하면서 집중적으로 끌어올릴 수 있었어요.</v>
@@ -7440,7 +7440,7 @@
       </c>
       <c r="E195" t="str" xml:space="preserve">
         <v xml:space="preserve">재수생의 맞는 학습 패턴과 함께 올바른 공부 방법을 지도하여 주시며_x000d_
-수험 생활에서의 어려움을 공감하며 본인의 경험과 함께 더불어 뜻깊은 조언을 해주신다. 또 외로운 수험 생활에서 일상의 대화가 되어주시기도 하며 더욱 공부에 집중할 수 있도록 최선을 다해주셔서 생활에 도움이 많이 되었다.</v>
+수험 생활에서의 어려움을 공감하며 본인의 경험과 함께 더불어 뜻깊은 조언을 해 주신다. 또 외로운 수험 생활에서 일상의 대화가 되어주시기도 하며 더욱 공부에 집중할 수 있도록 최선을 다해 주셔서 생활에 도움이 많이 되었다.</v>
       </c>
       <c r="F195" t="str">
         <v>혼자서 독학 재수를 하는 점에서 가장 불편하고도 어려운 부분이 즉각적인 질의 응답이 되어지지 않는 것인데 이 부분을 해결해주며 또 각 과목 마다 선생님이 배정되어 있으셔서 빠르게 피드백을 받고 질문을 할 수 있었다.</v>
@@ -7517,14 +7517,14 @@
 그리고 다른 과목들도 인강선생님들을 추천받거나, 학습자료들도 많이 도움을 받았습니다 !</v>
       </c>
       <c r="F197" t="str" xml:space="preserve">
-        <v xml:space="preserve">주마다 불러내시어, 과목별로 지금 어떤 공부들을 하고 있는지 점검을 해주셔서 _x000d_
+        <v xml:space="preserve">주마다 불러내시어, 과목별로 지금 어떤 공부들을 하고 있는지 점검을 해 주셔서 _x000d_
 일단 플래너와 주 학습 계획을 더 잘 세울 수 있게 되었습니다. _x000d_
 그리고 같이 어떤 공부를 어떻게 했는지 대화하다보면, 어떤 과목이 시간이 부족했으며 능률이 오르지 않았고, _x000d_
-실모 같은 경우도 어떤 유형들이 안되는지 잘 체크를 해주셔서 저의 문제점을 찾기 좋았던 것 같습니다. 또한 과목별로 제 스타일에 맞는 선생님들을 추천해 주셔서 도움을 많이 받았습니다 !</v>
+실모 같은 경우도 어떤 유형들이 안되는지 잘 체크를 해 주셔서 저의 문제점을 찾기 좋았던 것 같습니다. 또한 과목별로 제 스타일에 맞는 선생님들을 추천해 주셔서 도움을 많이 받았습니다 !</v>
       </c>
       <c r="G197" t="str" xml:space="preserve">
         <v xml:space="preserve">정신차리고 항상 자지 않으려고 노력은 하지만, 어쩔 수 없이 잠이 올 때 _x000d_
-수시로 깨워주시고 태도가 좋지 않을 때에도 잘 잡아주셔서 공부가 잘 되었던 것 같습니다. 그리고 학생의 컨디션도 잘 체크를 해주셔서 제가 몸이 좋지 않을때에는 제 편의를 봐주시면서 학습 관리 체크를 해주셨는데, n수 할때 도움이 많이 되었던 것 같습니다</v>
+수시로 깨워주시고 태도가 좋지 않을 때에도 잘 잡아주셔서 공부가 잘 되었던 것 같습니다. 그리고 학생의 컨디션도 잘 체크를 해 주셔서 제가 몸이 좋지 않을때에는 제 편의를 봐주시면서 학습 관리 체크를 해주셨는데, n수 할때 도움이 많이 되었던 것 같습니다</v>
       </c>
       <c r="H197" t="str" xml:space="preserve">
         <v xml:space="preserve">공부를 시작하기에 앞서, 20-30분 정도 일일테스트로 머리를 깨우고 공부를 하는게 도움이 많이 되었습니다. _x000d_
@@ -7594,8 +7594,8 @@
         <v>매 달 모의고사가 끝날 때마다 담임 선생님이 그 달에 쳤던 성적으로 어느 정도의 대학을 갈 수 있는지, 그리고 특정 과목의 몇 문제를 더 맞았을 때 대학 라인이 얼마나 바뀌는지 자세히 알려주셔서 도움이 됐습니다</v>
       </c>
       <c r="F199" t="str" xml:space="preserve">
-        <v xml:space="preserve">담임 선생님께서 보셨을 때 학습 시간이 부족해 보이는 과목을 짚어주시고, 어떤 방향으로 학습해 나가야할지 조언해주셔서 도움이 됐습니다_x000d_
-수능이 많이 다가왔을 때는 플래너 검사도 매일매일 해주셔서 방향을 잃지 않고 끝까지 완주했던 기억이 납니다</v>
+        <v xml:space="preserve">담임 선생님께서 보셨을 때 학습 시간이 부족해 보이는 과목을 짚어주시고, 어떤 방향으로 학습해 나가야할지 조언해 주셔서 도움이 됐습니다_x000d_
+수능이 많이 다가왔을 때는 플래너 검사도 매일매일 해 주셔서 방향을 잃지 않고 끝까지 완주했던 기억이 납니다</v>
       </c>
       <c r="G199" t="str">
         <v>급식을 먹고 나면 카페인 음료를 마셔도 식곤증으로 인해 졸음이 달아나지 않아 정신이 안 차려질 때가 있었는데 그 때마다 감독하시는 선생님이 깨워주셔서 정신차리고 공부를 이어갈 수 있어서 좋았습니다</v>
@@ -7607,7 +7607,7 @@
         <v>학원에 다니던 당시에는 제가 신경써야할 공부들이 너무 많고 떨어진 체력 때문에 선생님들께 감사인사도 제대로 못한 것 같습니다 뒤늦은 감사인사이지만 진심으로 감사합니다! 잘 이끌어주시고 가르쳐주셨던 안성이투스 선생님들 덕분에 아예 노베이스였던 제가 1년만에 인서울을 할 수 있었던 것 같습니다</v>
       </c>
       <c r="J199" t="str">
-        <v>국어 문학의 약점을 파악하고, 제게 맞는 풀이법과 학습 방법을 알려주셔서 공부 방향을 잡을 수 있었어요.</v>
+        <v>국어 문학의 약점을 파악하고, 제게 맞는 풀이법과 학습 방법을 알려주셔서 학습 방향을 잡을 수 있었어요.</v>
       </c>
       <c r="K199" t="str">
         <v/>
@@ -7701,19 +7701,19 @@
         <v>N수생</v>
       </c>
       <c r="E202" t="str">
-        <v>선생님께서 효율적이고 저에게 맞는  시간표를 짤 수 있게 도움을 많이 주십니다! 혼자서 1년간의 시간을 분배하기에는 어려운 부분이 있었어서 좋았어요 공부할 때 자주 돌아다니면서 상태 체크해주셔서 계속 집중해서 공부할 수 있었습니다. 어려운 문제를 질문하몀 천천히 잘 설명해주셔서 이해가 잘 됐어요</v>
+        <v>선생님께서 효율적이고 저에게 맞는  시간표를 짤 수 있게 도움을 많이 주십니다! 혼자서 1년간의 시간을 분배하기에는 어려운 부분이 있었어서 좋았어요 공부할 때 자주 돌아다니면서 상태 체크해 주셔서 계속 집중해서 공부할 수 있었습니다. 어려운 문제를 질문하몀 천천히 잘 설명해 주셔서 이해가 잘 됐어요</v>
       </c>
       <c r="F202" t="str">
         <v>혼자서는 꾸준히 규칙적으로 계속 공부하는걸 이어나가는게 힘든데 학습 관리 시스템 덕분에 도움을 많이 받았습니다 세세한 부분까지 관리받을 수 있어서 딴생각 안하고 공부만 잘 할수 있었던거같아요</v>
       </c>
       <c r="G202" t="str">
-        <v>선생님이 직접 돌아다니면서 관리해 주셔서 좋았어요 무작정 깨우지도 않고 너무 힘들 때는 어느정도 잘수 있게도 해주셔서 감사햇습니다 자주 돌아다니면서 면학 분위기 관리를 해주셔서 분위기 안좋았던 적이 거의 없었던거같아요 방해 안돼서 좋았습미다</v>
+        <v>선생님이 직접 돌아다니면서 관리해 주셔서 좋았어요 무작정 깨우지도 않고 너무 힘들 때는 어느정도 잘수 있게도 해 주셔서 감사햇습니다 자주 돌아다니면서 면학 분위기 관리를 해 주셔서 분위기 안좋았던 적이 거의 없었던거같아요 방해 안돼서 좋았습미다</v>
       </c>
       <c r="H202" t="str">
         <v>이투스 구독을 무료로 할 수 있어서 구독 갱신 같은 거 신경 안쓰고 학습 효율을 크게 높일수있었습니다! 이투스 안에 다양한 강의가 있어서 듣고싶은 거 제약없이 다 들을 수 있어서 좋았어요 무엇보다!!! 학원비에 구독비를 추가로 낼 필요가 없으니까 별도의 비용 부담 없이 이투스 강의를 들을수 있어서 경제적인 측면에서도 매우 좋앗습니다 ㅎㅎ</v>
       </c>
       <c r="I202" t="str">
-        <v>이투스에서 항상 저를 위해 신경써주셧던 선생님들께 진심으로 감사드립니다 !! 힘들고 지칠 때마다 따뜻한 말도 해주시고 현실적인 말도 해주셔서 다시 마음을 다잡고 할수있었어요 늘 묵묵히 응원도 해주시고 세심하게 관리해 주셔서 큰 힘이 되었습니다! 덕분에 학원에서 열심히 공부할 수있었어요</v>
+        <v>이투스에서 항상 저를 위해 신경써주셧던 선생님들께 진심으로 감사드립니다 !! 힘들고 지칠 때마다 따뜻한 말도 해 주시고 현실적인 말도 해 주셔서 다시 마음을 다잡고 할수있었어요 늘 묵묵히 응원도 해 주시고 세심하게 관리해 주셔서 큰 힘이 되었습니다! 덕분에 학원에서 열심히 공부할 수있었어요</v>
       </c>
       <c r="J202" t="str">
         <v>매번 학습일지를 작성하고 주기적인 피드백을 받으며 공부 계획을 잡아 원동력을 잃지 않고 공부할 수 있었어요.</v>
@@ -7814,7 +7814,7 @@
         <v>N수생</v>
       </c>
       <c r="E205" t="str">
-        <v>재수를 시작하고 저의 공부상태를 점검해주시고 저의 수준과 목표를 고려하여 어떤 강사의 어떤 커리큘럼을 따라가야할지에 대한 방향성을 잡아주었습니다. 또한 모의고사 성적관리도 꼼꼼히 해주며 부족한 부분들을 보완해주시려고 노력해주었습니다.</v>
+        <v>재수를 시작하고 저의 공부상태를 점검해 주시고 저의 수준과 목표를 고려하여 어떤 강사의 어떤 커리큘럼을 따라가야할지에 대한 방향성을 잡아주었습니다. 또한 모의고사 성적관리도 꼼꼼히 해주며 부족한 부분들을 보완해주시려고 노력해주었습니다.</v>
       </c>
       <c r="F205" t="str">
         <v>모의고사 성적들을 봐주시고 어떤점이 부족한지 보완해야 할점은 무엇인지를 같이 고민해주셨습니다. 또한 제가 필요한 자료들을 찾아주셔서 학습에 많은 도움이 되었습니다. 자습시간때도 지속적케어로 많은 도움을 받았습니다.</v>
@@ -7849,7 +7849,7 @@
         <v>N수생</v>
       </c>
       <c r="E206" t="str">
-        <v>공부 방법과 앞으로의 학습 방향을 잘 알려주시고 상담해주셔서 학습에 도움이 많이 되었습니다. 1:1로 원할 때 상담할 수 있어 좋았고, 선생님들께서 친절하시고 진중하게 상담에 임해주셨습니다. 성적이 나왔을 때 항상 같이 상담하며 멘탈을 잡아주셨고, 힘들 때나 지칠 때 학생들에게 깊게 공감해주시면서 응원해주셨습니다.</v>
+        <v>공부 방법과 앞으로의 학습 방향을 잘 알려주시고 상담해 주셔서 학습에 도움이 많이 되었습니다. 1:1로 원할 때 상담할 수 있어 좋았고, 선생님들께서 친절하시고 진중하게 상담에 임해주셨습니다. 성적이 나왔을 때 항상 같이 상담하며 멘탈을 잡아주셨고, 힘들 때나 지칠 때 학생들에게 깊게 공감해주시면서 응원해주셨습니다.</v>
       </c>
       <c r="F206" t="str">
         <v>선생님께서 학습 중 길을 잃을 때마다 상담해주시며 길을 잡도록 도와주셨습니다. 과목을 바꿔야할지, 논술로 바꿔야할지, 이런 큰 고민들을 함께 상담해주시며 문제들을 해결해 나갔는데, 이 부분이 앞으로의 공부 방향의 해결뿐만 아니라 멘탈적으로도 많은 도움이 되었습니다.</v>
@@ -7884,7 +7884,7 @@
         <v>N수생</v>
       </c>
       <c r="E207" t="str">
-        <v>어떤 점이 부족하고 어떻게 공부해야 하는지 친절히 알려주셨습니다. 또한 인강 선생님들마다의 특징도 잘 알고 계시고 무슨 교재가 지금 적절할지 조언해주셨습니다. 모의고사가 얼마 남지 않았을땐 어떻게 선택과 집중을 해야 하는지, 어떤 단원에 힘을 써야할지도 제 상황에 맞게 알려주시고 지도해주셔서 큰 도움이 되었고 힘이 되었습니다.</v>
+        <v>어떤 점이 부족하고 어떻게 공부해야 하는지 친절히 알려주셨습니다. 또한 인강 선생님들마다의 특징도 잘 알고 계시고 무슨 교재가 지금 적절할지 조언해주셨습니다. 모의고사가 얼마 남지 않았을땐 어떻게 선택과 집중을 해야 하는지, 어떤 단원에 힘을 써야할지도 제 상황에 맞게 알려주시고 지도해 주셔서 큰 도움이 되었고 힘이 되었습니다.</v>
       </c>
       <c r="F207" t="str">
         <v>무엇보다 부담 없이 과목별 선생님과 상담할 수 있는 것이 마음에 들었습니다. 인강을 들으면서 학습을 하다 보니 모르거나 궁금한 것이 있을때 바로 의견•조언을 얻기가 힘들어서 고민이었는데, 그럴때마다 바로바로 질문을 드리고 해답을 얻을 수 있는 것이 큰 도움이 되었습니다.</v>
@@ -7931,7 +7931,7 @@
         <v>이투스 전국 모의고사가 좋았던 이유는 매달 실시하기 때문에 본인의 성적변천을 잘 확인할 수 있었습니다. 또한 시험을 본 사람에게 성적표를 나누어 주는데 나에게 어떤 부분이 취약한지, 등급컷과 합격 가능권인 대학까지 다 알려주기 때문에 도움이 많이 되었다고 생각하는 콘텐츠중 하나입니다</v>
       </c>
       <c r="I208" t="str">
-        <v>관리 감독해주시고 학생 개개인에게 집중하여 상담해주시느라 고생하셨습니다 덕분에 좋은 환경에서 공부할 수 있었습니다 진심으로 다른 학생들에게도 추천하고 싶습니다 또한 아침부터 늦은 밤까지 학원에서 감독하시는게 쉽지 않으셨을텐데 지금이라도 감사의 말씀 전하고 싶습니다</v>
+        <v>관리 감독해 주시고 학생 개개인에게 집중하여 상담해주시느라 고생하셨습니다 덕분에 좋은 환경에서 공부할 수 있었습니다 진심으로 다른 학생들에게도 추천하고 싶습니다 또한 아침부터 늦은 밤까지 학원에서 감독하시는게 쉽지 않으셨을텐데 지금이라도 감사의 말씀 전하고 싶습니다</v>
       </c>
       <c r="J208" t="str">
         <v>매달 이투스 모의고사를 보며 실전 감각을 키우고, 성적 분석 리포트로 취약점을 확인해 학습 계획을 보완할 수 있었어요.</v>
@@ -7957,16 +7957,16 @@
         <v>습코칭을 받으면서 공부 방향을 잡는 데 큰 도움이 되었다. 특히 스터디플래너를 많이 써본 적이 없었는데 플래너 작성 방법부터 시간 관리, 효율적인 공부 방식까지 구체적으로 알려주셔서 정말 유용했다.</v>
       </c>
       <c r="F209" t="str">
-        <v>평소 계획을 세우고 공부하지 않고 그때그때 하고싶은 공부를 하여 공부 비중이 고르지않았다. 근데 주단위로 하루에 무엇을 얼만큼 공부할지 계획을 같이 세우고 피드백해주셔서 고르게 공부할 수 있었다.</v>
+        <v>평소 계획을 세우고 공부하지 않고 그때그때 하고싶은 공부를 하여 공부 비중이 고르지않았다. 근데 주단위로 하루에 무엇을 얼만큼 공부할지 계획을 같이 세우고 피드백해 주셔서 고르게 공부할 수 있었다.</v>
       </c>
       <c r="G209" t="str">
-        <v>잠이 많은 편이라 공부할 때 많이 졸았는데 학습 코칭 선생님께서 졸음 관리를 확실하게 지도해주셔서 많은 도움이 되었다. 졸릴 때는 자리에서 벗어나 밖에 서서 공부하라고 해 주시는 게 도움됐다.</v>
+        <v>잠이 많은 편이라 공부할 때 많이 졸았는데 학습 코칭 선생님께서 졸음 관리를 확실하게 지도해 주셔서 많은 도움이 되었다. 졸릴 때는 자리에서 벗어나 밖에 서서 공부하라고 해 주시는 게 도움됐다.</v>
       </c>
       <c r="H209" t="str">
         <v>실전처럼 모의고사를 볼 수 있는 환경이 마련되어 있어 실제 시험을 대비하는 데 큰 도움이 되었다. 시험 분위기를 미리 경험할 수 있어서 긴장감 조절에도 좋았고 문제 풀이 감각을 익히는 데 유익했다. 그리고 콘텐츠를 신청할 수 있는 방식이 가까워서 번거롭지 않고 편리하게 이용할 수 있었던 점도 좋았다.</v>
       </c>
       <c r="I209" t="str">
-        <v>선생님들께 진심으로 감사드립니다. 꾸준한 지도 덕분에 공부 방향을 잡고 노력할 수 있었습니다. 항상 세심하게 신경 써주시고 응원해주셔서 큰 힘이 되었습니다. 덕분에 포기하지 않고 계속 나아갈 수 있었습니다. 정말 감사합니다.</v>
+        <v>선생님들께 진심으로 감사드립니다. 꾸준한 지도 덕분에 공부 방향을 잡고 노력할 수 있었습니다. 항상 세심하게 신경 써주시고 응원해 주셔서 큰 힘이 되었습니다. 덕분에 포기하지 않고 계속 나아갈 수 있었습니다. 정말 감사합니다.</v>
       </c>
       <c r="J209" t="str">
         <v>철저한 자습실 관리와 졸음 관리, 주기적인 상담 덕분에 수능 전까지 긴장감을 유지하며 공부할 수 있었어요.</v>
@@ -8001,7 +8001,7 @@
         <v>더프, 강K같은 다른 사설 모의고사들을 많이 풀어봤는데, 이투스 모의고사는 사설 모의고사 중에서도 어려운 편이어서 실전에서 어려운 문제를 만났을 때를 대비할 수 있었던 것 같습니다.</v>
       </c>
       <c r="I210" t="str">
-        <v>이투스에서 여름방학 한달 간 지내는 동안 항상 질문하면 친절하게 대답해주시고 요청사항을 말하면 잘 들어주시고 공부에 집중할 수 있는 환경을 만들어 주셔서 감사했습니다^^.  덕분에 대학 합격했어요.</v>
+        <v>이투스에서 여름방학 한달 간 지내는 동안 항상 질문하면 친절하게 대답해 주시고 요청사항을 말하면 잘 들어주시고 공부에 집중할 수 있는 환경을 만들어 주셔서 감사했습니다^^.  덕분에 대학 합격했어요.</v>
       </c>
       <c r="J210" t="str">
         <v>학원에서 실전처럼 꾸준히 연습한 덕분에 실제 수능에서도 평소처럼 집중할 수 있었어요.</v>
@@ -8027,7 +8027,7 @@
         <v>주기적으로 했던것으로 기억하는데 그때는 그냥 단순히 가야할 방향을 점검하고 조정하는 정도로 생각했었는데 지나고 보니까 수험생 기간동안 이러한 요소를 잡아주는것은 매우 힘이 되었던것 같다. 또한 국어에서 약점을 지니고 있었는데 상담해 주시는 분이 국어 선생님이여서 약점 분석 부터 약점을 극복하기 위한 솔루션들을 주셨던것 같다. 이를 통해 국어 실력을 더욱 끌어올릴수 있었던것 같다.</v>
       </c>
       <c r="F211" t="str">
-        <v>1 대 1 질의 응답은 탐구 과목 위주로 신청했었는데 질문 받아주시는 분이 정말 친절하고 꼼꼼히 설명해주시고 꽤나 어려운 문제였는데도 손쉽게 알려주셔서 공부하는데 매우 유용했던것 같다.</v>
+        <v>1 대 1 질의 응답은 탐구 과목 위주로 신청했었는데 질문 받아주시는 분이 정말 친절하고 꼼꼼히 설명해 주시고 꽤나 어려운 문제였는데도 손쉽게 알려주셔서 공부하는데 매우 유용했던것 같다.</v>
       </c>
       <c r="G211" t="str">
         <v>수험생 생활이 끝나고 되돌아보면 휴대폰 수거는 매우 중요하고 필수적인것 같다. 지금 와서 생각해보면 어떻게 공부를 했나 싶을정도로 폰 중독에서 벗어나지 못하고있다. 아마도 이는 다른 수험생들에게도 필수적인 요소일 것이다</v>
@@ -8036,7 +8036,7 @@
         <v>영어공부를 딱히 따로 하지 않았는데 일년간, 그냥 단어 시험을 위해 공부를 했던것 매우 큰 도움이 되었던것 같다.  재시험 커트라인이 꽤나 빡빡했던것 같은데 그래서 더 도움이 되었던것 같다.</v>
       </c>
       <c r="I211" t="str">
-        <v>진짜 감사했습니다.  내원생이름도 외우시고 안부도 여쭤봐주시고 아침 일찍 출근하시고 상담도 해주시고 수험생들 공부 환경 만들어 주시려 애썼던것들 모두 감사합니다. 이 외에도 해주신것들이 많았던것 같은데 진짜 감사합니다.</v>
+        <v>진짜 감사했습니다.  내원생이름도 외우시고 안부도 여쭤봐주시고 아침 일찍 출근하시고 상담도 해 주시고 수험생들 공부 환경 만들어 주시려 애썼던것들 모두 감사합니다. 이 외에도 해 주신것들이 많았던것 같은데 진짜 감사합니다.</v>
       </c>
       <c r="J211" t="str">
         <v>학습 관리 시스템 덕분에 공부 시간을 체계적으로 관리하고, 계획·실행·피드백 과정을 꾸준히 이어갈 수 있었어요.</v>
@@ -8103,7 +8103,7 @@
         <v>요즘 같은 시대에 공부에 가장 방해가 되는 요소는 아무래도 휴대전화일 것 같은데요. 아침에 등원 하자마자 휴대폰을 제출하는 시스템이기 때문에 휴대폰을 보며 시간을 날리는 경우가 현저히 줄 수 밖에 없어서 좋았습니다. 서포터즈를 하는 경우와 같이 특수한 일이 있을 때는 허락을 받고 사용할 수 있어서 불편함이 없었습니다.</v>
       </c>
       <c r="H213" t="str">
-        <v>혼자 자습만 하다 보면 실전 모의고사를 푸는 감을 잃어버릴 수가 있어요. 하지만 매달 더프 모의고사와 이투스 모의고사와 같은 사설 모의고사를 치면서 그 감을 유지 할 수 있었습니다. 또 시험 후 결과를 보고 선생님께서 보완해야 할 부분과 방향을 제시해 주셔서 정말 좋았어요. 수학 모의고사 같은 경우는 무료로 풀이도 다 해주시고 1:1 상담도 해주셔서 무척이나 유용했던 기억이 있습니다!!</v>
+        <v>혼자 자습만 하다 보면 실전 모의고사를 푸는 감을 잃어버릴 수가 있어요. 하지만 매달 더프 모의고사와 이투스 모의고사와 같은 사설 모의고사를 치면서 그 감을 유지 할 수 있었습니다. 또 시험 후 결과를 보고 선생님께서 보완해야 할 부분과 방향을 제시해 주셔서 정말 좋았어요. 수학 모의고사 같은 경우는 무료로 풀이도 다 해 주시고 1:1 상담도 해 주셔서 무척이나 유용했던 기억이 있습니다!!</v>
       </c>
       <c r="I213" t="str">
         <v>이투스 학원을 졸업?한지 벌써 6개월이 흘렀네요.. 작년 2월부터 10월 말까지 직접적이든 간접적이든 저와 함께 해주셨던 선생님들이 계셨기에 지금 제가 서울에서 즐거운 시간을 보낼 수 있다고 생각해요. 솔직히 재수라는 게 절대 행복한 시간으로 기억 될 수다 없다고 생각했는데, 왜인지 저에게는 좋은 기억으로 남아 있습니다. 제가 있었던 부산 서면 이투스 247학원은 정이 넘치는 따뜻한 공간이었던 것 같아요!! 저의 인생에 좋은 영향을 주셔서 너무 감사합니다! 항상 무탈하세요!!</v>
@@ -8129,7 +8129,7 @@
         <v>N수생</v>
       </c>
       <c r="E214" t="str">
-        <v>수능이 얼마 안 남은 시점 긴장감과 부담감이 많았는데 선생님과의 상담을 통해 긴장이 많이 풀리고 자신감이 생겼습니다ㅏ 또한 학습 방법에 대한 자세한 조언들을 많이 해주셔서 공부 방향을 잡는 데에 많은 도움이 되었습니다</v>
+        <v>수능이 얼마 안 남은 시점 긴장감과 부담감이 많았는데 선생님과의 상담을 통해 긴장이 많이 풀리고 자신감이 생겼습니다ㅏ 또한 학습 방법에 대한 자세한 조언들을 많이 해 주셔서 공부 방향을 잡는 데에 많은 도움이 되었습니다</v>
       </c>
       <c r="F214" t="str">
         <v>과목에서 어떤 부분을 더 신경써야할지, 어느 부분은 어떻게 공부해야 좋을지에 대해 세세하게 짚어주셔서 학습하는데에 더 수월하고 빠른 방법으로 공부할 수 있어서 그 점이 가장 유용했습니다</v>
@@ -8142,7 +8142,7 @@
 모의고사 말고도 이투스에서 자체적인 모의고사를 보면서 모의고사를 보는 횟수를 늘리니 수능장에서의 감을 익히기 더 좋았습니다</v>
       </c>
       <c r="I214" t="str">
-        <v>짧은 시간동안 다녔지만 정말 의미있는 공부 시간을 보낸것같아 좋았습니다 조금 더 빨리 왔으면 좋았겠다는 후회를 많이 했어요 항상 친절하게 대해주셔서 감사했습니다ㅠㅠ 항상 건강하시구 좋은 일만 생기시길 빌게요 서울강동이투스화이띵</v>
+        <v>짧은 시간동안 다녔지만 정말 의미있는 공부 시간을 보낸것같아 좋았습니다 조금 더 빨리 왔으면 좋았겠다는 후회를 많이 했어요 항상 친절하게 대해 주셔서 감사했습니다ㅠㅠ 항상 건강하시구 좋은 일만 생기시길 빌게요 서울강동이투스화이띵</v>
       </c>
       <c r="J214" t="str">
         <v>평가원 모의고사와 실전 모의고사 후 과목별 상담을 통해 틀린 이유를 분석하고, 다음 시험을 위한 학습 방향을 잡을 수 있었어요.</v>
@@ -8165,10 +8165,10 @@
         <v>N수생</v>
       </c>
       <c r="E215" t="str">
-        <v>매주 정해진 시간에 그 주 학습에 대한 피드백을 받고, 각 과목에 대한 진도에 맞추어 그 주 학습 방법을 조언해주셔서 유용했다. 더 프리미엄 모의고사나 이투스 모의고사, 평가원 모의고사가 끝난 뒤, 작성한 오답노트를 통해 어떤 부분에서 문제를 틀렸는지 다각도로 분석해주시고 그 유형에 대해 빨리 풀 수 있는 숏컷이나 조건을 보고 바로 문제를 풀 수 있는 로직을 주셔서 다른 모의고사를 풀 때 도움이 되었다. 정해진 시간에 피드백을 받으니 루틴이 되어 학습을 할 때 긴장감도 생기고 재수 할 때 혼자가 아닌, 같이 공부하는 느낌이 들어 좋았다.</v>
+        <v>매주 정해진 시간에 그 주 학습에 대한 피드백을 받고, 각 과목에 대한 진도에 맞추어 그 주 학습 방법을 조언해 주셔서 유용했다. 더 프리미엄 모의고사나 이투스 모의고사, 평가원 모의고사가 끝난 뒤, 작성한 오답노트를 통해 어떤 부분에서 문제를 틀렸는지 다각도로 분석해 주시고 그 유형에 대해 빨리 풀 수 있는 숏컷이나 조건을 보고 바로 문제를 풀 수 있는 로직을 주셔서 다른 모의고사를 풀 때 도움이 되었다. 정해진 시간에 피드백을 받으니 루틴이 되어 학습을 할 때 긴장감도 생기고 재수 할 때 혼자가 아닌, 같이 공부하는 느낌이 들어 좋았다.</v>
       </c>
       <c r="F215" t="str">
-        <v>재수하기 전, 인강을 들을 때 수강율에 집착하고 주변 친구들의 추천을 통해 강의만 마구잡이로 많이 들어 그 해 수능에서 그닥 효과를 보지 못한 경험이 있었다. 이투스 학원에서 제공한 인강 추천 및 수강 관리 시스템으로 나에게 맞는 인강 강사 선생님을 나보다 인강에 대해 잘 아시는 분이 추천해주시니 한 인강 선생님의 커리큘럼을 성실하게 수행해내었다. 또 주마다 수강율 체크로 내가 지금 그 주에 소홀히 하고 있는 과목을 파악하고 이에 맞추어 그 주 인강 계획을 자세하게 수정해주시니 내가 그에 들일 노력을 대신 해주셔서 시간이 절약되는 효과를 누렸다.</v>
+        <v>재수하기 전, 인강을 들을 때 수강율에 집착하고 주변 친구들의 추천을 통해 강의만 마구잡이로 많이 들어 그 해 수능에서 그닥 효과를 보지 못한 경험이 있었다. 이투스 학원에서 제공한 인강 추천 및 수강 관리 시스템으로 나에게 맞는 인강 강사 선생님을 나보다 인강에 대해 잘 아시는 분이 추천해주시니 한 인강 선생님의 커리큘럼을 성실하게 수행해내었다. 또 주마다 수강율 체크로 내가 지금 그 주에 소홀히 하고 있는 과목을 파악하고 이에 맞추어 그 주 인강 계획을 자세하게 수정해주시니 내가 그에 들일 노력을 대신 해 주셔서 시간이 절약되는 효과를 누렸다.</v>
       </c>
       <c r="G215" t="str">
         <v>현역 때, 독서실이나 스터디카페에서는 인강 시청을 위해 패드를 키고 공부를 하는 것이 아닌 패드로 유튜브를 보거나 소셜미디어 앱으로 노는 경향이 있었고 이로 인해 순공 시간이 확실히 떨어졌다. 강제성이 부족해 실패를 겪으니, 이투스 학원에서 제공해주는 감독 시스템으로 패드를 통해 딴 짓을 못하게 되니 순공 시간이 비약적으로 늘고 공부에만 오로지 집중할 수 있는 환경이 만들어졌다. 또 공부 시간에 잠이 와 졸거나 책상에서 쪽잠을 잘때 감독관 선생님이 와서 깨워주시니 순공 시간이 늘어나는 효과와 함께 최대한 졸음을 깨우기 위해 노력하고 긴장감을 가지는 습관을 들게 되었다. 이를 통해 수능에서 현역 때의 수능 보다 좋은 결과를 얻은 것 같아 이투스의 생활 관리 시스템이 유용했다고 생각한다.</v>
@@ -8200,10 +8200,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E216" t="str">
-        <v>수능 공부를 본격적으로 시작했을 때 고3이라 나름 정보 수집을 해도 공부를 어떻게 해야 하는지, 뭐가 중요한지 잘 모르는 상태였습니다. 상담을 받으면서 선생님께서 '이 과목은 공부 방향이 괜찮은 것 같다', '저 과목은 공부 방법을 이렇게 바꿔보면 좋을 것 같다' 이런 식으로 조언해주셔서 수능 공부 방향을 잡는데 큰 도움이 되었고,  또한 자잘한 팁을 주신 것도 유용했습니다.</v>
+        <v>수능 공부를 본격적으로 시작했을 때 고3이라 나름 정보 수집을 해도 공부를 어떻게 해야 하는지, 뭐가 중요한지 잘 모르는 상태였습니다. 상담을 받으면서 선생님께서 '이 과목은 공부 방향이 괜찮은 것 같다', '저 과목은 공부 방법을 이렇게 바꿔보면 좋을 것 같다' 이런 식으로 조언해 주셔서 수능 공부 방향을 잡는데 큰 도움이 되었고,  또한 자잘한 팁을 주신 것도 유용했습니다.</v>
       </c>
       <c r="F216" t="str">
-        <v>저는 인강을 들으면서도 내가 내 수준에 맞게 잘 듣고 있는 게 맞을까?라는 의문이 계속 들었습니다. 특히 국어와 수학이 약해서 고민도 많고 걱정도 많았었는데, 선생님께서 조언을 잘 해주셔서 제 커리에 맞게 차근차근 해 나갈 수 있었습니다.</v>
+        <v>저는 인강을 들으면서도 내가 내 수준에 맞게 잘 듣고 있는 게 맞을까?라는 의문이 계속 들었습니다. 특히 국어와 수학이 약해서 고민도 많고 걱정도 많았었는데, 선생님께서 조언을 잘 해 주셔서 제 커리에 맞게 차근차근 해 나갈 수 있었습니다.</v>
       </c>
       <c r="G216" t="str">
         <v>저는 휴대폰이 근처에 있으면 공부 효율이 현저히 떨어지는 스타일이라 일부러 휴대폰을 걷는 곳으로 학원을 선택했었습니다. 확실히 휴대폰이 없으니 공부에 집중이 더 잘 되고 성취감도 있어서 생활 관리에 유용했습니다.</v>
@@ -8212,7 +8212,7 @@
         <v>혼자 공부하다 보면 영어 단어 암기의 중요성을 간과하게 되는 느낌이 있습니다. 저도 독학을 시작한 후로 영어 단어 암기에 소홀했는데 이투스에서 매일 단어 시험지를 나누어 주니 억지로라도 했던 것이 도움이 되었습니다.</v>
       </c>
       <c r="I216" t="str">
-        <v>수능 준비하는 동안 대학 걱정에 많이 힘들었는데, 선생님들이 항상 친절하고 정감있게 대해주신 것이 기억에 많이 남습니다. 그때 조금이나마 마음의 안정을 얻을 수 있었습니다. 짧은 시간이었지만 정말 감사했습니다!</v>
+        <v>수능 준비하는 동안 대학 걱정에 많이 힘들었는데, 선생님들이 항상 친절하고 정감있게 대해 주신 것이 기억에 많이 남습니다. 그때 조금이나마 마음의 안정을 얻을 수 있었습니다. 짧은 시간이었지만 정말 감사했습니다!</v>
       </c>
       <c r="J216" t="str">
         <v>정기적인 시험으로 위치를 파악하고, 담임 선생님의 맞춤 관리 덕분에 흔들림 없이 스스로를 통제할 수 있었어요."</v>
@@ -8306,7 +8306,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E219" t="str">
-        <v>현재 내 학습 수준과 남은 시간과 시기 등의 상황을 고려하여 적절한 강의와 커리큘럼을 추천해 주셔서 학습 방향을 보다 명확하게 설정하여 불필요한 시간 낭비 없이 효율적으로 공부할 수 있게 되었고 또한 학습 상담 과정에서 세심하게 제 고민과 부족한 부분을 파악해주시고 현실적인 조언과 구체적인 학습 방법까지 제시해 주셔서 신뢰가 갔으며 동기부여에도 큰 도움이 되었습니다.</v>
+        <v>현재 내 학습 수준과 남은 시간과 시기 등의 상황을 고려하여 적절한 강의와 커리큘럼을 추천해 주셔서 학습 방향을 보다 명확하게 설정하여 불필요한 시간 낭비 없이 효율적으로 공부할 수 있게 되었고 또한 학습 상담 과정에서 세심하게 제 고민과 부족한 부분을 파악해 주시고 현실적인 조언과 구체적인 학습 방법까지 제시해 주셔서 신뢰가 갔으며 동기부여에도 큰 도움이 되었습니다.</v>
       </c>
       <c r="F219" t="str">
         <v>현재 내 학습 수준과 남은 시간 등을 고려하여 교재와 인강을 체계적으로 추천해 주셔서 무엇부터 어떻게 공부해야 할지 명확하게 알 수 있어 매우 유용했습니다. 특히 개인에게 맞는 강의와 교재를 연결해주어 학습 효율이 높아졌고 시행착오를 줄일 수 있었습니다.</v>
@@ -8341,7 +8341,7 @@
         <v>N수생</v>
       </c>
       <c r="E220" t="str">
-        <v>아침부터 밤까지 한 공간에서 오래 공부하는 과정이 쉽지 않았고, 중간에 지치고 힘들었던 시기도 있었습니다. 그럴 때마다 선생님께서 학생 한 명 한 명의 상태를 세심하게 살펴주시고 진로와 학습에 대한 현실적인 조언을 해주셔서 다시 중심을 잡을 수 있었습니다. 덕분에 흔들리는 시기를 잘 극복하며 끝까지 버틸 수 있었습니다.</v>
+        <v>아침부터 밤까지 한 공간에서 오래 공부하는 과정이 쉽지 않았고, 중간에 지치고 힘들었던 시기도 있었습니다. 그럴 때마다 선생님께서 학생 한 명 한 명의 상태를 세심하게 살펴주시고 진로와 학습에 대한 현실적인 조언을 해 주셔서 다시 중심을 잡을 수 있었습니다. 덕분에 흔들리는 시기를 잘 극복하며 끝까지 버틸 수 있었습니다.</v>
       </c>
       <c r="F220" t="str">
         <v>매주 작성한 플래너를 확인하는 시간을 가졌는데, 이 시간이 저에겐 유용했습니다. 플래너를 바탕으로 공부 내용과 시간 활용을 세밀하게 점검해 주셨고, 공부 방향과 속도가 나에게 적절한지도 함께 확인해 주셨습니다. 또한 교재와 인강을 상황에 맞게 추천해 주시고, 모의고사 분석을 통해 만약 반복되는 실수가 있다면 그것을 교정할 수 있도록 하는 구체적인 행동 지침을 제시해 주셔서 큰 도움이 되었습니다.</v>
@@ -8412,7 +8412,7 @@
         <v>N수생</v>
       </c>
       <c r="E222" t="str">
-        <v>매주 상담을 진행하여 공부상황을 체크해 주시고 시험을 보고 정신적으로 흔들릴때마다 멘탈을 잡아주시고 초반 학습방법에 대한 상담에서도 얻을 것이 많았습니다. 질문도 항상 친절하게 답변해주시고 마지막까지 쳐지지 않게 응원해주셨습니다.</v>
+        <v>매주 상담을 진행하여 공부상황을 체크해 주시고 시험을 보고 정신적으로 흔들릴때마다 멘탈을 잡아주시고 초반 학습방법에 대한 상담에서도 얻을 것이 많았습니다. 질문도 항상 친절하게 답변해 주시고 마지막까지 쳐지지 않게 응원해주셨습니다.</v>
       </c>
       <c r="F222" t="str">
         <v>매달 자신이 어떤 위치에 있는지 확인하면서 부족한 점이 어딘지 확인할 수 있었습니다. 성적표를 보고 상담을 통해 과목별 비중을 조절할 수 있었고 시험 중 어떤 부분에서 막혔는가에 따라 피드백을 진핼할 수 있었습니다</v>
@@ -8424,7 +8424,7 @@
         <v>모의고사는 수능장에서 일어날 수 있는 많은 상황에 대비할 수 있고 자신의 위치를 파악할 수 있는 가장 좋은 방법입니다. 컨디션이 좋든 나쁘든 매달 모의고사를 실시하여 다양한 경험을 할 수 있었습니다.</v>
       </c>
       <c r="I222" t="str">
-        <v>길어진 수험생 생활로 자존감도 떨어지고 항상 생각만 많아져서 고민만 하면서 무기력하게 생활했는데 선생님들이 잘 받아주셔서 무사히 완주한거 같습니다. 담임 선생님 항상 무기력한 학생이였는데 매번 친절하게 상담해주셔서 감사합니다🙂</v>
+        <v>길어진 수험생 생활로 자존감도 떨어지고 항상 생각만 많아져서 고민만 하면서 무기력하게 생활했는데 선생님들이 잘 받아주셔서 무사히 완주한거 같습니다. 담임 선생님 항상 무기력한 학생이였는데 매번 친절하게 상담해 주셔서 감사합니다🙂</v>
       </c>
       <c r="J222" t="str">
         <v>선생님의 세심한 진도 체크와 관리 덕분에 플래너를 꾸준히 채워가며, 매일 성실하게 공부하는 좋은 습관이 생겼어요.</v>
@@ -8461,7 +8461,7 @@
       <c r="I223" t="str" xml:space="preserve">
         <v xml:space="preserve">이투스247학원 선생님들께,_x000d_
 _x000d_
-항상 학생들을 위해 세심하게 지도해주시고, 힘들 때마다 따뜻한 조언과 격려를 아끼지 않으셔서 진심으로 감사드립니다. 덕분에 흔들릴 때마다 다시 마음을 다잡고 끝까지 포기하지 않을 수 있었습니다._x000d_
+항상 학생들을 위해 세심하게 지도해 주시고, 힘들 때마다 따뜻한 조언과 격려를 아끼지 않으셔서 진심으로 감사드립니다. 덕분에 흔들릴 때마다 다시 마음을 다잡고 끝까지 포기하지 않을 수 있었습니다._x000d_
 _x000d_
 단순히 공부만이 아니라 생활과 멘탈까지 챙겨주신 덕분에 더 성장할 수 있었고, 그 과정 하나하나가 큰 힘이 되었습니다. 선생님들의 노력과 응원은 오래도록 잊지 않겠습니다._x000d_
 _x000d_
@@ -8528,7 +8528,7 @@
       </c>
       <c r="F225" t="str" xml:space="preserve">
         <v xml:space="preserve">특히 수학 부분에서 원장 선생님께서_x000d_
-지금 제 수준과 시기에 풀어야하는 교재들과 괜찮은 사설 모의고사들을 추천해주신게 도움이 많이 되었습니다._x000d_
+지금 제 수준과 시기에 풀어야하는 교재들과 괜찮은 사설 모의고사들을 추천해 주신게 도움이 많이 되었습니다._x000d_
 얼마남지 않은 시기에 최고의 효율을 발휘해 예체능임에도 불구하고 2등급이라는 좋은 성적을 받을 수 있었습니다.</v>
       </c>
       <c r="G225" t="str">
@@ -8538,7 +8538,7 @@
         <v>3,6모의고사를 못 본 저한테는 실전경험이 절실히 필요했습니다. 이투스 모의고사를 통해 수능장과 비슷한 상황에서 연습을 충분히 할 수 있었고 막판에 성적이 오른 가장 큰 요인 중 하나였습니다</v>
       </c>
       <c r="I225" t="str">
-        <v>도와주신 선생님들께 정말정말 감사드립니다. 3,4개월이라는 짧은 시간만에 인서울이라는 너무 큰 선물을 받았습니다. 축하해주신 선생님들도 너무 감사드려요. 나중에 꼭 찾아뵙겠습니다.</v>
+        <v>도와주신 선생님들께 정말정말 감사드립니다. 3,4개월이라는 짧은 시간만에 인서울이라는 너무 큰 선물을 받았습니다. 축하해 주신 선생님들도 너무 감사드려요. 나중에 꼭 찾아뵙겠습니다.</v>
       </c>
       <c r="J225" t="str">
         <v>맞춤형 학습 전략으로 공부 효율을 높이고, 언제든 친절하게 고민을 상담해 주신 덕분에 편안하게 학습에 집중할 수 있었어요.</v>
@@ -8568,13 +8568,13 @@
       </c>
       <c r="G226" t="str" xml:space="preserve">
         <v xml:space="preserve">학원의 면학 분위기 조성을 위하여 매 공부 시간마다 선생님들께서 돌아다니시면서 자는 사람들을 깨우고 공부에 집중할 수 있도록 하셨습니다._x000d_
-또한 시끄러운 사람이 있어 선생님들께 이야기하면 바로 조치를 취해주셔서 편안하게 조용한 환경에서 공부를 할 수 있었습니다.</v>
+또한 시끄러운 사람이 있어 선생님들께 이야기하면 바로 조치를 취해 주셔서 편안하게 조용한 환경에서 공부를 할 수 있었습니다.</v>
       </c>
       <c r="H226" t="str">
         <v>대성 모의고사와 교육청 모의고사, 평가원 모의고사로는 실전 모의고사 연습이 부족했었는데 이투스 모의고사도 봄으로써 더 많은 연습을 할 수 있어서 좋았습니다. 다양한 문제와 친절한 해설을 보면서 더욱 모의고사 푸는 연습을 할 수 있어서 도움이 많이 되었습니다.</v>
       </c>
       <c r="I226" t="str" xml:space="preserve">
-        <v xml:space="preserve">아침마다 이름 불러주시며 밝게 인사해주시고 공부에 집중할 수 있도록 도와주셔서 감사합니다! 선생님들께서 학생 한명한명  도와주시고 신경써주신 덕분에 좋은 환경에서 열심히 공부할 수 있었습니다!!_x000d_
+        <v xml:space="preserve">아침마다 이름 불러주시며 밝게 인사해 주시고 공부에 집중할 수 있도록 도와주셔서 감사합니다! 선생님들께서 학생 한명한명  도와주시고 신경써주신 덕분에 좋은 환경에서 열심히 공부할 수 있었습니다!!_x000d_
 감사합니다</v>
       </c>
       <c r="J226" t="str">
@@ -8604,7 +8604,7 @@
         <v>현역 때는 혼자 공부할 때는 인강을 듣더라도 미루게 되어서 제대로 듣지 못하는 경우가 많았는데 선생님이 세세히 체크해 주셔서 완강할 수 있었습니다. 그리고 내가 부족한 부분에 대란 인강을 추천해 주셔서 등급 올릴 수 있었습니다.</v>
       </c>
       <c r="G227" t="str">
-        <v>쉬는 시간에 자더라도 쉬는 시간이 끝나면 선생님이 끝나는 시간에 맞춰 깨워주셔서 공부 시간을 놓칠 일이 없어 좋았습니다. 또한 면학 분위기에 대한 관리도 세심하게 해주셔서 집중해서 공부할 수 있었습니다.</v>
+        <v>쉬는 시간에 자더라도 쉬는 시간이 끝나면 선생님이 끝나는 시간에 맞춰 깨워주셔서 공부 시간을 놓칠 일이 없어 좋았습니다. 또한 면학 분위기에 대한 관리도 세심하게 해 주셔서 집중해서 공부할 수 있었습니다.</v>
       </c>
       <c r="H227" t="str">
         <v>항상 시험을 보면 떨었었는데 정기적으로 이투스 모의고사를 응시해서 실전 감각을 키우고 시험 시간에 시간 배분하는 연습을 할 수 있어 도움이 많이 됐습니다. 또한 모의고사를 볼 때도 선생님들이 꼼꼼하게 감독해 주셔서 실전과 같은 환경에서 볼 수 있어 좋았습니다.</v>
@@ -8668,7 +8668,7 @@
         <v>N수생</v>
       </c>
       <c r="E229" t="str">
-        <v>모의고사 보고 부족한점을 이야기 해주시고 저는 논술로 목표 하고 있어서 어느 과목을 올려서 최저 맞히는데 상담도 해주셨습니다. 그리고 저의 경우 국어보다는 수학 사탐 영어 위주로 공부 하라고 코팅도 해주셨습니다</v>
+        <v>모의고사 보고 부족한점을 이야기 해 주시고 저는 논술로 목표 하고 있어서 어느 과목을 올려서 최저 맞히는데 상담도 해주셨습니다. 그리고 저의 경우 국어보다는 수학 사탐 영어 위주로 공부 하라고 코팅도 해주셨습니다</v>
       </c>
       <c r="F229" t="str">
         <v>플래너도 내가 직접 쓰면서 어떤 공부가 부족한지 눈에 잘 들어왔습니다. 그리고 공부를 한 내용을 직접 쓰기때문에 밀린공부도 없었고 효율적으로 공부 하게 되었습니다. 영어단어도 매일 봐서 단어를 따로 외우지 않아도 됬습니다</v>
@@ -8715,7 +8715,7 @@
         <v>원래 영어 공부를 가장 싫어하기도 하고 가장 안해서 성적이 매우 좋지 않았는데 매일 매일 단어를 외우고 테스트까지 보다 보니까 강제로라도 영어 공부를 조금이나마 하게 되었던 것 같고 복습 테스트도 있어서 기억에 오래 남았던 것 같습니다</v>
       </c>
       <c r="I230" t="str">
-        <v>친절하게 대해주시고 상담도 열심히 해주시고 이런저런 일도 많아서 대학 입시라는게 정말 힘들다고 느꼈지만 선생님들이 도와주셔서 도움이 되는게 많았던 것 같습니다. 그리 길게 다니지는 않았지만 감사했습니다.</v>
+        <v>친절하게 대해 주시고 상담도 열심히 해 주시고 이런저런 일도 많아서 대학 입시라는게 정말 힘들다고 느꼈지만 선생님들이 도와주셔서 도움이 되는게 많았던 것 같습니다. 그리 길게 다니지는 않았지만 감사했습니다.</v>
       </c>
       <c r="J230" t="str">
         <v>생활 관리 시스템은 규칙적인 생활 습관을 유지하는 데 큰 도움이 되었어요.</v>
@@ -8855,7 +8855,7 @@
         <v>영어공부에 있어서 영단어 공부는 매우 필수적이지만 스스로 하기에 쉽지 않다고 생각합니다. 다른 공부보다 항상 후순위로 밀려 생각보다 시간을 내서 공부하기 힘들기 때문입니다. 영단어 테스트를 매일, 반복적으로 보기 때문에 많은 도움을 받았던 것 같습니다.</v>
       </c>
       <c r="I234" t="str">
-        <v>학원에 계시는 모든 분들 정말 진심으로 응원해주시고 관리해주신다는 걸  정말 많이 느꼈습니다. 가끔 쓴소리도 해주시지만 그것또한 다 잘되라고 하시는 거라는 걸 잘 알고 있습니다. 수험기간 동안 수고많이해주셔서 정말 감사했습니다.</v>
+        <v>학원에 계시는 모든 분들 정말 진심으로 응원해 주시고 관리해 주신다는 걸  정말 많이 느꼈습니다. 가끔 쓴소리도 해주시지만 그것또한 다 잘되라고 하시는 거라는 걸 잘 알고 있습니다. 수험기간 동안 수고많이해 주셔서 정말 감사했습니다.</v>
       </c>
       <c r="J234" t="str">
         <v>담임 선생님과 성적 고민을 부담 없이 나눌 수 있어 좋았고, 멘토 선생님과 얘기를 하며 학습 향상에 도움이 되었어요.</v>
@@ -8896,7 +8896,7 @@
         <v>또 하나 도움이 많이 되었던 부분은 매주 진행되는 영단어 테스트였습니다. 영어는 꾸준함이 가장 중요한 과목인데, 혼자 공부하다 보면 다른 과목에 밀려 소홀해지기 쉬운 과목이기도 합니다. 그런데 매주 정기적으로 영단어 테스트가 있다 보니 영어를 완전히 놓지 않고 계속 붙잡고 갈 수 있었습니다. 이런 반복적인 관리 덕분에 자연스럽게 어휘력이 쌓였고, 영어 공부의 흐름을 끊지 않고 유지할 수 있었습니다. 단순히 단어를 외우는 것에서 끝나는 것이 아니라, 꾸준히 점검받는 과정이 있어서 더 책임감을 가지고 공부하게 된 것도 큰 도움이 되었습니다. 실제로 2026 수능 영어가 체감상 어려웠음에도 불구하고 87점을 받을 수 있었고, 정시에서도 영어 때문에 점수가 크게 깎이지 않았습니다. 이런 결과를 얻을 수 있었던 데에는 매주 진행되는 영단어 테스트를 통해 영어를 꾸준히 유지할 수 있었던 영향이 크다고 생각합니다.</v>
       </c>
       <c r="I235" t="str">
-        <v>마지막으로 영어 선생님과 실장님께 감사 인사를 드리고 싶습니다. 수험 생활을 하다 보면 예민해지고 작은 일에도 흔들리는 순간들이 많았는데, 그럴 때마다 항상 다정하게 대해주시고 질문에도 친절하게 답해주셔서 큰 힘이 되었습니다. 특히 ‘할 수 있다’고 계속해서 격려해주신 말들이 지칠 때마다 다시 버틸 수 있게 해주는 원동력이 되었습니다. 또 항상 밝게 인사해주시고 먼저 따뜻하게 말 걸어주셔서 학원에 오는 것 자체가 덜 부담스럽게 느껴졌던 것 같습니다. 사소해 보일 수 있지만 그런 분위기가 하루하루를 버티는 데 정말 큰 힘이 되었습니다. 중간중간 챙겨주신 맛있는 간식들도 큰 위로가 되었고, 덕분에 힘든 시기에도 포기하지 않고 끝까지 버틸 수 있었습니다. 1년이라는 시간을 무사히 버틸 수 있었던 데에는 선생님과 실장님의 도움이 정말 컸다고 생각합니다. 진심으로 감사드립니다.</v>
+        <v>마지막으로 영어 선생님과 실장님께 감사 인사를 드리고 싶습니다. 수험 생활을 하다 보면 예민해지고 작은 일에도 흔들리는 순간들이 많았는데, 그럴 때마다 항상 다정하게 대해 주시고 질문에도 친절하게 답해 주셔서 큰 힘이 되었습니다. 특히 ‘할 수 있다’고 계속해서 격려해 주신 말들이 지칠 때마다 다시 버틸 수 있게 해주는 원동력이 되었습니다. 또 항상 밝게 인사해 주시고 먼저 따뜻하게 말 걸어주셔서 학원에 오는 것 자체가 덜 부담스럽게 느껴졌던 것 같습니다. 사소해 보일 수 있지만 그런 분위기가 하루하루를 버티는 데 정말 큰 힘이 되었습니다. 중간중간 챙겨주신 맛있는 간식들도 큰 위로가 되었고, 덕분에 힘든 시기에도 포기하지 않고 끝까지 버틸 수 있었습니다. 1년이라는 시간을 무사히 버틸 수 있었던 데에는 선생님과 실장님의 도움이 정말 컸다고 생각합니다. 진심으로 감사드립니다.</v>
       </c>
       <c r="J235" t="str">
         <v>담임 선생님께서 일상의 대화로 힘이 되어주시고, 공부에 집중할 수 있도록 세심하게 도와주셔서 큰 도움이 되었어요.</v>
@@ -8919,7 +8919,7 @@
         <v>N수생</v>
       </c>
       <c r="E236" t="str">
-        <v>입시 정보를 평소에 확인하기 위해선 졸업한 학교에 가서 진로 선생님과 상담을 하거나 인터넷에서 번거롭게 일일히 찾아봐야 했는데, 학원에 입시 상담을 신청하면 친절하고 상세하게 설명해주셔서 시간낭비 없이 공부에 집중할 수 있었습니다.</v>
+        <v>입시 정보를 평소에 확인하기 위해선 졸업한 학교에 가서 진로 선생님과 상담을 하거나 인터넷에서 번거롭게 일일히 찾아봐야 했는데, 학원에 입시 상담을 신청하면 친절하고 상세하게 설명해 주셔서 시간낭비 없이 공부에 집중할 수 있었습니다.</v>
       </c>
       <c r="F236" t="str">
         <v>아무래도 인강 Q&amp;A 시스템을 이용하려면 답변을 받는데 시간이 꽤 많이 소요돼서 궁금한 것을 바로바로 알 순 없는데, 1:1 로 질문을 하면 인강 Q&amp;A 시스템을 활용하는 것 보다 상대적으로 매우 빠르게 답변을 들을 수 있어 쾌적했습니다.</v>
@@ -9044,7 +9044,7 @@
         <v>매주 목요일마다 정기적으로 테스트를 보면서 암기한 내용을 점검할 수 있어 좋았습니다. 시험이 있다는 사실이 동기부여가 되어 꾸준히 단어를 외우게 되었고 그 과정에서 평소에도 자연스럽게 단어를 반복해서 익히는 습관이 생겼습니다.</v>
       </c>
       <c r="I239" t="str">
-        <v>항상 신경 써주시고 도움 주신 선생님들께 감사드립니다. 학습 관리부터 생활 전반까지 세심하게 챙겨주시고 힘들 때마다 진심 어린 조언과 격려를 해주셔서 끝까지 포기하지 않고 버틸 수 있었습니다. 덕분에 공부 습관을 잡을 수 있었고 올바른 방향으로 나아갈 수 있었다고 생각합니다. 정말 감사합니다.</v>
+        <v>항상 신경 써주시고 도움 주신 선생님들께 감사드립니다. 학습 관리부터 생활 전반까지 세심하게 챙겨주시고 힘들 때마다 진심 어린 조언과 격려를 해 주셔서 끝까지 포기하지 않고 버틸 수 있었습니다. 덕분에 공부 습관을 잡을 수 있었고 올바른 방향으로 나아갈 수 있었다고 생각합니다. 정말 감사합니다.</v>
       </c>
       <c r="J239" t="str">
         <v>선생님께서 효율적이고 저에게 맞는 시간표를 짤 수 있게 도움을 많이 주셨어요.</v>
@@ -9140,7 +9140,7 @@
         <v>N수생</v>
       </c>
       <c r="E242" t="str">
-        <v>특정 과목에서 어려운 부분이 있으면 그 부분을 어떻게 해야 잘 풀어낼 수 있는지에 대해 아이디어를 주셔서 좋았습니다. 또한 주기적으로 풀고 있는 교재들을 점검해 주시고 다음으로 풀 교재들을 추천해주신 것도 도움이 많이 되었습니다.</v>
+        <v>특정 과목에서 어려운 부분이 있으면 그 부분을 어떻게 해야 잘 풀어낼 수 있는지에 대해 아이디어를 주셔서 좋았습니다. 또한 주기적으로 풀고 있는 교재들을 점검해 주시고 다음으로 풀 교재들을 추천해 주신 것도 도움이 많이 되었습니다.</v>
       </c>
       <c r="F242" t="str">
         <v>어떤 부분이 어려운지를 이야기 하면 멘토분들께서 본인이 풀어보셨던 문제집을 추천해주시기도 하는데 저는 이렇게 접한 교재로 도움을 정말 많이 받았습니다! 그리고 현재 풀고 있는 문제집을 말씀 드리면 어느정도로 교재의 장단점이나 어느정도로 학습해야 하는지도 알려주시는 경우가 있어서 좋았어요</v>
@@ -9152,7 +9152,7 @@
         <v>모든 사이트의 패스를 다 사려면 금액이 상당히 많이 드는데 이투스는 패스까지 무료로 준다는 게 금전적으로 메리트가 크다고 생각합니다! 저는 사회탐구를 이지영 선생님의 커리를 들었기 때문에 이투스 패스를 잘 활용했던 것 같습니다</v>
       </c>
       <c r="I242" t="str">
-        <v>항상 친절하게 관리해 주시고 상담도 해주시고 수업도 해주셔서 감사합니다. 상담하면서 심리적인 스트레스들을 해소할 수 있었던 것 같아서 좋았아요. 덕분에 1년 동안 편안한 환경에서 공부하여 대학에 올 수 있었습니다!</v>
+        <v>항상 친절하게 관리해 주시고 상담도 해 주시고 수업도 해 주셔서 감사합니다. 상담하면서 심리적인 스트레스들을 해소할 수 있었던 것 같아서 좋았아요. 덕분에 1년 동안 편안한 환경에서 공부하여 대학에 올 수 있었습니다!</v>
       </c>
       <c r="J242" t="str">
         <v>플래너와 휴대폰 관리 덕분에 과목 편식 없이 집중했고, 깊이 있는 상담이 큰 도움이 됐어요.</v>
@@ -9187,10 +9187,10 @@
         <v>저는 일일테스트는 딱히 없었고 오후에 진행하는 영어 듣기가 마음에 들었습니다. 딱 실제 영어 듣기를 하는 시간과 같은 시간에 수험생들이 중요치 않게 생각하여 만만하게 보는 영어 듣기를 진행해서 실제 시험장에서 듣기를 할 때 떨림이 감소하는 효과가 있었습니다.</v>
       </c>
       <c r="I243" t="str">
-        <v>약 6개월간 기초부터 심화까지 학습에 도움을 주시고 또 학습적인 측면 뿐만 아니라, 생활적인 부분에서도 많은 케어를 해주셔서 정말 감사드립니다. N수는 겨울 ~ 여름까지 얼마나 기초를 잘 닦아 놓느냐가 중요한데 이를 잘 할 수 있게 해주셔서 감사드립니다.</v>
+        <v>약 6개월간 기초부터 심화까지 학습에 도움을 주시고 또 학습적인 측면 뿐만 아니라, 생활적인 부분에서도 많은 케어를 해 주셔서 정말 감사드립니다. N수는 겨울 ~ 여름까지 얼마나 기초를 잘 닦아 놓느냐가 중요한데 이를 잘 할 수 있게 해 주셔서 감사드립니다.</v>
       </c>
       <c r="J243" t="str">
-        <v>성적이 나왔을 때 항상 같이 상담하며 멘탈을 잡아주셨고, 힘들 때나 지칠 때 학생들에게 깊게 공감해주시면서 응원해주셨어요.</v>
+        <v>성적이 나왔을 때 항상 같이 상담하며 멘탈을 잡아주셨고, 힘들 때나 지칠 때 학생들에게 깊게 공감해주시면서 응원해 주셨어요.</v>
       </c>
       <c r="K243" t="str">
         <v/>
@@ -9222,7 +9222,7 @@
         <v>아침마다 단어시험을 보는 시스템이 있어 꾸준히 어휘를 암기하는 데 큰 도움이 되었습니다. 반복적으로 점검할 수 있어 기억에 오래 남았고, 자연스럽게 영어 실력 향상에도 긍정적인 영향을 주었습니다.</v>
       </c>
       <c r="I244" t="str">
-        <v>선생님들께서 항상 친절하게 대해주시고 질문에도 성실히 답해 주셔서 좋았습니다. 학생 한 명 한 명을 신경 써 주시는 모습에서 책임감이 느껴졌고, 덕분에 더 열심히 공부할 수 있었습니다.</v>
+        <v>선생님들께서 항상 친절하게 대해 주시고 질문에도 성실히 답해 주셔서 좋았습니다. 학생 한 명 한 명을 신경 써 주시는 모습에서 책임감이 느껴졌고, 덕분에 더 열심히 공부할 수 있었습니다.</v>
       </c>
       <c r="J244" t="str">
         <v>학원의 생활 관리 시스템은 규칙적인 생활 습관을 형성하는 데 큰 도움이 되었어요.</v>
@@ -9257,13 +9257,13 @@
         <v>모의고사를 매월 보면서 저의 실력을 측정하는 것은 물론이고 실전 연습과 경험을 정말 많이 할 수 있었습니다. 특히 모의고사 전날이 정말 수능 전날인 것처럼 준비하고, 당일 아침부터 시험이 끝날 때까지의 시간을 고스란히 느끼면서 저만의 리듬과 루틴을 만들어 나갔던 것이 큰 도움이 되었습니다.</v>
       </c>
       <c r="I245" t="str" xml:space="preserve">
-        <v xml:space="preserve">우리 원장님 언제나 최대한 제가 원하는 거 할 수 있도록 자유롭게 공부할 수 있도록 편하게 해주신 점 감사드리고요. 저의 학습에 큰 도움을 주신 조교 선생님들께도 감사의 인사를 전합니다. 언젠가는 제가 저 자리에서 다른 학생들에게 제가 몸소 체득한 노하우를 전부 주고 싶다는 생각을 많이 했었는데, 이렇게 대치동에서 조교까지 하면서 지내는 지금의 시간이 꿈 같이 느껴지기만 합니다._x000d_
+        <v xml:space="preserve">우리 원장님 언제나 최대한 제가 원하는 거 할 수 있도록 자유롭게 공부할 수 있도록 편하게 해 주신 점 감사드리고요. 저의 학습에 큰 도움을 주신 조교 선생님들께도 감사의 인사를 전합니다. 언젠가는 제가 저 자리에서 다른 학생들에게 제가 몸소 체득한 노하우를 전부 주고 싶다는 생각을 많이 했었는데, 이렇게 대치동에서 조교까지 하면서 지내는 지금의 시간이 꿈 같이 느껴지기만 합니다._x000d_
 특히 저의 루틴을 유지할 수 있도록 많은 도움을 주시고 살펴주신 실장님께도 감사의 인사를 전합니다. 저의 요구사항이 참 많았었는데, 다 귀기울여 들어주셔서 참 감사했습니다._x000d_
 재수를 하는 기간 동안에 화창한 날도, 어두칙칙한 날도 있었습니다. 뭐든 이룰 수 있을 것 같은 날이 있었고, 모든 걸 놓아버리고 싶은 순간도 있었습니다. 돌이켜보면 제가 그 시간을 잘 지나올 수 있었던 것은 제 곁에서 묵묵히 도움을 주셨던, 저를 스쳐간 수많은 인연들 덕분이라는 생각이 듭니다. 정말 감사합니다._x000d_
 한 번 찾아뵙고 인사 드리겠습니다. 이만 줄입니다.</v>
       </c>
       <c r="J245" t="str">
-        <v>주단위로 하루에 무엇을 얼만큼 공부할지 계획을 같이 세우고 피드백해주셔서 고르게 공부할 수 있었어요.</v>
+        <v>주단위로 하루에 무엇을 얼만큼 공부할지 계획을 같이 세우고 피드백해 주셔서 고르게 공부할 수 있었어요.</v>
       </c>
       <c r="K245" t="str">
         <v/>
@@ -9318,22 +9318,22 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E247" t="str">
-        <v>각 과목별로 코칭을 받을 수 있어서 너무 좋았어요. 학습 상담을 통해 과목별로 제가 부족한 부분과 취약한 부분을 잘 보완할 수 있었어요. 또한 부족한 점을 베꿀 수 있는 자세한 대안까지 제안해주신 덕에 떨어졌던 자신감을 얻을 수 있었던 기회이기도 했습니다.</v>
+        <v>각 과목별로 코칭을 받을 수 있어서 너무 좋았어요. 학습 상담을 통해 과목별로 제가 부족한 부분과 취약한 부분을 잘 보완할 수 있었어요. 또한 부족한 점을 베꿀 수 있는 자세한 대안까지 제안해 주신 덕에 떨어졌던 자신감을 얻을 수 있었던 기회이기도 했습니다.</v>
       </c>
       <c r="F247" t="str">
         <v>공부를 어디서부터 어떻게 시작해야되고 계획해야되는지 막막한 저에게 공부할 큰 틀을 제안해주고 계획을 세우는 방법을 알려주는 이 시스템이 정날 유용했습니다. 제가 계획을 세우면 선생님께서 보고 피드백을 주셨기 때문에 더 효율적이고 도움이 되는 공부 계획을 세우고 실천할 수 있었습니다.</v>
       </c>
       <c r="G247" t="str">
-        <v>앉아서 공부하면 잠이 올 때가 정말 많은데 복도에서 공부할 수 있는 자리도 마련되어있고 그 외에 공부할 수 있는 공간도 엄청 다양해서 좋았습니다. 집중이 안될때 환경을 바꾸면서 공부하니 더 효율적으로 공부할 수 있었습니다. 또한 각 공간마다 감독도 잘 해주셔서 쾌적한 환경에서 공부에 집중할 수 있었어요.</v>
+        <v>앉아서 공부하면 잠이 올 때가 정말 많은데 복도에서 공부할 수 있는 자리도 마련되어있고 그 외에 공부할 수 있는 공간도 엄청 다양해서 좋았습니다. 집중이 안될때 환경을 바꾸면서 공부하니 더 효율적으로 공부할 수 있었습니다. 또한 각 공간마다 감독도 잘 해 주셔서 쾌적한 환경에서 공부에 집중할 수 있었어요.</v>
       </c>
       <c r="H247" t="str">
         <v>수능이 다가올수록 모의고사가 정말 중요한데 이투스 모의고사를 볼 수 있어서 정말 좋았어요. 이 그덕분에 감을 잃지않고 가져갈 수 있었고 시험을 보는 중에 내가 가져가야할 습관과 태도를 돌아보고 고치는 기회를 얻을 수 있었습니다.</v>
       </c>
       <c r="I247" t="str">
-        <v>생활과 학습 면에서 잘 케어해주셔서 정말 감사해요. 제가 이투스247학원에 있는 동안 혼자서 힘든 일이 정말 많았지만 선생님들께서 적극적으로 저에게 임해주셔서 저도 다시 힘내서 공부할 수 있었던 것 같습니다. 감사합니다</v>
+        <v>생활과 학습 면에서 잘 케어해 주셔서 정말 감사해요. 제가 이투스247학원에 있는 동안 혼자서 힘든 일이 정말 많았지만 선생님들께서 적극적으로 저에게 임해 주셔서 저도 다시 힘내서 공부할 수 있었던 것 같습니다. 감사합니다</v>
       </c>
       <c r="J247" t="str">
-        <v>학습에 집중할 수 있도록 선생님이 과목별로 상담도 해주시고, 플래너 작성한 것도 다시 점검해 주셔서 도움이 많이 됐어요!</v>
+        <v>학습에 집중할 수 있도록 선생님이 과목별로 상담도 해 주시고, 플래너 작성한 것도 다시 점검해 주셔서 도움이 많이 됐어요!</v>
       </c>
       <c r="K247" t="str">
         <v/>
@@ -9365,7 +9365,7 @@
         <v>인강사이트를 결제하는데에 꽤 부담이 되는 금액이 필요한데, 이투스를 사용할 수 있어 좋았다. 나는 타 인강사이트 하나와 이투스를 사용해 독학재수 내내 공부했다. 가끔 나눠주신 이투스 인강강사의 교재도 도움이 되었다.</v>
       </c>
       <c r="I248" t="str">
-        <v>학원의 면학 분위기와 따뜻한 관심 덕분에 이투스에서 두번째 수능을 마무리할 수 있었습니다. 재원기간동안 매주 상담을 해주신 담임 선생님, 아침마다 인사해주시던 선생님들, 졸 때마다 깨워주신 선생님 감사합니다.</v>
+        <v>학원의 면학 분위기와 따뜻한 관심 덕분에 이투스에서 두번째 수능을 마무리할 수 있었습니다. 재원기간동안 매주 상담을 해 주신 담임 선생님, 아침마다 인사해주시던 선생님들, 졸 때마다 깨워주신 선생님 감사합니다.</v>
       </c>
       <c r="J248" t="str">
         <v>조용하고 긴장감 있는 분위기 속에서 졸음 관리까지 확실히 받아, 장시간 안정적인 페이스로 공부에 온전히 집중할 수 있었어요.</v>
@@ -9391,7 +9391,7 @@
         <v>주기적인 학습 상담을 통해 주어진 시간동안 적어도 이정도 이상은 학습해야겠다는 기준이 생겼고 그에 맞추어 스스로 계획을 세워 차분하게 공부할 수 있었습니다. 진도 뿐만 아니라 중간중간 힘들어서 늦장을 부리고 싶을 때도 있었는데 이를 학습 상담을 통해 얻은 동기부여를 바탕으로 이겨낼 수 있었습니다.</v>
       </c>
       <c r="F249" t="str">
-        <v>스스로 문제를 풀다가 이해가 안되거나 문학 같은 경우, 인강을 통해 알고있던 내용과 다른 해석이 해설지에 적혀있는 경우엔 당황을 할 때가 있었는데 이러한 부분을 모아두었다가 1:1 질의응답을 통해 해결할 수 있어서 좋았습니다. 이해도 잘 되도록 설명해주셨어요.</v>
+        <v>스스로 문제를 풀다가 이해가 안되거나 문학 같은 경우, 인강을 통해 알고있던 내용과 다른 해석이 해설지에 적혀있는 경우엔 당황을 할 때가 있었는데 이러한 부분을 모아두었다가 1:1 질의응답을 통해 해결할 수 있어서 좋았습니다. 이해도 잘 되도록 설명해 주셨어요.</v>
       </c>
       <c r="G249" t="str">
         <v>사실 공부할 때 전자기기가 집중력에 가장 큰 영향을 미친다고 생각하는 입장인데, 아침에 등원을 하여 핸드폰을 제출하고 나면 끝나고 집에 갈 때까지 핸드폰에 대한 생각이 들지 않고 잊은 채로 공부만 바라볼 수 있어서 너무 좋았습니다. 특히 이 점은 집에서는 통제되기 힘든 부분이라고 생각되어 가장 좋았습니다.</v>
@@ -9435,7 +9435,7 @@
         <v>매일 진행되는 영단어 테스트가 큰 도움이 되었습니다. 원래 영어 실력이 나쁘지 않은 편이었지만, 꾸준히 영단어를 반복해서 학습하도록 관리해 주셔서 자연스럽게 어휘력이 더 강화되었습니다. 덕분에 따로 영어 공부에 많은 시간을 투자하지 않아도 안정적으로 좋은 성적을 유지할 수 있었습니다.</v>
       </c>
       <c r="I250" t="str">
-        <v>선생님들 덕분에 흐트러지지 않고 끝까지 체계적으로 준비하여 입시를 잘 마무리할 수 있었습니다! 항상 응원해주신 EM반 담임 선생님께 특히나 더 감사드립니다 안성이투스에서 공부하면서 정말정말 힘이 많이 되었습니다 감사합니다</v>
+        <v>선생님들 덕분에 흐트러지지 않고 끝까지 체계적으로 준비하여 입시를 잘 마무리할 수 있었습니다! 항상 응원해 주신 EM반 담임 선생님께 특히나 더 감사드립니다 안성이투스에서 공부하면서 정말정말 힘이 많이 되었습니다 감사합니다</v>
       </c>
       <c r="J250" t="str">
         <v>수능을 앞두고 상담을 통해 긴장을 덜고, 모의고사와 학습 조언으로 실전 감각을 키웠어요.</v>
@@ -9493,7 +9493,7 @@
         <v>N수생</v>
       </c>
       <c r="E252" t="str">
-        <v>300일 넘는 시간동안 7시 기상 1시 수면 생활을 하면서 재수 생활을 하면서 정신적으로 많이 무너질 뻔한 적이 많았다. 2 반복된 삶, 성적 압박감, 놀고 싶은 욕구를 통제해야 하는 것은 20살의 나에게 고되고 벅찼다. 때로는 무너질 때도 있었고, 밖으로 탈출하고 싶었을 때도 많았다. 그럴 때마다 원장님, 부원장님께서 내 힘든 사연에 대해 공감해주시고, 이해해주시고, 미래를 바라보는 올바른 방향으로 내 시각을 잡아주셨다. 그 덕분에 장기간 동안 크게 무너지지 않고 재수 생활을 할 수 있었다.</v>
+        <v>300일 넘는 시간동안 7시 기상 1시 수면 생활을 하면서 재수 생활을 하면서 정신적으로 많이 무너질 뻔한 적이 많았다. 2 반복된 삶, 성적 압박감, 놀고 싶은 욕구를 통제해야 하는 것은 20살의 나에게 고되고 벅찼다. 때로는 무너질 때도 있었고, 밖으로 탈출하고 싶었을 때도 많았다. 그럴 때마다 원장님, 부원장님께서 내 힘든 사연에 대해 공감해 주시고, 이해해 주시고, 미래를 바라보는 올바른 방향으로 내 시각을 잡아주셨다. 그 덕분에 장기간 동안 크게 무너지지 않고 재수 생활을 할 수 있었다.</v>
       </c>
       <c r="F252" t="str">
         <v>재수하는 학생이 잘못된 방향으로 공부하고, 수면의 통제가 스스로 되지 않는다면 실력의 발전을 기대할 수 없다. 그렇기에 학생 스스로가 목표를 계획하고, 스스로를 통제하는 것이 재수에서 가장 중요한 요소이다. 하루, 1주, 한 달의 목표를 수립하는 것을 도와주시고, 성적 관리, 국어, 영어, 수학 하프 모의고사 배부, 심지어 수면 관리까지, 수많은 관리를 받으면서 이투스 247 노량진에서 공부할 수 있었고, 이는 나를 재수 성공으로 이끈 큰 도움이었다.</v>
@@ -9551,9 +9551,9 @@
 또한 정해진 분량을 꾸준히 암기해야 한다는 점이 학습 습관 형성에도 긍정적인 영향을 주었습니다. 매일 일정량의 단어를 학습하고 점검하는 과정이 반복되면서 영어 공부에 대한 부담이 줄어들고, 점차 익숙해질 수 있었습니다.</v>
       </c>
       <c r="I253" t="str" xml:space="preserve">
-        <v xml:space="preserve">재수 기간 동안 항상 옆에서 지도해주시고 응원해주신 선생님들께 진심으로 감사드립니다._x000d_
-공부뿐만 아니라 학습 방향과 생활 습관까지 세심하게 신경 써 주신 덕분에 흔들리지 않고 꾸준히 노력할 수 있었습니다. 힘들고 지칠 때마다 해주신 조언과 격려가 큰 힘이 되었고, 덕분에 끝까지 포기하지 않고 나아갈 수 있었습니다._x000d_
-또한 학생 한 명 한 명을 진심으로 생각해주시고, 부족한 부분을 채워주기 위해 노력해주신 점에 깊이 감사드립니다. 선생님들 덕분에 단순한 성적 향상을 넘어서, 스스로 공부하는 방법과 태도를 배울 수 있었습니다._x000d_
+        <v xml:space="preserve">재수 기간 동안 항상 옆에서 지도해 주시고 응원해 주신 선생님들께 진심으로 감사드립니다._x000d_
+공부뿐만 아니라 학습 방향과 생활 습관까지 세심하게 신경 써 주신 덕분에 흔들리지 않고 꾸준히 노력할 수 있었습니다. 힘들고 지칠 때마다 해 주신 조언과 격려가 큰 힘이 되었고, 덕분에 끝까지 포기하지 않고 나아갈 수 있었습니다._x000d_
+또한 학생 한 명 한 명을 진심으로 생각해 주시고, 부족한 부분을 채워주기 위해 노력해 주신 점에 깊이 감사드립니다. 선생님들 덕분에 단순한 성적 향상을 넘어서, 스스로 공부하는 방법과 태도를 배울 수 있었습니다._x000d_
 앞으로도 선생님들께 배운 점을 바탕으로 더 노력하는 모습 보여드리겠습니다. 다시 한 번 진심으로 감사드립니다</v>
       </c>
       <c r="J253" t="str">
@@ -9580,7 +9580,7 @@
         <v>학원 생활 중 가장 만족스러웠던 부분은 체계적인 학습 관리 시스템이었습니다. 매일 정해진 스케줄에 따라 공부하며 흐트러지기 쉬운 생활 습관을 바로잡을 수 있었고, 특히 취약했던 과목의 오답 원인을 철저히 분석해 주는 코칭 덕분에 실질적인 성적 향상을 경험했습니다. 철저한 면학 분위기 속에서 스스로의 한계를 극복하며 끝까지 완주할 수 있는 힘을 얻었습니다.</v>
       </c>
       <c r="F254" t="str">
-        <v>일대일 질의응답 시간은 단순히 모르는 문제를 해결하는 것을 넘어, 제 사고의 논리적 허점을 정확히 파악할 수 있는 소중한 기회였습니다. 대규모 강의에서는 해결하기 어려운 개인적인 궁금증을 눈높이에 맞춰 설명해주셔서 개념을 더욱 입체적으로 이해할 수 있었습니다. 특히 제가 작성한 풀이 과정을 함께 검토하며 비효율적인 습관을 교정해 주신 덕분에 문제 접근 방식 자체가 훨씬 정교해졌고, 이는 실전에서의 자신감으로 이어졌습니다. 조급함을 덜고 학습의 본질에 집중할 수 있었던 가장 만족스러운 시간이었습니다.</v>
+        <v>일대일 질의응답 시간은 단순히 모르는 문제를 해결하는 것을 넘어, 제 사고의 논리적 허점을 정확히 파악할 수 있는 소중한 기회였습니다. 대규모 강의에서는 해결하기 어려운 개인적인 궁금증을 눈높이에 맞춰 설명해 주셔서 개념을 더욱 입체적으로 이해할 수 있었습니다. 특히 제가 작성한 풀이 과정을 함께 검토하며 비효율적인 습관을 교정해 주신 덕분에 문제 접근 방식 자체가 훨씬 정교해졌고, 이는 실전에서의 자신감으로 이어졌습니다. 조급함을 덜고 학습의 본질에 집중할 수 있었던 가장 만족스러운 시간이었습니다.</v>
       </c>
       <c r="G254" t="str">
         <v>학원의 강력한 와이파이 방화벽은 학습 몰입도를 최상으로 유지하는 데 결정적인 역할을 했습니다. 공부하는 도중 나도 모르게 SNS나 오락성 사이트에 접속하려는 유혹을 원천적으로 차단해 주어, 오로지 학습에만 전념할 수 있는 강제성을 부여해 주었습니다. 덕분에 스마트폰이나 태블릿을 활용하면서도 학습 도구로서의 기능에만 집중할 수 있었고, 불필요한 데이터 낭비나 집중력 분산을 막아주어 순수 공부 시간을 확보하는 데 큰 도움이 되었습니다. 스스로 통제하기 어려운 디지털 유혹으로부터 자유로워져 마음 편히 공부에만 몰두할 수 있었던 점이 정말 만족스러웠습니다.</v>
@@ -9594,7 +9594,7 @@
 수업 시간마다 열정적으로 핵심을 짚어주시고, 질문 하나하나에도 귀 기울여 주시며 함께 고민해 주셨던 모습들이 큰 힘이 되었습니다. 때로는 엄격한 가르침으로 중심을 잡아주시고, 때로는 따뜻한 조언으로 불안한 마음을 다독여 주신 선생님들의 헌신 덕분에 성적 그 이상의 소중한 배움을 얻었습니다. 가르쳐 주신 가르침 잊지 않고, 사회에서도 부끄럽지 않은 제자가 되도록 노력하겠습니다. 그동안 정말 감사했습니다.</v>
       </c>
       <c r="J254" t="str">
-        <v>선생님들께서 학생 한 명 한 명 세심하게 신경 써주시면서 학습과 멘탈을 챙겨주셔서 좋은 방향으로 나아갈 수 있었어요.</v>
+        <v>선생님들께서 학생 한 명 한 명 세심하게 신경 써 주시면서 학습과 멘탈을 챙겨주셔서 좋은 방향으로 나아갈 수 있었어요.</v>
       </c>
       <c r="K254" t="str">
         <v/>
@@ -9617,7 +9617,7 @@
         <v>모르는 문제가 생겼을때 거의 항상 조교선생님이 학원에 계셔서 질문하기 수월했고 현재 모의고사 성적과 내 목표대학에 맞춰서 계획을 체크해 주시고 그에 따른 피드백을 알려주셔서 유용했다. 또한 내가 어떤 부분이 부족하고 어떤 문제집을 풀면서 보완하면 좋을지도 구체적으로 알려주셔서 좋았다.</v>
       </c>
       <c r="F255" t="str">
-        <v>인강만 보고는 해결할 수 없었던 문제들을 직접 질문함으로써 내가 몰랐던 부분을 정확히 해결하고 나에게 맞는 인강선생님을 추천해주셨다. 또한 난이도 높은 문제들을 내 수준에 맞게 설명해주셔서 유용했다.</v>
+        <v>인강만 보고는 해결할 수 없었던 문제들을 직접 질문함으로써 내가 몰랐던 부분을 정확히 해결하고 나에게 맞는 인강선생님을 추천해주셨다. 또한 난이도 높은 문제들을 내 수준에 맞게 설명해 주셔서 유용했다.</v>
       </c>
       <c r="G255" t="str">
         <v>평소 아침잠이 많아 수능패턴에 몸을 맞추는것이 많이 힘들었는데 아침에 이투스학원에서 잘때마다 깨워주셔서 아침잠을 강제로 줄이고 몸을 수능패턴에 맞출 수 있었다. 또한 점심시간과 저녁시간도 수능에 맞춰져서 수능때 불편함을 느끼지 않았다.</v>
@@ -9626,7 +9626,7 @@
         <v>재수생이다보니 영어단어를 외울 시간이 부족했고 영어에 시간투자를 하는것이 아깝다고 생각해서 영어를 다른 과목에 비해 덜 공부했었는데 단어시험은 매일 보다보니 어쩔 수 없이 공부했고 그에 따라 매일 일정량씩 단어를 외워야 되서 영어에 많은 도움이 되었다.</v>
       </c>
       <c r="I255" t="str">
-        <v>1년 동안 재수하는 것이 너무 힘들것이라고 생각했었는데 이투스학원 선생님들이 계속 신경써주시고 상담도 자주해주셔서 버틸 수 있었던 것 같아요. 성적이 떨어져도 제 멘탈케어를 해주셔서 꾸준히 공부할 수 있었던 것 같습니다. 감사합니다.</v>
+        <v>1년 동안 재수하는 것이 너무 힘들것이라고 생각했었는데 이투스학원 선생님들이 계속 신경써주시고 상담도 자주해 주셔서 버틸 수 있었던 것 같아요. 성적이 떨어져도 제 멘탈케어를 해 주셔서 꾸준히 공부할 수 있었던 것 같습니다. 감사합니다.</v>
       </c>
       <c r="J255" t="str">
         <v>매주 플래너를 바탕으로 학습 점검이 이뤄져서 시간을 어떻게 활용하는지 선생님께서 세밀하게 관리해 주셔서 좋았어요.</v>
@@ -9661,7 +9661,7 @@
         <v>이투스 구독 시스템을 제공해줘서 부담 없이 다양한 강사님들의 강의를 듣고 선택할 수 있었습니다. 실제로 저는 김민정 선생님의 ebs 문학을 들었습니다. 두 개의 커리만 들어서 구독료를 매달 내기 좀 부담스러웠을 것 같은데 학원에서 제공해줘서 편하게 들을 수 있었습니다!</v>
       </c>
       <c r="I256" t="str">
-        <v>남들이 다 재수가 힘들다고 할 때 저는 정말 힘들지 않았는데 그 이유가 이투스247 학원 덕분이라고 생각합니다 ㅎㅎ 항상 공부하기 최적의 환경을 만들어주시고 다정하게 대해주셔서 감사했습니다! 학원 다니면서 공부 하는 법도 깨닫고 학원에서 쌓았던 것들을 발판 삼아 대학 공부도 열심히 하고 있습니다 감사합니다!!</v>
+        <v>남들이 다 재수가 힘들다고 할 때 저는 정말 힘들지 않았는데 그 이유가 이투스247 학원 덕분이라고 생각합니다 ㅎㅎ 항상 공부하기 최적의 환경을 만들어주시고 다정하게 대해 주셔서 감사했습니다! 학원 다니면서 공부 하는 법도 깨닫고 학원에서 쌓았던 것들을 발판 삼아 대학 공부도 열심히 하고 있습니다 감사합니다!!</v>
       </c>
       <c r="J256" t="str">
         <v>매달 내가 어느 정도 위치에 있고, 어떤 과목이 부족한지 모의고사를 통해 알 수 있어서 실전 감각도 익히고 도움이 많이 됐어요.</v>
@@ -9696,7 +9696,7 @@
         <v>각 인강 사이트마다 자신한테 맞는 선생들이 계시기 때문에 여러 패스를 끊어서 맞는 분을 찾는게 제일이지만 패스를 끊는 것도 비용이 들기 때문에 부담이 컸습니다. 그러나 이투스 247을 다니면 이투스 패스를 주어서 인강 선생님들 뵐 수 있다는 것이 비용적으로 부담이 줄었고 좋았습니다.</v>
       </c>
       <c r="I257" t="str">
-        <v>어떻게 공부를 해야 할지 모르던 저에게 올바른 방향을 제시해주시고 멘탈이 흔들릴 때나 지칠 때 잡아주시고 따뜻하게 대해주셔서 정말 감사했습니다. 덕분에 긴 수험 생활 잘 버틴 것 같습니다.!!</v>
+        <v>어떻게 공부를 해야 할지 모르던 저에게 올바른 방향을 제시해 주시고 멘탈이 흔들릴 때나 지칠 때 잡아주시고 따뜻하게 대해 주셔서 정말 감사했습니다. 덕분에 긴 수험 생활 잘 버틴 것 같습니다.!!</v>
       </c>
       <c r="J257" t="str">
         <v>졸음 지도 및 관리 덕분에 집중력을 유지하여, 순공 시간 확보에 큰 도움이 되었어요.</v>
@@ -9804,7 +9804,7 @@
         <v>감사했습니다 덕분에 좋은 대학생활 즐기고있어요 힘든일도이ㅛ았고 좋은일도 있었으나 결국 이겨내어 대학에 오게되었네요 이투스 관리감독 하시느라 힘드셨을텐데 앞으로도 힘내시길바랍니다!!</v>
       </c>
       <c r="J260" t="str">
-        <v>시기별로 상황에 맞춰 학습 방법을 추천해 주시고, 중간중간 점검도 해주셔서 취약 과목의 성적을 올리는 데 정말 많은 도움이 됐어요!</v>
+        <v>시기별로 상황에 맞춰 학습 방법을 추천해 주시고, 중간중간 점검도 해 주셔서 취약 과목의 성적을 올리는 데 정말 많은 도움이 됐어요!</v>
       </c>
       <c r="K260" t="str">
         <v/>
@@ -9836,10 +9836,10 @@
         <v>다양한 난이도의 모의고사를 풀며 실전 감각을 기를 수 있었습니다. 또한 학원 내 등수와 전국 등수가 함께 기재된 성적표를 통해 저의 위치를 객관적으로 파악할 수 있었고, 부족한 유형을 확인하여 보완할 수 있었습니다.</v>
       </c>
       <c r="I261" t="str">
-        <v>선생님들의 도움 덕분에 목표하던 학교에 진학하여 대학 생활을 즐기고 있습니다. 상담을 통해 해주신 말씀과 공부하며 얻은 것들을 바탕으로 앞으로도 열심히 살아가겠습니다. 진심으로 감사드립니다.</v>
+        <v>선생님들의 도움 덕분에 목표하던 학교에 진학하여 대학 생활을 즐기고 있습니다. 상담을 통해 해 주신 말씀과 공부하며 얻은 것들을 바탕으로 앞으로도 열심히 살아가겠습니다. 진심으로 감사드립니다.</v>
       </c>
       <c r="J261" t="str">
-        <v>모르는 문제 질문을 정말 많이 했는데 항상 친절하게 알려주시고, 따뜻한 응원도 해주셔서 큰 힘이 됐습니다!</v>
+        <v>모르는 문제 질문을 정말 많이 했는데 항상 친절하게 알려주시고, 따뜻한 응원도 해 주셔서 큰 힘이 됐습니다!</v>
       </c>
       <c r="K261" t="str">
         <v/>
@@ -9859,7 +9859,7 @@
         <v>N수생</v>
       </c>
       <c r="E262" t="str">
-        <v>수능을 망쳐서 원하는 대학을 가기에는 어려운 성적을 받았지만 선생님들께서 성적만 보고 판단하시지 않고 경쟁률 보시며 같이 상담해주시고 원서를 써서 원하는 대학에 붙을 수 있었습니다</v>
+        <v>수능을 망쳐서 원하는 대학을 가기에는 어려운 성적을 받았지만 선생님들께서 성적만 보고 판단하시지 않고 경쟁률 보시며 같이 상담해 주시고 원서를 써서 원하는 대학에 붙을 수 있었습니다</v>
       </c>
       <c r="F262" t="str">
         <v>한 강사의 커리큘럼만 추천하기보단 여러 강사들의 좋은 교재만 발췌해주시며 저의 스타일에 맞는 인강을 추천해 주시고 매주 진도를 확인하시며 그때 그때 저에게 필요한 플랜을 짜주신 것이 너무 인상적이었습니다</v>
@@ -9871,10 +9871,10 @@
         <v>매달 시험을 치르며 풀모의고사를 시간대로 풀 수 있는 시간대가 주어져 실전에서 도전해보지 못한 여러 방법을 적용해보며 모의고사속에서 저만의 스킬을 만들 수 있었고 다른 학생들과 같이 보며 등급과 성적을 볼 수 있어 동기부여가 되었습니다</v>
       </c>
       <c r="I262" t="str">
-        <v>제가 힘들 때마다 끝까지 믿어주시며 제가 힘든 소리를 하면 묵묵히 들어주시며 저의 의견을 존중해주시고 원서를 쓸 때도 진심으로 걱정하며 원서접수 마지막 날까지 같이 경쟁률 보며 챙겨주신 덕분에 대학에 갈 수 있었습니다 감사합니다</v>
+        <v>제가 힘들 때마다 끝까지 믿어주시며 제가 힘든 소리를 하면 묵묵히 들어주시며 저의 의견을 존중해 주시고 원서를 쓸 때도 진심으로 걱정하며 원서접수 마지막 날까지 같이 경쟁률 보며 챙겨주신 덕분에 대학에 갈 수 있었습니다 감사합니다</v>
       </c>
       <c r="J262" t="str">
-        <v>모의고사 결과를 바탕으로 부족한 부분을 짚어주시고, 논술 전형을 목표로 하는 저에게는 최저 충족을 위해 어떤 과목을 보완해야 할지도 함께 상담해주셨어요.</v>
+        <v>모의고사 결과를 바탕으로 부족한 부분을 짚어주시고, 논술 전형을 목표로 하는 저에게는 최저 충족을 위해 어떤 과목을 보완해야 할지도 함께 상담해 주셨어요.</v>
       </c>
       <c r="K262" t="str">
         <v>모의고사</v>
@@ -9929,14 +9929,14 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E264" t="str">
-        <v>공부를 하다보면 막막할때가 잦은데, 입시를 성공하신 선생님들의 학습 상담이 있어서 슬럼프나 막막할때 잘 넘어갈수 있었고, 때로는 엄격하지만 때로는 진중하고 재밌게 지친 수험 생활을 위로해주신점이 유용했습니다.</v>
+        <v>공부를 하다보면 막막할때가 잦은데, 입시를 성공하신 선생님들의 학습 상담이 있어서 슬럼프나 막막할때 잘 넘어갈수 있었고, 때로는 엄격하지만 때로는 진중하고 재밌게 지친 수험 생활을 위로해 주신점이 유용했습니다.</v>
       </c>
       <c r="F264" t="str" xml:space="preserve">
         <v xml:space="preserve">노베상태에서, 인강이나 책 선택조차 막막할 시기가 있었는데, 선생님이 계셔서 어떤 책을 어떻게 공부해야 할지 알수 있어서 유용했습니다._x000d_
-선생님이 추천해주신 책을 읽고 공부하니 비약적인 성적 상승을 이뤄서 기분이 좋았습니다.</v>
+선생님이 추천해 주신 책을 읽고 공부하니 비약적인 성적 상승을 이뤄서 기분이 좋았습니다.</v>
       </c>
       <c r="G264" t="str">
-        <v>고3 생활은 피곤한게 일상이였습니다. 학교를 끝나고 가는거다보니 상당히 심신이 지쳐있는 상태였고, 저녁을 먹고나면 졸기 십상인 상태였습니다. 하지먼 선생님들의 코칭 하에 면학 분위기를 형성해주시고, 잠을 쫓아주셔서 유용하고 좋았습니다.</v>
+        <v>고3 생활은 피곤한게 일상이였습니다. 학교를 끝나고 가는거다보니 상당히 심신이 지쳐있는 상태였고, 저녁을 먹고나면 졸기 십상인 상태였습니다. 하지먼 선생님들의 코칭 하에 면학 분위기를 형성해 주시고, 잠을 쫓아주셔서 유용하고 좋았습니다.</v>
       </c>
       <c r="H264" t="str">
         <v>여러 사설모의고사가 있지만, 이투스 모의고사를 통해 수능에 나올 유형이나 내용, 또한 나오진 않지만 공부에 도움이 되는 유형까지 다양하게 공부할 수 있었고, 수능 직전에 시간계산을 할때도 이투스 모의고사가 약방의 감초역할을 해줬습니다.</v>
@@ -9979,7 +9979,7 @@
         <v>이투스 전국모의고사를 매달 보는 것이 좋았습니다. 이투스 전국모의고사를 통해 다른 친구들과 나의 실력을 비교하는 기회를 제공받을 수 있었고, 무엇이 부족한지 파악할 수 있었습니다.</v>
       </c>
       <c r="I265" t="str">
-        <v>기숙학원에 있는동안 잘 케어해주셔서 감사합니다. 담임 선생님의 철저한 학습 관리와 멘토링 덕분에 반수에 성공해서 더 좋은 대학에 다닐 수 있게 되었습니다. 이투스247 기숙학원에서 관리해 주셔서 감사합니다.</v>
+        <v>기숙학원에 있는동안 잘 케어해 주셔서 감사합니다. 담임 선생님의 철저한 학습 관리와 멘토링 덕분에 반수에 성공해서 더 좋은 대학에 다닐 수 있게 되었습니다. 이투스247 기숙학원에서 관리해 주셔서 감사합니다.</v>
       </c>
       <c r="J265" t="str">
         <v>사소한 부분까지 함께 의견을 나누며 의지할 수 있는 선생님이 계셨다는 점이 수험 생활의 작은 힘이 되었어요.</v>
@@ -10169,7 +10169,7 @@
         <v>이투스 패스를 가장 우선으로 활용한 것은 아니었지만 몇가지 괜찮은 강의들이 있어 그것을 활용하기 위해 패스를 구독했다. 패스값을 학원에서 지원해주어서 원하는 강의를 추가적으로 들을 수 있어고 그것이 나에게 도움이 되었다.</v>
       </c>
       <c r="I269" t="str">
-        <v>저는 1년이 아닌 6개월만 다녔지만 1년간 수고 많으셨습니다! 매년 많은 학생들을 만나고 학샹들을 위해 희생해주셔서 감사합니다. 선생님들의 노력으로 많은 학생들이 도움을 받고 꿈을 펼치러 갈 수 있었고 갈 것 입니다! 다시 한 번 수고많으셨습니다!</v>
+        <v>저는 1년이 아닌 6개월만 다녔지만 1년간 수고 많으셨습니다! 매년 많은 학생들을 만나고 학샹들을 위해 희생해 주셔서 감사합니다. 선생님들의 노력으로 많은 학생들이 도움을 받고 꿈을 펼치러 갈 수 있었고 갈 것 입니다! 다시 한 번 수고많으셨습니다!</v>
       </c>
       <c r="J269" t="str">
         <v>개별 학습 데이터와 플래너, 방화벽 관리 덕분에 막막함을 줄이고 수험 생활을 잘 마무리했어요.</v>
@@ -10207,7 +10207,7 @@
         <v>배은지 선생님 제가 비록 재수생 같지도 않게 직장인 처럼 빨간날 마다 쉬고 주말에도 잘 나오지 않았지만 포기하지 않고 3주 마다 상담을 나눠 주시며 대회 상대가 돼줬던 것이 저의 재수 생활에 큰 활력이 됐습니다</v>
       </c>
       <c r="J270" t="str">
-        <v>전체적으로 스스로 공부하기 어려운 학생들에게 체계적인 관리와 즉각적인 피드백을 제공해준다는 점에서 만족도가 높은 학원이었어요.</v>
+        <v>전체적으로 스스로 공부하기 어려운 학생들에게 체계적인 관리와 즉각적인 피드백을 제공해 준다는 점에서 만족도가 높은 학원이었어요.</v>
       </c>
       <c r="K270" t="str">
         <v/>
@@ -10278,7 +10278,7 @@
         <v>처음 재수를 시작할 때 아무것도 모르는 노베이스 상태라 막막함이 컸는데, 선생님의 따뜻한 격려와 세심한 지도 덕분에 포기하지 않고 여기까지 올 수 있었습니다. 단순히 지식을 전달해 주시는 것을 넘어, 저의 학습 루틴과 멘탈까지 세밀하게 관리해 주신 덕분에 제 잠재력을 믿고 끝까지 완주할 수 있었습니다. 이제 저도 선생님처럼 누군가에게 선한 영향력을 주는 교육자가 되기 위해 노력하겠습니다. 그동안 베풀어 주신 은혜에 진심으로 감사드립니다</v>
       </c>
       <c r="J272" t="str">
-        <v>기초부터 심화까지 학습에 도움을 주시고 생활적인 부분에서도 많은 케어를 해주셔서 정말 감사드려요.</v>
+        <v>기초부터 심화까지 학습에 도움을 주시고 생활적인 부분에서도 많은 케어를 해 주셔서 정말 감사드려요.</v>
       </c>
       <c r="K272" t="str">
         <v/>
@@ -10298,10 +10298,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E273" t="str">
-        <v>내가 지금 하고 있는 공부법이 효율적인지 같이 고민해주시고 인강 사이트를 활용해서 공부하고 있다면 해당 강사에 대한 구체적인 로드맵도 함께 구상하는 시간을 가져서 도움이 많이 됐어요. 그리고 조교 선생님만의 공부법과 팁들을 많이 전수해주셔서 유익하게 공부 방법응 계획할 수 있었어요!</v>
+        <v>내가 지금 하고 있는 공부법이 효율적인지 같이 고민해 주시고 인강 사이트를 활용해서 공부하고 있다면 해당 강사에 대한 구체적인 로드맵도 함께 구상하는 시간을 가져서 도움이 많이 됐어요. 그리고 조교 선생님만의 공부법과 팁들을 많이 전수해 주셔서 유익하게 공부 방법응 계획할 수 있었어요!</v>
       </c>
       <c r="F273" t="str">
-        <v>수학 같은 경우는 해설지를 봐도 이해가 안 됐던 경우가 많았는데, 직접 문제를 함께 살펴보고 차근차근 설명해주신 점이 맘에 들었습니다. 또한 모르는 문제에 대해 바로 알려주는 것이 아니라 어떠한 점에서 막혔고 잘못된 습관이 있지는 않은지 점검해주신 후 능동적으로 문제릉 풀 수 있도록 도와주신 덕분에 스스로 문제를 풀어내는 능력을 기를 수 있었습니다!</v>
+        <v>수학 같은 경우는 해설지를 봐도 이해가 안 됐던 경우가 많았는데, 직접 문제를 함께 살펴보고 차근차근 설명해 주신 점이 맘에 들었습니다. 또한 모르는 문제에 대해 바로 알려주는 것이 아니라 어떠한 점에서 막혔고 잘못된 습관이 있지는 않은지 점검해 주신 후 능동적으로 문제릉 풀 수 있도록 도와주신 덕분에 스스로 문제를 풀어내는 능력을 기를 수 있었습니다!</v>
       </c>
       <c r="G273" t="str">
         <v>집에서 혼자 공부하거나 개인 스터디 카페에서 공부하는 경우 핸드폰 사용 절제가 잘 안됐는데 이투스247에서는 등원하자마자 핸드폰을 내기 때문에 오직 공부에만 몰두할 수 있는 환경에서 학습할 수 있어서 좋았습니다</v>
@@ -10310,7 +10310,7 @@
         <v>개인 공부만 하다보면 의지가 쉽게 떨어지기 마련인데 중간중간 전국 이투스 모의고사를 시행함으로서 나의 실력과 현재 위치를 직접적으로 체감할 수 있어 좋았습니다. 공부 자극도 돼서 꾸준한 학습을 이어가는데 도움이 많이 됐습니다!</v>
       </c>
       <c r="I273" t="str">
-        <v>학생 한명한명을 관리하는게 쉽지 않은 일인데 끝까지 함께 응원해주시고 여러모로 도와주셔서 너무 감사했습니다! 덕분에 지치지 않고 꾸준히 공부할 수 있었어요 ! 그리고 항상 맛있는 급식 주셔서 너무 감사했습니다!!</v>
+        <v>학생 한명한명을 관리하는게 쉽지 않은 일인데 끝까지 함께 응원해 주시고 여러모로 도와주셔서 너무 감사했습니다! 덕분에 지치지 않고 꾸준히 공부할 수 있었어요 ! 그리고 항상 맛있는 급식 주셔서 너무 감사했습니다!!</v>
       </c>
       <c r="J273" t="str">
         <v>출결 관리와 시간 관리가 철저해 자연스럽게 공부에 집중할 수 있었고, 전반적인 생활 습관을 바로잡는 데 도움이 되었어요.</v>
@@ -10368,7 +10368,7 @@
         <v>N수생</v>
       </c>
       <c r="E275" t="str">
-        <v>전반적인 성적, 부족한 과목과 파트를 자세히 파악해주시고 이를 토대로 구체적인 학습 방향을 제시해 주셔서 학습 계획 수립에 큰 도움이 되었습니다. 특히 저는 수학과 탐구 과목이 부족하였는데, 제시해주신 학습 방향대로 공부하니 성적 향상을 거둘 수 있었습니다.</v>
+        <v>전반적인 성적, 부족한 과목과 파트를 자세히 파악해 주시고 이를 토대로 구체적인 학습 방향을 제시해 주셔서 학습 계획 수립에 큰 도움이 되었습니다. 특히 저는 수학과 탐구 과목이 부족하였는데, 제시해 주신 학습 방향대로 공부하니 성적 향상을 거둘 수 있었습니다.</v>
       </c>
       <c r="F275" t="str">
         <v>수많은 콘텐츠가 넘쳐나는 현재 대학 입시 상황에서 무슨 교재와 강의를 선택해야 저의 현재 성적대에 도움이 될지 잘 모르겠어서 힘들었었는데 분석하신 제 성적을 바탕으로 각 과목의 교재와 강의를 꼼꼼히 추천해 주셔서 크게 도움이 되었습니다.</v>
@@ -10380,10 +10380,10 @@
         <v>영어가 현재 수능 체제에서 절대평가 과목이기도 해서 영어를 소홀히 하는 경향도 있었고 특히나 단어같은 경우는 귀찮아서 안 외우는 경우가 많았습니다. 단어를 선별해서 자료를 주신 덕에 외우기도 편리했고 다 같이 시험을 봐 강제성이 생긴 덕분에 꾸준히 단어를 외울 수 있었습니다.</v>
       </c>
       <c r="I275" t="str">
-        <v>힘들었던 재수 생활이었지만 독학기숙에서 시간을 보낼 수 있었기에 큰 힘이 되었던 것 같습니다. 힘들 때 상담해주시고, 방향성을 잡아주신 덕에 수월하게 공부했던 것 같습니다. 선생님들 덕분에 2026 입시를 마무리할 수 있었습니다. 감사합니다!</v>
+        <v>힘들었던 재수 생활이었지만 독학기숙에서 시간을 보낼 수 있었기에 큰 힘이 되었던 것 같습니다. 힘들 때 상담해 주시고, 방향성을 잡아주신 덕에 수월하게 공부했던 것 같습니다. 선생님들 덕분에 2026 입시를 마무리할 수 있었습니다. 감사합니다!</v>
       </c>
       <c r="J275" t="str">
-        <v>학습 계획을 하루와 주간 단위로 목표를 구체적으로 설정하고, 플래너로 중간 점검도 해주셔서 학습 방향을 명확하게 잡는 데 도움이 되었어요.</v>
+        <v>학습 계획을 하루와 주간 단위로 목표를 구체적으로 설정하고, 플래너로 중간 점검도 해 주셔서 학습 방향을 명확하게 잡는 데 도움이 되었어요.</v>
       </c>
       <c r="K275" t="str">
         <v>학습 계획</v>
@@ -10415,7 +10415,7 @@
         <v>단어를 외우는 계획을 잘 지키지 못하는 성격이어서, 매일매일 의무적으로 단어가 배부되고 저녁에 쓰는 것이 규칙적 생활에 도움이 되었고, 영어 실력을 높이는 방법이 된 것 같습니다.</v>
       </c>
       <c r="I276" t="str">
-        <v>이투스를 방학 때마다 꾸준히 다니고, 수능 직전 추석 휴일에도 다녔는데, 확실히 순공 시간을 늘리고 꾸준한 페이스를 유지하는 데 도움이 되었습니다. 이른 아침부터 문제를 나눠주시고, 관리해주신 것 정말 감사합니다.</v>
+        <v>이투스를 방학 때마다 꾸준히 다니고, 수능 직전 추석 휴일에도 다녔는데, 확실히 순공 시간을 늘리고 꾸준한 페이스를 유지하는 데 도움이 되었습니다. 이른 아침부터 문제를 나눠주시고, 관리해 주신 것 정말 감사합니다.</v>
       </c>
       <c r="J276" t="str">
         <v>한 해 동안 공부, 생활 관리를 넘어서 정말 많은 부분에서 도움을 받은 것 같아서 애틋한 마음이 드네요.</v>
@@ -10440,7 +10440,7 @@
       <c r="E277" t="str" xml:space="preserve">
         <v xml:space="preserve">학습 상담을 하면서 이후의 공부 계획과 방향성을 잡기 좋아서 만족스러웠다._x000d_
 _x000d_
-그동안 공부해온 산물들을 들고 담임 선생님과 이후에 어떻게 공부해내가면 좋을지를 얘기하였었는데 수시라면 수시전략대로 정시라면 정시대로 구체적 성적 향상에 도움 될만한 이야기를 해주셔서 그 학습 상담이 목표 대학에 합격하는 것에 대해 큰 도움이 되었던 것 같다.</v>
+그동안 공부해온 산물들을 들고 담임 선생님과 이후에 어떻게 공부해내가면 좋을지를 얘기하였었는데 수시라면 수시전략대로 정시라면 정시대로 구체적 성적 향상에 도움 될만한 이야기를 해 주셔서 그 학습 상담이 목표 대학에 합격하는 것에 대해 큰 도움이 되었던 것 같다.</v>
       </c>
       <c r="F277" t="str" xml:space="preserve">
         <v xml:space="preserve">언제든지 궁금한 게 생기면 1:1로 질문할 수 있다는 점이 큰 메리트를 가지고 있었던 것 같다._x000d_
@@ -10481,16 +10481,16 @@
         <v>취약 유형을 담임 선생님과 상담하면서 집중적으로 끌어올릴 수 있었다.또한 공부하다가 막히는 부분을 혼자 해결하기 힘들었는데 선생님과 상담하면서 방향성을 잡을 수 있게 되었다.독재의 단점이 혼자 공부하면서 방향성을 잡기 힘든건데 수원정자점에서 담임샘과 상담이 이러한 부분을 해결해주었다</v>
       </c>
       <c r="F278" t="str">
-        <v>인강의 경우 정말 괜찮은 강의가 많다 보니 그 중에 어떤것을 들어야 할지 많이 고민이 되었다. 그럴때마다 담임샘께 여쭤보면서 지금 나한태 적절한 수준의 강의는 무엇일지 알려주시고 추천을 해주셨다. 교재도 담임샘이 추천해주신 교재로 사용했었고 실제로 많이 도움되었다고 생각했다</v>
+        <v>인강의 경우 정말 괜찮은 강의가 많다 보니 그 중에 어떤것을 들어야 할지 많이 고민이 되었다. 그럴때마다 담임샘께 여쭤보면서 지금 나한태 적절한 수준의 강의는 무엇일지 알려주시고 추천을 해주셨다. 교재도 담임샘이 추천해 주신 교재로 사용했었고 실제로 많이 도움되었다고 생각했다</v>
       </c>
       <c r="G278" t="str">
-        <v>이투스 수원정자점을 다니면서 가장 좋았던 점은 생뢀관리였다.여기 오기전에 다니던 재종 학원애서는 생뢀관리샴이 계시긴 했었지만 몇시간에 한번 들어오실 정도로 생뢀관리를 안해주셨는데,이투스 학원에선 매 시간마다 들어오셔서 관리 해주신 점이 좋았다</v>
+        <v>이투스 수원정자점을 다니면서 가장 좋았던 점은 생뢀관리였다.여기 오기전에 다니던 재종 학원애서는 생뢀관리샴이 계시긴 했었지만 몇시간에 한번 들어오실 정도로 생뢀관리를 안해주셨는데,이투스 학원에선 매 시간마다 들어오셔서 관리 해 주신 점이 좋았다</v>
       </c>
       <c r="H278" t="str">
         <v>정시 공부를 하다보면 빠질 수 없는것이 실전 연습이다.이투스 학원에서 주관하는 실전 모의고사 연습은 실전 대비하기에 가장 효과적이었다. 매달 나오는 성적으로 현재 내 위치가 어느 정도인지 체감할 수 있었고 그에 따라 공부 계획도 수정할 수 있었다</v>
       </c>
       <c r="I278" t="str">
-        <v>수능공부 1년 동안 옆에서 많이 도와주시고 지켜봐주셔서 감사합니다! 공부하면서 많이 힘들고 불안할때마다 선생님들께서 조언주신것이 너무 도움되었어요.그리고 이벤트도 자주 진행해주셔서 버틸 수 있었습니다 감사합니다!</v>
+        <v>수능공부 1년 동안 옆에서 많이 도와주시고 지켜봐주셔서 감사합니다! 공부하면서 많이 힘들고 불안할때마다 선생님들께서 조언주신것이 너무 도움되었어요.그리고 이벤트도 자주 진행해 주셔서 버틸 수 있었습니다 감사합니다!</v>
       </c>
       <c r="J278" t="str">
         <v>주기적인 학습 상담과 1:1 질의응답, 휴대폰 관리와 모의고사 덕분에 끝까지 차분하게 공부할 수 있었어요.</v>
@@ -10525,7 +10525,7 @@
         <v>평소 영어에서 단어가 부족해서 많이 헤매고 그러면서도 열심히 외우다가 어느순간 안하게 됐습니다. 하지만 이투스에 와서 매일 시험을 보고 시험을 위해서라도 꾸준히 외우니 실력이 많이 늘어서 좋았어요</v>
       </c>
       <c r="I279" t="str">
-        <v>짧은 썸머기간동안 만나뵀지만 모두 진심으로 응원하고 격려해주셔서 너무 감사했습니다. 기숙 사감 선생님들도 생활 관리 선생님들도 과목 담당 선생님,논술 선생님, 그리고 저희 담당 선생님 모두 최적의 공부환경과 효율적인 학습을 위해 최선을 다해주셨어요! 덕분에 기숙생활 힘들지 않고 보람있게 마무리했습니다!</v>
+        <v>짧은 썸머기간동안 만나뵀지만 모두 진심으로 응원하고 격려해 주셔서 너무 감사했습니다. 기숙 사감 선생님들도 생활 관리 선생님들도 과목 담당 선생님,논술 선생님, 그리고 저희 담당 선생님 모두 최적의 공부환경과 효율적인 학습을 위해 최선을 다해 주셨어요! 덕분에 기숙생활 힘들지 않고 보람있게 마무리했습니다!</v>
       </c>
       <c r="J279" t="str">
         <v>스마트폰은 통제하기 어렵고 가장 큰 방해가 되는 요인인데 휴대폰을 제출하여 더 잘 집중할 수 있었어요.</v>
@@ -10693,19 +10693,19 @@
         <v>N수생</v>
       </c>
       <c r="E284" t="str">
-        <v>재수 중 초반 갈피가 안 잡혔을 때나 흐트러질 때쯤 혼자서 관리하기 어려운(핸드폰) 부분들을 관리해주시고 상담할 때 이제 거의 다 끝났다, 열심히 하라는 등의 격려 말을 해주셔서 멘탈 관리에 도움이 되었습니다.</v>
+        <v>재수 중 초반 갈피가 안 잡혔을 때나 흐트러질 때쯤 혼자서 관리하기 어려운(핸드폰) 부분들을 관리해 주시고 상담할 때 이제 거의 다 끝났다, 열심히 하라는 등의 격려 말을 해 주셔서 멘탈 관리에 도움이 되었습니다.</v>
       </c>
       <c r="F284" t="str">
-        <v>잘 모르는 커리큘럼을 잘 설명해주시고 제가 어떤 시기에 어떤 커리큘럼을 들어야하는지 자세히 조언해주시고 추천해 주셔서 좋았습니다. 제가 고민할 때 방향을 확실하게  잡아주셔서 유익했습니다.</v>
+        <v>잘 모르는 커리큘럼을 잘 설명해 주시고 제가 어떤 시기에 어떤 커리큘럼을 들어야하는지 자세히 조언해 주시고 추천해 주셔서 좋았습니다. 제가 고민할 때 방향을 확실하게  잡아주셔서 유익했습니다.</v>
       </c>
       <c r="G284" t="str">
         <v>제가 아침에 정말 많이 자고 사실 계속 잘 때 깨우실 때는 속으로 너무 짜증났는데 계속 깨워주시고 상담 때 일침도 날려주신 후에 정말 거짓말처럼 쭈욱 안 자서 너무 좋았습니다. 열정적으로 깨워주셔서 감사했습니다!</v>
       </c>
       <c r="H284" t="str">
-        <v>이투스 전국 모의고사를 통해서 계속 제 위치를 점검하고 실제 시험과 같은 분위기에서 연습할 수 있어서 좋았습니다. 결과가 나온 후 브리핑도 해주시고 반에서도 제 위치를 알 수 있는 게 큰 동력이 되었습니다.</v>
+        <v>이투스 전국 모의고사를 통해서 계속 제 위치를 점검하고 실제 시험과 같은 분위기에서 연습할 수 있어서 좋았습니다. 결과가 나온 후 브리핑도 해 주시고 반에서도 제 위치를 알 수 있는 게 큰 동력이 되었습니다.</v>
       </c>
       <c r="I284" t="str">
-        <v>계속 관리에 신경써주시고 조언도 해주시고 점검해주셔서 제가 만족할 수 있는 대학교이 올 수 있었습니다. 대학생활 너무 즐거워요! 이투스를 다녔던 걸 후회하지 않습니다. 감사합니다!</v>
+        <v>계속 관리에 신경써주시고 조언도 해 주시고 점검해 주셔서 제가 만족할 수 있는 대학교이 올 수 있었습니다. 대학생활 너무 즐거워요! 이투스를 다녔던 걸 후회하지 않습니다. 감사합니다!</v>
       </c>
       <c r="J284" t="str">
         <v>과목별로 시간 분배, 학습 방법을 선생님께서 노하우를 상세하게 알려주셔서 시험 때 문제 풀이에 정말 많은 도움이 됐어요!</v>
@@ -10728,7 +10728,7 @@
         <v>반수생</v>
       </c>
       <c r="E285" t="str">
-        <v>기숙학원에서의 생활상담은 단순한 고민 해결을 넘어서 큰 도움이 되었습니다. 규칙적인 생활에 적응하면서 생기는 스트레스나 학습에 대한 불안감을 상담을 통해 해소할 수 있었고, 상담 선생님께서 개인에 맞는 공부 방법과 생활 습관을 구체적으로 조언해주셔서 효율적으로 시간을 관리할 수 있었습니다. 덕분에 학업 집중도가 높아지고 심리적으로도 안정감을 느낄 수 있었습니다.</v>
+        <v>기숙학원에서의 생활상담은 단순한 고민 해결을 넘어서 큰 도움이 되었습니다. 규칙적인 생활에 적응하면서 생기는 스트레스나 학습에 대한 불안감을 상담을 통해 해소할 수 있었고, 상담 선생님께서 개인에 맞는 공부 방법과 생활 습관을 구체적으로 조언해 주셔서 효율적으로 시간을 관리할 수 있었습니다. 덕분에 학업 집중도가 높아지고 심리적으로도 안정감을 느낄 수 있었습니다.</v>
       </c>
       <c r="F285" t="str">
         <v>기숙학원에서의 성적 리포트 관리는 학습 방향을 잡는 데 매우 유용했습니다. 정기적으로 성적을 분석해 현재 위치를 객관적으로 파악할 수 있었고, 과목별 강점과 약점을 구체적으로 확인할 수 있었습니다. 이를 바탕으로 부족한 부분은 보완하고, 강점은 더욱 강화하는 전략적인 공부가 가능해졌습니다. 또한 목표 설정과 피드백이 반복되면서 학습 동기와 집중력이 크게 향상되었습니다.</v>
@@ -10740,10 +10740,10 @@
         <v>기숙학원에서 진행된 Voca 테스트는 영어 실력을 꾸준히 향상시키는 데 큰 도움이 되었습니다. 매일 정해진 분량의 단어를 반복적으로 암기하고 테스트를 통해 점검하면서 자연스럽게 어휘력이 쌓였습니다. 또한 틀린 단어를 다시 복습하는 과정이 체계적으로 이루어져 장기 기억으로 이어질 수 있었고, 꾸준한 긴장감 덕분에 학습 습관도 잡을 수 있었습니다. 이러한 반복 학습 시스템이 영어 성적 향상에 긍정적인 영향을 주었습니다.</v>
       </c>
       <c r="I285" t="str">
-        <v>항상 학생들을 위해 세심하게 지도해주신 선생님들께 진심으로 감사드립니다. 학업뿐만 아니라 생활 전반에 걸쳐 따뜻하게 신경 써주시고, 힘들 때마다 진심 어린 조언과 격려를 해주셔서 큰 힘이 되었습니다. 덕분에 흔들리지 않고 목표를 향해 꾸준히 나아갈 수 있었습니다. 앞으로도 이곳에서 배운 것들을 바탕으로 더욱 성장하는 모습으로 보답하겠습니다.</v>
+        <v>항상 학생들을 위해 세심하게 지도해 주신 선생님들께 진심으로 감사드립니다. 학업뿐만 아니라 생활 전반에 걸쳐 따뜻하게 신경 써주시고, 힘들 때마다 진심 어린 조언과 격려를 해 주셔서 큰 힘이 되었습니다. 덕분에 흔들리지 않고 목표를 향해 꾸준히 나아갈 수 있었습니다. 앞으로도 이곳에서 배운 것들을 바탕으로 더욱 성장하는 모습으로 보답하겠습니다.</v>
       </c>
       <c r="J285" t="str">
-        <v>단순히 학습 계획을 세워주는 것에 그치지 않고 실행할 수 있도록 점검도 해주시고, 생활 습관 등을 봐주셔서 해낼 수 있었어요.</v>
+        <v>단순히 학습 계획을 세워주는 것에 그치지 않고 실행할 수 있도록 점검도 해 주시고, 생활 습관 등을 봐주셔서 해낼 수 있었어요.</v>
       </c>
       <c r="K285" t="str">
         <v>학습 계획</v>
@@ -10810,7 +10810,7 @@
         <v>이투스 전국 모의고사는 실제 수능과 유사한 난이도와 문제 구성을 통해 실전 감각을 기르는 데 큰 도움이 되었습니다. 시험을 통해 자신의 위치를 객관적으로 파악할 수 있었고, 성적 분석 자료를 통해 취약한 과목과 단원을 정확히 확인할 수 있었습니다. 또한 반복적인 응시를 통해 시간 관리 능력과 문제 풀이 전략을 꾸준히 개선할 수 있어 실전 대비에 매우 유용했습니다.</v>
       </c>
       <c r="I287" t="str">
-        <v>1년 동안 늘 옆에서 지도해 주신 선생님들께 진심으로 감사드립니다. 힘들고 지칠 때마다 따뜻한 격려와 현실적인 조언을 해주셔서 끝까지 포기하지 않고 공부를 이어갈 수 있었습니다. 학습적인 부분뿐만 아니라 생활 태도와 마음가짐까지 세심하게 신경 써 주신 덕분에 많이 성장할 수 있었습니다. 항상 학생 한 명 한 명을 진심으로 대해주셔서 감사드리고, 그 덕분에 좋은 결과를 얻을 수 있었습니다.</v>
+        <v>1년 동안 늘 옆에서 지도해 주신 선생님들께 진심으로 감사드립니다. 힘들고 지칠 때마다 따뜻한 격려와 현실적인 조언을 해 주셔서 끝까지 포기하지 않고 공부를 이어갈 수 있었습니다. 학습적인 부분뿐만 아니라 생활 태도와 마음가짐까지 세심하게 신경 써 주신 덕분에 많이 성장할 수 있었습니다. 항상 학생 한 명 한 명을 진심으로 대해 주셔서 감사드리고, 그 덕분에 좋은 결과를 얻을 수 있었습니다.</v>
       </c>
       <c r="J287" t="str">
         <v>담임 선생님과 수학, 국어 선생님들이 따로 계셔서 원하는 분께 필요한 내용을 질문할 수 있는 점이 정말 좋았습니다.</v>
@@ -10880,7 +10880,7 @@
         <v>단어 외우기도 귀찮고 혼자하면 계속 미루다가 결국 안하게 되고 모르는 단어도 한번 보고 넘어가는게 끝인데 단어책을 멏회독 하면서 단어를 계속 보고 외우니까 훨씬 암기가 잘되고 물론 기간을 오래잡아야하지만 1년 공부한다 하고 단어장 여러개보다 한 단어장만 마스터해도 되니까 좋았다</v>
       </c>
       <c r="I289" t="str">
-        <v>열심히 봐주시고 상담도 깊이있게 해주셔서 감사했습니다 재수를 했어도 다시 학원 다니면서 했을거예요 나름 학원 다니면서 엄청 열심히 했다 생각하고 후회 없이 공부해보고 모르는 정보 없이 아쉬움 없이 공부할 수 있게 도와주셔서 감사했어요</v>
+        <v>열심히 봐주시고 상담도 깊이있게 해 주셔서 감사했습니다 재수를 했어도 다시 학원 다니면서 했을거예요 나름 학원 다니면서 엄청 열심히 했다 생각하고 후회 없이 공부해보고 모르는 정보 없이 아쉬움 없이 공부할 수 있게 도와주셔서 감사했어요</v>
       </c>
       <c r="J289" t="str">
         <v>원서를 쓸 때 강요 없이 진심으로 저의 의견을 존중해 주시면서 입시를 도와주신 덕분에 원하는 대학에 갈 수 있었습니다!</v>
@@ -10950,7 +10950,7 @@
         <v>우선, 매일 등원과 동시에 아침에 풀어야하는 국어 지문 1지문은 평가원 및 교육청 기출을 자주 접할 수 있도록 도와주었을 뿐 아니라 하루의 집중력을 긴 글을 통해 깨워주어 효율적의 학습의 시작을 마련해주었습니다. 그에 더해 매일 치러지는 영단어시험은 수능에 필요한 영단어들을 반복적으로 학습할 수 있도록 해주어 어휘력을 기르는데 큰 도움을 주었습니다.</v>
       </c>
       <c r="I291" t="str">
-        <v>학습 태도도 잘 잡혀있지 않았고 정신적으로도 많이 흔들리던 저를 잘 지탱해주셔서 감사합니다. 수능 공부 자체에 대한 실력 증진뿐만 아니라 학습 자체를 바라보는 태도에 대해 재정립할 수 있어서 정말 소중한 1년이었습니다🫠🫠 감사합니다!!</v>
+        <v>학습 태도도 잘 잡혀있지 않았고 정신적으로도 많이 흔들리던 저를 잘 지탱해 주셔서 감사합니다. 수능 공부 자체에 대한 실력 증진뿐만 아니라 학습 자체를 바라보는 태도에 대해 재정립할 수 있어서 정말 소중한 1년이었습니다🫠🫠 감사합니다!!</v>
       </c>
       <c r="J291" t="str">
         <v>노베이스라 인강과 교재 선택부터 막막했지만, 선생님께서 저에게 맞는 콘텐츠를 추천해 주신 덕분에 성적을 올릴 수 있었어요.</v>
@@ -10979,7 +10979,7 @@
         <v>성적 리포팅 및 관리가 도움이 되었습니다. 모의고사 응시 성적과 수능 예상 점수까지 리포팅되어 직관적으로 저의 위치를 알 수 있었고, 과목 간의 밸런스를 맞추기에도 수월했습니다. 월별로 성적 추이를 비교하며 공부하니 동기부여가 되어 더 열심히 공부했던 거 같습니다.</v>
       </c>
       <c r="G292" t="str">
-        <v>면학 분위기를 감독해주신 덕에 공부할 분위기가 조성되었고, 저도 흐트러지지 않고 공부에 집중할 수 있었습니다. 소음, 시설 관련 컴플레인이 생길 때마다 빠르게 처리해주시고 이해해주셔서 스트레스 없이 오직 공부에만 집중할 수 있었습니다.</v>
+        <v>면학 분위기를 감독해 주신 덕에 공부할 분위기가 조성되었고, 저도 흐트러지지 않고 공부에 집중할 수 있었습니다. 소음, 시설 관련 컴플레인이 생길 때마다 빠르게 처리해 주시고 이해해 주셔서 스트레스 없이 오직 공부에만 집중할 수 있었습니다.</v>
       </c>
       <c r="H292" t="str">
         <v>원래는 타 인강사이트의 패스를 수강하다가, 이투스 247 학원에서 재원생 콘텐츠로 이투스구독을 제공한 덕에 이투스 인강을 처음 수강했습니다. 스타강사들의 강의를 무료로 수강할 수 있다는게 정말 큰 메리트였습니다. 특히나 박광일, 정승제 선생님의 도움을 정말 많이 받았습니다.</v>
@@ -11011,7 +11011,7 @@
         <v>나의 상황에 맞는 학습플랜과 필요힌 공부 방법을 알려주셨고, 더 구체적으로 강의 수강 진도도 체크해 주시고 추천 강의도 알려주셔서 맞춤 공부하기 유용했습니다. 어려운 단원이나 특히 부족한 부분에 대해 보완할 수 있는 점을 정확히 알려주셨습니다.</v>
       </c>
       <c r="F293" t="str">
-        <v>나의 성적과 학업 목표에 따라 시간단위로  쪼개서 구체적이고 효율적으로 공부할 수 있도록 지도해주신 점이 좋았습니다. 특히 부족한 공부를 미루고 하고 싶은 공부 위주로 공부하는 습관이 있었는데 학원에서 준 계획표대로 실천하도록 노력했더니 균형 있는 공부를 할 수 있었습니다.</v>
+        <v>나의 성적과 학업 목표에 따라 시간단위로  쪼개서 구체적이고 효율적으로 공부할 수 있도록 지도해 주신 점이 좋았습니다. 특히 부족한 공부를 미루고 하고 싶은 공부 위주로 공부하는 습관이 있었는데 학원에서 준 계획표대로 실천하도록 노력했더니 균형 있는 공부를 할 수 있었습니다.</v>
       </c>
       <c r="G293" t="str">
         <v>공부를 방해하는 직접적인 요인을 강제적으로 제거함으로써 공부에만 오직 집중할 수 있는 환경이 만들어진 점이 가장 좋았습니다. 스터니카페나 다른 학원에서보다 더 통제적으로 핸드폰과 테블릿 사용을 조절할 수 있어서 공부에 집중하는데 효과적이었습니다.</v>
@@ -11055,7 +11055,7 @@
         <v>모의고사를 통해 실력 체크를 매주 할 수 있다는게 좋았고 오답을 바로바로 확인하고 질문할 수 있는 시스템이 큰 도움이 됐습니다. 모아두고 몰랐던 문제들만 다시 풀어보며 복습했더니 실전 시험에 큰 도움이 되었습니다.</v>
       </c>
       <c r="I294" t="str">
-        <v>질문이 많았는데 다 정성껏 봐주셔서 감사합니다.그리고 고민상담 또한 들어주고 옆에서 응원해주셔서 버틸 수 있었습니다. 힘들었던 고3시절 따뜻한 말 한마디들이 큰 힘이 되었습니다. 감사합니다</v>
+        <v>질문이 많았는데 다 정성껏 봐주셔서 감사합니다.그리고 고민상담 또한 들어주고 옆에서 응원해 주셔서 버틸 수 있었습니다. 힘들었던 고3시절 따뜻한 말 한마디들이 큰 힘이 되었습니다. 감사합니다</v>
       </c>
       <c r="J294" t="str">
         <v>선생님께서 성적 추이를 꼼꼼히 봐주시고 더 높은 목표를 제안해 주신 덕분에, 원하던 곳보다 더 좋은 학교에 합격할 수 있었어요!</v>
@@ -11090,7 +11090,7 @@
         <v>학원에서 주기적으로 실시되는 모의고사는 실제 시험과 유사한 환경을 경험하게 해주어 긴장감을 조절하는 데 큰 도움이 됩니다. 또한 자신의 현재 실력을 객관적으로 확인할 수 있어 부족한 과목이나 유형을 빠르게 파악하고 학습 방향을 수정할 수 있었습니다. 성적 추이를 통해 성장 과정을 눈으로 확인 할 수 있어 동기부여가 되었고, 시험 대비 전략을 세우는 데도 효과적이었습니다. 이러한 반복적인 훈련 덕분에 실전에서의 자신감과 안정감이 크게 향상되었습니다</v>
       </c>
       <c r="I295" t="str">
-        <v>학원에서 늘 따뜻한 격려와 세심한 지도를 해주신 선생님들께 진심으로 감사드립니다. 학습뿐만 아니라 생활 전반까지 꼼꼼히 챙겨주셔서 안정된 환경에서 공부할 수 있었고, 힘들 때마다 진심 어린 조 언과 응원으로 다시 일어설 수 있었습니다. 선생님들의 헌신적인 노력 덕분에 목표를 향해 흔들림 없이 나아갈 수 있었으며, 그 과정에서 큰 자신감과 성장을 경험할 수 있었습니다.</v>
+        <v>학원에서 늘 따뜻한 격려와 세심한 지도를 해 주신 선생님들께 진심으로 감사드립니다. 학습뿐만 아니라 생활 전반까지 꼼꼼히 챙겨주셔서 안정된 환경에서 공부할 수 있었고, 힘들 때마다 진심 어린 조 언과 응원으로 다시 일어설 수 있었습니다. 선생님들의 헌신적인 노력 덕분에 목표를 향해 흔들림 없이 나아갈 수 있었으며, 그 과정에서 큰 자신감과 성장을 경험할 수 있었습니다.</v>
       </c>
       <c r="J295" t="str">
         <v>학원에서 이투스 구독권을 지원해 주셔서 금전적인 부담을 줄이고 공부에만 매진할 수 있었습니다!</v>
@@ -11113,10 +11113,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E296" t="str">
-        <v>개인 담당 선생님이 배정되어 제 상황에 맞게 시간표를 짜주시고, 정기적인 상담을 통해 학습 방향을 잡아주셨습니다. 특히 주간 상담을 통해 진도를 꾸준히 체크해주셔서 공부 흐름을 유지하고, 부족한 과목을 개선할 수 있다는게 좋았습니다. 또한 과목별 담당 선생님이 따로 계셔서 모르는 문제를 바로 질문할 수 있다는 점도 좋았습니다. 혼자 공부할 때는 한 문제에 많은 시간을 쓰거나 해결하지 못하는 경우가 많았는데, 상담을 요청하면 다른 공부를 하고 있는 동안 불러서 친절하게 설명해주셔서 시간을 효율적으로 사용할 수 있었습니다. 무엇보다 혼자 공부할 때 쉽게 흐트러지던 습관이 많이 개선되었습니다. 집중이 흐트러지거나 졸 때는 선생님께서 직접 깨워주시기도 해서 학습 환경이 자연스럽게 유지되었습니다. 전체적으로 스스로 공부하기 어려운 학생들에게 체계적인 관리와 즉각적인 피드백을 제공해준다는 점에서 만족도가 높은 학원이었습니다!</v>
+        <v>개인 담당 선생님이 배정되어 제 상황에 맞게 시간표를 짜주시고, 정기적인 상담을 통해 학습 방향을 잡아주셨습니다. 특히 주간 상담을 통해 진도를 꾸준히 체크해 주셔서 공부 흐름을 유지하고, 부족한 과목을 개선할 수 있다는게 좋았습니다. 또한 과목별 담당 선생님이 따로 계셔서 모르는 문제를 바로 질문할 수 있다는 점도 좋았습니다. 혼자 공부할 때는 한 문제에 많은 시간을 쓰거나 해결하지 못하는 경우가 많았는데, 상담을 요청하면 다른 공부를 하고 있는 동안 불러서 친절하게 설명해 주셔서 시간을 효율적으로 사용할 수 있었습니다. 무엇보다 혼자 공부할 때 쉽게 흐트러지던 습관이 많이 개선되었습니다. 집중이 흐트러지거나 졸 때는 선생님께서 직접 깨워주시기도 해서 학습 환경이 자연스럽게 유지되었습니다. 전체적으로 스스로 공부하기 어려운 학생들에게 체계적인 관리와 즉각적인 피드백을 제공해 준다는 점에서 만족도가 높은 학원이었습니다!</v>
       </c>
       <c r="F296" t="str">
-        <v>혼자 공부할 때는 모르는 문제가 생기면 풀이를 찾아보거나 오랜 시간을 고민해야 해서 공부 흐름이 자주 끊겼습니다ㅜㅜ 하지만 학원에서는 질문을 신청해두면 다른 과목을 공부하는 동안 선생님께서 불러주셔서 시간을 낭비하지 않고 효율적으로 공부를 이어갈 수 있었습니다. 또한 단순히 정답만 알려주시는 것이 아니라, 문제 접근 방식과 어떻게 공부해야 하는지도 상담해주셔서 좋았습니다!  이해가 잘 되지 않는 부분은 다시 질문해도 부담 없이 친절하게 설명해주셔서 개념을 확실하게 정리할 수 있었습니다.</v>
+        <v>혼자 공부할 때는 모르는 문제가 생기면 풀이를 찾아보거나 오랜 시간을 고민해야 해서 공부 흐름이 자주 끊겼습니다ㅜㅜ 하지만 학원에서는 질문을 신청해두면 다른 과목을 공부하는 동안 선생님께서 불러주셔서 시간을 낭비하지 않고 효율적으로 공부를 이어갈 수 있었습니다. 또한 단순히 정답만 알려주시는 것이 아니라, 문제 접근 방식과 어떻게 공부해야 하는지도 상담해 주셔서 좋았습니다!  이해가 잘 되지 않는 부분은 다시 질문해도 부담 없이 친절하게 설명해 주셔서 개념을 확실하게 정리할 수 있었습니다.</v>
       </c>
       <c r="G296" t="str">
         <v>전체적으로 조용하고 집중할 수 있는 환경이 잘 조성되어 있어서 공부에 몰입할 수 있었습니다. 주변 친구들도 다 공부에 집중하는 분위기라 저도 흐트러지지 않고 꾸준히 앉아있게 되는 점이 좋았습니다. 특히 졸음 관리가 좋앗습니다. 혼자 공부할 때는 졸리면 그냥 자버리거나 끊기는 경우가 많았는데, 학원에서는 졸거나 집중이 흐트러질 때 선생님께서 직접 깨워주시거나 다시 집중할 수 있도록 도와주셔서 혼자 공부할 때보다 훨씬 오랜 시간 집중할 수 있었습니다. 덕분에 단순히 오래 앉아 있는 것이 아니라, 실제로 집중도 높은 공부 시간을 확보할 수 있었다고 느꼈습니다.</v>
@@ -11125,7 +11125,7 @@
         <v>영어는 단어가 매우 중요하다는 것을 알고 있어도 혼자 공부할 때는 외우는게 지루하게 느껴져서 대충 눈으로만 보고 넘어가는 경우가 많았습니다. 하지만 학원에서는 단어 시험이 주기적으로 진행되기 때문에 제대로 외울 수밖에 없는 환경이 만들어졌습니다. 단순히 시간을 주고 외우라고 하는 것이 아니라, 실제로 시험을 통해 확인되다 보니 더 집중해서 암기하게 되었고, 단어 실력이 확실히 향상되었다고 느꼈습니다. 이러한 반복적인 테스트 덕분에 단어 암기를 미루지 않게 되었고, 영어의 기본기를 다지는 데 도움이 되었습니다.</v>
       </c>
       <c r="I296" t="str">
-        <v>고1 겨울방학부터 고3 수능 직전까지 함께해주신 쌤들 너무너무 감사합니다!! 생각해보니까 꽤 긴 시간이었는데, 그동안 꾸준히 챙겨주시고 이끌어주셔서 끝까지 올 수 있었던 것 같아요 🥹 준성쌤!! 항상 하나하나 신경 써주시고 챙겨주셔서 진짜 든든했어요. 흐트러질 때마다 다시 잡아주셔서 끝까지 버틸 수 있었던 것 같아요!! 진짜 감사했습니다! 🥹🥰</v>
+        <v>고1 겨울방학부터 고3 수능 직전까지 함께해 주신 쌤들 너무너무 감사합니다!! 생각해보니까 꽤 긴 시간이었는데, 그동안 꾸준히 챙겨주시고 이끌어주셔서 끝까지 올 수 있었던 것 같아요 🥹 준성쌤!! 항상 하나하나 신경 써주시고 챙겨주셔서 진짜 든든했어요. 흐트러질 때마다 다시 잡아주셔서 끝까지 버틸 수 있었던 것 같아요!! 진짜 감사했습니다! 🥹🥰</v>
       </c>
       <c r="J296" t="str">
         <v>정기적으로 학습 상태를 점검하고, 앞으로의 계획을 선생님과 이야기 하면서 공부에 더 전념할 수 있었습니다.</v>
@@ -11183,16 +11183,16 @@
         <v>N수생</v>
       </c>
       <c r="E298" t="str">
-        <v>항상 주마다 담당 선생님과 시간별로 어떤 과목을 어떻게 공부할지 정했던 것이, 계획적으로 공부하는데 도움이 됐어요! 스케쥴링도 좋았지만, 선생님께서 개인 맞춤으로 좋은 교재도 추천을 잘 해주셔서 늘 길잡이가 있는 느낌이었어요. 공부 이외에도 고민이 있으면 상담할 수 있었기에 더 든든하기도 했어요. 😌</v>
+        <v>항상 주마다 담당 선생님과 시간별로 어떤 과목을 어떻게 공부할지 정했던 것이, 계획적으로 공부하는데 도움이 됐어요! 스케쥴링도 좋았지만, 선생님께서 개인 맞춤으로 좋은 교재도 추천을 잘 해 주셔서 늘 길잡이가 있는 느낌이었어요. 공부 이외에도 고민이 있으면 상담할 수 있었기에 더 든든하기도 했어요. 😌</v>
       </c>
       <c r="F298" t="str">
-        <v>우선 선생님께서 학습공간을 오가며 집중관리를 해주셔서, 졸거나 시간을 허비하는 일이 없었던 것 같아요. 그리고 개인 성적에 맞추어서 보완할 과목과 중점적으로 공부할 부분을 자세히 알려주셨던 게 도움이 많이 되었어요.</v>
+        <v>우선 선생님께서 학습공간을 오가며 집중관리를 해 주셔서, 졸거나 시간을 허비하는 일이 없었던 것 같아요. 그리고 개인 성적에 맞추어서 보완할 과목과 중점적으로 공부할 부분을 자세히 알려주셨던 게 도움이 많이 되었어요.</v>
       </c>
       <c r="G298" t="str">
         <v>공부에 있어서 가장 큰 장애물은 아마 핸드폰으로 인한 집중 흐트러짐이라 생각하는데요, 늘 등원시마다 휴대폰을 반납해야 했기에 수시로 폰을 보며 앚아서 시간을 날리는 일이 없었어요. 또한 wifi방화벽도 철저해서 태블릿로도 지정된  학습 사이트가 아니면 이용이 불가능해서 도움이 됐어요.</v>
       </c>
       <c r="H298" t="str">
-        <v>다른 장소나 모교를 찾아갈 필요 없이, 늘 등원하는 학원 그자리에서 모의고사를 볼 수 있는 점이 편리하기도 하고, 심적으로도 안정됐어요. 또 모의고사 결과도 잘 분석/조언 해주셔서 좋았어요!</v>
+        <v>다른 장소나 모교를 찾아갈 필요 없이, 늘 등원하는 학원 그자리에서 모의고사를 볼 수 있는 점이 편리하기도 하고, 심적으로도 안정됐어요. 또 모의고사 결과도 잘 분석/조언 해 주셔서 좋았어요!</v>
       </c>
       <c r="I298" t="str">
         <v>선생님들 잘 지내고 계시나요? 목표를 이루고 싶은데, 혼자 불안정하게 있었을 수도 있던 제게 길잡이가 되어주셔서 감사합니다. 한 해 동안 공부, 생활 관리를 넘어서 정말 많은 부분에서 도움을 받은 것 같아서 애틋한 마음이 드네요. 지금은 대학생이 되어 캠퍼스를 돌아다니는데, 그때의 제가 본다면 좋아할 것 같아요. 선생님들 덕분에 제가 끝까지 놓지 않고 헤쳐나갈 수 있던 것 같아요. 공부 이외에도 제게 많은 것들을 가르쳐주셔서 정말 감사합니다.</v>
@@ -11264,13 +11264,13 @@
         <v>매일 같은 환경에 있다보면 나도 모르게 멍을 때리거나 시간을 흘려 보낼 수 있는데, 플래너 관리가 있어 의식적으로 시간을 효율적으로 사용할 수 있었습니다. 또한 계획을 달성하지 못 한 날에도 담임 선생님과의 개인 면담을 통해 다시 한 번 동기를 부여 받고 다음날 다시 회복하면서 혼자 공부할 때 처럼 슬럼프에 빠지지 않을 수 있었습니다</v>
       </c>
       <c r="G300" t="str">
-        <v>졸음이 굉장히 많은 편이라 현역 때도, 재수 때도 힘들었는데 철저하게 감독하시고 바로바로 깨워주셔서 시간을 낭비하지 않을 수 있었습니다. 계속 조는 경우에는 스탠딩 책상으로 안내 해 주시고, 회복이 필요한 경우 양호실을 사용 할 수 있게 해주셔서 리프레쉬를 할 수 있었던 것 같습니다.</v>
+        <v>졸음이 굉장히 많은 편이라 현역 때도, 재수 때도 힘들었는데 철저하게 감독하시고 바로바로 깨워주셔서 시간을 낭비하지 않을 수 있었습니다. 계속 조는 경우에는 스탠딩 책상으로 안내 해 주시고, 회복이 필요한 경우 양호실을 사용 할 수 있게 해 주셔서 리프레쉬를 할 수 있었던 것 같습니다.</v>
       </c>
       <c r="H300" t="str">
         <v>영어에서 가장 기본이 되는 부분은 역시나 단어인데, 단어가 혼자 공부하기에는 가장 귀찮고 소홀 해질 수 있는 공부라고 생각합니다. 하지만 종례 시간 마다 모여서 단어 시험을 응시하니 어느정도의 강제성이 부여되어 꾸준히 단어를 외울 수 있었던 것 같습니다.</v>
       </c>
       <c r="I300" t="str">
-        <v>일 년 동안 말도 안 듣고 사고 뭉치였는데 끝까지 끌고 나가주신 갓투스 선생님들 정말 감사드립니다. 특히 항상 동기부여를 해주신 박재성 담임 선생님 진심으로 감사드리고, 지금은 안 계시지만 상담으로 제 멘탈을 항상 지켜주신 최봉호 선생님께도 감사드립니다</v>
+        <v>일 년 동안 말도 안 듣고 사고 뭉치였는데 끝까지 끌고 나가주신 갓투스 선생님들 정말 감사드립니다. 특히 항상 동기부여를 해 주신 박재성 담임 선생님 진심으로 감사드리고, 지금은 안 계시지만 상담으로 제 멘탈을 항상 지켜주신 최봉호 선생님께도 감사드립니다</v>
       </c>
       <c r="J300" t="str">
         <v>자제력이 많이 부족한 성격인데 학습 관련 사이트만 들어갈 수 있도록 방화벽이 있어 학습에만 집중할 수 있었습니다.</v>
@@ -11302,10 +11302,10 @@
         <v>핸드폰 수거를 통해 불필요한 핸드폰 사용을 줄일 수 있었습니다. 공부 환경에서 집중을 방해하는 핸드폰을 제거함으로써 온전히 공부에 집중할 수 있었고, 학습하는 내용에 대해 더 고민할 수 있는 환경이 조성될 수 있었습니다.</v>
       </c>
       <c r="H301" t="str">
-        <v>이투스 구독 패스를 제공해주셔서 다양한 선생님의 강의와 컨텐츠를 접할 수 있게 되어 도움이 되었습니다. 또한, 수험생 입장에서 인강 패스를 구매하기 위해 발생하는 경제적 부담도 덜 수 있었습니다.</v>
+        <v>이투스 구독 패스를 제공해 주셔서 다양한 선생님의 강의와 컨텐츠를 접할 수 있게 되어 도움이 되었습니다. 또한, 수험생 입장에서 인강 패스를 구매하기 위해 발생하는 경제적 부담도 덜 수 있었습니다.</v>
       </c>
       <c r="I301" t="str">
-        <v>매일 학습 환경을 관리해주시고 학습에 대한 상담을 진행해주신 덕분에 수능에 온전히 집중할 수 있었습니다. 다행히 수능에서도 좋은 성적을 받고 목표하던 대학에 진학하게 되어 더 감사한 마음입니다. 감사합니다.</v>
+        <v>매일 학습 환경을 관리해 주시고 학습에 대한 상담을 진행해 주신 덕분에 수능에 온전히 집중할 수 있었습니다. 다행히 수능에서도 좋은 성적을 받고 목표하던 대학에 진학하게 되어 더 감사한 마음입니다. 감사합니다.</v>
       </c>
       <c r="J301" t="str">
         <v>수시, 정시 방향성에 맞춰 입시 상담을 해주시는데 그에 맞춰 학습 방향도 같이 설계해 주셔서 목표 대학에 합격할 수 있었습니다.</v>
@@ -11340,7 +11340,7 @@
         <v>이투스 구독을 통해 정승제 선생님, 이지영 선생님 등 유명 강사들의 다양한 인강을 추가 비용 없이 수강할 수 있어 큰 도움이 되었습니다 수준 높은 강의를 활용해 부족한 부분을 보완하고, 효율적으로 공부하며 성적을 꾸준히 향상시킬 수 있었습니다</v>
       </c>
       <c r="I302" t="str" xml:space="preserve">
-        <v xml:space="preserve">1년 동안 저를 지도해주신 모든 선생님들께 정말 감사합니다 덕분에 지금 제가 대학생이 되어 캠퍼스 생활도 하고 즐겁게 지낼 수 있다고 생각합니다_x000d_
+        <v xml:space="preserve">1년 동안 저를 지도해 주신 모든 선생님들께 정말 감사합니다 덕분에 지금 제가 대학생이 되어 캠퍼스 생활도 하고 즐겁게 지낼 수 있다고 생각합니다_x000d_
 특히 멘탈 관리에 많은 도움을 주신 em반 담임 선생님 정은숙 선생님, 항상 맛있는 밥을 만들어주셨던 동원홈푸드 영양사님께 감사합니다!</v>
       </c>
       <c r="J302" t="str">
@@ -11370,7 +11370,7 @@
         <v>누군가 내 학습을 옆에서 피드백해주고 격려해주는 페이스메이커가 있다는 느낌을 1년 내내 받을 수 있었습니다. 같은 목표를 공유하며 계획을 세우고, 모의고사 직후에는 피드백을 해주시며 계획을 수정할 수 있었습니다. 콘텐츠 추천도 도와주셔서 가장 효율적으로 원하는 등급대에 도달할 수 있는 루트를 이용할 수 있었습니다!</v>
       </c>
       <c r="G303" t="str">
-        <v>아침 시간에 솔룸에 들어가면 졸음이 밀려올 수 밖에 없는 환경이지만, 독학기숙은 이걸 방지하기 위해 주간팀 선생님들이 순찰을 돌며 세심하게 졸음 관리를 해주셔서 졸음을 최소화할 수 있었습니다. 생활 관리도 매우 꼼꼼하게 이루어져서 자습실과 숙소에서 아무런 마찰이나 불편 없이 1년을 보냈던 것 같습니다!</v>
+        <v>아침 시간에 솔룸에 들어가면 졸음이 밀려올 수 밖에 없는 환경이지만, 독학기숙은 이걸 방지하기 위해 주간팀 선생님들이 순찰을 돌며 세심하게 졸음 관리를 해 주셔서 졸음을 최소화할 수 있었습니다. 생활 관리도 매우 꼼꼼하게 이루어져서 자습실과 숙소에서 아무런 마찰이나 불편 없이 1년을 보냈던 것 같습니다!</v>
       </c>
       <c r="H303" t="str">
         <v>이투스 모의고사는 실제 시험 현장과 매우 유사한 분위기 속에서 시험을 경험해볼 수 있다는 자체가 도움이 되는 경험이라고 생각합니다. 전국 단위에서 제 위치를 알아보고 부족한 점을 파악할 수 있고, 이투스 강사님들의 해설강의도 제공되어서 효과적으로 오답 정리를 할 수 있었습니다.</v>
@@ -11481,7 +11481,7 @@
         <v>요새의 인강패스 가격이 비싸짐에 따라 여러 회사의 패스를 사는 게 금전적으로 부담이 되었는데, 이투스에선 이를 지원해줘서 좋았습니다. 박광일, 정승제, 이지영 선생님의 강의를 무제한으로 들을 수 있었습니다. 특히 중간에 커리큘럼을 바꾸면서 타사의 강의와 비교해보기도 하며 학습 템포와 진도를 조절하는 데 도움이 되었습니다.</v>
       </c>
       <c r="I306" t="str">
-        <v>입시때 예민해져 불만도 많았고, 선생님들께 친절하게 대하지 못했음에도 배려해주시고 계속 웃으며 대해주셔서 감사합니다. 많은 학생들 관리하시느라 힘드셨을텐데 학생 하나하나에 신경써주시고 세세한 것 하나까지 기억해주시는 모습에 감동받기도 했습니다. 짧은 입시 기간이었지만 함께하며 정도 많이 들었고 선생님들을 잊지 못할 것 같습니다. 행복하세요.</v>
+        <v>입시때 예민해져 불만도 많았고, 선생님들께 친절하게 대하지 못했음에도 배려해 주시고 계속 웃으며 대해 주셔서 감사합니다. 많은 학생들 관리하시느라 힘드셨을텐데 학생 하나하나에 신경써주시고 세세한 것 하나까지 기억해주시는 모습에 감동받기도 했습니다. 짧은 입시 기간이었지만 함께하며 정도 많이 들었고 선생님들을 잊지 못할 것 같습니다. 행복하세요.</v>
       </c>
       <c r="J306" t="str">
         <v>모의고사 끝나면 매번 피드백 시간을 가졌는데 선생님이 객관적인 시선으로 필요한 부분을 찾아주셔서 큰 도움이 됐어요.</v>
@@ -11539,10 +11539,10 @@
         <v>N수생</v>
       </c>
       <c r="E308" t="str">
-        <v>인강이나 문제집을 찾을 시간이 많이 없었는데 어떤 걸 풀면 좋을지 추천해 주시고 진도 체크를 매주 해주셔서 도움이 되었다. 모의고사를 푼 이후에 틀린 문제를 기반으로 무엇을 보충하면 좋을지도 추천해주셨다.</v>
+        <v>인강이나 문제집을 찾을 시간이 많이 없었는데 어떤 걸 풀면 좋을지 추천해 주시고 진도 체크를 매주 해 주셔서 도움이 되었다. 모의고사를 푼 이후에 틀린 문제를 기반으로 무엇을 보충하면 좋을지도 추천해주셨다.</v>
       </c>
       <c r="F308" t="str">
-        <v>수학 문제를 풀면서 도저히 접근이 안되는 문제를 자주 질문했는데 이해를 할 수 있을 때까지 계속 설명해주셔서 풀 수 있는 문제가 는 것 같다. 해설지가 제대로 제공되지 않는 문제도 많아서 그 때 도움을 많이 받았다.</v>
+        <v>수학 문제를 풀면서 도저히 접근이 안되는 문제를 자주 질문했는데 이해를 할 수 있을 때까지 계속 설명해 주셔서 풀 수 있는 문제가 는 것 같다. 해설지가 제대로 제공되지 않는 문제도 많아서 그 때 도움을 많이 받았다.</v>
       </c>
       <c r="G308" t="str">
         <v>자습할 때 휴대폰을 보지 않는 게 어려웠는데 아예 수거를 하고 점심/저녁 시간에 학원 외부에서만 사용 가능하도록 되어 있어서 공부에만 집중할 수 있었다. 일요일 또한 자율등원이어도 휴대폰 제출이 필수여서 학원에 계속 나가게 된 것 같다.</v>
@@ -11551,10 +11551,10 @@
         <v>다른 업체의 사설 모의고사와 느낌이 달라서 새로운 유형의 문제를 풀기 좋았다. 낯선 문제를 풀 수 있는 기회가 생기기도 하고, 난이도가 사설 모의고사보다는 낮아서 풀만한 문제가 많았던 것 같다.</v>
       </c>
       <c r="I308" t="str">
-        <v>항상 요청 사항 잘 들어주시고 공부에 집중할 수 있도록 환경 마련해주셔서 감사합니다. 1년 동안 덕분에 공부 열심히 할 수 있었고 질문 잘 들어주셔서 어려운 문제도 풀 수 있었던 것 같습니다.</v>
+        <v>항상 요청 사항 잘 들어주시고 공부에 집중할 수 있도록 환경 마련해 주셔서 감사합니다. 1년 동안 덕분에 공부 열심히 할 수 있었고 질문 잘 들어주셔서 어려운 문제도 풀 수 있었던 것 같습니다.</v>
       </c>
       <c r="J308" t="str">
-        <v>항상 요청 사항 잘 들어주시고 공부에 집중할 수 있도록 환경 마련해주셔서 감사했어요.</v>
+        <v>항상 요청 사항 잘 들어주시고 공부에 집중할 수 있도록 환경 마련해 주셔서 감사했어요.</v>
       </c>
       <c r="K308" t="str">
         <v/>
@@ -11617,7 +11617,7 @@
         <v>반수생</v>
       </c>
       <c r="E310" t="str">
-        <v>다양한 대학교와 목표하는 대학교의 입결과 대학별로 더 중요치를 두는 과목 등에 대해서 자세하게 설명해주셔서 어느부분의 공부에 더욱 집중하여 학습해야 할지 알 수 있어서 많은 도움이 되았습니다!</v>
+        <v>다양한 대학교와 목표하는 대학교의 입결과 대학별로 더 중요치를 두는 과목 등에 대해서 자세하게 설명해 주셔서 어느부분의 공부에 더욱 집중하여 학습해야 할지 알 수 있어서 많은 도움이 되았습니다!</v>
       </c>
       <c r="F310" t="str">
         <v>매주 보는 개인 모의고사라던지, 평가원 모의고사, 달마다 학원에서 전체시행하는 더프모의고사같은 모의고사를 보고 나서 혼자서 사고하기 어려웠던 부분들에 대해 여쭈어보면 친절하게 알려주시고 그렇게 배운 부분이 하나의 자양분이 되어서 좋은 성적의 발판이 되었다고 생각합니다!</v>
@@ -11629,7 +11629,7 @@
         <v>영어단어가 영어에서 가장 중요하다고 생각하는데 힉원에서 보는 단어시험으로 인해 더욱 영어를 많이 접하게 되어서 영어 말하는 것 뿐 아니라 시험에서 필요한 듣기, 읽기 능력까지 다 함양되엏습니다!!</v>
       </c>
       <c r="I310" t="str">
-        <v>감사합니다! 항상 신경써주시고 잘 챙겨주시고 공부환경에 대해서 많이 배려해주셔서 감사해요. 제가 좀 까탈스러운편인데 배려해주신 부분이 너무 감사했습니다.. 항상 좋은 나날 되시길 부탁드려요!.!!</v>
+        <v>감사합니다! 항상 신경써주시고 잘 챙겨주시고 공부환경에 대해서 많이 배려해 주셔서 감사해요. 제가 좀 까탈스러운편인데 배려해 주신 부분이 너무 감사했습니다.. 항상 좋은 나날 되시길 부탁드려요!.!!</v>
       </c>
       <c r="J310" t="str">
         <v>모르는 문제를 여쭤볼 때 세세하게 풀이 방법을 알려주셔서 성적을 올리는 데 정말 많은 도움이 됐습니다!</v>
@@ -11658,7 +11658,7 @@
         <v>플래너 관리를 통해 규칙적인 학원 생활을 만들 수 있었고, 모의고사에서 여러 루틴을 시도해 저에게 맞는 루틴을 찾을 수 있었습니다. 또한 , 학습 방향이 맞는지 불안할 때 객관적인 시선으로 바라볼 수 있어서 좋았습니다.</v>
       </c>
       <c r="G311" t="str">
-        <v>졸음이 많은 편인데 , 선생님께서 졸음 관리를 철저하게 해주셔서 공부에 조금 더 몰두할 수 있었습니다. 졸음벨 시스템이 있어서 정말 졸릴 때는 눈을 붙이고 선생님께서 깨워주셨습니다.</v>
+        <v>졸음이 많은 편인데 , 선생님께서 졸음 관리를 철저하게 해 주셔서 공부에 조금 더 몰두할 수 있었습니다. 졸음벨 시스템이 있어서 정말 졸릴 때는 눈을 붙이고 선생님께서 깨워주셨습니다.</v>
       </c>
       <c r="H311" t="str">
         <v>이투스 인터넷 강의를 자유롭게 들을 수 있다는 점이 유용했습니다. 듣고 싶은 선생님과 이투스 선생님들의 컨텐츠를 다양하게 시도해보고 저에게 맞는 선생님을 찾을 수 있는 게 좋았습니다.</v>
@@ -11702,7 +11702,7 @@
         <v>1년 동안 학생들의 학습 코칭뿐만 아니라 멘탈 관리와 지친 학생들을 위한 간식 이벤트 등 많은 도움을 주셔서 매우 감사합니다! 덕분에 1년을 포기하지 않고  끝까지 잘 버틸 수 있었습니다.</v>
       </c>
       <c r="J312" t="str">
-        <v>학습 코칭뿐만 아니라 지친 학생들을 위해 다양한 이벤트도 진행해 주시고, 심리 상담도 해주셔서 끝까지 해낼 수 있었어요.</v>
+        <v>학습 코칭뿐만 아니라 지친 학생들을 위해 다양한 이벤트도 진행해 주시고, 심리 상담도 해 주셔서 끝까지 해낼 수 있었어요.</v>
       </c>
       <c r="K312" t="str">
         <v/>
@@ -11734,7 +11734,7 @@
         <v>재수를 하면서 수 많은 기출들과 모의고사들을 풀게 되는데 막판으로 갈수록 양질의 모의고사들을 얻기가 어려워집니다. 1달~2달에 한 번씩 치뤄지는 이투스 모의고사로 자기의 요즘 컨디션과 얼마나 성장했는지 체크도 하고 또 피드백까지 할수 있었던게 굉장한 도움이 되었던거 같습니다. 또 퀄리티 또한 입증이 되있기에 이투스에서 현장감을 느끼며 풀면서 실전성도 높일수가 있습니다.</v>
       </c>
       <c r="I313" t="str">
-        <v>1년 동안 질문에 친절히 답해주시고 힘들 때 격려로 끝까지 열심히 공부할 수 있게 도와주셔서 너무 감사합니다. 선생님들의 격려와 덕담이 없었더라면 끝까지 완주하지 못 했을거라고 생각합니다. 특히 제 담임이셨던 국어선생님 정말로 감사합니다.</v>
+        <v>1년 동안 질문에 친절히 답해 주시고 힘들 때 격려로 끝까지 열심히 공부할 수 있게 도와주셔서 너무 감사합니다. 선생님들의 격려와 덕담이 없었더라면 끝까지 완주하지 못 했을거라고 생각합니다. 특히 제 담임이셨던 국어선생님 정말로 감사합니다.</v>
       </c>
       <c r="J313" t="str">
         <v>재수 생활 동안 학습 계획과 생활 관리를 꾸준히 받아 끝까지 흔들리지 않고 공부할 수 있었어요.</v>
@@ -11769,7 +11769,7 @@
         <v>주기적인 모의고사로 내 위치를 확인할 수 있었던 점이 가장 좋아ㅛ습니다 수능 당일에 어떻게 하는것이 좋을지 어떤 루틴을 따를지 미리 생각할 수 있었던거 같아 좋았습니다 그래서 이투스 모의고사가 가장 좋았던거 같습니다</v>
       </c>
       <c r="I314" t="str">
-        <v>잘 이끌어주셔서 감사합니다 덕분에 좋은 결과가 있었던구 같습니다 힘든 수험 생활에도 불구하고 견딜 수 있었던 이유는 선생님들께서 열심히 독려해주시고 이끌어주셔서 그랬던거 같습니다 감사합니다</v>
+        <v>잘 이끌어주셔서 감사합니다 덕분에 좋은 결과가 있었던구 같습니다 힘든 수험 생활에도 불구하고 견딜 수 있었던 이유는 선생님들께서 열심히 독려해 주시고 이끌어주셔서 그랬던거 같습니다 감사합니다</v>
       </c>
       <c r="J314" t="str">
         <v>담당 과목 선생님들께서 상주하시면서 매주 학습 상담과 질의응답을 받아주셔서 정말 좋았어요.</v>
@@ -11795,7 +11795,7 @@
         <v>현재 실력에 대한 객관적인 평가와 보충할 점, 필요한 강의와 파트를 세세하게 파악해서 알려주시는 점이 좋았습니다. 특히 담임제로 이루어져서 공부 진도에 대해서도 체크 받고 주기적으로 공부 플랜을 조정하는 점이 학생 개개인에게 맞는 공부 방향을 알려주는 느낌이었습니다. 또한 전략적으로 과목들을 선택하도록 도와주셔서 실제 수능에서도 목표치 이상의 점수를 받을 수 있었고, 이에는 현명한 공부 플랜을 세워주셨던 선생님 덕분이라고 생각합니다. 또한, 단기적인 점수 향상이 필요했던 상황에서 가장 효율적일 수 있는 강의와 공부법을 알려주셔서 큰 도움이 됐습니다.</v>
       </c>
       <c r="F315" t="str">
-        <v>인강 선택지가 워낙 넓고, 실력과 집중 파트별로 다양한 인강들 중에서 현재 내 실력에 맞춰서 가장 적절한 인강을 추천해주신 점이 마음에 들었습니다. 또한, 인강별로 특징을 함께 설명해주셔서 선택지들 중 학생 개인이 유동적으로 들을 수 있어 큰 도움이 되었급니다. 인강 체계에 대해서 걱정이 많았었는데 다방면에서 많은 도움을 받았습니다.</v>
+        <v>인강 선택지가 워낙 넓고, 실력과 집중 파트별로 다양한 인강들 중에서 현재 내 실력에 맞춰서 가장 적절한 인강을 추천해 주신 점이 마음에 들었습니다. 또한, 인강별로 특징을 함께 설명해 주셔서 선택지들 중 학생 개인이 유동적으로 들을 수 있어 큰 도움이 되었급니다. 인강 체계에 대해서 걱정이 많았었는데 다방면에서 많은 도움을 받았습니다.</v>
       </c>
       <c r="G315" t="str">
         <v>확실히 공부하는 곳 내에서 조용하고 적절한 온도, 쾌적한 환경이 뒷받침 되니 공부 집중도가 향상됨을 느낄 수 있었습니다. 주변 학생들도 자거나 조는 학생이 없고, 조용한 환경이다 보니 더 집중해서 공부할 수 있었던 거 같습니다.</v>
@@ -11804,7 +11804,7 @@
         <v>공부하다 보면 전국모의고사나 사설 모의고사 등 많은 자료가 필요한데 이투스라는 큰 학원에서의 자료를 활용함으로써 질높은 수준의 모의고사를 풀 수 있었습니다. 다른 사설 모의고사에 비해 자료의 퀄리티와 통계가 좋아서 더욱 좋았습니다.</v>
       </c>
       <c r="I315" t="str">
-        <v>짧은 시간이었지만 많은 도움과 관심 주셨던 선생님들 덕분에 원하던 대학에 와서 만족스러운 대학생활을 즐기고 있습니다. 다방면에서 도와주시고 진심으로 응원해주셔서 감사했습니다. 수능 전 이투스에 다녔던 선택엔 후회가 없고 제 고3 최고의 선택이었던 거 같습니다!</v>
+        <v>짧은 시간이었지만 많은 도움과 관심 주셨던 선생님들 덕분에 원하던 대학에 와서 만족스러운 대학생활을 즐기고 있습니다. 다방면에서 도와주시고 진심으로 응원해 주셔서 감사했습니다. 수능 전 이투스에 다녔던 선택엔 후회가 없고 제 고3 최고의 선택이었던 거 같습니다!</v>
       </c>
       <c r="J315" t="str">
         <v>단기간의 점수 향상이 필요했는데 학원에서 상황에 맞춰 과목별로 학습 플랜을 세워 주셔서 효율적으로 공부할 수 있었어요!</v>
@@ -11839,7 +11839,7 @@
         <v>모의고사를 푸는 것 자체로 실전경험을 기를 수 있어서 좋다고 생각하고 모의고사를 다 풀고 틀린문제를 오답하는 과정에서 몰랐던 것을 알게 되거나 자주 하는 실수를 발견할 수 있어서 실력향상에 큰 도움이 되었습니다 이런 모의고사를 주기적으로 학원에서 시행하니 실력이 늘 수밖에 없었습니다</v>
       </c>
       <c r="I316" t="str">
-        <v>작년 저의 공부를 도와주시고 관리해 주셔서 정말 감사합니다 선생님들 덕분에 대학에 합격할 수 있었습니다 모의고사 성적이 나오면 제 성적을 분석해 주시고 상담해주신 선생님들 다시 한번 감사드립니다</v>
+        <v>작년 저의 공부를 도와주시고 관리해 주셔서 정말 감사합니다 선생님들 덕분에 대학에 합격할 수 있었습니다 모의고사 성적이 나오면 제 성적을 분석해 주시고 상담해 주신 선생님들 다시 한번 감사드립니다</v>
       </c>
       <c r="J316" t="str">
         <v>모의고사 등급을 잘 받아 학원에서 장학금을 주셨는데 공부하면서 많은 동기부여를 얻을 수 있었습니다!</v>
@@ -11862,7 +11862,7 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E317" t="str">
-        <v>모의고사 볼 때마다 모의고사 성적으로 대학 어디 갈 수 있는지 찝어주시고 목표를 설정해주셔서 내 위치를 파악할 수 있었고 동기부여를 얻을 수 있었다. 또한 입시설명회 등 입시정보를 많이 얻을 수 있는 자리를 만들어주어서 경험과 정보를 쌓는 데에 많은 도움이 되었다. 입시가 끝난 후 대학교에 원서를 넣을 때 성적에 맞춘 컨설팅을 통해 적절하게 원서를 작성했다.</v>
+        <v>모의고사 볼 때마다 모의고사 성적으로 대학 어디 갈 수 있는지 찝어주시고 목표를 설정해 주셔서 내 위치를 파악할 수 있었고 동기부여를 얻을 수 있었다. 또한 입시설명회 등 입시정보를 많이 얻을 수 있는 자리를 만들어주어서 경험과 정보를 쌓는 데에 많은 도움이 되었다. 입시가 끝난 후 대학교에 원서를 넣을 때 성적에 맞춘 컨설팅을 통해 적절하게 원서를 작성했다.</v>
       </c>
       <c r="F317" t="str">
         <v>모르는 문제를 질문하는 과정에서 내 스스로 메타인지가 길러져서, 내가 아는 것과 모르는 것을 확실히 구분할 수 있었다. 모르는 것을 질문하면서 선생님의 풀이와 나의 풀이를 비교할 수 있었다. 또한 선생님의 꿀팁들을 들으면서 학습적 측면에서 많은 성장을 할 수 있었다.</v>
@@ -11874,7 +11874,7 @@
         <v>영어 단어 일일테스트만 해도 외워야 하는 단어의 양이 충족되는 느낌이었다. 실제로 영어공부를 하나도 하지 않았는데도 단어 외운 것으로  커버가 되어서 노력 대비 성과가 좋게 나타났다. 그리고 꾸준히 해야한다는 강제성이 부여된게 좋았다.</v>
       </c>
       <c r="I317" t="str">
-        <v>선생님 덕분에 이름 들어본 대학에 오게 되었어요. 1년 동안 제 불안들 받아주시고 따듯하게 답변해주신거 정말 감사해요. 덕분에 많은 도움 되었고 많이 성장했습니다. 저도 선생님을 본받아서 남에게 친절을 베풀 수 있는 멋진 어른으로 성장하겠습니다.</v>
+        <v>선생님 덕분에 이름 들어본 대학에 오게 되었어요. 1년 동안 제 불안들 받아주시고 따듯하게 답변해 주신거 정말 감사해요. 덕분에 많은 도움 되었고 많이 성장했습니다. 저도 선생님을 본받아서 남에게 친절을 베풀 수 있는 멋진 어른으로 성장하겠습니다.</v>
       </c>
       <c r="J317" t="str">
         <v>혼자서 찾기 어려운 입시 정보를 학원에서 제공해 주셔서 원서 준비에 많은 도움이 됐어요.</v>
@@ -11900,7 +11900,7 @@
         <v>매주 담임 선생님과 함께 전 과목의 교재 진도를 계획하고, 일주일 후 그 계획을 실제로 수행했는지 선생님과 함께 교재를 통해 점검받을 수 있었다. 혼자 계획을 세우고 공부할 때보다 지속적인 피드백을 받을 수 있어 학습에 대한 긴장감을 유지할 수 있었고, 그 덕분에 끈기를 잃지 않고 꾸준히 공부할 수 있었다.</v>
       </c>
       <c r="F318" t="str">
-        <v>담임 선생님께서 다양한 과목의 인터넷 강의에 대한 이해도가 높아, 나의 수준과 현재 상황에 맞는 강의와 교재를 적절하게 추천해주신 점이 가장 유용했다. 덕분에 혼자서 선택에 시간을 낭비하지 않고 효율적으로 학습할 수 있었으며, 수강 진도까지 함께 관리해 주셔서 꾸준히 공부를 이어가는 데 큰 도움이 되었다.</v>
+        <v>담임 선생님께서 다양한 과목의 인터넷 강의에 대한 이해도가 높아, 나의 수준과 현재 상황에 맞는 강의와 교재를 적절하게 추천해 주신 점이 가장 유용했다. 덕분에 혼자서 선택에 시간을 낭비하지 않고 효율적으로 학습할 수 있었으며, 수강 진도까지 함께 관리해 주셔서 꾸준히 공부를 이어가는 데 큰 도움이 되었다.</v>
       </c>
       <c r="G318" t="str">
         <v>수능 공부와 관련된 앱/사이트에만 접속이 가능하니 학습에만 집중할 수 있었던 점이 가장 유용했다. 스스로 통제하기 어려운 상황에서도 외부적인 관리가 이루어지니 흐트러짐을 줄일 수 있었다.</v>
@@ -11909,7 +11909,7 @@
         <v>이투스 전국 모의고사는 문제의 수준이 높아 실전 대비에 큰 도움이 되었으며, 매달 꾸준히 응시하면서 수능과 유사한 긴장감과 시간 감각을 유지할 수 있었고 그 실전 감각이 수능장까지 이어져 도움이 되었다.</v>
       </c>
       <c r="I318" t="str">
-        <v>반년 동안 옆에서 꾸준히 신경 써주시고 챙겨주셔서 정말 감사했습니다. 공부가 잘 안 풀릴 때 같이 고민해주시고 방향을 잡아주신게 수능 날까지 버틸 수 있는 큰 힘이 됐던 것 같습니다. 감사합니다.</v>
+        <v>반년 동안 옆에서 꾸준히 신경 써주시고 챙겨주셔서 정말 감사했습니다. 공부가 잘 안 풀릴 때 같이 고민해 주시고 방향을 잡아주신게 수능 날까지 버틸 수 있는 큰 힘이 됐던 것 같습니다. 감사합니다.</v>
       </c>
       <c r="J318" t="str">
         <v>스스로 통제하기 어려운 상황에서 외부적인 관리가 이루어지니 흐트러짐을 줄일 수 있었어요.</v>
@@ -12004,7 +12004,7 @@
         <v>N수생</v>
       </c>
       <c r="E321" t="str">
-        <v>담임 선생님들이 계셔서 학습 외적인 부분에서도 도움을 받을 수 있다는 점이 좋았습니다. 기숙학원에서 재수를 하다보니 아무래도 정신적으로 힘들고 흔들릴 때가 많았는데 그럴 때마다 담임 선생님과의 대화를 통해 버티고 이겨낼 수 있었던 것 같습니다. 담임 선생님들이 진심으로 대해주셔서 좋았습니다.</v>
+        <v>담임 선생님들이 계셔서 학습 외적인 부분에서도 도움을 받을 수 있다는 점이 좋았습니다. 기숙학원에서 재수를 하다보니 아무래도 정신적으로 힘들고 흔들릴 때가 많았는데 그럴 때마다 담임 선생님과의 대화를 통해 버티고 이겨낼 수 있었던 것 같습니다. 담임 선생님들이 진심으로 대해 주셔서 좋았습니다.</v>
       </c>
       <c r="F321" t="str">
         <v>혼자서는 알아볼 수 없는 것들을 알 수 있어 좋았습니다. 또한, 성적분석만 나오는 것이 아니라 점수 변동 추이, 가능한 대학과 학과까지 자세하기 볼 수 있어 수험 생활 중 궁금증이 많이 해소되었습니다.</v>
@@ -12016,7 +12016,7 @@
         <v>독학기숙이다보니 인터넷강의만을 활용하여 공부하는데 이투스 구독권을 받아 무료로 이투스 강의를 들을 수 있다는 점이 좋았습니다. 더욱 더 선택지가 많아지고,  비용적으로 부담이 되는 인터넷강의를 무료로 들을 수 있어 평소에 궁금했던 선생님의 강의를 들어볼 수 있는게 좋았습니다.</v>
       </c>
       <c r="I321" t="str">
-        <v>대학 진학 결과가 제 생각만큼 좋지 않아서 이런 글을 써도 될까 고민했습니다. 그러나 작년 한해동안 학원에서 지내면서 정말 많이 배웠고 성장했습니다. 특히 제가 많이 울었는데 옆에서 같이 걱정해주시고 위로해주셨던 담임 선생님, 그리고 다른 반 담임 선생님이지만 상담시간 쪼개서 제 학습 상담까지 봐주셨던 선생님 정말 감사했습니다.</v>
+        <v>대학 진학 결과가 제 생각만큼 좋지 않아서 이런 글을 써도 될까 고민했습니다. 그러나 작년 한해동안 학원에서 지내면서 정말 많이 배웠고 성장했습니다. 특히 제가 많이 울었는데 옆에서 같이 걱정해 주시고 위로해주셨던 담임 선생님, 그리고 다른 반 담임 선생님이지만 상담시간 쪼개서 제 학습 상담까지 봐주셨던 선생님 정말 감사했습니다.</v>
       </c>
       <c r="J321" t="str">
         <v>담임 선생님들이 계셔서 학습 외적인 부분에서도 도움을 받을 수 있다는 점이 좋았어요.</v>
@@ -12039,7 +12039,7 @@
         <v>N수생</v>
       </c>
       <c r="E322" t="str">
-        <v>과목별로 학습 진행 상황에 대해 자세히 파악하고, 어떤 방향으로 나아가야할지 구체적으로 조언해주셨다. 또한 과목별로 구체적인 공부 방법도 알려주셔서 좋았다. 매주 플래너 검사도 꼼꼼히 해주시고 부족한 과목을 찾아내어 채울 수 있도록 도움을 주셔서 유용했다.</v>
+        <v>과목별로 학습 진행 상황에 대해 자세히 파악하고, 어떤 방향으로 나아가야할지 구체적으로 조언해주셨다. 또한 과목별로 구체적인 공부 방법도 알려주셔서 좋았다. 매주 플래너 검사도 꼼꼼히 해 주시고 부족한 과목을 찾아내어 채울 수 있도록 도움을 주셔서 유용했다.</v>
       </c>
       <c r="F322" t="str">
         <v>플래너를 검사하고 학습 진행 상황을 파악하여 단계에 맞는 학습 방법을 알려주셔서 유용하였다. 또한 플래너에서 부족한 부분을 찾아 보충하도록 도움을 주시고, 자세한 교재와 인강도 함께 추천해 주셔서 도움을 많이 받았다.</v>
@@ -12051,7 +12051,7 @@
         <v>다른 과목을 공부하느라 단어는 놓치기가 매우 쉬운데 단어 시험으로 매일 단어를 강제적으로 학습할 수 있게 하여 수능 영어에서 가장 중요한 부분을 매일 공부할 수 있었습니다. 모든 단어를 시험봐서 꼼꼼하고 자세하게 외우도록 하여 도움이 많이 되었습니다.</v>
       </c>
       <c r="I322" t="str">
-        <v>공부뿐만 아니라 생활이나 친구 관계에도 항상 신경 써주셔서 감사했습니다!! 덕분에 사소한 것에 흔들리지 않고 끝까지 열심히 공부할 수 있었습니다. 수업하시는 선생님들도 항상 열정적으로 수업해주시고 상담도 꼼꼼히 해주셔서 정말 도움이 많이 되었습니다. 다시 한번 감사드립니다!</v>
+        <v>공부뿐만 아니라 생활이나 친구 관계에도 항상 신경 써주셔서 감사했습니다!! 덕분에 사소한 것에 흔들리지 않고 끝까지 열심히 공부할 수 있었습니다. 수업하시는 선생님들도 항상 열정적으로 수업해 주시고 상담도 꼼꼼히 해 주셔서 정말 도움이 많이 되었습니다. 다시 한번 감사드립니다!</v>
       </c>
       <c r="J322" t="str">
         <v>플래너에서 부족한 부분을 찾아 보충하도록 도움을 주시고, 자세한 교재와 인강도 함께 추천해 주셔서 도움을 많이 받았어요.</v>
@@ -12074,7 +12074,7 @@
         <v>N수생</v>
       </c>
       <c r="E323" t="str">
-        <v>먼저 한약학과라는 학과를 소개해주시고 망설이는 저에게 확신을 갖게 해주는 선생님께 너무너무 감사드립니다. 또한 제 생기부와 수시 등급을 가지고 현실적으로 갈수 있는 곳을 알려주셔서 그때 당시에는 가슴아팠지만.. 장기적으로는 너무 다행이였습니다</v>
+        <v>먼저 한약학과라는 학과를 소개해 주시고 망설이는 저에게 확신을 갖게 해주는 선생님께 너무너무 감사드립니다. 또한 제 생기부와 수시 등급을 가지고 현실적으로 갈수 있는 곳을 알려주셔서 그때 당시에는 가슴아팠지만.. 장기적으로는 너무 다행이였습니다</v>
       </c>
       <c r="F323" t="str">
         <v>여러 다양한 인강 선생님들을 알수 있었고 2주에 한 번씩 상담을 하면서 최대한 인강을 안미루게 듣게되고 mbti가 p 90퍼인 저도 계획을 가지고 인강을 들을수 있게 되었습니다..ㅎㅎ</v>
@@ -12113,7 +12113,7 @@
 특히 좋았던 건 단어 시험 관리였어요. 영어 단어 암기는 꾸준히 유지하는 게 제일 어려운데, 시험으로 관리해줘서 일정 수준 이상의 암기량을 놓치지 않을 수 있었습니다. 그냥 알아서 외우라고 했으면 흐지부지됐을 것 같은데, 확인받는 구조 덕분에 긴장감도 생기고 꾸준히 이어나갈 수 있었어요.​​​​​​​​​​​​​​​​</v>
       </c>
       <c r="F324" t="str">
-        <v>1타 강사가 아니면 어떤 강사가 좋은지 정보가 별로 없었는데, 선생님께서 상담 후 저한테 잘 맞을 것 같은 강사를 추천해주셨습니다. 직접 들어보니 너무 만족스러웠고, 강사 선택으로 고민할 시간을 많이 단축할 수 있었습니다. 덕분에 처음부터 올바른 방향으로 나아가기가 훨씬 수월했습니다. 또 공부 페이스가 처질 때마다 새로운 교재를 추가해주셔서 다시 집중력을 끌어올리고 꾸준한 페이스를 유지할 수 있었습니다.​​​​​​​​​​​​​​​​</v>
+        <v>1타 강사가 아니면 어떤 강사가 좋은지 정보가 별로 없었는데, 선생님께서 상담 후 저한테 잘 맞을 것 같은 강사를 추천해주셨습니다. 직접 들어보니 너무 만족스러웠고, 강사 선택으로 고민할 시간을 많이 단축할 수 있었습니다. 덕분에 처음부터 올바른 방향으로 나아가기가 훨씬 수월했습니다. 또 공부 페이스가 처질 때마다 새로운 교재를 추가해 주셔서 다시 집중력을 끌어올리고 꾸준한 페이스를 유지할 수 있었습니다.​​​​​​​​​​​​​​​​</v>
       </c>
       <c r="G324" t="str">
         <v>재수 생활을 하다 보면 점심 이후에 쏟아지는 졸음을 이기는 게 보통 일이 아닌데, 학원에서 낮잠 시간을 따로 운영해줘서 짧게 자고 나면 오후 공부 집중력이 확실히 달랐습니다. 그냥 졸린 채로 억지로 버티는 것보다 잠깐 눈을 붙이고 다시 집중하는 게 훨씬 효율적이었어요. 졸음을 개인 의지로만 해결하려 했으면 오후 시간을 많이 날렸을 것 같은데, 체계적으로 관리해준 덕분에 하루 전체 공부량을 안정적으로 유지할 수 있었습니다.​​​​​​​​​​​​​​​​</v>
@@ -12122,10 +12122,10 @@
         <v>전국 모의고사를 학원에서 직접 응시할 수 있었던 게 정말 좋았습니다. 실제 수능과 비슷한 환경에서 시험을 치르다 보니 긴장감도 익숙해지고, 실전 감각을 꾸준히 유지할 수 있었어요. 성적표를 통해 전국에서 내 위치가 어느 정도인지 객관적으로 확인할 수 있어서 막연한 불안감이 줄었고, 부족한 부분이 어딘지 명확하게 파악해 다음 학습 계획에 바로 반영할 수 있었습니다. 혼자 공부했으면 내 실력을 제대로 가늠하기 어려웠을 텐데, 정기적으로 모의고사를 보면서 현실적인 목표 설정도 가능했어요.​​​​​​​​​​​​​​​​</v>
       </c>
       <c r="I324" t="str">
-        <v>1년 동안 옆에서 꼼꼼하게 챙겨주신 선생님들께 정말 감사드립니다. 힘들고 지칠 때마다 따뜻하게 격려해주신 덕분에 끝까지 포기하지 않고 버틸 수 있었어요. 덕분에 좋은 결과를 얻을 수 있었습니다. 감사합니다!​​​​​​​​​​​​​​​​</v>
+        <v>1년 동안 옆에서 꼼꼼하게 챙겨주신 선생님들께 정말 감사드립니다. 힘들고 지칠 때마다 따뜻하게 격려해 주신 덕분에 끝까지 포기하지 않고 버틸 수 있었어요. 덕분에 좋은 결과를 얻을 수 있었습니다. 감사합니다!​​​​​​​​​​​​​​​​</v>
       </c>
       <c r="J324" t="str">
-        <v>시기별로 인강 추천을 해주셔서 어떤 것을 들어야 할지 찾는 시간을 아껴 공부할 수 있었어요.</v>
+        <v>시기별로 인강 추천을 해 주셔서 어떤 것을 들어야 할지 찾는 시간을 아껴 공부할 수 있었어요.</v>
       </c>
       <c r="K324" t="str">
         <v>인강 추천</v>
@@ -12231,7 +12231,7 @@
         <v>이투스 전국 모의고사는 현재 내 위치를 객관적으로 확인할 수 있다는 점에서 도움이 됐다. 평소엔 내가 어느 정도 하고 있는지 감이 애매할 때가 많은데, 실제 시험처럼 점검해보면 약한 부분이 훨씬 선명하게 보인다. 특히 실전 시간 관리나 멘탈 흐름까지 같이 체크할 수 있어서 그냥 문제 푸는 거랑은 확실히 다르게 느껴졌다. 막연하게 불안해하기보다, 뭘 보완해야 하는지 방향을 잡는 데 유용했다.</v>
       </c>
       <c r="I327" t="str">
-        <v>선생님들께 감사했던 부분 중 하나는 제 체력이 정말 약한 편이라는 걸 그냥 의지 부족으로 보지 않고, 제 상황 자체를 이해해주셨다는 점이었다. 컨디션이 따라주지 않는 날에도 무작정 몰아붙이기보다 왜 힘든지 먼저 봐주시고, 그 안에서 할 수 있는 방향으로 같이 조정해주셔서 덜 지치고 더 오래 갈 수 있었다. 괜찮다고 넘기지 않고 공감해주시던 태도 덕분에 혼자만 뒤처지는 느낌도 덜했고, 그래서 더 버텨볼 힘이 났다</v>
+        <v>선생님들께 감사했던 부분 중 하나는 제 체력이 정말 약한 편이라는 걸 그냥 의지 부족으로 보지 않고, 제 상황 자체를 이해해주셨다는 점이었다. 컨디션이 따라주지 않는 날에도 무작정 몰아붙이기보다 왜 힘든지 먼저 봐주시고, 그 안에서 할 수 있는 방향으로 같이 조정해 주셔서 덜 지치고 더 오래 갈 수 있었다. 괜찮다고 넘기지 않고 공감해주시던 태도 덕분에 혼자만 뒤처지는 느낌도 덜했고, 그래서 더 버텨볼 힘이 났다</v>
       </c>
       <c r="J327" t="str">
         <v>선생님과 함께 세운 학습 계획이 유용했던 건, 그냥 “공부해라”가 아니라 뭘 얼마나 어떻게 해야 하는지를 계속 보이게 만들어준다는 점이었어요.</v>
@@ -12257,7 +12257,7 @@
         <v>불안했던 저를 안심시켜주시고 친절하게 뭐든 알려주셨습니다!!! 특히 국어 부분에서 모르는 것을 물어보면서 약점들을 바로 잡을 수 있었고, 의지도 많이 되었던 것 같습니다. 친근하신 인상이셔서 물어보기도 쉬웠던 것 겉습니다</v>
       </c>
       <c r="F328" t="str">
-        <v>국어 같은 경우, 답지만 보고 스스로 이해하기는 추상적인 경우가 많은데 1대1 질의응답을 통해 이런 문제점들을 해결할 수 있었고, 언매 같은 경우 모르는 것을 질문하면서 추가로 알아야할 개념까지 설명해주셔서 더 도움이 되었던 것 같습니다</v>
+        <v>국어 같은 경우, 답지만 보고 스스로 이해하기는 추상적인 경우가 많은데 1대1 질의응답을 통해 이런 문제점들을 해결할 수 있었고, 언매 같은 경우 모르는 것을 질문하면서 추가로 알아야할 개념까지 설명해 주셔서 더 도움이 되었던 것 같습니다</v>
       </c>
       <c r="G328" t="str">
         <v>귀찮게 출결 때 자리에 안 앉아있어도 되고, 등원했을 때 카드만 딱 찍으면 되서 시간 절약도 장점이라면 장점인 것 같습니다. 또한 이러한 절약을 통해 공부 시간을 더 확보해 빠른 시간안에 공부에 몰입할 수 있었습니다</v>
@@ -12301,7 +12301,7 @@
         <v>제공된 콘텐츠 중에서는 단어 단어 테스트와 이투스 모의고사가 특히 유용했습니다. 단어 테스트를 통해 어휘를 반복적으로 점검하며 암기 효과를 높일 수 있었고, 이투스 모의고사를 통해 실제 시험과 유사한 환경에서 자신의 실력을 확인하고 부족한 부분을 파악할 수 있었습니다. 이러한 콘텐츠들이 학습의 방향을 잡고 실력을 향상시키는 데 큰 도움이 되었습니다.</v>
       </c>
       <c r="I329" t="str">
-        <v>이투스247학원 선생님들께 진심으로 감사의 말씀을 전해드립니다. 항상 학생들의 학습과 생활을 세심하게 살펴주시고, 힘들 때마다 따뜻하게 상담해 주셔서 큰 힘이 되었습니다. 덕분에 흔들리지 않고 꾸준히 공부할 수 있었으며, 스스로를 관리하는 능력도 많이 성장할 수 있었습니다. 앞으로도 선생님들께서 해주신 지도와 응원을 잊지 않고 더욱 노력하겠습니다. 진심으로 감사합니다.</v>
+        <v>이투스247학원 선생님들께 진심으로 감사의 말씀을 전해드립니다. 항상 학생들의 학습과 생활을 세심하게 살펴주시고, 힘들 때마다 따뜻하게 상담해 주셔서 큰 힘이 되었습니다. 덕분에 흔들리지 않고 꾸준히 공부할 수 있었으며, 스스로를 관리하는 능력도 많이 성장할 수 있었습니다. 앞으로도 선생님들께서 해 주신 지도와 응원을 잊지 않고 더욱 노력하겠습니다. 진심으로 감사합니다.</v>
       </c>
       <c r="J329" t="str">
         <v>학습 관리 시스템은 학습 중 딴짓을 하지 않도록 환경을 만들어 주어 집중력을 유지하는 데 큰 도움이 되었어요.</v>
@@ -12336,7 +12336,7 @@
         <v>이투스 패스 증정은 학습의 폭을 넓히는 데 큰 도움이 되었습니다. 다양한 과목과 수준별 강의를 자유롭게 선택해 들을 수 있어 부족한 부분을 보완하기에 매우 효율적이었고, 필요에 따라 여러 강사의 강의를 비교하며 자신에게 맞는 수업을 찾을 수 있었습니다. 또한 추가 비용 부담 없이 양질의 인강을 활용할 수 있어 경제적인 측면에서도 만족도가 높았고, 전반적인 학습 효율을 높이는 데 큰 도움이 되었습니다.</v>
       </c>
       <c r="I330" t="str">
-        <v>수험 기간 동안 아낌없는 지원과 세심한 지도를 해주셔서 진심으로 감사드립니다. 학습뿐만 아니라 생활 관리와 입시 상담까지 전반적으로 도움을 주신 덕분에 끝까지 흔들리지 않고 목표를 향해 나아갈 수 있었습니다. 항상 학생의 입장에서 생각해주시고 응원해주셔서 큰 힘이 되었으며, 그 덕분에 좋은 결과를 얻을 수 있었습니다. 다시 한 번 깊이 감사드립니다.</v>
+        <v>수험 기간 동안 아낌없는 지원과 세심한 지도를 해 주셔서 진심으로 감사드립니다. 학습뿐만 아니라 생활 관리와 입시 상담까지 전반적으로 도움을 주신 덕분에 끝까지 흔들리지 않고 목표를 향해 나아갈 수 있었습니다. 항상 학생의 입장에서 생각해 주시고 응원해 주셔서 큰 힘이 되었으며, 그 덕분에 좋은 결과를 얻을 수 있었습니다. 다시 한 번 깊이 감사드립니다.</v>
       </c>
       <c r="J330" t="str">
         <v>비용 부담 없이 원하는 인강을 수강하도록 이투스 구독권을 무료로 제공해 주셔서 감사했습니다.</v>
@@ -12373,7 +12373,7 @@
       </c>
       <c r="I331" t="str" xml:space="preserve">
         <v xml:space="preserve">은애쌤, 감사합니다!!!!! _x000d_
-이걸 보실지는 모르겠지만 항상 한결같은 모습으로 저를 상담해주시고, 상담 외에도 엄마같은 느낌으로 저를 격려해주시고 응원해주셔서 감사합니다 _x000d_
+이걸 보실지는 모르겠지만 항상 한결같은 모습으로 저를 상담해 주시고, 상담 외에도 엄마같은 느낌으로 저를 격려해 주시고 응원해 주셔서 감사합니다 _x000d_
 그리고 매달 신경써주셔서 감사합니다ㅠ _x000d_
 덕분에 열심히 할 수 있었어요! _x000d_
 조만간 찾아갈게요!!!~</v>
@@ -12411,10 +12411,10 @@
         <v>목동 이투스 247점에서는 단어테스트반을 모집하여 매주 영단어 테스트를 봅니다. 학생들이 가장 귀찮아하고 소홀히하는 영단어 외우기를 같은 학생들과 함께 매주 테스트를 보며 매주 빼먹지 않게 외우게된다는 장점이 있습니다.</v>
       </c>
       <c r="I332" t="str">
-        <v>항상 입시 스트레스로와 몸 건강으로 인해 학원에게 피해를 많이 끼쳤지만 그럼에도 불구하고 항상 격려해주시고 힘을 내게 도와주셔서 덕분에 끝까지 입시를 마칠 수 있었습니다. 모두 선생님들 덕분입니다. 제 입시에서 이투스 247 선생님들을 만난것이 가장 큰 행운이였습니다 감사합니다..!</v>
+        <v>항상 입시 스트레스로와 몸 건강으로 인해 학원에게 피해를 많이 끼쳤지만 그럼에도 불구하고 항상 격려해 주시고 힘을 내게 도와주셔서 덕분에 끝까지 입시를 마칠 수 있었습니다. 모두 선생님들 덕분입니다. 제 입시에서 이투스 247 선생님들을 만난것이 가장 큰 행운이였습니다 감사합니다..!</v>
       </c>
       <c r="J332" t="str">
-        <v>매너 타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다 같이 집중할 수 있는 공부 환경을 제공해주셨어요.</v>
+        <v>매너 타임이라는 시스템을 통해 특정 시간대에 자습실에서 학생들의 이동 소음에 신경 쓰이지 않고 다 같이 집중할 수 있는 공부 환경을 제공해 주셨어요.</v>
       </c>
       <c r="K332" t="str">
         <v/>
@@ -12434,16 +12434,16 @@
         <v>N수생</v>
       </c>
       <c r="E333" t="str">
-        <v>학습과정에 있어서 불편하거나 막히는 부분이 있을 때마다 말씀드리면 항상 빠르게 수용해주시고 상황에 맞춰 자세하고 친절하게 상담해주셨습니다. 그래서 이후 학습을 더욱 편안하고 효율적으로 진행할수 있었고 덕분에 학습에 대한 부담도 줄어들었습니다</v>
+        <v>학습과정에 있어서 불편하거나 막히는 부분이 있을 때마다 말씀드리면 항상 빠르게 수용해 주시고 상황에 맞춰 자세하고 친절하게 상담해주셨습니다. 그래서 이후 학습을 더욱 편안하고 효율적으로 진행할수 있었고 덕분에 학습에 대한 부담도 줄어들었습니다</v>
       </c>
       <c r="F333" t="str">
-        <v>저는 제 상태도 모르고 아는 내용을 반복적으로 강의 시청만 했었는데, 이 부분에 대해서 담임 선생님께서 확실하게 해야 될 것과 과감하게 버려야 할 부분을 정해주셔서 학습 속도와 효율성이 높아진 것 같습니다.</v>
+        <v>저는 제 상태도 모르고 아는 내용을 반복적으로 강의 시청만 했었는데, 이 부분에 대해서 담임 선생님께서 확실하게 해야 될 것과 과감하게 버려야 할 부분을 정해 주셔서 학습 속도와 효율성이 높아진 것 같습니다.</v>
       </c>
       <c r="G333" t="str">
         <v>저는 평소에 전자기기가 있으면 공부에 집중을 하지 못하는 타입인데, 이곳에서는 강제적으로 휴대폰을 사용하지 못하니 자투리 시간이나 식사 시간에 쪽잠을 자거나 산책하며 휴식을 취하는 등 건강한 생활을 하게되어 훨씬 좋았던 것 같습니다.</v>
       </c>
       <c r="H333" t="str">
-        <v>평소에 영단어를 무작정 암기하기만 하고 따로 테스트를 보지 않았었는데, 이투스247 학원에서는 따로 매일매일 테스트 용지를 제공해주셔서 정말로 내가 암기를 한건지 아닌지 위치를 확실하게 알 수 있어서 유용했습니다.</v>
+        <v>평소에 영단어를 무작정 암기하기만 하고 따로 테스트를 보지 않았었는데, 이투스247 학원에서는 따로 매일매일 테스트 용지를 제공해 주셔서 정말로 내가 암기를 한건지 아닌지 위치를 확실하게 알 수 있어서 유용했습니다.</v>
       </c>
       <c r="I333" t="str">
         <v>선생님들의 따뜻한 관심과 미소 덕분에 공부하는게 덜 힘들었던 것 같습니다. 학습하는데 있어 사소한 불편사항도 바로 들어주셔서 너무 좋았어요.. 덕분에 정말 편한 환경에서 공부하게 된 것 같습니다 정말 감사했습니당 ㅎㅎ</v>
@@ -12469,7 +12469,7 @@
         <v>N수생</v>
       </c>
       <c r="E334" t="str">
-        <v>선생님들이 과목별로 다르게 저한테 맞는 공부법을 알려주셨습니다. 선생님 본인의 수험 생활에서 효과를 보셨던 방법들부터 선배님들의 방법까지 소개해주셔서 도움이 많이 됐습니다. 학습 뿐만아니라 생활부분에서도 힘든 점이나 어려운 점이 있으면 쉽게 말할 수 있는 분위기여서 학원 생활에 있어 큰 어려움은 없었습니다. 선생님들 덕분에 수월한 수험 생활을 한 것 같습니다.</v>
+        <v>선생님들이 과목별로 다르게 저한테 맞는 공부법을 알려주셨습니다. 선생님 본인의 수험 생활에서 효과를 보셨던 방법들부터 선배님들의 방법까지 소개해 주셔서 도움이 많이 됐습니다. 학습 뿐만아니라 생활부분에서도 힘든 점이나 어려운 점이 있으면 쉽게 말할 수 있는 분위기여서 학원 생활에 있어 큰 어려움은 없었습니다. 선생님들 덕분에 수월한 수험 생활을 한 것 같습니다.</v>
       </c>
       <c r="F334" t="str">
         <v>매달 정기고사나 모의고사가 끝나면 필수로 해야하는 상담이 있었는데 결과가 좋든 좋지 않든 선생님께서 편안하게 상담을 진행해주셨고, 잘 한 부분은 아낌없는 칭찬과 아쉬운 부분은 어떻게 해결해나가야하는지에 대해 보완점도 제시해 주셔서 유용했습니다.</v>
@@ -12481,7 +12481,7 @@
         <v>원내에서 자신의 위치, 전국단위에서의 자신의 위치를 확인할 수 있어서 위치파악에 유용했고, 매달 정기고사가 있다는 점 자체에 긴장감을 심어주어 공부에 자극이 되고 다음번에는 더 좋은 성적을 받아야 되겠다는 원동력이 되기도 했습니다.</v>
       </c>
       <c r="I334" t="str">
-        <v>선생님들! 수험 생활 내내 옆에서 정신적 지지를 해주셔서 감사합니다. 선생님들이 있어서 지루하고 무료했던 제 수험 생활이 조금이나마 즐거웠던 것 같습니다. 항상 생각했던 건데 저는 다시 돌아가도 꼳 이투스 독학 기숙을 선택할 것 같습니다.</v>
+        <v>선생님들! 수험 생활 내내 옆에서 정신적 지지를 해 주셔서 감사합니다. 선생님들이 있어서 지루하고 무료했던 제 수험 생활이 조금이나마 즐거웠던 것 같습니다. 항상 생각했던 건데 저는 다시 돌아가도 꼳 이투스 독학 기숙을 선택할 것 같습니다.</v>
       </c>
       <c r="J334" t="str">
         <v>과목별로 공부 방법을 추천해 주셨는데 저와 너무 잘 맞아서 성적 올리는 데 도움이 됐어요.</v>
@@ -12516,7 +12516,7 @@
         <v>학력평가나 모의평가를 시행하지 않는 달에 이투스 모의고사로 나의 실력을 점검할 수 있는 기회를 주어 현재 나의 상황을 점검하고 앞으로의 공부 계획을 세울 수 있도록 도와주어서 좋았던 것 같다.</v>
       </c>
       <c r="I335" t="str">
-        <v>선생님들 안녕하세요! 오랜만에 이렇게 후기를 남기면서 인사드립니다. 사실 학원 들어올 때까지만 해도 지방대 공대에 다니고 있어서 잘해봐야 국숭세단 정도 갈 줄 알았는데 학원에와서 5개월 정도 공부하고 이제는 제가 중앙대에 다니고 있네요. 이게 다 저를 잘 캐어해주신 선생님들 덕분인 듯 합니다. 정말 감사드려요!</v>
+        <v>선생님들 안녕하세요! 오랜만에 이렇게 후기를 남기면서 인사드립니다. 사실 학원 들어올 때까지만 해도 지방대 공대에 다니고 있어서 잘해봐야 국숭세단 정도 갈 줄 알았는데 학원에와서 5개월 정도 공부하고 이제는 제가 중앙대에 다니고 있네요. 이게 다 저를 잘 캐어해 주신 선생님들 덕분인 듯 합니다. 정말 감사드려요!</v>
       </c>
       <c r="J335" t="str">
         <v>데일리 테스트를 실시해 취약한 과목에 대하여 어떻게 풀면 좋을지 감을 잡을 수 있었어요.</v>
@@ -12574,7 +12574,7 @@
         <v>반수생</v>
       </c>
       <c r="E337" t="str">
-        <v>선생님께서 공부를 전체적으로 어떤 방식으로 해나가야하는지 계속해서 조언해주셔서 도움아 돠었습니다.또 모의고사를 본 후 선생님께서 개선해야 할점을 알려주신점도 도움이 많이 되었습니다.어떤부분에 대해 내가 약하고 어떤 부분에서 실수가 계속해서 일어나는지 알게 되고 고치게 도움을 많이 주십니다</v>
+        <v>선생님께서 공부를 전체적으로 어떤 방식으로 해나가야하는지 계속해서 조언해 주셔서 도움아 돠었습니다.또 모의고사를 본 후 선생님께서 개선해야 할점을 알려주신점도 도움이 많이 되었습니다.어떤부분에 대해 내가 약하고 어떤 부분에서 실수가 계속해서 일어나는지 알게 되고 고치게 도움을 많이 주십니다</v>
       </c>
       <c r="F337" t="str">
         <v>인터넷강의의 가장 큰 단점은 커리가 너무 많다는점인데 선생님과 상담후 나에게 딱 맞는 강의를 수강하는데 도움이 많이 되었습니다.반수생이었던 저는 시간이 부족해 선택과 집중이 되게 중요했는데 선생님의 도움이 없었더라면 혼자 방황했을꺼 같습니다.</v>
@@ -12621,10 +12621,10 @@
         <v>이투스247에서 제공하는 VOCA 콘텐츠를 통해 꾸준하고 접근성 편한 영어 단어 공부를 이어갈 수 있었습니다. 사실 영어라는 과목이 수능에서 차지하는 비중이 적다보니 선뜻 공부할 마음이 생기지 않을 때도 있고, 지속적인 학습이 어렵습니다. 하지만 이투스247의 VOCA 콘텐츠 덕분에 영어 학습을 저의 학습 루틴에 포함시키고 꾸준하게 영어 실력을 키워나갈 수 있었기에 매우 유용했습니다.</v>
       </c>
       <c r="I338" t="str">
-        <v>끝나지 않을 것 같던 수험 생활도 어느새 끝이 나고 그렇게 바라던 약학대학에 입학해 즐겁게 다니고 있습니다. 이투스247 학원의 선생님들께서 진심으로 임해주신 덕분이라고 언제나 생각합니다. 제 인생에서 잊을 수 없는 한 페이지가 될 것 같아요. 정말 감사했습니다!</v>
+        <v>끝나지 않을 것 같던 수험 생활도 어느새 끝이 나고 그렇게 바라던 약학대학에 입학해 즐겁게 다니고 있습니다. 이투스247 학원의 선생님들께서 진심으로 임해 주신 덕분이라고 언제나 생각합니다. 제 인생에서 잊을 수 없는 한 페이지가 될 것 같아요. 정말 감사했습니다!</v>
       </c>
       <c r="J338" t="str">
-        <v>학습 상담 외에도 생활, 멘탈 관련 상담도 해주셔서 단단해진 마음으로 공부에 임할 수 있었어요.</v>
+        <v>학습 상담 외에도 생활, 멘탈 관련 상담도 해 주셔서 단단해진 마음으로 공부에 임할 수 있었어요.</v>
       </c>
       <c r="K338" t="str">
         <v>학습 관리</v>
@@ -12644,10 +12644,10 @@
         <v>재학생(고3)</v>
       </c>
       <c r="E339" t="str">
-        <v>모의고사 성적을 바탕으로 지원 가능한 대학을 설명해주셨는데 구체적으로 지금 성적에서 몇 점, 몇 문제만 더 맞으면 학교 라인을 높일 수 있다고 말씀해주셔서 더욱 동기부여를 받고 열심히 공부할 수 있는 계기가 되었던 것 같습니다</v>
+        <v>모의고사 성적을 바탕으로 지원 가능한 대학을 설명해주셨는데 구체적으로 지금 성적에서 몇 점, 몇 문제만 더 맞으면 학교 라인을 높일 수 있다고 말씀해 주셔서 더욱 동기부여를 받고 열심히 공부할 수 있는 계기가 되었던 것 같습니다</v>
       </c>
       <c r="F339" t="str">
-        <v>국영수탐구 뿐만 아니라 논술 전형 응시 예정이었어서 특정 학교 논술 관련해서 궁금한 점을 여쭤본 적이 있었는데 선생님께서 저에게 도움이 될 수 있는 답변을 해주셔서 실제로 논술을 준비하는 과정에서 도움이 되었던 경험이 있습니다</v>
+        <v>국영수탐구 뿐만 아니라 논술 전형 응시 예정이었어서 특정 학교 논술 관련해서 궁금한 점을 여쭤본 적이 있었는데 선생님께서 저에게 도움이 될 수 있는 답변을 해 주셔서 실제로 논술을 준비하는 과정에서 도움이 되었던 경험이 있습니다</v>
       </c>
       <c r="G339" t="str">
         <v>아무래도 스카 혹은 집에서 독학 재수를 하는 경우에는 휴대폰을 가끔은 보게 되어 온전히 집중하지 못하는 경우가 많은데 이투스에서는 등원하면서 휴대폰을 제출해서 하루종일 공부와 해야 할 일에만 집중할 수 있었다는 점이 좋았습니다</v>
@@ -12656,7 +12656,7 @@
         <v>타사 인강들만 사용하고 있었어서 이투스 강의를 듣지 못하는 점이 아쉬웠었는데 구독을 통해서 이투스에서만 들을 수 있는 선생님들의 강의를 필요할 때마다 수강할 수 있었다는 점이 학습적인 측면에서 매우 좋았던 것 같습니다</v>
       </c>
       <c r="I339" t="str">
-        <v>학교 끝나자마자 이투스에 와서 공부하는 생활이 마냥 쉽지만은 않았고 체력적, 정신적으로 힘든 순간이 많았는데 상담 실장님, 부원장님께서 항상 좋은 말씀만 해주시고 신경써주셔서 끝까지 학원 다니면서 합격이라는 결과까지 낼 수 있었던 같습니다 ㅠㅠ !! 저에게는 이투스 다니는게 나름 소소한 행복이고 낙이었어서 진심으로 감사하다는 말씀 드리고 싶습니다 🥹☺️</v>
+        <v>학교 끝나자마자 이투스에 와서 공부하는 생활이 마냥 쉽지만은 않았고 체력적, 정신적으로 힘든 순간이 많았는데 상담 실장님, 부원장님께서 항상 좋은 말씀만 해 주시고 신경써주셔서 끝까지 학원 다니면서 합격이라는 결과까지 낼 수 있었던 같습니다 ㅠㅠ !! 저에게는 이투스 다니는게 나름 소소한 행복이고 낙이었어서 진심으로 감사하다는 말씀 드리고 싶습니다 🥹☺️</v>
       </c>
       <c r="J339" t="str">
         <v>논술을 준비하고 있었는데 선생님께서 궁금한 것들을 세세하게 알려주셔서 도움이 됐어요.</v>
@@ -12691,7 +12691,7 @@
         <v>혼자서 단어를 외우려고 하다보면 의지 부족으로 루틴이 꾸준히 이어지지 못하는데, 학원에서는 일괄적으로 단어 시험을 봐서 단어를 외우는 습관을 들일 수 있었다. 매일 영단어를 외우고 시험보고, 또 반복하다 보니 확실하게 영단어를 습득할 수 있었다.</v>
       </c>
       <c r="I340" t="str">
-        <v>약 10개월 간 잘 지도해주신 덕에 수능에서 좋은 결과를 얻을 수 있었습니다. 덕분에 지금 간 대학에 만족하며 잘 다니고 있습니다ㅎㅎ 아낌없는 조언 해주시고 좋은 공부 습관과 생활 습관을 만들어주셔서 감사합니다!</v>
+        <v>약 10개월 간 잘 지도해 주신 덕에 수능에서 좋은 결과를 얻을 수 있었습니다. 덕분에 지금 간 대학에 만족하며 잘 다니고 있습니다ㅎㅎ 아낌없는 조언 해 주시고 좋은 공부 습관과 생활 습관을 만들어주셔서 감사합니다!</v>
       </c>
       <c r="J340" t="str">
         <v>선생님들이 면학 분위기를 꼼꼼하게 관리하시기 때문에 학원에 있는 동안 공부에만 집중할 수 있었어요.</v>
@@ -12762,7 +12762,7 @@
         <v>이투스 모의고사를 통해 나의 현재 위치를 객관적으로 파악할 수 있었고 부족한 부분을 확인해 보완할 수 있었다. 이를 바탕으로 앞으로의 공부 방향을 보다 구체적으로 설정하는 데 도움이 되었다.</v>
       </c>
       <c r="I342" t="str">
-        <v>이투스 247 선생님들께 진심으로 감사드립니다. 항상 학생 한 명 한 명을 세심하게 지도해주시고 힘든 순간마다 따뜻한 조언과 격려로 큰 힘이 되어주셨습니다. 덕분에 흔들리지 않고 끝까지 공부할 수 있었고 더 나은 방향으로 나아갈 수 있었습니다. 감사합니다.</v>
+        <v>이투스 247 선생님들께 진심으로 감사드립니다. 항상 학생 한 명 한 명을 세심하게 지도해 주시고 힘든 순간마다 따뜻한 조언과 격려로 큰 힘이 되어주셨습니다. 덕분에 흔들리지 않고 끝까지 공부할 수 있었고 더 나은 방향으로 나아갈 수 있었습니다. 감사합니다.</v>
       </c>
       <c r="J342" t="str">
         <v>면학 분위기 감독과 졸음 관리는 학습 집중도를 유지하는 데 큰 도움이 되었어요.</v>
@@ -12837,7 +12837,7 @@
 또한 혼자 공부할 경우 약점 과목 시험을 피하게 되는 경향이 있는데, 일일 테스트를 통해 전 과목을 균형 있게 점검할 수 있어 약점은 보완하고 강점은 더욱 강화할 수 있었습니다.</v>
       </c>
       <c r="I344" t="str" xml:space="preserve">
-        <v xml:space="preserve">재수 생활을 돌아보면, 혼자였다면 끝까지 버틸 수 있었을까 싶을 만큼 선생님들께서 항상 곁에서 든든한 조력자가 되어주셨습니다. 학생들이 최상의 환경에서 학습에 몰두할 수 있도록 세심하게 지원해주신 점에 깊이 감사드립니다._x000d_
+        <v xml:space="preserve">재수 생활을 돌아보면, 혼자였다면 끝까지 버틸 수 있었을까 싶을 만큼 선생님들께서 항상 곁에서 든든한 조력자가 되어주셨습니다. 학생들이 최상의 환경에서 학습에 몰두할 수 있도록 세심하게 지원해 주신 점에 깊이 감사드립니다._x000d_
 또한 공부 중 답답함이나 고민이 생길 때마다 꼼꼼하게 살펴주시고, 실질적으로 도움이 되는 조언을 아끼지 않으셔서 지치지 않고 끝까지 학습을 이어갈 수 있었습니다.</v>
       </c>
       <c r="J344" t="str">
@@ -12945,7 +12945,7 @@
         <v>N수생</v>
       </c>
       <c r="E347" t="str">
-        <v>상담이 필요할때마다 상담을 최대한 빠르게 응해주신 점이 좋았습니다. 모의고사를 본 후에 최대한 빠른 시간에 모의고사를 직접 검토해주시고 아직 부족한 점이나 채워야할 점들을 피드백해주셔서 좋았습니다. 또 모의고사와 플래너를 함께 피드백해주셔서 앞으로의 방향을 가르쳐주신 점이 도움이 되었습니다. 상담을 하면서 가지고 있는 고민이나 생활 습관 같은 사소한 것들도 마음 편하게 얘기할 수 있어서 외로운 수험 생활동안 학원에서만큼이라도 공부에만 집중할 수 있었던 것 같습니다.</v>
+        <v>상담이 필요할때마다 상담을 최대한 빠르게 응해 주신 점이 좋았습니다. 모의고사를 본 후에 최대한 빠른 시간에 모의고사를 직접 검토해 주시고 아직 부족한 점이나 채워야할 점들을 피드백해 주셔서 좋았습니다. 또 모의고사와 플래너를 함께 피드백해 주셔서 앞으로의 방향을 가르쳐주신 점이 도움이 되었습니다. 상담을 하면서 가지고 있는 고민이나 생활 습관 같은 사소한 것들도 마음 편하게 얘기할 수 있어서 외로운 수험 생활동안 학원에서만큼이라도 공부에만 집중할 수 있었던 것 같습니다.</v>
       </c>
       <c r="F347" t="str">
         <v>독학재수에서의 가장 큰 단점이 자신이 어느정도까지 공부를 했는지, 어느정도에 위치해 있는지, 어떤 점이 잘못되었는지 를 스스로 알아차리기 힘든 것인데, 성적 레포팅과 피드백을 거치면서 내가 어떤 잘못된 공부 방법을 가지고 있는지 내가 이때까지 성장했는지를 제 3자의 눈으로 볼 수 있었다는 점이 가장 좋았습니다.</v>
@@ -12980,10 +12980,10 @@
         <v>N수생</v>
       </c>
       <c r="E348" t="str">
-        <v>담임 선생님께서 상담하실 때 마다 각 과목 별 공부가 어떻게 진행되고 있는지 구체적으로 상담해주시고(예를 들면 어떤 인강을 듣고 있는지, 또는 어떤 문제집을 풀고 있는지) 해당 내용이 끝난 다음에는 어떤 커리큘럼을 밟으면 좋은지 상담해주시는 등 구체적인 공부방향 설정에 큰 도움을 주셨습니다.</v>
+        <v>담임 선생님께서 상담하실 때 마다 각 과목 별 공부가 어떻게 진행되고 있는지 구체적으로 상담해 주시고(예를 들면 어떤 인강을 듣고 있는지, 또는 어떤 문제집을 풀고 있는지) 해당 내용이 끝난 다음에는 어떤 커리큘럼을 밟으면 좋은지 상담해주시는 등 구체적인 공부방향 설정에 큰 도움을 주셨습니다.</v>
       </c>
       <c r="F348" t="str">
-        <v>플래너를 주기적으로 검사함을 통해 하루에 몇 시간 정도 공부하는지 또 과목별로 균형 있게 학습하고 있는 지를 확인해 주시고 그에 따라 학습 피드백을 해주시는 것이 좋았습니다. 또 상담을 통해 또는 스스로 세운 계획을 얼마나 잘 지키고 있는지 점검함을 통해 학습 관리를 잘 해주신 부분이 좋았습니다.</v>
+        <v>플래너를 주기적으로 검사함을 통해 하루에 몇 시간 정도 공부하는지 또 과목별로 균형 있게 학습하고 있는 지를 확인해 주시고 그에 따라 학습 피드백을 해주시는 것이 좋았습니다. 또 상담을 통해 또는 스스로 세운 계획을 얼마나 잘 지키고 있는지 점검함을 통해 학습 관리를 잘 해 주신 부분이 좋았습니다.</v>
       </c>
       <c r="G348" t="str">
         <v>담임 선생님들이 주기적으로 면학 분위기 조성에 힘쓰시는 것이 느껴졌습니다. 일단 오전, 오후마다 선생님들이 졸고 있는 학생들을 깨우셨고 휴가 전후로 전체적으로 분위기가 헤이해지면 더 강하게 면학 분위기 관리에 힘을 쓰셨습니다. 덕분에 분위기에 휩쓸리지 않고 공부할 수 있어서 좋았습니다.</v>
@@ -13140,9 +13140,9 @@
 _x000d_
 아마도 가장 많이 질문하러 갔던 덕곤쌤, 무시하지 않고 늦게까지 남아 어떤 질문이든 받아주셔서 감사합니다._x000d_
 _x000d_
-매주 상담하며 끝까지 믿어주신 재현쌤, 합격 전부터 응원해주시고 합격증 보내드렸을 때 진심으로 축하해주셔서 감사합니다._x000d_
+매주 상담하며 끝까지 믿어주신 재현쌤, 합격 전부터 응원해 주시고 합격증 보내드렸을 때 진심으로 축하해 주셔서 감사합니다._x000d_
 _x000d_
-그리고 마지막으로 가장 많은 시간 함께한 단비쌤, 컨디션이 좋지 않거나 아플 때 편의를 봐주셨던 것 외에도 생활전반을 책임져주셔서 감사합니다. 수능 전 주에 육사 합격했을 때 같이 축하해주셔서 감사해요. 정말 큰 힘이 됐습니다.</v>
+그리고 마지막으로 가장 많은 시간 함께한 단비쌤, 컨디션이 좋지 않거나 아플 때 편의를 봐주셨던 것 외에도 생활전반을 책임져주셔서 감사합니다. 수능 전 주에 육사 합격했을 때 같이 축하해 주셔서 감사해요. 정말 큰 힘이 됐습니다.</v>
       </c>
       <c r="J352" t="str">
         <v>처음 상담 받으러 갔을 때부터 수능 전 마지막 모의고사 날까지 항상 관심을 가져주신 원장 선생님께 정말 감사했어요.</v>
@@ -13177,7 +13177,7 @@
         <v>객관적으로 스스로를 돌아볼 수 있는 기회가 되어 가장 좋았고, 그 외에도 시간 조절이나 시험지 운용과 같은 점에서도 여러 시뮬레이션을 해보고 가장 적합한 시험 방식을 찾아갈 수 있다는 점에서도 긍정적으로 작용했습니다.</v>
       </c>
       <c r="I353" t="str">
-        <v>군더더기 없이 딱 n수생에게 필요한 환경을 조성해 주시고, 그에 맞는 태도를 취해주셔서 더 감사했습니다! 평소에 다른 사람과 대화하는 것을 좋아하는 성격이라 너무 친화적인 분위기였다면 저에게 독이 되었을텐데, 쉬는 시간에는 적절하게 대화도 나눠주시고, 공부할 때는 딱 몰입할 수 있게 해주셨기에 좋은 성과를 낼 수 있었다고 생각합니다! 앞으로도 응원하겠습니다😊</v>
+        <v>군더더기 없이 딱 n수생에게 필요한 환경을 조성해 주시고, 그에 맞는 태도를 취해 주셔서 더 감사했습니다! 평소에 다른 사람과 대화하는 것을 좋아하는 성격이라 너무 친화적인 분위기였다면 저에게 독이 되었을텐데, 쉬는 시간에는 적절하게 대화도 나눠주시고, 공부할 때는 딱 몰입할 수 있게 해주셨기에 좋은 성과를 낼 수 있었다고 생각합니다! 앞으로도 응원하겠습니다😊</v>
       </c>
       <c r="J353" t="str">
         <v>학원에서 제가 필요로 하는 학습 자료를 찾아주셔서 시간을 효율적으로 활용할 수 있었어요.</v>
@@ -13212,7 +13212,7 @@
         <v>집에서 혼자 모의고사를 풀면 시간이나 방식을 제대로 지키지 않게 된다. 하지만 여기서는 모의고사 환경을 조성해줘 실제 수능을 보는듯한 마음가짐으로 모의고사를 볼 수 있었다. 또 성적이 나와 나의 대략적 위치를 파악하기가 용의했다.</v>
       </c>
       <c r="I354" t="str">
-        <v>힘들 때마다 응원해주셔서 감사합니다. 선생님들 덕분에 대학갈 수 있었어요!! 특히 공부하라고 따끔하게 한마디 해주신거 당시엔 너무너무 속상했는데 지금 생각하니 정말 좋은 동기부여였던 것 같아요 사랑합니다!!!</v>
+        <v>힘들 때마다 응원해 주셔서 감사합니다. 선생님들 덕분에 대학갈 수 있었어요!! 특히 공부하라고 따끔하게 한마디 해 주신거 당시엔 너무너무 속상했는데 지금 생각하니 정말 좋은 동기부여였던 것 같아요 사랑합니다!!!</v>
       </c>
       <c r="J354" t="str">
         <v>실제 수험장과 똑같은 환경으로 관리해 주셔서 실전처럼 매일 공부할 수 있었어요.</v>
@@ -13235,7 +13235,7 @@
         <v>반수생</v>
       </c>
       <c r="E355" t="str">
-        <v>개인적으로 몸이 좋지 않았는데 이를 배려를 정말 많이 해주셔서 에어컨 세기도 약하게 조절해주시고 룸메이트도 최대한 저랑 맞는 사람이랑 쓸 수 있도록 도와주셨습니다. 또한 교무실에 상비약이 배치되어 있어 가벼운 감기는 상비약을 먹으면서 회복하고 심한 감기일 때는 밖에 있는 병원에 갈 수 있어서 좋았습니다</v>
+        <v>개인적으로 몸이 좋지 않았는데 이를 배려를 정말 많이 해 주셔서 에어컨 세기도 약하게 조절해 주시고 룸메이트도 최대한 저랑 맞는 사람이랑 쓸 수 있도록 도와주셨습니다. 또한 교무실에 상비약이 배치되어 있어 가벼운 감기는 상비약을 먹으면서 회복하고 심한 감기일 때는 밖에 있는 병원에 갈 수 있어서 좋았습니다</v>
       </c>
       <c r="F355" t="str" xml:space="preserve">
         <v xml:space="preserve">평소 의욕만 앞서 무리하게 계획을 세우거나, 기분에 따라 학습량이 들쑥날쑥해지는 편이었습니다. 하지만 학원에서 제공하는 학습 계획 플래너 관리를 받으면서 공부의 질이 완전히 달라졌습니다._x000d_
@@ -13320,7 +13320,7 @@
         <v>솔직히 이투스모의고사는 사설이라서 그렇게 중요하지않겠지라는 생각으로 이투스모의고사를 생각했었는데 실제 재원생으로 이투스247을 다니면서 이투스모의고사가 제가 수능생활을 유지할수있게하는 큰 도움이 된것같습니다 아무래도 수능생활에서 6월9월모의고사 수능 이렇게 중요한모의고사는 3개라고 볼수 있는데 그 사이의 텀이 너무 긴데, 그 사이동안 긴장이 풀어지면서 해아해질수 있는 기간을 이투스모의고사가 적절히 그 기간동안 긴장의 끈을 놓지않게 텐션을 유지해주면서 나의 성적대가 지금 어느정도인지 내가 공부하고있는 지금 이 방향이 잘가고있는지 확인할수있게만든 중요한 이정표의 역할이 되었다고 생각합니다 그래서 이투스모의고사를 통해 수능때까지의 긴장의끈을 놓지않고 달리며 수능때좋은성적을 거뒀던것같습니다</v>
       </c>
       <c r="I357" t="str">
-        <v>늦은나이에 공부를 시작하느라 뭐가뭔지도 모르고 수능의기조가 어떤지도 몰랐는데 이튜스선생님들을 만나고 쓴소리와 격려의말을 들으면서 제가부족한점과 지금 고쳐야할점을 회피하지않고 직면하게되면서 지금 이 수험 생활에서 중요하게 뭔지 다시금 생각하게 해주셨고, 격려의 말을 통해 나라는 학생도 수능에서의 성공을 꿈꿀수 있는사람으로서 다시 생각하게해쥬셨던것같습니다 많이 모자랐는데도 그저 지나가는 학생이 아닌 정말 끌어서 제가원하는 목표를 이루게 하기위해 힘드실텐데도 본인들의 에너지를 써가면서 저를 설득하고 공부하게끔 다시도와주시는 모습을 수능끝나고 뼈저리게 감사한 마음을 느꼈던것같습니다 이투스247김포점에서 선생님들을 만나고 꿈을 이루게 된것에 너무 감사드리고 저를 지나가는 학생이 아니라 진심으로 대해주셔서 정말 감사합니다 덕분에 꿈을 이룬것같습니다 항상 행복하세요 선생님들 !❤️</v>
+        <v>늦은나이에 공부를 시작하느라 뭐가뭔지도 모르고 수능의기조가 어떤지도 몰랐는데 이튜스선생님들을 만나고 쓴소리와 격려의말을 들으면서 제가부족한점과 지금 고쳐야할점을 회피하지않고 직면하게되면서 지금 이 수험 생활에서 중요하게 뭔지 다시금 생각하게 해주셨고, 격려의 말을 통해 나라는 학생도 수능에서의 성공을 꿈꿀수 있는사람으로서 다시 생각하게해쥬셨던것같습니다 많이 모자랐는데도 그저 지나가는 학생이 아닌 정말 끌어서 제가원하는 목표를 이루게 하기위해 힘드실텐데도 본인들의 에너지를 써가면서 저를 설득하고 공부하게끔 다시도와주시는 모습을 수능끝나고 뼈저리게 감사한 마음을 느꼈던것같습니다 이투스247김포점에서 선생님들을 만나고 꿈을 이루게 된것에 너무 감사드리고 저를 지나가는 학생이 아니라 진심으로 대해 주셔서 정말 감사합니다 덕분에 꿈을 이룬것같습니다 항상 행복하세요 선생님들 !❤️</v>
       </c>
       <c r="J357" t="str">
         <v>담임 선생님께서 부족한 과목을 보완할 수 있는 교재를 추천해 주셨는데 잘 맞았어요!</v>
@@ -13355,7 +13355,7 @@
         <v>본인은 인터넷 강의 사이트에 고민이 많았는데,학원에 다니면 이투스로 강의를 들을 수 있다고 해서 듣게 되었습니다.덕분에 이투스강의로 정착을 하게됐고 과목별로 난이도와 단원을 고를 수 있어서 좋았습니다. 또한 듣고 싶은 강의를 마음껏 들을 수 있고 헷갈린 건 q&amp;a 창을 통해 물을 수 있어서 학습에 도움이 됐습니다.</v>
       </c>
       <c r="I358" t="str">
-        <v>항상 수업에 열심히 임하시고 가르치셔서 감사했어요.궁금한 점이나 헷갈린 걸 여쭤봐도 친절히 설명해주셔서 기억에 남습니다.여러모로 인생조언도 배웠습니다. 건강하시고 좋은 일만 가득하시길 바랍니다.</v>
+        <v>항상 수업에 열심히 임하시고 가르치셔서 감사했어요.궁금한 점이나 헷갈린 걸 여쭤봐도 친절히 설명해 주셔서 기억에 남습니다.여러모로 인생조언도 배웠습니다. 건강하시고 좋은 일만 가득하시길 바랍니다.</v>
       </c>
       <c r="J358" t="str">
         <v>학원에서 실행 가능한 계획을 세우도록 도와주고, 관리해 주셔서 공부에 도움이 많이 됐어요!</v>
@@ -13416,7 +13416,7 @@
         <v>커리큘럼을 선생님과 함께 구성할 수 있어 좋았고, 제가 몰랐던 문제집을 추천받을 수 있어 도움이 되었습니다. 또한 매달 실시하는 모의고사 성적을 바탕으로 상담을 진행하며, 현재 제 학습 상태를 객관적으로 파악하고 앞으로의 학습 방향을 설계할 수 있어 좋았습니다.</v>
       </c>
       <c r="F360" t="str">
-        <v>인강 수강 여부와 진도를 꾸준히 확인해주셔서 학습을 미루지 않고 계획대로 이어갈 수 있었습니다. 또한 수강 현황을 바탕으로 부족한 부분을 빠르게 파악해 보완할 수 있었고, 스스로 공부할 때보다 체계적으로 학습 방향을 유지하는 데 큰 도움이 되었습니다.</v>
+        <v>인강 수강 여부와 진도를 꾸준히 확인해 주셔서 학습을 미루지 않고 계획대로 이어갈 수 있었습니다. 또한 수강 현황을 바탕으로 부족한 부분을 빠르게 파악해 보완할 수 있었고, 스스로 공부할 때보다 체계적으로 학습 방향을 유지하는 데 큰 도움이 되었습니다.</v>
       </c>
       <c r="G360" t="str">
         <v>핸드폰을 걷는 환경이 조성되면서 불필요한 알림이나 SNS에 방해받지 않고 공부에 집중할 수 있었습니다. 이전보다 학습 몰입도가 높아졌고, 시간을 더 효율적으로 활용할 수 있었습니다. 또한 스스로 통제하기 어려웠던 사용 습관을 자연스럽게 개선하는 데에도 도움이 되었습니다.</v>
@@ -13425,7 +13425,7 @@
         <v>이투스 구독을 통해 다양한 강의를 자유롭게 선택해 들을 수 있어, 제 수준과 필요한 과목에 맞는 학습이 가능했습니다. 이해가 부족한 부분은 여러 강사의 설명을 비교하며 보완할 수 있었고, 최신 출제 경향이 반영된 강의를 통해 효율적으로 시험을 준비할 수 있어 큰 도움이 되었습니다.</v>
       </c>
       <c r="I360" t="str">
-        <v>선생님들께서 항상 세심하게 지도해주시고, 학습 방향을 잡아주신 덕분에 흔들리지 않고 끝까지 공부를 이어갈 수 있었습니다. 매달 진행된 상담과 피드백을 통해 제 현재 상태를 객관적으로 파악하고 부족한 부분을 보완할 수 있어 많은 도움이 되었습니다. 진심으로 감사드립니다.</v>
+        <v>선생님들께서 항상 세심하게 지도해 주시고, 학습 방향을 잡아주신 덕분에 흔들리지 않고 끝까지 공부를 이어갈 수 있었습니다. 매달 진행된 상담과 피드백을 통해 제 현재 상태를 객관적으로 파악하고 부족한 부분을 보완할 수 있어 많은 도움이 되었습니다. 진심으로 감사드립니다.</v>
       </c>
       <c r="J360" t="str">
         <v>매달 실시하는 모의고사를 통해 앞으로의 학습 방향을 선생님이 함께 설계해 주신 것이 좋았습니다.</v>
@@ -13460,7 +13460,7 @@
         <v>매일 일정한 시간에 단어 테스트를 보는 것도 좋았던 점이라고 생각합니다. 영어가 약한 편이라 단어를 외우는 게 항상 밀리거나 제대로 안 되는 경우가 많았는데, 매일 정해진 시간에 테스트를 보니까 어쩔 수 없이 계속 보게 되어서 도움이 됐습니다. 그냥 혼자 할 때는 미루게 되는 경우가 많았는데, 테스트가 있으니까 꾸준히 반복하게 되는 점이 좋았습니다.  또 한 번 보고 끝나는 게 아니라 틀린 단어를 다시 복습하게 되면서 자연스럽게 반복 학습이 되었습니다. 계속 같은 단어를 여러 번 보게 되니까 점점 익숙해지고, 예전보다 단어가 덜 부담스럽게 느껴졌습니다.  전체적으로 매일 단어 테스트를 통해 영어 공부를 꾸준히 이어갈 수 있었고, 약했던 부분을 조금씩 보완할 수 있어서 만족스러웠습니다.</v>
       </c>
       <c r="I361" t="str">
-        <v>데스크 선생님과 담임 선생님 모두 항상 웃는 얼굴로 대해주셔서 좋았습니다. 학원에 갈 때마다 밝게 인사해주시고 친절하게 대해주셔서 수험 생활 중에 작은 부분이지만 힘이 많이 됐습니다. 혼자 공부하다 보면 지치거나 기분이 다운될 때가 많은데, 그런 분위기 덕분에 조금이나마 편하게 다닐 수 있었던 것 같습니다.  또 중간에 성적이 잘 안 나오거나 공부가 잘 안 풀려서 낙담할 때도 있었는데, 그럴 때마다 항상 응원해주시고 괜찮다고 말해주셔서 다시 마음 잡는 데 도움이 됐습니다. 단순한 관리만 하는 게 아니라 학생 입장에서 이해해주시고 말해주시는 느낌이 들어서 더 의지가 됐습니다.  전체적으로 공부 환경뿐만 아니라 사람적인 부분에서도 도움을 많이 받았고, 그런 점들이 수험 생활을 버티는 데 큰 힘이 됐다고 생각합니다.</v>
+        <v>데스크 선생님과 담임 선생님 모두 항상 웃는 얼굴로 대해 주셔서 좋았습니다. 학원에 갈 때마다 밝게 인사해 주시고 친절하게 대해 주셔서 수험 생활 중에 작은 부분이지만 힘이 많이 됐습니다. 혼자 공부하다 보면 지치거나 기분이 다운될 때가 많은데, 그런 분위기 덕분에 조금이나마 편하게 다닐 수 있었던 것 같습니다.  또 중간에 성적이 잘 안 나오거나 공부가 잘 안 풀려서 낙담할 때도 있었는데, 그럴 때마다 항상 응원해 주시고 괜찮다고 말해 주셔서 다시 마음 잡는 데 도움이 됐습니다. 단순한 관리만 하는 게 아니라 학생 입장에서 이해해 주시고 말해주시는 느낌이 들어서 더 의지가 됐습니다.  전체적으로 공부 환경뿐만 아니라 사람적인 부분에서도 도움을 많이 받았고, 그런 점들이 수험 생활을 버티는 데 큰 힘이 됐다고 생각합니다.</v>
       </c>
       <c r="J361" t="str">
         <v>이투스247학원의 학습 계획이랑 플래너 관리도 도움이 많이 됐어요.</v>
@@ -13566,7 +13566,7 @@
 반복적인 테스트를 통해 실전에서 문장을 해석하는 속도가 비약적으로 빨라졌고, 이는 영어 성적을 안정적으로 유지하는 핵심 동력이 되었습니다. 스스로 공부했다면 자칫 소홀해질 수 있었던 어휘 학습을 매일 점검받으며 흔들림 없는 실력을 쌓을 수 있었던 점이 수험 생활 중 가장 유익했던 부분이었습니다.</v>
       </c>
       <c r="I363" t="str">
-        <v>중간중간 내가 최저를 못맞출까 불안했을때 선생님들이 끝까지 하면된다는 말을 들으며 끝까지 버틴 끝에 제가 원하던 최저를 맞춰 대학을 갈수있었던거 같아 끝까지 응원해주신 선생님들께 감사합니다!</v>
+        <v>중간중간 내가 최저를 못맞출까 불안했을때 선생님들이 끝까지 하면된다는 말을 들으며 끝까지 버틴 끝에 제가 원하던 최저를 맞춰 대학을 갈수있었던거 같아 끝까지 응원해 주신 선생님들께 감사합니다!</v>
       </c>
       <c r="J363" t="str">
         <v>눈치 보지 않고 모르는 문제를 바로 선생님께 질문해 해결할 수 있는 점이 정말 좋았습니다!</v>
@@ -13589,7 +13589,7 @@
         <v>N수생</v>
       </c>
       <c r="E364" t="str">
-        <v>처음 입소 당시 공부를 어디서부터 어떻게 해야 하는지 막막했는데 선생님께서 잘 알려주시고 이끌어주셔서 공부 방향을 잡게되고 중간에 흐트러지지 않게 지도해주셔서 성적 향상을 이룰 수 있어서 학습 코칭 시스템이 유용했다고 생각합니다</v>
+        <v>처음 입소 당시 공부를 어디서부터 어떻게 해야 하는지 막막했는데 선생님께서 잘 알려주시고 이끌어주셔서 공부 방향을 잡게되고 중간에 흐트러지지 않게 지도해 주셔서 성적 향상을 이룰 수 있어서 학습 코칭 시스템이 유용했다고 생각합니다</v>
       </c>
       <c r="F364" t="str">
         <v>6,9모 학원 모의고사를 정기적으로 보고 지원가능대학 라인을 확인함으로써 적당한 긴장감과 도전의식을 가지며 공부할 수 있었다고 생각해서 이 학습 관리 시스템이 유용했다고 생각이 되었습니다</v>
@@ -13601,7 +13601,7 @@
         <v>학원 내 모의고사를 봄으로써 내가 아는 것과 모르는 것 어중간하게 아는 것을 구분을 할 수 있어서 추후 학습 계획을 세우고 오답정리를 할 때 취약점을 빠르게 보완하고 성적 향상을 이룰 수 있게 해줘서 원내 모의고사가 좋았습니다</v>
       </c>
       <c r="I364" t="str" xml:space="preserve">
-        <v xml:space="preserve">2월부터 11월까지 잘 지도해주셔서 감사합니다 전역 후에 입시하느라 되게 막막하고 불안하고 했었는데 여기서 빡세게 공부해서 숭실대 잘 다니고 있어요_x000d_
+        <v xml:space="preserve">2월부터 11월까지 잘 지도해 주셔서 감사합니다 전역 후에 입시하느라 되게 막막하고 불안하고 했었는데 여기서 빡세게 공부해서 숭실대 잘 다니고 있어요_x000d_
 제 인생에서 인서울은 연이 아닌듯 싶었는데 정말 감사합니다 그리고 원내에서 계획표 쓰고 6시 기상하고 하는 시스템 지금도 스스로 잘 유지해서 요번에 한능검하고 사조사 2급 자격증 취득했어요 대입성공과 규칙적이고 계획적인 습관,도전의식도 기를 수 있었던 시간이라고 생각해요 감사합니다</v>
       </c>
       <c r="J364" t="str">
@@ -13672,11 +13672,11 @@
         <v>저는 이투스에서 정승제 선생님의 강의를 계속 수강했었는데, 다른 인강 교재들이나 강의도 다 듣고 있었기 때문에 반수를 하는 제 입장에서는 재정적인 부담도 어쩔 수 없이 있었습니다. 그런데 이투스를 다니면서 저한테 인강을 무료로 볼 수 있게 되어 부담도 적고 듣고 싶은 과목 골라 들을 수 있어서 좋았습니다.</v>
       </c>
       <c r="I366" t="str" xml:space="preserve">
-        <v xml:space="preserve">그동안 정말 감사했습니다~ 선생님들 덕분에 대학생활을 훨씬 더 즐겁고 의미 있게 보낼 수 있었던 것 같아요!! 중간중간 힘들 때도 많았고, 지치고 포기하고 싶었던 순간들도 있었지만, 그럴 때마다 항상 따뜻하게 대해주시고 친절하게 도와주셔서 끝까지 잘 버틸 수 있었던 것 같습니다._x000d_
+        <v xml:space="preserve">그동안 정말 감사했습니다~ 선생님들 덕분에 대학생활을 훨씬 더 즐겁고 의미 있게 보낼 수 있었던 것 같아요!! 중간중간 힘들 때도 많았고, 지치고 포기하고 싶었던 순간들도 있었지만, 그럴 때마다 항상 따뜻하게 대해 주시고 친절하게 도와주셔서 끝까지 잘 버틸 수 있었던 것 같습니다._x000d_
  늘 밝은 분위기로 맞아주시고 세심하게 신경 써주셔서 정말 감사했습니다.</v>
       </c>
       <c r="J366" t="str">
-        <v>주기적으로 학습 상담을 해주셔서 커리큘럼에 대한 고민 없이 공부에만 집중할 수 있었어요!</v>
+        <v>주기적으로 학습 상담을 해 주셔서 커리큘럼에 대한 고민 없이 공부에만 집중할 수 있었어요!</v>
       </c>
       <c r="K366" t="str">
         <v>학습 관리</v>
@@ -13708,7 +13708,7 @@
         <v>매일매일 VOCA 테스트를 통해 수능 중요 단어들을 매일매일 숙지하는 시간이 필수적으로 생겨서 좋았고, 영어듣기 테스트를 매일 진행하여 듣기를 소홀히 하지 못하도록 늘 영어 듣는 귀를 훈련시키는 시간이 매우 도움이 되었습니다.</v>
       </c>
       <c r="I367" t="str">
-        <v>늘 부족하고 잠도 많이 자고 서툴렀던 저에게 항상 친절하고 세세하게 설명해주시고 모르는 부분에 대해 물어보면 늘 친절하고 알기 쉽게 설명해주셔서 감사합니다. 또 마음이 지치고 힘들 때마다 항상 응원해주시고 북돋아주셔서 그 말들 덕분에 남은 하루를 버텼던 것 같습니다. 다시 한 번 감사합니다.</v>
+        <v>늘 부족하고 잠도 많이 자고 서툴렀던 저에게 항상 친절하고 세세하게 설명해 주시고 모르는 부분에 대해 물어보면 늘 친절하고 알기 쉽게 설명해 주셔서 감사합니다. 또 마음이 지치고 힘들 때마다 항상 응원해 주시고 북돋아주셔서 그 말들 덕분에 남은 하루를 버텼던 것 같습니다. 다시 한 번 감사합니다.</v>
       </c>
       <c r="J367" t="str">
         <v>개인별 담임 선생님이 계셔서 각자 어떤 방식으로 공부하는지 매주 확인하는 것이 좋은 시스템이었다고 생각해요.</v>
@@ -13731,7 +13731,7 @@
         <v>N수생</v>
       </c>
       <c r="E368" t="str">
-        <v>생활상담이 체계적으로 잘 이루어졌다는 점이 가장 큰 장점이라고 느꼈습니다. 단순히 공부만 관리해주는 것이 아니라, 개인적인 고민이나 스트레스, 진로에 대한 부분까지 편하게 이야기할 수 있어서 심리적으로 큰 안정감을 얻을 수 있었습니다. 선생님들께서 항상 친절하게 공감해주시고, 현실적이면서도 도움이 되는 조언을 해주셔서 혼자서 고민할 때보다 훨씬 방향을 잡기 수월했습니다. 또한 정기적인 상담을 통해 현재 상태를 점검하고 생활 습관이나 학습 태도를 개선할 수 있었던 점도 매우 좋았습니다. 이런 부분 덕분에 학원 생활에 잘 적응할 수 있었고, 전반적으로 공부에 더 집중할 수 있는 환경이 만들어졌다고 생각합니다.</v>
+        <v>생활상담이 체계적으로 잘 이루어졌다는 점이 가장 큰 장점이라고 느꼈습니다. 단순히 공부만 관리해주는 것이 아니라, 개인적인 고민이나 스트레스, 진로에 대한 부분까지 편하게 이야기할 수 있어서 심리적으로 큰 안정감을 얻을 수 있었습니다. 선생님들께서 항상 친절하게 공감해 주시고, 현실적이면서도 도움이 되는 조언을 해 주셔서 혼자서 고민할 때보다 훨씬 방향을 잡기 수월했습니다. 또한 정기적인 상담을 통해 현재 상태를 점검하고 생활 습관이나 학습 태도를 개선할 수 있었던 점도 매우 좋았습니다. 이런 부분 덕분에 학원 생활에 잘 적응할 수 있었고, 전반적으로 공부에 더 집중할 수 있는 환경이 만들어졌다고 생각합니다.</v>
       </c>
       <c r="F368" t="str">
         <v>1대1 질의응답 시스템을 선택한 이유는 모르는 내용을 바로 해결할 수 있어 학습 효율이 높았기 때문입니다. 수업 중 이해가 부족했던 부분이나 문제 풀이 과정에서 막힌 부분을 바로 질문하고 자세한 설명을 들을 수 있어서 이해도가 크게 향상되었습니다. 또한 개인 수준에 맞춰 설명해주시기 때문에 부담 없이 질문할 수 있었고, 부족한 점을 정확히 보완할 수 있어 공부에 큰 도움이 되었습니다.</v>
@@ -13743,7 +13743,7 @@
         <v>매일 꾸준히 학습 내용을 점검할 수 있었기 때문입니다. 하루 동안 공부한 내용을 바로 테스트를 통해 확인하면서 이해가 부족한 부분을 빠르게 파악하고 보완할 수 있었습니다. 또한 매일 시험이 있다는 긴장감 덕분에 자연스럽게 복습 습관이 형성되었고, 학습 리듬을 유지하는 데에도 큰 도움이 되었습니다. 이러한 반복적인 점검 과정이 실력 향상에 효과적이었다고 느꼈습니다.</v>
       </c>
       <c r="I368" t="str">
-        <v>진짜 기초도 거의없고 공부패턴도 안잡혀있었는데 매일 열심히 지도해주시고 격려도 해주셔서 내신8등급에서 영대까지 갔어요! 덕분에 공부뿐만아니라 많은것들을 바운것같아요 너무감사드립니다 선생님들 !!</v>
+        <v>진짜 기초도 거의없고 공부패턴도 안잡혀있었는데 매일 열심히 지도해 주시고 격려도 해 주셔서 내신8등급에서 영대까지 갔어요! 덕분에 공부뿐만아니라 많은것들을 바운것같아요 너무감사드립니다 선생님들 !!</v>
       </c>
       <c r="J368" t="str">
         <v>면학 분위기 감독 및 졸음 관리로 학습에 집중할 수 있는 환경이 잘 조성되어 있었어요.</v>
@@ -13766,7 +13766,7 @@
         <v>N수생</v>
       </c>
       <c r="E369" t="str">
-        <v>수시 원서 접수 상담 과정에서 다양한 자료를 제공받아 대학을 대학선택에 큰 도움을 받았고, 세 차례의 상담을 통해  학생에게 더 적합한 대학을 구체적으로 판단해주셔서 원서 접수를 보다 수월하게 진행할 수 있었습니다.</v>
+        <v>수시 원서 접수 상담 과정에서 다양한 자료를 제공받아 대학을 대학선택에 큰 도움을 받았고, 세 차례의 상담을 통해  학생에게 더 적합한 대학을 구체적으로 판단해 주셔서 원서 접수를 보다 수월하게 진행할 수 있었습니다.</v>
       </c>
       <c r="F369" t="str">
         <v>매달 한 번씩 진행된 상담을 통해 학습 과정에서의 고민을 해소할 수 있어 도움이 되었으며, 지속적인 상담으로 체계적인 케어를 받는다는 느낌을 받았습니다. 또한 플래너 관리를 통해 부족한 부분을 보완할 수 있었습니다.</v>
@@ -13778,7 +13778,7 @@
         <v>강남 지점에서는 밴드 미션을 통해 영단어 시험을 진행했는데 학습에 큰 도움이 되었습니다. 특히, 밴드 미션을 했을 때  상점을 부여하는 시스템이 꾸준한 학습을 유지하는 데 원동력이 되었습니다.</v>
       </c>
       <c r="I369" t="str">
-        <v>5월부터 시작해서 11월까지 공부하느라 힘든 순간도 많았었는데 아침마다 반갑게 인사해주시고 상담할 때마다 할 수 있다고 격려해주셔서 멘탈적으로 많은 도움이 되었습니다! 또 주기적으로 이벤트를 진행해주셔서 지루하지 않고 재밌게 학원을 다녔던 기억이 있습니다. 늘 감사합니다!!</v>
+        <v>5월부터 시작해서 11월까지 공부하느라 힘든 순간도 많았었는데 아침마다 반갑게 인사해 주시고 상담할 때마다 할 수 있다고 격려해 주셔서 멘탈적으로 많은 도움이 되었습니다! 또 주기적으로 이벤트를 진행해 주셔서 지루하지 않고 재밌게 학원을 다녔던 기억이 있습니다. 늘 감사합니다!!</v>
       </c>
       <c r="J369" t="str">
         <v>플래너 관리를 통해 부족한 부분을 보완할 수 있었어요.</v>
@@ -13803,7 +13803,7 @@
       <c r="E370" t="str" xml:space="preserve">
         <v xml:space="preserve">다른 학원들처럼 딱딱한 분위기가 아닌 편안한 분위기에서 제 의견을 잘 들어주시면서 학습 계획을 짜주셨습니다._x000d_
 계획만 짜놓고 방치하는 게 아닌_x000d_
-진도율까지 확인해주셔서 과제를 미루지 않고 끝내는 데에 도움이 되었습니다</v>
+진도율까지 확인해 주셔서 과제를 미루지 않고 끝내는 데에 도움이 되었습니다</v>
       </c>
       <c r="F370" t="str">
         <v>과외처럼 1대1 대면으로 모르는 게 더이상 없어질 때까지 질문을 드릴 수 있는 게 가장 큰 메리트였고 여러 선생님께 여러 풀이법을 들을 수 있는 점이 문제 접근성을 높이는 데에 도움이 되었습니다</v>
@@ -13812,11 +13812,11 @@
         <v>카드로 간단하게 출석체크가 가능하고 번호를 입력해서도 가능했습니다. 그리고 출입 시에 초인종을 눌러야만 문을 통과할 수 있는 게 보안 측면에서도 학업 측면에서도 도움이 되었습니다.</v>
       </c>
       <c r="H370" t="str">
-        <v>현역이라서 모의고사 시험 경험이 부족했는데 실전같은 분위기에서 omr 체크까지 연습하며 모의고사를 칠 수 있는 건 큰 장점이었습니다. 오답 해설 강의까지 해주셔서 실전력과 함께 얻어가는 게 많았습니다</v>
+        <v>현역이라서 모의고사 시험 경험이 부족했는데 실전같은 분위기에서 omr 체크까지 연습하며 모의고사를 칠 수 있는 건 큰 장점이었습니다. 오답 해설 강의까지 해 주셔서 실전력과 함께 얻어가는 게 많았습니다</v>
       </c>
       <c r="I370" t="str" xml:space="preserve">
         <v xml:space="preserve">다른 학원은 삭막한 분위기 때문에 다니기 싫었는데 말도 많이 걸어주시고 친근하게 다가와주셔서 심리안정이 많이 됐습니다_x000d_
-학업 측면 말고도 멘탈 관리, 학과 정보까지 다 상담해주셔서 1년이 빨리 지나갔습니다 감사합니다!!</v>
+학업 측면 말고도 멘탈 관리, 학과 정보까지 다 상담해 주셔서 1년이 빨리 지나갔습니다 감사합니다!!</v>
       </c>
       <c r="J370" t="str">
         <v>다른 학원들처럼 딱딱한 분위기가 아닌 편안한 분위기에서 제 의견을 잘 들어주시면서 학습 계획을 짜주셨었어요.</v>

</xml_diff>